<commit_message>
Update trains and loco export 2026-04-04 18:47:57
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -3376,22 +3376,22 @@
       </c>
       <c r="G58" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8121</t>
+          <t>VLINE-8120</t>
         </is>
       </c>
       <c r="H58" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8406</t>
+          <t>VLINE-8404</t>
         </is>
       </c>
       <c r="I58" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8727</t>
+          <t>VLINE-8726</t>
         </is>
       </c>
       <c r="J58" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8817</t>
+          <t>VLINE-8816</t>
         </is>
       </c>
     </row>
@@ -3428,22 +3428,22 @@
       </c>
       <c r="G59" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8124</t>
+          <t>VLINE-8121</t>
         </is>
       </c>
       <c r="H59" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8408</t>
+          <t>VLINE-8406</t>
         </is>
       </c>
       <c r="I59" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8729</t>
+          <t>VLINE-8727</t>
         </is>
       </c>
       <c r="J59" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8818</t>
+          <t>VLINE-8817</t>
         </is>
       </c>
     </row>
@@ -3480,22 +3480,22 @@
       </c>
       <c r="G60" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8126</t>
+          <t>VLINE-8124</t>
         </is>
       </c>
       <c r="H60" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8411</t>
+          <t>VLINE-8408</t>
         </is>
       </c>
       <c r="I60" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8730</t>
+          <t>VLINE-8729</t>
         </is>
       </c>
       <c r="J60" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8819</t>
+          <t>VLINE-8818</t>
         </is>
       </c>
     </row>
@@ -3532,22 +3532,22 @@
       </c>
       <c r="G61" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8127</t>
+          <t>VLINE-8126</t>
         </is>
       </c>
       <c r="H61" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8413</t>
+          <t>VLINE-8411</t>
         </is>
       </c>
       <c r="I61" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8731</t>
+          <t>VLINE-8730</t>
         </is>
       </c>
       <c r="J61" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8822</t>
+          <t>VLINE-8819</t>
         </is>
       </c>
     </row>
@@ -3584,22 +3584,22 @@
       </c>
       <c r="G62" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8128</t>
+          <t>VLINE-8127</t>
         </is>
       </c>
       <c r="H62" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8415</t>
+          <t>VLINE-8413</t>
         </is>
       </c>
       <c r="I62" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8733</t>
+          <t>VLINE-8731</t>
         </is>
       </c>
       <c r="J62" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8860</t>
+          <t>VLINE-8822</t>
         </is>
       </c>
     </row>
@@ -3636,22 +3636,22 @@
       </c>
       <c r="G63" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8129</t>
+          <t>VLINE-8128</t>
         </is>
       </c>
       <c r="H63" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8417</t>
+          <t>VLINE-8415</t>
         </is>
       </c>
       <c r="I63" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8735</t>
+          <t>VLINE-8733</t>
         </is>
       </c>
       <c r="J63" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8861</t>
+          <t>VLINE-8860</t>
         </is>
       </c>
     </row>
@@ -3688,22 +3688,22 @@
       </c>
       <c r="G64" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8132</t>
+          <t>VLINE-8129</t>
         </is>
       </c>
       <c r="H64" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8418</t>
+          <t>VLINE-8417</t>
         </is>
       </c>
       <c r="I64" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8736</t>
+          <t>VLINE-8735</t>
         </is>
       </c>
       <c r="J64" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8862</t>
+          <t>VLINE-8861</t>
         </is>
       </c>
     </row>
@@ -3740,22 +3740,22 @@
       </c>
       <c r="G65" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8134</t>
+          <t>VLINE-8132</t>
         </is>
       </c>
       <c r="H65" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8419</t>
+          <t>VLINE-8418</t>
         </is>
       </c>
       <c r="I65" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8737</t>
+          <t>VLINE-8736</t>
         </is>
       </c>
       <c r="J65" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8863</t>
+          <t>VLINE-8862</t>
         </is>
       </c>
     </row>
@@ -3787,27 +3787,27 @@
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>TT131</t>
+          <t>TT130</t>
         </is>
       </c>
       <c r="G66" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8136</t>
+          <t>VLINE-8134</t>
         </is>
       </c>
       <c r="H66" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8420</t>
+          <t>VLINE-8419</t>
         </is>
       </c>
       <c r="I66" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8739</t>
+          <t>VLINE-8737</t>
         </is>
       </c>
       <c r="J66" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8864</t>
+          <t>VLINE-8863</t>
         </is>
       </c>
     </row>
@@ -3839,27 +3839,27 @@
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT131</t>
         </is>
       </c>
       <c r="G67" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8145</t>
+          <t>VLINE-8136</t>
         </is>
       </c>
       <c r="H67" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8421</t>
+          <t>VLINE-8420</t>
         </is>
       </c>
       <c r="I67" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8740</t>
+          <t>VLINE-8739</t>
         </is>
       </c>
       <c r="J67" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8865</t>
+          <t>VLINE-8864</t>
         </is>
       </c>
     </row>
@@ -3891,27 +3891,27 @@
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT202</t>
         </is>
       </c>
       <c r="G68" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8148</t>
+          <t>VLINE-8145</t>
         </is>
       </c>
       <c r="H68" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8422</t>
+          <t>VLINE-8421</t>
         </is>
       </c>
       <c r="I68" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8741</t>
+          <t>VLINE-8740</t>
         </is>
       </c>
       <c r="J68" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8866</t>
+          <t>VLINE-8865</t>
         </is>
       </c>
     </row>
@@ -3943,27 +3943,27 @@
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>VL352</t>
+          <t>TT206</t>
         </is>
       </c>
       <c r="G69" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8150</t>
+          <t>VLINE-8148</t>
         </is>
       </c>
       <c r="H69" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8424</t>
+          <t>VLINE-8422</t>
         </is>
       </c>
       <c r="I69" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8742</t>
+          <t>VLINE-8741</t>
         </is>
       </c>
       <c r="J69" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8867</t>
+          <t>VLINE-8866</t>
         </is>
       </c>
     </row>
@@ -3995,27 +3995,27 @@
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>VL353</t>
+          <t>VL352</t>
         </is>
       </c>
       <c r="G70" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8151</t>
+          <t>VLINE-8150</t>
         </is>
       </c>
       <c r="H70" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8425</t>
+          <t>VLINE-8424</t>
         </is>
       </c>
       <c r="I70" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8743</t>
+          <t>VLINE-8742</t>
         </is>
       </c>
       <c r="J70" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8868</t>
+          <t>VLINE-8867</t>
         </is>
       </c>
     </row>
@@ -4047,27 +4047,27 @@
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>VL357</t>
+          <t>VL353</t>
         </is>
       </c>
       <c r="G71" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8152</t>
+          <t>VLINE-8151</t>
         </is>
       </c>
       <c r="H71" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8426</t>
+          <t>VLINE-8425</t>
         </is>
       </c>
       <c r="I71" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8744</t>
+          <t>VLINE-8743</t>
         </is>
       </c>
       <c r="J71" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8869</t>
+          <t>VLINE-8868</t>
         </is>
       </c>
     </row>
@@ -4099,27 +4099,27 @@
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8004</t>
+          <t>VL357</t>
         </is>
       </c>
       <c r="G72" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8153</t>
+          <t>VLINE-8152</t>
         </is>
       </c>
       <c r="H72" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8427</t>
+          <t>VLINE-8426</t>
         </is>
       </c>
       <c r="I72" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8745</t>
+          <t>VLINE-8744</t>
         </is>
       </c>
       <c r="J72" s="1" t="inlineStr">
         <is>
-          <t>WH001</t>
+          <t>VLINE-8869</t>
         </is>
       </c>
     </row>
@@ -4151,27 +4151,27 @@
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8007</t>
+          <t>VLINE-8004</t>
         </is>
       </c>
       <c r="G73" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8154</t>
+          <t>VLINE-8153</t>
         </is>
       </c>
       <c r="H73" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8428</t>
+          <t>VLINE-8427</t>
         </is>
       </c>
       <c r="I73" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8746</t>
+          <t>VLINE-8745</t>
         </is>
       </c>
       <c r="J73" s="1" t="inlineStr">
         <is>
-          <t>WH003</t>
+          <t>WH001</t>
         </is>
       </c>
     </row>
@@ -4203,27 +4203,27 @@
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8011</t>
+          <t>VLINE-8007</t>
         </is>
       </c>
       <c r="G74" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8155</t>
+          <t>VLINE-8154</t>
         </is>
       </c>
       <c r="H74" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8429</t>
+          <t>VLINE-8428</t>
         </is>
       </c>
       <c r="I74" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8748</t>
+          <t>VLINE-8746</t>
         </is>
       </c>
       <c r="J74" s="1" t="inlineStr">
         <is>
-          <t>WL02</t>
+          <t>WH003</t>
         </is>
       </c>
     </row>
@@ -4255,27 +4255,27 @@
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8013</t>
+          <t>VLINE-8011</t>
         </is>
       </c>
       <c r="G75" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8157</t>
+          <t>VLINE-8155</t>
         </is>
       </c>
       <c r="H75" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8430</t>
+          <t>VLINE-8429</t>
         </is>
       </c>
       <c r="I75" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8750</t>
+          <t>VLINE-8748</t>
         </is>
       </c>
       <c r="J75" s="1" t="inlineStr">
         <is>
-          <t>X12-X14</t>
+          <t>WL02</t>
         </is>
       </c>
     </row>
@@ -4307,27 +4307,27 @@
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8019</t>
+          <t>VLINE-8013</t>
         </is>
       </c>
       <c r="G76" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8158</t>
+          <t>VLINE-8157</t>
         </is>
       </c>
       <c r="H76" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8432</t>
+          <t>VLINE-8430</t>
         </is>
       </c>
       <c r="I76" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8751</t>
+          <t>VLINE-8750</t>
         </is>
       </c>
       <c r="J76" s="1" t="inlineStr">
         <is>
-          <t>X31</t>
+          <t>X12-X14</t>
         </is>
       </c>
     </row>
@@ -4359,27 +4359,27 @@
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8020</t>
+          <t>VLINE-8019</t>
         </is>
       </c>
       <c r="G77" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8159</t>
+          <t>VLINE-8158</t>
         </is>
       </c>
       <c r="H77" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8434</t>
+          <t>VLINE-8432</t>
         </is>
       </c>
       <c r="I77" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8752</t>
+          <t>VLINE-8751</t>
         </is>
       </c>
       <c r="J77" s="1" t="inlineStr">
         <is>
-          <t>XP2000</t>
+          <t>X31</t>
         </is>
       </c>
     </row>
@@ -4411,27 +4411,27 @@
       </c>
       <c r="F78" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8023</t>
+          <t>VLINE-8020</t>
         </is>
       </c>
       <c r="G78" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8160</t>
+          <t>VLINE-8159</t>
         </is>
       </c>
       <c r="H78" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8441</t>
+          <t>VLINE-8434</t>
         </is>
       </c>
       <c r="I78" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8753</t>
+          <t>VLINE-8752</t>
         </is>
       </c>
       <c r="J78" s="1" t="inlineStr">
         <is>
-          <t>XP2003</t>
+          <t>XP2000</t>
         </is>
       </c>
     </row>
@@ -4463,27 +4463,27 @@
       </c>
       <c r="F79" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8025</t>
+          <t>VLINE-8023</t>
         </is>
       </c>
       <c r="G79" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8161</t>
+          <t>VLINE-8160</t>
         </is>
       </c>
       <c r="H79" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8443</t>
+          <t>VLINE-8441</t>
         </is>
       </c>
       <c r="I79" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8754</t>
+          <t>VLINE-8753</t>
         </is>
       </c>
       <c r="J79" s="1" t="inlineStr">
         <is>
-          <t>XP2004</t>
+          <t>XP2003</t>
         </is>
       </c>
     </row>
@@ -4515,27 +4515,27 @@
       </c>
       <c r="F80" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8026</t>
+          <t>VLINE-8025</t>
         </is>
       </c>
       <c r="G80" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8162</t>
+          <t>VLINE-8161</t>
         </is>
       </c>
       <c r="H80" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8444</t>
+          <t>VLINE-8443</t>
         </is>
       </c>
       <c r="I80" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8755</t>
+          <t>VLINE-8754</t>
         </is>
       </c>
       <c r="J80" s="1" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>XP2004</t>
         </is>
       </c>
     </row>
@@ -4567,27 +4567,27 @@
       </c>
       <c r="F81" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8027</t>
+          <t>VLINE-8026</t>
         </is>
       </c>
       <c r="G81" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8171</t>
+          <t>VLINE-8162</t>
         </is>
       </c>
       <c r="H81" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8446</t>
+          <t>VLINE-8444</t>
         </is>
       </c>
       <c r="I81" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8756</t>
+          <t>VLINE-8755</t>
         </is>
       </c>
       <c r="J81" s="1" t="inlineStr">
         <is>
-          <t>XP2007</t>
+          <t>XP2005</t>
         </is>
       </c>
     </row>
@@ -4619,27 +4619,27 @@
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8028</t>
+          <t>VLINE-8027</t>
         </is>
       </c>
       <c r="G82" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8172</t>
+          <t>VLINE-8171</t>
         </is>
       </c>
       <c r="H82" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8447</t>
+          <t>VLINE-8446</t>
         </is>
       </c>
       <c r="I82" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8757</t>
+          <t>VLINE-8756</t>
         </is>
       </c>
       <c r="J82" s="1" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>XP2007</t>
         </is>
       </c>
     </row>
@@ -4671,27 +4671,27 @@
       </c>
       <c r="F83" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8030</t>
+          <t>VLINE-8028</t>
         </is>
       </c>
       <c r="G83" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8179</t>
+          <t>VLINE-8172</t>
         </is>
       </c>
       <c r="H83" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8449</t>
+          <t>VLINE-8447</t>
         </is>
       </c>
       <c r="I83" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8758</t>
+          <t>VLINE-8757</t>
         </is>
       </c>
       <c r="J83" s="1" t="inlineStr">
         <is>
-          <t>XP2010</t>
+          <t>XP2008</t>
         </is>
       </c>
     </row>
@@ -4723,27 +4723,27 @@
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8032</t>
+          <t>VLINE-8030</t>
         </is>
       </c>
       <c r="G84" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8180</t>
+          <t>VLINE-8179</t>
         </is>
       </c>
       <c r="H84" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8450</t>
+          <t>VLINE-8449</t>
         </is>
       </c>
       <c r="I84" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8759</t>
+          <t>VLINE-8758</t>
         </is>
       </c>
       <c r="J84" s="1" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>XP2010</t>
         </is>
       </c>
     </row>
@@ -4775,27 +4775,27 @@
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8036</t>
+          <t>VLINE-8032</t>
         </is>
       </c>
       <c r="G85" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8181</t>
+          <t>VLINE-8180</t>
         </is>
       </c>
       <c r="H85" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8451</t>
+          <t>VLINE-8450</t>
         </is>
       </c>
       <c r="I85" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8760</t>
+          <t>VLINE-8759</t>
         </is>
       </c>
       <c r="J85" s="1" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>XP2011</t>
         </is>
       </c>
     </row>
@@ -4827,27 +4827,27 @@
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8051</t>
+          <t>VLINE-8036</t>
         </is>
       </c>
       <c r="G86" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8182</t>
+          <t>VLINE-8181</t>
         </is>
       </c>
       <c r="H86" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8452</t>
+          <t>VLINE-8451</t>
         </is>
       </c>
       <c r="I86" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8761</t>
+          <t>VLINE-8760</t>
         </is>
       </c>
       <c r="J86" s="1" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>XP2012</t>
         </is>
       </c>
     </row>
@@ -4879,27 +4879,27 @@
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8052</t>
+          <t>VLINE-8051</t>
         </is>
       </c>
       <c r="G87" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8183</t>
+          <t>VLINE-8182</t>
         </is>
       </c>
       <c r="H87" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8453</t>
+          <t>VLINE-8452</t>
         </is>
       </c>
       <c r="I87" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8762</t>
+          <t>VLINE-8761</t>
         </is>
       </c>
       <c r="J87" s="1" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>XP2013</t>
         </is>
       </c>
     </row>
@@ -4931,27 +4931,27 @@
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8053</t>
+          <t>VLINE-8052</t>
         </is>
       </c>
       <c r="G88" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8184</t>
+          <t>VLINE-8183</t>
         </is>
       </c>
       <c r="H88" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8454</t>
+          <t>VLINE-8453</t>
         </is>
       </c>
       <c r="I88" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8770</t>
+          <t>VLINE-8762</t>
         </is>
       </c>
       <c r="J88" s="1" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>XP2014</t>
         </is>
       </c>
     </row>
@@ -4983,27 +4983,27 @@
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8055</t>
+          <t>VLINE-8053</t>
         </is>
       </c>
       <c r="G89" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8185</t>
+          <t>VLINE-8184</t>
         </is>
       </c>
       <c r="H89" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8455</t>
+          <t>VLINE-8454</t>
         </is>
       </c>
       <c r="I89" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8772</t>
+          <t>VLINE-8770</t>
         </is>
       </c>
       <c r="J89" s="1" t="inlineStr">
         <is>
-          <t>XP2016</t>
+          <t>XP2015</t>
         </is>
       </c>
     </row>
@@ -5035,27 +5035,27 @@
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8056</t>
+          <t>VLINE-8055</t>
         </is>
       </c>
       <c r="G90" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8186</t>
+          <t>VLINE-8185</t>
         </is>
       </c>
       <c r="H90" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8456</t>
+          <t>VLINE-8455</t>
         </is>
       </c>
       <c r="I90" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8774</t>
+          <t>VLINE-8772</t>
         </is>
       </c>
       <c r="J90" s="1" t="inlineStr">
         <is>
-          <t>XP2017</t>
+          <t>XP2016</t>
         </is>
       </c>
     </row>
@@ -5087,27 +5087,27 @@
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8057</t>
+          <t>VLINE-8056</t>
         </is>
       </c>
       <c r="G91" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8187</t>
+          <t>VLINE-8186</t>
         </is>
       </c>
       <c r="H91" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8457</t>
+          <t>VLINE-8456</t>
         </is>
       </c>
       <c r="I91" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8776</t>
+          <t>VLINE-8774</t>
         </is>
       </c>
       <c r="J91" s="1" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>XP2017</t>
         </is>
       </c>
     </row>
@@ -5139,27 +5139,27 @@
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8058</t>
+          <t>VLINE-8057</t>
         </is>
       </c>
       <c r="G92" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8189</t>
+          <t>VLINE-8187</t>
         </is>
       </c>
       <c r="H92" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8460</t>
+          <t>VLINE-8457</t>
         </is>
       </c>
       <c r="I92" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8778</t>
+          <t>VLINE-8776</t>
         </is>
       </c>
       <c r="J92" s="1" t="inlineStr">
         <is>
-          <t>XR552</t>
+          <t>XP2019</t>
         </is>
       </c>
     </row>
@@ -5191,27 +5191,27 @@
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8059</t>
+          <t>VLINE-8058</t>
         </is>
       </c>
       <c r="G93" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8303</t>
+          <t>VLINE-8189</t>
         </is>
       </c>
       <c r="H93" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8461</t>
+          <t>VLINE-8460</t>
         </is>
       </c>
       <c r="I93" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8780</t>
+          <t>VLINE-8778</t>
         </is>
       </c>
       <c r="J93" s="1" t="inlineStr">
         <is>
-          <t>XRN001</t>
+          <t>XR550</t>
         </is>
       </c>
     </row>
@@ -5243,27 +5243,27 @@
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8061</t>
+          <t>VLINE-8059</t>
         </is>
       </c>
       <c r="G94" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8304</t>
+          <t>VLINE-8303</t>
         </is>
       </c>
       <c r="H94" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8464</t>
+          <t>VLINE-8461</t>
         </is>
       </c>
       <c r="I94" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8793</t>
+          <t>VLINE-8780</t>
         </is>
       </c>
       <c r="J94" s="1" t="inlineStr">
         <is>
-          <t>XRN004</t>
+          <t>XR552</t>
         </is>
       </c>
     </row>
@@ -5295,27 +5295,27 @@
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8072</t>
+          <t>VLINE-8061</t>
         </is>
       </c>
       <c r="G95" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8311</t>
+          <t>VLINE-8304</t>
         </is>
       </c>
       <c r="H95" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8465</t>
+          <t>VLINE-8464</t>
         </is>
       </c>
       <c r="I95" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8795</t>
+          <t>VLINE-8793</t>
         </is>
       </c>
       <c r="J95" s="1" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>XRN001</t>
         </is>
       </c>
     </row>
@@ -5347,27 +5347,27 @@
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8074</t>
+          <t>VLINE-8072</t>
         </is>
       </c>
       <c r="G96" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8313</t>
+          <t>VLINE-8311</t>
         </is>
       </c>
       <c r="H96" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8468</t>
+          <t>VLINE-8465</t>
         </is>
       </c>
       <c r="I96" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8797</t>
+          <t>VLINE-8795</t>
         </is>
       </c>
       <c r="J96" s="1" t="inlineStr">
         <is>
-          <t>XRN006</t>
+          <t>XRN004</t>
         </is>
       </c>
     </row>
@@ -5399,27 +5399,27 @@
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8075</t>
+          <t>VLINE-8074</t>
         </is>
       </c>
       <c r="G97" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8314</t>
+          <t>VLINE-8313</t>
         </is>
       </c>
       <c r="H97" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8469</t>
+          <t>VLINE-8468</t>
         </is>
       </c>
       <c r="I97" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8799</t>
+          <t>VLINE-8797</t>
         </is>
       </c>
       <c r="J97" s="1" t="inlineStr">
         <is>
-          <t>XRN007</t>
+          <t>XRN005</t>
         </is>
       </c>
     </row>
@@ -5451,27 +5451,27 @@
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8076</t>
+          <t>VLINE-8075</t>
         </is>
       </c>
       <c r="G98" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8316</t>
+          <t>VLINE-8314</t>
         </is>
       </c>
       <c r="H98" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8605</t>
+          <t>VLINE-8469</t>
         </is>
       </c>
       <c r="I98" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8800</t>
+          <t>VLINE-8799</t>
         </is>
       </c>
       <c r="J98" s="1" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>XRN006</t>
         </is>
       </c>
     </row>
@@ -5503,27 +5503,27 @@
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8077</t>
+          <t>VLINE-8076</t>
         </is>
       </c>
       <c r="G99" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8318</t>
+          <t>VLINE-8316</t>
         </is>
       </c>
       <c r="H99" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8610</t>
+          <t>VLINE-8605</t>
         </is>
       </c>
       <c r="I99" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8801</t>
+          <t>VLINE-8800</t>
         </is>
       </c>
       <c r="J99" s="1" t="inlineStr">
         <is>
-          <t>XRN011</t>
+          <t>XRN007</t>
         </is>
       </c>
     </row>
@@ -5555,27 +5555,27 @@
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8080</t>
+          <t>VLINE-8077</t>
         </is>
       </c>
       <c r="G100" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8321</t>
+          <t>VLINE-8318</t>
         </is>
       </c>
       <c r="H100" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8612</t>
+          <t>VLINE-8610</t>
         </is>
       </c>
       <c r="I100" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8802</t>
+          <t>VLINE-8801</t>
         </is>
       </c>
       <c r="J100" s="1" t="inlineStr">
         <is>
-          <t>XRN014</t>
+          <t>XRN009</t>
         </is>
       </c>
     </row>
@@ -5607,27 +5607,27 @@
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8081</t>
+          <t>VLINE-8080</t>
         </is>
       </c>
       <c r="G101" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8324</t>
+          <t>VLINE-8321</t>
         </is>
       </c>
       <c r="H101" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8615</t>
+          <t>VLINE-8612</t>
         </is>
       </c>
       <c r="I101" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8803</t>
+          <t>VLINE-8802</t>
         </is>
       </c>
       <c r="J101" s="1" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>XRN011</t>
         </is>
       </c>
     </row>
@@ -5659,27 +5659,27 @@
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8084</t>
+          <t>VLINE-8081</t>
         </is>
       </c>
       <c r="G102" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8332</t>
+          <t>VLINE-8324</t>
         </is>
       </c>
       <c r="H102" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8620</t>
+          <t>VLINE-8615</t>
         </is>
       </c>
       <c r="I102" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8804</t>
+          <t>VLINE-8803</t>
         </is>
       </c>
       <c r="J102" s="1" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>XRN014</t>
         </is>
       </c>
     </row>
@@ -5711,27 +5711,27 @@
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8088</t>
+          <t>VLINE-8084</t>
         </is>
       </c>
       <c r="G103" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8336</t>
+          <t>VLINE-8332</t>
         </is>
       </c>
       <c r="H103" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8625</t>
+          <t>VLINE-8620</t>
         </is>
       </c>
       <c r="I103" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8805</t>
+          <t>VLINE-8804</t>
         </is>
       </c>
       <c r="J103" s="1" t="inlineStr">
         <is>
-          <t>XRN020</t>
+          <t>XRN017</t>
         </is>
       </c>
     </row>
@@ -5763,27 +5763,27 @@
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8089</t>
+          <t>VLINE-8088</t>
         </is>
       </c>
       <c r="G104" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8337</t>
+          <t>VLINE-8336</t>
         </is>
       </c>
       <c r="H104" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8630</t>
+          <t>VLINE-8625</t>
         </is>
       </c>
       <c r="I104" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8806</t>
+          <t>VLINE-8805</t>
         </is>
       </c>
       <c r="J104" s="1" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>XRN018</t>
         </is>
       </c>
     </row>
@@ -5815,27 +5815,27 @@
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8104</t>
+          <t>VLINE-8089</t>
         </is>
       </c>
       <c r="G105" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8338</t>
+          <t>VLINE-8337</t>
         </is>
       </c>
       <c r="H105" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8671</t>
+          <t>VLINE-8630</t>
         </is>
       </c>
       <c r="I105" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8807</t>
+          <t>VLINE-8806</t>
         </is>
       </c>
       <c r="J105" s="1" t="inlineStr">
         <is>
-          <t>XRN023</t>
+          <t>XRN020</t>
         </is>
       </c>
     </row>
@@ -5867,27 +5867,27 @@
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8107</t>
+          <t>VLINE-8104</t>
         </is>
       </c>
       <c r="G106" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8339</t>
+          <t>VLINE-8338</t>
         </is>
       </c>
       <c r="H106" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8706</t>
+          <t>VLINE-8671</t>
         </is>
       </c>
       <c r="I106" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8808</t>
+          <t>VLINE-8807</t>
         </is>
       </c>
       <c r="J106" s="1" t="inlineStr">
         <is>
-          <t>XRN025</t>
+          <t>XRN021</t>
         </is>
       </c>
     </row>
@@ -5919,27 +5919,27 @@
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8110</t>
+          <t>VLINE-8107</t>
         </is>
       </c>
       <c r="G107" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8362</t>
+          <t>VLINE-8339</t>
         </is>
       </c>
       <c r="H107" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8711</t>
+          <t>VLINE-8706</t>
         </is>
       </c>
       <c r="I107" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8809</t>
+          <t>VLINE-8808</t>
         </is>
       </c>
       <c r="J107" s="1" t="inlineStr">
         <is>
-          <t>XRN026</t>
+          <t>XRN023</t>
         </is>
       </c>
     </row>
@@ -5971,27 +5971,27 @@
       </c>
       <c r="F108" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8111</t>
+          <t>VLINE-8110</t>
         </is>
       </c>
       <c r="G108" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8363</t>
+          <t>VLINE-8362</t>
         </is>
       </c>
       <c r="H108" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8714</t>
+          <t>VLINE-8711</t>
         </is>
       </c>
       <c r="I108" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8810</t>
+          <t>VLINE-8809</t>
         </is>
       </c>
       <c r="J108" s="1" t="inlineStr">
         <is>
-          <t>XRN027</t>
+          <t>XRN025</t>
         </is>
       </c>
     </row>
@@ -6023,27 +6023,27 @@
       </c>
       <c r="F109" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8113</t>
+          <t>VLINE-8111</t>
         </is>
       </c>
       <c r="G109" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8365</t>
+          <t>VLINE-8363</t>
         </is>
       </c>
       <c r="H109" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8717</t>
+          <t>VLINE-8714</t>
         </is>
       </c>
       <c r="I109" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8811</t>
+          <t>VLINE-8810</t>
         </is>
       </c>
       <c r="J109" s="1" t="inlineStr">
         <is>
-          <t>Y163</t>
+          <t>XRN026</t>
         </is>
       </c>
     </row>
@@ -6075,22 +6075,27 @@
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8114</t>
+          <t>VLINE-8113</t>
         </is>
       </c>
       <c r="G110" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8366</t>
+          <t>VLINE-8365</t>
         </is>
       </c>
       <c r="H110" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8721</t>
+          <t>VLINE-8717</t>
         </is>
       </c>
       <c r="I110" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8812</t>
+          <t>VLINE-8811</t>
+        </is>
+      </c>
+      <c r="J110" s="1" t="inlineStr">
+        <is>
+          <t>XRN027</t>
         </is>
       </c>
     </row>
@@ -6122,22 +6127,27 @@
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8115</t>
+          <t>VLINE-8114</t>
         </is>
       </c>
       <c r="G111" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8369</t>
+          <t>VLINE-8366</t>
         </is>
       </c>
       <c r="H111" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8723</t>
+          <t>VLINE-8721</t>
         </is>
       </c>
       <c r="I111" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8813</t>
+          <t>VLINE-8812</t>
+        </is>
+      </c>
+      <c r="J111" s="1" t="inlineStr">
+        <is>
+          <t>Y163</t>
         </is>
       </c>
     </row>
@@ -6169,22 +6179,22 @@
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8119</t>
+          <t>VLINE-8115</t>
         </is>
       </c>
       <c r="G112" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8403</t>
+          <t>VLINE-8369</t>
         </is>
       </c>
       <c r="H112" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8725</t>
+          <t>VLINE-8723</t>
         </is>
       </c>
       <c r="I112" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8814</t>
+          <t>VLINE-8813</t>
         </is>
       </c>
     </row>
@@ -6216,22 +6226,22 @@
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8120</t>
+          <t>VLINE-8119</t>
         </is>
       </c>
       <c r="G113" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8404</t>
+          <t>VLINE-8403</t>
         </is>
       </c>
       <c r="H113" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8726</t>
+          <t>VLINE-8725</t>
         </is>
       </c>
       <c r="I113" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8816</t>
+          <t>VLINE-8814</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update trains and loco export 2026-04-04 20:04:37
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -467,7 +467,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>HM2707</t>
+          <t>HM2706</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>HM2751</t>
+          <t>HM2707</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t>HM2753</t>
+          <t>HM2751</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>HM2754</t>
+          <t>HM2753</t>
         </is>
       </c>
     </row>
@@ -635,7 +635,7 @@
       </c>
       <c r="H5" s="1" t="inlineStr">
         <is>
-          <t>HM2755</t>
+          <t>HM2754</t>
         </is>
       </c>
     </row>
@@ -677,7 +677,7 @@
       </c>
       <c r="H6" s="1" t="inlineStr">
         <is>
-          <t>HM2756</t>
+          <t>HM2755</t>
         </is>
       </c>
     </row>
@@ -719,7 +719,7 @@
       </c>
       <c r="H7" s="1" t="inlineStr">
         <is>
-          <t>HM2757</t>
+          <t>HM2756</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="H8" s="1" t="inlineStr">
         <is>
-          <t>JHRTST</t>
+          <t>HM2757</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="H9" s="1" t="inlineStr">
         <is>
-          <t>JP2296-5</t>
+          <t>JHRTST</t>
         </is>
       </c>
     </row>
@@ -845,7 +845,7 @@
       </c>
       <c r="H10" s="1" t="inlineStr">
         <is>
-          <t>JP2296-6</t>
+          <t>JP2296-5</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       </c>
       <c r="H11" s="1" t="inlineStr">
         <is>
-          <t>JP2298-5</t>
+          <t>JP2296-6</t>
         </is>
       </c>
     </row>
@@ -929,7 +929,7 @@
       </c>
       <c r="H12" s="1" t="inlineStr">
         <is>
-          <t>JP2299-6</t>
+          <t>JP2298-5</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="H13" s="1" t="inlineStr">
         <is>
-          <t>JP2300-6</t>
+          <t>JP2299-6</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="H14" s="1" t="inlineStr">
         <is>
-          <t>JP2333-6</t>
+          <t>JP2300-6</t>
         </is>
       </c>
     </row>
@@ -1055,7 +1055,7 @@
       </c>
       <c r="H15" s="1" t="inlineStr">
         <is>
-          <t>JP2335-6</t>
+          <t>JP2333-6</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="H16" s="1" t="inlineStr">
         <is>
-          <t>JP2337-5</t>
+          <t>JP2335-6</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="H17" s="1" t="inlineStr">
         <is>
-          <t>JP2340-5</t>
+          <t>JP2337-5</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="H18" s="1" t="inlineStr">
         <is>
-          <t>JP2474-5</t>
+          <t>JP2340-5</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="H19" s="1" t="inlineStr">
         <is>
-          <t>JP2532-5</t>
+          <t>JP2474-5</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="H20" s="1" t="inlineStr">
         <is>
-          <t>JP2535-5</t>
+          <t>JP2532-5</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       </c>
       <c r="H21" s="1" t="inlineStr">
         <is>
-          <t>JP2536-5</t>
+          <t>JP2535-5</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="H22" s="1" t="inlineStr">
         <is>
-          <t>JP2537-1</t>
+          <t>JP2536-5</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="H23" s="1" t="inlineStr">
         <is>
-          <t>JP2537-5</t>
+          <t>JP2537-1</t>
         </is>
       </c>
     </row>
@@ -1433,7 +1433,7 @@
       </c>
       <c r="H24" s="1" t="inlineStr">
         <is>
-          <t>JP2540-5</t>
+          <t>JP2537-5</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="H25" s="1" t="inlineStr">
         <is>
-          <t>JP2542-1</t>
+          <t>JP2540-5</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="H26" s="1" t="inlineStr">
         <is>
-          <t>JP2542-5</t>
+          <t>JP2542-1</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="H27" s="1" t="inlineStr">
         <is>
-          <t>JP2544-6</t>
+          <t>JP2542-5</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="H28" s="1" t="inlineStr">
         <is>
-          <t>JP2546-5</t>
+          <t>JP2544-6</t>
         </is>
       </c>
     </row>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="H29" s="1" t="inlineStr">
         <is>
-          <t>JP9750-6</t>
+          <t>JP2546-5</t>
         </is>
       </c>
     </row>
@@ -1685,7 +1685,7 @@
       </c>
       <c r="H30" s="1" t="inlineStr">
         <is>
-          <t>LDP003</t>
+          <t>JP9750-6</t>
         </is>
       </c>
     </row>
@@ -1727,7 +1727,7 @@
       </c>
       <c r="H31" s="1" t="inlineStr">
         <is>
-          <t>LDP007</t>
+          <t>LDP003</t>
         </is>
       </c>
     </row>
@@ -1769,7 +1769,7 @@
       </c>
       <c r="H32" s="1" t="inlineStr">
         <is>
-          <t>LDP009</t>
+          <t>LDP007</t>
         </is>
       </c>
     </row>
@@ -1811,7 +1811,7 @@
       </c>
       <c r="H33" s="1" t="inlineStr">
         <is>
-          <t>LE2851</t>
+          <t>LDP009</t>
         </is>
       </c>
     </row>
@@ -1848,12 +1848,12 @@
       </c>
       <c r="G34" s="1" t="inlineStr">
         <is>
-          <t>GM27</t>
+          <t>GM22</t>
         </is>
       </c>
       <c r="H34" s="1" t="inlineStr">
         <is>
-          <t>LE2852</t>
+          <t>LE2851</t>
         </is>
       </c>
     </row>
@@ -1890,12 +1890,12 @@
       </c>
       <c r="G35" s="1" t="inlineStr">
         <is>
-          <t>GM46</t>
+          <t>GM27</t>
         </is>
       </c>
       <c r="H35" s="1" t="inlineStr">
         <is>
-          <t>LE2853</t>
+          <t>LE2852</t>
         </is>
       </c>
     </row>
@@ -1932,12 +1932,12 @@
       </c>
       <c r="G36" s="1" t="inlineStr">
         <is>
-          <t>GWA001</t>
+          <t>GM46</t>
         </is>
       </c>
       <c r="H36" s="1" t="inlineStr">
         <is>
-          <t>LE2854</t>
+          <t>LE2853</t>
         </is>
       </c>
     </row>
@@ -1974,12 +1974,12 @@
       </c>
       <c r="G37" s="1" t="inlineStr">
         <is>
-          <t>GWA002</t>
+          <t>GWA001</t>
         </is>
       </c>
       <c r="H37" s="1" t="inlineStr">
         <is>
-          <t>LE2855</t>
+          <t>LE2854</t>
         </is>
       </c>
     </row>
@@ -2016,12 +2016,12 @@
       </c>
       <c r="G38" s="1" t="inlineStr">
         <is>
-          <t>GWA004</t>
+          <t>GWA002</t>
         </is>
       </c>
       <c r="H38" s="1" t="inlineStr">
         <is>
-          <t>LE2858</t>
+          <t>LE2855</t>
         </is>
       </c>
     </row>
@@ -2058,12 +2058,12 @@
       </c>
       <c r="G39" s="1" t="inlineStr">
         <is>
-          <t>GWA005</t>
+          <t>GWA004</t>
         </is>
       </c>
       <c r="H39" s="1" t="inlineStr">
         <is>
-          <t>LE2862</t>
+          <t>LE2856</t>
         </is>
       </c>
     </row>
@@ -2100,12 +2100,12 @@
       </c>
       <c r="G40" s="1" t="inlineStr">
         <is>
-          <t>GWA007</t>
+          <t>GWA005</t>
         </is>
       </c>
       <c r="H40" s="1" t="inlineStr">
         <is>
-          <t>LE2863</t>
+          <t>LE2858</t>
         </is>
       </c>
     </row>
@@ -2142,12 +2142,12 @@
       </c>
       <c r="G41" s="1" t="inlineStr">
         <is>
-          <t>GWA010</t>
+          <t>GWA007</t>
         </is>
       </c>
       <c r="H41" s="1" t="inlineStr">
         <is>
-          <t>LE2864</t>
+          <t>LE2862</t>
         </is>
       </c>
     </row>
@@ -2184,12 +2184,12 @@
       </c>
       <c r="G42" s="1" t="inlineStr">
         <is>
-          <t>GWB101</t>
+          <t>GWA010</t>
         </is>
       </c>
       <c r="H42" s="1" t="inlineStr">
         <is>
-          <t>LZ3120</t>
+          <t>LE2863</t>
         </is>
       </c>
     </row>
@@ -2226,12 +2226,12 @@
       </c>
       <c r="G43" s="1" t="inlineStr">
         <is>
-          <t>GWB102</t>
+          <t>GWB101</t>
         </is>
       </c>
       <c r="H43" s="1" t="inlineStr">
         <is>
-          <t>M24</t>
+          <t>LE2864</t>
         </is>
       </c>
     </row>
@@ -2268,12 +2268,12 @@
       </c>
       <c r="G44" s="1" t="inlineStr">
         <is>
-          <t>GWB103</t>
+          <t>GWB102</t>
         </is>
       </c>
       <c r="H44" s="1" t="inlineStr">
         <is>
-          <t>M31</t>
+          <t>LZ3120</t>
         </is>
       </c>
     </row>
@@ -2310,12 +2310,12 @@
       </c>
       <c r="G45" s="1" t="inlineStr">
         <is>
-          <t>GWB105</t>
+          <t>GWB103</t>
         </is>
       </c>
       <c r="H45" s="1" t="inlineStr">
         <is>
-          <t>MAN001</t>
+          <t>M24</t>
         </is>
       </c>
     </row>
@@ -2352,12 +2352,12 @@
       </c>
       <c r="G46" s="1" t="inlineStr">
         <is>
-          <t>GWB106</t>
+          <t>GWB105</t>
         </is>
       </c>
       <c r="H46" s="1" t="inlineStr">
         <is>
-          <t>MAN002</t>
+          <t>M31</t>
         </is>
       </c>
     </row>
@@ -2394,12 +2394,12 @@
       </c>
       <c r="G47" s="1" t="inlineStr">
         <is>
-          <t>GWU005</t>
+          <t>GWB106</t>
         </is>
       </c>
       <c r="H47" s="1" t="inlineStr">
         <is>
-          <t>MAN003</t>
+          <t>MAN001</t>
         </is>
       </c>
     </row>
@@ -2436,12 +2436,12 @@
       </c>
       <c r="G48" s="1" t="inlineStr">
         <is>
-          <t>GWU013</t>
+          <t>GWU005</t>
         </is>
       </c>
       <c r="H48" s="1" t="inlineStr">
         <is>
-          <t>MAN005</t>
+          <t>MAN002</t>
         </is>
       </c>
     </row>
@@ -2478,12 +2478,12 @@
       </c>
       <c r="G49" s="1" t="inlineStr">
         <is>
-          <t>GWU014</t>
+          <t>GWU013</t>
         </is>
       </c>
       <c r="H49" s="1" t="inlineStr">
         <is>
-          <t>MAN007</t>
+          <t>MAN003</t>
         </is>
       </c>
     </row>
@@ -2520,12 +2520,12 @@
       </c>
       <c r="G50" s="1" t="inlineStr">
         <is>
-          <t>H3</t>
+          <t>GWU014</t>
         </is>
       </c>
       <c r="H50" s="1" t="inlineStr">
         <is>
-          <t>MAN008</t>
+          <t>MAN005</t>
         </is>
       </c>
     </row>
@@ -2562,12 +2562,12 @@
       </c>
       <c r="G51" s="1" t="inlineStr">
         <is>
-          <t>HM2701</t>
+          <t>H3</t>
         </is>
       </c>
       <c r="H51" s="1" t="inlineStr">
         <is>
-          <t>MAN009</t>
+          <t>MAN007</t>
         </is>
       </c>
     </row>
@@ -2604,12 +2604,12 @@
       </c>
       <c r="G52" s="1" t="inlineStr">
         <is>
-          <t>HM2702</t>
+          <t>HM2701</t>
         </is>
       </c>
       <c r="H52" s="1" t="inlineStr">
         <is>
-          <t>MAN010</t>
+          <t>MAN008</t>
         </is>
       </c>
     </row>
@@ -2646,12 +2646,12 @@
       </c>
       <c r="G53" s="1" t="inlineStr">
         <is>
-          <t>HM2703</t>
+          <t>HM2702</t>
         </is>
       </c>
       <c r="H53" s="1" t="inlineStr">
         <is>
-          <t>MAN011</t>
+          <t>MAN009</t>
         </is>
       </c>
     </row>
@@ -2688,12 +2688,12 @@
       </c>
       <c r="G54" s="1" t="inlineStr">
         <is>
-          <t>HM2704</t>
+          <t>HM2703</t>
         </is>
       </c>
       <c r="H54" s="1" t="inlineStr">
         <is>
-          <t>MAN012</t>
+          <t>MAN010</t>
         </is>
       </c>
     </row>
@@ -2730,12 +2730,12 @@
       </c>
       <c r="G55" s="1" t="inlineStr">
         <is>
-          <t>HM2705</t>
+          <t>HM2704</t>
         </is>
       </c>
       <c r="H55" s="1" t="inlineStr">
         <is>
-          <t>MAN013</t>
+          <t>MAN011</t>
         </is>
       </c>
     </row>
@@ -2772,3636 +2772,3656 @@
       </c>
       <c r="G56" s="1" t="inlineStr">
         <is>
-          <t>HM2706</t>
+          <t>HM2705</t>
         </is>
       </c>
       <c r="H56" s="1" t="inlineStr">
         <is>
-          <t>MAN014</t>
+          <t>MAN012</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>MAN015</t>
+          <t>MAN013</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
-          <t>MM-544M</t>
+          <t>MM-536M</t>
         </is>
       </c>
       <c r="C58" s="1" t="inlineStr">
         <is>
-          <t>MM-858M</t>
+          <t>MM-844M</t>
         </is>
       </c>
       <c r="D58" s="1" t="inlineStr">
         <is>
-          <t>MM-9941M</t>
+          <t>MM-9933M</t>
         </is>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>NR40</t>
+          <t>NR37</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>P2505</t>
+          <t>P2501</t>
         </is>
       </c>
       <c r="G58" s="1" t="inlineStr">
         <is>
-          <t>RL302</t>
+          <t>R766</t>
         </is>
       </c>
       <c r="H58" s="1" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TE2813</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>MAN016</t>
+          <t>MAN014</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
-          <t>MM-546M</t>
+          <t>MM-542M</t>
         </is>
       </c>
       <c r="C59" s="1" t="inlineStr">
         <is>
-          <t>MM-860M</t>
+          <t>MM-852M</t>
         </is>
       </c>
       <c r="D59" s="1" t="inlineStr">
         <is>
-          <t>MM-9943M</t>
+          <t>MM-9938M</t>
         </is>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>NR43</t>
+          <t>NR38</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>P2506</t>
+          <t>P2502</t>
         </is>
       </c>
       <c r="G59" s="1" t="inlineStr">
         <is>
-          <t>RL304</t>
+          <t>RB2353</t>
         </is>
       </c>
       <c r="H59" s="1" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TE2814</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>MAN017</t>
+          <t>MAN015</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
-          <t>MM-551M</t>
+          <t>MM-544M</t>
         </is>
       </c>
       <c r="C60" s="1" t="inlineStr">
         <is>
-          <t>MM-862M</t>
+          <t>MM-858M</t>
         </is>
       </c>
       <c r="D60" s="1" t="inlineStr">
         <is>
-          <t>MM-9945M</t>
+          <t>MM-9941M</t>
         </is>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>NR44</t>
+          <t>NR39</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>P2507</t>
+          <t>P2503</t>
         </is>
       </c>
       <c r="G60" s="1" t="inlineStr">
         <is>
-          <t>RL307</t>
+          <t>RCTST4</t>
         </is>
       </c>
       <c r="H60" s="1" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TJ096</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>MM-4M</t>
+          <t>MAN016</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
-          <t>MM-588M</t>
+          <t>MM-546M</t>
         </is>
       </c>
       <c r="C61" s="1" t="inlineStr">
         <is>
-          <t>MM-868M</t>
+          <t>MM-860M</t>
         </is>
       </c>
       <c r="D61" s="1" t="inlineStr">
         <is>
-          <t>MM-9946M</t>
+          <t>MM-9943M</t>
         </is>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>NR45</t>
+          <t>NR40</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>P2508</t>
+          <t>P2505</t>
         </is>
       </c>
       <c r="G61" s="1" t="inlineStr">
         <is>
-          <t>RL309</t>
+          <t>RL301</t>
         </is>
       </c>
       <c r="H61" s="1" t="inlineStr">
         <is>
-          <t>TT07</t>
+          <t>TJ107</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>MM-9M</t>
+          <t>MAN017</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
-          <t>MM-602M</t>
+          <t>MM-551M</t>
         </is>
       </c>
       <c r="C62" s="1" t="inlineStr">
         <is>
-          <t>MM-872M</t>
+          <t>MM-862M</t>
         </is>
       </c>
       <c r="D62" s="1" t="inlineStr">
         <is>
-          <t>MM-9950M</t>
+          <t>MM-9945M</t>
         </is>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>NR51</t>
+          <t>NR43</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>P2509</t>
+          <t>P2506</t>
         </is>
       </c>
       <c r="G62" s="1" t="inlineStr">
         <is>
-          <t>RL310</t>
+          <t>RL302</t>
         </is>
       </c>
       <c r="H62" s="1" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TT03</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>MM-16M</t>
+          <t>MM-4M</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
-          <t>MM-624M</t>
+          <t>MM-588M</t>
         </is>
       </c>
       <c r="C63" s="1" t="inlineStr">
         <is>
-          <t>MM-874M</t>
+          <t>MM-868M</t>
         </is>
       </c>
       <c r="D63" s="1" t="inlineStr">
         <is>
-          <t>MM-9951M</t>
+          <t>MM-9946M</t>
         </is>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>NR52</t>
+          <t>NR44</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>P2510</t>
+          <t>P2507</t>
         </is>
       </c>
       <c r="G63" s="1" t="inlineStr">
         <is>
-          <t>S312</t>
+          <t>RL304</t>
         </is>
       </c>
       <c r="H63" s="1" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TT04</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>MM-18M</t>
+          <t>MM-9M</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
-          <t>MM-636M</t>
+          <t>MM-602M</t>
         </is>
       </c>
       <c r="C64" s="1" t="inlineStr">
         <is>
-          <t>MM-876M</t>
+          <t>MM-872M</t>
         </is>
       </c>
       <c r="D64" s="1" t="inlineStr">
         <is>
-          <t>MM-9952M</t>
+          <t>MM-9950M</t>
         </is>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>NR53</t>
+          <t>NR45</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>P2511</t>
+          <t>P2508</t>
         </is>
       </c>
       <c r="G64" s="1" t="inlineStr">
         <is>
-          <t>S317</t>
+          <t>RL307</t>
         </is>
       </c>
       <c r="H64" s="1" t="inlineStr">
         <is>
-          <t>TT106</t>
+          <t>TT05</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>MM-20M</t>
+          <t>MM-16M</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
-          <t>MM-640M</t>
+          <t>MM-624M</t>
         </is>
       </c>
       <c r="C65" s="1" t="inlineStr">
         <is>
-          <t>MM-882M</t>
+          <t>MM-874M</t>
         </is>
       </c>
       <c r="D65" s="1" t="inlineStr">
         <is>
-          <t>MM-9953M</t>
+          <t>MM-9951M</t>
         </is>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>NR51</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>P2513</t>
+          <t>P2509</t>
         </is>
       </c>
       <c r="G65" s="1" t="inlineStr">
         <is>
-          <t>S3301</t>
+          <t>RL309</t>
         </is>
       </c>
       <c r="H65" s="1" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TT07</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>MM-22M</t>
+          <t>MM-18M</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
-          <t>MM-654M</t>
+          <t>MM-636M</t>
         </is>
       </c>
       <c r="C66" s="1" t="inlineStr">
         <is>
-          <t>MM-894M</t>
+          <t>MM-876M</t>
         </is>
       </c>
       <c r="D66" s="1" t="inlineStr">
         <is>
-          <t>MM-9954M</t>
+          <t>MM-9952M</t>
         </is>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>NR57</t>
+          <t>NR52</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>P2514</t>
+          <t>P2510</t>
         </is>
       </c>
       <c r="G66" s="1" t="inlineStr">
         <is>
-          <t>S3302</t>
+          <t>RL310</t>
         </is>
       </c>
       <c r="H66" s="1" t="inlineStr">
         <is>
-          <t>TT108</t>
+          <t>TT08</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>MM-28M</t>
+          <t>MM-20M</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
-          <t>MM-656M</t>
+          <t>MM-640M</t>
         </is>
       </c>
       <c r="C67" s="1" t="inlineStr">
         <is>
-          <t>MM-896M</t>
+          <t>MM-882M</t>
         </is>
       </c>
       <c r="D67" s="1" t="inlineStr">
         <is>
-          <t>MM-9955M</t>
+          <t>MM-9953M</t>
         </is>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>NR59</t>
+          <t>NR53</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>P2515</t>
+          <t>P2511</t>
         </is>
       </c>
       <c r="G67" s="1" t="inlineStr">
         <is>
-          <t>S3304</t>
+          <t>S312</t>
         </is>
       </c>
       <c r="H67" s="1" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TT103</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>MM-34M</t>
+          <t>MM-22M</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
-          <t>MM-660M</t>
+          <t>MM-654M</t>
         </is>
       </c>
       <c r="C68" s="1" t="inlineStr">
         <is>
-          <t>MM-902M</t>
+          <t>MM-894M</t>
         </is>
       </c>
       <c r="D68" s="1" t="inlineStr">
         <is>
-          <t>MM-9957M</t>
+          <t>MM-9954M</t>
         </is>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>NR61</t>
+          <t>NR54</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>P2516</t>
+          <t>P2513</t>
         </is>
       </c>
       <c r="G68" s="1" t="inlineStr">
         <is>
-          <t>S3306</t>
+          <t>S317</t>
         </is>
       </c>
       <c r="H68" s="1" t="inlineStr">
         <is>
-          <t>TT112</t>
+          <t>TT106</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>MM-42M</t>
+          <t>MM-28M</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
-          <t>MM-661M</t>
+          <t>MM-656M</t>
         </is>
       </c>
       <c r="C69" s="1" t="inlineStr">
         <is>
-          <t>MM-904M</t>
+          <t>MM-896M</t>
         </is>
       </c>
       <c r="D69" s="1" t="inlineStr">
         <is>
-          <t>MM-9959M</t>
+          <t>MM-9955M</t>
         </is>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>NR62</t>
+          <t>NR57</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>PB1</t>
+          <t>P2514</t>
         </is>
       </c>
       <c r="G69" s="1" t="inlineStr">
         <is>
-          <t>S3307</t>
+          <t>S3301</t>
         </is>
       </c>
       <c r="H69" s="1" t="inlineStr">
         <is>
-          <t>TT114</t>
+          <t>TT107</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>MM-46M</t>
+          <t>MM-34M</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
         <is>
-          <t>MM-664M</t>
+          <t>MM-660M</t>
         </is>
       </c>
       <c r="C70" s="1" t="inlineStr">
         <is>
-          <t>MM-906M</t>
+          <t>MM-902M</t>
         </is>
       </c>
       <c r="D70" s="1" t="inlineStr">
         <is>
-          <t>MM-9960M</t>
+          <t>MM-9957M</t>
         </is>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR59</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>P2515</t>
         </is>
       </c>
       <c r="G70" s="1" t="inlineStr">
         <is>
-          <t>S3309</t>
+          <t>S3302</t>
         </is>
       </c>
       <c r="H70" s="1" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT108</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>MM-50M</t>
+          <t>MM-42M</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
-          <t>MM-666M</t>
+          <t>MM-661M</t>
         </is>
       </c>
       <c r="C71" s="1" t="inlineStr">
         <is>
-          <t>MM-908M</t>
+          <t>MM-904M</t>
         </is>
       </c>
       <c r="D71" s="1" t="inlineStr">
         <is>
-          <t>MM-9961M</t>
+          <t>MM-9959M</t>
         </is>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR61</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>P2516</t>
         </is>
       </c>
       <c r="G71" s="1" t="inlineStr">
         <is>
-          <t>S3310</t>
+          <t>S3304</t>
         </is>
       </c>
       <c r="H71" s="1" t="inlineStr">
         <is>
-          <t>TT116</t>
+          <t>TT110</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>MM-54M</t>
+          <t>MM-46M</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
         <is>
-          <t>MM-668M</t>
+          <t>MM-664M</t>
         </is>
       </c>
       <c r="C72" s="1" t="inlineStr">
         <is>
-          <t>MM-910M</t>
+          <t>MM-906M</t>
         </is>
       </c>
       <c r="D72" s="1" t="inlineStr">
         <is>
-          <t>MM-9962M</t>
+          <t>MM-9960M</t>
         </is>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>NR66</t>
+          <t>NR62</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>PHC002</t>
+          <t>PB1</t>
         </is>
       </c>
       <c r="G72" s="1" t="inlineStr">
         <is>
-          <t>S7001</t>
+          <t>S3306</t>
         </is>
       </c>
       <c r="H72" s="1" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT112</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>MM-58M</t>
+          <t>MM-50M</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
         <is>
-          <t>MM-673M</t>
+          <t>MM-666M</t>
         </is>
       </c>
       <c r="C73" s="1" t="inlineStr">
         <is>
-          <t>MM-912M</t>
+          <t>MM-908M</t>
         </is>
       </c>
       <c r="D73" s="1" t="inlineStr">
         <is>
-          <t>MM-9963M</t>
+          <t>MM-9961M</t>
         </is>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>NR67</t>
+          <t>NR64</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>Q4001</t>
+          <t>PB4</t>
         </is>
       </c>
       <c r="G73" s="1" t="inlineStr">
         <is>
-          <t>S7002</t>
+          <t>S3307</t>
         </is>
       </c>
       <c r="H73" s="1" t="inlineStr">
         <is>
-          <t>TT122</t>
+          <t>TT114</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>MM-64M</t>
+          <t>MM-54M</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
-          <t>MM-674M</t>
+          <t>MM-668M</t>
         </is>
       </c>
       <c r="C74" s="1" t="inlineStr">
         <is>
-          <t>MM-914M</t>
+          <t>MM-910M</t>
         </is>
       </c>
       <c r="D74" s="1" t="inlineStr">
         <is>
-          <t>MM-9964M</t>
+          <t>MM-9962M</t>
         </is>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR65</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>Q4003</t>
+          <t>PHC001</t>
         </is>
       </c>
       <c r="G74" s="1" t="inlineStr">
         <is>
-          <t>S7003</t>
+          <t>S3309</t>
         </is>
       </c>
       <c r="H74" s="1" t="inlineStr">
         <is>
-          <t>TT127</t>
+          <t>TT115</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>MM-74M</t>
+          <t>MM-58M</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
         <is>
-          <t>MM-680M</t>
+          <t>MM-673M</t>
         </is>
       </c>
       <c r="C75" s="1" t="inlineStr">
         <is>
-          <t>MM-920M</t>
+          <t>MM-912M</t>
         </is>
       </c>
       <c r="D75" s="1" t="inlineStr">
         <is>
-          <t>MM-9965M</t>
+          <t>MM-9963M</t>
         </is>
       </c>
       <c r="E75" s="1" t="inlineStr">
         <is>
-          <t>NR69</t>
+          <t>NR66</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>PHC002</t>
         </is>
       </c>
       <c r="G75" s="1" t="inlineStr">
         <is>
-          <t>S7005</t>
+          <t>S3310</t>
         </is>
       </c>
       <c r="H75" s="1" t="inlineStr">
         <is>
-          <t>TT128</t>
+          <t>TT116</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>MM-76M</t>
+          <t>MM-64M</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
         <is>
-          <t>MM-708M</t>
+          <t>MM-674M</t>
         </is>
       </c>
       <c r="C76" s="1" t="inlineStr">
         <is>
-          <t>MM-922M</t>
+          <t>MM-914M</t>
         </is>
       </c>
       <c r="D76" s="1" t="inlineStr">
         <is>
-          <t>MM-9966M</t>
+          <t>MM-9964M</t>
         </is>
       </c>
       <c r="E76" s="1" t="inlineStr">
         <is>
-          <t>NR71</t>
+          <t>NR67</t>
         </is>
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>Q4005</t>
+          <t>Q4001</t>
         </is>
       </c>
       <c r="G76" s="1" t="inlineStr">
         <is>
-          <t>S7006</t>
+          <t>S7001</t>
         </is>
       </c>
       <c r="H76" s="1" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT117</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>MM-82M</t>
+          <t>MM-74M</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
         <is>
-          <t>MM-722M</t>
+          <t>MM-680M</t>
         </is>
       </c>
       <c r="C77" s="1" t="inlineStr">
         <is>
-          <t>MM-924M</t>
+          <t>MM-920M</t>
         </is>
       </c>
       <c r="D77" s="1" t="inlineStr">
         <is>
-          <t>MM-9967M</t>
+          <t>MM-9965M</t>
         </is>
       </c>
       <c r="E77" s="1" t="inlineStr">
         <is>
-          <t>NR72</t>
+          <t>NR68</t>
         </is>
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
-          <t>Q4006</t>
+          <t>Q4003</t>
         </is>
       </c>
       <c r="G77" s="1" t="inlineStr">
         <is>
-          <t>S7007</t>
+          <t>S7002</t>
         </is>
       </c>
       <c r="H77" s="1" t="inlineStr">
         <is>
-          <t>TT131</t>
+          <t>TT122</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>MM-86M</t>
+          <t>MM-76M</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
         <is>
-          <t>MM-726M</t>
+          <t>MM-708M</t>
         </is>
       </c>
       <c r="C78" s="1" t="inlineStr">
         <is>
-          <t>MM-926M</t>
+          <t>MM-922M</t>
         </is>
       </c>
       <c r="D78" s="1" t="inlineStr">
         <is>
-          <t>MM-9969M</t>
+          <t>MM-9966M</t>
         </is>
       </c>
       <c r="E78" s="1" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR69</t>
         </is>
       </c>
       <c r="F78" s="1" t="inlineStr">
         <is>
-          <t>Q4007</t>
+          <t>Q4004</t>
         </is>
       </c>
       <c r="G78" s="1" t="inlineStr">
         <is>
-          <t>S7012</t>
+          <t>S7003</t>
         </is>
       </c>
       <c r="H78" s="1" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT127</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>MM-88M</t>
+          <t>MM-82M</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
         <is>
-          <t>MM-728M</t>
+          <t>MM-722M</t>
         </is>
       </c>
       <c r="C79" s="1" t="inlineStr">
         <is>
-          <t>MM-934M</t>
+          <t>MM-924M</t>
         </is>
       </c>
       <c r="D79" s="1" t="inlineStr">
         <is>
-          <t>MMY032</t>
+          <t>MM-9967M</t>
         </is>
       </c>
       <c r="E79" s="1" t="inlineStr">
         <is>
-          <t>NR77</t>
+          <t>NR71</t>
         </is>
       </c>
       <c r="F79" s="1" t="inlineStr">
         <is>
-          <t>Q4009</t>
+          <t>Q4005</t>
         </is>
       </c>
       <c r="G79" s="1" t="inlineStr">
         <is>
-          <t>S7014</t>
+          <t>S7005</t>
         </is>
       </c>
       <c r="H79" s="1" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT128</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>MM-92M</t>
+          <t>MM-86M</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
         <is>
-          <t>MM-734M</t>
+          <t>MM-726M</t>
         </is>
       </c>
       <c r="C80" s="1" t="inlineStr">
         <is>
-          <t>MM-936M</t>
+          <t>MM-926M</t>
         </is>
       </c>
       <c r="D80" s="1" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MM-9969M</t>
         </is>
       </c>
       <c r="E80" s="1" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR72</t>
         </is>
       </c>
       <c r="F80" s="1" t="inlineStr">
         <is>
-          <t>Q4011</t>
+          <t>Q4006</t>
         </is>
       </c>
       <c r="G80" s="1" t="inlineStr">
         <is>
-          <t>S7020</t>
+          <t>S7006</t>
         </is>
       </c>
       <c r="H80" s="1" t="inlineStr">
         <is>
-          <t>VL352</t>
+          <t>TT130</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>MM-99M</t>
+          <t>MM-88M</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
         <is>
-          <t>MM-736M</t>
+          <t>MM-728M</t>
         </is>
       </c>
       <c r="C81" s="1" t="inlineStr">
         <is>
-          <t>MM-948M</t>
+          <t>MM-934M</t>
         </is>
       </c>
       <c r="D81" s="1" t="inlineStr">
         <is>
-          <t>MRL004</t>
+          <t>MMY032</t>
         </is>
       </c>
       <c r="E81" s="1" t="inlineStr">
         <is>
-          <t>NR81</t>
+          <t>NR75</t>
         </is>
       </c>
       <c r="F81" s="1" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>Q4007</t>
         </is>
       </c>
       <c r="G81" s="1" t="inlineStr">
         <is>
-          <t>S7022</t>
+          <t>S7007</t>
         </is>
       </c>
       <c r="H81" s="1" t="inlineStr">
         <is>
-          <t>VL353</t>
+          <t>TT131</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>MM-114M</t>
+          <t>MM-92M</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
         <is>
-          <t>MM-740M</t>
+          <t>MM-734M</t>
         </is>
       </c>
       <c r="C82" s="1" t="inlineStr">
         <is>
-          <t>MM-956M</t>
+          <t>MM-936M</t>
         </is>
       </c>
       <c r="D82" s="1" t="inlineStr">
         <is>
-          <t>MRL006</t>
+          <t>MRL001</t>
         </is>
       </c>
       <c r="E82" s="1" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR77</t>
         </is>
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>Q4009</t>
         </is>
       </c>
       <c r="G82" s="1" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>S7012</t>
         </is>
       </c>
       <c r="H82" s="1" t="inlineStr">
         <is>
-          <t>VL357</t>
+          <t>TT202</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>MM-120M</t>
+          <t>MM-99M</t>
         </is>
       </c>
       <c r="B83" s="1" t="inlineStr">
         <is>
-          <t>MM-744M</t>
+          <t>MM-736M</t>
         </is>
       </c>
       <c r="C83" s="1" t="inlineStr">
         <is>
-          <t>MM-962M</t>
+          <t>MM-948M</t>
         </is>
       </c>
       <c r="D83" s="1" t="inlineStr">
         <is>
-          <t>N452</t>
+          <t>MRL004</t>
         </is>
       </c>
       <c r="E83" s="1" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR78</t>
         </is>
       </c>
       <c r="F83" s="1" t="inlineStr">
         <is>
-          <t>Q4014</t>
+          <t>Q4011</t>
         </is>
       </c>
       <c r="G83" s="1" t="inlineStr">
         <is>
-          <t>SCT002</t>
+          <t>S7014</t>
         </is>
       </c>
       <c r="H83" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8004</t>
+          <t>TT206</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>MM-134M</t>
+          <t>MM-114M</t>
         </is>
       </c>
       <c r="B84" s="1" t="inlineStr">
         <is>
-          <t>MM-752M</t>
+          <t>MM-740M</t>
         </is>
       </c>
       <c r="C84" s="1" t="inlineStr">
         <is>
-          <t>MM-964M</t>
+          <t>MM-956M</t>
         </is>
       </c>
       <c r="D84" s="1" t="inlineStr">
         <is>
-          <t>N457</t>
+          <t>MRL006</t>
         </is>
       </c>
       <c r="E84" s="1" t="inlineStr">
         <is>
-          <t>NR84</t>
+          <t>NR81</t>
         </is>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>Q4015</t>
+          <t>Q4012</t>
         </is>
       </c>
       <c r="G84" s="1" t="inlineStr">
         <is>
-          <t>SCT006</t>
+          <t>S7020</t>
         </is>
       </c>
       <c r="H84" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8007</t>
+          <t>VL352</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>MM-146M</t>
+          <t>MM-120M</t>
         </is>
       </c>
       <c r="B85" s="1" t="inlineStr">
         <is>
-          <t>MM-756M</t>
+          <t>MM-744M</t>
         </is>
       </c>
       <c r="C85" s="1" t="inlineStr">
         <is>
-          <t>MM-966M</t>
+          <t>MM-962M</t>
         </is>
       </c>
       <c r="D85" s="1" t="inlineStr">
         <is>
-          <t>N458</t>
+          <t>N452</t>
         </is>
       </c>
       <c r="E85" s="1" t="inlineStr">
         <is>
-          <t>NR85</t>
+          <t>NR82</t>
         </is>
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>Q4013</t>
         </is>
       </c>
       <c r="G85" s="1" t="inlineStr">
         <is>
-          <t>SCT007</t>
+          <t>S7022</t>
         </is>
       </c>
       <c r="H85" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8011</t>
+          <t>VL353</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>MM-168M</t>
+          <t>MM-134M</t>
         </is>
       </c>
       <c r="B86" s="1" t="inlineStr">
         <is>
-          <t>MM-760M</t>
+          <t>MM-752M</t>
         </is>
       </c>
       <c r="C86" s="1" t="inlineStr">
         <is>
-          <t>MM-970M</t>
+          <t>MM-964M</t>
         </is>
       </c>
       <c r="D86" s="1" t="inlineStr">
         <is>
-          <t>N465</t>
+          <t>N457</t>
         </is>
       </c>
       <c r="E86" s="1" t="inlineStr">
         <is>
-          <t>NR86</t>
+          <t>NR83</t>
         </is>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>Q4017</t>
+          <t>Q4014</t>
         </is>
       </c>
       <c r="G86" s="1" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>SCT001</t>
         </is>
       </c>
       <c r="H86" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8013</t>
+          <t>VL357</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>MM-182M</t>
+          <t>MM-146M</t>
         </is>
       </c>
       <c r="B87" s="1" t="inlineStr">
         <is>
-          <t>MM-764M</t>
+          <t>MM-756M</t>
         </is>
       </c>
       <c r="C87" s="1" t="inlineStr">
         <is>
-          <t>MM-972M</t>
+          <t>MM-966M</t>
         </is>
       </c>
       <c r="D87" s="1" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>N458</t>
         </is>
       </c>
       <c r="E87" s="1" t="inlineStr">
         <is>
-          <t>NR87</t>
+          <t>NR84</t>
         </is>
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>Q4019</t>
+          <t>Q4015</t>
         </is>
       </c>
       <c r="G87" s="1" t="inlineStr">
         <is>
-          <t>SCT011</t>
+          <t>SCT002</t>
         </is>
       </c>
       <c r="H87" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8019</t>
+          <t>VLINE-8004</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>MM-184M</t>
+          <t>MM-168M</t>
         </is>
       </c>
       <c r="B88" s="1" t="inlineStr">
         <is>
-          <t>MM-774M</t>
+          <t>MM-760M</t>
         </is>
       </c>
       <c r="C88" s="1" t="inlineStr">
         <is>
-          <t>MM-974M</t>
+          <t>MM-970M</t>
         </is>
       </c>
       <c r="D88" s="1" t="inlineStr">
         <is>
-          <t>N467</t>
+          <t>N465</t>
         </is>
       </c>
       <c r="E88" s="1" t="inlineStr">
         <is>
-          <t>NR88</t>
+          <t>NR85</t>
         </is>
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>Q4016</t>
         </is>
       </c>
       <c r="G88" s="1" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>SCT006</t>
         </is>
       </c>
       <c r="H88" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8020</t>
+          <t>VLINE-8007</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>MM-186M</t>
+          <t>MM-182M</t>
         </is>
       </c>
       <c r="B89" s="1" t="inlineStr">
         <is>
-          <t>MM-776M</t>
+          <t>MM-764M</t>
         </is>
       </c>
       <c r="C89" s="1" t="inlineStr">
         <is>
-          <t>MM-980M</t>
+          <t>MM-972M</t>
         </is>
       </c>
       <c r="D89" s="1" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>N466</t>
         </is>
       </c>
       <c r="E89" s="1" t="inlineStr">
         <is>
-          <t>NR90</t>
+          <t>NR86</t>
         </is>
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>Q4017</t>
         </is>
       </c>
       <c r="G89" s="1" t="inlineStr">
         <is>
-          <t>SCT014</t>
+          <t>SCT007</t>
         </is>
       </c>
       <c r="H89" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8023</t>
+          <t>VLINE-8011</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>MM-190M</t>
+          <t>MM-184M</t>
         </is>
       </c>
       <c r="B90" s="1" t="inlineStr">
         <is>
-          <t>MM-778M</t>
+          <t>MM-774M</t>
         </is>
       </c>
       <c r="C90" s="1" t="inlineStr">
         <is>
-          <t>MM-982M</t>
+          <t>MM-974M</t>
         </is>
       </c>
       <c r="D90" s="1" t="inlineStr">
         <is>
-          <t>N473</t>
+          <t>N467</t>
         </is>
       </c>
       <c r="E90" s="1" t="inlineStr">
         <is>
-          <t>NR92</t>
+          <t>NR87</t>
         </is>
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>QBX005</t>
+          <t>Q4019</t>
         </is>
       </c>
       <c r="G90" s="1" t="inlineStr">
         <is>
-          <t>SCT015</t>
+          <t>SCT009</t>
         </is>
       </c>
       <c r="H90" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8025</t>
+          <t>VLINE-8013</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>MM-206M</t>
+          <t>MM-186M</t>
         </is>
       </c>
       <c r="B91" s="1" t="inlineStr">
         <is>
-          <t>MM-780M</t>
+          <t>MM-776M</t>
         </is>
       </c>
       <c r="C91" s="1" t="inlineStr">
         <is>
-          <t>MM-984M</t>
+          <t>MM-980M</t>
         </is>
       </c>
       <c r="D91" s="1" t="inlineStr">
         <is>
-          <t>NR1</t>
+          <t>N469</t>
         </is>
       </c>
       <c r="E91" s="1" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR88</t>
         </is>
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>QBX006</t>
+          <t>QBX003</t>
         </is>
       </c>
       <c r="G91" s="1" t="inlineStr">
         <is>
-          <t>SO2</t>
+          <t>SCT011</t>
         </is>
       </c>
       <c r="H91" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8026</t>
+          <t>VLINE-8019</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>MM-218M</t>
+          <t>MM-190M</t>
         </is>
       </c>
       <c r="B92" s="1" t="inlineStr">
         <is>
-          <t>MM-784M</t>
+          <t>MM-778M</t>
         </is>
       </c>
       <c r="C92" s="1" t="inlineStr">
         <is>
-          <t>MM-986M</t>
+          <t>MM-982M</t>
         </is>
       </c>
       <c r="D92" s="1" t="inlineStr">
         <is>
-          <t>NR2</t>
+          <t>N473</t>
         </is>
       </c>
       <c r="E92" s="1" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR90</t>
         </is>
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>QBX004</t>
         </is>
       </c>
       <c r="G92" s="1" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>SCT013</t>
         </is>
       </c>
       <c r="H92" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8027</t>
+          <t>VLINE-8020</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>MM-222M</t>
+          <t>MM-206M</t>
         </is>
       </c>
       <c r="B93" s="1" t="inlineStr">
         <is>
-          <t>MM-790M</t>
+          <t>MM-780M</t>
         </is>
       </c>
       <c r="C93" s="1" t="inlineStr">
         <is>
-          <t>MM-9903M</t>
+          <t>MM-984M</t>
         </is>
       </c>
       <c r="D93" s="1" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>NR1</t>
         </is>
       </c>
       <c r="E93" s="1" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR92</t>
         </is>
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>QBX005</t>
         </is>
       </c>
       <c r="G93" s="1" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>SCT014</t>
         </is>
       </c>
       <c r="H93" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8028</t>
+          <t>VLINE-8023</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>MM-224M</t>
+          <t>MM-218M</t>
         </is>
       </c>
       <c r="B94" s="1" t="inlineStr">
         <is>
-          <t>MM-792M</t>
+          <t>MM-784M</t>
         </is>
       </c>
       <c r="C94" s="1" t="inlineStr">
         <is>
-          <t>MM-9904M</t>
+          <t>MM-986M</t>
         </is>
       </c>
       <c r="D94" s="1" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>NR2</t>
         </is>
       </c>
       <c r="E94" s="1" t="inlineStr">
         <is>
-          <t>NR96</t>
+          <t>NR93</t>
         </is>
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>QBX006</t>
         </is>
       </c>
       <c r="G94" s="1" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>SCT015</t>
         </is>
       </c>
       <c r="H94" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8030</t>
+          <t>VLINE-8025</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>MM-242M</t>
+          <t>MM-222M</t>
         </is>
       </c>
       <c r="B95" s="1" t="inlineStr">
         <is>
-          <t>MM-798M</t>
+          <t>MM-790M</t>
         </is>
       </c>
       <c r="C95" s="1" t="inlineStr">
         <is>
-          <t>MM-9906M</t>
+          <t>MM-9903M</t>
         </is>
       </c>
       <c r="D95" s="1" t="inlineStr">
         <is>
-          <t>NR7</t>
+          <t>NR4</t>
         </is>
       </c>
       <c r="E95" s="1" t="inlineStr">
         <is>
-          <t>NR98</t>
+          <t>NR94</t>
         </is>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>QE004</t>
+          <t>QE001</t>
         </is>
       </c>
       <c r="G95" s="1" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>SO2</t>
         </is>
       </c>
       <c r="H95" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8032</t>
+          <t>VLINE-8026</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>MM-256M</t>
+          <t>MM-224M</t>
         </is>
       </c>
       <c r="B96" s="1" t="inlineStr">
         <is>
-          <t>MM-800M</t>
+          <t>MM-792M</t>
         </is>
       </c>
       <c r="C96" s="1" t="inlineStr">
         <is>
-          <t>MM-9907M</t>
+          <t>MM-9904M</t>
         </is>
       </c>
       <c r="D96" s="1" t="inlineStr">
         <is>
-          <t>NR8</t>
+          <t>NR5</t>
         </is>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>NR99</t>
+          <t>NR95</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>QE006</t>
+          <t>QE002</t>
         </is>
       </c>
       <c r="G96" s="1" t="inlineStr">
         <is>
-          <t>T363</t>
+          <t>SSR101</t>
         </is>
       </c>
       <c r="H96" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8036</t>
+          <t>VLINE-8027</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>MM-264M</t>
+          <t>MM-242M</t>
         </is>
       </c>
       <c r="B97" s="1" t="inlineStr">
         <is>
-          <t>MM-802M</t>
+          <t>MM-798M</t>
         </is>
       </c>
       <c r="C97" s="1" t="inlineStr">
         <is>
-          <t>MM-9909M</t>
+          <t>MM-9906M</t>
         </is>
       </c>
       <c r="D97" s="1" t="inlineStr">
         <is>
-          <t>NR9</t>
+          <t>NR7</t>
         </is>
       </c>
       <c r="E97" s="1" t="inlineStr">
         <is>
-          <t>NR101</t>
+          <t>NR96</t>
         </is>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>QL001</t>
+          <t>QE003</t>
         </is>
       </c>
       <c r="G97" s="1" t="inlineStr">
         <is>
-          <t>T386</t>
+          <t>SSR102</t>
         </is>
       </c>
       <c r="H97" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8051</t>
+          <t>VLINE-8028</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>MM-268M</t>
+          <t>MM-256M</t>
         </is>
       </c>
       <c r="B98" s="1" t="inlineStr">
         <is>
-          <t>MM-804M</t>
+          <t>MM-800M</t>
         </is>
       </c>
       <c r="C98" s="1" t="inlineStr">
         <is>
-          <t>MM-9912M</t>
+          <t>MM-9907M</t>
         </is>
       </c>
       <c r="D98" s="1" t="inlineStr">
         <is>
-          <t>NR12</t>
+          <t>NR8</t>
         </is>
       </c>
       <c r="E98" s="1" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR98</t>
         </is>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>QL002</t>
+          <t>QE004</t>
         </is>
       </c>
       <c r="G98" s="1" t="inlineStr">
         <is>
-          <t>TDX101</t>
+          <t>SSR103</t>
         </is>
       </c>
       <c r="H98" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8052</t>
+          <t>VLINE-8030</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>MM-282M</t>
+          <t>MM-264M</t>
         </is>
       </c>
       <c r="B99" s="1" t="inlineStr">
         <is>
-          <t>MM-808M</t>
+          <t>MM-802M</t>
         </is>
       </c>
       <c r="C99" s="1" t="inlineStr">
         <is>
-          <t>MM-9913M</t>
+          <t>MM-9909M</t>
         </is>
       </c>
       <c r="D99" s="1" t="inlineStr">
         <is>
-          <t>NR15</t>
+          <t>NR9</t>
         </is>
       </c>
       <c r="E99" s="1" t="inlineStr">
         <is>
-          <t>NR103</t>
+          <t>NR99</t>
         </is>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>QE006</t>
         </is>
       </c>
       <c r="G99" s="1" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>SSR104</t>
         </is>
       </c>
       <c r="H99" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8053</t>
+          <t>VLINE-8032</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>MM-352M</t>
+          <t>MM-268M</t>
         </is>
       </c>
       <c r="B100" s="1" t="inlineStr">
         <is>
-          <t>MM-810M</t>
+          <t>MM-804M</t>
         </is>
       </c>
       <c r="C100" s="1" t="inlineStr">
         <is>
-          <t>MM-9914M</t>
+          <t>MM-9912M</t>
         </is>
       </c>
       <c r="D100" s="1" t="inlineStr">
         <is>
-          <t>NR16</t>
+          <t>NR12</t>
         </is>
       </c>
       <c r="E100" s="1" t="inlineStr">
         <is>
-          <t>NR105</t>
+          <t>NR101</t>
         </is>
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>QL001</t>
         </is>
       </c>
       <c r="G100" s="1" t="inlineStr">
         <is>
-          <t>TE2802</t>
+          <t>T363</t>
         </is>
       </c>
       <c r="H100" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8055</t>
+          <t>VLINE-8036</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>MM-372M</t>
+          <t>MM-282M</t>
         </is>
       </c>
       <c r="B101" s="1" t="inlineStr">
         <is>
-          <t>MM-814M</t>
+          <t>MM-808M</t>
         </is>
       </c>
       <c r="C101" s="1" t="inlineStr">
         <is>
-          <t>MM-9915M</t>
+          <t>MM-9913M</t>
         </is>
       </c>
       <c r="D101" s="1" t="inlineStr">
         <is>
-          <t>NR18</t>
+          <t>NR13</t>
         </is>
       </c>
       <c r="E101" s="1" t="inlineStr">
         <is>
-          <t>NR108</t>
+          <t>NR102</t>
         </is>
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>QL008</t>
+          <t>QL002</t>
         </is>
       </c>
       <c r="G101" s="1" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>T386</t>
         </is>
       </c>
       <c r="H101" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8056</t>
+          <t>VLINE-8051</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>MM-378M</t>
+          <t>MM-352M</t>
         </is>
       </c>
       <c r="B102" s="1" t="inlineStr">
         <is>
-          <t>MM-816M</t>
+          <t>MM-810M</t>
         </is>
       </c>
       <c r="C102" s="1" t="inlineStr">
         <is>
-          <t>MM-9917M</t>
+          <t>MM-9914M</t>
         </is>
       </c>
       <c r="D102" s="1" t="inlineStr">
         <is>
-          <t>NR19</t>
+          <t>NR15</t>
         </is>
       </c>
       <c r="E102" s="1" t="inlineStr">
         <is>
-          <t>NR110</t>
+          <t>NR103</t>
         </is>
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>QL010</t>
+          <t>QL004</t>
         </is>
       </c>
       <c r="G102" s="1" t="inlineStr">
         <is>
-          <t>TE2804</t>
+          <t>TDX101</t>
         </is>
       </c>
       <c r="H102" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8057</t>
+          <t>VLINE-8052</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>MM-382M</t>
+          <t>MM-372M</t>
         </is>
       </c>
       <c r="B103" s="1" t="inlineStr">
         <is>
-          <t>MM-818M</t>
+          <t>MM-814M</t>
         </is>
       </c>
       <c r="C103" s="1" t="inlineStr">
         <is>
-          <t>MM-9918M</t>
+          <t>MM-9915M</t>
         </is>
       </c>
       <c r="D103" s="1" t="inlineStr">
         <is>
-          <t>NR21</t>
+          <t>NR16</t>
         </is>
       </c>
       <c r="E103" s="1" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR105</t>
         </is>
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>QL011</t>
+          <t>QL007</t>
         </is>
       </c>
       <c r="G103" s="1" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>TE2801</t>
         </is>
       </c>
       <c r="H103" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8058</t>
+          <t>VLINE-8053</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>MM-392M</t>
+          <t>MM-378M</t>
         </is>
       </c>
       <c r="B104" s="1" t="inlineStr">
         <is>
-          <t>MM-820M</t>
+          <t>MM-816M</t>
         </is>
       </c>
       <c r="C104" s="1" t="inlineStr">
         <is>
-          <t>MM-9919M</t>
+          <t>MM-9917M</t>
         </is>
       </c>
       <c r="D104" s="1" t="inlineStr">
         <is>
-          <t>NR25</t>
+          <t>NR18</t>
         </is>
       </c>
       <c r="E104" s="1" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR108</t>
         </is>
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>QL014</t>
+          <t>QL008</t>
         </is>
       </c>
       <c r="G104" s="1" t="inlineStr">
         <is>
-          <t>TE2806</t>
+          <t>TE2802</t>
         </is>
       </c>
       <c r="H104" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8059</t>
+          <t>VLINE-8055</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>MM-444M</t>
+          <t>MM-382M</t>
         </is>
       </c>
       <c r="B105" s="1" t="inlineStr">
         <is>
-          <t>MM-824M</t>
+          <t>MM-818M</t>
         </is>
       </c>
       <c r="C105" s="1" t="inlineStr">
         <is>
-          <t>MM-9920M</t>
+          <t>MM-9918M</t>
         </is>
       </c>
       <c r="D105" s="1" t="inlineStr">
         <is>
-          <t>NR27</t>
+          <t>NR19</t>
         </is>
       </c>
       <c r="E105" s="1" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR110</t>
         </is>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>QL017</t>
+          <t>QL010</t>
         </is>
       </c>
       <c r="G105" s="1" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>TE2803</t>
         </is>
       </c>
       <c r="H105" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8061</t>
+          <t>VLINE-8056</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>MM-464M</t>
+          <t>MM-392M</t>
         </is>
       </c>
       <c r="B106" s="1" t="inlineStr">
         <is>
-          <t>MM-826M</t>
+          <t>MM-820M</t>
         </is>
       </c>
       <c r="C106" s="1" t="inlineStr">
         <is>
-          <t>MM-9922M</t>
+          <t>MM-9919M</t>
         </is>
       </c>
       <c r="D106" s="1" t="inlineStr">
         <is>
-          <t>NR28</t>
+          <t>NR21</t>
         </is>
       </c>
       <c r="E106" s="1" t="inlineStr">
         <is>
-          <t>NR118</t>
+          <t>NR112</t>
         </is>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>QL018</t>
+          <t>QL011</t>
         </is>
       </c>
       <c r="G106" s="1" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>TE2804</t>
         </is>
       </c>
       <c r="H106" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8072</t>
+          <t>VLINE-8057</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>MM-486M</t>
+          <t>MM-444M</t>
         </is>
       </c>
       <c r="B107" s="1" t="inlineStr">
         <is>
-          <t>MM-828M</t>
+          <t>MM-824M</t>
         </is>
       </c>
       <c r="C107" s="1" t="inlineStr">
         <is>
-          <t>MM-9924M</t>
+          <t>MM-9920M</t>
         </is>
       </c>
       <c r="D107" s="1" t="inlineStr">
         <is>
-          <t>NR30</t>
+          <t>NR25</t>
         </is>
       </c>
       <c r="E107" s="1" t="inlineStr">
         <is>
-          <t>NR119</t>
+          <t>NR113</t>
         </is>
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QL014</t>
         </is>
       </c>
       <c r="G107" s="1" t="inlineStr">
         <is>
-          <t>TE2809</t>
+          <t>TE2805</t>
         </is>
       </c>
       <c r="H107" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8074</t>
+          <t>VLINE-8058</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>MM-496M</t>
+          <t>MM-464M</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
         <is>
-          <t>MM-830M</t>
+          <t>MM-826M</t>
         </is>
       </c>
       <c r="C108" s="1" t="inlineStr">
         <is>
-          <t>MM-9926M</t>
+          <t>MM-9922M</t>
         </is>
       </c>
       <c r="D108" s="1" t="inlineStr">
         <is>
-          <t>NR31</t>
+          <t>NR27</t>
         </is>
       </c>
       <c r="E108" s="1" t="inlineStr">
         <is>
-          <t>NR120</t>
+          <t>NR115</t>
         </is>
       </c>
       <c r="F108" s="1" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QL017</t>
         </is>
       </c>
       <c r="G108" s="1" t="inlineStr">
         <is>
-          <t>TE2810</t>
+          <t>TE2806</t>
         </is>
       </c>
       <c r="H108" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8075</t>
+          <t>VLINE-8059</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>MM-514M</t>
+          <t>MM-486M</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
         <is>
-          <t>MM-832M</t>
+          <t>MM-828M</t>
         </is>
       </c>
       <c r="C109" s="1" t="inlineStr">
         <is>
-          <t>MM-9928M</t>
+          <t>MM-9924M</t>
         </is>
       </c>
       <c r="D109" s="1" t="inlineStr">
         <is>
-          <t>NR34</t>
+          <t>NR28</t>
         </is>
       </c>
       <c r="E109" s="1" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>NR118</t>
         </is>
       </c>
       <c r="F109" s="1" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QL018</t>
         </is>
       </c>
       <c r="G109" s="1" t="inlineStr">
         <is>
-          <t>TE2812</t>
+          <t>TE2807</t>
         </is>
       </c>
       <c r="H109" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8076</t>
+          <t>VLINE-8061</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>MM-526M</t>
+          <t>MM-496M</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
         <is>
-          <t>MM-834M</t>
+          <t>MM-830M</t>
         </is>
       </c>
       <c r="C110" s="1" t="inlineStr">
         <is>
-          <t>MM-9929M</t>
+          <t>MM-9926M</t>
         </is>
       </c>
       <c r="D110" s="1" t="inlineStr">
         <is>
-          <t>NR36</t>
+          <t>NR30</t>
         </is>
       </c>
       <c r="E110" s="1" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>NR119</t>
         </is>
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>R766</t>
+          <t>QR1744</t>
         </is>
       </c>
       <c r="G110" s="1" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>TE2808</t>
         </is>
       </c>
       <c r="H110" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8077</t>
+          <t>VLINE-8072</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>MM-534M</t>
+          <t>MM-514M</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
         <is>
-          <t>MM-838M</t>
+          <t>MM-832M</t>
         </is>
       </c>
       <c r="C111" s="1" t="inlineStr">
         <is>
-          <t>MM-9932M</t>
+          <t>MM-9928M</t>
         </is>
       </c>
       <c r="D111" s="1" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>NR31</t>
         </is>
       </c>
       <c r="E111" s="1" t="inlineStr">
         <is>
-          <t>P2501</t>
+          <t>NR120</t>
         </is>
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>QR1771</t>
         </is>
       </c>
       <c r="G111" s="1" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>TE2809</t>
         </is>
       </c>
       <c r="H111" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8080</t>
+          <t>VLINE-8074</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>MM-536M</t>
+          <t>MM-526M</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
         <is>
-          <t>MM-844M</t>
+          <t>MM-834M</t>
         </is>
       </c>
       <c r="C112" s="1" t="inlineStr">
         <is>
-          <t>MM-9933M</t>
+          <t>MM-9929M</t>
         </is>
       </c>
       <c r="D112" s="1" t="inlineStr">
         <is>
-          <t>NR38</t>
+          <t>NR34</t>
         </is>
       </c>
       <c r="E112" s="1" t="inlineStr">
         <is>
-          <t>P2502</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>RCTST4</t>
+          <t>QR5404</t>
         </is>
       </c>
       <c r="G112" s="1" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>TE2810</t>
         </is>
       </c>
       <c r="H112" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8081</t>
+          <t>VLINE-8075</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>MM-542M</t>
+          <t>MM-534M</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
         <is>
-          <t>MM-852M</t>
+          <t>MM-838M</t>
         </is>
       </c>
       <c r="C113" s="1" t="inlineStr">
         <is>
-          <t>MM-9938M</t>
+          <t>MM-9932M</t>
         </is>
       </c>
       <c r="D113" s="1" t="inlineStr">
         <is>
-          <t>NR39</t>
+          <t>NR36</t>
         </is>
       </c>
       <c r="E113" s="1" t="inlineStr">
         <is>
-          <t>P2503</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>R711</t>
         </is>
       </c>
       <c r="G113" s="1" t="inlineStr">
         <is>
-          <t>TJ107</t>
+          <t>TE2812</t>
         </is>
       </c>
       <c r="H113" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8084</t>
+          <t>VLINE-8076</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8088</t>
+          <t>VLINE-8077</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8336</t>
+          <t>VLINE-8318</t>
         </is>
       </c>
       <c r="C115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8625</t>
+          <t>VLINE-8610</t>
         </is>
       </c>
       <c r="D115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8805</t>
+          <t>VLINE-8801</t>
         </is>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>XRN009</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8089</t>
+          <t>VLINE-8080</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8337</t>
+          <t>VLINE-8321</t>
         </is>
       </c>
       <c r="C116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8630</t>
+          <t>VLINE-8612</t>
         </is>
       </c>
       <c r="D116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8806</t>
+          <t>VLINE-8802</t>
         </is>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>XRN020</t>
+          <t>XRN011</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8104</t>
+          <t>VLINE-8081</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8338</t>
+          <t>VLINE-8324</t>
         </is>
       </c>
       <c r="C117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8671</t>
+          <t>VLINE-8615</t>
         </is>
       </c>
       <c r="D117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8807</t>
+          <t>VLINE-8803</t>
         </is>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>XRN014</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8107</t>
+          <t>VLINE-8084</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8339</t>
+          <t>VLINE-8332</t>
         </is>
       </c>
       <c r="C118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8706</t>
+          <t>VLINE-8620</t>
         </is>
       </c>
       <c r="D118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8808</t>
+          <t>VLINE-8804</t>
         </is>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>XRN023</t>
+          <t>XRN017</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8110</t>
+          <t>VLINE-8088</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8362</t>
+          <t>VLINE-8336</t>
         </is>
       </c>
       <c r="C119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8711</t>
+          <t>VLINE-8625</t>
         </is>
       </c>
       <c r="D119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8809</t>
+          <t>VLINE-8805</t>
         </is>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>XRN025</t>
+          <t>XRN018</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8111</t>
+          <t>VLINE-8089</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8363</t>
+          <t>VLINE-8337</t>
         </is>
       </c>
       <c r="C120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8714</t>
+          <t>VLINE-8630</t>
         </is>
       </c>
       <c r="D120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8810</t>
+          <t>VLINE-8806</t>
         </is>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>XRN026</t>
+          <t>XRN020</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8113</t>
+          <t>VLINE-8104</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8365</t>
+          <t>VLINE-8338</t>
         </is>
       </c>
       <c r="C121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8717</t>
+          <t>VLINE-8671</t>
         </is>
       </c>
       <c r="D121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8811</t>
+          <t>VLINE-8807</t>
         </is>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>XRN027</t>
+          <t>XRN021</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8114</t>
+          <t>VLINE-8107</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8366</t>
+          <t>VLINE-8339</t>
         </is>
       </c>
       <c r="C122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8721</t>
+          <t>VLINE-8706</t>
         </is>
       </c>
       <c r="D122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8812</t>
+          <t>VLINE-8808</t>
         </is>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>Y163</t>
+          <t>XRN023</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8115</t>
+          <t>VLINE-8110</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8369</t>
+          <t>VLINE-8362</t>
         </is>
       </c>
       <c r="C123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8723</t>
+          <t>VLINE-8711</t>
         </is>
       </c>
       <c r="D123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8813</t>
+          <t>VLINE-8809</t>
+        </is>
+      </c>
+      <c r="E123" s="1" t="inlineStr">
+        <is>
+          <t>XRN025</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8119</t>
+          <t>VLINE-8111</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8403</t>
+          <t>VLINE-8363</t>
         </is>
       </c>
       <c r="C124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8725</t>
+          <t>VLINE-8714</t>
         </is>
       </c>
       <c r="D124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8814</t>
+          <t>VLINE-8810</t>
+        </is>
+      </c>
+      <c r="E124" s="1" t="inlineStr">
+        <is>
+          <t>XRN026</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8120</t>
+          <t>VLINE-8113</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8404</t>
+          <t>VLINE-8365</t>
         </is>
       </c>
       <c r="C125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8726</t>
+          <t>VLINE-8717</t>
         </is>
       </c>
       <c r="D125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8816</t>
+          <t>VLINE-8811</t>
+        </is>
+      </c>
+      <c r="E125" s="1" t="inlineStr">
+        <is>
+          <t>XRN027</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8121</t>
+          <t>VLINE-8114</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8406</t>
+          <t>VLINE-8366</t>
         </is>
       </c>
       <c r="C126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8727</t>
+          <t>VLINE-8721</t>
         </is>
       </c>
       <c r="D126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8817</t>
+          <t>VLINE-8812</t>
+        </is>
+      </c>
+      <c r="E126" s="1" t="inlineStr">
+        <is>
+          <t>Y163</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8124</t>
+          <t>VLINE-8115</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8408</t>
+          <t>VLINE-8369</t>
         </is>
       </c>
       <c r="C127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8729</t>
+          <t>VLINE-8723</t>
         </is>
       </c>
       <c r="D127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8818</t>
+          <t>VLINE-8813</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8126</t>
+          <t>VLINE-8119</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8411</t>
+          <t>VLINE-8403</t>
         </is>
       </c>
       <c r="C128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8730</t>
+          <t>VLINE-8725</t>
         </is>
       </c>
       <c r="D128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8819</t>
+          <t>VLINE-8814</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8127</t>
+          <t>VLINE-8120</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8413</t>
+          <t>VLINE-8404</t>
         </is>
       </c>
       <c r="C129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8731</t>
+          <t>VLINE-8726</t>
         </is>
       </c>
       <c r="D129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8822</t>
+          <t>VLINE-8816</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8128</t>
+          <t>VLINE-8121</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8415</t>
+          <t>VLINE-8406</t>
         </is>
       </c>
       <c r="C130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8733</t>
+          <t>VLINE-8727</t>
         </is>
       </c>
       <c r="D130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8860</t>
+          <t>VLINE-8817</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8129</t>
+          <t>VLINE-8124</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8417</t>
+          <t>VLINE-8408</t>
         </is>
       </c>
       <c r="C131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8735</t>
+          <t>VLINE-8729</t>
         </is>
       </c>
       <c r="D131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8861</t>
+          <t>VLINE-8818</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8132</t>
+          <t>VLINE-8126</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8418</t>
+          <t>VLINE-8411</t>
         </is>
       </c>
       <c r="C132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8736</t>
+          <t>VLINE-8730</t>
         </is>
       </c>
       <c r="D132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8862</t>
+          <t>VLINE-8819</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8134</t>
+          <t>VLINE-8127</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8419</t>
+          <t>VLINE-8413</t>
         </is>
       </c>
       <c r="C133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8737</t>
+          <t>VLINE-8731</t>
         </is>
       </c>
       <c r="D133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8863</t>
+          <t>VLINE-8822</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8136</t>
+          <t>VLINE-8128</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8420</t>
+          <t>VLINE-8415</t>
         </is>
       </c>
       <c r="C134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8739</t>
+          <t>VLINE-8733</t>
         </is>
       </c>
       <c r="D134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8864</t>
+          <t>VLINE-8860</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8145</t>
+          <t>VLINE-8129</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8421</t>
+          <t>VLINE-8417</t>
         </is>
       </c>
       <c r="C135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8740</t>
+          <t>VLINE-8735</t>
         </is>
       </c>
       <c r="D135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8865</t>
+          <t>VLINE-8861</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8148</t>
+          <t>VLINE-8132</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8422</t>
+          <t>VLINE-8418</t>
         </is>
       </c>
       <c r="C136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8741</t>
+          <t>VLINE-8736</t>
         </is>
       </c>
       <c r="D136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8866</t>
+          <t>VLINE-8862</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8150</t>
+          <t>VLINE-8134</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8424</t>
+          <t>VLINE-8419</t>
         </is>
       </c>
       <c r="C137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8742</t>
+          <t>VLINE-8737</t>
         </is>
       </c>
       <c r="D137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8867</t>
+          <t>VLINE-8863</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8151</t>
+          <t>VLINE-8136</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8425</t>
+          <t>VLINE-8420</t>
         </is>
       </c>
       <c r="C138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8743</t>
+          <t>VLINE-8739</t>
         </is>
       </c>
       <c r="D138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8868</t>
+          <t>VLINE-8864</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8152</t>
+          <t>VLINE-8145</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8426</t>
+          <t>VLINE-8421</t>
         </is>
       </c>
       <c r="C139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8744</t>
+          <t>VLINE-8740</t>
         </is>
       </c>
       <c r="D139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8869</t>
+          <t>VLINE-8865</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8153</t>
+          <t>VLINE-8148</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8427</t>
+          <t>VLINE-8422</t>
         </is>
       </c>
       <c r="C140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8745</t>
+          <t>VLINE-8741</t>
         </is>
       </c>
       <c r="D140" s="1" t="inlineStr">
         <is>
-          <t>WH001</t>
+          <t>VLINE-8866</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8154</t>
+          <t>VLINE-8150</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8428</t>
+          <t>VLINE-8424</t>
         </is>
       </c>
       <c r="C141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8746</t>
+          <t>VLINE-8742</t>
         </is>
       </c>
       <c r="D141" s="1" t="inlineStr">
         <is>
-          <t>WH003</t>
+          <t>VLINE-8867</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8155</t>
+          <t>VLINE-8151</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8429</t>
+          <t>VLINE-8425</t>
         </is>
       </c>
       <c r="C142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8748</t>
+          <t>VLINE-8743</t>
         </is>
       </c>
       <c r="D142" s="1" t="inlineStr">
         <is>
-          <t>WL02</t>
+          <t>VLINE-8868</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8157</t>
+          <t>VLINE-8152</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8430</t>
+          <t>VLINE-8426</t>
         </is>
       </c>
       <c r="C143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8750</t>
+          <t>VLINE-8744</t>
         </is>
       </c>
       <c r="D143" s="1" t="inlineStr">
         <is>
-          <t>X12-X14</t>
+          <t>VLINE-8869</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8158</t>
+          <t>VLINE-8153</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8432</t>
+          <t>VLINE-8427</t>
         </is>
       </c>
       <c r="C144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8751</t>
+          <t>VLINE-8745</t>
         </is>
       </c>
       <c r="D144" s="1" t="inlineStr">
         <is>
-          <t>X31</t>
+          <t>WH001</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8159</t>
+          <t>VLINE-8154</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8434</t>
+          <t>VLINE-8428</t>
         </is>
       </c>
       <c r="C145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8752</t>
+          <t>VLINE-8746</t>
         </is>
       </c>
       <c r="D145" s="1" t="inlineStr">
         <is>
-          <t>XP2000</t>
+          <t>WH003</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8160</t>
+          <t>VLINE-8155</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8441</t>
+          <t>VLINE-8429</t>
         </is>
       </c>
       <c r="C146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8753</t>
+          <t>VLINE-8748</t>
         </is>
       </c>
       <c r="D146" s="1" t="inlineStr">
         <is>
-          <t>XP2003</t>
+          <t>WL02</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8161</t>
+          <t>VLINE-8157</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8443</t>
+          <t>VLINE-8430</t>
         </is>
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8754</t>
+          <t>VLINE-8750</t>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
         <is>
-          <t>XP2004</t>
+          <t>X12-X14</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8162</t>
+          <t>VLINE-8158</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8444</t>
+          <t>VLINE-8432</t>
         </is>
       </c>
       <c r="C148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8755</t>
+          <t>VLINE-8751</t>
         </is>
       </c>
       <c r="D148" s="1" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>X31</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8171</t>
+          <t>VLINE-8159</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8446</t>
+          <t>VLINE-8434</t>
         </is>
       </c>
       <c r="C149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8756</t>
+          <t>VLINE-8752</t>
         </is>
       </c>
       <c r="D149" s="1" t="inlineStr">
         <is>
-          <t>XP2007</t>
+          <t>XP2000</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8172</t>
+          <t>VLINE-8160</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8447</t>
+          <t>VLINE-8441</t>
         </is>
       </c>
       <c r="C150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8757</t>
+          <t>VLINE-8753</t>
         </is>
       </c>
       <c r="D150" s="1" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>XP2003</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8179</t>
+          <t>VLINE-8161</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8449</t>
+          <t>VLINE-8443</t>
         </is>
       </c>
       <c r="C151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8758</t>
+          <t>VLINE-8754</t>
         </is>
       </c>
       <c r="D151" s="1" t="inlineStr">
         <is>
-          <t>XP2010</t>
+          <t>XP2004</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8180</t>
+          <t>VLINE-8162</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8450</t>
+          <t>VLINE-8444</t>
         </is>
       </c>
       <c r="C152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8759</t>
+          <t>VLINE-8755</t>
         </is>
       </c>
       <c r="D152" s="1" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>XP2005</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8181</t>
+          <t>VLINE-8171</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8451</t>
+          <t>VLINE-8446</t>
         </is>
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8760</t>
+          <t>VLINE-8756</t>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>XP2007</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8182</t>
+          <t>VLINE-8172</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8452</t>
+          <t>VLINE-8447</t>
         </is>
       </c>
       <c r="C154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8761</t>
+          <t>VLINE-8757</t>
         </is>
       </c>
       <c r="D154" s="1" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>XP2008</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8183</t>
+          <t>VLINE-8179</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8453</t>
+          <t>VLINE-8449</t>
         </is>
       </c>
       <c r="C155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8762</t>
+          <t>VLINE-8758</t>
         </is>
       </c>
       <c r="D155" s="1" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>XP2010</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8184</t>
+          <t>VLINE-8180</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8454</t>
+          <t>VLINE-8450</t>
         </is>
       </c>
       <c r="C156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8770</t>
+          <t>VLINE-8759</t>
         </is>
       </c>
       <c r="D156" s="1" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>XP2011</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8185</t>
+          <t>VLINE-8181</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8455</t>
+          <t>VLINE-8451</t>
         </is>
       </c>
       <c r="C157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8772</t>
+          <t>VLINE-8760</t>
         </is>
       </c>
       <c r="D157" s="1" t="inlineStr">
         <is>
-          <t>XP2016</t>
+          <t>XP2012</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8186</t>
+          <t>VLINE-8182</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8456</t>
+          <t>VLINE-8452</t>
         </is>
       </c>
       <c r="C158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8774</t>
+          <t>VLINE-8761</t>
         </is>
       </c>
       <c r="D158" s="1" t="inlineStr">
         <is>
-          <t>XP2017</t>
+          <t>XP2013</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8187</t>
+          <t>VLINE-8183</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8457</t>
+          <t>VLINE-8453</t>
         </is>
       </c>
       <c r="C159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8776</t>
+          <t>VLINE-8762</t>
         </is>
       </c>
       <c r="D159" s="1" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>XP2014</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8189</t>
+          <t>VLINE-8184</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8460</t>
+          <t>VLINE-8454</t>
         </is>
       </c>
       <c r="C160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8778</t>
+          <t>VLINE-8770</t>
         </is>
       </c>
       <c r="D160" s="1" t="inlineStr">
         <is>
-          <t>XR550</t>
+          <t>XP2015</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8303</t>
+          <t>VLINE-8185</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8461</t>
+          <t>VLINE-8455</t>
         </is>
       </c>
       <c r="C161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8780</t>
+          <t>VLINE-8772</t>
         </is>
       </c>
       <c r="D161" s="1" t="inlineStr">
         <is>
-          <t>XR552</t>
+          <t>XP2016</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8304</t>
+          <t>VLINE-8186</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8464</t>
+          <t>VLINE-8456</t>
         </is>
       </c>
       <c r="C162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8793</t>
+          <t>VLINE-8774</t>
         </is>
       </c>
       <c r="D162" s="1" t="inlineStr">
         <is>
-          <t>XRN001</t>
+          <t>XP2017</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8311</t>
+          <t>VLINE-8187</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8465</t>
+          <t>VLINE-8457</t>
         </is>
       </c>
       <c r="C163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8795</t>
+          <t>VLINE-8776</t>
         </is>
       </c>
       <c r="D163" s="1" t="inlineStr">
         <is>
-          <t>XRN004</t>
+          <t>XP2019</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8313</t>
+          <t>VLINE-8189</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8468</t>
+          <t>VLINE-8460</t>
         </is>
       </c>
       <c r="C164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8797</t>
+          <t>VLINE-8778</t>
         </is>
       </c>
       <c r="D164" s="1" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>XR550</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8314</t>
+          <t>VLINE-8303</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8469</t>
+          <t>VLINE-8461</t>
         </is>
       </c>
       <c r="C165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8799</t>
+          <t>VLINE-8780</t>
         </is>
       </c>
       <c r="D165" s="1" t="inlineStr">
         <is>
-          <t>XRN006</t>
+          <t>XR552</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8316</t>
+          <t>VLINE-8304</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8605</t>
+          <t>VLINE-8464</t>
         </is>
       </c>
       <c r="C166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8800</t>
+          <t>VLINE-8793</t>
         </is>
       </c>
       <c r="D166" s="1" t="inlineStr">
         <is>
-          <t>XRN007</t>
+          <t>XRN001</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8318</t>
+          <t>VLINE-8311</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8610</t>
+          <t>VLINE-8465</t>
         </is>
       </c>
       <c r="C167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8801</t>
+          <t>VLINE-8795</t>
         </is>
       </c>
       <c r="D167" s="1" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>XRN004</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8321</t>
+          <t>VLINE-8313</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8612</t>
+          <t>VLINE-8468</t>
         </is>
       </c>
       <c r="C168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8802</t>
+          <t>VLINE-8797</t>
         </is>
       </c>
       <c r="D168" s="1" t="inlineStr">
         <is>
-          <t>XRN011</t>
+          <t>XRN005</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8324</t>
+          <t>VLINE-8314</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8615</t>
+          <t>VLINE-8469</t>
         </is>
       </c>
       <c r="C169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8803</t>
+          <t>VLINE-8799</t>
         </is>
       </c>
       <c r="D169" s="1" t="inlineStr">
         <is>
-          <t>XRN014</t>
+          <t>XRN006</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8332</t>
+          <t>VLINE-8316</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8620</t>
+          <t>VLINE-8605</t>
         </is>
       </c>
       <c r="C170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8804</t>
+          <t>VLINE-8800</t>
         </is>
       </c>
       <c r="D170" s="1" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>XRN007</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update trains and loco export 2026-04-04 22:53:37
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -2789,37 +2789,37 @@
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
-          <t>MM-418M</t>
+          <t>MM-392M</t>
         </is>
       </c>
       <c r="C58" s="1" t="inlineStr">
         <is>
-          <t>MM-816M</t>
+          <t>MM-814M</t>
         </is>
       </c>
       <c r="D58" s="1" t="inlineStr">
         <is>
-          <t>MM-9915M</t>
+          <t>MM-9914M</t>
         </is>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>NR12</t>
+          <t>NR9</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>NR103</t>
+          <t>NR102</t>
         </is>
       </c>
       <c r="G58" s="1" t="inlineStr">
         <is>
-          <t>QL001</t>
+          <t>QE006</t>
         </is>
       </c>
       <c r="H58" s="1" t="inlineStr">
         <is>
-          <t>T363</t>
+          <t>SSR104</t>
         </is>
       </c>
     </row>
@@ -2831,37 +2831,37 @@
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
-          <t>MM-430M</t>
+          <t>MM-418M</t>
         </is>
       </c>
       <c r="C59" s="1" t="inlineStr">
         <is>
-          <t>MM-818M</t>
+          <t>MM-816M</t>
         </is>
       </c>
       <c r="D59" s="1" t="inlineStr">
         <is>
-          <t>MM-9917M</t>
+          <t>MM-9915M</t>
         </is>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>NR15</t>
+          <t>NR12</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>NR105</t>
+          <t>NR103</t>
         </is>
       </c>
       <c r="G59" s="1" t="inlineStr">
         <is>
-          <t>QL002</t>
+          <t>QL001</t>
         </is>
       </c>
       <c r="H59" s="1" t="inlineStr">
         <is>
-          <t>T386</t>
+          <t>T363</t>
         </is>
       </c>
     </row>
@@ -2873,37 +2873,37 @@
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
-          <t>MM-444M</t>
+          <t>MM-430M</t>
         </is>
       </c>
       <c r="C60" s="1" t="inlineStr">
         <is>
-          <t>MM-820M</t>
+          <t>MM-818M</t>
         </is>
       </c>
       <c r="D60" s="1" t="inlineStr">
         <is>
-          <t>MM-9918M</t>
+          <t>MM-9917M</t>
         </is>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>NR16</t>
+          <t>NR15</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>NR108</t>
+          <t>NR105</t>
         </is>
       </c>
       <c r="G60" s="1" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>QL002</t>
         </is>
       </c>
       <c r="H60" s="1" t="inlineStr">
         <is>
-          <t>TDX101</t>
+          <t>T386</t>
         </is>
       </c>
     </row>
@@ -2915,37 +2915,37 @@
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
-          <t>MM-464M</t>
+          <t>MM-444M</t>
         </is>
       </c>
       <c r="C61" s="1" t="inlineStr">
         <is>
-          <t>MM-824M</t>
+          <t>MM-820M</t>
         </is>
       </c>
       <c r="D61" s="1" t="inlineStr">
         <is>
-          <t>MM-9919M</t>
+          <t>MM-9918M</t>
         </is>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>NR18</t>
+          <t>NR16</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR108</t>
         </is>
       </c>
       <c r="G61" s="1" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>QL004</t>
         </is>
       </c>
       <c r="H61" s="1" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>TDX101</t>
         </is>
       </c>
     </row>
@@ -2957,37 +2957,37 @@
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
-          <t>MM-486M</t>
+          <t>MM-464M</t>
         </is>
       </c>
       <c r="C62" s="1" t="inlineStr">
         <is>
-          <t>MM-826M</t>
+          <t>MM-824M</t>
         </is>
       </c>
       <c r="D62" s="1" t="inlineStr">
         <is>
-          <t>MM-9920M</t>
+          <t>MM-9919M</t>
         </is>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>NR19</t>
+          <t>NR18</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>NR110</t>
+          <t>NR109</t>
         </is>
       </c>
       <c r="G62" s="1" t="inlineStr">
         <is>
-          <t>QL008</t>
+          <t>QL007</t>
         </is>
       </c>
       <c r="H62" s="1" t="inlineStr">
         <is>
-          <t>TE2802</t>
+          <t>TE2801</t>
         </is>
       </c>
     </row>
@@ -2999,37 +2999,37 @@
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
-          <t>MM-496M</t>
+          <t>MM-486M</t>
         </is>
       </c>
       <c r="C63" s="1" t="inlineStr">
         <is>
-          <t>MM-828M</t>
+          <t>MM-826M</t>
         </is>
       </c>
       <c r="D63" s="1" t="inlineStr">
         <is>
-          <t>MM-9922M</t>
+          <t>MM-9920M</t>
         </is>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>NR21</t>
+          <t>NR19</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR110</t>
         </is>
       </c>
       <c r="G63" s="1" t="inlineStr">
         <is>
-          <t>QL010</t>
+          <t>QL008</t>
         </is>
       </c>
       <c r="H63" s="1" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>TE2802</t>
         </is>
       </c>
     </row>
@@ -3041,37 +3041,37 @@
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
-          <t>MM-514M</t>
+          <t>MM-496M</t>
         </is>
       </c>
       <c r="C64" s="1" t="inlineStr">
         <is>
-          <t>MM-830M</t>
+          <t>MM-828M</t>
         </is>
       </c>
       <c r="D64" s="1" t="inlineStr">
         <is>
-          <t>MM-9923M</t>
+          <t>MM-9922M</t>
         </is>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>NR25</t>
+          <t>NR21</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR112</t>
         </is>
       </c>
       <c r="G64" s="1" t="inlineStr">
         <is>
-          <t>QL011</t>
+          <t>QL010</t>
         </is>
       </c>
       <c r="H64" s="1" t="inlineStr">
         <is>
-          <t>TE2804</t>
+          <t>TE2803</t>
         </is>
       </c>
     </row>
@@ -3083,37 +3083,37 @@
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
-          <t>MM-526M</t>
+          <t>MM-514M</t>
         </is>
       </c>
       <c r="C65" s="1" t="inlineStr">
         <is>
-          <t>MM-832M</t>
+          <t>MM-830M</t>
         </is>
       </c>
       <c r="D65" s="1" t="inlineStr">
         <is>
-          <t>MM-9924M</t>
+          <t>MM-9923M</t>
         </is>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>NR27</t>
+          <t>NR25</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR113</t>
         </is>
       </c>
       <c r="G65" s="1" t="inlineStr">
         <is>
-          <t>QL014</t>
+          <t>QL011</t>
         </is>
       </c>
       <c r="H65" s="1" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>TE2804</t>
         </is>
       </c>
     </row>
@@ -3125,37 +3125,37 @@
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
-          <t>MM-534M</t>
+          <t>MM-526M</t>
         </is>
       </c>
       <c r="C66" s="1" t="inlineStr">
         <is>
-          <t>MM-834M</t>
+          <t>MM-832M</t>
         </is>
       </c>
       <c r="D66" s="1" t="inlineStr">
         <is>
-          <t>MM-9926M</t>
+          <t>MM-9924M</t>
         </is>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>NR28</t>
+          <t>NR27</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>NR118</t>
+          <t>NR115</t>
         </is>
       </c>
       <c r="G66" s="1" t="inlineStr">
         <is>
-          <t>QL018</t>
+          <t>QL014</t>
         </is>
       </c>
       <c r="H66" s="1" t="inlineStr">
         <is>
-          <t>TE2806</t>
+          <t>TE2805</t>
         </is>
       </c>
     </row>
@@ -3167,37 +3167,37 @@
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
-          <t>MM-536M</t>
+          <t>MM-534M</t>
         </is>
       </c>
       <c r="C67" s="1" t="inlineStr">
         <is>
-          <t>MM-838M</t>
+          <t>MM-834M</t>
         </is>
       </c>
       <c r="D67" s="1" t="inlineStr">
         <is>
-          <t>MM-9928M</t>
+          <t>MM-9926M</t>
         </is>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>NR30</t>
+          <t>NR28</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>NR119</t>
+          <t>NR118</t>
         </is>
       </c>
       <c r="G67" s="1" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QL018</t>
         </is>
       </c>
       <c r="H67" s="1" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>TE2806</t>
         </is>
       </c>
     </row>
@@ -3209,37 +3209,37 @@
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
-          <t>MM-542M</t>
+          <t>MM-536M</t>
         </is>
       </c>
       <c r="C68" s="1" t="inlineStr">
         <is>
-          <t>MM-844M</t>
+          <t>MM-838M</t>
         </is>
       </c>
       <c r="D68" s="1" t="inlineStr">
         <is>
-          <t>MM-9929M</t>
+          <t>MM-9928M</t>
         </is>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>NR31</t>
+          <t>NR30</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>NR120</t>
+          <t>NR119</t>
         </is>
       </c>
       <c r="G68" s="1" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QR1744</t>
         </is>
       </c>
       <c r="H68" s="1" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>TE2807</t>
         </is>
       </c>
     </row>
@@ -3251,37 +3251,37 @@
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
-          <t>MM-544M</t>
+          <t>MM-542M</t>
         </is>
       </c>
       <c r="C69" s="1" t="inlineStr">
         <is>
-          <t>MM-852M</t>
+          <t>MM-844M</t>
         </is>
       </c>
       <c r="D69" s="1" t="inlineStr">
         <is>
-          <t>MM-9932M</t>
+          <t>MM-9929M</t>
         </is>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>NR34</t>
+          <t>NR31</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>NR122</t>
+          <t>NR120</t>
         </is>
       </c>
       <c r="G69" s="1" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QR1771</t>
         </is>
       </c>
       <c r="H69" s="1" t="inlineStr">
         <is>
-          <t>TE2809</t>
+          <t>TE2808</t>
         </is>
       </c>
     </row>
@@ -3293,37 +3293,37 @@
       </c>
       <c r="B70" s="1" t="inlineStr">
         <is>
-          <t>MM-546M</t>
+          <t>MM-544M</t>
         </is>
       </c>
       <c r="C70" s="1" t="inlineStr">
         <is>
-          <t>MM-858M</t>
+          <t>MM-852M</t>
         </is>
       </c>
       <c r="D70" s="1" t="inlineStr">
         <is>
-          <t>MM-9933M</t>
+          <t>MM-9932M</t>
         </is>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>NR36</t>
+          <t>NR34</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>NR122</t>
         </is>
       </c>
       <c r="G70" s="1" t="inlineStr">
         <is>
-          <t>R711</t>
+          <t>QR5404</t>
         </is>
       </c>
       <c r="H70" s="1" t="inlineStr">
         <is>
-          <t>TE2810</t>
+          <t>TE2809</t>
         </is>
       </c>
     </row>
@@ -3335,37 +3335,37 @@
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
-          <t>MM-551M</t>
+          <t>MM-546M</t>
         </is>
       </c>
       <c r="C71" s="1" t="inlineStr">
         <is>
-          <t>MM-860M</t>
+          <t>MM-858M</t>
         </is>
       </c>
       <c r="D71" s="1" t="inlineStr">
         <is>
-          <t>MM-9936M</t>
+          <t>MM-9933M</t>
         </is>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>NR36</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="G71" s="1" t="inlineStr">
         <is>
-          <t>R766</t>
+          <t>R711</t>
         </is>
       </c>
       <c r="H71" s="1" t="inlineStr">
         <is>
-          <t>TE2812</t>
+          <t>TE2810</t>
         </is>
       </c>
     </row>
@@ -3377,37 +3377,37 @@
       </c>
       <c r="B72" s="1" t="inlineStr">
         <is>
-          <t>MM-588M</t>
+          <t>MM-551M</t>
         </is>
       </c>
       <c r="C72" s="1" t="inlineStr">
         <is>
-          <t>MM-862M</t>
+          <t>MM-860M</t>
         </is>
       </c>
       <c r="D72" s="1" t="inlineStr">
         <is>
-          <t>MM-9938M</t>
+          <t>MM-9936M</t>
         </is>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>NR38</t>
+          <t>NR37</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>P2501</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="G72" s="1" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>R766</t>
         </is>
       </c>
       <c r="H72" s="1" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>TE2812</t>
         </is>
       </c>
     </row>
@@ -3419,37 +3419,37 @@
       </c>
       <c r="B73" s="1" t="inlineStr">
         <is>
-          <t>MM-602M</t>
+          <t>MM-588M</t>
         </is>
       </c>
       <c r="C73" s="1" t="inlineStr">
         <is>
-          <t>MM-868M</t>
+          <t>MM-862M</t>
         </is>
       </c>
       <c r="D73" s="1" t="inlineStr">
         <is>
-          <t>MM-9941M</t>
+          <t>MM-9938M</t>
         </is>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>NR39</t>
+          <t>NR38</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>P2502</t>
+          <t>P2501</t>
         </is>
       </c>
       <c r="G73" s="1" t="inlineStr">
         <is>
-          <t>RCTST4</t>
+          <t>RB2353</t>
         </is>
       </c>
       <c r="H73" s="1" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>TE2813</t>
         </is>
       </c>
     </row>
@@ -3461,37 +3461,37 @@
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
-          <t>MM-624M</t>
+          <t>MM-602M</t>
         </is>
       </c>
       <c r="C74" s="1" t="inlineStr">
         <is>
-          <t>MM-872M</t>
+          <t>MM-868M</t>
         </is>
       </c>
       <c r="D74" s="1" t="inlineStr">
         <is>
-          <t>MM-9943M</t>
+          <t>MM-9941M</t>
         </is>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>NR40</t>
+          <t>NR39</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>P2503</t>
+          <t>P2502</t>
         </is>
       </c>
       <c r="G74" s="1" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>RCTST4</t>
         </is>
       </c>
       <c r="H74" s="1" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>TE2814</t>
         </is>
       </c>
     </row>
@@ -3503,37 +3503,37 @@
       </c>
       <c r="B75" s="1" t="inlineStr">
         <is>
-          <t>MM-636M</t>
+          <t>MM-624M</t>
         </is>
       </c>
       <c r="C75" s="1" t="inlineStr">
         <is>
-          <t>MM-874M</t>
+          <t>MM-872M</t>
         </is>
       </c>
       <c r="D75" s="1" t="inlineStr">
         <is>
-          <t>MM-9945M</t>
+          <t>MM-9943M</t>
         </is>
       </c>
       <c r="E75" s="1" t="inlineStr">
         <is>
-          <t>NR43</t>
+          <t>NR40</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>P2505</t>
+          <t>P2503</t>
         </is>
       </c>
       <c r="G75" s="1" t="inlineStr">
         <is>
-          <t>RL302</t>
+          <t>RL301</t>
         </is>
       </c>
       <c r="H75" s="1" t="inlineStr">
         <is>
-          <t>TJ107</t>
+          <t>TJ096</t>
         </is>
       </c>
     </row>
@@ -3545,37 +3545,37 @@
       </c>
       <c r="B76" s="1" t="inlineStr">
         <is>
-          <t>MM-640M</t>
+          <t>MM-636M</t>
         </is>
       </c>
       <c r="C76" s="1" t="inlineStr">
         <is>
-          <t>MM-876M</t>
+          <t>MM-874M</t>
         </is>
       </c>
       <c r="D76" s="1" t="inlineStr">
         <is>
-          <t>MM-9946M</t>
+          <t>MM-9945M</t>
         </is>
       </c>
       <c r="E76" s="1" t="inlineStr">
         <is>
-          <t>NR44</t>
+          <t>NR43</t>
         </is>
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>P2506</t>
+          <t>P2505</t>
         </is>
       </c>
       <c r="G76" s="1" t="inlineStr">
         <is>
-          <t>RL304</t>
+          <t>RL302</t>
         </is>
       </c>
       <c r="H76" s="1" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TJ107</t>
         </is>
       </c>
     </row>
@@ -3587,37 +3587,37 @@
       </c>
       <c r="B77" s="1" t="inlineStr">
         <is>
-          <t>MM-654M</t>
+          <t>MM-640M</t>
         </is>
       </c>
       <c r="C77" s="1" t="inlineStr">
         <is>
-          <t>MM-882M</t>
+          <t>MM-876M</t>
         </is>
       </c>
       <c r="D77" s="1" t="inlineStr">
         <is>
-          <t>MM-9950M</t>
+          <t>MM-9946M</t>
         </is>
       </c>
       <c r="E77" s="1" t="inlineStr">
         <is>
-          <t>NR45</t>
+          <t>NR44</t>
         </is>
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
-          <t>P2507</t>
+          <t>P2506</t>
         </is>
       </c>
       <c r="G77" s="1" t="inlineStr">
         <is>
-          <t>RL307</t>
+          <t>RL304</t>
         </is>
       </c>
       <c r="H77" s="1" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TT03</t>
         </is>
       </c>
     </row>
@@ -3629,37 +3629,37 @@
       </c>
       <c r="B78" s="1" t="inlineStr">
         <is>
-          <t>MM-656M</t>
+          <t>MM-654M</t>
         </is>
       </c>
       <c r="C78" s="1" t="inlineStr">
         <is>
-          <t>MM-894M</t>
+          <t>MM-882M</t>
         </is>
       </c>
       <c r="D78" s="1" t="inlineStr">
         <is>
-          <t>MM-9951M</t>
+          <t>MM-9950M</t>
         </is>
       </c>
       <c r="E78" s="1" t="inlineStr">
         <is>
-          <t>NR51</t>
+          <t>NR45</t>
         </is>
       </c>
       <c r="F78" s="1" t="inlineStr">
         <is>
-          <t>P2508</t>
+          <t>P2507</t>
         </is>
       </c>
       <c r="G78" s="1" t="inlineStr">
         <is>
-          <t>RL309</t>
+          <t>RL307</t>
         </is>
       </c>
       <c r="H78" s="1" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TT04</t>
         </is>
       </c>
     </row>
@@ -3671,37 +3671,37 @@
       </c>
       <c r="B79" s="1" t="inlineStr">
         <is>
-          <t>MM-660M</t>
+          <t>MM-656M</t>
         </is>
       </c>
       <c r="C79" s="1" t="inlineStr">
         <is>
-          <t>MM-896M</t>
+          <t>MM-894M</t>
         </is>
       </c>
       <c r="D79" s="1" t="inlineStr">
         <is>
-          <t>MM-9952M</t>
+          <t>MM-9951M</t>
         </is>
       </c>
       <c r="E79" s="1" t="inlineStr">
         <is>
-          <t>NR52</t>
+          <t>NR51</t>
         </is>
       </c>
       <c r="F79" s="1" t="inlineStr">
         <is>
-          <t>P2509</t>
+          <t>P2508</t>
         </is>
       </c>
       <c r="G79" s="1" t="inlineStr">
         <is>
-          <t>RL310</t>
+          <t>RL309</t>
         </is>
       </c>
       <c r="H79" s="1" t="inlineStr">
         <is>
-          <t>TT07</t>
+          <t>TT05</t>
         </is>
       </c>
     </row>
@@ -3713,37 +3713,37 @@
       </c>
       <c r="B80" s="1" t="inlineStr">
         <is>
-          <t>MM-661M</t>
+          <t>MM-660M</t>
         </is>
       </c>
       <c r="C80" s="1" t="inlineStr">
         <is>
-          <t>MM-902M</t>
+          <t>MM-896M</t>
         </is>
       </c>
       <c r="D80" s="1" t="inlineStr">
         <is>
-          <t>MM-9953M</t>
+          <t>MM-9952M</t>
         </is>
       </c>
       <c r="E80" s="1" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>NR52</t>
         </is>
       </c>
       <c r="F80" s="1" t="inlineStr">
         <is>
-          <t>P2510</t>
+          <t>P2509</t>
         </is>
       </c>
       <c r="G80" s="1" t="inlineStr">
         <is>
-          <t>S312</t>
+          <t>RL310</t>
         </is>
       </c>
       <c r="H80" s="1" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TT07</t>
         </is>
       </c>
     </row>
@@ -3755,37 +3755,37 @@
       </c>
       <c r="B81" s="1" t="inlineStr">
         <is>
-          <t>MM-664M</t>
+          <t>MM-661M</t>
         </is>
       </c>
       <c r="C81" s="1" t="inlineStr">
         <is>
-          <t>MM-904M</t>
+          <t>MM-902M</t>
         </is>
       </c>
       <c r="D81" s="1" t="inlineStr">
         <is>
-          <t>MM-9954M</t>
+          <t>MM-9953M</t>
         </is>
       </c>
       <c r="E81" s="1" t="inlineStr">
         <is>
-          <t>NR57</t>
+          <t>NR54</t>
         </is>
       </c>
       <c r="F81" s="1" t="inlineStr">
         <is>
-          <t>P2511</t>
+          <t>P2510</t>
         </is>
       </c>
       <c r="G81" s="1" t="inlineStr">
         <is>
-          <t>S317</t>
+          <t>S312</t>
         </is>
       </c>
       <c r="H81" s="1" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TT08</t>
         </is>
       </c>
     </row>
@@ -3797,37 +3797,37 @@
       </c>
       <c r="B82" s="1" t="inlineStr">
         <is>
-          <t>MM-666M</t>
+          <t>MM-664M</t>
         </is>
       </c>
       <c r="C82" s="1" t="inlineStr">
         <is>
-          <t>MM-906M</t>
+          <t>MM-904M</t>
         </is>
       </c>
       <c r="D82" s="1" t="inlineStr">
         <is>
-          <t>MM-9955M</t>
+          <t>MM-9954M</t>
         </is>
       </c>
       <c r="E82" s="1" t="inlineStr">
         <is>
-          <t>NR59</t>
+          <t>NR57</t>
         </is>
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
-          <t>P2513</t>
+          <t>P2511</t>
         </is>
       </c>
       <c r="G82" s="1" t="inlineStr">
         <is>
-          <t>S3301</t>
+          <t>S317</t>
         </is>
       </c>
       <c r="H82" s="1" t="inlineStr">
         <is>
-          <t>TT106</t>
+          <t>TT103</t>
         </is>
       </c>
     </row>
@@ -3839,37 +3839,37 @@
       </c>
       <c r="B83" s="1" t="inlineStr">
         <is>
-          <t>MM-668M</t>
+          <t>MM-666M</t>
         </is>
       </c>
       <c r="C83" s="1" t="inlineStr">
         <is>
-          <t>MM-908M</t>
+          <t>MM-906M</t>
         </is>
       </c>
       <c r="D83" s="1" t="inlineStr">
         <is>
-          <t>MM-9957M</t>
+          <t>MM-9955M</t>
         </is>
       </c>
       <c r="E83" s="1" t="inlineStr">
         <is>
-          <t>NR61</t>
+          <t>NR59</t>
         </is>
       </c>
       <c r="F83" s="1" t="inlineStr">
         <is>
-          <t>P2514</t>
+          <t>P2513</t>
         </is>
       </c>
       <c r="G83" s="1" t="inlineStr">
         <is>
-          <t>S3302</t>
+          <t>S3301</t>
         </is>
       </c>
       <c r="H83" s="1" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TT106</t>
         </is>
       </c>
     </row>
@@ -3881,37 +3881,37 @@
       </c>
       <c r="B84" s="1" t="inlineStr">
         <is>
-          <t>MM-673M</t>
+          <t>MM-668M</t>
         </is>
       </c>
       <c r="C84" s="1" t="inlineStr">
         <is>
-          <t>MM-910M</t>
+          <t>MM-908M</t>
         </is>
       </c>
       <c r="D84" s="1" t="inlineStr">
         <is>
-          <t>MM-9959M</t>
+          <t>MM-9957M</t>
         </is>
       </c>
       <c r="E84" s="1" t="inlineStr">
         <is>
-          <t>NR62</t>
+          <t>NR61</t>
         </is>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>P2515</t>
+          <t>P2514</t>
         </is>
       </c>
       <c r="G84" s="1" t="inlineStr">
         <is>
-          <t>S3304</t>
+          <t>S3302</t>
         </is>
       </c>
       <c r="H84" s="1" t="inlineStr">
         <is>
-          <t>TT108</t>
+          <t>TT107</t>
         </is>
       </c>
     </row>
@@ -3923,37 +3923,37 @@
       </c>
       <c r="B85" s="1" t="inlineStr">
         <is>
-          <t>MM-674M</t>
+          <t>MM-673M</t>
         </is>
       </c>
       <c r="C85" s="1" t="inlineStr">
         <is>
-          <t>MM-912M</t>
+          <t>MM-910M</t>
         </is>
       </c>
       <c r="D85" s="1" t="inlineStr">
         <is>
-          <t>MM-9960M</t>
+          <t>MM-9959M</t>
         </is>
       </c>
       <c r="E85" s="1" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR62</t>
         </is>
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>P2516</t>
+          <t>P2515</t>
         </is>
       </c>
       <c r="G85" s="1" t="inlineStr">
         <is>
-          <t>S3305</t>
+          <t>S3304</t>
         </is>
       </c>
       <c r="H85" s="1" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TT108</t>
         </is>
       </c>
     </row>
@@ -3965,37 +3965,37 @@
       </c>
       <c r="B86" s="1" t="inlineStr">
         <is>
-          <t>MM-680M</t>
+          <t>MM-674M</t>
         </is>
       </c>
       <c r="C86" s="1" t="inlineStr">
         <is>
-          <t>MM-914M</t>
+          <t>MM-912M</t>
         </is>
       </c>
       <c r="D86" s="1" t="inlineStr">
         <is>
-          <t>MM-9961M</t>
+          <t>MM-9960M</t>
         </is>
       </c>
       <c r="E86" s="1" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR64</t>
         </is>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>PB2</t>
+          <t>P2516</t>
         </is>
       </c>
       <c r="G86" s="1" t="inlineStr">
         <is>
-          <t>S3306</t>
+          <t>S3305</t>
         </is>
       </c>
       <c r="H86" s="1" t="inlineStr">
         <is>
-          <t>TT114</t>
+          <t>TT110</t>
         </is>
       </c>
     </row>
@@ -4007,37 +4007,37 @@
       </c>
       <c r="B87" s="1" t="inlineStr">
         <is>
-          <t>MM-708M</t>
+          <t>MM-680M</t>
         </is>
       </c>
       <c r="C87" s="1" t="inlineStr">
         <is>
-          <t>MM-920M</t>
+          <t>MM-914M</t>
         </is>
       </c>
       <c r="D87" s="1" t="inlineStr">
         <is>
-          <t>MM-9962M</t>
+          <t>MM-9961M</t>
         </is>
       </c>
       <c r="E87" s="1" t="inlineStr">
         <is>
-          <t>NR66</t>
+          <t>NR65</t>
         </is>
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>PB2</t>
         </is>
       </c>
       <c r="G87" s="1" t="inlineStr">
         <is>
-          <t>S3307</t>
+          <t>S3306</t>
         </is>
       </c>
       <c r="H87" s="1" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT114</t>
         </is>
       </c>
     </row>
@@ -4049,37 +4049,37 @@
       </c>
       <c r="B88" s="1" t="inlineStr">
         <is>
-          <t>MM-722M</t>
+          <t>MM-708M</t>
         </is>
       </c>
       <c r="C88" s="1" t="inlineStr">
         <is>
-          <t>MM-922M</t>
+          <t>MM-920M</t>
         </is>
       </c>
       <c r="D88" s="1" t="inlineStr">
         <is>
-          <t>MM-9963M</t>
+          <t>MM-9962M</t>
         </is>
       </c>
       <c r="E88" s="1" t="inlineStr">
         <is>
-          <t>NR67</t>
+          <t>NR66</t>
         </is>
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>PB4</t>
         </is>
       </c>
       <c r="G88" s="1" t="inlineStr">
         <is>
-          <t>S3309</t>
+          <t>S3307</t>
         </is>
       </c>
       <c r="H88" s="1" t="inlineStr">
         <is>
-          <t>TT116</t>
+          <t>TT115</t>
         </is>
       </c>
     </row>
@@ -4091,37 +4091,37 @@
       </c>
       <c r="B89" s="1" t="inlineStr">
         <is>
-          <t>MM-726M</t>
+          <t>MM-722M</t>
         </is>
       </c>
       <c r="C89" s="1" t="inlineStr">
         <is>
-          <t>MM-924M</t>
+          <t>MM-922M</t>
         </is>
       </c>
       <c r="D89" s="1" t="inlineStr">
         <is>
-          <t>MM-9964M</t>
+          <t>MM-9963M</t>
         </is>
       </c>
       <c r="E89" s="1" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR67</t>
         </is>
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>PHC002</t>
+          <t>PHC001</t>
         </is>
       </c>
       <c r="G89" s="1" t="inlineStr">
         <is>
-          <t>S3310</t>
+          <t>S3309</t>
         </is>
       </c>
       <c r="H89" s="1" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT116</t>
         </is>
       </c>
     </row>
@@ -4133,37 +4133,37 @@
       </c>
       <c r="B90" s="1" t="inlineStr">
         <is>
-          <t>MM-728M</t>
+          <t>MM-726M</t>
         </is>
       </c>
       <c r="C90" s="1" t="inlineStr">
         <is>
-          <t>MM-926M</t>
+          <t>MM-924M</t>
         </is>
       </c>
       <c r="D90" s="1" t="inlineStr">
         <is>
-          <t>MM-9965M</t>
+          <t>MM-9964M</t>
         </is>
       </c>
       <c r="E90" s="1" t="inlineStr">
         <is>
-          <t>NR69</t>
+          <t>NR68</t>
         </is>
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>Q4001</t>
+          <t>PHC002</t>
         </is>
       </c>
       <c r="G90" s="1" t="inlineStr">
         <is>
-          <t>S7001</t>
+          <t>S3310</t>
         </is>
       </c>
       <c r="H90" s="1" t="inlineStr">
         <is>
-          <t>TT122</t>
+          <t>TT117</t>
         </is>
       </c>
     </row>
@@ -4175,37 +4175,37 @@
       </c>
       <c r="B91" s="1" t="inlineStr">
         <is>
-          <t>MM-734M</t>
+          <t>MM-728M</t>
         </is>
       </c>
       <c r="C91" s="1" t="inlineStr">
         <is>
-          <t>MM-934M</t>
+          <t>MM-926M</t>
         </is>
       </c>
       <c r="D91" s="1" t="inlineStr">
         <is>
-          <t>MM-9966M</t>
+          <t>MM-9965M</t>
         </is>
       </c>
       <c r="E91" s="1" t="inlineStr">
         <is>
-          <t>NR71</t>
+          <t>NR69</t>
         </is>
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>Q4003</t>
+          <t>Q4001</t>
         </is>
       </c>
       <c r="G91" s="1" t="inlineStr">
         <is>
-          <t>S7002</t>
+          <t>S7001</t>
         </is>
       </c>
       <c r="H91" s="1" t="inlineStr">
         <is>
-          <t>TT127</t>
+          <t>TT122</t>
         </is>
       </c>
     </row>
@@ -4217,37 +4217,37 @@
       </c>
       <c r="B92" s="1" t="inlineStr">
         <is>
-          <t>MM-736M</t>
+          <t>MM-734M</t>
         </is>
       </c>
       <c r="C92" s="1" t="inlineStr">
         <is>
-          <t>MM-936M</t>
+          <t>MM-934M</t>
         </is>
       </c>
       <c r="D92" s="1" t="inlineStr">
         <is>
-          <t>MM-9967M</t>
+          <t>MM-9966M</t>
         </is>
       </c>
       <c r="E92" s="1" t="inlineStr">
         <is>
-          <t>NR72</t>
+          <t>NR71</t>
         </is>
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>Q4003</t>
         </is>
       </c>
       <c r="G92" s="1" t="inlineStr">
         <is>
-          <t>S7003</t>
+          <t>S7002</t>
         </is>
       </c>
       <c r="H92" s="1" t="inlineStr">
         <is>
-          <t>TT128</t>
+          <t>TT127</t>
         </is>
       </c>
     </row>
@@ -4259,37 +4259,37 @@
       </c>
       <c r="B93" s="1" t="inlineStr">
         <is>
-          <t>MM-740M</t>
+          <t>MM-736M</t>
         </is>
       </c>
       <c r="C93" s="1" t="inlineStr">
         <is>
-          <t>MM-948M</t>
+          <t>MM-936M</t>
         </is>
       </c>
       <c r="D93" s="1" t="inlineStr">
         <is>
-          <t>MM-9969M</t>
+          <t>MM-9967M</t>
         </is>
       </c>
       <c r="E93" s="1" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR72</t>
         </is>
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>Q4005</t>
+          <t>Q4004</t>
         </is>
       </c>
       <c r="G93" s="1" t="inlineStr">
         <is>
-          <t>S7005</t>
+          <t>S7003</t>
         </is>
       </c>
       <c r="H93" s="1" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT128</t>
         </is>
       </c>
     </row>
@@ -4301,37 +4301,37 @@
       </c>
       <c r="B94" s="1" t="inlineStr">
         <is>
-          <t>MM-744M</t>
+          <t>MM-740M</t>
         </is>
       </c>
       <c r="C94" s="1" t="inlineStr">
         <is>
-          <t>MM-956M</t>
+          <t>MM-948M</t>
         </is>
       </c>
       <c r="D94" s="1" t="inlineStr">
         <is>
-          <t>MM-9970M</t>
+          <t>MM-9969M</t>
         </is>
       </c>
       <c r="E94" s="1" t="inlineStr">
         <is>
-          <t>NR77</t>
+          <t>NR75</t>
         </is>
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>Q4006</t>
+          <t>Q4005</t>
         </is>
       </c>
       <c r="G94" s="1" t="inlineStr">
         <is>
-          <t>S7006</t>
+          <t>S7005</t>
         </is>
       </c>
       <c r="H94" s="1" t="inlineStr">
         <is>
-          <t>TT131</t>
+          <t>TT130</t>
         </is>
       </c>
     </row>
@@ -4343,37 +4343,37 @@
       </c>
       <c r="B95" s="1" t="inlineStr">
         <is>
-          <t>MM-752M</t>
+          <t>MM-744M</t>
         </is>
       </c>
       <c r="C95" s="1" t="inlineStr">
         <is>
-          <t>MM-962M</t>
+          <t>MM-956M</t>
         </is>
       </c>
       <c r="D95" s="1" t="inlineStr">
         <is>
-          <t>MMY032</t>
+          <t>MM-9970M</t>
         </is>
       </c>
       <c r="E95" s="1" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR77</t>
         </is>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>Q4007</t>
+          <t>Q4006</t>
         </is>
       </c>
       <c r="G95" s="1" t="inlineStr">
         <is>
-          <t>S7007</t>
+          <t>S7006</t>
         </is>
       </c>
       <c r="H95" s="1" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT131</t>
         </is>
       </c>
     </row>
@@ -4385,37 +4385,37 @@
       </c>
       <c r="B96" s="1" t="inlineStr">
         <is>
-          <t>MM-756M</t>
+          <t>MM-752M</t>
         </is>
       </c>
       <c r="C96" s="1" t="inlineStr">
         <is>
-          <t>MM-964M</t>
+          <t>MM-962M</t>
         </is>
       </c>
       <c r="D96" s="1" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MMY032</t>
         </is>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>NR81</t>
+          <t>NR78</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>Q4009</t>
+          <t>Q4007</t>
         </is>
       </c>
       <c r="G96" s="1" t="inlineStr">
         <is>
-          <t>S7012</t>
+          <t>S7007</t>
         </is>
       </c>
       <c r="H96" s="1" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT202</t>
         </is>
       </c>
     </row>
@@ -4427,37 +4427,37 @@
       </c>
       <c r="B97" s="1" t="inlineStr">
         <is>
-          <t>MM-760M</t>
+          <t>MM-756M</t>
         </is>
       </c>
       <c r="C97" s="1" t="inlineStr">
         <is>
-          <t>MM-966M</t>
+          <t>MM-964M</t>
         </is>
       </c>
       <c r="D97" s="1" t="inlineStr">
         <is>
-          <t>MRL004</t>
+          <t>MRL001</t>
         </is>
       </c>
       <c r="E97" s="1" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR81</t>
         </is>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>Q4011</t>
+          <t>Q4009</t>
         </is>
       </c>
       <c r="G97" s="1" t="inlineStr">
         <is>
-          <t>S7014</t>
+          <t>S7012</t>
         </is>
       </c>
       <c r="H97" s="1" t="inlineStr">
         <is>
-          <t>VL352</t>
+          <t>TT206</t>
         </is>
       </c>
     </row>
@@ -4469,37 +4469,37 @@
       </c>
       <c r="B98" s="1" t="inlineStr">
         <is>
-          <t>MM-764M</t>
+          <t>MM-760M</t>
         </is>
       </c>
       <c r="C98" s="1" t="inlineStr">
         <is>
-          <t>MM-970M</t>
+          <t>MM-966M</t>
         </is>
       </c>
       <c r="D98" s="1" t="inlineStr">
         <is>
-          <t>MRL006</t>
+          <t>MRL004</t>
         </is>
       </c>
       <c r="E98" s="1" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR82</t>
         </is>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>Q4011</t>
         </is>
       </c>
       <c r="G98" s="1" t="inlineStr">
         <is>
-          <t>S7020</t>
+          <t>S7014</t>
         </is>
       </c>
       <c r="H98" s="1" t="inlineStr">
         <is>
-          <t>VL353</t>
+          <t>VL352</t>
         </is>
       </c>
     </row>
@@ -4511,37 +4511,37 @@
       </c>
       <c r="B99" s="1" t="inlineStr">
         <is>
-          <t>MM-774M</t>
+          <t>MM-764M</t>
         </is>
       </c>
       <c r="C99" s="1" t="inlineStr">
         <is>
-          <t>MM-972M</t>
+          <t>MM-970M</t>
         </is>
       </c>
       <c r="D99" s="1" t="inlineStr">
         <is>
-          <t>N452</t>
+          <t>MRL006</t>
         </is>
       </c>
       <c r="E99" s="1" t="inlineStr">
         <is>
-          <t>NR84</t>
+          <t>NR83</t>
         </is>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>Q4012</t>
         </is>
       </c>
       <c r="G99" s="1" t="inlineStr">
         <is>
-          <t>S7022</t>
+          <t>S7020</t>
         </is>
       </c>
       <c r="H99" s="1" t="inlineStr">
         <is>
-          <t>VL357</t>
+          <t>VL353</t>
         </is>
       </c>
     </row>
@@ -4553,37 +4553,37 @@
       </c>
       <c r="B100" s="1" t="inlineStr">
         <is>
-          <t>MM-776M</t>
+          <t>MM-774M</t>
         </is>
       </c>
       <c r="C100" s="1" t="inlineStr">
         <is>
-          <t>MM-974M</t>
+          <t>MM-972M</t>
         </is>
       </c>
       <c r="D100" s="1" t="inlineStr">
         <is>
-          <t>N457</t>
+          <t>N452</t>
         </is>
       </c>
       <c r="E100" s="1" t="inlineStr">
         <is>
-          <t>NR85</t>
+          <t>NR84</t>
         </is>
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>Q4014</t>
+          <t>Q4013</t>
         </is>
       </c>
       <c r="G100" s="1" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>S7022</t>
         </is>
       </c>
       <c r="H100" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8004</t>
+          <t>VL357</t>
         </is>
       </c>
     </row>
@@ -4595,37 +4595,37 @@
       </c>
       <c r="B101" s="1" t="inlineStr">
         <is>
-          <t>MM-778M</t>
+          <t>MM-776M</t>
         </is>
       </c>
       <c r="C101" s="1" t="inlineStr">
         <is>
-          <t>MM-980M</t>
+          <t>MM-974M</t>
         </is>
       </c>
       <c r="D101" s="1" t="inlineStr">
         <is>
-          <t>N458</t>
+          <t>N457</t>
         </is>
       </c>
       <c r="E101" s="1" t="inlineStr">
         <is>
-          <t>NR86</t>
+          <t>NR85</t>
         </is>
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>Q4015</t>
+          <t>Q4014</t>
         </is>
       </c>
       <c r="G101" s="1" t="inlineStr">
         <is>
-          <t>SCT002</t>
+          <t>SCT001</t>
         </is>
       </c>
       <c r="H101" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8007</t>
+          <t>VLINE-8004</t>
         </is>
       </c>
     </row>
@@ -4637,37 +4637,37 @@
       </c>
       <c r="B102" s="1" t="inlineStr">
         <is>
-          <t>MM-780M</t>
+          <t>MM-778M</t>
         </is>
       </c>
       <c r="C102" s="1" t="inlineStr">
         <is>
-          <t>MM-982M</t>
+          <t>MM-980M</t>
         </is>
       </c>
       <c r="D102" s="1" t="inlineStr">
         <is>
-          <t>N465</t>
+          <t>N458</t>
         </is>
       </c>
       <c r="E102" s="1" t="inlineStr">
         <is>
-          <t>NR87</t>
+          <t>NR86</t>
         </is>
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>Q4015</t>
         </is>
       </c>
       <c r="G102" s="1" t="inlineStr">
         <is>
-          <t>SCT006</t>
+          <t>SCT002</t>
         </is>
       </c>
       <c r="H102" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8011</t>
+          <t>VLINE-8007</t>
         </is>
       </c>
     </row>
@@ -4679,37 +4679,37 @@
       </c>
       <c r="B103" s="1" t="inlineStr">
         <is>
-          <t>MM-784M</t>
+          <t>MM-780M</t>
         </is>
       </c>
       <c r="C103" s="1" t="inlineStr">
         <is>
-          <t>MM-984M</t>
+          <t>MM-982M</t>
         </is>
       </c>
       <c r="D103" s="1" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>N465</t>
         </is>
       </c>
       <c r="E103" s="1" t="inlineStr">
         <is>
-          <t>NR88</t>
+          <t>NR87</t>
         </is>
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>Q4017</t>
+          <t>Q4016</t>
         </is>
       </c>
       <c r="G103" s="1" t="inlineStr">
         <is>
-          <t>SCT007</t>
+          <t>SCT006</t>
         </is>
       </c>
       <c r="H103" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8013</t>
+          <t>VLINE-8011</t>
         </is>
       </c>
     </row>
@@ -4721,37 +4721,37 @@
       </c>
       <c r="B104" s="1" t="inlineStr">
         <is>
-          <t>MM-790M</t>
+          <t>MM-784M</t>
         </is>
       </c>
       <c r="C104" s="1" t="inlineStr">
         <is>
-          <t>MM-986M</t>
+          <t>MM-984M</t>
         </is>
       </c>
       <c r="D104" s="1" t="inlineStr">
         <is>
-          <t>N467</t>
+          <t>N466</t>
         </is>
       </c>
       <c r="E104" s="1" t="inlineStr">
         <is>
-          <t>NR90</t>
+          <t>NR88</t>
         </is>
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>Q4019</t>
+          <t>Q4017</t>
         </is>
       </c>
       <c r="G104" s="1" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>SCT007</t>
         </is>
       </c>
       <c r="H104" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8019</t>
+          <t>VLINE-8013</t>
         </is>
       </c>
     </row>
@@ -4763,37 +4763,37 @@
       </c>
       <c r="B105" s="1" t="inlineStr">
         <is>
-          <t>MM-792M</t>
+          <t>MM-790M</t>
         </is>
       </c>
       <c r="C105" s="1" t="inlineStr">
         <is>
-          <t>MM-9903M</t>
+          <t>MM-986M</t>
         </is>
       </c>
       <c r="D105" s="1" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>N467</t>
         </is>
       </c>
       <c r="E105" s="1" t="inlineStr">
         <is>
-          <t>NR92</t>
+          <t>NR90</t>
         </is>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>Q4019</t>
         </is>
       </c>
       <c r="G105" s="1" t="inlineStr">
         <is>
-          <t>SCT011</t>
+          <t>SCT009</t>
         </is>
       </c>
       <c r="H105" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8020</t>
+          <t>VLINE-8019</t>
         </is>
       </c>
     </row>
@@ -4805,37 +4805,37 @@
       </c>
       <c r="B106" s="1" t="inlineStr">
         <is>
-          <t>MM-796M</t>
+          <t>MM-792M</t>
         </is>
       </c>
       <c r="C106" s="1" t="inlineStr">
         <is>
-          <t>MM-9904M</t>
+          <t>MM-9903M</t>
         </is>
       </c>
       <c r="D106" s="1" t="inlineStr">
         <is>
-          <t>N473</t>
+          <t>N469</t>
         </is>
       </c>
       <c r="E106" s="1" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR92</t>
         </is>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>QBX003</t>
         </is>
       </c>
       <c r="G106" s="1" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>SCT011</t>
         </is>
       </c>
       <c r="H106" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8023</t>
+          <t>VLINE-8020</t>
         </is>
       </c>
     </row>
@@ -4847,1656 +4847,1661 @@
       </c>
       <c r="B107" s="1" t="inlineStr">
         <is>
-          <t>MM-798M</t>
+          <t>MM-796M</t>
         </is>
       </c>
       <c r="C107" s="1" t="inlineStr">
         <is>
-          <t>MM-9906M</t>
+          <t>MM-9904M</t>
         </is>
       </c>
       <c r="D107" s="1" t="inlineStr">
         <is>
-          <t>NR1</t>
+          <t>N473</t>
         </is>
       </c>
       <c r="E107" s="1" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR93</t>
         </is>
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>QBX005</t>
+          <t>QBX004</t>
         </is>
       </c>
       <c r="G107" s="1" t="inlineStr">
         <is>
-          <t>SCT014</t>
+          <t>SCT013</t>
         </is>
       </c>
       <c r="H107" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8025</t>
+          <t>VLINE-8023</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>MM-282M</t>
+          <t>MM-278M</t>
         </is>
       </c>
       <c r="B108" s="1" t="inlineStr">
         <is>
-          <t>MM-800M</t>
+          <t>MM-798M</t>
         </is>
       </c>
       <c r="C108" s="1" t="inlineStr">
         <is>
-          <t>MM-9907M</t>
+          <t>MM-9906M</t>
         </is>
       </c>
       <c r="D108" s="1" t="inlineStr">
         <is>
-          <t>NR2</t>
+          <t>NR1</t>
         </is>
       </c>
       <c r="E108" s="1" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR94</t>
         </is>
       </c>
       <c r="F108" s="1" t="inlineStr">
         <is>
-          <t>QBX006</t>
+          <t>QBX005</t>
         </is>
       </c>
       <c r="G108" s="1" t="inlineStr">
         <is>
-          <t>SCT015</t>
+          <t>SCT014</t>
         </is>
       </c>
       <c r="H108" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8026</t>
+          <t>VLINE-8025</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>MM-352M</t>
+          <t>MM-282M</t>
         </is>
       </c>
       <c r="B109" s="1" t="inlineStr">
         <is>
-          <t>MM-802M</t>
+          <t>MM-800M</t>
         </is>
       </c>
       <c r="C109" s="1" t="inlineStr">
         <is>
-          <t>MM-9908M</t>
+          <t>MM-9907M</t>
         </is>
       </c>
       <c r="D109" s="1" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>NR2</t>
         </is>
       </c>
       <c r="E109" s="1" t="inlineStr">
         <is>
-          <t>NR96</t>
+          <t>NR95</t>
         </is>
       </c>
       <c r="F109" s="1" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>QBX006</t>
         </is>
       </c>
       <c r="G109" s="1" t="inlineStr">
         <is>
-          <t>SO2</t>
+          <t>SCT015</t>
         </is>
       </c>
       <c r="H109" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8027</t>
+          <t>VLINE-8026</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>MM-372M</t>
+          <t>MM-352M</t>
         </is>
       </c>
       <c r="B110" s="1" t="inlineStr">
         <is>
-          <t>MM-804M</t>
+          <t>MM-802M</t>
         </is>
       </c>
       <c r="C110" s="1" t="inlineStr">
         <is>
-          <t>MM-9909M</t>
+          <t>MM-9908M</t>
         </is>
       </c>
       <c r="D110" s="1" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>NR4</t>
         </is>
       </c>
       <c r="E110" s="1" t="inlineStr">
         <is>
-          <t>NR98</t>
+          <t>NR96</t>
         </is>
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>QE001</t>
         </is>
       </c>
       <c r="G110" s="1" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>SO2</t>
         </is>
       </c>
       <c r="H110" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8028</t>
+          <t>VLINE-8027</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>MM-378M</t>
+          <t>MM-372M</t>
         </is>
       </c>
       <c r="B111" s="1" t="inlineStr">
         <is>
-          <t>MM-808M</t>
+          <t>MM-804M</t>
         </is>
       </c>
       <c r="C111" s="1" t="inlineStr">
         <is>
-          <t>MM-9912M</t>
+          <t>MM-9909M</t>
         </is>
       </c>
       <c r="D111" s="1" t="inlineStr">
         <is>
-          <t>NR7</t>
+          <t>NR5</t>
         </is>
       </c>
       <c r="E111" s="1" t="inlineStr">
         <is>
-          <t>NR99</t>
+          <t>NR98</t>
         </is>
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>QE002</t>
         </is>
       </c>
       <c r="G111" s="1" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>SSR101</t>
         </is>
       </c>
       <c r="H111" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8030</t>
+          <t>VLINE-8028</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>MM-382M</t>
+          <t>MM-378M</t>
         </is>
       </c>
       <c r="B112" s="1" t="inlineStr">
         <is>
-          <t>MM-810M</t>
+          <t>MM-808M</t>
         </is>
       </c>
       <c r="C112" s="1" t="inlineStr">
         <is>
-          <t>MM-9913M</t>
+          <t>MM-9912M</t>
         </is>
       </c>
       <c r="D112" s="1" t="inlineStr">
         <is>
-          <t>NR8</t>
+          <t>NR7</t>
         </is>
       </c>
       <c r="E112" s="1" t="inlineStr">
         <is>
-          <t>NR101</t>
+          <t>NR99</t>
         </is>
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>QE004</t>
+          <t>QE003</t>
         </is>
       </c>
       <c r="G112" s="1" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>SSR102</t>
         </is>
       </c>
       <c r="H112" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8032</t>
+          <t>VLINE-8030</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>MM-392M</t>
+          <t>MM-382M</t>
         </is>
       </c>
       <c r="B113" s="1" t="inlineStr">
         <is>
-          <t>MM-814M</t>
+          <t>MM-810M</t>
         </is>
       </c>
       <c r="C113" s="1" t="inlineStr">
         <is>
-          <t>MM-9914M</t>
+          <t>MM-9913M</t>
         </is>
       </c>
       <c r="D113" s="1" t="inlineStr">
         <is>
-          <t>NR9</t>
+          <t>NR8</t>
         </is>
       </c>
       <c r="E113" s="1" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR101</t>
         </is>
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>QE006</t>
+          <t>QE004</t>
         </is>
       </c>
       <c r="G113" s="1" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>SSR103</t>
         </is>
       </c>
       <c r="H113" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8036</t>
+          <t>VLINE-8032</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8051</t>
+          <t>VLINE-8036</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8182</t>
+          <t>VLINE-8181</t>
         </is>
       </c>
       <c r="C115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8450</t>
+          <t>VLINE-8449</t>
         </is>
       </c>
       <c r="D115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8758</t>
+          <t>VLINE-8757</t>
         </is>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>XP2010</t>
+          <t>XP2008</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8052</t>
+          <t>VLINE-8051</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8183</t>
+          <t>VLINE-8182</t>
         </is>
       </c>
       <c r="C116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8451</t>
+          <t>VLINE-8450</t>
         </is>
       </c>
       <c r="D116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8759</t>
+          <t>VLINE-8758</t>
         </is>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>XP2010</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8053</t>
+          <t>VLINE-8052</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8184</t>
+          <t>VLINE-8183</t>
         </is>
       </c>
       <c r="C117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8452</t>
+          <t>VLINE-8451</t>
         </is>
       </c>
       <c r="D117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8760</t>
+          <t>VLINE-8759</t>
         </is>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>XP2011</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8055</t>
+          <t>VLINE-8053</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8185</t>
+          <t>VLINE-8184</t>
         </is>
       </c>
       <c r="C118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8453</t>
+          <t>VLINE-8452</t>
         </is>
       </c>
       <c r="D118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8761</t>
+          <t>VLINE-8760</t>
         </is>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>XP2012</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8056</t>
+          <t>VLINE-8055</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8186</t>
+          <t>VLINE-8185</t>
         </is>
       </c>
       <c r="C119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8454</t>
+          <t>VLINE-8453</t>
         </is>
       </c>
       <c r="D119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8762</t>
+          <t>VLINE-8761</t>
         </is>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>XP2013</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8057</t>
+          <t>VLINE-8056</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8187</t>
+          <t>VLINE-8186</t>
         </is>
       </c>
       <c r="C120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8455</t>
+          <t>VLINE-8454</t>
         </is>
       </c>
       <c r="D120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8770</t>
+          <t>VLINE-8762</t>
         </is>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>XP2014</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8058</t>
+          <t>VLINE-8057</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8189</t>
+          <t>VLINE-8187</t>
         </is>
       </c>
       <c r="C121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8456</t>
+          <t>VLINE-8455</t>
         </is>
       </c>
       <c r="D121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8772</t>
+          <t>VLINE-8770</t>
         </is>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>XP2016</t>
+          <t>XP2015</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8059</t>
+          <t>VLINE-8058</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8303</t>
+          <t>VLINE-8189</t>
         </is>
       </c>
       <c r="C122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8457</t>
+          <t>VLINE-8456</t>
         </is>
       </c>
       <c r="D122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8774</t>
+          <t>VLINE-8772</t>
         </is>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>XP2017</t>
+          <t>XP2016</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8061</t>
+          <t>VLINE-8059</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8304</t>
+          <t>VLINE-8303</t>
         </is>
       </c>
       <c r="C123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8460</t>
+          <t>VLINE-8457</t>
         </is>
       </c>
       <c r="D123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8776</t>
+          <t>VLINE-8774</t>
         </is>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>XP2017</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8072</t>
+          <t>VLINE-8061</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8306</t>
+          <t>VLINE-8304</t>
         </is>
       </c>
       <c r="C124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8461</t>
+          <t>VLINE-8460</t>
         </is>
       </c>
       <c r="D124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8778</t>
+          <t>VLINE-8776</t>
         </is>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>XR552</t>
+          <t>XP2019</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8074</t>
+          <t>VLINE-8072</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8311</t>
+          <t>VLINE-8306</t>
         </is>
       </c>
       <c r="C125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8464</t>
+          <t>VLINE-8461</t>
         </is>
       </c>
       <c r="D125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8780</t>
+          <t>VLINE-8778</t>
         </is>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>XRN001</t>
+          <t>XR552</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8075</t>
+          <t>VLINE-8074</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8313</t>
+          <t>VLINE-8311</t>
         </is>
       </c>
       <c r="C126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8465</t>
+          <t>VLINE-8464</t>
         </is>
       </c>
       <c r="D126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8793</t>
+          <t>VLINE-8780</t>
         </is>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>XRN004</t>
+          <t>XRN001</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8076</t>
+          <t>VLINE-8075</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8314</t>
+          <t>VLINE-8313</t>
         </is>
       </c>
       <c r="C127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8468</t>
+          <t>VLINE-8465</t>
         </is>
       </c>
       <c r="D127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8795</t>
+          <t>VLINE-8793</t>
         </is>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>XRN004</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8077</t>
+          <t>VLINE-8076</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8316</t>
+          <t>VLINE-8314</t>
         </is>
       </c>
       <c r="C128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8469</t>
+          <t>VLINE-8468</t>
         </is>
       </c>
       <c r="D128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8797</t>
+          <t>VLINE-8795</t>
         </is>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>XRN006</t>
+          <t>XRN005</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8080</t>
+          <t>VLINE-8077</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8318</t>
+          <t>VLINE-8316</t>
         </is>
       </c>
       <c r="C129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8605</t>
+          <t>VLINE-8469</t>
         </is>
       </c>
       <c r="D129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8799</t>
+          <t>VLINE-8797</t>
         </is>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>XRN007</t>
+          <t>XRN006</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8081</t>
+          <t>VLINE-8080</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8321</t>
+          <t>VLINE-8318</t>
         </is>
       </c>
       <c r="C130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8610</t>
+          <t>VLINE-8605</t>
         </is>
       </c>
       <c r="D130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8800</t>
+          <t>VLINE-8799</t>
         </is>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>XRN007</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8084</t>
+          <t>VLINE-8081</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8324</t>
+          <t>VLINE-8321</t>
         </is>
       </c>
       <c r="C131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8612</t>
+          <t>VLINE-8610</t>
         </is>
       </c>
       <c r="D131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8801</t>
+          <t>VLINE-8800</t>
         </is>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>XRN011</t>
+          <t>XRN009</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8088</t>
+          <t>VLINE-8084</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8332</t>
+          <t>VLINE-8324</t>
         </is>
       </c>
       <c r="C132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8615</t>
+          <t>VLINE-8612</t>
         </is>
       </c>
       <c r="D132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8802</t>
+          <t>VLINE-8801</t>
         </is>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>XRN014</t>
+          <t>XRN011</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8089</t>
+          <t>VLINE-8088</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8336</t>
+          <t>VLINE-8332</t>
         </is>
       </c>
       <c r="C133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8620</t>
+          <t>VLINE-8615</t>
         </is>
       </c>
       <c r="D133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8803</t>
+          <t>VLINE-8802</t>
         </is>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>XRN014</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8104</t>
+          <t>VLINE-8089</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8337</t>
+          <t>VLINE-8336</t>
         </is>
       </c>
       <c r="C134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8625</t>
+          <t>VLINE-8620</t>
         </is>
       </c>
       <c r="D134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8804</t>
+          <t>VLINE-8803</t>
         </is>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>XRN017</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8107</t>
+          <t>VLINE-8104</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8338</t>
+          <t>VLINE-8337</t>
         </is>
       </c>
       <c r="C135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8630</t>
+          <t>VLINE-8625</t>
         </is>
       </c>
       <c r="D135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8805</t>
+          <t>VLINE-8804</t>
         </is>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>XRN020</t>
+          <t>XRN018</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8110</t>
+          <t>VLINE-8107</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8339</t>
+          <t>VLINE-8338</t>
         </is>
       </c>
       <c r="C136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8671</t>
+          <t>VLINE-8630</t>
         </is>
       </c>
       <c r="D136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8806</t>
+          <t>VLINE-8805</t>
         </is>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>XRN020</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8111</t>
+          <t>VLINE-8110</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8362</t>
+          <t>VLINE-8339</t>
         </is>
       </c>
       <c r="C137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8706</t>
+          <t>VLINE-8671</t>
         </is>
       </c>
       <c r="D137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8807</t>
+          <t>VLINE-8806</t>
         </is>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>XRN023</t>
+          <t>XRN021</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8113</t>
+          <t>VLINE-8111</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8363</t>
+          <t>VLINE-8362</t>
         </is>
       </c>
       <c r="C138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8711</t>
+          <t>VLINE-8706</t>
         </is>
       </c>
       <c r="D138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8808</t>
+          <t>VLINE-8807</t>
         </is>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>XRN025</t>
+          <t>XRN023</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8114</t>
+          <t>VLINE-8113</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8365</t>
+          <t>VLINE-8363</t>
         </is>
       </c>
       <c r="C139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8714</t>
+          <t>VLINE-8711</t>
         </is>
       </c>
       <c r="D139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8809</t>
+          <t>VLINE-8808</t>
         </is>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>XRN026</t>
+          <t>XRN025</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8115</t>
+          <t>VLINE-8114</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8366</t>
+          <t>VLINE-8365</t>
         </is>
       </c>
       <c r="C140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8717</t>
+          <t>VLINE-8714</t>
         </is>
       </c>
       <c r="D140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8810</t>
+          <t>VLINE-8809</t>
         </is>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>XRN027</t>
+          <t>XRN026</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8119</t>
+          <t>VLINE-8115</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8369</t>
+          <t>VLINE-8366</t>
         </is>
       </c>
       <c r="C141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8720</t>
+          <t>VLINE-8717</t>
         </is>
       </c>
       <c r="D141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8811</t>
+          <t>VLINE-8810</t>
         </is>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>Y163</t>
+          <t>XRN027</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8120</t>
+          <t>VLINE-8119</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8403</t>
+          <t>VLINE-8369</t>
         </is>
       </c>
       <c r="C142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8721</t>
+          <t>VLINE-8720</t>
         </is>
       </c>
       <c r="D142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8812</t>
+          <t>VLINE-8811</t>
+        </is>
+      </c>
+      <c r="E142" s="1" t="inlineStr">
+        <is>
+          <t>Y163</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8121</t>
+          <t>VLINE-8120</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8404</t>
+          <t>VLINE-8403</t>
         </is>
       </c>
       <c r="C143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8723</t>
+          <t>VLINE-8721</t>
         </is>
       </c>
       <c r="D143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8813</t>
+          <t>VLINE-8812</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8124</t>
+          <t>VLINE-8121</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8406</t>
+          <t>VLINE-8404</t>
         </is>
       </c>
       <c r="C144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8725</t>
+          <t>VLINE-8723</t>
         </is>
       </c>
       <c r="D144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8814</t>
+          <t>VLINE-8813</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8126</t>
+          <t>VLINE-8124</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8408</t>
+          <t>VLINE-8406</t>
         </is>
       </c>
       <c r="C145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8726</t>
+          <t>VLINE-8725</t>
         </is>
       </c>
       <c r="D145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8816</t>
+          <t>VLINE-8814</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8127</t>
+          <t>VLINE-8126</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8410</t>
+          <t>VLINE-8408</t>
         </is>
       </c>
       <c r="C146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8727</t>
+          <t>VLINE-8726</t>
         </is>
       </c>
       <c r="D146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8817</t>
+          <t>VLINE-8816</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8128</t>
+          <t>VLINE-8127</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8411</t>
+          <t>VLINE-8410</t>
         </is>
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8729</t>
+          <t>VLINE-8727</t>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8818</t>
+          <t>VLINE-8817</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8129</t>
+          <t>VLINE-8128</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8413</t>
+          <t>VLINE-8411</t>
         </is>
       </c>
       <c r="C148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8730</t>
+          <t>VLINE-8729</t>
         </is>
       </c>
       <c r="D148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8819</t>
+          <t>VLINE-8818</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8132</t>
+          <t>VLINE-8129</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8415</t>
+          <t>VLINE-8413</t>
         </is>
       </c>
       <c r="C149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8731</t>
+          <t>VLINE-8730</t>
         </is>
       </c>
       <c r="D149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8822</t>
+          <t>VLINE-8819</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8134</t>
+          <t>VLINE-8132</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8417</t>
+          <t>VLINE-8415</t>
         </is>
       </c>
       <c r="C150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8733</t>
+          <t>VLINE-8731</t>
         </is>
       </c>
       <c r="D150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8860</t>
+          <t>VLINE-8822</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8136</t>
+          <t>VLINE-8134</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8418</t>
+          <t>VLINE-8417</t>
         </is>
       </c>
       <c r="C151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8735</t>
+          <t>VLINE-8733</t>
         </is>
       </c>
       <c r="D151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8861</t>
+          <t>VLINE-8860</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8145</t>
+          <t>VLINE-8136</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8419</t>
+          <t>VLINE-8418</t>
         </is>
       </c>
       <c r="C152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8736</t>
+          <t>VLINE-8735</t>
         </is>
       </c>
       <c r="D152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8862</t>
+          <t>VLINE-8861</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8148</t>
+          <t>VLINE-8145</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8420</t>
+          <t>VLINE-8419</t>
         </is>
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8737</t>
+          <t>VLINE-8736</t>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8863</t>
+          <t>VLINE-8862</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8150</t>
+          <t>VLINE-8148</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8421</t>
+          <t>VLINE-8420</t>
         </is>
       </c>
       <c r="C154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8739</t>
+          <t>VLINE-8737</t>
         </is>
       </c>
       <c r="D154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8864</t>
+          <t>VLINE-8863</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8151</t>
+          <t>VLINE-8150</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8422</t>
+          <t>VLINE-8421</t>
         </is>
       </c>
       <c r="C155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8740</t>
+          <t>VLINE-8739</t>
         </is>
       </c>
       <c r="D155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8865</t>
+          <t>VLINE-8864</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8152</t>
+          <t>VLINE-8151</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8424</t>
+          <t>VLINE-8422</t>
         </is>
       </c>
       <c r="C156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8741</t>
+          <t>VLINE-8740</t>
         </is>
       </c>
       <c r="D156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8866</t>
+          <t>VLINE-8865</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8153</t>
+          <t>VLINE-8152</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8425</t>
+          <t>VLINE-8424</t>
         </is>
       </c>
       <c r="C157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8742</t>
+          <t>VLINE-8741</t>
         </is>
       </c>
       <c r="D157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8867</t>
+          <t>VLINE-8866</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8154</t>
+          <t>VLINE-8153</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8426</t>
+          <t>VLINE-8425</t>
         </is>
       </c>
       <c r="C158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8743</t>
+          <t>VLINE-8742</t>
         </is>
       </c>
       <c r="D158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8868</t>
+          <t>VLINE-8867</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8155</t>
+          <t>VLINE-8154</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8427</t>
+          <t>VLINE-8426</t>
         </is>
       </c>
       <c r="C159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8744</t>
+          <t>VLINE-8743</t>
         </is>
       </c>
       <c r="D159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8869</t>
+          <t>VLINE-8868</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8157</t>
+          <t>VLINE-8155</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8428</t>
+          <t>VLINE-8427</t>
         </is>
       </c>
       <c r="C160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8745</t>
+          <t>VLINE-8744</t>
         </is>
       </c>
       <c r="D160" s="1" t="inlineStr">
         <is>
-          <t>WH001</t>
+          <t>VLINE-8869</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8158</t>
+          <t>VLINE-8157</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8429</t>
+          <t>VLINE-8428</t>
         </is>
       </c>
       <c r="C161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8746</t>
+          <t>VLINE-8745</t>
         </is>
       </c>
       <c r="D161" s="1" t="inlineStr">
         <is>
-          <t>WH003</t>
+          <t>WH001</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8159</t>
+          <t>VLINE-8158</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8430</t>
+          <t>VLINE-8429</t>
         </is>
       </c>
       <c r="C162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8748</t>
+          <t>VLINE-8746</t>
         </is>
       </c>
       <c r="D162" s="1" t="inlineStr">
         <is>
-          <t>WL02</t>
+          <t>WH003</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8160</t>
+          <t>VLINE-8159</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8432</t>
+          <t>VLINE-8430</t>
         </is>
       </c>
       <c r="C163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8750</t>
+          <t>VLINE-8748</t>
         </is>
       </c>
       <c r="D163" s="1" t="inlineStr">
         <is>
-          <t>X12-X14</t>
+          <t>WL02</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8161</t>
+          <t>VLINE-8160</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8434</t>
+          <t>VLINE-8432</t>
         </is>
       </c>
       <c r="C164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8751</t>
+          <t>VLINE-8750</t>
         </is>
       </c>
       <c r="D164" s="1" t="inlineStr">
         <is>
-          <t>X31</t>
+          <t>X12-X14</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8162</t>
+          <t>VLINE-8161</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8441</t>
+          <t>VLINE-8434</t>
         </is>
       </c>
       <c r="C165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8752</t>
+          <t>VLINE-8751</t>
         </is>
       </c>
       <c r="D165" s="1" t="inlineStr">
         <is>
-          <t>XP2000</t>
+          <t>X31</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8171</t>
+          <t>VLINE-8162</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8443</t>
+          <t>VLINE-8441</t>
         </is>
       </c>
       <c r="C166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8753</t>
+          <t>VLINE-8752</t>
         </is>
       </c>
       <c r="D166" s="1" t="inlineStr">
         <is>
-          <t>XP2003</t>
+          <t>XP2000</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8172</t>
+          <t>VLINE-8171</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8444</t>
+          <t>VLINE-8443</t>
         </is>
       </c>
       <c r="C167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8754</t>
+          <t>VLINE-8753</t>
         </is>
       </c>
       <c r="D167" s="1" t="inlineStr">
         <is>
-          <t>XP2004</t>
+          <t>XP2003</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8179</t>
+          <t>VLINE-8172</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8446</t>
+          <t>VLINE-8444</t>
         </is>
       </c>
       <c r="C168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8755</t>
+          <t>VLINE-8754</t>
         </is>
       </c>
       <c r="D168" s="1" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>XP2004</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8180</t>
+          <t>VLINE-8179</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8447</t>
+          <t>VLINE-8446</t>
         </is>
       </c>
       <c r="C169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8756</t>
+          <t>VLINE-8755</t>
         </is>
       </c>
       <c r="D169" s="1" t="inlineStr">
         <is>
-          <t>XP2007</t>
+          <t>XP2005</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8181</t>
+          <t>VLINE-8180</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8449</t>
+          <t>VLINE-8447</t>
         </is>
       </c>
       <c r="C170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8757</t>
+          <t>VLINE-8756</t>
         </is>
       </c>
       <c r="D170" s="1" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>XP2007</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update trains and loco export 2026-04-05 11:21:09
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -2799,27 +2799,27 @@
       </c>
       <c r="D58" s="1" t="inlineStr">
         <is>
-          <t>MM-796M</t>
+          <t>MM-792M</t>
         </is>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>MM-972M</t>
+          <t>MM-970M</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MMY032</t>
         </is>
       </c>
       <c r="G58" s="1" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR72</t>
         </is>
       </c>
       <c r="H58" s="1" t="inlineStr">
         <is>
-          <t>PHC002</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
@@ -2841,27 +2841,27 @@
       </c>
       <c r="D59" s="1" t="inlineStr">
         <is>
-          <t>MM-798M</t>
+          <t>MM-796M</t>
         </is>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>MM-974M</t>
+          <t>MM-972M</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>MRL004</t>
+          <t>MRL001</t>
         </is>
       </c>
       <c r="G59" s="1" t="inlineStr">
         <is>
-          <t>NR77</t>
+          <t>NR75</t>
         </is>
       </c>
       <c r="H59" s="1" t="inlineStr">
         <is>
-          <t>Q4001</t>
+          <t>PHC002</t>
         </is>
       </c>
     </row>
@@ -2883,27 +2883,27 @@
       </c>
       <c r="D60" s="1" t="inlineStr">
         <is>
-          <t>MM-800M</t>
+          <t>MM-798M</t>
         </is>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>MM-976M</t>
+          <t>MM-974M</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>MRL006</t>
+          <t>MRL004</t>
         </is>
       </c>
       <c r="G60" s="1" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR77</t>
         </is>
       </c>
       <c r="H60" s="1" t="inlineStr">
         <is>
-          <t>Q4003</t>
+          <t>Q4001</t>
         </is>
       </c>
     </row>
@@ -2925,27 +2925,27 @@
       </c>
       <c r="D61" s="1" t="inlineStr">
         <is>
-          <t>MM-802M</t>
+          <t>MM-800M</t>
         </is>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>MM-980M</t>
+          <t>MM-976M</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>N452</t>
+          <t>MRL006</t>
         </is>
       </c>
       <c r="G61" s="1" t="inlineStr">
         <is>
-          <t>NR81</t>
+          <t>NR78</t>
         </is>
       </c>
       <c r="H61" s="1" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>Q4003</t>
         </is>
       </c>
     </row>
@@ -2967,27 +2967,27 @@
       </c>
       <c r="D62" s="1" t="inlineStr">
         <is>
-          <t>MM-804M</t>
+          <t>MM-802M</t>
         </is>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>MM-982M</t>
+          <t>MM-980M</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>N453</t>
+          <t>N452</t>
         </is>
       </c>
       <c r="G62" s="1" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR81</t>
         </is>
       </c>
       <c r="H62" s="1" t="inlineStr">
         <is>
-          <t>Q4005</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
@@ -3009,27 +3009,27 @@
       </c>
       <c r="D63" s="1" t="inlineStr">
         <is>
-          <t>MM-808M</t>
+          <t>MM-804M</t>
         </is>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>MM-984M</t>
+          <t>MM-982M</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>N457</t>
+          <t>N453</t>
         </is>
       </c>
       <c r="G63" s="1" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR82</t>
         </is>
       </c>
       <c r="H63" s="1" t="inlineStr">
         <is>
-          <t>Q4006</t>
+          <t>Q4005</t>
         </is>
       </c>
     </row>
@@ -3051,27 +3051,27 @@
       </c>
       <c r="D64" s="1" t="inlineStr">
         <is>
-          <t>MM-810M</t>
+          <t>MM-808M</t>
         </is>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>MM-986M</t>
+          <t>MM-984M</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>N458</t>
+          <t>N457</t>
         </is>
       </c>
       <c r="G64" s="1" t="inlineStr">
         <is>
-          <t>NR84</t>
+          <t>NR83</t>
         </is>
       </c>
       <c r="H64" s="1" t="inlineStr">
         <is>
-          <t>Q4007</t>
+          <t>Q4006</t>
         </is>
       </c>
     </row>
@@ -3093,27 +3093,27 @@
       </c>
       <c r="D65" s="1" t="inlineStr">
         <is>
-          <t>MM-814M</t>
+          <t>MM-810M</t>
         </is>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>MM-9902M</t>
+          <t>MM-986M</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>N465</t>
+          <t>N458</t>
         </is>
       </c>
       <c r="G65" s="1" t="inlineStr">
         <is>
-          <t>NR85</t>
+          <t>NR84</t>
         </is>
       </c>
       <c r="H65" s="1" t="inlineStr">
         <is>
-          <t>Q4009</t>
+          <t>Q4007</t>
         </is>
       </c>
     </row>
@@ -3135,27 +3135,27 @@
       </c>
       <c r="D66" s="1" t="inlineStr">
         <is>
-          <t>MM-816M</t>
+          <t>MM-814M</t>
         </is>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>MM-9903M</t>
+          <t>MM-9902M</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>N465</t>
         </is>
       </c>
       <c r="G66" s="1" t="inlineStr">
         <is>
-          <t>NR86</t>
+          <t>NR85</t>
         </is>
       </c>
       <c r="H66" s="1" t="inlineStr">
         <is>
-          <t>Q4011</t>
+          <t>Q4009</t>
         </is>
       </c>
     </row>
@@ -3177,27 +3177,27 @@
       </c>
       <c r="D67" s="1" t="inlineStr">
         <is>
-          <t>MM-818M</t>
+          <t>MM-816M</t>
         </is>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>MM-9904M</t>
+          <t>MM-9903M</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>N467</t>
+          <t>N466</t>
         </is>
       </c>
       <c r="G67" s="1" t="inlineStr">
         <is>
-          <t>NR87</t>
+          <t>NR86</t>
         </is>
       </c>
       <c r="H67" s="1" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>Q4011</t>
         </is>
       </c>
     </row>
@@ -3219,27 +3219,27 @@
       </c>
       <c r="D68" s="1" t="inlineStr">
         <is>
-          <t>MM-820M</t>
+          <t>MM-818M</t>
         </is>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>MM-9906M</t>
+          <t>MM-9904M</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>N467</t>
         </is>
       </c>
       <c r="G68" s="1" t="inlineStr">
         <is>
-          <t>NR88</t>
+          <t>NR87</t>
         </is>
       </c>
       <c r="H68" s="1" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
@@ -3261,27 +3261,27 @@
       </c>
       <c r="D69" s="1" t="inlineStr">
         <is>
-          <t>MM-824M</t>
+          <t>MM-820M</t>
         </is>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>MM-9907M</t>
+          <t>MM-9906M</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>N473</t>
+          <t>N469</t>
         </is>
       </c>
       <c r="G69" s="1" t="inlineStr">
         <is>
-          <t>NR89</t>
+          <t>NR88</t>
         </is>
       </c>
       <c r="H69" s="1" t="inlineStr">
         <is>
-          <t>Q4014</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
@@ -3303,27 +3303,27 @@
       </c>
       <c r="D70" s="1" t="inlineStr">
         <is>
-          <t>MM-826M</t>
+          <t>MM-824M</t>
         </is>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>MM-9908M</t>
+          <t>MM-9907M</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>NR1</t>
+          <t>N473</t>
         </is>
       </c>
       <c r="G70" s="1" t="inlineStr">
         <is>
-          <t>NR90</t>
+          <t>NR89</t>
         </is>
       </c>
       <c r="H70" s="1" t="inlineStr">
         <is>
-          <t>Q4015</t>
+          <t>Q4014</t>
         </is>
       </c>
     </row>
@@ -3345,27 +3345,27 @@
       </c>
       <c r="D71" s="1" t="inlineStr">
         <is>
-          <t>MM-828M</t>
+          <t>MM-826M</t>
         </is>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>MM-9909M</t>
+          <t>MM-9908M</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>NR2</t>
+          <t>NR1</t>
         </is>
       </c>
       <c r="G71" s="1" t="inlineStr">
         <is>
-          <t>NR91</t>
+          <t>NR90</t>
         </is>
       </c>
       <c r="H71" s="1" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>Q4015</t>
         </is>
       </c>
     </row>
@@ -3382,32 +3382,32 @@
       </c>
       <c r="C72" s="1" t="inlineStr">
         <is>
-          <t>MM-588M</t>
+          <t>MM-580M</t>
         </is>
       </c>
       <c r="D72" s="1" t="inlineStr">
         <is>
-          <t>MM-830M</t>
+          <t>MM-828M</t>
         </is>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>MM-9912M</t>
+          <t>MM-9909M</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>NR2</t>
         </is>
       </c>
       <c r="G72" s="1" t="inlineStr">
         <is>
-          <t>NR92</t>
+          <t>NR91</t>
         </is>
       </c>
       <c r="H72" s="1" t="inlineStr">
         <is>
-          <t>Q4017</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
@@ -3424,32 +3424,32 @@
       </c>
       <c r="C73" s="1" t="inlineStr">
         <is>
-          <t>MM-602M</t>
+          <t>MM-588M</t>
         </is>
       </c>
       <c r="D73" s="1" t="inlineStr">
         <is>
-          <t>MM-832M</t>
+          <t>MM-830M</t>
         </is>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>MM-9913M</t>
+          <t>MM-9912M</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>NR4</t>
         </is>
       </c>
       <c r="G73" s="1" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR92</t>
         </is>
       </c>
       <c r="H73" s="1" t="inlineStr">
         <is>
-          <t>Q4019</t>
+          <t>Q4017</t>
         </is>
       </c>
     </row>
@@ -3466,32 +3466,32 @@
       </c>
       <c r="C74" s="1" t="inlineStr">
         <is>
-          <t>MM-616M</t>
+          <t>MM-602M</t>
         </is>
       </c>
       <c r="D74" s="1" t="inlineStr">
         <is>
-          <t>MM-834M</t>
+          <t>MM-832M</t>
         </is>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>MM-9914M</t>
+          <t>MM-9913M</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>NR7</t>
+          <t>NR5</t>
         </is>
       </c>
       <c r="G74" s="1" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR93</t>
         </is>
       </c>
       <c r="H74" s="1" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>Q4019</t>
         </is>
       </c>
     </row>
@@ -3508,32 +3508,32 @@
       </c>
       <c r="C75" s="1" t="inlineStr">
         <is>
-          <t>MM-624M</t>
+          <t>MM-616M</t>
         </is>
       </c>
       <c r="D75" s="1" t="inlineStr">
         <is>
-          <t>MM-838M</t>
+          <t>MM-834M</t>
         </is>
       </c>
       <c r="E75" s="1" t="inlineStr">
         <is>
-          <t>MM-9915M</t>
+          <t>MM-9914M</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>NR8</t>
+          <t>NR7</t>
         </is>
       </c>
       <c r="G75" s="1" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR94</t>
         </is>
       </c>
       <c r="H75" s="1" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
@@ -3550,32 +3550,32 @@
       </c>
       <c r="C76" s="1" t="inlineStr">
         <is>
-          <t>MM-632M</t>
+          <t>MM-624M</t>
         </is>
       </c>
       <c r="D76" s="1" t="inlineStr">
         <is>
-          <t>MM-842M</t>
+          <t>MM-838M</t>
         </is>
       </c>
       <c r="E76" s="1" t="inlineStr">
         <is>
-          <t>MM-9917M</t>
+          <t>MM-9915M</t>
         </is>
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>NR9</t>
+          <t>NR8</t>
         </is>
       </c>
       <c r="G76" s="1" t="inlineStr">
         <is>
-          <t>NR96</t>
+          <t>NR95</t>
         </is>
       </c>
       <c r="H76" s="1" t="inlineStr">
         <is>
-          <t>QBX005</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
@@ -3592,32 +3592,32 @@
       </c>
       <c r="C77" s="1" t="inlineStr">
         <is>
-          <t>MM-636M</t>
+          <t>MM-632M</t>
         </is>
       </c>
       <c r="D77" s="1" t="inlineStr">
         <is>
-          <t>MM-844M</t>
+          <t>MM-842M</t>
         </is>
       </c>
       <c r="E77" s="1" t="inlineStr">
         <is>
-          <t>MM-9918M</t>
+          <t>MM-9917M</t>
         </is>
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
-          <t>NR12</t>
+          <t>NR9</t>
         </is>
       </c>
       <c r="G77" s="1" t="inlineStr">
         <is>
-          <t>NR98</t>
+          <t>NR96</t>
         </is>
       </c>
       <c r="H77" s="1" t="inlineStr">
         <is>
-          <t>QBX006</t>
+          <t>QBX005</t>
         </is>
       </c>
     </row>
@@ -3634,32 +3634,32 @@
       </c>
       <c r="C78" s="1" t="inlineStr">
         <is>
-          <t>MM-640M</t>
+          <t>MM-636M</t>
         </is>
       </c>
       <c r="D78" s="1" t="inlineStr">
         <is>
-          <t>MM-852M</t>
+          <t>MM-844M</t>
         </is>
       </c>
       <c r="E78" s="1" t="inlineStr">
         <is>
-          <t>MM-9919M</t>
+          <t>MM-9918M</t>
         </is>
       </c>
       <c r="F78" s="1" t="inlineStr">
         <is>
-          <t>NR15</t>
+          <t>NR12</t>
         </is>
       </c>
       <c r="G78" s="1" t="inlineStr">
         <is>
-          <t>NR99</t>
+          <t>NR98</t>
         </is>
       </c>
       <c r="H78" s="1" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>QBX006</t>
         </is>
       </c>
     </row>
@@ -3676,32 +3676,32 @@
       </c>
       <c r="C79" s="1" t="inlineStr">
         <is>
-          <t>MM-654M</t>
+          <t>MM-640M</t>
         </is>
       </c>
       <c r="D79" s="1" t="inlineStr">
         <is>
-          <t>MM-858M</t>
+          <t>MM-852M</t>
         </is>
       </c>
       <c r="E79" s="1" t="inlineStr">
         <is>
-          <t>MM-9920M</t>
+          <t>MM-9919M</t>
         </is>
       </c>
       <c r="F79" s="1" t="inlineStr">
         <is>
-          <t>NR16</t>
+          <t>NR15</t>
         </is>
       </c>
       <c r="G79" s="1" t="inlineStr">
         <is>
-          <t>NR101</t>
+          <t>NR99</t>
         </is>
       </c>
       <c r="H79" s="1" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>QE001</t>
         </is>
       </c>
     </row>
@@ -3718,32 +3718,32 @@
       </c>
       <c r="C80" s="1" t="inlineStr">
         <is>
-          <t>MM-656M</t>
+          <t>MM-654M</t>
         </is>
       </c>
       <c r="D80" s="1" t="inlineStr">
         <is>
-          <t>MM-860M</t>
+          <t>MM-858M</t>
         </is>
       </c>
       <c r="E80" s="1" t="inlineStr">
         <is>
-          <t>MM-9922M</t>
+          <t>MM-9920M</t>
         </is>
       </c>
       <c r="F80" s="1" t="inlineStr">
         <is>
-          <t>NR18</t>
+          <t>NR16</t>
         </is>
       </c>
       <c r="G80" s="1" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR101</t>
         </is>
       </c>
       <c r="H80" s="1" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
@@ -3760,32 +3760,32 @@
       </c>
       <c r="C81" s="1" t="inlineStr">
         <is>
-          <t>MM-660M</t>
+          <t>MM-656M</t>
         </is>
       </c>
       <c r="D81" s="1" t="inlineStr">
         <is>
-          <t>MM-862M</t>
+          <t>MM-860M</t>
         </is>
       </c>
       <c r="E81" s="1" t="inlineStr">
         <is>
-          <t>MM-9923M</t>
+          <t>MM-9922M</t>
         </is>
       </c>
       <c r="F81" s="1" t="inlineStr">
         <is>
-          <t>NR19</t>
+          <t>NR18</t>
         </is>
       </c>
       <c r="G81" s="1" t="inlineStr">
         <is>
-          <t>NR103</t>
+          <t>NR102</t>
         </is>
       </c>
       <c r="H81" s="1" t="inlineStr">
         <is>
-          <t>QE004</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
@@ -3802,32 +3802,32 @@
       </c>
       <c r="C82" s="1" t="inlineStr">
         <is>
-          <t>MM-661M</t>
+          <t>MM-660M</t>
         </is>
       </c>
       <c r="D82" s="1" t="inlineStr">
         <is>
-          <t>MM-868M</t>
+          <t>MM-862M</t>
         </is>
       </c>
       <c r="E82" s="1" t="inlineStr">
         <is>
-          <t>MM-9924M</t>
+          <t>MM-9923M</t>
         </is>
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
-          <t>NR21</t>
+          <t>NR19</t>
         </is>
       </c>
       <c r="G82" s="1" t="inlineStr">
         <is>
-          <t>NR105</t>
+          <t>NR103</t>
         </is>
       </c>
       <c r="H82" s="1" t="inlineStr">
         <is>
-          <t>QE006</t>
+          <t>QE004</t>
         </is>
       </c>
     </row>
@@ -3844,32 +3844,32 @@
       </c>
       <c r="C83" s="1" t="inlineStr">
         <is>
-          <t>MM-662M</t>
+          <t>MM-661M</t>
         </is>
       </c>
       <c r="D83" s="1" t="inlineStr">
         <is>
-          <t>MM-872M</t>
+          <t>MM-868M</t>
         </is>
       </c>
       <c r="E83" s="1" t="inlineStr">
         <is>
-          <t>MM-9926M</t>
+          <t>MM-9924M</t>
         </is>
       </c>
       <c r="F83" s="1" t="inlineStr">
         <is>
-          <t>NR25</t>
+          <t>NR21</t>
         </is>
       </c>
       <c r="G83" s="1" t="inlineStr">
         <is>
-          <t>NR108</t>
+          <t>NR105</t>
         </is>
       </c>
       <c r="H83" s="1" t="inlineStr">
         <is>
-          <t>QL001</t>
+          <t>QE006</t>
         </is>
       </c>
     </row>
@@ -3886,32 +3886,32 @@
       </c>
       <c r="C84" s="1" t="inlineStr">
         <is>
-          <t>MM-664M</t>
+          <t>MM-662M</t>
         </is>
       </c>
       <c r="D84" s="1" t="inlineStr">
         <is>
-          <t>MM-874M</t>
+          <t>MM-872M</t>
         </is>
       </c>
       <c r="E84" s="1" t="inlineStr">
         <is>
-          <t>MM-9928M</t>
+          <t>MM-9926M</t>
         </is>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>NR27</t>
+          <t>NR25</t>
         </is>
       </c>
       <c r="G84" s="1" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR108</t>
         </is>
       </c>
       <c r="H84" s="1" t="inlineStr">
         <is>
-          <t>QL002</t>
+          <t>QL001</t>
         </is>
       </c>
     </row>
@@ -3928,32 +3928,32 @@
       </c>
       <c r="C85" s="1" t="inlineStr">
         <is>
-          <t>MM-666M</t>
+          <t>MM-664M</t>
         </is>
       </c>
       <c r="D85" s="1" t="inlineStr">
         <is>
-          <t>MM-876M</t>
+          <t>MM-874M</t>
         </is>
       </c>
       <c r="E85" s="1" t="inlineStr">
         <is>
-          <t>MM-9929M</t>
+          <t>MM-9928M</t>
         </is>
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>NR28</t>
+          <t>NR27</t>
         </is>
       </c>
       <c r="G85" s="1" t="inlineStr">
         <is>
-          <t>NR110</t>
+          <t>NR109</t>
         </is>
       </c>
       <c r="H85" s="1" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>QL002</t>
         </is>
       </c>
     </row>
@@ -3970,32 +3970,32 @@
       </c>
       <c r="C86" s="1" t="inlineStr">
         <is>
-          <t>MM-668M</t>
+          <t>MM-666M</t>
         </is>
       </c>
       <c r="D86" s="1" t="inlineStr">
         <is>
-          <t>MM-882M</t>
+          <t>MM-876M</t>
         </is>
       </c>
       <c r="E86" s="1" t="inlineStr">
         <is>
-          <t>MM-9932M</t>
+          <t>MM-9929M</t>
         </is>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>NR30</t>
+          <t>NR28</t>
         </is>
       </c>
       <c r="G86" s="1" t="inlineStr">
         <is>
-          <t>NR111</t>
+          <t>NR110</t>
         </is>
       </c>
       <c r="H86" s="1" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>QL004</t>
         </is>
       </c>
     </row>
@@ -4012,32 +4012,32 @@
       </c>
       <c r="C87" s="1" t="inlineStr">
         <is>
-          <t>MM-673M</t>
+          <t>MM-668M</t>
         </is>
       </c>
       <c r="D87" s="1" t="inlineStr">
         <is>
-          <t>MM-894M</t>
+          <t>MM-882M</t>
         </is>
       </c>
       <c r="E87" s="1" t="inlineStr">
         <is>
-          <t>MM-9933M</t>
+          <t>MM-9932M</t>
         </is>
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>NR31</t>
+          <t>NR30</t>
         </is>
       </c>
       <c r="G87" s="1" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR111</t>
         </is>
       </c>
       <c r="H87" s="1" t="inlineStr">
         <is>
-          <t>QL008</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
@@ -4054,32 +4054,32 @@
       </c>
       <c r="C88" s="1" t="inlineStr">
         <is>
-          <t>MM-674M</t>
+          <t>MM-673M</t>
         </is>
       </c>
       <c r="D88" s="1" t="inlineStr">
         <is>
-          <t>MM-896M</t>
+          <t>MM-894M</t>
         </is>
       </c>
       <c r="E88" s="1" t="inlineStr">
         <is>
-          <t>MM-9934M</t>
+          <t>MM-9933M</t>
         </is>
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>NR34</t>
+          <t>NR31</t>
         </is>
       </c>
       <c r="G88" s="1" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR112</t>
         </is>
       </c>
       <c r="H88" s="1" t="inlineStr">
         <is>
-          <t>QL010</t>
+          <t>QL008</t>
         </is>
       </c>
     </row>
@@ -4096,32 +4096,32 @@
       </c>
       <c r="C89" s="1" t="inlineStr">
         <is>
-          <t>MM-680M</t>
+          <t>MM-674M</t>
         </is>
       </c>
       <c r="D89" s="1" t="inlineStr">
         <is>
-          <t>MM-902M</t>
+          <t>MM-896M</t>
         </is>
       </c>
       <c r="E89" s="1" t="inlineStr">
         <is>
-          <t>MM-9936M</t>
+          <t>MM-9934M</t>
         </is>
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>NR36</t>
+          <t>NR34</t>
         </is>
       </c>
       <c r="G89" s="1" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR113</t>
         </is>
       </c>
       <c r="H89" s="1" t="inlineStr">
         <is>
-          <t>QL011</t>
+          <t>QL010</t>
         </is>
       </c>
     </row>
@@ -4138,32 +4138,32 @@
       </c>
       <c r="C90" s="1" t="inlineStr">
         <is>
-          <t>MM-708M</t>
+          <t>MM-680M</t>
         </is>
       </c>
       <c r="D90" s="1" t="inlineStr">
         <is>
-          <t>MM-904M</t>
+          <t>MM-902M</t>
         </is>
       </c>
       <c r="E90" s="1" t="inlineStr">
         <is>
-          <t>MM-9938M</t>
+          <t>MM-9936M</t>
         </is>
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>NR36</t>
         </is>
       </c>
       <c r="G90" s="1" t="inlineStr">
         <is>
-          <t>NR118</t>
+          <t>NR115</t>
         </is>
       </c>
       <c r="H90" s="1" t="inlineStr">
         <is>
-          <t>QL014</t>
+          <t>QL011</t>
         </is>
       </c>
     </row>
@@ -4180,32 +4180,32 @@
       </c>
       <c r="C91" s="1" t="inlineStr">
         <is>
-          <t>MM-710M</t>
+          <t>MM-708M</t>
         </is>
       </c>
       <c r="D91" s="1" t="inlineStr">
         <is>
-          <t>MM-906M</t>
+          <t>MM-904M</t>
         </is>
       </c>
       <c r="E91" s="1" t="inlineStr">
         <is>
-          <t>MM-9941M</t>
+          <t>MM-9938M</t>
         </is>
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>NR38</t>
+          <t>NR37</t>
         </is>
       </c>
       <c r="G91" s="1" t="inlineStr">
         <is>
-          <t>NR119</t>
+          <t>NR118</t>
         </is>
       </c>
       <c r="H91" s="1" t="inlineStr">
         <is>
-          <t>QL018</t>
+          <t>QL014</t>
         </is>
       </c>
     </row>
@@ -4222,32 +4222,32 @@
       </c>
       <c r="C92" s="1" t="inlineStr">
         <is>
-          <t>MM-716M</t>
+          <t>MM-710M</t>
         </is>
       </c>
       <c r="D92" s="1" t="inlineStr">
         <is>
-          <t>MM-908M</t>
+          <t>MM-906M</t>
         </is>
       </c>
       <c r="E92" s="1" t="inlineStr">
         <is>
-          <t>MM-9943M</t>
+          <t>MM-9941M</t>
         </is>
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>NR39</t>
+          <t>NR38</t>
         </is>
       </c>
       <c r="G92" s="1" t="inlineStr">
         <is>
-          <t>NR120</t>
+          <t>NR119</t>
         </is>
       </c>
       <c r="H92" s="1" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QL018</t>
         </is>
       </c>
     </row>
@@ -4264,32 +4264,32 @@
       </c>
       <c r="C93" s="1" t="inlineStr">
         <is>
-          <t>MM-722M</t>
+          <t>MM-716M</t>
         </is>
       </c>
       <c r="D93" s="1" t="inlineStr">
         <is>
-          <t>MM-910M</t>
+          <t>MM-908M</t>
         </is>
       </c>
       <c r="E93" s="1" t="inlineStr">
         <is>
-          <t>MM-9945M</t>
+          <t>MM-9943M</t>
         </is>
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>NR40</t>
+          <t>NR39</t>
         </is>
       </c>
       <c r="G93" s="1" t="inlineStr">
         <is>
-          <t>NR122</t>
+          <t>NR120</t>
         </is>
       </c>
       <c r="H93" s="1" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QR1744</t>
         </is>
       </c>
     </row>
@@ -4306,32 +4306,32 @@
       </c>
       <c r="C94" s="1" t="inlineStr">
         <is>
-          <t>MM-726M</t>
+          <t>MM-722M</t>
         </is>
       </c>
       <c r="D94" s="1" t="inlineStr">
         <is>
-          <t>MM-912M</t>
+          <t>MM-910M</t>
         </is>
       </c>
       <c r="E94" s="1" t="inlineStr">
         <is>
-          <t>MM-9946M</t>
+          <t>MM-9945M</t>
         </is>
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>NR43</t>
+          <t>NR40</t>
         </is>
       </c>
       <c r="G94" s="1" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>NR122</t>
         </is>
       </c>
       <c r="H94" s="1" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QR1771</t>
         </is>
       </c>
     </row>
@@ -4348,32 +4348,32 @@
       </c>
       <c r="C95" s="1" t="inlineStr">
         <is>
-          <t>MM-728M</t>
+          <t>MM-726M</t>
         </is>
       </c>
       <c r="D95" s="1" t="inlineStr">
         <is>
-          <t>MM-914M</t>
+          <t>MM-912M</t>
         </is>
       </c>
       <c r="E95" s="1" t="inlineStr">
         <is>
-          <t>MM-9950M</t>
+          <t>MM-9946M</t>
         </is>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>NR44</t>
+          <t>NR43</t>
         </is>
       </c>
       <c r="G95" s="1" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="H95" s="1" t="inlineStr">
         <is>
-          <t>R711</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
@@ -4390,32 +4390,32 @@
       </c>
       <c r="C96" s="1" t="inlineStr">
         <is>
-          <t>MM-734M</t>
+          <t>MM-728M</t>
         </is>
       </c>
       <c r="D96" s="1" t="inlineStr">
         <is>
-          <t>MM-920M</t>
+          <t>MM-914M</t>
         </is>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>MM-9951M</t>
+          <t>MM-9950M</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>NR45</t>
+          <t>NR44</t>
         </is>
       </c>
       <c r="G96" s="1" t="inlineStr">
         <is>
-          <t>P2501</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="H96" s="1" t="inlineStr">
         <is>
-          <t>R766</t>
+          <t>R711</t>
         </is>
       </c>
     </row>
@@ -4432,32 +4432,32 @@
       </c>
       <c r="C97" s="1" t="inlineStr">
         <is>
-          <t>MM-736M</t>
+          <t>MM-734M</t>
         </is>
       </c>
       <c r="D97" s="1" t="inlineStr">
         <is>
-          <t>MM-922M</t>
+          <t>MM-920M</t>
         </is>
       </c>
       <c r="E97" s="1" t="inlineStr">
         <is>
-          <t>MM-9952M</t>
+          <t>MM-9951M</t>
         </is>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>NR48</t>
+          <t>NR45</t>
         </is>
       </c>
       <c r="G97" s="1" t="inlineStr">
         <is>
-          <t>P2502</t>
+          <t>P2501</t>
         </is>
       </c>
       <c r="H97" s="1" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>R766</t>
         </is>
       </c>
     </row>
@@ -4474,32 +4474,32 @@
       </c>
       <c r="C98" s="1" t="inlineStr">
         <is>
-          <t>MM-738M</t>
+          <t>MM-736M</t>
         </is>
       </c>
       <c r="D98" s="1" t="inlineStr">
         <is>
-          <t>MM-924M</t>
+          <t>MM-922M</t>
         </is>
       </c>
       <c r="E98" s="1" t="inlineStr">
         <is>
-          <t>MM-9953M</t>
+          <t>MM-9952M</t>
         </is>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>NR51</t>
+          <t>NR48</t>
         </is>
       </c>
       <c r="G98" s="1" t="inlineStr">
         <is>
-          <t>P2503</t>
+          <t>P2502</t>
         </is>
       </c>
       <c r="H98" s="1" t="inlineStr">
         <is>
-          <t>RCTST4</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
@@ -4516,32 +4516,32 @@
       </c>
       <c r="C99" s="1" t="inlineStr">
         <is>
-          <t>MM-740M</t>
+          <t>MM-738M</t>
         </is>
       </c>
       <c r="D99" s="1" t="inlineStr">
         <is>
-          <t>MM-926M</t>
+          <t>MM-924M</t>
         </is>
       </c>
       <c r="E99" s="1" t="inlineStr">
         <is>
-          <t>MM-9954M</t>
+          <t>MM-9953M</t>
         </is>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>NR52</t>
+          <t>NR51</t>
         </is>
       </c>
       <c r="G99" s="1" t="inlineStr">
         <is>
-          <t>P2505</t>
+          <t>P2503</t>
         </is>
       </c>
       <c r="H99" s="1" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>RCTST4</t>
         </is>
       </c>
     </row>
@@ -4558,32 +4558,32 @@
       </c>
       <c r="C100" s="1" t="inlineStr">
         <is>
-          <t>MM-742M</t>
+          <t>MM-740M</t>
         </is>
       </c>
       <c r="D100" s="1" t="inlineStr">
         <is>
-          <t>MM-934M</t>
+          <t>MM-926M</t>
         </is>
       </c>
       <c r="E100" s="1" t="inlineStr">
         <is>
-          <t>MM-9955M</t>
+          <t>MM-9954M</t>
         </is>
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>NR53</t>
+          <t>NR52</t>
         </is>
       </c>
       <c r="G100" s="1" t="inlineStr">
         <is>
-          <t>P2506</t>
+          <t>P2505</t>
         </is>
       </c>
       <c r="H100" s="1" t="inlineStr">
         <is>
-          <t>RL302</t>
+          <t>RL301</t>
         </is>
       </c>
     </row>
@@ -4600,32 +4600,32 @@
       </c>
       <c r="C101" s="1" t="inlineStr">
         <is>
-          <t>MM-744M</t>
+          <t>MM-742M</t>
         </is>
       </c>
       <c r="D101" s="1" t="inlineStr">
         <is>
-          <t>MM-936M</t>
+          <t>MM-934M</t>
         </is>
       </c>
       <c r="E101" s="1" t="inlineStr">
         <is>
-          <t>MM-9957M</t>
+          <t>MM-9955M</t>
         </is>
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>NR53</t>
         </is>
       </c>
       <c r="G101" s="1" t="inlineStr">
         <is>
-          <t>P2507</t>
+          <t>P2506</t>
         </is>
       </c>
       <c r="H101" s="1" t="inlineStr">
         <is>
-          <t>RL304</t>
+          <t>RL302</t>
         </is>
       </c>
     </row>
@@ -4642,32 +4642,32 @@
       </c>
       <c r="C102" s="1" t="inlineStr">
         <is>
-          <t>MM-752M</t>
+          <t>MM-744M</t>
         </is>
       </c>
       <c r="D102" s="1" t="inlineStr">
         <is>
-          <t>MM-940M</t>
+          <t>MM-936M</t>
         </is>
       </c>
       <c r="E102" s="1" t="inlineStr">
         <is>
-          <t>MM-9959M</t>
+          <t>MM-9957M</t>
         </is>
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>NR57</t>
+          <t>NR54</t>
         </is>
       </c>
       <c r="G102" s="1" t="inlineStr">
         <is>
-          <t>P2508</t>
+          <t>P2507</t>
         </is>
       </c>
       <c r="H102" s="1" t="inlineStr">
         <is>
-          <t>RL305</t>
+          <t>RL304</t>
         </is>
       </c>
     </row>
@@ -4684,32 +4684,32 @@
       </c>
       <c r="C103" s="1" t="inlineStr">
         <is>
-          <t>MM-756M</t>
+          <t>MM-752M</t>
         </is>
       </c>
       <c r="D103" s="1" t="inlineStr">
         <is>
-          <t>MM-944M</t>
+          <t>MM-940M</t>
         </is>
       </c>
       <c r="E103" s="1" t="inlineStr">
         <is>
-          <t>MM-9960M</t>
+          <t>MM-9959M</t>
         </is>
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>NR59</t>
+          <t>NR57</t>
         </is>
       </c>
       <c r="G103" s="1" t="inlineStr">
         <is>
-          <t>P2509</t>
+          <t>P2508</t>
         </is>
       </c>
       <c r="H103" s="1" t="inlineStr">
         <is>
-          <t>RL307</t>
+          <t>RL305</t>
         </is>
       </c>
     </row>
@@ -4726,32 +4726,32 @@
       </c>
       <c r="C104" s="1" t="inlineStr">
         <is>
-          <t>MM-760M</t>
+          <t>MM-756M</t>
         </is>
       </c>
       <c r="D104" s="1" t="inlineStr">
         <is>
-          <t>MM-948M</t>
+          <t>MM-944M</t>
         </is>
       </c>
       <c r="E104" s="1" t="inlineStr">
         <is>
-          <t>MM-9961M</t>
+          <t>MM-9960M</t>
         </is>
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>NR61</t>
+          <t>NR59</t>
         </is>
       </c>
       <c r="G104" s="1" t="inlineStr">
         <is>
-          <t>P2510</t>
+          <t>P2509</t>
         </is>
       </c>
       <c r="H104" s="1" t="inlineStr">
         <is>
-          <t>RL309</t>
+          <t>RL307</t>
         </is>
       </c>
     </row>
@@ -4768,32 +4768,32 @@
       </c>
       <c r="C105" s="1" t="inlineStr">
         <is>
-          <t>MM-764M</t>
+          <t>MM-760M</t>
         </is>
       </c>
       <c r="D105" s="1" t="inlineStr">
         <is>
-          <t>MM-952M</t>
+          <t>MM-948M</t>
         </is>
       </c>
       <c r="E105" s="1" t="inlineStr">
         <is>
-          <t>MM-9962M</t>
+          <t>MM-9961M</t>
         </is>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>NR62</t>
+          <t>NR61</t>
         </is>
       </c>
       <c r="G105" s="1" t="inlineStr">
         <is>
-          <t>P2511</t>
+          <t>P2510</t>
         </is>
       </c>
       <c r="H105" s="1" t="inlineStr">
         <is>
-          <t>RL310</t>
+          <t>RL309</t>
         </is>
       </c>
     </row>
@@ -4810,32 +4810,32 @@
       </c>
       <c r="C106" s="1" t="inlineStr">
         <is>
-          <t>MM-768M</t>
+          <t>MM-764M</t>
         </is>
       </c>
       <c r="D106" s="1" t="inlineStr">
         <is>
-          <t>MM-954M</t>
+          <t>MM-952M</t>
         </is>
       </c>
       <c r="E106" s="1" t="inlineStr">
         <is>
-          <t>MM-9963M</t>
+          <t>MM-9962M</t>
         </is>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR62</t>
         </is>
       </c>
       <c r="G106" s="1" t="inlineStr">
         <is>
-          <t>P2513</t>
+          <t>P2511</t>
         </is>
       </c>
       <c r="H106" s="1" t="inlineStr">
         <is>
-          <t>S312</t>
+          <t>RL310</t>
         </is>
       </c>
     </row>
@@ -4852,32 +4852,32 @@
       </c>
       <c r="C107" s="1" t="inlineStr">
         <is>
-          <t>MM-774M</t>
+          <t>MM-768M</t>
         </is>
       </c>
       <c r="D107" s="1" t="inlineStr">
         <is>
-          <t>MM-956M</t>
+          <t>MM-954M</t>
         </is>
       </c>
       <c r="E107" s="1" t="inlineStr">
         <is>
-          <t>MM-9964M</t>
+          <t>MM-9963M</t>
         </is>
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR64</t>
         </is>
       </c>
       <c r="G107" s="1" t="inlineStr">
         <is>
-          <t>P2514</t>
+          <t>P2513</t>
         </is>
       </c>
       <c r="H107" s="1" t="inlineStr">
         <is>
-          <t>S317</t>
+          <t>S312</t>
         </is>
       </c>
     </row>
@@ -4894,32 +4894,32 @@
       </c>
       <c r="C108" s="1" t="inlineStr">
         <is>
-          <t>MM-776M</t>
+          <t>MM-774M</t>
         </is>
       </c>
       <c r="D108" s="1" t="inlineStr">
         <is>
-          <t>MM-958M</t>
+          <t>MM-956M</t>
         </is>
       </c>
       <c r="E108" s="1" t="inlineStr">
         <is>
-          <t>MM-9965M</t>
+          <t>MM-9964M</t>
         </is>
       </c>
       <c r="F108" s="1" t="inlineStr">
         <is>
-          <t>NR66</t>
+          <t>NR65</t>
         </is>
       </c>
       <c r="G108" s="1" t="inlineStr">
         <is>
-          <t>P2515</t>
+          <t>P2514</t>
         </is>
       </c>
       <c r="H108" s="1" t="inlineStr">
         <is>
-          <t>S3301</t>
+          <t>S317</t>
         </is>
       </c>
     </row>
@@ -4936,32 +4936,32 @@
       </c>
       <c r="C109" s="1" t="inlineStr">
         <is>
-          <t>MM-778M</t>
+          <t>MM-776M</t>
         </is>
       </c>
       <c r="D109" s="1" t="inlineStr">
         <is>
-          <t>MM-962M</t>
+          <t>MM-958M</t>
         </is>
       </c>
       <c r="E109" s="1" t="inlineStr">
         <is>
-          <t>MM-9966M</t>
+          <t>MM-9965M</t>
         </is>
       </c>
       <c r="F109" s="1" t="inlineStr">
         <is>
-          <t>NR67</t>
+          <t>NR66</t>
         </is>
       </c>
       <c r="G109" s="1" t="inlineStr">
         <is>
-          <t>P2516</t>
+          <t>P2515</t>
         </is>
       </c>
       <c r="H109" s="1" t="inlineStr">
         <is>
-          <t>S3302</t>
+          <t>S3301</t>
         </is>
       </c>
     </row>
@@ -4978,32 +4978,32 @@
       </c>
       <c r="C110" s="1" t="inlineStr">
         <is>
-          <t>MM-780M</t>
+          <t>MM-778M</t>
         </is>
       </c>
       <c r="D110" s="1" t="inlineStr">
         <is>
-          <t>MM-964M</t>
+          <t>MM-962M</t>
         </is>
       </c>
       <c r="E110" s="1" t="inlineStr">
         <is>
-          <t>MM-9967M</t>
+          <t>MM-9966M</t>
         </is>
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR67</t>
         </is>
       </c>
       <c r="G110" s="1" t="inlineStr">
         <is>
-          <t>PB1</t>
+          <t>P2516</t>
         </is>
       </c>
       <c r="H110" s="1" t="inlineStr">
         <is>
-          <t>S3304</t>
+          <t>S3302</t>
         </is>
       </c>
     </row>
@@ -5020,32 +5020,32 @@
       </c>
       <c r="C111" s="1" t="inlineStr">
         <is>
-          <t>MM-784M</t>
+          <t>MM-780M</t>
         </is>
       </c>
       <c r="D111" s="1" t="inlineStr">
         <is>
-          <t>MM-966M</t>
+          <t>MM-964M</t>
         </is>
       </c>
       <c r="E111" s="1" t="inlineStr">
         <is>
-          <t>MM-9969M</t>
+          <t>MM-9967M</t>
         </is>
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>NR69</t>
+          <t>NR68</t>
         </is>
       </c>
       <c r="G111" s="1" t="inlineStr">
         <is>
-          <t>PB2</t>
+          <t>PB1</t>
         </is>
       </c>
       <c r="H111" s="1" t="inlineStr">
         <is>
-          <t>S3305</t>
+          <t>S3304</t>
         </is>
       </c>
     </row>
@@ -5062,32 +5062,32 @@
       </c>
       <c r="C112" s="1" t="inlineStr">
         <is>
-          <t>MM-790M</t>
+          <t>MM-784M</t>
         </is>
       </c>
       <c r="D112" s="1" t="inlineStr">
         <is>
-          <t>MM-968M</t>
+          <t>MM-966M</t>
         </is>
       </c>
       <c r="E112" s="1" t="inlineStr">
         <is>
-          <t>MM-9970M</t>
+          <t>MM-9969M</t>
         </is>
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>NR71</t>
+          <t>NR69</t>
         </is>
       </c>
       <c r="G112" s="1" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>PB2</t>
         </is>
       </c>
       <c r="H112" s="1" t="inlineStr">
         <is>
-          <t>S3306</t>
+          <t>S3305</t>
         </is>
       </c>
     </row>
@@ -5104,2079 +5104,2084 @@
       </c>
       <c r="C113" s="1" t="inlineStr">
         <is>
-          <t>MM-792M</t>
+          <t>MM-790M</t>
         </is>
       </c>
       <c r="D113" s="1" t="inlineStr">
         <is>
-          <t>MM-970M</t>
+          <t>MM-968M</t>
         </is>
       </c>
       <c r="E113" s="1" t="inlineStr">
         <is>
-          <t>MMY032</t>
+          <t>MM-9970M</t>
         </is>
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>NR72</t>
+          <t>NR71</t>
         </is>
       </c>
       <c r="G113" s="1" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>PB4</t>
         </is>
       </c>
       <c r="H113" s="1" t="inlineStr">
         <is>
-          <t>S3307</t>
+          <t>S3306</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>S3309</t>
+          <t>S3307</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
         <is>
-          <t>TT108</t>
+          <t>TT107</t>
         </is>
       </c>
       <c r="C115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8110</t>
+          <t>VLINE-8107</t>
         </is>
       </c>
       <c r="D115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8311</t>
+          <t>VLINE-8306</t>
         </is>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8449</t>
+          <t>VLINE-8447</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8754</t>
+          <t>VLINE-8753</t>
         </is>
       </c>
       <c r="G115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8819</t>
+          <t>VLINE-8818</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>S3310</t>
+          <t>S3309</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TT108</t>
         </is>
       </c>
       <c r="C116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8111</t>
+          <t>VLINE-8110</t>
         </is>
       </c>
       <c r="D116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8313</t>
+          <t>VLINE-8311</t>
         </is>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8450</t>
+          <t>VLINE-8449</t>
         </is>
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8755</t>
+          <t>VLINE-8754</t>
         </is>
       </c>
       <c r="G116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8822</t>
+          <t>VLINE-8819</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>S7001</t>
+          <t>S3310</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
         <is>
-          <t>TT113</t>
+          <t>TT110</t>
         </is>
       </c>
       <c r="C117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8113</t>
+          <t>VLINE-8111</t>
         </is>
       </c>
       <c r="D117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8314</t>
+          <t>VLINE-8313</t>
         </is>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8451</t>
+          <t>VLINE-8450</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8756</t>
+          <t>VLINE-8755</t>
         </is>
       </c>
       <c r="G117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8860</t>
+          <t>VLINE-8822</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>S7002</t>
+          <t>S7001</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
         <is>
-          <t>TT114</t>
+          <t>TT113</t>
         </is>
       </c>
       <c r="C118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8114</t>
+          <t>VLINE-8113</t>
         </is>
       </c>
       <c r="D118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8316</t>
+          <t>VLINE-8314</t>
         </is>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8452</t>
+          <t>VLINE-8451</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8757</t>
+          <t>VLINE-8756</t>
         </is>
       </c>
       <c r="G118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8861</t>
+          <t>VLINE-8860</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>S7003</t>
+          <t>S7002</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT114</t>
         </is>
       </c>
       <c r="C119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8115</t>
+          <t>VLINE-8114</t>
         </is>
       </c>
       <c r="D119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8318</t>
+          <t>VLINE-8316</t>
         </is>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8453</t>
+          <t>VLINE-8452</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8758</t>
+          <t>VLINE-8757</t>
         </is>
       </c>
       <c r="G119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8862</t>
+          <t>VLINE-8861</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>S7005</t>
+          <t>S7003</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
         <is>
-          <t>TT116</t>
+          <t>TT115</t>
         </is>
       </c>
       <c r="C120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8119</t>
+          <t>VLINE-8115</t>
         </is>
       </c>
       <c r="D120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8321</t>
+          <t>VLINE-8318</t>
         </is>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8454</t>
+          <t>VLINE-8453</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8759</t>
+          <t>VLINE-8758</t>
         </is>
       </c>
       <c r="G120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8863</t>
+          <t>VLINE-8862</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>S7006</t>
+          <t>S7005</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT116</t>
         </is>
       </c>
       <c r="C121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8120</t>
+          <t>VLINE-8119</t>
         </is>
       </c>
       <c r="D121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8323</t>
+          <t>VLINE-8321</t>
         </is>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8455</t>
+          <t>VLINE-8454</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8760</t>
+          <t>VLINE-8759</t>
         </is>
       </c>
       <c r="G121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8864</t>
+          <t>VLINE-8863</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>S7007</t>
+          <t>S7006</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
         <is>
-          <t>TT122</t>
+          <t>TT117</t>
         </is>
       </c>
       <c r="C122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8121</t>
+          <t>VLINE-8120</t>
         </is>
       </c>
       <c r="D122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8324</t>
+          <t>VLINE-8323</t>
         </is>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8456</t>
+          <t>VLINE-8455</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8761</t>
+          <t>VLINE-8760</t>
         </is>
       </c>
       <c r="G122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8865</t>
+          <t>VLINE-8864</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>S7008</t>
+          <t>S7007</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
         <is>
-          <t>TT127</t>
+          <t>TT122</t>
         </is>
       </c>
       <c r="C123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8123</t>
+          <t>VLINE-8121</t>
         </is>
       </c>
       <c r="D123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8325</t>
+          <t>VLINE-8324</t>
         </is>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8457</t>
+          <t>VLINE-8456</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8762</t>
+          <t>VLINE-8761</t>
         </is>
       </c>
       <c r="G123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8866</t>
+          <t>VLINE-8865</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>S7012</t>
+          <t>S7008</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
         <is>
-          <t>TT128</t>
+          <t>TT127</t>
         </is>
       </c>
       <c r="C124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8124</t>
+          <t>VLINE-8123</t>
         </is>
       </c>
       <c r="D124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8328</t>
+          <t>VLINE-8325</t>
         </is>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8460</t>
+          <t>VLINE-8457</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8763</t>
+          <t>VLINE-8762</t>
         </is>
       </c>
       <c r="G124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8867</t>
+          <t>VLINE-8866</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>S7014</t>
+          <t>S7012</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT128</t>
         </is>
       </c>
       <c r="C125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8126</t>
+          <t>VLINE-8124</t>
         </is>
       </c>
       <c r="D125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8329</t>
+          <t>VLINE-8328</t>
         </is>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8461</t>
+          <t>VLINE-8460</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8765</t>
+          <t>VLINE-8763</t>
         </is>
       </c>
       <c r="G125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8868</t>
+          <t>VLINE-8867</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>S7015</t>
+          <t>S7014</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
         <is>
-          <t>TT131</t>
+          <t>TT130</t>
         </is>
       </c>
       <c r="C126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8127</t>
+          <t>VLINE-8126</t>
         </is>
       </c>
       <c r="D126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8332</t>
+          <t>VLINE-8329</t>
         </is>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8464</t>
+          <t>VLINE-8461</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8766</t>
+          <t>VLINE-8765</t>
         </is>
       </c>
       <c r="G126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8869</t>
+          <t>VLINE-8868</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>S7017</t>
+          <t>S7015</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT131</t>
         </is>
       </c>
       <c r="C127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8128</t>
+          <t>VLINE-8127</t>
         </is>
       </c>
       <c r="D127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8336</t>
+          <t>VLINE-8332</t>
         </is>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8465</t>
+          <t>VLINE-8464</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8767</t>
+          <t>VLINE-8766</t>
         </is>
       </c>
       <c r="G127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8890</t>
+          <t>VLINE-8869</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>S7018</t>
+          <t>S7017</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT202</t>
         </is>
       </c>
       <c r="C128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8129</t>
+          <t>VLINE-8128</t>
         </is>
       </c>
       <c r="D128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8337</t>
+          <t>VLINE-8336</t>
         </is>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8468</t>
+          <t>VLINE-8465</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8768</t>
+          <t>VLINE-8767</t>
         </is>
       </c>
       <c r="G128" s="1" t="inlineStr">
         <is>
-          <t>WH001</t>
+          <t>VLINE-8890</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>S7020</t>
+          <t>S7018</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
         <is>
-          <t>VL352</t>
+          <t>TT206</t>
         </is>
       </c>
       <c r="C129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8131</t>
+          <t>VLINE-8129</t>
         </is>
       </c>
       <c r="D129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8338</t>
+          <t>VLINE-8337</t>
         </is>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8469</t>
+          <t>VLINE-8468</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8769</t>
+          <t>VLINE-8768</t>
         </is>
       </c>
       <c r="G129" s="1" t="inlineStr">
         <is>
-          <t>WH003</t>
+          <t>WH001</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>S7022</t>
+          <t>S7020</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
         <is>
-          <t>VL353</t>
+          <t>VL352</t>
         </is>
       </c>
       <c r="C130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8132</t>
+          <t>VLINE-8131</t>
         </is>
       </c>
       <c r="D130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8339</t>
+          <t>VLINE-8338</t>
         </is>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8605</t>
+          <t>VLINE-8469</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8770</t>
+          <t>VLINE-8769</t>
         </is>
       </c>
       <c r="G130" s="1" t="inlineStr">
         <is>
-          <t>WL02</t>
+          <t>WH003</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>S7022</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
         <is>
-          <t>VL357</t>
+          <t>VL353</t>
         </is>
       </c>
       <c r="C131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8133</t>
+          <t>VLINE-8132</t>
         </is>
       </c>
       <c r="D131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8362</t>
+          <t>VLINE-8339</t>
         </is>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8610</t>
+          <t>VLINE-8605</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8772</t>
+          <t>VLINE-8770</t>
         </is>
       </c>
       <c r="G131" s="1" t="inlineStr">
         <is>
-          <t>X12-X14</t>
+          <t>WL02</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>SCT002</t>
+          <t>SCT001</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8004</t>
+          <t>VL357</t>
         </is>
       </c>
       <c r="C132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8134</t>
+          <t>VLINE-8133</t>
         </is>
       </c>
       <c r="D132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8363</t>
+          <t>VLINE-8362</t>
         </is>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8612</t>
+          <t>VLINE-8610</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8773</t>
+          <t>VLINE-8772</t>
         </is>
       </c>
       <c r="G132" s="1" t="inlineStr">
         <is>
-          <t>X31</t>
+          <t>X12-X14</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>SCT006</t>
+          <t>SCT002</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8007</t>
+          <t>VLINE-8004</t>
         </is>
       </c>
       <c r="C133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8136</t>
+          <t>VLINE-8134</t>
         </is>
       </c>
       <c r="D133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8365</t>
+          <t>VLINE-8363</t>
         </is>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8615</t>
+          <t>VLINE-8612</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8774</t>
+          <t>VLINE-8773</t>
         </is>
       </c>
       <c r="G133" s="1" t="inlineStr">
         <is>
-          <t>XP2000</t>
+          <t>X31</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>SCT007</t>
+          <t>SCT006</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8011</t>
+          <t>VLINE-8007</t>
         </is>
       </c>
       <c r="C134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8137</t>
+          <t>VLINE-8136</t>
         </is>
       </c>
       <c r="D134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8366</t>
+          <t>VLINE-8365</t>
         </is>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8617</t>
+          <t>VLINE-8615</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8776</t>
+          <t>VLINE-8774</t>
         </is>
       </c>
       <c r="G134" s="1" t="inlineStr">
         <is>
-          <t>XP2003</t>
+          <t>XP2000</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>SCT007</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8013</t>
+          <t>VLINE-8011</t>
         </is>
       </c>
       <c r="C135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8140</t>
+          <t>VLINE-8137</t>
         </is>
       </c>
       <c r="D135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8368</t>
+          <t>VLINE-8366</t>
         </is>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8620</t>
+          <t>VLINE-8617</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8778</t>
+          <t>VLINE-8776</t>
         </is>
       </c>
       <c r="G135" s="1" t="inlineStr">
         <is>
-          <t>XP2004</t>
+          <t>XP2003</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>SCT011</t>
+          <t>SCT009</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8019</t>
+          <t>VLINE-8013</t>
         </is>
       </c>
       <c r="C136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8141</t>
+          <t>VLINE-8140</t>
         </is>
       </c>
       <c r="D136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8369</t>
+          <t>VLINE-8368</t>
         </is>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8625</t>
+          <t>VLINE-8620</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8779</t>
+          <t>VLINE-8778</t>
         </is>
       </c>
       <c r="G136" s="1" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>XP2004</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>SCT011</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8020</t>
+          <t>VLINE-8019</t>
         </is>
       </c>
       <c r="C137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8142</t>
+          <t>VLINE-8141</t>
         </is>
       </c>
       <c r="D137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8403</t>
+          <t>VLINE-8369</t>
         </is>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8630</t>
+          <t>VLINE-8625</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8780</t>
+          <t>VLINE-8779</t>
         </is>
       </c>
       <c r="G137" s="1" t="inlineStr">
         <is>
-          <t>XP2007</t>
+          <t>XP2005</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>SCT014</t>
+          <t>SCT013</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8023</t>
+          <t>VLINE-8020</t>
         </is>
       </c>
       <c r="C138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8144</t>
+          <t>VLINE-8142</t>
         </is>
       </c>
       <c r="D138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8404</t>
+          <t>VLINE-8403</t>
         </is>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8671</t>
+          <t>VLINE-8630</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8781</t>
+          <t>VLINE-8780</t>
         </is>
       </c>
       <c r="G138" s="1" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>XP2007</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>SCT015</t>
+          <t>SCT014</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8025</t>
+          <t>VLINE-8023</t>
         </is>
       </c>
       <c r="C139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8145</t>
+          <t>VLINE-8144</t>
         </is>
       </c>
       <c r="D139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8406</t>
+          <t>VLINE-8404</t>
         </is>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8706</t>
+          <t>VLINE-8671</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8782</t>
+          <t>VLINE-8781</t>
         </is>
       </c>
       <c r="G139" s="1" t="inlineStr">
         <is>
-          <t>XP2010</t>
+          <t>XP2008</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>SO2</t>
+          <t>SCT015</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8026</t>
+          <t>VLINE-8025</t>
         </is>
       </c>
       <c r="C140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8148</t>
+          <t>VLINE-8145</t>
         </is>
       </c>
       <c r="D140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8408</t>
+          <t>VLINE-8406</t>
         </is>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8711</t>
+          <t>VLINE-8706</t>
         </is>
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8783</t>
+          <t>VLINE-8782</t>
         </is>
       </c>
       <c r="G140" s="1" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>XP2010</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>SO2</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8027</t>
+          <t>VLINE-8026</t>
         </is>
       </c>
       <c r="C141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8150</t>
+          <t>VLINE-8148</t>
         </is>
       </c>
       <c r="D141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8410</t>
+          <t>VLINE-8408</t>
         </is>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8714</t>
+          <t>VLINE-8711</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8784</t>
+          <t>VLINE-8783</t>
         </is>
       </c>
       <c r="G141" s="1" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>XP2011</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>SSR101</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8028</t>
+          <t>VLINE-8027</t>
         </is>
       </c>
       <c r="C142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8151</t>
+          <t>VLINE-8150</t>
         </is>
       </c>
       <c r="D142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8411</t>
+          <t>VLINE-8410</t>
         </is>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8717</t>
+          <t>VLINE-8714</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8786</t>
+          <t>VLINE-8784</t>
         </is>
       </c>
       <c r="G142" s="1" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>XP2012</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>SSR102</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8029</t>
+          <t>VLINE-8028</t>
         </is>
       </c>
       <c r="C143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8152</t>
+          <t>VLINE-8151</t>
         </is>
       </c>
       <c r="D143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8413</t>
+          <t>VLINE-8411</t>
         </is>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8720</t>
+          <t>VLINE-8717</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8787</t>
+          <t>VLINE-8786</t>
         </is>
       </c>
       <c r="G143" s="1" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>XP2013</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>SSR103</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8030</t>
+          <t>VLINE-8029</t>
         </is>
       </c>
       <c r="C144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8153</t>
+          <t>VLINE-8152</t>
         </is>
       </c>
       <c r="D144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8415</t>
+          <t>VLINE-8413</t>
         </is>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8721</t>
+          <t>VLINE-8720</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8788</t>
+          <t>VLINE-8787</t>
         </is>
       </c>
       <c r="G144" s="1" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>XP2014</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>T363</t>
+          <t>SSR104</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8031</t>
+          <t>VLINE-8030</t>
         </is>
       </c>
       <c r="C145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8154</t>
+          <t>VLINE-8153</t>
         </is>
       </c>
       <c r="D145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8417</t>
+          <t>VLINE-8415</t>
         </is>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8723</t>
+          <t>VLINE-8721</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8790</t>
+          <t>VLINE-8788</t>
         </is>
       </c>
       <c r="G145" s="1" t="inlineStr">
         <is>
-          <t>XP2016</t>
+          <t>XP2015</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>T386</t>
+          <t>T363</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8032</t>
+          <t>VLINE-8031</t>
         </is>
       </c>
       <c r="C146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8155</t>
+          <t>VLINE-8154</t>
         </is>
       </c>
       <c r="D146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8418</t>
+          <t>VLINE-8417</t>
         </is>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8725</t>
+          <t>VLINE-8723</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8792</t>
+          <t>VLINE-8790</t>
         </is>
       </c>
       <c r="G146" s="1" t="inlineStr">
         <is>
-          <t>XP2017</t>
+          <t>XP2016</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>TDX101</t>
+          <t>T386</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8036</t>
+          <t>VLINE-8032</t>
         </is>
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8157</t>
+          <t>VLINE-8155</t>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8419</t>
+          <t>VLINE-8418</t>
         </is>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8726</t>
+          <t>VLINE-8725</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8793</t>
+          <t>VLINE-8792</t>
         </is>
       </c>
       <c r="G147" s="1" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>XP2017</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>TDX101</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8038</t>
+          <t>VLINE-8036</t>
         </is>
       </c>
       <c r="C148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8158</t>
+          <t>VLINE-8157</t>
         </is>
       </c>
       <c r="D148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8420</t>
+          <t>VLINE-8419</t>
         </is>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8727</t>
+          <t>VLINE-8726</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8794</t>
+          <t>VLINE-8793</t>
         </is>
       </c>
       <c r="G148" s="1" t="inlineStr">
         <is>
-          <t>XR552</t>
+          <t>XP2019</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>TE2802</t>
+          <t>TE2801</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8042</t>
+          <t>VLINE-8038</t>
         </is>
       </c>
       <c r="C149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8159</t>
+          <t>VLINE-8158</t>
         </is>
       </c>
       <c r="D149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8421</t>
+          <t>VLINE-8420</t>
         </is>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8729</t>
+          <t>VLINE-8727</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8795</t>
+          <t>VLINE-8794</t>
         </is>
       </c>
       <c r="G149" s="1" t="inlineStr">
         <is>
-          <t>XRN001</t>
+          <t>XR552</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>TE2802</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8051</t>
+          <t>VLINE-8042</t>
         </is>
       </c>
       <c r="C150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8160</t>
+          <t>VLINE-8159</t>
         </is>
       </c>
       <c r="D150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8422</t>
+          <t>VLINE-8421</t>
         </is>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8730</t>
+          <t>VLINE-8729</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8796</t>
+          <t>VLINE-8795</t>
         </is>
       </c>
       <c r="G150" s="1" t="inlineStr">
         <is>
-          <t>XRN004</t>
+          <t>XRN001</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>TE2804</t>
+          <t>TE2803</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8052</t>
+          <t>VLINE-8051</t>
         </is>
       </c>
       <c r="C151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8161</t>
+          <t>VLINE-8160</t>
         </is>
       </c>
       <c r="D151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8424</t>
+          <t>VLINE-8422</t>
         </is>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8731</t>
+          <t>VLINE-8730</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8797</t>
+          <t>VLINE-8796</t>
         </is>
       </c>
       <c r="G151" s="1" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>XRN004</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>TE2804</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8053</t>
+          <t>VLINE-8052</t>
         </is>
       </c>
       <c r="C152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8162</t>
+          <t>VLINE-8161</t>
         </is>
       </c>
       <c r="D152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8425</t>
+          <t>VLINE-8424</t>
         </is>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8733</t>
+          <t>VLINE-8731</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8799</t>
+          <t>VLINE-8797</t>
         </is>
       </c>
       <c r="G152" s="1" t="inlineStr">
         <is>
-          <t>XRN006</t>
+          <t>XRN005</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>TE2806</t>
+          <t>TE2805</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8055</t>
+          <t>VLINE-8053</t>
         </is>
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8171</t>
+          <t>VLINE-8162</t>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8426</t>
+          <t>VLINE-8425</t>
         </is>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8735</t>
+          <t>VLINE-8733</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8800</t>
+          <t>VLINE-8799</t>
         </is>
       </c>
       <c r="G153" s="1" t="inlineStr">
         <is>
-          <t>XRN007</t>
+          <t>XRN006</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>TE2806</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8056</t>
+          <t>VLINE-8055</t>
         </is>
       </c>
       <c r="C154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8172</t>
+          <t>VLINE-8171</t>
         </is>
       </c>
       <c r="D154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8427</t>
+          <t>VLINE-8426</t>
         </is>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8736</t>
+          <t>VLINE-8735</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8801</t>
+          <t>VLINE-8800</t>
         </is>
       </c>
       <c r="G154" s="1" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>XRN007</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>TE2807</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8057</t>
+          <t>VLINE-8056</t>
         </is>
       </c>
       <c r="C155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8176</t>
+          <t>VLINE-8172</t>
         </is>
       </c>
       <c r="D155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8428</t>
+          <t>VLINE-8427</t>
         </is>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8737</t>
+          <t>VLINE-8736</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8802</t>
+          <t>VLINE-8801</t>
         </is>
       </c>
       <c r="G155" s="1" t="inlineStr">
         <is>
-          <t>XRN011</t>
+          <t>XRN009</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>TE2809</t>
+          <t>TE2808</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8058</t>
+          <t>VLINE-8057</t>
         </is>
       </c>
       <c r="C156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8179</t>
+          <t>VLINE-8176</t>
         </is>
       </c>
       <c r="D156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8429</t>
+          <t>VLINE-8428</t>
         </is>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8739</t>
+          <t>VLINE-8737</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8803</t>
+          <t>VLINE-8802</t>
         </is>
       </c>
       <c r="G156" s="1" t="inlineStr">
         <is>
-          <t>XRN014</t>
+          <t>XRN011</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>TE2810</t>
+          <t>TE2809</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8059</t>
+          <t>VLINE-8058</t>
         </is>
       </c>
       <c r="C157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8180</t>
+          <t>VLINE-8179</t>
         </is>
       </c>
       <c r="D157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8430</t>
+          <t>VLINE-8429</t>
         </is>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8740</t>
+          <t>VLINE-8739</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8804</t>
+          <t>VLINE-8803</t>
         </is>
       </c>
       <c r="G157" s="1" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>XRN014</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>TE2812</t>
+          <t>TE2810</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8061</t>
+          <t>VLINE-8059</t>
         </is>
       </c>
       <c r="C158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8181</t>
+          <t>VLINE-8180</t>
         </is>
       </c>
       <c r="D158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8431</t>
+          <t>VLINE-8430</t>
         </is>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8741</t>
+          <t>VLINE-8740</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8805</t>
+          <t>VLINE-8804</t>
         </is>
       </c>
       <c r="G158" s="1" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>XRN017</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>TE2812</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8072</t>
+          <t>VLINE-8061</t>
         </is>
       </c>
       <c r="C159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8182</t>
+          <t>VLINE-8181</t>
         </is>
       </c>
       <c r="D159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8432</t>
+          <t>VLINE-8431</t>
         </is>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8742</t>
+          <t>VLINE-8741</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8806</t>
+          <t>VLINE-8805</t>
         </is>
       </c>
       <c r="G159" s="1" t="inlineStr">
         <is>
-          <t>XRN020</t>
+          <t>XRN018</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>TE2813</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8074</t>
+          <t>VLINE-8072</t>
         </is>
       </c>
       <c r="C160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8183</t>
+          <t>VLINE-8182</t>
         </is>
       </c>
       <c r="D160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8433</t>
+          <t>VLINE-8432</t>
         </is>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8743</t>
+          <t>VLINE-8742</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8807</t>
+          <t>VLINE-8806</t>
         </is>
       </c>
       <c r="G160" s="1" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>XRN020</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>TE2814</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8075</t>
+          <t>VLINE-8074</t>
         </is>
       </c>
       <c r="C161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8184</t>
+          <t>VLINE-8183</t>
         </is>
       </c>
       <c r="D161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8434</t>
+          <t>VLINE-8433</t>
         </is>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8744</t>
+          <t>VLINE-8743</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8808</t>
+          <t>VLINE-8807</t>
         </is>
       </c>
       <c r="G161" s="1" t="inlineStr">
         <is>
-          <t>XRN023</t>
+          <t>XRN021</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>TJ107</t>
+          <t>TJ096</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8076</t>
+          <t>VLINE-8075</t>
         </is>
       </c>
       <c r="C162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8185</t>
+          <t>VLINE-8184</t>
         </is>
       </c>
       <c r="D162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8435</t>
+          <t>VLINE-8434</t>
         </is>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8745</t>
+          <t>VLINE-8744</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8809</t>
+          <t>VLINE-8808</t>
         </is>
       </c>
       <c r="G162" s="1" t="inlineStr">
         <is>
-          <t>XRN025</t>
+          <t>XRN023</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TJ107</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8077</t>
+          <t>VLINE-8076</t>
         </is>
       </c>
       <c r="C163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8186</t>
+          <t>VLINE-8185</t>
         </is>
       </c>
       <c r="D163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8438</t>
+          <t>VLINE-8435</t>
         </is>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8746</t>
+          <t>VLINE-8745</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8810</t>
+          <t>VLINE-8809</t>
         </is>
       </c>
       <c r="G163" s="1" t="inlineStr">
         <is>
-          <t>XRN026</t>
+          <t>XRN025</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TT03</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8080</t>
+          <t>VLINE-8077</t>
         </is>
       </c>
       <c r="C164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8187</t>
+          <t>VLINE-8186</t>
         </is>
       </c>
       <c r="D164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8440</t>
+          <t>VLINE-8438</t>
         </is>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8747</t>
+          <t>VLINE-8746</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8811</t>
+          <t>VLINE-8810</t>
         </is>
       </c>
       <c r="G164" s="1" t="inlineStr">
         <is>
-          <t>XRN027</t>
+          <t>XRN026</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TT04</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8081</t>
+          <t>VLINE-8080</t>
         </is>
       </c>
       <c r="C165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8188</t>
+          <t>VLINE-8187</t>
         </is>
       </c>
       <c r="D165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8441</t>
+          <t>VLINE-8440</t>
         </is>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8748</t>
+          <t>VLINE-8747</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8812</t>
+          <t>VLINE-8811</t>
         </is>
       </c>
       <c r="G165" s="1" t="inlineStr">
         <is>
-          <t>Y163</t>
+          <t>XRN027</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>TT07</t>
+          <t>TT05</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8084</t>
+          <t>VLINE-8081</t>
         </is>
       </c>
       <c r="C166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8189</t>
+          <t>VLINE-8188</t>
         </is>
       </c>
       <c r="D166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8442</t>
+          <t>VLINE-8441</t>
         </is>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8749</t>
+          <t>VLINE-8748</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8813</t>
+          <t>VLINE-8812</t>
+        </is>
+      </c>
+      <c r="G166" s="1" t="inlineStr">
+        <is>
+          <t>Y163</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TT07</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8088</t>
+          <t>VLINE-8084</t>
         </is>
       </c>
       <c r="C167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8293</t>
+          <t>VLINE-8189</t>
         </is>
       </c>
       <c r="D167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8443</t>
+          <t>VLINE-8442</t>
         </is>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8750</t>
+          <t>VLINE-8749</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8814</t>
+          <t>VLINE-8813</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TT08</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8089</t>
+          <t>VLINE-8088</t>
         </is>
       </c>
       <c r="C168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8303</t>
+          <t>VLINE-8293</t>
         </is>
       </c>
       <c r="D168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8444</t>
+          <t>VLINE-8443</t>
         </is>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8751</t>
+          <t>VLINE-8750</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8816</t>
+          <t>VLINE-8814</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>TT106</t>
+          <t>TT103</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8104</t>
+          <t>VLINE-8089</t>
         </is>
       </c>
       <c r="C169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8304</t>
+          <t>VLINE-8303</t>
         </is>
       </c>
       <c r="D169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8446</t>
+          <t>VLINE-8444</t>
         </is>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8752</t>
+          <t>VLINE-8751</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8817</t>
+          <t>VLINE-8816</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TT106</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8107</t>
+          <t>VLINE-8104</t>
         </is>
       </c>
       <c r="C170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8306</t>
+          <t>VLINE-8304</t>
         </is>
       </c>
       <c r="D170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8447</t>
+          <t>VLINE-8446</t>
         </is>
       </c>
       <c r="E170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8753</t>
+          <t>VLINE-8752</t>
         </is>
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8818</t>
+          <t>VLINE-8817</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update trains and loco export 2026-04-05 11:50:36
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -2799,27 +2799,27 @@
       </c>
       <c r="D58" s="1" t="inlineStr">
         <is>
-          <t>MM-792M</t>
+          <t>MM-790M</t>
         </is>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>MM-970M</t>
+          <t>MM-968M</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>MMY032</t>
+          <t>MM-9970M</t>
         </is>
       </c>
       <c r="G58" s="1" t="inlineStr">
         <is>
-          <t>NR72</t>
+          <t>NR71</t>
         </is>
       </c>
       <c r="H58" s="1" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>PB4</t>
         </is>
       </c>
     </row>
@@ -2841,27 +2841,27 @@
       </c>
       <c r="D59" s="1" t="inlineStr">
         <is>
-          <t>MM-796M</t>
+          <t>MM-792M</t>
         </is>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>MM-972M</t>
+          <t>MM-970M</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MMY032</t>
         </is>
       </c>
       <c r="G59" s="1" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR72</t>
         </is>
       </c>
       <c r="H59" s="1" t="inlineStr">
         <is>
-          <t>PHC002</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
@@ -2883,27 +2883,27 @@
       </c>
       <c r="D60" s="1" t="inlineStr">
         <is>
-          <t>MM-798M</t>
+          <t>MM-796M</t>
         </is>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>MM-974M</t>
+          <t>MM-972M</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>MRL004</t>
+          <t>MRL001</t>
         </is>
       </c>
       <c r="G60" s="1" t="inlineStr">
         <is>
-          <t>NR77</t>
+          <t>NR75</t>
         </is>
       </c>
       <c r="H60" s="1" t="inlineStr">
         <is>
-          <t>Q4001</t>
+          <t>PHC002</t>
         </is>
       </c>
     </row>
@@ -2925,27 +2925,27 @@
       </c>
       <c r="D61" s="1" t="inlineStr">
         <is>
-          <t>MM-800M</t>
+          <t>MM-798M</t>
         </is>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>MM-976M</t>
+          <t>MM-974M</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>MRL006</t>
+          <t>MRL004</t>
         </is>
       </c>
       <c r="G61" s="1" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR77</t>
         </is>
       </c>
       <c r="H61" s="1" t="inlineStr">
         <is>
-          <t>Q4003</t>
+          <t>Q4001</t>
         </is>
       </c>
     </row>
@@ -2967,27 +2967,27 @@
       </c>
       <c r="D62" s="1" t="inlineStr">
         <is>
-          <t>MM-802M</t>
+          <t>MM-800M</t>
         </is>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>MM-980M</t>
+          <t>MM-976M</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>N452</t>
+          <t>MRL006</t>
         </is>
       </c>
       <c r="G62" s="1" t="inlineStr">
         <is>
-          <t>NR81</t>
+          <t>NR78</t>
         </is>
       </c>
       <c r="H62" s="1" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>Q4003</t>
         </is>
       </c>
     </row>
@@ -3009,27 +3009,27 @@
       </c>
       <c r="D63" s="1" t="inlineStr">
         <is>
-          <t>MM-804M</t>
+          <t>MM-802M</t>
         </is>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>MM-982M</t>
+          <t>MM-980M</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>N453</t>
+          <t>N452</t>
         </is>
       </c>
       <c r="G63" s="1" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR81</t>
         </is>
       </c>
       <c r="H63" s="1" t="inlineStr">
         <is>
-          <t>Q4005</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
@@ -3051,27 +3051,27 @@
       </c>
       <c r="D64" s="1" t="inlineStr">
         <is>
-          <t>MM-808M</t>
+          <t>MM-804M</t>
         </is>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>MM-984M</t>
+          <t>MM-982M</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>N457</t>
+          <t>N453</t>
         </is>
       </c>
       <c r="G64" s="1" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR82</t>
         </is>
       </c>
       <c r="H64" s="1" t="inlineStr">
         <is>
-          <t>Q4006</t>
+          <t>Q4005</t>
         </is>
       </c>
     </row>
@@ -3093,27 +3093,27 @@
       </c>
       <c r="D65" s="1" t="inlineStr">
         <is>
-          <t>MM-810M</t>
+          <t>MM-808M</t>
         </is>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>MM-986M</t>
+          <t>MM-984M</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>N458</t>
+          <t>N457</t>
         </is>
       </c>
       <c r="G65" s="1" t="inlineStr">
         <is>
-          <t>NR84</t>
+          <t>NR83</t>
         </is>
       </c>
       <c r="H65" s="1" t="inlineStr">
         <is>
-          <t>Q4007</t>
+          <t>Q4006</t>
         </is>
       </c>
     </row>
@@ -3135,27 +3135,27 @@
       </c>
       <c r="D66" s="1" t="inlineStr">
         <is>
-          <t>MM-814M</t>
+          <t>MM-810M</t>
         </is>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>MM-9902M</t>
+          <t>MM-986M</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>N465</t>
+          <t>N458</t>
         </is>
       </c>
       <c r="G66" s="1" t="inlineStr">
         <is>
-          <t>NR85</t>
+          <t>NR84</t>
         </is>
       </c>
       <c r="H66" s="1" t="inlineStr">
         <is>
-          <t>Q4009</t>
+          <t>Q4007</t>
         </is>
       </c>
     </row>
@@ -3177,27 +3177,27 @@
       </c>
       <c r="D67" s="1" t="inlineStr">
         <is>
-          <t>MM-816M</t>
+          <t>MM-814M</t>
         </is>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>MM-9903M</t>
+          <t>MM-9902M</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>N465</t>
         </is>
       </c>
       <c r="G67" s="1" t="inlineStr">
         <is>
-          <t>NR86</t>
+          <t>NR85</t>
         </is>
       </c>
       <c r="H67" s="1" t="inlineStr">
         <is>
-          <t>Q4011</t>
+          <t>Q4009</t>
         </is>
       </c>
     </row>
@@ -3219,27 +3219,27 @@
       </c>
       <c r="D68" s="1" t="inlineStr">
         <is>
-          <t>MM-818M</t>
+          <t>MM-816M</t>
         </is>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>MM-9904M</t>
+          <t>MM-9903M</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>N467</t>
+          <t>N466</t>
         </is>
       </c>
       <c r="G68" s="1" t="inlineStr">
         <is>
-          <t>NR87</t>
+          <t>NR86</t>
         </is>
       </c>
       <c r="H68" s="1" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>Q4011</t>
         </is>
       </c>
     </row>
@@ -3261,27 +3261,27 @@
       </c>
       <c r="D69" s="1" t="inlineStr">
         <is>
-          <t>MM-820M</t>
+          <t>MM-818M</t>
         </is>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>MM-9906M</t>
+          <t>MM-9904M</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>N467</t>
         </is>
       </c>
       <c r="G69" s="1" t="inlineStr">
         <is>
-          <t>NR88</t>
+          <t>NR87</t>
         </is>
       </c>
       <c r="H69" s="1" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
@@ -3303,27 +3303,27 @@
       </c>
       <c r="D70" s="1" t="inlineStr">
         <is>
-          <t>MM-824M</t>
+          <t>MM-820M</t>
         </is>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>MM-9907M</t>
+          <t>MM-9906M</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>N473</t>
+          <t>N469</t>
         </is>
       </c>
       <c r="G70" s="1" t="inlineStr">
         <is>
-          <t>NR89</t>
+          <t>NR88</t>
         </is>
       </c>
       <c r="H70" s="1" t="inlineStr">
         <is>
-          <t>Q4014</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
@@ -3345,27 +3345,27 @@
       </c>
       <c r="D71" s="1" t="inlineStr">
         <is>
-          <t>MM-826M</t>
+          <t>MM-824M</t>
         </is>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>MM-9908M</t>
+          <t>MM-9907M</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>NR1</t>
+          <t>N473</t>
         </is>
       </c>
       <c r="G71" s="1" t="inlineStr">
         <is>
-          <t>NR90</t>
+          <t>NR89</t>
         </is>
       </c>
       <c r="H71" s="1" t="inlineStr">
         <is>
-          <t>Q4015</t>
+          <t>Q4014</t>
         </is>
       </c>
     </row>
@@ -3387,27 +3387,27 @@
       </c>
       <c r="D72" s="1" t="inlineStr">
         <is>
-          <t>MM-828M</t>
+          <t>MM-826M</t>
         </is>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>MM-9909M</t>
+          <t>MM-9908M</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>NR2</t>
+          <t>NR1</t>
         </is>
       </c>
       <c r="G72" s="1" t="inlineStr">
         <is>
-          <t>NR91</t>
+          <t>NR90</t>
         </is>
       </c>
       <c r="H72" s="1" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>Q4015</t>
         </is>
       </c>
     </row>
@@ -3429,27 +3429,27 @@
       </c>
       <c r="D73" s="1" t="inlineStr">
         <is>
-          <t>MM-830M</t>
+          <t>MM-828M</t>
         </is>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>MM-9912M</t>
+          <t>MM-9909M</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>NR2</t>
         </is>
       </c>
       <c r="G73" s="1" t="inlineStr">
         <is>
-          <t>NR92</t>
+          <t>NR91</t>
         </is>
       </c>
       <c r="H73" s="1" t="inlineStr">
         <is>
-          <t>Q4017</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
@@ -3471,27 +3471,27 @@
       </c>
       <c r="D74" s="1" t="inlineStr">
         <is>
-          <t>MM-832M</t>
+          <t>MM-830M</t>
         </is>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>MM-9913M</t>
+          <t>MM-9912M</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>NR4</t>
         </is>
       </c>
       <c r="G74" s="1" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR92</t>
         </is>
       </c>
       <c r="H74" s="1" t="inlineStr">
         <is>
-          <t>Q4019</t>
+          <t>Q4017</t>
         </is>
       </c>
     </row>
@@ -3508,32 +3508,32 @@
       </c>
       <c r="C75" s="1" t="inlineStr">
         <is>
-          <t>MM-616M</t>
+          <t>MM-608M</t>
         </is>
       </c>
       <c r="D75" s="1" t="inlineStr">
         <is>
-          <t>MM-834M</t>
+          <t>MM-832M</t>
         </is>
       </c>
       <c r="E75" s="1" t="inlineStr">
         <is>
-          <t>MM-9914M</t>
+          <t>MM-9913M</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>NR7</t>
+          <t>NR5</t>
         </is>
       </c>
       <c r="G75" s="1" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR93</t>
         </is>
       </c>
       <c r="H75" s="1" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>Q4019</t>
         </is>
       </c>
     </row>
@@ -3550,32 +3550,32 @@
       </c>
       <c r="C76" s="1" t="inlineStr">
         <is>
-          <t>MM-624M</t>
+          <t>MM-616M</t>
         </is>
       </c>
       <c r="D76" s="1" t="inlineStr">
         <is>
-          <t>MM-838M</t>
+          <t>MM-834M</t>
         </is>
       </c>
       <c r="E76" s="1" t="inlineStr">
         <is>
-          <t>MM-9915M</t>
+          <t>MM-9914M</t>
         </is>
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>NR8</t>
+          <t>NR7</t>
         </is>
       </c>
       <c r="G76" s="1" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR94</t>
         </is>
       </c>
       <c r="H76" s="1" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
@@ -3592,32 +3592,32 @@
       </c>
       <c r="C77" s="1" t="inlineStr">
         <is>
-          <t>MM-632M</t>
+          <t>MM-624M</t>
         </is>
       </c>
       <c r="D77" s="1" t="inlineStr">
         <is>
-          <t>MM-842M</t>
+          <t>MM-838M</t>
         </is>
       </c>
       <c r="E77" s="1" t="inlineStr">
         <is>
-          <t>MM-9917M</t>
+          <t>MM-9915M</t>
         </is>
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
-          <t>NR9</t>
+          <t>NR8</t>
         </is>
       </c>
       <c r="G77" s="1" t="inlineStr">
         <is>
-          <t>NR96</t>
+          <t>NR95</t>
         </is>
       </c>
       <c r="H77" s="1" t="inlineStr">
         <is>
-          <t>QBX005</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
@@ -3634,32 +3634,32 @@
       </c>
       <c r="C78" s="1" t="inlineStr">
         <is>
-          <t>MM-636M</t>
+          <t>MM-632M</t>
         </is>
       </c>
       <c r="D78" s="1" t="inlineStr">
         <is>
-          <t>MM-844M</t>
+          <t>MM-842M</t>
         </is>
       </c>
       <c r="E78" s="1" t="inlineStr">
         <is>
-          <t>MM-9918M</t>
+          <t>MM-9917M</t>
         </is>
       </c>
       <c r="F78" s="1" t="inlineStr">
         <is>
-          <t>NR12</t>
+          <t>NR9</t>
         </is>
       </c>
       <c r="G78" s="1" t="inlineStr">
         <is>
-          <t>NR98</t>
+          <t>NR96</t>
         </is>
       </c>
       <c r="H78" s="1" t="inlineStr">
         <is>
-          <t>QBX006</t>
+          <t>QBX005</t>
         </is>
       </c>
     </row>
@@ -3676,32 +3676,32 @@
       </c>
       <c r="C79" s="1" t="inlineStr">
         <is>
-          <t>MM-640M</t>
+          <t>MM-636M</t>
         </is>
       </c>
       <c r="D79" s="1" t="inlineStr">
         <is>
-          <t>MM-852M</t>
+          <t>MM-844M</t>
         </is>
       </c>
       <c r="E79" s="1" t="inlineStr">
         <is>
-          <t>MM-9919M</t>
+          <t>MM-9918M</t>
         </is>
       </c>
       <c r="F79" s="1" t="inlineStr">
         <is>
-          <t>NR15</t>
+          <t>NR12</t>
         </is>
       </c>
       <c r="G79" s="1" t="inlineStr">
         <is>
-          <t>NR99</t>
+          <t>NR98</t>
         </is>
       </c>
       <c r="H79" s="1" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>QBX006</t>
         </is>
       </c>
     </row>
@@ -3718,32 +3718,32 @@
       </c>
       <c r="C80" s="1" t="inlineStr">
         <is>
-          <t>MM-654M</t>
+          <t>MM-640M</t>
         </is>
       </c>
       <c r="D80" s="1" t="inlineStr">
         <is>
-          <t>MM-858M</t>
+          <t>MM-852M</t>
         </is>
       </c>
       <c r="E80" s="1" t="inlineStr">
         <is>
-          <t>MM-9920M</t>
+          <t>MM-9919M</t>
         </is>
       </c>
       <c r="F80" s="1" t="inlineStr">
         <is>
-          <t>NR16</t>
+          <t>NR15</t>
         </is>
       </c>
       <c r="G80" s="1" t="inlineStr">
         <is>
-          <t>NR101</t>
+          <t>NR99</t>
         </is>
       </c>
       <c r="H80" s="1" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>QE001</t>
         </is>
       </c>
     </row>
@@ -3760,32 +3760,32 @@
       </c>
       <c r="C81" s="1" t="inlineStr">
         <is>
-          <t>MM-656M</t>
+          <t>MM-654M</t>
         </is>
       </c>
       <c r="D81" s="1" t="inlineStr">
         <is>
-          <t>MM-860M</t>
+          <t>MM-858M</t>
         </is>
       </c>
       <c r="E81" s="1" t="inlineStr">
         <is>
-          <t>MM-9922M</t>
+          <t>MM-9920M</t>
         </is>
       </c>
       <c r="F81" s="1" t="inlineStr">
         <is>
-          <t>NR18</t>
+          <t>NR16</t>
         </is>
       </c>
       <c r="G81" s="1" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR101</t>
         </is>
       </c>
       <c r="H81" s="1" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
@@ -3802,32 +3802,32 @@
       </c>
       <c r="C82" s="1" t="inlineStr">
         <is>
-          <t>MM-660M</t>
+          <t>MM-656M</t>
         </is>
       </c>
       <c r="D82" s="1" t="inlineStr">
         <is>
-          <t>MM-862M</t>
+          <t>MM-860M</t>
         </is>
       </c>
       <c r="E82" s="1" t="inlineStr">
         <is>
-          <t>MM-9923M</t>
+          <t>MM-9922M</t>
         </is>
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
-          <t>NR19</t>
+          <t>NR18</t>
         </is>
       </c>
       <c r="G82" s="1" t="inlineStr">
         <is>
-          <t>NR103</t>
+          <t>NR102</t>
         </is>
       </c>
       <c r="H82" s="1" t="inlineStr">
         <is>
-          <t>QE004</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
@@ -3844,32 +3844,32 @@
       </c>
       <c r="C83" s="1" t="inlineStr">
         <is>
-          <t>MM-661M</t>
+          <t>MM-660M</t>
         </is>
       </c>
       <c r="D83" s="1" t="inlineStr">
         <is>
-          <t>MM-868M</t>
+          <t>MM-862M</t>
         </is>
       </c>
       <c r="E83" s="1" t="inlineStr">
         <is>
-          <t>MM-9924M</t>
+          <t>MM-9923M</t>
         </is>
       </c>
       <c r="F83" s="1" t="inlineStr">
         <is>
-          <t>NR21</t>
+          <t>NR19</t>
         </is>
       </c>
       <c r="G83" s="1" t="inlineStr">
         <is>
-          <t>NR105</t>
+          <t>NR103</t>
         </is>
       </c>
       <c r="H83" s="1" t="inlineStr">
         <is>
-          <t>QE006</t>
+          <t>QE004</t>
         </is>
       </c>
     </row>
@@ -3886,32 +3886,32 @@
       </c>
       <c r="C84" s="1" t="inlineStr">
         <is>
-          <t>MM-662M</t>
+          <t>MM-661M</t>
         </is>
       </c>
       <c r="D84" s="1" t="inlineStr">
         <is>
-          <t>MM-872M</t>
+          <t>MM-868M</t>
         </is>
       </c>
       <c r="E84" s="1" t="inlineStr">
         <is>
-          <t>MM-9926M</t>
+          <t>MM-9924M</t>
         </is>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>NR25</t>
+          <t>NR21</t>
         </is>
       </c>
       <c r="G84" s="1" t="inlineStr">
         <is>
-          <t>NR108</t>
+          <t>NR105</t>
         </is>
       </c>
       <c r="H84" s="1" t="inlineStr">
         <is>
-          <t>QL001</t>
+          <t>QE006</t>
         </is>
       </c>
     </row>
@@ -3928,32 +3928,32 @@
       </c>
       <c r="C85" s="1" t="inlineStr">
         <is>
-          <t>MM-664M</t>
+          <t>MM-662M</t>
         </is>
       </c>
       <c r="D85" s="1" t="inlineStr">
         <is>
-          <t>MM-874M</t>
+          <t>MM-872M</t>
         </is>
       </c>
       <c r="E85" s="1" t="inlineStr">
         <is>
-          <t>MM-9928M</t>
+          <t>MM-9926M</t>
         </is>
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>NR27</t>
+          <t>NR25</t>
         </is>
       </c>
       <c r="G85" s="1" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR108</t>
         </is>
       </c>
       <c r="H85" s="1" t="inlineStr">
         <is>
-          <t>QL002</t>
+          <t>QL001</t>
         </is>
       </c>
     </row>
@@ -3970,32 +3970,32 @@
       </c>
       <c r="C86" s="1" t="inlineStr">
         <is>
-          <t>MM-666M</t>
+          <t>MM-664M</t>
         </is>
       </c>
       <c r="D86" s="1" t="inlineStr">
         <is>
-          <t>MM-876M</t>
+          <t>MM-874M</t>
         </is>
       </c>
       <c r="E86" s="1" t="inlineStr">
         <is>
-          <t>MM-9929M</t>
+          <t>MM-9928M</t>
         </is>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>NR28</t>
+          <t>NR27</t>
         </is>
       </c>
       <c r="G86" s="1" t="inlineStr">
         <is>
-          <t>NR110</t>
+          <t>NR109</t>
         </is>
       </c>
       <c r="H86" s="1" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>QL002</t>
         </is>
       </c>
     </row>
@@ -4012,32 +4012,32 @@
       </c>
       <c r="C87" s="1" t="inlineStr">
         <is>
-          <t>MM-668M</t>
+          <t>MM-666M</t>
         </is>
       </c>
       <c r="D87" s="1" t="inlineStr">
         <is>
-          <t>MM-882M</t>
+          <t>MM-876M</t>
         </is>
       </c>
       <c r="E87" s="1" t="inlineStr">
         <is>
-          <t>MM-9932M</t>
+          <t>MM-9929M</t>
         </is>
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>NR30</t>
+          <t>NR28</t>
         </is>
       </c>
       <c r="G87" s="1" t="inlineStr">
         <is>
-          <t>NR111</t>
+          <t>NR110</t>
         </is>
       </c>
       <c r="H87" s="1" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>QL004</t>
         </is>
       </c>
     </row>
@@ -4054,32 +4054,32 @@
       </c>
       <c r="C88" s="1" t="inlineStr">
         <is>
-          <t>MM-673M</t>
+          <t>MM-668M</t>
         </is>
       </c>
       <c r="D88" s="1" t="inlineStr">
         <is>
-          <t>MM-894M</t>
+          <t>MM-882M</t>
         </is>
       </c>
       <c r="E88" s="1" t="inlineStr">
         <is>
-          <t>MM-9933M</t>
+          <t>MM-9932M</t>
         </is>
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>NR31</t>
+          <t>NR30</t>
         </is>
       </c>
       <c r="G88" s="1" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR111</t>
         </is>
       </c>
       <c r="H88" s="1" t="inlineStr">
         <is>
-          <t>QL008</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
@@ -4096,32 +4096,32 @@
       </c>
       <c r="C89" s="1" t="inlineStr">
         <is>
-          <t>MM-674M</t>
+          <t>MM-673M</t>
         </is>
       </c>
       <c r="D89" s="1" t="inlineStr">
         <is>
-          <t>MM-896M</t>
+          <t>MM-894M</t>
         </is>
       </c>
       <c r="E89" s="1" t="inlineStr">
         <is>
-          <t>MM-9934M</t>
+          <t>MM-9933M</t>
         </is>
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>NR34</t>
+          <t>NR31</t>
         </is>
       </c>
       <c r="G89" s="1" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR112</t>
         </is>
       </c>
       <c r="H89" s="1" t="inlineStr">
         <is>
-          <t>QL010</t>
+          <t>QL008</t>
         </is>
       </c>
     </row>
@@ -4138,32 +4138,32 @@
       </c>
       <c r="C90" s="1" t="inlineStr">
         <is>
-          <t>MM-680M</t>
+          <t>MM-674M</t>
         </is>
       </c>
       <c r="D90" s="1" t="inlineStr">
         <is>
-          <t>MM-902M</t>
+          <t>MM-896M</t>
         </is>
       </c>
       <c r="E90" s="1" t="inlineStr">
         <is>
-          <t>MM-9936M</t>
+          <t>MM-9934M</t>
         </is>
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>NR36</t>
+          <t>NR34</t>
         </is>
       </c>
       <c r="G90" s="1" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR113</t>
         </is>
       </c>
       <c r="H90" s="1" t="inlineStr">
         <is>
-          <t>QL011</t>
+          <t>QL010</t>
         </is>
       </c>
     </row>
@@ -4180,32 +4180,32 @@
       </c>
       <c r="C91" s="1" t="inlineStr">
         <is>
-          <t>MM-708M</t>
+          <t>MM-680M</t>
         </is>
       </c>
       <c r="D91" s="1" t="inlineStr">
         <is>
-          <t>MM-904M</t>
+          <t>MM-902M</t>
         </is>
       </c>
       <c r="E91" s="1" t="inlineStr">
         <is>
-          <t>MM-9938M</t>
+          <t>MM-9936M</t>
         </is>
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>NR36</t>
         </is>
       </c>
       <c r="G91" s="1" t="inlineStr">
         <is>
-          <t>NR118</t>
+          <t>NR115</t>
         </is>
       </c>
       <c r="H91" s="1" t="inlineStr">
         <is>
-          <t>QL014</t>
+          <t>QL011</t>
         </is>
       </c>
     </row>
@@ -4222,32 +4222,32 @@
       </c>
       <c r="C92" s="1" t="inlineStr">
         <is>
-          <t>MM-710M</t>
+          <t>MM-708M</t>
         </is>
       </c>
       <c r="D92" s="1" t="inlineStr">
         <is>
-          <t>MM-906M</t>
+          <t>MM-904M</t>
         </is>
       </c>
       <c r="E92" s="1" t="inlineStr">
         <is>
-          <t>MM-9941M</t>
+          <t>MM-9938M</t>
         </is>
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>NR38</t>
+          <t>NR37</t>
         </is>
       </c>
       <c r="G92" s="1" t="inlineStr">
         <is>
-          <t>NR119</t>
+          <t>NR118</t>
         </is>
       </c>
       <c r="H92" s="1" t="inlineStr">
         <is>
-          <t>QL018</t>
+          <t>QL014</t>
         </is>
       </c>
     </row>
@@ -4264,32 +4264,32 @@
       </c>
       <c r="C93" s="1" t="inlineStr">
         <is>
-          <t>MM-716M</t>
+          <t>MM-710M</t>
         </is>
       </c>
       <c r="D93" s="1" t="inlineStr">
         <is>
-          <t>MM-908M</t>
+          <t>MM-906M</t>
         </is>
       </c>
       <c r="E93" s="1" t="inlineStr">
         <is>
-          <t>MM-9943M</t>
+          <t>MM-9941M</t>
         </is>
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>NR39</t>
+          <t>NR38</t>
         </is>
       </c>
       <c r="G93" s="1" t="inlineStr">
         <is>
-          <t>NR120</t>
+          <t>NR119</t>
         </is>
       </c>
       <c r="H93" s="1" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QL018</t>
         </is>
       </c>
     </row>
@@ -4306,32 +4306,32 @@
       </c>
       <c r="C94" s="1" t="inlineStr">
         <is>
-          <t>MM-722M</t>
+          <t>MM-716M</t>
         </is>
       </c>
       <c r="D94" s="1" t="inlineStr">
         <is>
-          <t>MM-910M</t>
+          <t>MM-908M</t>
         </is>
       </c>
       <c r="E94" s="1" t="inlineStr">
         <is>
-          <t>MM-9945M</t>
+          <t>MM-9943M</t>
         </is>
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>NR40</t>
+          <t>NR39</t>
         </is>
       </c>
       <c r="G94" s="1" t="inlineStr">
         <is>
-          <t>NR122</t>
+          <t>NR120</t>
         </is>
       </c>
       <c r="H94" s="1" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QR1744</t>
         </is>
       </c>
     </row>
@@ -4348,32 +4348,32 @@
       </c>
       <c r="C95" s="1" t="inlineStr">
         <is>
-          <t>MM-726M</t>
+          <t>MM-722M</t>
         </is>
       </c>
       <c r="D95" s="1" t="inlineStr">
         <is>
-          <t>MM-912M</t>
+          <t>MM-910M</t>
         </is>
       </c>
       <c r="E95" s="1" t="inlineStr">
         <is>
-          <t>MM-9946M</t>
+          <t>MM-9945M</t>
         </is>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>NR43</t>
+          <t>NR40</t>
         </is>
       </c>
       <c r="G95" s="1" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>NR122</t>
         </is>
       </c>
       <c r="H95" s="1" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QR1771</t>
         </is>
       </c>
     </row>
@@ -4390,32 +4390,32 @@
       </c>
       <c r="C96" s="1" t="inlineStr">
         <is>
-          <t>MM-728M</t>
+          <t>MM-726M</t>
         </is>
       </c>
       <c r="D96" s="1" t="inlineStr">
         <is>
-          <t>MM-914M</t>
+          <t>MM-912M</t>
         </is>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>MM-9950M</t>
+          <t>MM-9946M</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>NR44</t>
+          <t>NR43</t>
         </is>
       </c>
       <c r="G96" s="1" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="H96" s="1" t="inlineStr">
         <is>
-          <t>R711</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
@@ -4432,32 +4432,32 @@
       </c>
       <c r="C97" s="1" t="inlineStr">
         <is>
-          <t>MM-734M</t>
+          <t>MM-728M</t>
         </is>
       </c>
       <c r="D97" s="1" t="inlineStr">
         <is>
-          <t>MM-920M</t>
+          <t>MM-914M</t>
         </is>
       </c>
       <c r="E97" s="1" t="inlineStr">
         <is>
-          <t>MM-9951M</t>
+          <t>MM-9950M</t>
         </is>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>NR45</t>
+          <t>NR44</t>
         </is>
       </c>
       <c r="G97" s="1" t="inlineStr">
         <is>
-          <t>P2501</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="H97" s="1" t="inlineStr">
         <is>
-          <t>R766</t>
+          <t>R711</t>
         </is>
       </c>
     </row>
@@ -4474,32 +4474,32 @@
       </c>
       <c r="C98" s="1" t="inlineStr">
         <is>
-          <t>MM-736M</t>
+          <t>MM-734M</t>
         </is>
       </c>
       <c r="D98" s="1" t="inlineStr">
         <is>
-          <t>MM-922M</t>
+          <t>MM-920M</t>
         </is>
       </c>
       <c r="E98" s="1" t="inlineStr">
         <is>
-          <t>MM-9952M</t>
+          <t>MM-9951M</t>
         </is>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>NR48</t>
+          <t>NR45</t>
         </is>
       </c>
       <c r="G98" s="1" t="inlineStr">
         <is>
-          <t>P2502</t>
+          <t>P2501</t>
         </is>
       </c>
       <c r="H98" s="1" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>R766</t>
         </is>
       </c>
     </row>
@@ -4516,32 +4516,32 @@
       </c>
       <c r="C99" s="1" t="inlineStr">
         <is>
-          <t>MM-738M</t>
+          <t>MM-736M</t>
         </is>
       </c>
       <c r="D99" s="1" t="inlineStr">
         <is>
-          <t>MM-924M</t>
+          <t>MM-922M</t>
         </is>
       </c>
       <c r="E99" s="1" t="inlineStr">
         <is>
-          <t>MM-9953M</t>
+          <t>MM-9952M</t>
         </is>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>NR51</t>
+          <t>NR48</t>
         </is>
       </c>
       <c r="G99" s="1" t="inlineStr">
         <is>
-          <t>P2503</t>
+          <t>P2502</t>
         </is>
       </c>
       <c r="H99" s="1" t="inlineStr">
         <is>
-          <t>RCTST4</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
@@ -4558,32 +4558,32 @@
       </c>
       <c r="C100" s="1" t="inlineStr">
         <is>
-          <t>MM-740M</t>
+          <t>MM-738M</t>
         </is>
       </c>
       <c r="D100" s="1" t="inlineStr">
         <is>
-          <t>MM-926M</t>
+          <t>MM-924M</t>
         </is>
       </c>
       <c r="E100" s="1" t="inlineStr">
         <is>
-          <t>MM-9954M</t>
+          <t>MM-9953M</t>
         </is>
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>NR52</t>
+          <t>NR51</t>
         </is>
       </c>
       <c r="G100" s="1" t="inlineStr">
         <is>
-          <t>P2505</t>
+          <t>P2503</t>
         </is>
       </c>
       <c r="H100" s="1" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>RCTST4</t>
         </is>
       </c>
     </row>
@@ -4600,32 +4600,32 @@
       </c>
       <c r="C101" s="1" t="inlineStr">
         <is>
-          <t>MM-742M</t>
+          <t>MM-740M</t>
         </is>
       </c>
       <c r="D101" s="1" t="inlineStr">
         <is>
-          <t>MM-934M</t>
+          <t>MM-926M</t>
         </is>
       </c>
       <c r="E101" s="1" t="inlineStr">
         <is>
-          <t>MM-9955M</t>
+          <t>MM-9954M</t>
         </is>
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>NR53</t>
+          <t>NR52</t>
         </is>
       </c>
       <c r="G101" s="1" t="inlineStr">
         <is>
-          <t>P2506</t>
+          <t>P2505</t>
         </is>
       </c>
       <c r="H101" s="1" t="inlineStr">
         <is>
-          <t>RL302</t>
+          <t>RL301</t>
         </is>
       </c>
     </row>
@@ -4642,32 +4642,32 @@
       </c>
       <c r="C102" s="1" t="inlineStr">
         <is>
-          <t>MM-744M</t>
+          <t>MM-742M</t>
         </is>
       </c>
       <c r="D102" s="1" t="inlineStr">
         <is>
-          <t>MM-936M</t>
+          <t>MM-934M</t>
         </is>
       </c>
       <c r="E102" s="1" t="inlineStr">
         <is>
-          <t>MM-9957M</t>
+          <t>MM-9955M</t>
         </is>
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>NR53</t>
         </is>
       </c>
       <c r="G102" s="1" t="inlineStr">
         <is>
-          <t>P2507</t>
+          <t>P2506</t>
         </is>
       </c>
       <c r="H102" s="1" t="inlineStr">
         <is>
-          <t>RL304</t>
+          <t>RL302</t>
         </is>
       </c>
     </row>
@@ -4684,32 +4684,32 @@
       </c>
       <c r="C103" s="1" t="inlineStr">
         <is>
-          <t>MM-752M</t>
+          <t>MM-744M</t>
         </is>
       </c>
       <c r="D103" s="1" t="inlineStr">
         <is>
-          <t>MM-940M</t>
+          <t>MM-936M</t>
         </is>
       </c>
       <c r="E103" s="1" t="inlineStr">
         <is>
-          <t>MM-9959M</t>
+          <t>MM-9957M</t>
         </is>
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>NR57</t>
+          <t>NR54</t>
         </is>
       </c>
       <c r="G103" s="1" t="inlineStr">
         <is>
-          <t>P2508</t>
+          <t>P2507</t>
         </is>
       </c>
       <c r="H103" s="1" t="inlineStr">
         <is>
-          <t>RL305</t>
+          <t>RL304</t>
         </is>
       </c>
     </row>
@@ -4726,32 +4726,32 @@
       </c>
       <c r="C104" s="1" t="inlineStr">
         <is>
-          <t>MM-756M</t>
+          <t>MM-752M</t>
         </is>
       </c>
       <c r="D104" s="1" t="inlineStr">
         <is>
-          <t>MM-944M</t>
+          <t>MM-940M</t>
         </is>
       </c>
       <c r="E104" s="1" t="inlineStr">
         <is>
-          <t>MM-9960M</t>
+          <t>MM-9959M</t>
         </is>
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>NR59</t>
+          <t>NR57</t>
         </is>
       </c>
       <c r="G104" s="1" t="inlineStr">
         <is>
-          <t>P2509</t>
+          <t>P2508</t>
         </is>
       </c>
       <c r="H104" s="1" t="inlineStr">
         <is>
-          <t>RL307</t>
+          <t>RL305</t>
         </is>
       </c>
     </row>
@@ -4768,32 +4768,32 @@
       </c>
       <c r="C105" s="1" t="inlineStr">
         <is>
-          <t>MM-760M</t>
+          <t>MM-756M</t>
         </is>
       </c>
       <c r="D105" s="1" t="inlineStr">
         <is>
-          <t>MM-948M</t>
+          <t>MM-944M</t>
         </is>
       </c>
       <c r="E105" s="1" t="inlineStr">
         <is>
-          <t>MM-9961M</t>
+          <t>MM-9960M</t>
         </is>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>NR61</t>
+          <t>NR59</t>
         </is>
       </c>
       <c r="G105" s="1" t="inlineStr">
         <is>
-          <t>P2510</t>
+          <t>P2509</t>
         </is>
       </c>
       <c r="H105" s="1" t="inlineStr">
         <is>
-          <t>RL309</t>
+          <t>RL307</t>
         </is>
       </c>
     </row>
@@ -4810,32 +4810,32 @@
       </c>
       <c r="C106" s="1" t="inlineStr">
         <is>
-          <t>MM-764M</t>
+          <t>MM-760M</t>
         </is>
       </c>
       <c r="D106" s="1" t="inlineStr">
         <is>
-          <t>MM-952M</t>
+          <t>MM-948M</t>
         </is>
       </c>
       <c r="E106" s="1" t="inlineStr">
         <is>
-          <t>MM-9962M</t>
+          <t>MM-9961M</t>
         </is>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>NR62</t>
+          <t>NR61</t>
         </is>
       </c>
       <c r="G106" s="1" t="inlineStr">
         <is>
-          <t>P2511</t>
+          <t>P2510</t>
         </is>
       </c>
       <c r="H106" s="1" t="inlineStr">
         <is>
-          <t>RL310</t>
+          <t>RL309</t>
         </is>
       </c>
     </row>
@@ -4852,32 +4852,32 @@
       </c>
       <c r="C107" s="1" t="inlineStr">
         <is>
-          <t>MM-768M</t>
+          <t>MM-764M</t>
         </is>
       </c>
       <c r="D107" s="1" t="inlineStr">
         <is>
-          <t>MM-954M</t>
+          <t>MM-952M</t>
         </is>
       </c>
       <c r="E107" s="1" t="inlineStr">
         <is>
-          <t>MM-9963M</t>
+          <t>MM-9962M</t>
         </is>
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR62</t>
         </is>
       </c>
       <c r="G107" s="1" t="inlineStr">
         <is>
-          <t>P2513</t>
+          <t>P2511</t>
         </is>
       </c>
       <c r="H107" s="1" t="inlineStr">
         <is>
-          <t>S312</t>
+          <t>RL310</t>
         </is>
       </c>
     </row>
@@ -4894,32 +4894,32 @@
       </c>
       <c r="C108" s="1" t="inlineStr">
         <is>
-          <t>MM-774M</t>
+          <t>MM-768M</t>
         </is>
       </c>
       <c r="D108" s="1" t="inlineStr">
         <is>
-          <t>MM-956M</t>
+          <t>MM-954M</t>
         </is>
       </c>
       <c r="E108" s="1" t="inlineStr">
         <is>
-          <t>MM-9964M</t>
+          <t>MM-9963M</t>
         </is>
       </c>
       <c r="F108" s="1" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR64</t>
         </is>
       </c>
       <c r="G108" s="1" t="inlineStr">
         <is>
-          <t>P2514</t>
+          <t>P2513</t>
         </is>
       </c>
       <c r="H108" s="1" t="inlineStr">
         <is>
-          <t>S317</t>
+          <t>S312</t>
         </is>
       </c>
     </row>
@@ -4936,32 +4936,32 @@
       </c>
       <c r="C109" s="1" t="inlineStr">
         <is>
-          <t>MM-776M</t>
+          <t>MM-774M</t>
         </is>
       </c>
       <c r="D109" s="1" t="inlineStr">
         <is>
-          <t>MM-958M</t>
+          <t>MM-956M</t>
         </is>
       </c>
       <c r="E109" s="1" t="inlineStr">
         <is>
-          <t>MM-9965M</t>
+          <t>MM-9964M</t>
         </is>
       </c>
       <c r="F109" s="1" t="inlineStr">
         <is>
-          <t>NR66</t>
+          <t>NR65</t>
         </is>
       </c>
       <c r="G109" s="1" t="inlineStr">
         <is>
-          <t>P2515</t>
+          <t>P2514</t>
         </is>
       </c>
       <c r="H109" s="1" t="inlineStr">
         <is>
-          <t>S3301</t>
+          <t>S317</t>
         </is>
       </c>
     </row>
@@ -4978,32 +4978,32 @@
       </c>
       <c r="C110" s="1" t="inlineStr">
         <is>
-          <t>MM-778M</t>
+          <t>MM-776M</t>
         </is>
       </c>
       <c r="D110" s="1" t="inlineStr">
         <is>
-          <t>MM-962M</t>
+          <t>MM-958M</t>
         </is>
       </c>
       <c r="E110" s="1" t="inlineStr">
         <is>
-          <t>MM-9966M</t>
+          <t>MM-9965M</t>
         </is>
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>NR67</t>
+          <t>NR66</t>
         </is>
       </c>
       <c r="G110" s="1" t="inlineStr">
         <is>
-          <t>P2516</t>
+          <t>P2515</t>
         </is>
       </c>
       <c r="H110" s="1" t="inlineStr">
         <is>
-          <t>S3302</t>
+          <t>S3301</t>
         </is>
       </c>
     </row>
@@ -5020,32 +5020,32 @@
       </c>
       <c r="C111" s="1" t="inlineStr">
         <is>
-          <t>MM-780M</t>
+          <t>MM-778M</t>
         </is>
       </c>
       <c r="D111" s="1" t="inlineStr">
         <is>
-          <t>MM-964M</t>
+          <t>MM-962M</t>
         </is>
       </c>
       <c r="E111" s="1" t="inlineStr">
         <is>
-          <t>MM-9967M</t>
+          <t>MM-9966M</t>
         </is>
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR67</t>
         </is>
       </c>
       <c r="G111" s="1" t="inlineStr">
         <is>
-          <t>PB1</t>
+          <t>P2516</t>
         </is>
       </c>
       <c r="H111" s="1" t="inlineStr">
         <is>
-          <t>S3304</t>
+          <t>S3302</t>
         </is>
       </c>
     </row>
@@ -5062,32 +5062,32 @@
       </c>
       <c r="C112" s="1" t="inlineStr">
         <is>
-          <t>MM-784M</t>
+          <t>MM-780M</t>
         </is>
       </c>
       <c r="D112" s="1" t="inlineStr">
         <is>
-          <t>MM-966M</t>
+          <t>MM-964M</t>
         </is>
       </c>
       <c r="E112" s="1" t="inlineStr">
         <is>
-          <t>MM-9969M</t>
+          <t>MM-9967M</t>
         </is>
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>NR69</t>
+          <t>NR68</t>
         </is>
       </c>
       <c r="G112" s="1" t="inlineStr">
         <is>
-          <t>PB2</t>
+          <t>PB1</t>
         </is>
       </c>
       <c r="H112" s="1" t="inlineStr">
         <is>
-          <t>S3305</t>
+          <t>S3304</t>
         </is>
       </c>
     </row>
@@ -5104,2084 +5104,2089 @@
       </c>
       <c r="C113" s="1" t="inlineStr">
         <is>
-          <t>MM-790M</t>
+          <t>MM-784M</t>
         </is>
       </c>
       <c r="D113" s="1" t="inlineStr">
         <is>
-          <t>MM-968M</t>
+          <t>MM-966M</t>
         </is>
       </c>
       <c r="E113" s="1" t="inlineStr">
         <is>
-          <t>MM-9970M</t>
+          <t>MM-9969M</t>
         </is>
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>NR71</t>
+          <t>NR69</t>
         </is>
       </c>
       <c r="G113" s="1" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>PB2</t>
         </is>
       </c>
       <c r="H113" s="1" t="inlineStr">
         <is>
-          <t>S3306</t>
+          <t>S3305</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>S3307</t>
+          <t>S3306</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TT106</t>
         </is>
       </c>
       <c r="C115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8107</t>
+          <t>VLINE-8104</t>
         </is>
       </c>
       <c r="D115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8306</t>
+          <t>VLINE-8304</t>
         </is>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8447</t>
+          <t>VLINE-8446</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8753</t>
+          <t>VLINE-8752</t>
         </is>
       </c>
       <c r="G115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8818</t>
+          <t>VLINE-8817</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>S3309</t>
+          <t>S3307</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
         <is>
-          <t>TT108</t>
+          <t>TT107</t>
         </is>
       </c>
       <c r="C116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8110</t>
+          <t>VLINE-8107</t>
         </is>
       </c>
       <c r="D116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8311</t>
+          <t>VLINE-8306</t>
         </is>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8449</t>
+          <t>VLINE-8447</t>
         </is>
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8754</t>
+          <t>VLINE-8753</t>
         </is>
       </c>
       <c r="G116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8819</t>
+          <t>VLINE-8818</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>S3310</t>
+          <t>S3309</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TT108</t>
         </is>
       </c>
       <c r="C117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8111</t>
+          <t>VLINE-8110</t>
         </is>
       </c>
       <c r="D117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8313</t>
+          <t>VLINE-8311</t>
         </is>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8450</t>
+          <t>VLINE-8449</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8755</t>
+          <t>VLINE-8754</t>
         </is>
       </c>
       <c r="G117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8822</t>
+          <t>VLINE-8819</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>S7001</t>
+          <t>S3310</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
         <is>
-          <t>TT113</t>
+          <t>TT110</t>
         </is>
       </c>
       <c r="C118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8113</t>
+          <t>VLINE-8111</t>
         </is>
       </c>
       <c r="D118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8314</t>
+          <t>VLINE-8313</t>
         </is>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8451</t>
+          <t>VLINE-8450</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8756</t>
+          <t>VLINE-8755</t>
         </is>
       </c>
       <c r="G118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8860</t>
+          <t>VLINE-8822</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>S7002</t>
+          <t>S7001</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
         <is>
-          <t>TT114</t>
+          <t>TT113</t>
         </is>
       </c>
       <c r="C119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8114</t>
+          <t>VLINE-8113</t>
         </is>
       </c>
       <c r="D119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8316</t>
+          <t>VLINE-8314</t>
         </is>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8452</t>
+          <t>VLINE-8451</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8757</t>
+          <t>VLINE-8756</t>
         </is>
       </c>
       <c r="G119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8861</t>
+          <t>VLINE-8860</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>S7003</t>
+          <t>S7002</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT114</t>
         </is>
       </c>
       <c r="C120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8115</t>
+          <t>VLINE-8114</t>
         </is>
       </c>
       <c r="D120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8318</t>
+          <t>VLINE-8316</t>
         </is>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8453</t>
+          <t>VLINE-8452</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8758</t>
+          <t>VLINE-8757</t>
         </is>
       </c>
       <c r="G120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8862</t>
+          <t>VLINE-8861</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>S7005</t>
+          <t>S7003</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
         <is>
-          <t>TT116</t>
+          <t>TT115</t>
         </is>
       </c>
       <c r="C121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8119</t>
+          <t>VLINE-8115</t>
         </is>
       </c>
       <c r="D121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8321</t>
+          <t>VLINE-8318</t>
         </is>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8454</t>
+          <t>VLINE-8453</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8759</t>
+          <t>VLINE-8758</t>
         </is>
       </c>
       <c r="G121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8863</t>
+          <t>VLINE-8862</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>S7006</t>
+          <t>S7005</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT116</t>
         </is>
       </c>
       <c r="C122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8120</t>
+          <t>VLINE-8119</t>
         </is>
       </c>
       <c r="D122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8323</t>
+          <t>VLINE-8321</t>
         </is>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8455</t>
+          <t>VLINE-8454</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8760</t>
+          <t>VLINE-8759</t>
         </is>
       </c>
       <c r="G122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8864</t>
+          <t>VLINE-8863</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>S7007</t>
+          <t>S7006</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
         <is>
-          <t>TT122</t>
+          <t>TT117</t>
         </is>
       </c>
       <c r="C123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8121</t>
+          <t>VLINE-8120</t>
         </is>
       </c>
       <c r="D123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8324</t>
+          <t>VLINE-8323</t>
         </is>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8456</t>
+          <t>VLINE-8455</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8761</t>
+          <t>VLINE-8760</t>
         </is>
       </c>
       <c r="G123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8865</t>
+          <t>VLINE-8864</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>S7008</t>
+          <t>S7007</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
         <is>
-          <t>TT127</t>
+          <t>TT122</t>
         </is>
       </c>
       <c r="C124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8123</t>
+          <t>VLINE-8121</t>
         </is>
       </c>
       <c r="D124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8325</t>
+          <t>VLINE-8324</t>
         </is>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8457</t>
+          <t>VLINE-8456</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8762</t>
+          <t>VLINE-8761</t>
         </is>
       </c>
       <c r="G124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8866</t>
+          <t>VLINE-8865</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>S7012</t>
+          <t>S7008</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
         <is>
-          <t>TT128</t>
+          <t>TT127</t>
         </is>
       </c>
       <c r="C125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8124</t>
+          <t>VLINE-8123</t>
         </is>
       </c>
       <c r="D125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8328</t>
+          <t>VLINE-8325</t>
         </is>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8460</t>
+          <t>VLINE-8457</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8763</t>
+          <t>VLINE-8762</t>
         </is>
       </c>
       <c r="G125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8867</t>
+          <t>VLINE-8866</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>S7014</t>
+          <t>S7012</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT128</t>
         </is>
       </c>
       <c r="C126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8126</t>
+          <t>VLINE-8124</t>
         </is>
       </c>
       <c r="D126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8329</t>
+          <t>VLINE-8328</t>
         </is>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8461</t>
+          <t>VLINE-8460</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8765</t>
+          <t>VLINE-8763</t>
         </is>
       </c>
       <c r="G126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8868</t>
+          <t>VLINE-8867</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>S7015</t>
+          <t>S7014</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
         <is>
-          <t>TT131</t>
+          <t>TT130</t>
         </is>
       </c>
       <c r="C127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8127</t>
+          <t>VLINE-8126</t>
         </is>
       </c>
       <c r="D127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8332</t>
+          <t>VLINE-8329</t>
         </is>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8464</t>
+          <t>VLINE-8461</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8766</t>
+          <t>VLINE-8765</t>
         </is>
       </c>
       <c r="G127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8869</t>
+          <t>VLINE-8868</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>S7017</t>
+          <t>S7015</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT131</t>
         </is>
       </c>
       <c r="C128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8128</t>
+          <t>VLINE-8127</t>
         </is>
       </c>
       <c r="D128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8336</t>
+          <t>VLINE-8332</t>
         </is>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8465</t>
+          <t>VLINE-8464</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8767</t>
+          <t>VLINE-8766</t>
         </is>
       </c>
       <c r="G128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8890</t>
+          <t>VLINE-8869</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>S7018</t>
+          <t>S7017</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT202</t>
         </is>
       </c>
       <c r="C129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8129</t>
+          <t>VLINE-8128</t>
         </is>
       </c>
       <c r="D129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8337</t>
+          <t>VLINE-8336</t>
         </is>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8468</t>
+          <t>VLINE-8465</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8768</t>
+          <t>VLINE-8767</t>
         </is>
       </c>
       <c r="G129" s="1" t="inlineStr">
         <is>
-          <t>WH001</t>
+          <t>VLINE-8890</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>S7020</t>
+          <t>S7018</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
         <is>
-          <t>VL352</t>
+          <t>TT206</t>
         </is>
       </c>
       <c r="C130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8131</t>
+          <t>VLINE-8129</t>
         </is>
       </c>
       <c r="D130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8338</t>
+          <t>VLINE-8337</t>
         </is>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8469</t>
+          <t>VLINE-8468</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8769</t>
+          <t>VLINE-8768</t>
         </is>
       </c>
       <c r="G130" s="1" t="inlineStr">
         <is>
-          <t>WH003</t>
+          <t>WH001</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>S7022</t>
+          <t>S7020</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
         <is>
-          <t>VL353</t>
+          <t>VL352</t>
         </is>
       </c>
       <c r="C131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8132</t>
+          <t>VLINE-8131</t>
         </is>
       </c>
       <c r="D131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8339</t>
+          <t>VLINE-8338</t>
         </is>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8605</t>
+          <t>VLINE-8469</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8770</t>
+          <t>VLINE-8769</t>
         </is>
       </c>
       <c r="G131" s="1" t="inlineStr">
         <is>
-          <t>WL02</t>
+          <t>WH003</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>S7022</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
         <is>
-          <t>VL357</t>
+          <t>VL353</t>
         </is>
       </c>
       <c r="C132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8133</t>
+          <t>VLINE-8132</t>
         </is>
       </c>
       <c r="D132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8362</t>
+          <t>VLINE-8339</t>
         </is>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8610</t>
+          <t>VLINE-8605</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8772</t>
+          <t>VLINE-8770</t>
         </is>
       </c>
       <c r="G132" s="1" t="inlineStr">
         <is>
-          <t>X12-X14</t>
+          <t>WL02</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>SCT002</t>
+          <t>SCT001</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8004</t>
+          <t>VL357</t>
         </is>
       </c>
       <c r="C133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8134</t>
+          <t>VLINE-8133</t>
         </is>
       </c>
       <c r="D133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8363</t>
+          <t>VLINE-8362</t>
         </is>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8612</t>
+          <t>VLINE-8610</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8773</t>
+          <t>VLINE-8772</t>
         </is>
       </c>
       <c r="G133" s="1" t="inlineStr">
         <is>
-          <t>X31</t>
+          <t>X12-X14</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>SCT006</t>
+          <t>SCT002</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8007</t>
+          <t>VLINE-8004</t>
         </is>
       </c>
       <c r="C134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8136</t>
+          <t>VLINE-8134</t>
         </is>
       </c>
       <c r="D134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8365</t>
+          <t>VLINE-8363</t>
         </is>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8615</t>
+          <t>VLINE-8612</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8774</t>
+          <t>VLINE-8773</t>
         </is>
       </c>
       <c r="G134" s="1" t="inlineStr">
         <is>
-          <t>XP2000</t>
+          <t>X31</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>SCT007</t>
+          <t>SCT006</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8011</t>
+          <t>VLINE-8007</t>
         </is>
       </c>
       <c r="C135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8137</t>
+          <t>VLINE-8136</t>
         </is>
       </c>
       <c r="D135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8366</t>
+          <t>VLINE-8365</t>
         </is>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8617</t>
+          <t>VLINE-8615</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8776</t>
+          <t>VLINE-8774</t>
         </is>
       </c>
       <c r="G135" s="1" t="inlineStr">
         <is>
-          <t>XP2003</t>
+          <t>XP2000</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>SCT007</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8013</t>
+          <t>VLINE-8011</t>
         </is>
       </c>
       <c r="C136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8140</t>
+          <t>VLINE-8137</t>
         </is>
       </c>
       <c r="D136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8368</t>
+          <t>VLINE-8366</t>
         </is>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8620</t>
+          <t>VLINE-8617</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8778</t>
+          <t>VLINE-8776</t>
         </is>
       </c>
       <c r="G136" s="1" t="inlineStr">
         <is>
-          <t>XP2004</t>
+          <t>XP2003</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>SCT011</t>
+          <t>SCT009</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8019</t>
+          <t>VLINE-8013</t>
         </is>
       </c>
       <c r="C137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8141</t>
+          <t>VLINE-8140</t>
         </is>
       </c>
       <c r="D137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8369</t>
+          <t>VLINE-8368</t>
         </is>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8625</t>
+          <t>VLINE-8620</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8779</t>
+          <t>VLINE-8778</t>
         </is>
       </c>
       <c r="G137" s="1" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>XP2004</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>SCT011</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8020</t>
+          <t>VLINE-8019</t>
         </is>
       </c>
       <c r="C138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8142</t>
+          <t>VLINE-8141</t>
         </is>
       </c>
       <c r="D138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8403</t>
+          <t>VLINE-8369</t>
         </is>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8630</t>
+          <t>VLINE-8625</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8780</t>
+          <t>VLINE-8779</t>
         </is>
       </c>
       <c r="G138" s="1" t="inlineStr">
         <is>
-          <t>XP2007</t>
+          <t>XP2005</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>SCT014</t>
+          <t>SCT013</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8023</t>
+          <t>VLINE-8020</t>
         </is>
       </c>
       <c r="C139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8144</t>
+          <t>VLINE-8142</t>
         </is>
       </c>
       <c r="D139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8404</t>
+          <t>VLINE-8403</t>
         </is>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8671</t>
+          <t>VLINE-8630</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8781</t>
+          <t>VLINE-8780</t>
         </is>
       </c>
       <c r="G139" s="1" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>XP2007</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>SCT015</t>
+          <t>SCT014</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8025</t>
+          <t>VLINE-8023</t>
         </is>
       </c>
       <c r="C140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8145</t>
+          <t>VLINE-8144</t>
         </is>
       </c>
       <c r="D140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8406</t>
+          <t>VLINE-8404</t>
         </is>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8706</t>
+          <t>VLINE-8671</t>
         </is>
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8782</t>
+          <t>VLINE-8781</t>
         </is>
       </c>
       <c r="G140" s="1" t="inlineStr">
         <is>
-          <t>XP2010</t>
+          <t>XP2008</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>SO2</t>
+          <t>SCT015</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8026</t>
+          <t>VLINE-8025</t>
         </is>
       </c>
       <c r="C141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8148</t>
+          <t>VLINE-8145</t>
         </is>
       </c>
       <c r="D141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8408</t>
+          <t>VLINE-8406</t>
         </is>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8711</t>
+          <t>VLINE-8706</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8783</t>
+          <t>VLINE-8782</t>
         </is>
       </c>
       <c r="G141" s="1" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>XP2010</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>SO2</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8027</t>
+          <t>VLINE-8026</t>
         </is>
       </c>
       <c r="C142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8150</t>
+          <t>VLINE-8148</t>
         </is>
       </c>
       <c r="D142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8410</t>
+          <t>VLINE-8408</t>
         </is>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8714</t>
+          <t>VLINE-8711</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8784</t>
+          <t>VLINE-8783</t>
         </is>
       </c>
       <c r="G142" s="1" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>XP2011</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>SSR101</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8028</t>
+          <t>VLINE-8027</t>
         </is>
       </c>
       <c r="C143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8151</t>
+          <t>VLINE-8150</t>
         </is>
       </c>
       <c r="D143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8411</t>
+          <t>VLINE-8410</t>
         </is>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8717</t>
+          <t>VLINE-8714</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8786</t>
+          <t>VLINE-8784</t>
         </is>
       </c>
       <c r="G143" s="1" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>XP2012</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>SSR102</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8029</t>
+          <t>VLINE-8028</t>
         </is>
       </c>
       <c r="C144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8152</t>
+          <t>VLINE-8151</t>
         </is>
       </c>
       <c r="D144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8413</t>
+          <t>VLINE-8411</t>
         </is>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8720</t>
+          <t>VLINE-8717</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8787</t>
+          <t>VLINE-8786</t>
         </is>
       </c>
       <c r="G144" s="1" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>XP2013</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>SSR103</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8030</t>
+          <t>VLINE-8029</t>
         </is>
       </c>
       <c r="C145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8153</t>
+          <t>VLINE-8152</t>
         </is>
       </c>
       <c r="D145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8415</t>
+          <t>VLINE-8413</t>
         </is>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8721</t>
+          <t>VLINE-8720</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8788</t>
+          <t>VLINE-8787</t>
         </is>
       </c>
       <c r="G145" s="1" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>XP2014</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>T363</t>
+          <t>SSR104</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8031</t>
+          <t>VLINE-8030</t>
         </is>
       </c>
       <c r="C146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8154</t>
+          <t>VLINE-8153</t>
         </is>
       </c>
       <c r="D146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8417</t>
+          <t>VLINE-8415</t>
         </is>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8723</t>
+          <t>VLINE-8721</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8790</t>
+          <t>VLINE-8788</t>
         </is>
       </c>
       <c r="G146" s="1" t="inlineStr">
         <is>
-          <t>XP2016</t>
+          <t>XP2015</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>T386</t>
+          <t>T363</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8032</t>
+          <t>VLINE-8031</t>
         </is>
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8155</t>
+          <t>VLINE-8154</t>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8418</t>
+          <t>VLINE-8417</t>
         </is>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8725</t>
+          <t>VLINE-8723</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8792</t>
+          <t>VLINE-8790</t>
         </is>
       </c>
       <c r="G147" s="1" t="inlineStr">
         <is>
-          <t>XP2017</t>
+          <t>XP2016</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>TDX101</t>
+          <t>T386</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8036</t>
+          <t>VLINE-8032</t>
         </is>
       </c>
       <c r="C148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8157</t>
+          <t>VLINE-8155</t>
         </is>
       </c>
       <c r="D148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8419</t>
+          <t>VLINE-8418</t>
         </is>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8726</t>
+          <t>VLINE-8725</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8793</t>
+          <t>VLINE-8792</t>
         </is>
       </c>
       <c r="G148" s="1" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>XP2017</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>TDX101</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8038</t>
+          <t>VLINE-8036</t>
         </is>
       </c>
       <c r="C149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8158</t>
+          <t>VLINE-8157</t>
         </is>
       </c>
       <c r="D149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8420</t>
+          <t>VLINE-8419</t>
         </is>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8727</t>
+          <t>VLINE-8726</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8794</t>
+          <t>VLINE-8793</t>
         </is>
       </c>
       <c r="G149" s="1" t="inlineStr">
         <is>
-          <t>XR552</t>
+          <t>XP2019</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>TE2802</t>
+          <t>TE2801</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8042</t>
+          <t>VLINE-8038</t>
         </is>
       </c>
       <c r="C150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8159</t>
+          <t>VLINE-8158</t>
         </is>
       </c>
       <c r="D150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8421</t>
+          <t>VLINE-8420</t>
         </is>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8729</t>
+          <t>VLINE-8727</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8795</t>
+          <t>VLINE-8794</t>
         </is>
       </c>
       <c r="G150" s="1" t="inlineStr">
         <is>
-          <t>XRN001</t>
+          <t>XR552</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>TE2802</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8051</t>
+          <t>VLINE-8042</t>
         </is>
       </c>
       <c r="C151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8160</t>
+          <t>VLINE-8159</t>
         </is>
       </c>
       <c r="D151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8422</t>
+          <t>VLINE-8421</t>
         </is>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8730</t>
+          <t>VLINE-8729</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8796</t>
+          <t>VLINE-8795</t>
         </is>
       </c>
       <c r="G151" s="1" t="inlineStr">
         <is>
-          <t>XRN004</t>
+          <t>XRN001</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>TE2804</t>
+          <t>TE2803</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8052</t>
+          <t>VLINE-8051</t>
         </is>
       </c>
       <c r="C152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8161</t>
+          <t>VLINE-8160</t>
         </is>
       </c>
       <c r="D152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8424</t>
+          <t>VLINE-8422</t>
         </is>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8731</t>
+          <t>VLINE-8730</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8797</t>
+          <t>VLINE-8796</t>
         </is>
       </c>
       <c r="G152" s="1" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>XRN004</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>TE2804</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8053</t>
+          <t>VLINE-8052</t>
         </is>
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8162</t>
+          <t>VLINE-8161</t>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8425</t>
+          <t>VLINE-8424</t>
         </is>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8733</t>
+          <t>VLINE-8731</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8799</t>
+          <t>VLINE-8797</t>
         </is>
       </c>
       <c r="G153" s="1" t="inlineStr">
         <is>
-          <t>XRN006</t>
+          <t>XRN005</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>TE2806</t>
+          <t>TE2805</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8055</t>
+          <t>VLINE-8053</t>
         </is>
       </c>
       <c r="C154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8171</t>
+          <t>VLINE-8162</t>
         </is>
       </c>
       <c r="D154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8426</t>
+          <t>VLINE-8425</t>
         </is>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8735</t>
+          <t>VLINE-8733</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8800</t>
+          <t>VLINE-8799</t>
         </is>
       </c>
       <c r="G154" s="1" t="inlineStr">
         <is>
-          <t>XRN007</t>
+          <t>XRN006</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>TE2806</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8056</t>
+          <t>VLINE-8055</t>
         </is>
       </c>
       <c r="C155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8172</t>
+          <t>VLINE-8171</t>
         </is>
       </c>
       <c r="D155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8427</t>
+          <t>VLINE-8426</t>
         </is>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8736</t>
+          <t>VLINE-8735</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8801</t>
+          <t>VLINE-8800</t>
         </is>
       </c>
       <c r="G155" s="1" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>XRN007</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>TE2807</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8057</t>
+          <t>VLINE-8056</t>
         </is>
       </c>
       <c r="C156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8176</t>
+          <t>VLINE-8172</t>
         </is>
       </c>
       <c r="D156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8428</t>
+          <t>VLINE-8427</t>
         </is>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8737</t>
+          <t>VLINE-8736</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8802</t>
+          <t>VLINE-8801</t>
         </is>
       </c>
       <c r="G156" s="1" t="inlineStr">
         <is>
-          <t>XRN011</t>
+          <t>XRN009</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>TE2809</t>
+          <t>TE2808</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8058</t>
+          <t>VLINE-8057</t>
         </is>
       </c>
       <c r="C157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8179</t>
+          <t>VLINE-8176</t>
         </is>
       </c>
       <c r="D157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8429</t>
+          <t>VLINE-8428</t>
         </is>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8739</t>
+          <t>VLINE-8737</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8803</t>
+          <t>VLINE-8802</t>
         </is>
       </c>
       <c r="G157" s="1" t="inlineStr">
         <is>
-          <t>XRN014</t>
+          <t>XRN011</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>TE2810</t>
+          <t>TE2809</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8059</t>
+          <t>VLINE-8058</t>
         </is>
       </c>
       <c r="C158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8180</t>
+          <t>VLINE-8179</t>
         </is>
       </c>
       <c r="D158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8430</t>
+          <t>VLINE-8429</t>
         </is>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8740</t>
+          <t>VLINE-8739</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8804</t>
+          <t>VLINE-8803</t>
         </is>
       </c>
       <c r="G158" s="1" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>XRN014</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>TE2812</t>
+          <t>TE2810</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8061</t>
+          <t>VLINE-8059</t>
         </is>
       </c>
       <c r="C159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8181</t>
+          <t>VLINE-8180</t>
         </is>
       </c>
       <c r="D159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8431</t>
+          <t>VLINE-8430</t>
         </is>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8741</t>
+          <t>VLINE-8740</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8805</t>
+          <t>VLINE-8804</t>
         </is>
       </c>
       <c r="G159" s="1" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>XRN017</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>TE2812</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8072</t>
+          <t>VLINE-8061</t>
         </is>
       </c>
       <c r="C160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8182</t>
+          <t>VLINE-8181</t>
         </is>
       </c>
       <c r="D160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8432</t>
+          <t>VLINE-8431</t>
         </is>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8742</t>
+          <t>VLINE-8741</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8806</t>
+          <t>VLINE-8805</t>
         </is>
       </c>
       <c r="G160" s="1" t="inlineStr">
         <is>
-          <t>XRN020</t>
+          <t>XRN018</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>TE2813</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8074</t>
+          <t>VLINE-8072</t>
         </is>
       </c>
       <c r="C161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8183</t>
+          <t>VLINE-8182</t>
         </is>
       </c>
       <c r="D161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8433</t>
+          <t>VLINE-8432</t>
         </is>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8743</t>
+          <t>VLINE-8742</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8807</t>
+          <t>VLINE-8806</t>
         </is>
       </c>
       <c r="G161" s="1" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>XRN020</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>TE2814</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8075</t>
+          <t>VLINE-8074</t>
         </is>
       </c>
       <c r="C162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8184</t>
+          <t>VLINE-8183</t>
         </is>
       </c>
       <c r="D162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8434</t>
+          <t>VLINE-8433</t>
         </is>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8744</t>
+          <t>VLINE-8743</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8808</t>
+          <t>VLINE-8807</t>
         </is>
       </c>
       <c r="G162" s="1" t="inlineStr">
         <is>
-          <t>XRN023</t>
+          <t>XRN021</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>TJ107</t>
+          <t>TJ096</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8076</t>
+          <t>VLINE-8075</t>
         </is>
       </c>
       <c r="C163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8185</t>
+          <t>VLINE-8184</t>
         </is>
       </c>
       <c r="D163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8435</t>
+          <t>VLINE-8434</t>
         </is>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8745</t>
+          <t>VLINE-8744</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8809</t>
+          <t>VLINE-8808</t>
         </is>
       </c>
       <c r="G163" s="1" t="inlineStr">
         <is>
-          <t>XRN025</t>
+          <t>XRN023</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TJ107</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8077</t>
+          <t>VLINE-8076</t>
         </is>
       </c>
       <c r="C164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8186</t>
+          <t>VLINE-8185</t>
         </is>
       </c>
       <c r="D164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8438</t>
+          <t>VLINE-8435</t>
         </is>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8746</t>
+          <t>VLINE-8745</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8810</t>
+          <t>VLINE-8809</t>
         </is>
       </c>
       <c r="G164" s="1" t="inlineStr">
         <is>
-          <t>XRN026</t>
+          <t>XRN025</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TT03</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8080</t>
+          <t>VLINE-8077</t>
         </is>
       </c>
       <c r="C165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8187</t>
+          <t>VLINE-8186</t>
         </is>
       </c>
       <c r="D165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8440</t>
+          <t>VLINE-8438</t>
         </is>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8747</t>
+          <t>VLINE-8746</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8811</t>
+          <t>VLINE-8810</t>
         </is>
       </c>
       <c r="G165" s="1" t="inlineStr">
         <is>
-          <t>XRN027</t>
+          <t>XRN026</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TT04</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8081</t>
+          <t>VLINE-8080</t>
         </is>
       </c>
       <c r="C166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8188</t>
+          <t>VLINE-8187</t>
         </is>
       </c>
       <c r="D166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8441</t>
+          <t>VLINE-8440</t>
         </is>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8748</t>
+          <t>VLINE-8747</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8812</t>
+          <t>VLINE-8811</t>
         </is>
       </c>
       <c r="G166" s="1" t="inlineStr">
         <is>
-          <t>Y163</t>
+          <t>XRN027</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>TT07</t>
+          <t>TT05</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8084</t>
+          <t>VLINE-8081</t>
         </is>
       </c>
       <c r="C167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8189</t>
+          <t>VLINE-8188</t>
         </is>
       </c>
       <c r="D167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8442</t>
+          <t>VLINE-8441</t>
         </is>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8749</t>
+          <t>VLINE-8748</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8813</t>
+          <t>VLINE-8812</t>
+        </is>
+      </c>
+      <c r="G167" s="1" t="inlineStr">
+        <is>
+          <t>Y163</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TT07</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8088</t>
+          <t>VLINE-8084</t>
         </is>
       </c>
       <c r="C168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8293</t>
+          <t>VLINE-8189</t>
         </is>
       </c>
       <c r="D168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8443</t>
+          <t>VLINE-8442</t>
         </is>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8750</t>
+          <t>VLINE-8749</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8814</t>
+          <t>VLINE-8813</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TT08</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8089</t>
+          <t>VLINE-8088</t>
         </is>
       </c>
       <c r="C169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8303</t>
+          <t>VLINE-8293</t>
         </is>
       </c>
       <c r="D169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8444</t>
+          <t>VLINE-8443</t>
         </is>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8751</t>
+          <t>VLINE-8750</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8816</t>
+          <t>VLINE-8814</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>TT106</t>
+          <t>TT103</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8104</t>
+          <t>VLINE-8089</t>
         </is>
       </c>
       <c r="C170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8304</t>
+          <t>VLINE-8303</t>
         </is>
       </c>
       <c r="D170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8446</t>
+          <t>VLINE-8444</t>
         </is>
       </c>
       <c r="E170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8752</t>
+          <t>VLINE-8751</t>
         </is>
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8817</t>
+          <t>VLINE-8816</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update trains and loco export 2026-04-05 16:33:19
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -2819,7 +2819,7 @@
       </c>
       <c r="H58" s="1" t="inlineStr">
         <is>
-          <t>P2505</t>
+          <t>P2504</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2861,7 @@
       </c>
       <c r="H59" s="1" t="inlineStr">
         <is>
-          <t>P2506</t>
+          <t>P2505</t>
         </is>
       </c>
     </row>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="H60" s="1" t="inlineStr">
         <is>
-          <t>P2507</t>
+          <t>P2506</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="H61" s="1" t="inlineStr">
         <is>
-          <t>P2508</t>
+          <t>P2507</t>
         </is>
       </c>
     </row>
@@ -2987,7 +2987,7 @@
       </c>
       <c r="H62" s="1" t="inlineStr">
         <is>
-          <t>P2509</t>
+          <t>P2508</t>
         </is>
       </c>
     </row>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="H63" s="1" t="inlineStr">
         <is>
-          <t>P2510</t>
+          <t>P2509</t>
         </is>
       </c>
     </row>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="H64" s="1" t="inlineStr">
         <is>
-          <t>P2511</t>
+          <t>P2510</t>
         </is>
       </c>
     </row>
@@ -3113,7 +3113,7 @@
       </c>
       <c r="H65" s="1" t="inlineStr">
         <is>
-          <t>P2513</t>
+          <t>P2511</t>
         </is>
       </c>
     </row>
@@ -3155,7 +3155,7 @@
       </c>
       <c r="H66" s="1" t="inlineStr">
         <is>
-          <t>P2514</t>
+          <t>P2513</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
       </c>
       <c r="H67" s="1" t="inlineStr">
         <is>
-          <t>P2515</t>
+          <t>P2514</t>
         </is>
       </c>
     </row>
@@ -3239,7 +3239,7 @@
       </c>
       <c r="H68" s="1" t="inlineStr">
         <is>
-          <t>P2516</t>
+          <t>P2515</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="H69" s="1" t="inlineStr">
         <is>
-          <t>PB1</t>
+          <t>P2516</t>
         </is>
       </c>
     </row>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="H70" s="1" t="inlineStr">
         <is>
-          <t>PB2</t>
+          <t>PB1</t>
         </is>
       </c>
     </row>
@@ -3365,7 +3365,7 @@
       </c>
       <c r="H71" s="1" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>PB2</t>
         </is>
       </c>
     </row>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="H72" s="1" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>PB4</t>
         </is>
       </c>
     </row>
@@ -3449,7 +3449,7 @@
       </c>
       <c r="H73" s="1" t="inlineStr">
         <is>
-          <t>PHC002</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
@@ -3491,7 +3491,7 @@
       </c>
       <c r="H74" s="1" t="inlineStr">
         <is>
-          <t>Q4001</t>
+          <t>PHC002</t>
         </is>
       </c>
     </row>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="H75" s="1" t="inlineStr">
         <is>
-          <t>Q4003</t>
+          <t>Q4001</t>
         </is>
       </c>
     </row>
@@ -3575,7 +3575,7 @@
       </c>
       <c r="H76" s="1" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>Q4003</t>
         </is>
       </c>
     </row>
@@ -3617,7 +3617,7 @@
       </c>
       <c r="H77" s="1" t="inlineStr">
         <is>
-          <t>Q4005</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
@@ -3659,7 +3659,7 @@
       </c>
       <c r="H78" s="1" t="inlineStr">
         <is>
-          <t>Q4006</t>
+          <t>Q4005</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3701,7 @@
       </c>
       <c r="H79" s="1" t="inlineStr">
         <is>
-          <t>Q4007</t>
+          <t>Q4006</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="H80" s="1" t="inlineStr">
         <is>
-          <t>Q4009</t>
+          <t>Q4007</t>
         </is>
       </c>
     </row>
@@ -3785,7 +3785,7 @@
       </c>
       <c r="H81" s="1" t="inlineStr">
         <is>
-          <t>Q4011</t>
+          <t>Q4009</t>
         </is>
       </c>
     </row>
@@ -3827,7 +3827,7 @@
       </c>
       <c r="H82" s="1" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>Q4011</t>
         </is>
       </c>
     </row>
@@ -3869,7 +3869,7 @@
       </c>
       <c r="H83" s="1" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
@@ -3911,7 +3911,7 @@
       </c>
       <c r="H84" s="1" t="inlineStr">
         <is>
-          <t>Q4014</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
@@ -3953,7 +3953,7 @@
       </c>
       <c r="H85" s="1" t="inlineStr">
         <is>
-          <t>Q4015</t>
+          <t>Q4014</t>
         </is>
       </c>
     </row>
@@ -3995,7 +3995,7 @@
       </c>
       <c r="H86" s="1" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>Q4015</t>
         </is>
       </c>
     </row>
@@ -4037,7 +4037,7 @@
       </c>
       <c r="H87" s="1" t="inlineStr">
         <is>
-          <t>Q4017</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
@@ -4079,7 +4079,7 @@
       </c>
       <c r="H88" s="1" t="inlineStr">
         <is>
-          <t>Q4019</t>
+          <t>Q4017</t>
         </is>
       </c>
     </row>
@@ -4121,7 +4121,7 @@
       </c>
       <c r="H89" s="1" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>Q4019</t>
         </is>
       </c>
     </row>
@@ -4163,7 +4163,7 @@
       </c>
       <c r="H90" s="1" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
@@ -4205,7 +4205,7 @@
       </c>
       <c r="H91" s="1" t="inlineStr">
         <is>
-          <t>QBX005</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
@@ -4247,7 +4247,7 @@
       </c>
       <c r="H92" s="1" t="inlineStr">
         <is>
-          <t>QBX006</t>
+          <t>QBX005</t>
         </is>
       </c>
     </row>
@@ -4289,7 +4289,7 @@
       </c>
       <c r="H93" s="1" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>QBX006</t>
         </is>
       </c>
     </row>
@@ -4331,7 +4331,7 @@
       </c>
       <c r="H94" s="1" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>QE001</t>
         </is>
       </c>
     </row>
@@ -4373,7 +4373,7 @@
       </c>
       <c r="H95" s="1" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
@@ -4415,7 +4415,7 @@
       </c>
       <c r="H96" s="1" t="inlineStr">
         <is>
-          <t>QE004</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
@@ -4457,7 +4457,7 @@
       </c>
       <c r="H97" s="1" t="inlineStr">
         <is>
-          <t>QE006</t>
+          <t>QE004</t>
         </is>
       </c>
     </row>
@@ -4499,7 +4499,7 @@
       </c>
       <c r="H98" s="1" t="inlineStr">
         <is>
-          <t>QL001</t>
+          <t>QE006</t>
         </is>
       </c>
     </row>
@@ -4541,7 +4541,7 @@
       </c>
       <c r="H99" s="1" t="inlineStr">
         <is>
-          <t>QL002</t>
+          <t>QL001</t>
         </is>
       </c>
     </row>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="H100" s="1" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>QL002</t>
         </is>
       </c>
     </row>
@@ -4625,7 +4625,7 @@
       </c>
       <c r="H101" s="1" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>QL004</t>
         </is>
       </c>
     </row>
@@ -4667,7 +4667,7 @@
       </c>
       <c r="H102" s="1" t="inlineStr">
         <is>
-          <t>QL008</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
@@ -4709,7 +4709,7 @@
       </c>
       <c r="H103" s="1" t="inlineStr">
         <is>
-          <t>QL010</t>
+          <t>QL008</t>
         </is>
       </c>
     </row>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="H104" s="1" t="inlineStr">
         <is>
-          <t>QL011</t>
+          <t>QL010</t>
         </is>
       </c>
     </row>
@@ -4793,7 +4793,7 @@
       </c>
       <c r="H105" s="1" t="inlineStr">
         <is>
-          <t>QL014</t>
+          <t>QL011</t>
         </is>
       </c>
     </row>
@@ -4835,7 +4835,7 @@
       </c>
       <c r="H106" s="1" t="inlineStr">
         <is>
-          <t>QL018</t>
+          <t>QL014</t>
         </is>
       </c>
     </row>
@@ -4877,7 +4877,7 @@
       </c>
       <c r="H107" s="1" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QL018</t>
         </is>
       </c>
     </row>
@@ -4919,7 +4919,7 @@
       </c>
       <c r="H108" s="1" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QR1744</t>
         </is>
       </c>
     </row>
@@ -4961,7 +4961,7 @@
       </c>
       <c r="H109" s="1" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QR1771</t>
         </is>
       </c>
     </row>
@@ -5003,7 +5003,7 @@
       </c>
       <c r="H110" s="1" t="inlineStr">
         <is>
-          <t>R711</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
@@ -5045,7 +5045,7 @@
       </c>
       <c r="H111" s="1" t="inlineStr">
         <is>
-          <t>R766</t>
+          <t>R711</t>
         </is>
       </c>
     </row>
@@ -5087,7 +5087,7 @@
       </c>
       <c r="H112" s="1" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>R766</t>
         </is>
       </c>
     </row>
@@ -5129,2149 +5129,2154 @@
       </c>
       <c r="H113" s="1" t="inlineStr">
         <is>
-          <t>RCTST4</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>RCTST4</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>TE2806</t>
         </is>
       </c>
       <c r="C115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8056</t>
+          <t>VLINE-8055</t>
         </is>
       </c>
       <c r="D115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8172</t>
+          <t>VLINE-8171</t>
         </is>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8426</t>
+          <t>VLINE-8425</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8735</t>
+          <t>VLINE-8733</t>
         </is>
       </c>
       <c r="G115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8800</t>
+          <t>VLINE-8799</t>
         </is>
       </c>
       <c r="H115" s="1" t="inlineStr">
         <is>
-          <t>XRN006</t>
+          <t>XRN005</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>RL302</t>
+          <t>RL301</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>TE2807</t>
         </is>
       </c>
       <c r="C116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8057</t>
+          <t>VLINE-8056</t>
         </is>
       </c>
       <c r="D116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8176</t>
+          <t>VLINE-8172</t>
         </is>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8427</t>
+          <t>VLINE-8426</t>
         </is>
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8736</t>
+          <t>VLINE-8735</t>
         </is>
       </c>
       <c r="G116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8801</t>
+          <t>VLINE-8800</t>
         </is>
       </c>
       <c r="H116" s="1" t="inlineStr">
         <is>
-          <t>XRN007</t>
+          <t>XRN006</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>RL304</t>
+          <t>RL302</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
         <is>
-          <t>TE2809</t>
+          <t>TE2808</t>
         </is>
       </c>
       <c r="C117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8058</t>
+          <t>VLINE-8057</t>
         </is>
       </c>
       <c r="D117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8179</t>
+          <t>VLINE-8176</t>
         </is>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8428</t>
+          <t>VLINE-8427</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8737</t>
+          <t>VLINE-8736</t>
         </is>
       </c>
       <c r="G117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8802</t>
+          <t>VLINE-8801</t>
         </is>
       </c>
       <c r="H117" s="1" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>XRN007</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>RL305</t>
+          <t>RL304</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
         <is>
-          <t>TE2810</t>
+          <t>TE2809</t>
         </is>
       </c>
       <c r="C118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8059</t>
+          <t>VLINE-8058</t>
         </is>
       </c>
       <c r="D118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8180</t>
+          <t>VLINE-8179</t>
         </is>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8429</t>
+          <t>VLINE-8428</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8739</t>
+          <t>VLINE-8737</t>
         </is>
       </c>
       <c r="G118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8803</t>
+          <t>VLINE-8802</t>
         </is>
       </c>
       <c r="H118" s="1" t="inlineStr">
         <is>
-          <t>XRN011</t>
+          <t>XRN009</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>RL307</t>
+          <t>RL305</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
         <is>
-          <t>TE2812</t>
+          <t>TE2810</t>
         </is>
       </c>
       <c r="C119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8061</t>
+          <t>VLINE-8059</t>
         </is>
       </c>
       <c r="D119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8181</t>
+          <t>VLINE-8180</t>
         </is>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8430</t>
+          <t>VLINE-8429</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8740</t>
+          <t>VLINE-8739</t>
         </is>
       </c>
       <c r="G119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8804</t>
+          <t>VLINE-8803</t>
         </is>
       </c>
       <c r="H119" s="1" t="inlineStr">
         <is>
-          <t>XRN014</t>
+          <t>XRN011</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>RL309</t>
+          <t>RL307</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>TE2812</t>
         </is>
       </c>
       <c r="C120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8072</t>
+          <t>VLINE-8061</t>
         </is>
       </c>
       <c r="D120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8182</t>
+          <t>VLINE-8181</t>
         </is>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8431</t>
+          <t>VLINE-8430</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8741</t>
+          <t>VLINE-8740</t>
         </is>
       </c>
       <c r="G120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8805</t>
+          <t>VLINE-8804</t>
         </is>
       </c>
       <c r="H120" s="1" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>XRN014</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>RL310</t>
+          <t>RL309</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>TE2813</t>
         </is>
       </c>
       <c r="C121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8074</t>
+          <t>VLINE-8072</t>
         </is>
       </c>
       <c r="D121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8183</t>
+          <t>VLINE-8182</t>
         </is>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8432</t>
+          <t>VLINE-8431</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8742</t>
+          <t>VLINE-8741</t>
         </is>
       </c>
       <c r="G121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8806</t>
+          <t>VLINE-8805</t>
         </is>
       </c>
       <c r="H121" s="1" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>XRN017</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>S312</t>
+          <t>RL310</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>TE2814</t>
         </is>
       </c>
       <c r="C122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8075</t>
+          <t>VLINE-8074</t>
         </is>
       </c>
       <c r="D122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8184</t>
+          <t>VLINE-8183</t>
         </is>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8433</t>
+          <t>VLINE-8432</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8743</t>
+          <t>VLINE-8742</t>
         </is>
       </c>
       <c r="G122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8807</t>
+          <t>VLINE-8806</t>
         </is>
       </c>
       <c r="H122" s="1" t="inlineStr">
         <is>
-          <t>XRN020</t>
+          <t>XRN018</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>S317</t>
+          <t>S312</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
         <is>
-          <t>TJ107</t>
+          <t>TJ096</t>
         </is>
       </c>
       <c r="C123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8076</t>
+          <t>VLINE-8075</t>
         </is>
       </c>
       <c r="D123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8185</t>
+          <t>VLINE-8184</t>
         </is>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8434</t>
+          <t>VLINE-8433</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8744</t>
+          <t>VLINE-8743</t>
         </is>
       </c>
       <c r="G123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8808</t>
+          <t>VLINE-8807</t>
         </is>
       </c>
       <c r="H123" s="1" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>XRN020</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>S3301</t>
+          <t>S317</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TJ107</t>
         </is>
       </c>
       <c r="C124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8077</t>
+          <t>VLINE-8076</t>
         </is>
       </c>
       <c r="D124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8186</t>
+          <t>VLINE-8185</t>
         </is>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8435</t>
+          <t>VLINE-8434</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8745</t>
+          <t>VLINE-8744</t>
         </is>
       </c>
       <c r="G124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8809</t>
+          <t>VLINE-8808</t>
         </is>
       </c>
       <c r="H124" s="1" t="inlineStr">
         <is>
-          <t>XRN023</t>
+          <t>XRN021</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>S3302</t>
+          <t>S3301</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TT03</t>
         </is>
       </c>
       <c r="C125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8080</t>
+          <t>VLINE-8077</t>
         </is>
       </c>
       <c r="D125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8187</t>
+          <t>VLINE-8186</t>
         </is>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8438</t>
+          <t>VLINE-8435</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8746</t>
+          <t>VLINE-8745</t>
         </is>
       </c>
       <c r="G125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8810</t>
+          <t>VLINE-8809</t>
         </is>
       </c>
       <c r="H125" s="1" t="inlineStr">
         <is>
-          <t>XRN025</t>
+          <t>XRN023</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>S3304</t>
+          <t>S3302</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TT04</t>
         </is>
       </c>
       <c r="C126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8081</t>
+          <t>VLINE-8080</t>
         </is>
       </c>
       <c r="D126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8188</t>
+          <t>VLINE-8187</t>
         </is>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8440</t>
+          <t>VLINE-8438</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8747</t>
+          <t>VLINE-8746</t>
         </is>
       </c>
       <c r="G126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8811</t>
+          <t>VLINE-8810</t>
         </is>
       </c>
       <c r="H126" s="1" t="inlineStr">
         <is>
-          <t>XRN026</t>
+          <t>XRN025</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>S3305</t>
+          <t>S3304</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
         <is>
-          <t>TT07</t>
+          <t>TT05</t>
         </is>
       </c>
       <c r="C127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8084</t>
+          <t>VLINE-8081</t>
         </is>
       </c>
       <c r="D127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8189</t>
+          <t>VLINE-8188</t>
         </is>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8441</t>
+          <t>VLINE-8440</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8748</t>
+          <t>VLINE-8747</t>
         </is>
       </c>
       <c r="G127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8812</t>
+          <t>VLINE-8811</t>
         </is>
       </c>
       <c r="H127" s="1" t="inlineStr">
         <is>
-          <t>XRN027</t>
+          <t>XRN026</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>S3306</t>
+          <t>S3305</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TT07</t>
         </is>
       </c>
       <c r="C128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8088</t>
+          <t>VLINE-8084</t>
         </is>
       </c>
       <c r="D128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8291</t>
+          <t>VLINE-8189</t>
         </is>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8442</t>
+          <t>VLINE-8441</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8749</t>
+          <t>VLINE-8748</t>
         </is>
       </c>
       <c r="G128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8813</t>
+          <t>VLINE-8812</t>
         </is>
       </c>
       <c r="H128" s="1" t="inlineStr">
         <is>
-          <t>Y163</t>
+          <t>XRN027</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>S3307</t>
+          <t>S3306</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TT08</t>
         </is>
       </c>
       <c r="C129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8089</t>
+          <t>VLINE-8088</t>
         </is>
       </c>
       <c r="D129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8293</t>
+          <t>VLINE-8291</t>
         </is>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8443</t>
+          <t>VLINE-8442</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8750</t>
+          <t>VLINE-8749</t>
         </is>
       </c>
       <c r="G129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8814</t>
+          <t>VLINE-8813</t>
+        </is>
+      </c>
+      <c r="H129" s="1" t="inlineStr">
+        <is>
+          <t>Y163</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>S3309</t>
+          <t>S3307</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
         <is>
-          <t>TT106</t>
+          <t>TT103</t>
         </is>
       </c>
       <c r="C130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8104</t>
+          <t>VLINE-8089</t>
         </is>
       </c>
       <c r="D130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8303</t>
+          <t>VLINE-8293</t>
         </is>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8444</t>
+          <t>VLINE-8443</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8751</t>
+          <t>VLINE-8750</t>
         </is>
       </c>
       <c r="G130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8816</t>
+          <t>VLINE-8814</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>S3310</t>
+          <t>S3309</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TT106</t>
         </is>
       </c>
       <c r="C131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8107</t>
+          <t>VLINE-8104</t>
         </is>
       </c>
       <c r="D131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8304</t>
+          <t>VLINE-8303</t>
         </is>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8446</t>
+          <t>VLINE-8444</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8752</t>
+          <t>VLINE-8751</t>
         </is>
       </c>
       <c r="G131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8817</t>
+          <t>VLINE-8816</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>S7001</t>
+          <t>S3310</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
         <is>
-          <t>TT108</t>
+          <t>TT107</t>
         </is>
       </c>
       <c r="C132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8110</t>
+          <t>VLINE-8107</t>
         </is>
       </c>
       <c r="D132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8306</t>
+          <t>VLINE-8304</t>
         </is>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8447</t>
+          <t>VLINE-8446</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8753</t>
+          <t>VLINE-8752</t>
         </is>
       </c>
       <c r="G132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8818</t>
+          <t>VLINE-8817</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>S7002</t>
+          <t>S7001</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TT108</t>
         </is>
       </c>
       <c r="C133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8111</t>
+          <t>VLINE-8110</t>
         </is>
       </c>
       <c r="D133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8311</t>
+          <t>VLINE-8306</t>
         </is>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8449</t>
+          <t>VLINE-8447</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8754</t>
+          <t>VLINE-8753</t>
         </is>
       </c>
       <c r="G133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8819</t>
+          <t>VLINE-8818</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>S7003</t>
+          <t>S7002</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
         <is>
-          <t>TT113</t>
+          <t>TT110</t>
         </is>
       </c>
       <c r="C134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8113</t>
+          <t>VLINE-8111</t>
         </is>
       </c>
       <c r="D134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8313</t>
+          <t>VLINE-8311</t>
         </is>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8450</t>
+          <t>VLINE-8449</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8755</t>
+          <t>VLINE-8754</t>
         </is>
       </c>
       <c r="G134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8822</t>
+          <t>VLINE-8819</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>S7004</t>
+          <t>S7003</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
         <is>
-          <t>TT114</t>
+          <t>TT113</t>
         </is>
       </c>
       <c r="C135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8114</t>
+          <t>VLINE-8113</t>
         </is>
       </c>
       <c r="D135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8314</t>
+          <t>VLINE-8313</t>
         </is>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8451</t>
+          <t>VLINE-8450</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8756</t>
+          <t>VLINE-8755</t>
         </is>
       </c>
       <c r="G135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8860</t>
+          <t>VLINE-8822</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>S7005</t>
+          <t>S7004</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT114</t>
         </is>
       </c>
       <c r="C136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8115</t>
+          <t>VLINE-8114</t>
         </is>
       </c>
       <c r="D136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8316</t>
+          <t>VLINE-8314</t>
         </is>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8452</t>
+          <t>VLINE-8451</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8757</t>
+          <t>VLINE-8756</t>
         </is>
       </c>
       <c r="G136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8861</t>
+          <t>VLINE-8860</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>S7006</t>
+          <t>S7005</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
         <is>
-          <t>TT116</t>
+          <t>TT115</t>
         </is>
       </c>
       <c r="C137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8119</t>
+          <t>VLINE-8115</t>
         </is>
       </c>
       <c r="D137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8318</t>
+          <t>VLINE-8316</t>
         </is>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8453</t>
+          <t>VLINE-8452</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8758</t>
+          <t>VLINE-8757</t>
         </is>
       </c>
       <c r="G137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8862</t>
+          <t>VLINE-8861</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>S7007</t>
+          <t>S7006</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT116</t>
         </is>
       </c>
       <c r="C138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8120</t>
+          <t>VLINE-8119</t>
         </is>
       </c>
       <c r="D138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8321</t>
+          <t>VLINE-8318</t>
         </is>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8454</t>
+          <t>VLINE-8453</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8759</t>
+          <t>VLINE-8758</t>
         </is>
       </c>
       <c r="G138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8863</t>
+          <t>VLINE-8862</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>S7008</t>
+          <t>S7007</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
         <is>
-          <t>TT122</t>
+          <t>TT117</t>
         </is>
       </c>
       <c r="C139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8121</t>
+          <t>VLINE-8120</t>
         </is>
       </c>
       <c r="D139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8323</t>
+          <t>VLINE-8321</t>
         </is>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8455</t>
+          <t>VLINE-8454</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8760</t>
+          <t>VLINE-8759</t>
         </is>
       </c>
       <c r="G139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8864</t>
+          <t>VLINE-8863</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>S7012</t>
+          <t>S7008</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
         <is>
-          <t>TT127</t>
+          <t>TT122</t>
         </is>
       </c>
       <c r="C140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8123</t>
+          <t>VLINE-8121</t>
         </is>
       </c>
       <c r="D140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8324</t>
+          <t>VLINE-8323</t>
         </is>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8456</t>
+          <t>VLINE-8455</t>
         </is>
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8761</t>
+          <t>VLINE-8760</t>
         </is>
       </c>
       <c r="G140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8865</t>
+          <t>VLINE-8864</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>S7013</t>
+          <t>S7012</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
         <is>
-          <t>TT128</t>
+          <t>TT127</t>
         </is>
       </c>
       <c r="C141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8124</t>
+          <t>VLINE-8123</t>
         </is>
       </c>
       <c r="D141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8325</t>
+          <t>VLINE-8324</t>
         </is>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8457</t>
+          <t>VLINE-8456</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8762</t>
+          <t>VLINE-8761</t>
         </is>
       </c>
       <c r="G141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8866</t>
+          <t>VLINE-8865</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>S7014</t>
+          <t>S7013</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT128</t>
         </is>
       </c>
       <c r="C142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8126</t>
+          <t>VLINE-8124</t>
         </is>
       </c>
       <c r="D142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8328</t>
+          <t>VLINE-8325</t>
         </is>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8460</t>
+          <t>VLINE-8457</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8763</t>
+          <t>VLINE-8762</t>
         </is>
       </c>
       <c r="G142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8867</t>
+          <t>VLINE-8866</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>S7015</t>
+          <t>S7014</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
         <is>
-          <t>TT131</t>
+          <t>TT130</t>
         </is>
       </c>
       <c r="C143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8127</t>
+          <t>VLINE-8126</t>
         </is>
       </c>
       <c r="D143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8329</t>
+          <t>VLINE-8328</t>
         </is>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8461</t>
+          <t>VLINE-8460</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8765</t>
+          <t>VLINE-8763</t>
         </is>
       </c>
       <c r="G143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8868</t>
+          <t>VLINE-8867</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>S7017</t>
+          <t>S7015</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT131</t>
         </is>
       </c>
       <c r="C144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8128</t>
+          <t>VLINE-8127</t>
         </is>
       </c>
       <c r="D144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8332</t>
+          <t>VLINE-8329</t>
         </is>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8464</t>
+          <t>VLINE-8461</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8766</t>
+          <t>VLINE-8765</t>
         </is>
       </c>
       <c r="G144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8869</t>
+          <t>VLINE-8868</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>S7018</t>
+          <t>S7017</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT202</t>
         </is>
       </c>
       <c r="C145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8129</t>
+          <t>VLINE-8128</t>
         </is>
       </c>
       <c r="D145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8336</t>
+          <t>VLINE-8332</t>
         </is>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8465</t>
+          <t>VLINE-8464</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8767</t>
+          <t>VLINE-8766</t>
         </is>
       </c>
       <c r="G145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8890</t>
+          <t>VLINE-8869</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>S7020</t>
+          <t>S7018</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
         <is>
-          <t>VL352</t>
+          <t>TT206</t>
         </is>
       </c>
       <c r="C146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8131</t>
+          <t>VLINE-8129</t>
         </is>
       </c>
       <c r="D146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8337</t>
+          <t>VLINE-8336</t>
         </is>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8468</t>
+          <t>VLINE-8465</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8768</t>
+          <t>VLINE-8767</t>
         </is>
       </c>
       <c r="G146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8891</t>
+          <t>VLINE-8890</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>S7022</t>
+          <t>S7020</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
         <is>
-          <t>VL353</t>
+          <t>VL352</t>
         </is>
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8132</t>
+          <t>VLINE-8131</t>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8338</t>
+          <t>VLINE-8337</t>
         </is>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8469</t>
+          <t>VLINE-8468</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8769</t>
+          <t>VLINE-8768</t>
         </is>
       </c>
       <c r="G147" s="1" t="inlineStr">
         <is>
-          <t>WH001</t>
+          <t>VLINE-8891</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>S7022</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
         <is>
-          <t>VL357</t>
+          <t>VL353</t>
         </is>
       </c>
       <c r="C148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8133</t>
+          <t>VLINE-8132</t>
         </is>
       </c>
       <c r="D148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8339</t>
+          <t>VLINE-8338</t>
         </is>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8605</t>
+          <t>VLINE-8469</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8770</t>
+          <t>VLINE-8769</t>
         </is>
       </c>
       <c r="G148" s="1" t="inlineStr">
         <is>
-          <t>WH003</t>
+          <t>WH001</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>SCT002</t>
+          <t>SCT001</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8004</t>
+          <t>VL357</t>
         </is>
       </c>
       <c r="C149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8134</t>
+          <t>VLINE-8133</t>
         </is>
       </c>
       <c r="D149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8362</t>
+          <t>VLINE-8339</t>
         </is>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8610</t>
+          <t>VLINE-8605</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8772</t>
+          <t>VLINE-8770</t>
         </is>
       </c>
       <c r="G149" s="1" t="inlineStr">
         <is>
-          <t>WL02</t>
+          <t>WH003</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>SCT006</t>
+          <t>SCT002</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8007</t>
+          <t>VLINE-8004</t>
         </is>
       </c>
       <c r="C150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8136</t>
+          <t>VLINE-8134</t>
         </is>
       </c>
       <c r="D150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8363</t>
+          <t>VLINE-8362</t>
         </is>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8612</t>
+          <t>VLINE-8610</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8773</t>
+          <t>VLINE-8772</t>
         </is>
       </c>
       <c r="G150" s="1" t="inlineStr">
         <is>
-          <t>X12-X14</t>
+          <t>WL02</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>SCT007</t>
+          <t>SCT006</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8011</t>
+          <t>VLINE-8007</t>
         </is>
       </c>
       <c r="C151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8137</t>
+          <t>VLINE-8136</t>
         </is>
       </c>
       <c r="D151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8365</t>
+          <t>VLINE-8363</t>
         </is>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8615</t>
+          <t>VLINE-8612</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8774</t>
+          <t>VLINE-8773</t>
         </is>
       </c>
       <c r="G151" s="1" t="inlineStr">
         <is>
-          <t>X31</t>
+          <t>X12-X14</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>SCT007</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8013</t>
+          <t>VLINE-8011</t>
         </is>
       </c>
       <c r="C152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8140</t>
+          <t>VLINE-8137</t>
         </is>
       </c>
       <c r="D152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8366</t>
+          <t>VLINE-8365</t>
         </is>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8617</t>
+          <t>VLINE-8615</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8776</t>
+          <t>VLINE-8774</t>
         </is>
       </c>
       <c r="G152" s="1" t="inlineStr">
         <is>
-          <t>XP2000</t>
+          <t>X31</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>SCT011</t>
+          <t>SCT009</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8019</t>
+          <t>VLINE-8013</t>
         </is>
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8141</t>
+          <t>VLINE-8140</t>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8368</t>
+          <t>VLINE-8366</t>
         </is>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8620</t>
+          <t>VLINE-8617</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8778</t>
+          <t>VLINE-8776</t>
         </is>
       </c>
       <c r="G153" s="1" t="inlineStr">
         <is>
-          <t>XP2003</t>
+          <t>XP2000</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>SCT011</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8020</t>
+          <t>VLINE-8019</t>
         </is>
       </c>
       <c r="C154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8142</t>
+          <t>VLINE-8141</t>
         </is>
       </c>
       <c r="D154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8369</t>
+          <t>VLINE-8368</t>
         </is>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8625</t>
+          <t>VLINE-8620</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8779</t>
+          <t>VLINE-8778</t>
         </is>
       </c>
       <c r="G154" s="1" t="inlineStr">
         <is>
-          <t>XP2004</t>
+          <t>XP2003</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>SCT014</t>
+          <t>SCT013</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8023</t>
+          <t>VLINE-8020</t>
         </is>
       </c>
       <c r="C155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8144</t>
+          <t>VLINE-8142</t>
         </is>
       </c>
       <c r="D155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8403</t>
+          <t>VLINE-8369</t>
         </is>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8630</t>
+          <t>VLINE-8625</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8780</t>
+          <t>VLINE-8779</t>
         </is>
       </c>
       <c r="G155" s="1" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>XP2004</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>SCT015</t>
+          <t>SCT014</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8025</t>
+          <t>VLINE-8023</t>
         </is>
       </c>
       <c r="C156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8145</t>
+          <t>VLINE-8144</t>
         </is>
       </c>
       <c r="D156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8404</t>
+          <t>VLINE-8403</t>
         </is>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8671</t>
+          <t>VLINE-8630</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8781</t>
+          <t>VLINE-8780</t>
         </is>
       </c>
       <c r="G156" s="1" t="inlineStr">
         <is>
-          <t>XP2007</t>
+          <t>XP2005</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>SO2</t>
+          <t>SCT015</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8026</t>
+          <t>VLINE-8025</t>
         </is>
       </c>
       <c r="C157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8148</t>
+          <t>VLINE-8145</t>
         </is>
       </c>
       <c r="D157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8406</t>
+          <t>VLINE-8404</t>
         </is>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8706</t>
+          <t>VLINE-8671</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8782</t>
+          <t>VLINE-8781</t>
         </is>
       </c>
       <c r="G157" s="1" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>XP2007</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>SO2</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8027</t>
+          <t>VLINE-8026</t>
         </is>
       </c>
       <c r="C158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8150</t>
+          <t>VLINE-8148</t>
         </is>
       </c>
       <c r="D158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8408</t>
+          <t>VLINE-8406</t>
         </is>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8711</t>
+          <t>VLINE-8706</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8783</t>
+          <t>VLINE-8782</t>
         </is>
       </c>
       <c r="G158" s="1" t="inlineStr">
         <is>
-          <t>XP2010</t>
+          <t>XP2008</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>SSR101</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8028</t>
+          <t>VLINE-8027</t>
         </is>
       </c>
       <c r="C159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8151</t>
+          <t>VLINE-8150</t>
         </is>
       </c>
       <c r="D159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8410</t>
+          <t>VLINE-8408</t>
         </is>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8714</t>
+          <t>VLINE-8711</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8784</t>
+          <t>VLINE-8783</t>
         </is>
       </c>
       <c r="G159" s="1" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>XP2010</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>SSR102</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8029</t>
+          <t>VLINE-8028</t>
         </is>
       </c>
       <c r="C160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8152</t>
+          <t>VLINE-8151</t>
         </is>
       </c>
       <c r="D160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8411</t>
+          <t>VLINE-8410</t>
         </is>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8717</t>
+          <t>VLINE-8714</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8786</t>
+          <t>VLINE-8784</t>
         </is>
       </c>
       <c r="G160" s="1" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>XP2011</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>SSR103</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8030</t>
+          <t>VLINE-8029</t>
         </is>
       </c>
       <c r="C161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8153</t>
+          <t>VLINE-8152</t>
         </is>
       </c>
       <c r="D161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8413</t>
+          <t>VLINE-8411</t>
         </is>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8720</t>
+          <t>VLINE-8717</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8787</t>
+          <t>VLINE-8786</t>
         </is>
       </c>
       <c r="G161" s="1" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>XP2012</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>T363</t>
+          <t>SSR104</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8031</t>
+          <t>VLINE-8030</t>
         </is>
       </c>
       <c r="C162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8154</t>
+          <t>VLINE-8153</t>
         </is>
       </c>
       <c r="D162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8415</t>
+          <t>VLINE-8413</t>
         </is>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8721</t>
+          <t>VLINE-8720</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8788</t>
+          <t>VLINE-8787</t>
         </is>
       </c>
       <c r="G162" s="1" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>XP2013</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>T386</t>
+          <t>T363</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8032</t>
+          <t>VLINE-8031</t>
         </is>
       </c>
       <c r="C163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8155</t>
+          <t>VLINE-8154</t>
         </is>
       </c>
       <c r="D163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8417</t>
+          <t>VLINE-8415</t>
         </is>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8723</t>
+          <t>VLINE-8721</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8790</t>
+          <t>VLINE-8788</t>
         </is>
       </c>
       <c r="G163" s="1" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>XP2014</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>TDX101</t>
+          <t>T386</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8036</t>
+          <t>VLINE-8032</t>
         </is>
       </c>
       <c r="C164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8157</t>
+          <t>VLINE-8155</t>
         </is>
       </c>
       <c r="D164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8418</t>
+          <t>VLINE-8417</t>
         </is>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8725</t>
+          <t>VLINE-8723</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8792</t>
+          <t>VLINE-8790</t>
         </is>
       </c>
       <c r="G164" s="1" t="inlineStr">
         <is>
-          <t>XP2016</t>
+          <t>XP2015</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>TDX101</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8038</t>
+          <t>VLINE-8036</t>
         </is>
       </c>
       <c r="C165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8158</t>
+          <t>VLINE-8157</t>
         </is>
       </c>
       <c r="D165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8419</t>
+          <t>VLINE-8418</t>
         </is>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8726</t>
+          <t>VLINE-8725</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8793</t>
+          <t>VLINE-8792</t>
         </is>
       </c>
       <c r="G165" s="1" t="inlineStr">
         <is>
-          <t>XP2017</t>
+          <t>XP2016</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>TE2802</t>
+          <t>TE2801</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8042</t>
+          <t>VLINE-8038</t>
         </is>
       </c>
       <c r="C166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8159</t>
+          <t>VLINE-8158</t>
         </is>
       </c>
       <c r="D166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8420</t>
+          <t>VLINE-8419</t>
         </is>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8727</t>
+          <t>VLINE-8726</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8794</t>
+          <t>VLINE-8793</t>
         </is>
       </c>
       <c r="G166" s="1" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>XP2017</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>TE2802</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8051</t>
+          <t>VLINE-8042</t>
         </is>
       </c>
       <c r="C167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8160</t>
+          <t>VLINE-8159</t>
         </is>
       </c>
       <c r="D167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8421</t>
+          <t>VLINE-8420</t>
         </is>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8729</t>
+          <t>VLINE-8727</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8795</t>
+          <t>VLINE-8794</t>
         </is>
       </c>
       <c r="G167" s="1" t="inlineStr">
         <is>
-          <t>XR552</t>
+          <t>XP2019</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>TE2804</t>
+          <t>TE2803</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8052</t>
+          <t>VLINE-8051</t>
         </is>
       </c>
       <c r="C168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8161</t>
+          <t>VLINE-8160</t>
         </is>
       </c>
       <c r="D168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8422</t>
+          <t>VLINE-8421</t>
         </is>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8730</t>
+          <t>VLINE-8729</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8796</t>
+          <t>VLINE-8795</t>
         </is>
       </c>
       <c r="G168" s="1" t="inlineStr">
         <is>
-          <t>XRN001</t>
+          <t>XR552</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>TE2804</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8053</t>
+          <t>VLINE-8052</t>
         </is>
       </c>
       <c r="C169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8162</t>
+          <t>VLINE-8161</t>
         </is>
       </c>
       <c r="D169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8424</t>
+          <t>VLINE-8422</t>
         </is>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8731</t>
+          <t>VLINE-8730</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8797</t>
+          <t>VLINE-8796</t>
         </is>
       </c>
       <c r="G169" s="1" t="inlineStr">
         <is>
-          <t>XRN004</t>
+          <t>XRN001</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>TE2806</t>
+          <t>TE2805</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8055</t>
+          <t>VLINE-8053</t>
         </is>
       </c>
       <c r="C170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8171</t>
+          <t>VLINE-8162</t>
         </is>
       </c>
       <c r="D170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8425</t>
+          <t>VLINE-8424</t>
         </is>
       </c>
       <c r="E170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8733</t>
+          <t>VLINE-8731</t>
         </is>
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8799</t>
+          <t>VLINE-8797</t>
         </is>
       </c>
       <c r="G170" s="1" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>XRN004</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update trains and loco export 2026-04-05 19:50:12
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -2794,32 +2794,32 @@
       </c>
       <c r="C58" s="1" t="inlineStr">
         <is>
-          <t>MM-242M</t>
+          <t>MM-224M</t>
         </is>
       </c>
       <c r="D58" s="1" t="inlineStr">
         <is>
-          <t>MM-734M</t>
+          <t>MM-722M</t>
         </is>
       </c>
       <c r="E58" s="1" t="inlineStr">
         <is>
-          <t>MM-912M</t>
+          <t>MM-906M</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
         <is>
-          <t>MM-9945M</t>
+          <t>MM-9938M</t>
         </is>
       </c>
       <c r="G58" s="1" t="inlineStr">
         <is>
-          <t>NR38</t>
+          <t>NR31</t>
         </is>
       </c>
       <c r="H58" s="1" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR110</t>
         </is>
       </c>
     </row>
@@ -2836,32 +2836,32 @@
       </c>
       <c r="C59" s="1" t="inlineStr">
         <is>
-          <t>MM-256M</t>
+          <t>MM-242M</t>
         </is>
       </c>
       <c r="D59" s="1" t="inlineStr">
         <is>
-          <t>MM-736M</t>
+          <t>MM-726M</t>
         </is>
       </c>
       <c r="E59" s="1" t="inlineStr">
         <is>
-          <t>MM-914M</t>
+          <t>MM-908M</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
         <is>
-          <t>MM-9946M</t>
+          <t>MM-9941M</t>
         </is>
       </c>
       <c r="G59" s="1" t="inlineStr">
         <is>
-          <t>NR39</t>
+          <t>NR34</t>
         </is>
       </c>
       <c r="H59" s="1" t="inlineStr">
         <is>
-          <t>NR118</t>
+          <t>NR111</t>
         </is>
       </c>
     </row>
@@ -2878,32 +2878,32 @@
       </c>
       <c r="C60" s="1" t="inlineStr">
         <is>
-          <t>MM-258M</t>
+          <t>MM-256M</t>
         </is>
       </c>
       <c r="D60" s="1" t="inlineStr">
         <is>
-          <t>MM-738M</t>
+          <t>MM-728M</t>
         </is>
       </c>
       <c r="E60" s="1" t="inlineStr">
         <is>
-          <t>MM-920M</t>
+          <t>MM-910M</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
         <is>
-          <t>MM-9949M</t>
+          <t>MM-9943M</t>
         </is>
       </c>
       <c r="G60" s="1" t="inlineStr">
         <is>
-          <t>NR40</t>
+          <t>NR36</t>
         </is>
       </c>
       <c r="H60" s="1" t="inlineStr">
         <is>
-          <t>NR119</t>
+          <t>NR112</t>
         </is>
       </c>
     </row>
@@ -2920,32 +2920,32 @@
       </c>
       <c r="C61" s="1" t="inlineStr">
         <is>
-          <t>MM-264M</t>
+          <t>MM-258M</t>
         </is>
       </c>
       <c r="D61" s="1" t="inlineStr">
         <is>
-          <t>MM-740M</t>
+          <t>MM-734M</t>
         </is>
       </c>
       <c r="E61" s="1" t="inlineStr">
         <is>
-          <t>MM-922M</t>
+          <t>MM-912M</t>
         </is>
       </c>
       <c r="F61" s="1" t="inlineStr">
         <is>
-          <t>MM-9950M</t>
+          <t>MM-9945M</t>
         </is>
       </c>
       <c r="G61" s="1" t="inlineStr">
         <is>
-          <t>NR43</t>
+          <t>NR37</t>
         </is>
       </c>
       <c r="H61" s="1" t="inlineStr">
         <is>
-          <t>NR120</t>
+          <t>NR113</t>
         </is>
       </c>
     </row>
@@ -2962,32 +2962,32 @@
       </c>
       <c r="C62" s="1" t="inlineStr">
         <is>
-          <t>MM-268M</t>
+          <t>MM-264M</t>
         </is>
       </c>
       <c r="D62" s="1" t="inlineStr">
         <is>
-          <t>MM-742M</t>
+          <t>MM-736M</t>
         </is>
       </c>
       <c r="E62" s="1" t="inlineStr">
         <is>
-          <t>MM-924M</t>
+          <t>MM-914M</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
         <is>
-          <t>MM-9951M</t>
+          <t>MM-9946M</t>
         </is>
       </c>
       <c r="G62" s="1" t="inlineStr">
         <is>
-          <t>NR44</t>
+          <t>NR38</t>
         </is>
       </c>
       <c r="H62" s="1" t="inlineStr">
         <is>
-          <t>NR122</t>
+          <t>NR115</t>
         </is>
       </c>
     </row>
@@ -3004,32 +3004,32 @@
       </c>
       <c r="C63" s="1" t="inlineStr">
         <is>
-          <t>MM-278M</t>
+          <t>MM-268M</t>
         </is>
       </c>
       <c r="D63" s="1" t="inlineStr">
         <is>
-          <t>MM-744M</t>
+          <t>MM-738M</t>
         </is>
       </c>
       <c r="E63" s="1" t="inlineStr">
         <is>
-          <t>MM-926M</t>
+          <t>MM-920M</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
         <is>
-          <t>MM-9952M</t>
+          <t>MM-9949M</t>
         </is>
       </c>
       <c r="G63" s="1" t="inlineStr">
         <is>
-          <t>NR45</t>
+          <t>NR39</t>
         </is>
       </c>
       <c r="H63" s="1" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>NR118</t>
         </is>
       </c>
     </row>
@@ -3046,32 +3046,32 @@
       </c>
       <c r="C64" s="1" t="inlineStr">
         <is>
-          <t>MM-282M</t>
+          <t>MM-278M</t>
         </is>
       </c>
       <c r="D64" s="1" t="inlineStr">
         <is>
-          <t>MM-752M</t>
+          <t>MM-740M</t>
         </is>
       </c>
       <c r="E64" s="1" t="inlineStr">
         <is>
-          <t>MM-934M</t>
+          <t>MM-922M</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
         <is>
-          <t>MM-9953M</t>
+          <t>MM-9950M</t>
         </is>
       </c>
       <c r="G64" s="1" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>NR40</t>
         </is>
       </c>
       <c r="H64" s="1" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>NR119</t>
         </is>
       </c>
     </row>
@@ -3088,32 +3088,32 @@
       </c>
       <c r="C65" s="1" t="inlineStr">
         <is>
-          <t>MM-352M</t>
+          <t>MM-282M</t>
         </is>
       </c>
       <c r="D65" s="1" t="inlineStr">
         <is>
-          <t>MM-756M</t>
+          <t>MM-742M</t>
         </is>
       </c>
       <c r="E65" s="1" t="inlineStr">
         <is>
-          <t>MM-936M</t>
+          <t>MM-924M</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
         <is>
-          <t>MM-9954M</t>
+          <t>MM-9951M</t>
         </is>
       </c>
       <c r="G65" s="1" t="inlineStr">
         <is>
-          <t>NR48</t>
+          <t>NR43</t>
         </is>
       </c>
       <c r="H65" s="1" t="inlineStr">
         <is>
-          <t>P2501</t>
+          <t>NR120</t>
         </is>
       </c>
     </row>
@@ -3130,32 +3130,32 @@
       </c>
       <c r="C66" s="1" t="inlineStr">
         <is>
-          <t>MM-358M</t>
+          <t>MM-284M</t>
         </is>
       </c>
       <c r="D66" s="1" t="inlineStr">
         <is>
-          <t>MM-760M</t>
+          <t>MM-744M</t>
         </is>
       </c>
       <c r="E66" s="1" t="inlineStr">
         <is>
-          <t>MM-938M</t>
+          <t>MM-926M</t>
         </is>
       </c>
       <c r="F66" s="1" t="inlineStr">
         <is>
-          <t>MM-9955M</t>
+          <t>MM-9952M</t>
         </is>
       </c>
       <c r="G66" s="1" t="inlineStr">
         <is>
-          <t>NR51</t>
+          <t>NR44</t>
         </is>
       </c>
       <c r="H66" s="1" t="inlineStr">
         <is>
-          <t>P2502</t>
+          <t>NR122</t>
         </is>
       </c>
     </row>
@@ -3172,32 +3172,32 @@
       </c>
       <c r="C67" s="1" t="inlineStr">
         <is>
-          <t>MM-372M</t>
+          <t>MM-352M</t>
         </is>
       </c>
       <c r="D67" s="1" t="inlineStr">
         <is>
-          <t>MM-764M</t>
+          <t>MM-752M</t>
         </is>
       </c>
       <c r="E67" s="1" t="inlineStr">
         <is>
-          <t>MM-940M</t>
+          <t>MM-934M</t>
         </is>
       </c>
       <c r="F67" s="1" t="inlineStr">
         <is>
-          <t>MM-9957M</t>
+          <t>MM-9953M</t>
         </is>
       </c>
       <c r="G67" s="1" t="inlineStr">
         <is>
-          <t>NR52</t>
+          <t>NR45</t>
         </is>
       </c>
       <c r="H67" s="1" t="inlineStr">
         <is>
-          <t>P2503</t>
+          <t>P14</t>
         </is>
       </c>
     </row>
@@ -3214,32 +3214,32 @@
       </c>
       <c r="C68" s="1" t="inlineStr">
         <is>
-          <t>MM-378M</t>
+          <t>MM-358M</t>
         </is>
       </c>
       <c r="D68" s="1" t="inlineStr">
         <is>
-          <t>MM-768M</t>
+          <t>MM-756M</t>
         </is>
       </c>
       <c r="E68" s="1" t="inlineStr">
         <is>
-          <t>MM-944M</t>
+          <t>MM-936M</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
         <is>
-          <t>MM-9959M</t>
+          <t>MM-9954M</t>
         </is>
       </c>
       <c r="G68" s="1" t="inlineStr">
         <is>
-          <t>NR53</t>
+          <t>NR47</t>
         </is>
       </c>
       <c r="H68" s="1" t="inlineStr">
         <is>
-          <t>P2504</t>
+          <t>P16</t>
         </is>
       </c>
     </row>
@@ -3256,32 +3256,32 @@
       </c>
       <c r="C69" s="1" t="inlineStr">
         <is>
-          <t>MM-382M</t>
+          <t>MM-372M</t>
         </is>
       </c>
       <c r="D69" s="1" t="inlineStr">
         <is>
-          <t>MM-774M</t>
+          <t>MM-760M</t>
         </is>
       </c>
       <c r="E69" s="1" t="inlineStr">
         <is>
-          <t>MM-948M</t>
+          <t>MM-938M</t>
         </is>
       </c>
       <c r="F69" s="1" t="inlineStr">
         <is>
-          <t>MM-9960M</t>
+          <t>MM-9955M</t>
         </is>
       </c>
       <c r="G69" s="1" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>NR48</t>
         </is>
       </c>
       <c r="H69" s="1" t="inlineStr">
         <is>
-          <t>P2505</t>
+          <t>P2501</t>
         </is>
       </c>
     </row>
@@ -3298,32 +3298,32 @@
       </c>
       <c r="C70" s="1" t="inlineStr">
         <is>
-          <t>MM-392M</t>
+          <t>MM-378M</t>
         </is>
       </c>
       <c r="D70" s="1" t="inlineStr">
         <is>
-          <t>MM-776M</t>
+          <t>MM-764M</t>
         </is>
       </c>
       <c r="E70" s="1" t="inlineStr">
         <is>
-          <t>MM-952M</t>
+          <t>MM-940M</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
         <is>
-          <t>MM-9961M</t>
+          <t>MM-9957M</t>
         </is>
       </c>
       <c r="G70" s="1" t="inlineStr">
         <is>
-          <t>NR57</t>
+          <t>NR51</t>
         </is>
       </c>
       <c r="H70" s="1" t="inlineStr">
         <is>
-          <t>P2506</t>
+          <t>P2502</t>
         </is>
       </c>
     </row>
@@ -3340,32 +3340,32 @@
       </c>
       <c r="C71" s="1" t="inlineStr">
         <is>
-          <t>MM-418M</t>
+          <t>MM-382M</t>
         </is>
       </c>
       <c r="D71" s="1" t="inlineStr">
         <is>
-          <t>MM-778M</t>
+          <t>MM-768M</t>
         </is>
       </c>
       <c r="E71" s="1" t="inlineStr">
         <is>
-          <t>MM-954M</t>
+          <t>MM-944M</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
         <is>
-          <t>MM-9962M</t>
+          <t>MM-9959M</t>
         </is>
       </c>
       <c r="G71" s="1" t="inlineStr">
         <is>
-          <t>NR59</t>
+          <t>NR52</t>
         </is>
       </c>
       <c r="H71" s="1" t="inlineStr">
         <is>
-          <t>P2507</t>
+          <t>P2503</t>
         </is>
       </c>
     </row>
@@ -3382,32 +3382,32 @@
       </c>
       <c r="C72" s="1" t="inlineStr">
         <is>
-          <t>MM-430M</t>
+          <t>MM-392M</t>
         </is>
       </c>
       <c r="D72" s="1" t="inlineStr">
         <is>
-          <t>MM-780M</t>
+          <t>MM-774M</t>
         </is>
       </c>
       <c r="E72" s="1" t="inlineStr">
         <is>
-          <t>MM-956M</t>
+          <t>MM-948M</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
         <is>
-          <t>MM-9963M</t>
+          <t>MM-9960M</t>
         </is>
       </c>
       <c r="G72" s="1" t="inlineStr">
         <is>
-          <t>NR61</t>
+          <t>NR53</t>
         </is>
       </c>
       <c r="H72" s="1" t="inlineStr">
         <is>
-          <t>P2508</t>
+          <t>P2504</t>
         </is>
       </c>
     </row>
@@ -3424,32 +3424,32 @@
       </c>
       <c r="C73" s="1" t="inlineStr">
         <is>
-          <t>MM-444M</t>
+          <t>MM-418M</t>
         </is>
       </c>
       <c r="D73" s="1" t="inlineStr">
         <is>
-          <t>MM-784M</t>
+          <t>MM-776M</t>
         </is>
       </c>
       <c r="E73" s="1" t="inlineStr">
         <is>
-          <t>MM-958M</t>
+          <t>MM-952M</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
         <is>
-          <t>MM-9964M</t>
+          <t>MM-9961M</t>
         </is>
       </c>
       <c r="G73" s="1" t="inlineStr">
         <is>
-          <t>NR62</t>
+          <t>NR54</t>
         </is>
       </c>
       <c r="H73" s="1" t="inlineStr">
         <is>
-          <t>P2509</t>
+          <t>P2505</t>
         </is>
       </c>
     </row>
@@ -3466,32 +3466,32 @@
       </c>
       <c r="C74" s="1" t="inlineStr">
         <is>
-          <t>MM-464M</t>
+          <t>MM-430M</t>
         </is>
       </c>
       <c r="D74" s="1" t="inlineStr">
         <is>
-          <t>MM-790M</t>
+          <t>MM-778M</t>
         </is>
       </c>
       <c r="E74" s="1" t="inlineStr">
         <is>
-          <t>MM-962M</t>
+          <t>MM-954M</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
         <is>
-          <t>MM-9965M</t>
+          <t>MM-9962M</t>
         </is>
       </c>
       <c r="G74" s="1" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR57</t>
         </is>
       </c>
       <c r="H74" s="1" t="inlineStr">
         <is>
-          <t>P2510</t>
+          <t>P2506</t>
         </is>
       </c>
     </row>
@@ -3508,32 +3508,32 @@
       </c>
       <c r="C75" s="1" t="inlineStr">
         <is>
-          <t>MM-486M</t>
+          <t>MM-444M</t>
         </is>
       </c>
       <c r="D75" s="1" t="inlineStr">
         <is>
-          <t>MM-792M</t>
+          <t>MM-780M</t>
         </is>
       </c>
       <c r="E75" s="1" t="inlineStr">
         <is>
-          <t>MM-964M</t>
+          <t>MM-956M</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
         <is>
-          <t>MM-9966M</t>
+          <t>MM-9963M</t>
         </is>
       </c>
       <c r="G75" s="1" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR59</t>
         </is>
       </c>
       <c r="H75" s="1" t="inlineStr">
         <is>
-          <t>P2511</t>
+          <t>P2507</t>
         </is>
       </c>
     </row>
@@ -3550,32 +3550,32 @@
       </c>
       <c r="C76" s="1" t="inlineStr">
         <is>
-          <t>MM-496M</t>
+          <t>MM-464M</t>
         </is>
       </c>
       <c r="D76" s="1" t="inlineStr">
         <is>
-          <t>MM-796M</t>
+          <t>MM-784M</t>
         </is>
       </c>
       <c r="E76" s="1" t="inlineStr">
         <is>
-          <t>MM-966M</t>
+          <t>MM-958M</t>
         </is>
       </c>
       <c r="F76" s="1" t="inlineStr">
         <is>
-          <t>MM-9967M</t>
+          <t>MM-9964M</t>
         </is>
       </c>
       <c r="G76" s="1" t="inlineStr">
         <is>
-          <t>NR66</t>
+          <t>NR61</t>
         </is>
       </c>
       <c r="H76" s="1" t="inlineStr">
         <is>
-          <t>P2513</t>
+          <t>P2508</t>
         </is>
       </c>
     </row>
@@ -3592,32 +3592,32 @@
       </c>
       <c r="C77" s="1" t="inlineStr">
         <is>
-          <t>MM-514M</t>
+          <t>MM-486M</t>
         </is>
       </c>
       <c r="D77" s="1" t="inlineStr">
         <is>
-          <t>MM-798M</t>
+          <t>MM-790M</t>
         </is>
       </c>
       <c r="E77" s="1" t="inlineStr">
         <is>
-          <t>MM-968M</t>
+          <t>MM-962M</t>
         </is>
       </c>
       <c r="F77" s="1" t="inlineStr">
         <is>
-          <t>MM-9969M</t>
+          <t>MM-9965M</t>
         </is>
       </c>
       <c r="G77" s="1" t="inlineStr">
         <is>
-          <t>NR67</t>
+          <t>NR62</t>
         </is>
       </c>
       <c r="H77" s="1" t="inlineStr">
         <is>
-          <t>P2514</t>
+          <t>P2509</t>
         </is>
       </c>
     </row>
@@ -3634,32 +3634,32 @@
       </c>
       <c r="C78" s="1" t="inlineStr">
         <is>
-          <t>MM-526M</t>
+          <t>MM-496M</t>
         </is>
       </c>
       <c r="D78" s="1" t="inlineStr">
         <is>
-          <t>MM-800M</t>
+          <t>MM-792M</t>
         </is>
       </c>
       <c r="E78" s="1" t="inlineStr">
         <is>
-          <t>MM-970M</t>
+          <t>MM-964M</t>
         </is>
       </c>
       <c r="F78" s="1" t="inlineStr">
         <is>
-          <t>MM-9970M</t>
+          <t>MM-9966M</t>
         </is>
       </c>
       <c r="G78" s="1" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR64</t>
         </is>
       </c>
       <c r="H78" s="1" t="inlineStr">
         <is>
-          <t>P2515</t>
+          <t>P2510</t>
         </is>
       </c>
     </row>
@@ -3676,32 +3676,32 @@
       </c>
       <c r="C79" s="1" t="inlineStr">
         <is>
-          <t>MM-534M</t>
+          <t>MM-514M</t>
         </is>
       </c>
       <c r="D79" s="1" t="inlineStr">
         <is>
-          <t>MM-802M</t>
+          <t>MM-796M</t>
         </is>
       </c>
       <c r="E79" s="1" t="inlineStr">
         <is>
-          <t>MM-972M</t>
+          <t>MM-966M</t>
         </is>
       </c>
       <c r="F79" s="1" t="inlineStr">
         <is>
-          <t>MMY032</t>
+          <t>MM-9967M</t>
         </is>
       </c>
       <c r="G79" s="1" t="inlineStr">
         <is>
-          <t>NR69</t>
+          <t>NR65</t>
         </is>
       </c>
       <c r="H79" s="1" t="inlineStr">
         <is>
-          <t>P2516</t>
+          <t>P2511</t>
         </is>
       </c>
     </row>
@@ -3718,32 +3718,32 @@
       </c>
       <c r="C80" s="1" t="inlineStr">
         <is>
-          <t>MM-536M</t>
+          <t>MM-526M</t>
         </is>
       </c>
       <c r="D80" s="1" t="inlineStr">
         <is>
-          <t>MM-804M</t>
+          <t>MM-798M</t>
         </is>
       </c>
       <c r="E80" s="1" t="inlineStr">
         <is>
-          <t>MM-974M</t>
+          <t>MM-968M</t>
         </is>
       </c>
       <c r="F80" s="1" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MM-9968M</t>
         </is>
       </c>
       <c r="G80" s="1" t="inlineStr">
         <is>
-          <t>NR71</t>
+          <t>NR66</t>
         </is>
       </c>
       <c r="H80" s="1" t="inlineStr">
         <is>
-          <t>PB1</t>
+          <t>P2513</t>
         </is>
       </c>
     </row>
@@ -3760,32 +3760,32 @@
       </c>
       <c r="C81" s="1" t="inlineStr">
         <is>
-          <t>MM-542M</t>
+          <t>MM-534M</t>
         </is>
       </c>
       <c r="D81" s="1" t="inlineStr">
         <is>
-          <t>MM-808M</t>
+          <t>MM-800M</t>
         </is>
       </c>
       <c r="E81" s="1" t="inlineStr">
         <is>
-          <t>MM-976M</t>
+          <t>MM-970M</t>
         </is>
       </c>
       <c r="F81" s="1" t="inlineStr">
         <is>
-          <t>MRL004</t>
+          <t>MM-9969M</t>
         </is>
       </c>
       <c r="G81" s="1" t="inlineStr">
         <is>
-          <t>NR72</t>
+          <t>NR67</t>
         </is>
       </c>
       <c r="H81" s="1" t="inlineStr">
         <is>
-          <t>PB2</t>
+          <t>P2514</t>
         </is>
       </c>
     </row>
@@ -3802,32 +3802,32 @@
       </c>
       <c r="C82" s="1" t="inlineStr">
         <is>
-          <t>MM-544M</t>
+          <t>MM-536M</t>
         </is>
       </c>
       <c r="D82" s="1" t="inlineStr">
         <is>
-          <t>MM-810M</t>
+          <t>MM-802M</t>
         </is>
       </c>
       <c r="E82" s="1" t="inlineStr">
         <is>
-          <t>MM-980M</t>
+          <t>MM-972M</t>
         </is>
       </c>
       <c r="F82" s="1" t="inlineStr">
         <is>
-          <t>MRL006</t>
+          <t>MM-9970M</t>
         </is>
       </c>
       <c r="G82" s="1" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR68</t>
         </is>
       </c>
       <c r="H82" s="1" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>P2515</t>
         </is>
       </c>
     </row>
@@ -3844,32 +3844,32 @@
       </c>
       <c r="C83" s="1" t="inlineStr">
         <is>
-          <t>MM-546M</t>
+          <t>MM-542M</t>
         </is>
       </c>
       <c r="D83" s="1" t="inlineStr">
         <is>
-          <t>MM-814M</t>
+          <t>MM-804M</t>
         </is>
       </c>
       <c r="E83" s="1" t="inlineStr">
         <is>
-          <t>MM-982M</t>
+          <t>MM-974M</t>
         </is>
       </c>
       <c r="F83" s="1" t="inlineStr">
         <is>
-          <t>N452</t>
+          <t>MMY032</t>
         </is>
       </c>
       <c r="G83" s="1" t="inlineStr">
         <is>
-          <t>NR77</t>
+          <t>NR69</t>
         </is>
       </c>
       <c r="H83" s="1" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>P2516</t>
         </is>
       </c>
     </row>
@@ -3886,32 +3886,32 @@
       </c>
       <c r="C84" s="1" t="inlineStr">
         <is>
-          <t>MM-551M</t>
+          <t>MM-544M</t>
         </is>
       </c>
       <c r="D84" s="1" t="inlineStr">
         <is>
-          <t>MM-816M</t>
+          <t>MM-808M</t>
         </is>
       </c>
       <c r="E84" s="1" t="inlineStr">
         <is>
-          <t>MM-984M</t>
+          <t>MM-976M</t>
         </is>
       </c>
       <c r="F84" s="1" t="inlineStr">
         <is>
-          <t>N453</t>
+          <t>MRL001</t>
         </is>
       </c>
       <c r="G84" s="1" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR71</t>
         </is>
       </c>
       <c r="H84" s="1" t="inlineStr">
         <is>
-          <t>PHC002</t>
+          <t>PB1</t>
         </is>
       </c>
     </row>
@@ -3928,32 +3928,32 @@
       </c>
       <c r="C85" s="1" t="inlineStr">
         <is>
-          <t>MM-552M</t>
+          <t>MM-546M</t>
         </is>
       </c>
       <c r="D85" s="1" t="inlineStr">
         <is>
-          <t>MM-818M</t>
+          <t>MM-810M</t>
         </is>
       </c>
       <c r="E85" s="1" t="inlineStr">
         <is>
-          <t>MM-986M</t>
+          <t>MM-980M</t>
         </is>
       </c>
       <c r="F85" s="1" t="inlineStr">
         <is>
-          <t>N457</t>
+          <t>MRL004</t>
         </is>
       </c>
       <c r="G85" s="1" t="inlineStr">
         <is>
-          <t>NR81</t>
+          <t>NR72</t>
         </is>
       </c>
       <c r="H85" s="1" t="inlineStr">
         <is>
-          <t>Q4001</t>
+          <t>PB2</t>
         </is>
       </c>
     </row>
@@ -3970,32 +3970,32 @@
       </c>
       <c r="C86" s="1" t="inlineStr">
         <is>
-          <t>MM-580M</t>
+          <t>MM-550M</t>
         </is>
       </c>
       <c r="D86" s="1" t="inlineStr">
         <is>
-          <t>MM-820M</t>
+          <t>MM-814M</t>
         </is>
       </c>
       <c r="E86" s="1" t="inlineStr">
         <is>
-          <t>MM-9902M</t>
+          <t>MM-982M</t>
         </is>
       </c>
       <c r="F86" s="1" t="inlineStr">
         <is>
-          <t>N458</t>
+          <t>MRL006</t>
         </is>
       </c>
       <c r="G86" s="1" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR75</t>
         </is>
       </c>
       <c r="H86" s="1" t="inlineStr">
         <is>
-          <t>Q4003</t>
+          <t>PB4</t>
         </is>
       </c>
     </row>
@@ -4012,32 +4012,32 @@
       </c>
       <c r="C87" s="1" t="inlineStr">
         <is>
-          <t>MM-588M</t>
+          <t>MM-551M</t>
         </is>
       </c>
       <c r="D87" s="1" t="inlineStr">
         <is>
-          <t>MM-824M</t>
+          <t>MM-816M</t>
         </is>
       </c>
       <c r="E87" s="1" t="inlineStr">
         <is>
-          <t>MM-9903M</t>
+          <t>MM-984M</t>
         </is>
       </c>
       <c r="F87" s="1" t="inlineStr">
         <is>
-          <t>N461</t>
+          <t>N452</t>
         </is>
       </c>
       <c r="G87" s="1" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR77</t>
         </is>
       </c>
       <c r="H87" s="1" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
@@ -4054,32 +4054,32 @@
       </c>
       <c r="C88" s="1" t="inlineStr">
         <is>
-          <t>MM-602M</t>
+          <t>MM-552M</t>
         </is>
       </c>
       <c r="D88" s="1" t="inlineStr">
         <is>
-          <t>MM-826M</t>
+          <t>MM-818M</t>
         </is>
       </c>
       <c r="E88" s="1" t="inlineStr">
         <is>
-          <t>MM-9904M</t>
+          <t>MM-986M</t>
         </is>
       </c>
       <c r="F88" s="1" t="inlineStr">
         <is>
-          <t>N465</t>
+          <t>N453</t>
         </is>
       </c>
       <c r="G88" s="1" t="inlineStr">
         <is>
-          <t>NR84</t>
+          <t>NR78</t>
         </is>
       </c>
       <c r="H88" s="1" t="inlineStr">
         <is>
-          <t>Q4005</t>
+          <t>PHC002</t>
         </is>
       </c>
     </row>
@@ -4096,32 +4096,32 @@
       </c>
       <c r="C89" s="1" t="inlineStr">
         <is>
-          <t>MM-608M</t>
+          <t>MM-580M</t>
         </is>
       </c>
       <c r="D89" s="1" t="inlineStr">
         <is>
-          <t>MM-828M</t>
+          <t>MM-820M</t>
         </is>
       </c>
       <c r="E89" s="1" t="inlineStr">
         <is>
-          <t>MM-9906M</t>
+          <t>MM-9902M</t>
         </is>
       </c>
       <c r="F89" s="1" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>N457</t>
         </is>
       </c>
       <c r="G89" s="1" t="inlineStr">
         <is>
-          <t>NR85</t>
+          <t>NR81</t>
         </is>
       </c>
       <c r="H89" s="1" t="inlineStr">
         <is>
-          <t>Q4006</t>
+          <t>Q4001</t>
         </is>
       </c>
     </row>
@@ -4138,32 +4138,32 @@
       </c>
       <c r="C90" s="1" t="inlineStr">
         <is>
-          <t>MM-616M</t>
+          <t>MM-588M</t>
         </is>
       </c>
       <c r="D90" s="1" t="inlineStr">
         <is>
-          <t>MM-830M</t>
+          <t>MM-824M</t>
         </is>
       </c>
       <c r="E90" s="1" t="inlineStr">
         <is>
-          <t>MM-9907M</t>
+          <t>MM-9903M</t>
         </is>
       </c>
       <c r="F90" s="1" t="inlineStr">
         <is>
-          <t>N467</t>
+          <t>N458</t>
         </is>
       </c>
       <c r="G90" s="1" t="inlineStr">
         <is>
-          <t>NR86</t>
+          <t>NR82</t>
         </is>
       </c>
       <c r="H90" s="1" t="inlineStr">
         <is>
-          <t>Q4007</t>
+          <t>Q4003</t>
         </is>
       </c>
     </row>
@@ -4180,32 +4180,32 @@
       </c>
       <c r="C91" s="1" t="inlineStr">
         <is>
-          <t>MM-624M</t>
+          <t>MM-602M</t>
         </is>
       </c>
       <c r="D91" s="1" t="inlineStr">
         <is>
-          <t>MM-832M</t>
+          <t>MM-826M</t>
         </is>
       </c>
       <c r="E91" s="1" t="inlineStr">
         <is>
-          <t>MM-9908M</t>
+          <t>MM-9904M</t>
         </is>
       </c>
       <c r="F91" s="1" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>N461</t>
         </is>
       </c>
       <c r="G91" s="1" t="inlineStr">
         <is>
-          <t>NR87</t>
+          <t>NR83</t>
         </is>
       </c>
       <c r="H91" s="1" t="inlineStr">
         <is>
-          <t>Q4009</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
@@ -4222,32 +4222,32 @@
       </c>
       <c r="C92" s="1" t="inlineStr">
         <is>
-          <t>MM-632M</t>
+          <t>MM-608M</t>
         </is>
       </c>
       <c r="D92" s="1" t="inlineStr">
         <is>
-          <t>MM-834M</t>
+          <t>MM-828M</t>
         </is>
       </c>
       <c r="E92" s="1" t="inlineStr">
         <is>
-          <t>MM-9909M</t>
+          <t>MM-9906M</t>
         </is>
       </c>
       <c r="F92" s="1" t="inlineStr">
         <is>
-          <t>N473</t>
+          <t>N465</t>
         </is>
       </c>
       <c r="G92" s="1" t="inlineStr">
         <is>
-          <t>NR88</t>
+          <t>NR84</t>
         </is>
       </c>
       <c r="H92" s="1" t="inlineStr">
         <is>
-          <t>Q4011</t>
+          <t>Q4005</t>
         </is>
       </c>
     </row>
@@ -4264,32 +4264,32 @@
       </c>
       <c r="C93" s="1" t="inlineStr">
         <is>
-          <t>MM-636M</t>
+          <t>MM-616M</t>
         </is>
       </c>
       <c r="D93" s="1" t="inlineStr">
         <is>
-          <t>MM-838M</t>
+          <t>MM-830M</t>
         </is>
       </c>
       <c r="E93" s="1" t="inlineStr">
         <is>
-          <t>MM-9912M</t>
+          <t>MM-9907M</t>
         </is>
       </c>
       <c r="F93" s="1" t="inlineStr">
         <is>
-          <t>NR1</t>
+          <t>N466</t>
         </is>
       </c>
       <c r="G93" s="1" t="inlineStr">
         <is>
-          <t>NR89</t>
+          <t>NR85</t>
         </is>
       </c>
       <c r="H93" s="1" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>Q4006</t>
         </is>
       </c>
     </row>
@@ -4306,32 +4306,32 @@
       </c>
       <c r="C94" s="1" t="inlineStr">
         <is>
-          <t>MM-640M</t>
+          <t>MM-624M</t>
         </is>
       </c>
       <c r="D94" s="1" t="inlineStr">
         <is>
-          <t>MM-840M</t>
+          <t>MM-832M</t>
         </is>
       </c>
       <c r="E94" s="1" t="inlineStr">
         <is>
-          <t>MM-9913M</t>
+          <t>MM-9908M</t>
         </is>
       </c>
       <c r="F94" s="1" t="inlineStr">
         <is>
-          <t>NR2</t>
+          <t>N467</t>
         </is>
       </c>
       <c r="G94" s="1" t="inlineStr">
         <is>
-          <t>NR90</t>
+          <t>NR86</t>
         </is>
       </c>
       <c r="H94" s="1" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>Q4007</t>
         </is>
       </c>
     </row>
@@ -4348,32 +4348,32 @@
       </c>
       <c r="C95" s="1" t="inlineStr">
         <is>
-          <t>MM-654M</t>
+          <t>MM-632M</t>
         </is>
       </c>
       <c r="D95" s="1" t="inlineStr">
         <is>
-          <t>MM-842M</t>
+          <t>MM-834M</t>
         </is>
       </c>
       <c r="E95" s="1" t="inlineStr">
         <is>
-          <t>MM-9914M</t>
+          <t>MM-9909M</t>
         </is>
       </c>
       <c r="F95" s="1" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>N469</t>
         </is>
       </c>
       <c r="G95" s="1" t="inlineStr">
         <is>
-          <t>NR91</t>
+          <t>NR87</t>
         </is>
       </c>
       <c r="H95" s="1" t="inlineStr">
         <is>
-          <t>Q4014</t>
+          <t>Q4009</t>
         </is>
       </c>
     </row>
@@ -4390,32 +4390,32 @@
       </c>
       <c r="C96" s="1" t="inlineStr">
         <is>
-          <t>MM-656M</t>
+          <t>MM-636M</t>
         </is>
       </c>
       <c r="D96" s="1" t="inlineStr">
         <is>
-          <t>MM-844M</t>
+          <t>MM-838M</t>
         </is>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>MM-9915M</t>
+          <t>MM-9912M</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>N473</t>
         </is>
       </c>
       <c r="G96" s="1" t="inlineStr">
         <is>
-          <t>NR92</t>
+          <t>NR88</t>
         </is>
       </c>
       <c r="H96" s="1" t="inlineStr">
         <is>
-          <t>Q4015</t>
+          <t>Q4011</t>
         </is>
       </c>
     </row>
@@ -4432,32 +4432,32 @@
       </c>
       <c r="C97" s="1" t="inlineStr">
         <is>
-          <t>MM-660M</t>
+          <t>MM-640M</t>
         </is>
       </c>
       <c r="D97" s="1" t="inlineStr">
         <is>
-          <t>MM-852M</t>
+          <t>MM-840M</t>
         </is>
       </c>
       <c r="E97" s="1" t="inlineStr">
         <is>
-          <t>MM-9917M</t>
+          <t>MM-9913M</t>
         </is>
       </c>
       <c r="F97" s="1" t="inlineStr">
         <is>
-          <t>NR7</t>
+          <t>NR1</t>
         </is>
       </c>
       <c r="G97" s="1" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR89</t>
         </is>
       </c>
       <c r="H97" s="1" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
@@ -4474,32 +4474,32 @@
       </c>
       <c r="C98" s="1" t="inlineStr">
         <is>
-          <t>MM-661M</t>
+          <t>MM-654M</t>
         </is>
       </c>
       <c r="D98" s="1" t="inlineStr">
         <is>
-          <t>MM-858M</t>
+          <t>MM-842M</t>
         </is>
       </c>
       <c r="E98" s="1" t="inlineStr">
         <is>
-          <t>MM-9918M</t>
+          <t>MM-9914M</t>
         </is>
       </c>
       <c r="F98" s="1" t="inlineStr">
         <is>
-          <t>NR8</t>
+          <t>NR2</t>
         </is>
       </c>
       <c r="G98" s="1" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR90</t>
         </is>
       </c>
       <c r="H98" s="1" t="inlineStr">
         <is>
-          <t>Q4017</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
@@ -4516,32 +4516,32 @@
       </c>
       <c r="C99" s="1" t="inlineStr">
         <is>
-          <t>MM-662M</t>
+          <t>MM-656M</t>
         </is>
       </c>
       <c r="D99" s="1" t="inlineStr">
         <is>
-          <t>MM-860M</t>
+          <t>MM-844M</t>
         </is>
       </c>
       <c r="E99" s="1" t="inlineStr">
         <is>
-          <t>MM-9919M</t>
+          <t>MM-9915M</t>
         </is>
       </c>
       <c r="F99" s="1" t="inlineStr">
         <is>
-          <t>NR9</t>
+          <t>NR4</t>
         </is>
       </c>
       <c r="G99" s="1" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR91</t>
         </is>
       </c>
       <c r="H99" s="1" t="inlineStr">
         <is>
-          <t>Q4019</t>
+          <t>Q4014</t>
         </is>
       </c>
     </row>
@@ -4558,32 +4558,32 @@
       </c>
       <c r="C100" s="1" t="inlineStr">
         <is>
-          <t>MM-664M</t>
+          <t>MM-660M</t>
         </is>
       </c>
       <c r="D100" s="1" t="inlineStr">
         <is>
-          <t>MM-862M</t>
+          <t>MM-852M</t>
         </is>
       </c>
       <c r="E100" s="1" t="inlineStr">
         <is>
-          <t>MM-9920M</t>
+          <t>MM-9917M</t>
         </is>
       </c>
       <c r="F100" s="1" t="inlineStr">
         <is>
-          <t>NR12</t>
+          <t>NR5</t>
         </is>
       </c>
       <c r="G100" s="1" t="inlineStr">
         <is>
-          <t>NR96</t>
+          <t>NR92</t>
         </is>
       </c>
       <c r="H100" s="1" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>Q4015</t>
         </is>
       </c>
     </row>
@@ -4600,32 +4600,32 @@
       </c>
       <c r="C101" s="1" t="inlineStr">
         <is>
-          <t>MM-666M</t>
+          <t>MM-661M</t>
         </is>
       </c>
       <c r="D101" s="1" t="inlineStr">
         <is>
-          <t>MM-868M</t>
+          <t>MM-858M</t>
         </is>
       </c>
       <c r="E101" s="1" t="inlineStr">
         <is>
-          <t>MM-9922M</t>
+          <t>MM-9918M</t>
         </is>
       </c>
       <c r="F101" s="1" t="inlineStr">
         <is>
-          <t>NR15</t>
+          <t>NR7</t>
         </is>
       </c>
       <c r="G101" s="1" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>NR93</t>
         </is>
       </c>
       <c r="H101" s="1" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
@@ -4642,32 +4642,32 @@
       </c>
       <c r="C102" s="1" t="inlineStr">
         <is>
-          <t>MM-668M</t>
+          <t>MM-662M</t>
         </is>
       </c>
       <c r="D102" s="1" t="inlineStr">
         <is>
-          <t>MM-870M</t>
+          <t>MM-860M</t>
         </is>
       </c>
       <c r="E102" s="1" t="inlineStr">
         <is>
-          <t>MM-9923M</t>
+          <t>MM-9919M</t>
         </is>
       </c>
       <c r="F102" s="1" t="inlineStr">
         <is>
-          <t>NR16</t>
+          <t>NR8</t>
         </is>
       </c>
       <c r="G102" s="1" t="inlineStr">
         <is>
-          <t>NR98</t>
+          <t>NR94</t>
         </is>
       </c>
       <c r="H102" s="1" t="inlineStr">
         <is>
-          <t>QBX005</t>
+          <t>Q4017</t>
         </is>
       </c>
     </row>
@@ -4684,32 +4684,32 @@
       </c>
       <c r="C103" s="1" t="inlineStr">
         <is>
-          <t>MM-673M</t>
+          <t>MM-664M</t>
         </is>
       </c>
       <c r="D103" s="1" t="inlineStr">
         <is>
-          <t>MM-872M</t>
+          <t>MM-862M</t>
         </is>
       </c>
       <c r="E103" s="1" t="inlineStr">
         <is>
-          <t>MM-9924M</t>
+          <t>MM-9920M</t>
         </is>
       </c>
       <c r="F103" s="1" t="inlineStr">
         <is>
-          <t>NR18</t>
+          <t>NR9</t>
         </is>
       </c>
       <c r="G103" s="1" t="inlineStr">
         <is>
-          <t>NR99</t>
+          <t>NR95</t>
         </is>
       </c>
       <c r="H103" s="1" t="inlineStr">
         <is>
-          <t>QBX006</t>
+          <t>Q4019</t>
         </is>
       </c>
     </row>
@@ -4726,32 +4726,32 @@
       </c>
       <c r="C104" s="1" t="inlineStr">
         <is>
-          <t>MM-674M</t>
+          <t>MM-666M</t>
         </is>
       </c>
       <c r="D104" s="1" t="inlineStr">
         <is>
-          <t>MM-874M</t>
+          <t>MM-868M</t>
         </is>
       </c>
       <c r="E104" s="1" t="inlineStr">
         <is>
-          <t>MM-9926M</t>
+          <t>MM-9922M</t>
         </is>
       </c>
       <c r="F104" s="1" t="inlineStr">
         <is>
-          <t>NR19</t>
+          <t>NR12</t>
         </is>
       </c>
       <c r="G104" s="1" t="inlineStr">
         <is>
-          <t>NR101</t>
+          <t>NR96</t>
         </is>
       </c>
       <c r="H104" s="1" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
@@ -4768,32 +4768,32 @@
       </c>
       <c r="C105" s="1" t="inlineStr">
         <is>
-          <t>MM-676M</t>
+          <t>MM-668M</t>
         </is>
       </c>
       <c r="D105" s="1" t="inlineStr">
         <is>
-          <t>MM-876M</t>
+          <t>MM-870M</t>
         </is>
       </c>
       <c r="E105" s="1" t="inlineStr">
         <is>
-          <t>MM-9928M</t>
+          <t>MM-9923M</t>
         </is>
       </c>
       <c r="F105" s="1" t="inlineStr">
         <is>
-          <t>NR21</t>
+          <t>NR15</t>
         </is>
       </c>
       <c r="G105" s="1" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR97</t>
         </is>
       </c>
       <c r="H105" s="1" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
@@ -4810,32 +4810,32 @@
       </c>
       <c r="C106" s="1" t="inlineStr">
         <is>
-          <t>MM-680M</t>
+          <t>MM-673M</t>
         </is>
       </c>
       <c r="D106" s="1" t="inlineStr">
         <is>
-          <t>MM-882M</t>
+          <t>MM-872M</t>
         </is>
       </c>
       <c r="E106" s="1" t="inlineStr">
         <is>
-          <t>MM-9929M</t>
+          <t>MM-9924M</t>
         </is>
       </c>
       <c r="F106" s="1" t="inlineStr">
         <is>
-          <t>NR25</t>
+          <t>NR16</t>
         </is>
       </c>
       <c r="G106" s="1" t="inlineStr">
         <is>
-          <t>NR103</t>
+          <t>NR98</t>
         </is>
       </c>
       <c r="H106" s="1" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>QBX005</t>
         </is>
       </c>
     </row>
@@ -4852,32 +4852,32 @@
       </c>
       <c r="C107" s="1" t="inlineStr">
         <is>
-          <t>MM-706M</t>
+          <t>MM-674M</t>
         </is>
       </c>
       <c r="D107" s="1" t="inlineStr">
         <is>
-          <t>MM-894M</t>
+          <t>MM-874M</t>
         </is>
       </c>
       <c r="E107" s="1" t="inlineStr">
         <is>
-          <t>MM-9932M</t>
+          <t>MM-9926M</t>
         </is>
       </c>
       <c r="F107" s="1" t="inlineStr">
         <is>
-          <t>NR27</t>
+          <t>NR18</t>
         </is>
       </c>
       <c r="G107" s="1" t="inlineStr">
         <is>
-          <t>NR105</t>
+          <t>NR99</t>
         </is>
       </c>
       <c r="H107" s="1" t="inlineStr">
         <is>
-          <t>QE004</t>
+          <t>QBX006</t>
         </is>
       </c>
     </row>
@@ -4894,32 +4894,32 @@
       </c>
       <c r="C108" s="1" t="inlineStr">
         <is>
-          <t>MM-708M</t>
+          <t>MM-676M</t>
         </is>
       </c>
       <c r="D108" s="1" t="inlineStr">
         <is>
-          <t>MM-896M</t>
+          <t>MM-876M</t>
         </is>
       </c>
       <c r="E108" s="1" t="inlineStr">
         <is>
-          <t>MM-9933M</t>
+          <t>MM-9928M</t>
         </is>
       </c>
       <c r="F108" s="1" t="inlineStr">
         <is>
-          <t>NR28</t>
+          <t>NR19</t>
         </is>
       </c>
       <c r="G108" s="1" t="inlineStr">
         <is>
-          <t>NR108</t>
+          <t>NR101</t>
         </is>
       </c>
       <c r="H108" s="1" t="inlineStr">
         <is>
-          <t>QE006</t>
+          <t>QE001</t>
         </is>
       </c>
     </row>
@@ -4936,32 +4936,32 @@
       </c>
       <c r="C109" s="1" t="inlineStr">
         <is>
-          <t>MM-710M</t>
+          <t>MM-680M</t>
         </is>
       </c>
       <c r="D109" s="1" t="inlineStr">
         <is>
-          <t>MM-902M</t>
+          <t>MM-882M</t>
         </is>
       </c>
       <c r="E109" s="1" t="inlineStr">
         <is>
-          <t>MM-9934M</t>
+          <t>MM-9929M</t>
         </is>
       </c>
       <c r="F109" s="1" t="inlineStr">
         <is>
-          <t>NR30</t>
+          <t>NR21</t>
         </is>
       </c>
       <c r="G109" s="1" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR102</t>
         </is>
       </c>
       <c r="H109" s="1" t="inlineStr">
         <is>
-          <t>QL001</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
@@ -4978,32 +4978,32 @@
       </c>
       <c r="C110" s="1" t="inlineStr">
         <is>
-          <t>MM-716M</t>
+          <t>MM-706M</t>
         </is>
       </c>
       <c r="D110" s="1" t="inlineStr">
         <is>
-          <t>MM-904M</t>
+          <t>MM-894M</t>
         </is>
       </c>
       <c r="E110" s="1" t="inlineStr">
         <is>
-          <t>MM-9936M</t>
+          <t>MM-9932M</t>
         </is>
       </c>
       <c r="F110" s="1" t="inlineStr">
         <is>
-          <t>NR31</t>
+          <t>NR25</t>
         </is>
       </c>
       <c r="G110" s="1" t="inlineStr">
         <is>
-          <t>NR110</t>
+          <t>NR103</t>
         </is>
       </c>
       <c r="H110" s="1" t="inlineStr">
         <is>
-          <t>QL002</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
@@ -5015,37 +5015,37 @@
       </c>
       <c r="B111" s="1" t="inlineStr">
         <is>
-          <t>MM-218M</t>
+          <t>MM-216M</t>
         </is>
       </c>
       <c r="C111" s="1" t="inlineStr">
         <is>
-          <t>MM-722M</t>
+          <t>MM-708M</t>
         </is>
       </c>
       <c r="D111" s="1" t="inlineStr">
         <is>
-          <t>MM-906M</t>
+          <t>MM-896M</t>
         </is>
       </c>
       <c r="E111" s="1" t="inlineStr">
         <is>
-          <t>MM-9938M</t>
+          <t>MM-9933M</t>
         </is>
       </c>
       <c r="F111" s="1" t="inlineStr">
         <is>
-          <t>NR34</t>
+          <t>NR27</t>
         </is>
       </c>
       <c r="G111" s="1" t="inlineStr">
         <is>
-          <t>NR111</t>
+          <t>NR105</t>
         </is>
       </c>
       <c r="H111" s="1" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>QE004</t>
         </is>
       </c>
     </row>
@@ -5057,37 +5057,37 @@
       </c>
       <c r="B112" s="1" t="inlineStr">
         <is>
-          <t>MM-222M</t>
+          <t>MM-218M</t>
         </is>
       </c>
       <c r="C112" s="1" t="inlineStr">
         <is>
-          <t>MM-726M</t>
+          <t>MM-710M</t>
         </is>
       </c>
       <c r="D112" s="1" t="inlineStr">
         <is>
-          <t>MM-908M</t>
+          <t>MM-902M</t>
         </is>
       </c>
       <c r="E112" s="1" t="inlineStr">
         <is>
-          <t>MM-9941M</t>
+          <t>MM-9934M</t>
         </is>
       </c>
       <c r="F112" s="1" t="inlineStr">
         <is>
-          <t>NR36</t>
+          <t>NR28</t>
         </is>
       </c>
       <c r="G112" s="1" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR108</t>
         </is>
       </c>
       <c r="H112" s="1" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>QE006</t>
         </is>
       </c>
     </row>
@@ -5099,2234 +5099,2254 @@
       </c>
       <c r="B113" s="1" t="inlineStr">
         <is>
-          <t>MM-224M</t>
+          <t>MM-222M</t>
         </is>
       </c>
       <c r="C113" s="1" t="inlineStr">
         <is>
-          <t>MM-728M</t>
+          <t>MM-716M</t>
         </is>
       </c>
       <c r="D113" s="1" t="inlineStr">
         <is>
-          <t>MM-910M</t>
+          <t>MM-904M</t>
         </is>
       </c>
       <c r="E113" s="1" t="inlineStr">
         <is>
-          <t>MM-9943M</t>
+          <t>MM-9936M</t>
         </is>
       </c>
       <c r="F113" s="1" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>NR30</t>
         </is>
       </c>
       <c r="G113" s="1" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR109</t>
         </is>
       </c>
       <c r="H113" s="1" t="inlineStr">
         <is>
-          <t>QL008</t>
+          <t>QL001</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>QL010</t>
+          <t>QL002</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>SCT015</t>
         </is>
       </c>
       <c r="C115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8029</t>
+          <t>VLINE-8025</t>
         </is>
       </c>
       <c r="D115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8152</t>
+          <t>VLINE-8145</t>
         </is>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8411</t>
+          <t>VLINE-8404</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8717</t>
+          <t>VLINE-8671</t>
         </is>
       </c>
       <c r="G115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8786</t>
+          <t>VLINE-8781</t>
         </is>
       </c>
       <c r="H115" s="1" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>XP2007</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>QL011</t>
+          <t>QL004</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>SO2</t>
         </is>
       </c>
       <c r="C116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8030</t>
+          <t>VLINE-8026</t>
         </is>
       </c>
       <c r="D116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8153</t>
+          <t>VLINE-8148</t>
         </is>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8413</t>
+          <t>VLINE-8406</t>
         </is>
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8720</t>
+          <t>VLINE-8706</t>
         </is>
       </c>
       <c r="G116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8787</t>
+          <t>VLINE-8782</t>
         </is>
       </c>
       <c r="H116" s="1" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>XP2008</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>QL014</t>
+          <t>QL007</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
         <is>
-          <t>T363</t>
+          <t>SSR101</t>
         </is>
       </c>
       <c r="C117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8031</t>
+          <t>VLINE-8027</t>
         </is>
       </c>
       <c r="D117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8154</t>
+          <t>VLINE-8150</t>
         </is>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8415</t>
+          <t>VLINE-8408</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8721</t>
+          <t>VLINE-8711</t>
         </is>
       </c>
       <c r="G117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8788</t>
+          <t>VLINE-8783</t>
         </is>
       </c>
       <c r="H117" s="1" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>XP2010</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>QL018</t>
+          <t>QL008</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
         <is>
-          <t>T386</t>
+          <t>SSR102</t>
         </is>
       </c>
       <c r="C118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8032</t>
+          <t>VLINE-8028</t>
         </is>
       </c>
       <c r="D118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8155</t>
+          <t>VLINE-8151</t>
         </is>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8417</t>
+          <t>VLINE-8410</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8723</t>
+          <t>VLINE-8714</t>
         </is>
       </c>
       <c r="G118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8790</t>
+          <t>VLINE-8784</t>
         </is>
       </c>
       <c r="H118" s="1" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>XP2011</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QL010</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
         <is>
-          <t>TDX101</t>
+          <t>SSR103</t>
         </is>
       </c>
       <c r="C119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8036</t>
+          <t>VLINE-8029</t>
         </is>
       </c>
       <c r="D119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8157</t>
+          <t>VLINE-8152</t>
         </is>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8418</t>
+          <t>VLINE-8411</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8725</t>
+          <t>VLINE-8717</t>
         </is>
       </c>
       <c r="G119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8792</t>
+          <t>VLINE-8786</t>
         </is>
       </c>
       <c r="H119" s="1" t="inlineStr">
         <is>
-          <t>XP2016</t>
+          <t>XP2012</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QL011</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>SSR104</t>
         </is>
       </c>
       <c r="C120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8038</t>
+          <t>VLINE-8030</t>
         </is>
       </c>
       <c r="D120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8158</t>
+          <t>VLINE-8153</t>
         </is>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8419</t>
+          <t>VLINE-8413</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8726</t>
+          <t>VLINE-8720</t>
         </is>
       </c>
       <c r="G120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8793</t>
+          <t>VLINE-8787</t>
         </is>
       </c>
       <c r="H120" s="1" t="inlineStr">
         <is>
-          <t>XP2017</t>
+          <t>XP2013</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QL014</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
         <is>
-          <t>TE2802</t>
+          <t>T363</t>
         </is>
       </c>
       <c r="C121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8042</t>
+          <t>VLINE-8031</t>
         </is>
       </c>
       <c r="D121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8159</t>
+          <t>VLINE-8154</t>
         </is>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8420</t>
+          <t>VLINE-8415</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8727</t>
+          <t>VLINE-8721</t>
         </is>
       </c>
       <c r="G121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8794</t>
+          <t>VLINE-8788</t>
         </is>
       </c>
       <c r="H121" s="1" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>XP2014</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>R711</t>
+          <t>QL018</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>T386</t>
         </is>
       </c>
       <c r="C122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8051</t>
+          <t>VLINE-8032</t>
         </is>
       </c>
       <c r="D122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8160</t>
+          <t>VLINE-8155</t>
         </is>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8421</t>
+          <t>VLINE-8417</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8729</t>
+          <t>VLINE-8723</t>
         </is>
       </c>
       <c r="G122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8795</t>
+          <t>VLINE-8790</t>
         </is>
       </c>
       <c r="H122" s="1" t="inlineStr">
         <is>
-          <t>XR552</t>
+          <t>XP2015</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>R766</t>
+          <t>QR1744</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
         <is>
-          <t>TE2804</t>
+          <t>TDX101</t>
         </is>
       </c>
       <c r="C123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8052</t>
+          <t>VLINE-8036</t>
         </is>
       </c>
       <c r="D123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8161</t>
+          <t>VLINE-8157</t>
         </is>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8422</t>
+          <t>VLINE-8418</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8730</t>
+          <t>VLINE-8725</t>
         </is>
       </c>
       <c r="G123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8796</t>
+          <t>VLINE-8792</t>
         </is>
       </c>
       <c r="H123" s="1" t="inlineStr">
         <is>
-          <t>XRN001</t>
+          <t>XP2016</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>QR1771</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>TE2801</t>
         </is>
       </c>
       <c r="C124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8053</t>
+          <t>VLINE-8038</t>
         </is>
       </c>
       <c r="D124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8162</t>
+          <t>VLINE-8158</t>
         </is>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8424</t>
+          <t>VLINE-8419</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8731</t>
+          <t>VLINE-8726</t>
         </is>
       </c>
       <c r="G124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8797</t>
+          <t>VLINE-8793</t>
         </is>
       </c>
       <c r="H124" s="1" t="inlineStr">
         <is>
-          <t>XRN004</t>
+          <t>XP2017</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>RCTST4</t>
+          <t>QR5404</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
         <is>
-          <t>TE2806</t>
+          <t>TE2802</t>
         </is>
       </c>
       <c r="C125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8055</t>
+          <t>VLINE-8042</t>
         </is>
       </c>
       <c r="D125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8171</t>
+          <t>VLINE-8159</t>
         </is>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8425</t>
+          <t>VLINE-8420</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8733</t>
+          <t>VLINE-8727</t>
         </is>
       </c>
       <c r="G125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8799</t>
+          <t>VLINE-8794</t>
         </is>
       </c>
       <c r="H125" s="1" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>XP2019</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>R711</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>TE2803</t>
         </is>
       </c>
       <c r="C126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8056</t>
+          <t>VLINE-8051</t>
         </is>
       </c>
       <c r="D126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8172</t>
+          <t>VLINE-8160</t>
         </is>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8426</t>
+          <t>VLINE-8421</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8735</t>
+          <t>VLINE-8729</t>
         </is>
       </c>
       <c r="G126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8800</t>
+          <t>VLINE-8795</t>
         </is>
       </c>
       <c r="H126" s="1" t="inlineStr">
         <is>
-          <t>XRN006</t>
+          <t>XR552</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>RL302</t>
+          <t>R766</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>TE2804</t>
         </is>
       </c>
       <c r="C127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8057</t>
+          <t>VLINE-8052</t>
         </is>
       </c>
       <c r="D127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8176</t>
+          <t>VLINE-8161</t>
         </is>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8427</t>
+          <t>VLINE-8422</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8736</t>
+          <t>VLINE-8730</t>
         </is>
       </c>
       <c r="G127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8801</t>
+          <t>VLINE-8796</t>
         </is>
       </c>
       <c r="H127" s="1" t="inlineStr">
         <is>
-          <t>XRN007</t>
+          <t>XRN001</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>RL304</t>
+          <t>RB2353</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
         <is>
-          <t>TE2809</t>
+          <t>TE2805</t>
         </is>
       </c>
       <c r="C128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8058</t>
+          <t>VLINE-8053</t>
         </is>
       </c>
       <c r="D128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8179</t>
+          <t>VLINE-8162</t>
         </is>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8428</t>
+          <t>VLINE-8424</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8737</t>
+          <t>VLINE-8731</t>
         </is>
       </c>
       <c r="G128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8802</t>
+          <t>VLINE-8797</t>
         </is>
       </c>
       <c r="H128" s="1" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>XRN004</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>RL305</t>
+          <t>RCTST4</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
         <is>
-          <t>TE2810</t>
+          <t>TE2806</t>
         </is>
       </c>
       <c r="C129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8059</t>
+          <t>VLINE-8055</t>
         </is>
       </c>
       <c r="D129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8180</t>
+          <t>VLINE-8171</t>
         </is>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8429</t>
+          <t>VLINE-8425</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8739</t>
+          <t>VLINE-8733</t>
         </is>
       </c>
       <c r="G129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8803</t>
+          <t>VLINE-8799</t>
         </is>
       </c>
       <c r="H129" s="1" t="inlineStr">
         <is>
-          <t>XRN011</t>
+          <t>XRN005</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>RL307</t>
+          <t>RL301</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
         <is>
-          <t>TE2812</t>
+          <t>TE2807</t>
         </is>
       </c>
       <c r="C130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8061</t>
+          <t>VLINE-8056</t>
         </is>
       </c>
       <c r="D130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8181</t>
+          <t>VLINE-8172</t>
         </is>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8430</t>
+          <t>VLINE-8426</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8740</t>
+          <t>VLINE-8735</t>
         </is>
       </c>
       <c r="G130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8804</t>
+          <t>VLINE-8800</t>
         </is>
       </c>
       <c r="H130" s="1" t="inlineStr">
         <is>
-          <t>XRN014</t>
+          <t>XRN006</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>RL309</t>
+          <t>RL302</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>TE2808</t>
         </is>
       </c>
       <c r="C131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8072</t>
+          <t>VLINE-8057</t>
         </is>
       </c>
       <c r="D131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8182</t>
+          <t>VLINE-8176</t>
         </is>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8431</t>
+          <t>VLINE-8427</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8741</t>
+          <t>VLINE-8736</t>
         </is>
       </c>
       <c r="G131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8805</t>
+          <t>VLINE-8801</t>
         </is>
       </c>
       <c r="H131" s="1" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>XRN007</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>RL310</t>
+          <t>RL304</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>TE2809</t>
         </is>
       </c>
       <c r="C132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8074</t>
+          <t>VLINE-8058</t>
         </is>
       </c>
       <c r="D132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8183</t>
+          <t>VLINE-8179</t>
         </is>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8432</t>
+          <t>VLINE-8428</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8742</t>
+          <t>VLINE-8737</t>
         </is>
       </c>
       <c r="G132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8806</t>
+          <t>VLINE-8802</t>
         </is>
       </c>
       <c r="H132" s="1" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>XRN009</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>S312</t>
+          <t>RL305</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>TE2810</t>
         </is>
       </c>
       <c r="C133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8075</t>
+          <t>VLINE-8059</t>
         </is>
       </c>
       <c r="D133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8184</t>
+          <t>VLINE-8180</t>
         </is>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8433</t>
+          <t>VLINE-8429</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8743</t>
+          <t>VLINE-8739</t>
         </is>
       </c>
       <c r="G133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8807</t>
+          <t>VLINE-8803</t>
         </is>
       </c>
       <c r="H133" s="1" t="inlineStr">
         <is>
-          <t>XRN020</t>
+          <t>XRN011</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>S317</t>
+          <t>RL307</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
         <is>
-          <t>TJ107</t>
+          <t>TE2812</t>
         </is>
       </c>
       <c r="C134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8076</t>
+          <t>VLINE-8061</t>
         </is>
       </c>
       <c r="D134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8185</t>
+          <t>VLINE-8181</t>
         </is>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8434</t>
+          <t>VLINE-8430</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8744</t>
+          <t>VLINE-8740</t>
         </is>
       </c>
       <c r="G134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8808</t>
+          <t>VLINE-8804</t>
         </is>
       </c>
       <c r="H134" s="1" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>XRN014</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>S3301</t>
+          <t>RL309</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TE2813</t>
         </is>
       </c>
       <c r="C135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8077</t>
+          <t>VLINE-8072</t>
         </is>
       </c>
       <c r="D135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8186</t>
+          <t>VLINE-8182</t>
         </is>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8435</t>
+          <t>VLINE-8431</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8745</t>
+          <t>VLINE-8741</t>
         </is>
       </c>
       <c r="G135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8809</t>
+          <t>VLINE-8805</t>
         </is>
       </c>
       <c r="H135" s="1" t="inlineStr">
         <is>
-          <t>XRN023</t>
+          <t>XRN017</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>S3302</t>
+          <t>RL310</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TE2814</t>
         </is>
       </c>
       <c r="C136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8080</t>
+          <t>VLINE-8074</t>
         </is>
       </c>
       <c r="D136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8187</t>
+          <t>VLINE-8183</t>
         </is>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8438</t>
+          <t>VLINE-8432</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8746</t>
+          <t>VLINE-8742</t>
         </is>
       </c>
       <c r="G136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8810</t>
+          <t>VLINE-8806</t>
         </is>
       </c>
       <c r="H136" s="1" t="inlineStr">
         <is>
-          <t>XRN025</t>
+          <t>XRN018</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>S3304</t>
+          <t>S312</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TJ096</t>
         </is>
       </c>
       <c r="C137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8081</t>
+          <t>VLINE-8075</t>
         </is>
       </c>
       <c r="D137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8188</t>
+          <t>VLINE-8184</t>
         </is>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8440</t>
+          <t>VLINE-8433</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8747</t>
+          <t>VLINE-8743</t>
         </is>
       </c>
       <c r="G137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8811</t>
+          <t>VLINE-8807</t>
         </is>
       </c>
       <c r="H137" s="1" t="inlineStr">
         <is>
-          <t>XRN026</t>
+          <t>XRN020</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>S3305</t>
+          <t>S317</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
         <is>
-          <t>TT07</t>
+          <t>TJ107</t>
         </is>
       </c>
       <c r="C138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8084</t>
+          <t>VLINE-8076</t>
         </is>
       </c>
       <c r="D138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8189</t>
+          <t>VLINE-8185</t>
         </is>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8441</t>
+          <t>VLINE-8434</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8748</t>
+          <t>VLINE-8744</t>
         </is>
       </c>
       <c r="G138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8812</t>
+          <t>VLINE-8808</t>
         </is>
       </c>
       <c r="H138" s="1" t="inlineStr">
         <is>
-          <t>XRN027</t>
+          <t>XRN021</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>S3306</t>
+          <t>S3301</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TT03</t>
         </is>
       </c>
       <c r="C139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8088</t>
+          <t>VLINE-8077</t>
         </is>
       </c>
       <c r="D139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8291</t>
+          <t>VLINE-8186</t>
         </is>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8442</t>
+          <t>VLINE-8435</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8749</t>
+          <t>VLINE-8745</t>
         </is>
       </c>
       <c r="G139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8813</t>
+          <t>VLINE-8809</t>
         </is>
       </c>
       <c r="H139" s="1" t="inlineStr">
         <is>
-          <t>Y163</t>
+          <t>XRN023</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>S3307</t>
+          <t>S3302</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TT04</t>
         </is>
       </c>
       <c r="C140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8089</t>
+          <t>VLINE-8080</t>
         </is>
       </c>
       <c r="D140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8293</t>
+          <t>VLINE-8187</t>
         </is>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8443</t>
+          <t>VLINE-8438</t>
         </is>
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8750</t>
+          <t>VLINE-8746</t>
         </is>
       </c>
       <c r="G140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8814</t>
+          <t>VLINE-8810</t>
+        </is>
+      </c>
+      <c r="H140" s="1" t="inlineStr">
+        <is>
+          <t>XRN025</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>S3309</t>
+          <t>S3304</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
         <is>
-          <t>TT106</t>
+          <t>TT05</t>
         </is>
       </c>
       <c r="C141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8104</t>
+          <t>VLINE-8081</t>
         </is>
       </c>
       <c r="D141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8303</t>
+          <t>VLINE-8188</t>
         </is>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8444</t>
+          <t>VLINE-8440</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8751</t>
+          <t>VLINE-8747</t>
         </is>
       </c>
       <c r="G141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8816</t>
+          <t>VLINE-8811</t>
+        </is>
+      </c>
+      <c r="H141" s="1" t="inlineStr">
+        <is>
+          <t>XRN026</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>S3310</t>
+          <t>S3305</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TT07</t>
         </is>
       </c>
       <c r="C142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8107</t>
+          <t>VLINE-8084</t>
         </is>
       </c>
       <c r="D142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8304</t>
+          <t>VLINE-8189</t>
         </is>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8446</t>
+          <t>VLINE-8441</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8752</t>
+          <t>VLINE-8748</t>
         </is>
       </c>
       <c r="G142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8817</t>
+          <t>VLINE-8812</t>
+        </is>
+      </c>
+      <c r="H142" s="1" t="inlineStr">
+        <is>
+          <t>XRN027</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>S7001</t>
+          <t>S3306</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
         <is>
-          <t>TT108</t>
+          <t>TT08</t>
         </is>
       </c>
       <c r="C143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8110</t>
+          <t>VLINE-8088</t>
         </is>
       </c>
       <c r="D143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8306</t>
+          <t>VLINE-8291</t>
         </is>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8447</t>
+          <t>VLINE-8442</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8753</t>
+          <t>VLINE-8749</t>
         </is>
       </c>
       <c r="G143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8818</t>
+          <t>VLINE-8813</t>
+        </is>
+      </c>
+      <c r="H143" s="1" t="inlineStr">
+        <is>
+          <t>Y163</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>S7002</t>
+          <t>S3307</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TT103</t>
         </is>
       </c>
       <c r="C144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8111</t>
+          <t>VLINE-8089</t>
         </is>
       </c>
       <c r="D144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8311</t>
+          <t>VLINE-8293</t>
         </is>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8449</t>
+          <t>VLINE-8443</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8754</t>
+          <t>VLINE-8750</t>
         </is>
       </c>
       <c r="G144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8819</t>
+          <t>VLINE-8814</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>S7003</t>
+          <t>S3309</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
         <is>
-          <t>TT113</t>
+          <t>TT106</t>
         </is>
       </c>
       <c r="C145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8113</t>
+          <t>VLINE-8104</t>
         </is>
       </c>
       <c r="D145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8313</t>
+          <t>VLINE-8303</t>
         </is>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8450</t>
+          <t>VLINE-8444</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8755</t>
+          <t>VLINE-8751</t>
         </is>
       </c>
       <c r="G145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8822</t>
+          <t>VLINE-8816</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>S7004</t>
+          <t>S3310</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
         <is>
-          <t>TT114</t>
+          <t>TT107</t>
         </is>
       </c>
       <c r="C146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8114</t>
+          <t>VLINE-8107</t>
         </is>
       </c>
       <c r="D146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8314</t>
+          <t>VLINE-8304</t>
         </is>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8451</t>
+          <t>VLINE-8446</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8756</t>
+          <t>VLINE-8752</t>
         </is>
       </c>
       <c r="G146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8860</t>
+          <t>VLINE-8817</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>S7005</t>
+          <t>S7001</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT108</t>
         </is>
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8115</t>
+          <t>VLINE-8110</t>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8316</t>
+          <t>VLINE-8306</t>
         </is>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8452</t>
+          <t>VLINE-8447</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8757</t>
+          <t>VLINE-8753</t>
         </is>
       </c>
       <c r="G147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8861</t>
+          <t>VLINE-8818</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>S7006</t>
+          <t>S7002</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
         <is>
-          <t>TT116</t>
+          <t>TT110</t>
         </is>
       </c>
       <c r="C148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8119</t>
+          <t>VLINE-8111</t>
         </is>
       </c>
       <c r="D148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8318</t>
+          <t>VLINE-8311</t>
         </is>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8453</t>
+          <t>VLINE-8449</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8758</t>
+          <t>VLINE-8754</t>
         </is>
       </c>
       <c r="G148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8862</t>
+          <t>VLINE-8819</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>S7007</t>
+          <t>S7003</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT113</t>
         </is>
       </c>
       <c r="C149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8120</t>
+          <t>VLINE-8113</t>
         </is>
       </c>
       <c r="D149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8321</t>
+          <t>VLINE-8313</t>
         </is>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8454</t>
+          <t>VLINE-8450</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8759</t>
+          <t>VLINE-8755</t>
         </is>
       </c>
       <c r="G149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8863</t>
+          <t>VLINE-8822</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>S7008</t>
+          <t>S7004</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
         <is>
-          <t>TT122</t>
+          <t>TT114</t>
         </is>
       </c>
       <c r="C150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8121</t>
+          <t>VLINE-8114</t>
         </is>
       </c>
       <c r="D150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8323</t>
+          <t>VLINE-8314</t>
         </is>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8455</t>
+          <t>VLINE-8451</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8760</t>
+          <t>VLINE-8756</t>
         </is>
       </c>
       <c r="G150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8864</t>
+          <t>VLINE-8860</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>S7012</t>
+          <t>S7005</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
         <is>
-          <t>TT127</t>
+          <t>TT115</t>
         </is>
       </c>
       <c r="C151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8123</t>
+          <t>VLINE-8115</t>
         </is>
       </c>
       <c r="D151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8324</t>
+          <t>VLINE-8316</t>
         </is>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8456</t>
+          <t>VLINE-8452</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8761</t>
+          <t>VLINE-8757</t>
         </is>
       </c>
       <c r="G151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8865</t>
+          <t>VLINE-8861</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>S7013</t>
+          <t>S7006</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
         <is>
-          <t>TT128</t>
+          <t>TT116</t>
         </is>
       </c>
       <c r="C152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8124</t>
+          <t>VLINE-8119</t>
         </is>
       </c>
       <c r="D152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8325</t>
+          <t>VLINE-8318</t>
         </is>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8457</t>
+          <t>VLINE-8453</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8762</t>
+          <t>VLINE-8758</t>
         </is>
       </c>
       <c r="G152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8866</t>
+          <t>VLINE-8862</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>S7014</t>
+          <t>S7007</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT117</t>
         </is>
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8126</t>
+          <t>VLINE-8120</t>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8328</t>
+          <t>VLINE-8321</t>
         </is>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8460</t>
+          <t>VLINE-8454</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8763</t>
+          <t>VLINE-8759</t>
         </is>
       </c>
       <c r="G153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8867</t>
+          <t>VLINE-8863</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>S7015</t>
+          <t>S7008</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
         <is>
-          <t>TT131</t>
+          <t>TT122</t>
         </is>
       </c>
       <c r="C154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8127</t>
+          <t>VLINE-8121</t>
         </is>
       </c>
       <c r="D154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8329</t>
+          <t>VLINE-8323</t>
         </is>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8461</t>
+          <t>VLINE-8455</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8765</t>
+          <t>VLINE-8760</t>
         </is>
       </c>
       <c r="G154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8868</t>
+          <t>VLINE-8864</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>S7017</t>
+          <t>S7012</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT127</t>
         </is>
       </c>
       <c r="C155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8128</t>
+          <t>VLINE-8123</t>
         </is>
       </c>
       <c r="D155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8332</t>
+          <t>VLINE-8324</t>
         </is>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8464</t>
+          <t>VLINE-8456</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8766</t>
+          <t>VLINE-8761</t>
         </is>
       </c>
       <c r="G155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8869</t>
+          <t>VLINE-8865</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>S7018</t>
+          <t>S7013</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT128</t>
         </is>
       </c>
       <c r="C156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8129</t>
+          <t>VLINE-8124</t>
         </is>
       </c>
       <c r="D156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8336</t>
+          <t>VLINE-8325</t>
         </is>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8465</t>
+          <t>VLINE-8457</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8767</t>
+          <t>VLINE-8762</t>
         </is>
       </c>
       <c r="G156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8890</t>
+          <t>VLINE-8866</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>S7020</t>
+          <t>S7014</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
         <is>
-          <t>VL352</t>
+          <t>TT130</t>
         </is>
       </c>
       <c r="C157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8131</t>
+          <t>VLINE-8126</t>
         </is>
       </c>
       <c r="D157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8337</t>
+          <t>VLINE-8328</t>
         </is>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8468</t>
+          <t>VLINE-8460</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8768</t>
+          <t>VLINE-8763</t>
         </is>
       </c>
       <c r="G157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8891</t>
+          <t>VLINE-8867</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>S7022</t>
+          <t>S7015</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
         <is>
-          <t>VL353</t>
+          <t>TT131</t>
         </is>
       </c>
       <c r="C158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8132</t>
+          <t>VLINE-8127</t>
         </is>
       </c>
       <c r="D158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8338</t>
+          <t>VLINE-8329</t>
         </is>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8469</t>
+          <t>VLINE-8461</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8769</t>
+          <t>VLINE-8765</t>
         </is>
       </c>
       <c r="G158" s="1" t="inlineStr">
         <is>
-          <t>WH001</t>
+          <t>VLINE-8868</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>S7017</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
         <is>
-          <t>VL357</t>
+          <t>TT202</t>
         </is>
       </c>
       <c r="C159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8133</t>
+          <t>VLINE-8128</t>
         </is>
       </c>
       <c r="D159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8339</t>
+          <t>VLINE-8332</t>
         </is>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8605</t>
+          <t>VLINE-8464</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8770</t>
+          <t>VLINE-8766</t>
         </is>
       </c>
       <c r="G159" s="1" t="inlineStr">
         <is>
-          <t>WH003</t>
+          <t>VLINE-8869</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>SCT002</t>
+          <t>S7018</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8004</t>
+          <t>TT206</t>
         </is>
       </c>
       <c r="C160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8134</t>
+          <t>VLINE-8129</t>
         </is>
       </c>
       <c r="D160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8362</t>
+          <t>VLINE-8336</t>
         </is>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8610</t>
+          <t>VLINE-8465</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8772</t>
+          <t>VLINE-8767</t>
         </is>
       </c>
       <c r="G160" s="1" t="inlineStr">
         <is>
-          <t>WL02</t>
+          <t>VLINE-8890</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>SCT006</t>
+          <t>S7020</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8007</t>
+          <t>VL352</t>
         </is>
       </c>
       <c r="C161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8136</t>
+          <t>VLINE-8131</t>
         </is>
       </c>
       <c r="D161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8363</t>
+          <t>VLINE-8337</t>
         </is>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8612</t>
+          <t>VLINE-8468</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8773</t>
+          <t>VLINE-8768</t>
         </is>
       </c>
       <c r="G161" s="1" t="inlineStr">
         <is>
-          <t>X12-X14</t>
+          <t>VLINE-8891</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>SCT007</t>
+          <t>S7022</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8011</t>
+          <t>VL353</t>
         </is>
       </c>
       <c r="C162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8137</t>
+          <t>VLINE-8132</t>
         </is>
       </c>
       <c r="D162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8365</t>
+          <t>VLINE-8338</t>
         </is>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8615</t>
+          <t>VLINE-8469</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8774</t>
+          <t>VLINE-8769</t>
         </is>
       </c>
       <c r="G162" s="1" t="inlineStr">
         <is>
-          <t>X31</t>
+          <t>WH001</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>SCT001</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8013</t>
+          <t>VL357</t>
         </is>
       </c>
       <c r="C163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8140</t>
+          <t>VLINE-8133</t>
         </is>
       </c>
       <c r="D163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8366</t>
+          <t>VLINE-8339</t>
         </is>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8617</t>
+          <t>VLINE-8605</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8776</t>
+          <t>VLINE-8770</t>
         </is>
       </c>
       <c r="G163" s="1" t="inlineStr">
         <is>
-          <t>XP2000</t>
+          <t>WH003</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>SCT011</t>
+          <t>SCT002</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8019</t>
+          <t>VLINE-8004</t>
         </is>
       </c>
       <c r="C164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8141</t>
+          <t>VLINE-8134</t>
         </is>
       </c>
       <c r="D164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8368</t>
+          <t>VLINE-8362</t>
         </is>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8620</t>
+          <t>VLINE-8610</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8778</t>
+          <t>VLINE-8772</t>
         </is>
       </c>
       <c r="G164" s="1" t="inlineStr">
         <is>
-          <t>XP2003</t>
+          <t>WL02</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>SCT006</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8020</t>
+          <t>VLINE-8007</t>
         </is>
       </c>
       <c r="C165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8142</t>
+          <t>VLINE-8136</t>
         </is>
       </c>
       <c r="D165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8369</t>
+          <t>VLINE-8363</t>
         </is>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8625</t>
+          <t>VLINE-8612</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8779</t>
+          <t>VLINE-8773</t>
         </is>
       </c>
       <c r="G165" s="1" t="inlineStr">
         <is>
-          <t>XP2004</t>
+          <t>X12-X14</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>SCT014</t>
+          <t>SCT007</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8023</t>
+          <t>VLINE-8011</t>
         </is>
       </c>
       <c r="C166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8144</t>
+          <t>VLINE-8137</t>
         </is>
       </c>
       <c r="D166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8403</t>
+          <t>VLINE-8365</t>
         </is>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8630</t>
+          <t>VLINE-8615</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8780</t>
+          <t>VLINE-8774</t>
         </is>
       </c>
       <c r="G166" s="1" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>X31</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>SCT015</t>
+          <t>SCT009</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8025</t>
+          <t>VLINE-8013</t>
         </is>
       </c>
       <c r="C167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8145</t>
+          <t>VLINE-8140</t>
         </is>
       </c>
       <c r="D167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8404</t>
+          <t>VLINE-8366</t>
         </is>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8671</t>
+          <t>VLINE-8617</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8781</t>
+          <t>VLINE-8776</t>
         </is>
       </c>
       <c r="G167" s="1" t="inlineStr">
         <is>
-          <t>XP2007</t>
+          <t>XP2000</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>SO2</t>
+          <t>SCT011</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8026</t>
+          <t>VLINE-8019</t>
         </is>
       </c>
       <c r="C168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8148</t>
+          <t>VLINE-8141</t>
         </is>
       </c>
       <c r="D168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8406</t>
+          <t>VLINE-8368</t>
         </is>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8706</t>
+          <t>VLINE-8620</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8782</t>
+          <t>VLINE-8778</t>
         </is>
       </c>
       <c r="G168" s="1" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>XP2003</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>SCT013</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8027</t>
+          <t>VLINE-8020</t>
         </is>
       </c>
       <c r="C169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8150</t>
+          <t>VLINE-8142</t>
         </is>
       </c>
       <c r="D169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8408</t>
+          <t>VLINE-8369</t>
         </is>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8711</t>
+          <t>VLINE-8625</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8783</t>
+          <t>VLINE-8779</t>
         </is>
       </c>
       <c r="G169" s="1" t="inlineStr">
         <is>
-          <t>XP2010</t>
+          <t>XP2004</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>SCT014</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8028</t>
+          <t>VLINE-8023</t>
         </is>
       </c>
       <c r="C170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8151</t>
+          <t>VLINE-8144</t>
         </is>
       </c>
       <c r="D170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8410</t>
+          <t>VLINE-8403</t>
         </is>
       </c>
       <c r="E170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8714</t>
+          <t>VLINE-8630</t>
         </is>
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8784</t>
+          <t>VLINE-8780</t>
         </is>
       </c>
       <c r="G170" s="1" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>XP2005</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update trains and loco export 2026-04-06 12:42:07
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -5141,37 +5141,37 @@
       </c>
       <c r="B115" s="1" t="inlineStr">
         <is>
-          <t>P2513</t>
+          <t>P2511</t>
         </is>
       </c>
       <c r="C115" s="1" t="inlineStr">
         <is>
-          <t>RL307</t>
+          <t>RL306</t>
         </is>
       </c>
       <c r="D115" s="1" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>TE2807</t>
         </is>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8052</t>
+          <t>VLINE-8051</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8161</t>
+          <t>VLINE-8160</t>
         </is>
       </c>
       <c r="G115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8422</t>
+          <t>VLINE-8421</t>
         </is>
       </c>
       <c r="H115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8730</t>
+          <t>VLINE-8729</t>
         </is>
       </c>
     </row>
@@ -5183,37 +5183,37 @@
       </c>
       <c r="B116" s="1" t="inlineStr">
         <is>
-          <t>P2514</t>
+          <t>P2513</t>
         </is>
       </c>
       <c r="C116" s="1" t="inlineStr">
         <is>
-          <t>RL309</t>
+          <t>RL307</t>
         </is>
       </c>
       <c r="D116" s="1" t="inlineStr">
         <is>
-          <t>TE2809</t>
+          <t>TE2808</t>
         </is>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8053</t>
+          <t>VLINE-8052</t>
         </is>
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8162</t>
+          <t>VLINE-8161</t>
         </is>
       </c>
       <c r="G116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8424</t>
+          <t>VLINE-8422</t>
         </is>
       </c>
       <c r="H116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8731</t>
+          <t>VLINE-8730</t>
         </is>
       </c>
     </row>
@@ -5225,37 +5225,37 @@
       </c>
       <c r="B117" s="1" t="inlineStr">
         <is>
-          <t>P2515</t>
+          <t>P2514</t>
         </is>
       </c>
       <c r="C117" s="1" t="inlineStr">
         <is>
-          <t>RL310</t>
+          <t>RL309</t>
         </is>
       </c>
       <c r="D117" s="1" t="inlineStr">
         <is>
-          <t>TE2810</t>
+          <t>TE2809</t>
         </is>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8055</t>
+          <t>VLINE-8053</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8171</t>
+          <t>VLINE-8162</t>
         </is>
       </c>
       <c r="G117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8425</t>
+          <t>VLINE-8424</t>
         </is>
       </c>
       <c r="H117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8733</t>
+          <t>VLINE-8731</t>
         </is>
       </c>
     </row>
@@ -5267,37 +5267,37 @@
       </c>
       <c r="B118" s="1" t="inlineStr">
         <is>
-          <t>P2516</t>
+          <t>P2515</t>
         </is>
       </c>
       <c r="C118" s="1" t="inlineStr">
         <is>
-          <t>S312</t>
+          <t>RL310</t>
         </is>
       </c>
       <c r="D118" s="1" t="inlineStr">
         <is>
-          <t>TE2812</t>
+          <t>TE2810</t>
         </is>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8056</t>
+          <t>VLINE-8055</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8172</t>
+          <t>VLINE-8171</t>
         </is>
       </c>
       <c r="G118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8426</t>
+          <t>VLINE-8425</t>
         </is>
       </c>
       <c r="H118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8735</t>
+          <t>VLINE-8733</t>
         </is>
       </c>
     </row>
@@ -5309,37 +5309,37 @@
       </c>
       <c r="B119" s="1" t="inlineStr">
         <is>
-          <t>PB1</t>
+          <t>P2516</t>
         </is>
       </c>
       <c r="C119" s="1" t="inlineStr">
         <is>
-          <t>S317</t>
+          <t>S312</t>
         </is>
       </c>
       <c r="D119" s="1" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>TE2812</t>
         </is>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8057</t>
+          <t>VLINE-8056</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8176</t>
+          <t>VLINE-8172</t>
         </is>
       </c>
       <c r="G119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8427</t>
+          <t>VLINE-8426</t>
         </is>
       </c>
       <c r="H119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8736</t>
+          <t>VLINE-8735</t>
         </is>
       </c>
     </row>
@@ -5351,37 +5351,37 @@
       </c>
       <c r="B120" s="1" t="inlineStr">
         <is>
-          <t>PB2</t>
+          <t>PB1</t>
         </is>
       </c>
       <c r="C120" s="1" t="inlineStr">
         <is>
-          <t>S3301</t>
+          <t>S317</t>
         </is>
       </c>
       <c r="D120" s="1" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>TE2813</t>
         </is>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8058</t>
+          <t>VLINE-8057</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8179</t>
+          <t>VLINE-8176</t>
         </is>
       </c>
       <c r="G120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8428</t>
+          <t>VLINE-8427</t>
         </is>
       </c>
       <c r="H120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8737</t>
+          <t>VLINE-8736</t>
         </is>
       </c>
     </row>
@@ -5393,37 +5393,37 @@
       </c>
       <c r="B121" s="1" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>PB2</t>
         </is>
       </c>
       <c r="C121" s="1" t="inlineStr">
         <is>
-          <t>S3302</t>
+          <t>S3301</t>
         </is>
       </c>
       <c r="D121" s="1" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>TE2814</t>
         </is>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8059</t>
+          <t>VLINE-8058</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8180</t>
+          <t>VLINE-8179</t>
         </is>
       </c>
       <c r="G121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8429</t>
+          <t>VLINE-8428</t>
         </is>
       </c>
       <c r="H121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8739</t>
+          <t>VLINE-8737</t>
         </is>
       </c>
     </row>
@@ -5435,37 +5435,37 @@
       </c>
       <c r="B122" s="1" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>PB4</t>
         </is>
       </c>
       <c r="C122" s="1" t="inlineStr">
         <is>
-          <t>S3304</t>
+          <t>S3302</t>
         </is>
       </c>
       <c r="D122" s="1" t="inlineStr">
         <is>
-          <t>TJ107</t>
+          <t>TJ096</t>
         </is>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8061</t>
+          <t>VLINE-8059</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8181</t>
+          <t>VLINE-8180</t>
         </is>
       </c>
       <c r="G122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8430</t>
+          <t>VLINE-8429</t>
         </is>
       </c>
       <c r="H122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8740</t>
+          <t>VLINE-8739</t>
         </is>
       </c>
     </row>
@@ -5477,37 +5477,37 @@
       </c>
       <c r="B123" s="1" t="inlineStr">
         <is>
-          <t>PHC002</t>
+          <t>PHC001</t>
         </is>
       </c>
       <c r="C123" s="1" t="inlineStr">
         <is>
-          <t>S3305</t>
+          <t>S3304</t>
         </is>
       </c>
       <c r="D123" s="1" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TJ107</t>
         </is>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8072</t>
+          <t>VLINE-8061</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8182</t>
+          <t>VLINE-8181</t>
         </is>
       </c>
       <c r="G123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8431</t>
+          <t>VLINE-8430</t>
         </is>
       </c>
       <c r="H123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8741</t>
+          <t>VLINE-8740</t>
         </is>
       </c>
     </row>
@@ -5519,37 +5519,37 @@
       </c>
       <c r="B124" s="1" t="inlineStr">
         <is>
-          <t>Q4001</t>
+          <t>PHC002</t>
         </is>
       </c>
       <c r="C124" s="1" t="inlineStr">
         <is>
-          <t>S3306</t>
+          <t>S3305</t>
         </is>
       </c>
       <c r="D124" s="1" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TT03</t>
         </is>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8074</t>
+          <t>VLINE-8072</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8183</t>
+          <t>VLINE-8182</t>
         </is>
       </c>
       <c r="G124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8432</t>
+          <t>VLINE-8431</t>
         </is>
       </c>
       <c r="H124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8742</t>
+          <t>VLINE-8741</t>
         </is>
       </c>
     </row>
@@ -5561,37 +5561,37 @@
       </c>
       <c r="B125" s="1" t="inlineStr">
         <is>
-          <t>Q4003</t>
+          <t>Q4001</t>
         </is>
       </c>
       <c r="C125" s="1" t="inlineStr">
         <is>
-          <t>S3307</t>
+          <t>S3306</t>
         </is>
       </c>
       <c r="D125" s="1" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TT04</t>
         </is>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8075</t>
+          <t>VLINE-8074</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8184</t>
+          <t>VLINE-8183</t>
         </is>
       </c>
       <c r="G125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8433</t>
+          <t>VLINE-8432</t>
         </is>
       </c>
       <c r="H125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8743</t>
+          <t>VLINE-8742</t>
         </is>
       </c>
     </row>
@@ -5603,37 +5603,37 @@
       </c>
       <c r="B126" s="1" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>Q4003</t>
         </is>
       </c>
       <c r="C126" s="1" t="inlineStr">
         <is>
-          <t>S3309</t>
+          <t>S3307</t>
         </is>
       </c>
       <c r="D126" s="1" t="inlineStr">
         <is>
-          <t>TT07</t>
+          <t>TT05</t>
         </is>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8076</t>
+          <t>VLINE-8075</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8185</t>
+          <t>VLINE-8184</t>
         </is>
       </c>
       <c r="G126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8434</t>
+          <t>VLINE-8433</t>
         </is>
       </c>
       <c r="H126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8744</t>
+          <t>VLINE-8743</t>
         </is>
       </c>
     </row>
@@ -5645,37 +5645,37 @@
       </c>
       <c r="B127" s="1" t="inlineStr">
         <is>
-          <t>Q4005</t>
+          <t>Q4004</t>
         </is>
       </c>
       <c r="C127" s="1" t="inlineStr">
         <is>
-          <t>S3310</t>
+          <t>S3309</t>
         </is>
       </c>
       <c r="D127" s="1" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TT07</t>
         </is>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8077</t>
+          <t>VLINE-8076</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8186</t>
+          <t>VLINE-8185</t>
         </is>
       </c>
       <c r="G127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8435</t>
+          <t>VLINE-8434</t>
         </is>
       </c>
       <c r="H127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8745</t>
+          <t>VLINE-8744</t>
         </is>
       </c>
     </row>
@@ -5687,37 +5687,37 @@
       </c>
       <c r="B128" s="1" t="inlineStr">
         <is>
-          <t>Q4006</t>
+          <t>Q4005</t>
         </is>
       </c>
       <c r="C128" s="1" t="inlineStr">
         <is>
-          <t>S7001</t>
+          <t>S3310</t>
         </is>
       </c>
       <c r="D128" s="1" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TT08</t>
         </is>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8080</t>
+          <t>VLINE-8077</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8187</t>
+          <t>VLINE-8186</t>
         </is>
       </c>
       <c r="G128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8438</t>
+          <t>VLINE-8435</t>
         </is>
       </c>
       <c r="H128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8746</t>
+          <t>VLINE-8745</t>
         </is>
       </c>
     </row>
@@ -5729,37 +5729,37 @@
       </c>
       <c r="B129" s="1" t="inlineStr">
         <is>
-          <t>Q4007</t>
+          <t>Q4006</t>
         </is>
       </c>
       <c r="C129" s="1" t="inlineStr">
         <is>
-          <t>S7002</t>
+          <t>S7001</t>
         </is>
       </c>
       <c r="D129" s="1" t="inlineStr">
         <is>
-          <t>TT106</t>
+          <t>TT103</t>
         </is>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8081</t>
+          <t>VLINE-8080</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8188</t>
+          <t>VLINE-8187</t>
         </is>
       </c>
       <c r="G129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8440</t>
+          <t>VLINE-8438</t>
         </is>
       </c>
       <c r="H129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8747</t>
+          <t>VLINE-8746</t>
         </is>
       </c>
     </row>
@@ -5771,37 +5771,37 @@
       </c>
       <c r="B130" s="1" t="inlineStr">
         <is>
-          <t>Q4009</t>
+          <t>Q4007</t>
         </is>
       </c>
       <c r="C130" s="1" t="inlineStr">
         <is>
-          <t>S7003</t>
+          <t>S7002</t>
         </is>
       </c>
       <c r="D130" s="1" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TT106</t>
         </is>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8084</t>
+          <t>VLINE-8081</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8189</t>
+          <t>VLINE-8188</t>
         </is>
       </c>
       <c r="G130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8441</t>
+          <t>VLINE-8440</t>
         </is>
       </c>
       <c r="H130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8748</t>
+          <t>VLINE-8747</t>
         </is>
       </c>
     </row>
@@ -5813,37 +5813,37 @@
       </c>
       <c r="B131" s="1" t="inlineStr">
         <is>
-          <t>Q4011</t>
+          <t>Q4009</t>
         </is>
       </c>
       <c r="C131" s="1" t="inlineStr">
         <is>
-          <t>S7004</t>
+          <t>S7003</t>
         </is>
       </c>
       <c r="D131" s="1" t="inlineStr">
         <is>
-          <t>TT108</t>
+          <t>TT107</t>
         </is>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8088</t>
+          <t>VLINE-8084</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8291</t>
+          <t>VLINE-8189</t>
         </is>
       </c>
       <c r="G131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8442</t>
+          <t>VLINE-8441</t>
         </is>
       </c>
       <c r="H131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8749</t>
+          <t>VLINE-8748</t>
         </is>
       </c>
     </row>
@@ -5855,37 +5855,37 @@
       </c>
       <c r="B132" s="1" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>Q4011</t>
         </is>
       </c>
       <c r="C132" s="1" t="inlineStr">
         <is>
-          <t>S7005</t>
+          <t>S7004</t>
         </is>
       </c>
       <c r="D132" s="1" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TT108</t>
         </is>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8089</t>
+          <t>VLINE-8088</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8293</t>
+          <t>VLINE-8291</t>
         </is>
       </c>
       <c r="G132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8443</t>
+          <t>VLINE-8442</t>
         </is>
       </c>
       <c r="H132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8750</t>
+          <t>VLINE-8749</t>
         </is>
       </c>
     </row>
@@ -5897,37 +5897,37 @@
       </c>
       <c r="B133" s="1" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>Q4012</t>
         </is>
       </c>
       <c r="C133" s="1" t="inlineStr">
         <is>
-          <t>S7006</t>
+          <t>S7005</t>
         </is>
       </c>
       <c r="D133" s="1" t="inlineStr">
         <is>
-          <t>TT113</t>
+          <t>TT110</t>
         </is>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8104</t>
+          <t>VLINE-8089</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8303</t>
+          <t>VLINE-8293</t>
         </is>
       </c>
       <c r="G133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8444</t>
+          <t>VLINE-8443</t>
         </is>
       </c>
       <c r="H133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8751</t>
+          <t>VLINE-8750</t>
         </is>
       </c>
     </row>
@@ -5939,37 +5939,37 @@
       </c>
       <c r="B134" s="1" t="inlineStr">
         <is>
-          <t>Q4014</t>
+          <t>Q4013</t>
         </is>
       </c>
       <c r="C134" s="1" t="inlineStr">
         <is>
-          <t>S7007</t>
+          <t>S7006</t>
         </is>
       </c>
       <c r="D134" s="1" t="inlineStr">
         <is>
-          <t>TT114</t>
+          <t>TT113</t>
         </is>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8107</t>
+          <t>VLINE-8104</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8304</t>
+          <t>VLINE-8303</t>
         </is>
       </c>
       <c r="G134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8446</t>
+          <t>VLINE-8444</t>
         </is>
       </c>
       <c r="H134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8752</t>
+          <t>VLINE-8751</t>
         </is>
       </c>
     </row>
@@ -5981,37 +5981,37 @@
       </c>
       <c r="B135" s="1" t="inlineStr">
         <is>
-          <t>Q4015</t>
+          <t>Q4014</t>
         </is>
       </c>
       <c r="C135" s="1" t="inlineStr">
         <is>
-          <t>S7008</t>
+          <t>S7007</t>
         </is>
       </c>
       <c r="D135" s="1" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT114</t>
         </is>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8110</t>
+          <t>VLINE-8107</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8306</t>
+          <t>VLINE-8304</t>
         </is>
       </c>
       <c r="G135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8447</t>
+          <t>VLINE-8446</t>
         </is>
       </c>
       <c r="H135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8753</t>
+          <t>VLINE-8752</t>
         </is>
       </c>
     </row>
@@ -6023,37 +6023,37 @@
       </c>
       <c r="B136" s="1" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>Q4015</t>
         </is>
       </c>
       <c r="C136" s="1" t="inlineStr">
         <is>
-          <t>S7009</t>
+          <t>S7008</t>
         </is>
       </c>
       <c r="D136" s="1" t="inlineStr">
         <is>
-          <t>TT116</t>
+          <t>TT115</t>
         </is>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8111</t>
+          <t>VLINE-8110</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8311</t>
+          <t>VLINE-8306</t>
         </is>
       </c>
       <c r="G136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8449</t>
+          <t>VLINE-8447</t>
         </is>
       </c>
       <c r="H136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8754</t>
+          <t>VLINE-8753</t>
         </is>
       </c>
     </row>
@@ -6065,37 +6065,37 @@
       </c>
       <c r="B137" s="1" t="inlineStr">
         <is>
-          <t>Q4017</t>
+          <t>Q4016</t>
         </is>
       </c>
       <c r="C137" s="1" t="inlineStr">
         <is>
-          <t>S7012</t>
+          <t>S7009</t>
         </is>
       </c>
       <c r="D137" s="1" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT116</t>
         </is>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8113</t>
+          <t>VLINE-8111</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8313</t>
+          <t>VLINE-8311</t>
         </is>
       </c>
       <c r="G137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8450</t>
+          <t>VLINE-8449</t>
         </is>
       </c>
       <c r="H137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8755</t>
+          <t>VLINE-8754</t>
         </is>
       </c>
     </row>
@@ -6107,37 +6107,37 @@
       </c>
       <c r="B138" s="1" t="inlineStr">
         <is>
-          <t>Q4019</t>
+          <t>Q4017</t>
         </is>
       </c>
       <c r="C138" s="1" t="inlineStr">
         <is>
-          <t>S7013</t>
+          <t>S7012</t>
         </is>
       </c>
       <c r="D138" s="1" t="inlineStr">
         <is>
-          <t>TT122</t>
+          <t>TT117</t>
         </is>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8114</t>
+          <t>VLINE-8113</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8314</t>
+          <t>VLINE-8313</t>
         </is>
       </c>
       <c r="G138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8451</t>
+          <t>VLINE-8450</t>
         </is>
       </c>
       <c r="H138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8756</t>
+          <t>VLINE-8755</t>
         </is>
       </c>
     </row>
@@ -6149,37 +6149,37 @@
       </c>
       <c r="B139" s="1" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>Q4019</t>
         </is>
       </c>
       <c r="C139" s="1" t="inlineStr">
         <is>
-          <t>S7014</t>
+          <t>S7013</t>
         </is>
       </c>
       <c r="D139" s="1" t="inlineStr">
         <is>
-          <t>TT127</t>
+          <t>TT122</t>
         </is>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8115</t>
+          <t>VLINE-8114</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8316</t>
+          <t>VLINE-8314</t>
         </is>
       </c>
       <c r="G139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8452</t>
+          <t>VLINE-8451</t>
         </is>
       </c>
       <c r="H139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8757</t>
+          <t>VLINE-8756</t>
         </is>
       </c>
     </row>
@@ -6191,37 +6191,37 @@
       </c>
       <c r="B140" s="1" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>QBX003</t>
         </is>
       </c>
       <c r="C140" s="1" t="inlineStr">
         <is>
-          <t>S7015</t>
+          <t>S7014</t>
         </is>
       </c>
       <c r="D140" s="1" t="inlineStr">
         <is>
-          <t>TT128</t>
+          <t>TT127</t>
         </is>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8119</t>
+          <t>VLINE-8115</t>
         </is>
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8318</t>
+          <t>VLINE-8316</t>
         </is>
       </c>
       <c r="G140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8453</t>
+          <t>VLINE-8452</t>
         </is>
       </c>
       <c r="H140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8758</t>
+          <t>VLINE-8757</t>
         </is>
       </c>
     </row>
@@ -6233,37 +6233,37 @@
       </c>
       <c r="B141" s="1" t="inlineStr">
         <is>
-          <t>QBX005</t>
+          <t>QBX004</t>
         </is>
       </c>
       <c r="C141" s="1" t="inlineStr">
         <is>
-          <t>S7017</t>
+          <t>S7015</t>
         </is>
       </c>
       <c r="D141" s="1" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT128</t>
         </is>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8120</t>
+          <t>VLINE-8119</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8321</t>
+          <t>VLINE-8318</t>
         </is>
       </c>
       <c r="G141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8454</t>
+          <t>VLINE-8453</t>
         </is>
       </c>
       <c r="H141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8759</t>
+          <t>VLINE-8758</t>
         </is>
       </c>
     </row>
@@ -6275,37 +6275,37 @@
       </c>
       <c r="B142" s="1" t="inlineStr">
         <is>
-          <t>QBX006</t>
+          <t>QBX005</t>
         </is>
       </c>
       <c r="C142" s="1" t="inlineStr">
         <is>
-          <t>S7018</t>
+          <t>S7017</t>
         </is>
       </c>
       <c r="D142" s="1" t="inlineStr">
         <is>
-          <t>TT131</t>
+          <t>TT130</t>
         </is>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8121</t>
+          <t>VLINE-8120</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8323</t>
+          <t>VLINE-8321</t>
         </is>
       </c>
       <c r="G142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8455</t>
+          <t>VLINE-8454</t>
         </is>
       </c>
       <c r="H142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8760</t>
+          <t>VLINE-8759</t>
         </is>
       </c>
     </row>
@@ -6317,37 +6317,37 @@
       </c>
       <c r="B143" s="1" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>QBX006</t>
         </is>
       </c>
       <c r="C143" s="1" t="inlineStr">
         <is>
-          <t>S7020</t>
+          <t>S7018</t>
         </is>
       </c>
       <c r="D143" s="1" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT131</t>
         </is>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8123</t>
+          <t>VLINE-8121</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8324</t>
+          <t>VLINE-8323</t>
         </is>
       </c>
       <c r="G143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8456</t>
+          <t>VLINE-8455</t>
         </is>
       </c>
       <c r="H143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8761</t>
+          <t>VLINE-8760</t>
         </is>
       </c>
     </row>
@@ -6359,37 +6359,37 @@
       </c>
       <c r="B144" s="1" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>QE001</t>
         </is>
       </c>
       <c r="C144" s="1" t="inlineStr">
         <is>
-          <t>S7022</t>
+          <t>S7020</t>
         </is>
       </c>
       <c r="D144" s="1" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT202</t>
         </is>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8124</t>
+          <t>VLINE-8123</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8325</t>
+          <t>VLINE-8324</t>
         </is>
       </c>
       <c r="G144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8457</t>
+          <t>VLINE-8456</t>
         </is>
       </c>
       <c r="H144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8762</t>
+          <t>VLINE-8761</t>
         </is>
       </c>
     </row>
@@ -6401,37 +6401,37 @@
       </c>
       <c r="B145" s="1" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>QE002</t>
         </is>
       </c>
       <c r="C145" s="1" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>S7022</t>
         </is>
       </c>
       <c r="D145" s="1" t="inlineStr">
         <is>
-          <t>VL352</t>
+          <t>TT206</t>
         </is>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8126</t>
+          <t>VLINE-8124</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8328</t>
+          <t>VLINE-8325</t>
         </is>
       </c>
       <c r="G145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8460</t>
+          <t>VLINE-8457</t>
         </is>
       </c>
       <c r="H145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8763</t>
+          <t>VLINE-8762</t>
         </is>
       </c>
     </row>
@@ -6443,37 +6443,37 @@
       </c>
       <c r="B146" s="1" t="inlineStr">
         <is>
-          <t>QE004</t>
+          <t>QE003</t>
         </is>
       </c>
       <c r="C146" s="1" t="inlineStr">
         <is>
-          <t>SCT002</t>
+          <t>SCT001</t>
         </is>
       </c>
       <c r="D146" s="1" t="inlineStr">
         <is>
-          <t>VL353</t>
+          <t>VL352</t>
         </is>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8127</t>
+          <t>VLINE-8126</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8329</t>
+          <t>VLINE-8328</t>
         </is>
       </c>
       <c r="G146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8461</t>
+          <t>VLINE-8460</t>
         </is>
       </c>
       <c r="H146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8764</t>
+          <t>VLINE-8763</t>
         </is>
       </c>
     </row>
@@ -6485,37 +6485,37 @@
       </c>
       <c r="B147" s="1" t="inlineStr">
         <is>
-          <t>QE006</t>
+          <t>QE004</t>
         </is>
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t>SCT006</t>
+          <t>SCT002</t>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
         <is>
-          <t>VL357</t>
+          <t>VL353</t>
         </is>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8128</t>
+          <t>VLINE-8127</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8332</t>
+          <t>VLINE-8329</t>
         </is>
       </c>
       <c r="G147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8464</t>
+          <t>VLINE-8461</t>
         </is>
       </c>
       <c r="H147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8765</t>
+          <t>VLINE-8764</t>
         </is>
       </c>
     </row>
@@ -6527,37 +6527,37 @@
       </c>
       <c r="B148" s="1" t="inlineStr">
         <is>
-          <t>QL001</t>
+          <t>QE006</t>
         </is>
       </c>
       <c r="C148" s="1" t="inlineStr">
         <is>
-          <t>SCT007</t>
+          <t>SCT006</t>
         </is>
       </c>
       <c r="D148" s="1" t="inlineStr">
         <is>
-          <t>VL359</t>
+          <t>VL357</t>
         </is>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8129</t>
+          <t>VLINE-8128</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8336</t>
+          <t>VLINE-8332</t>
         </is>
       </c>
       <c r="G148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8465</t>
+          <t>VLINE-8464</t>
         </is>
       </c>
       <c r="H148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8766</t>
+          <t>VLINE-8765</t>
         </is>
       </c>
     </row>
@@ -6569,37 +6569,37 @@
       </c>
       <c r="B149" s="1" t="inlineStr">
         <is>
-          <t>QL002</t>
+          <t>QL001</t>
         </is>
       </c>
       <c r="C149" s="1" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>SCT007</t>
         </is>
       </c>
       <c r="D149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8004</t>
+          <t>VL359</t>
         </is>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8131</t>
+          <t>VLINE-8129</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8337</t>
+          <t>VLINE-8336</t>
         </is>
       </c>
       <c r="G149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8468</t>
+          <t>VLINE-8465</t>
         </is>
       </c>
       <c r="H149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8767</t>
+          <t>VLINE-8766</t>
         </is>
       </c>
     </row>
@@ -6611,37 +6611,37 @@
       </c>
       <c r="B150" s="1" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>QL002</t>
         </is>
       </c>
       <c r="C150" s="1" t="inlineStr">
         <is>
-          <t>SCT011</t>
+          <t>SCT009</t>
         </is>
       </c>
       <c r="D150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8007</t>
+          <t>VLINE-8004</t>
         </is>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8132</t>
+          <t>VLINE-8131</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8338</t>
+          <t>VLINE-8337</t>
         </is>
       </c>
       <c r="G150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8469</t>
+          <t>VLINE-8468</t>
         </is>
       </c>
       <c r="H150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8768</t>
+          <t>VLINE-8767</t>
         </is>
       </c>
     </row>
@@ -6653,37 +6653,37 @@
       </c>
       <c r="B151" s="1" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>QL004</t>
         </is>
       </c>
       <c r="C151" s="1" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>SCT011</t>
         </is>
       </c>
       <c r="D151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8011</t>
+          <t>VLINE-8007</t>
         </is>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8133</t>
+          <t>VLINE-8132</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8339</t>
+          <t>VLINE-8338</t>
         </is>
       </c>
       <c r="G151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8605</t>
+          <t>VLINE-8469</t>
         </is>
       </c>
       <c r="H151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8769</t>
+          <t>VLINE-8768</t>
         </is>
       </c>
     </row>
@@ -6695,37 +6695,37 @@
       </c>
       <c r="B152" s="1" t="inlineStr">
         <is>
-          <t>QL008</t>
+          <t>QL007</t>
         </is>
       </c>
       <c r="C152" s="1" t="inlineStr">
         <is>
-          <t>SCT014</t>
+          <t>SCT013</t>
         </is>
       </c>
       <c r="D152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8013</t>
+          <t>VLINE-8011</t>
         </is>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8134</t>
+          <t>VLINE-8133</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8362</t>
+          <t>VLINE-8339</t>
         </is>
       </c>
       <c r="G152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8610</t>
+          <t>VLINE-8605</t>
         </is>
       </c>
       <c r="H152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8770</t>
+          <t>VLINE-8769</t>
         </is>
       </c>
     </row>
@@ -6737,37 +6737,37 @@
       </c>
       <c r="B153" s="1" t="inlineStr">
         <is>
-          <t>QL010</t>
+          <t>QL008</t>
         </is>
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t>SCT015</t>
+          <t>SCT014</t>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8019</t>
+          <t>VLINE-8013</t>
         </is>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8136</t>
+          <t>VLINE-8134</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8363</t>
+          <t>VLINE-8362</t>
         </is>
       </c>
       <c r="G153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8612</t>
+          <t>VLINE-8610</t>
         </is>
       </c>
       <c r="H153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8772</t>
+          <t>VLINE-8770</t>
         </is>
       </c>
     </row>
@@ -6779,37 +6779,37 @@
       </c>
       <c r="B154" s="1" t="inlineStr">
         <is>
-          <t>QL011</t>
+          <t>QL010</t>
         </is>
       </c>
       <c r="C154" s="1" t="inlineStr">
         <is>
-          <t>SO2</t>
+          <t>SCT015</t>
         </is>
       </c>
       <c r="D154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8020</t>
+          <t>VLINE-8019</t>
         </is>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8137</t>
+          <t>VLINE-8136</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8365</t>
+          <t>VLINE-8363</t>
         </is>
       </c>
       <c r="G154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8615</t>
+          <t>VLINE-8612</t>
         </is>
       </c>
       <c r="H154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8773</t>
+          <t>VLINE-8772</t>
         </is>
       </c>
     </row>
@@ -6821,37 +6821,37 @@
       </c>
       <c r="B155" s="1" t="inlineStr">
         <is>
-          <t>QL012</t>
+          <t>QL011</t>
         </is>
       </c>
       <c r="C155" s="1" t="inlineStr">
         <is>
-          <t>SO3</t>
+          <t>SO2</t>
         </is>
       </c>
       <c r="D155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8023</t>
+          <t>VLINE-8020</t>
         </is>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8140</t>
+          <t>VLINE-8137</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8366</t>
+          <t>VLINE-8365</t>
         </is>
       </c>
       <c r="G155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8617</t>
+          <t>VLINE-8615</t>
         </is>
       </c>
       <c r="H155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8774</t>
+          <t>VLINE-8773</t>
         </is>
       </c>
     </row>
@@ -6863,1137 +6863,1152 @@
       </c>
       <c r="B156" s="1" t="inlineStr">
         <is>
-          <t>QL014</t>
+          <t>QL012</t>
         </is>
       </c>
       <c r="C156" s="1" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>SO3</t>
         </is>
       </c>
       <c r="D156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8025</t>
+          <t>VLINE-8023</t>
         </is>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8141</t>
+          <t>VLINE-8140</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8368</t>
+          <t>VLINE-8366</t>
         </is>
       </c>
       <c r="G156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8620</t>
+          <t>VLINE-8617</t>
         </is>
       </c>
       <c r="H156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8776</t>
+          <t>VLINE-8774</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>NR122</t>
+          <t>NR121</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
         <is>
-          <t>QL017</t>
+          <t>QL014</t>
         </is>
       </c>
       <c r="C157" s="1" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>SSR101</t>
         </is>
       </c>
       <c r="D157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8026</t>
+          <t>VLINE-8025</t>
         </is>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8142</t>
+          <t>VLINE-8141</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8369</t>
+          <t>VLINE-8368</t>
         </is>
       </c>
       <c r="G157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8625</t>
+          <t>VLINE-8620</t>
         </is>
       </c>
       <c r="H157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8778</t>
+          <t>VLINE-8776</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>NR122</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
         <is>
-          <t>QL018</t>
+          <t>QL017</t>
         </is>
       </c>
       <c r="C158" s="1" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>SSR102</t>
         </is>
       </c>
       <c r="D158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8027</t>
+          <t>VLINE-8026</t>
         </is>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8144</t>
+          <t>VLINE-8142</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8403</t>
+          <t>VLINE-8369</t>
         </is>
       </c>
       <c r="G158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8630</t>
+          <t>VLINE-8625</t>
         </is>
       </c>
       <c r="H158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8779</t>
+          <t>VLINE-8778</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QL018</t>
         </is>
       </c>
       <c r="C159" s="1" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>SSR103</t>
         </is>
       </c>
       <c r="D159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8028</t>
+          <t>VLINE-8027</t>
         </is>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8145</t>
+          <t>VLINE-8144</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8404</t>
+          <t>VLINE-8403</t>
         </is>
       </c>
       <c r="G159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8671</t>
+          <t>VLINE-8630</t>
         </is>
       </c>
       <c r="H159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8780</t>
+          <t>VLINE-8779</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>P2501</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QR1744</t>
         </is>
       </c>
       <c r="C160" s="1" t="inlineStr">
         <is>
-          <t>T363</t>
+          <t>SSR104</t>
         </is>
       </c>
       <c r="D160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8029</t>
+          <t>VLINE-8028</t>
         </is>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8148</t>
+          <t>VLINE-8145</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8406</t>
+          <t>VLINE-8404</t>
         </is>
       </c>
       <c r="G160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8706</t>
+          <t>VLINE-8671</t>
         </is>
       </c>
       <c r="H160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8781</t>
+          <t>VLINE-8780</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>P2502</t>
+          <t>P2501</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QR1771</t>
         </is>
       </c>
       <c r="C161" s="1" t="inlineStr">
         <is>
-          <t>T381</t>
+          <t>T363</t>
         </is>
       </c>
       <c r="D161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8030</t>
+          <t>VLINE-8029</t>
         </is>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8150</t>
+          <t>VLINE-8148</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8408</t>
+          <t>VLINE-8406</t>
         </is>
       </c>
       <c r="G161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8711</t>
+          <t>VLINE-8706</t>
         </is>
       </c>
       <c r="H161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8782</t>
+          <t>VLINE-8781</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>P2503</t>
+          <t>P2502</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
         <is>
-          <t>R711</t>
+          <t>QR5404</t>
         </is>
       </c>
       <c r="C162" s="1" t="inlineStr">
         <is>
-          <t>T386</t>
+          <t>T381</t>
         </is>
       </c>
       <c r="D162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8031</t>
+          <t>VLINE-8030</t>
         </is>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8151</t>
+          <t>VLINE-8150</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8410</t>
+          <t>VLINE-8408</t>
         </is>
       </c>
       <c r="G162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8714</t>
+          <t>VLINE-8711</t>
         </is>
       </c>
       <c r="H162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8783</t>
+          <t>VLINE-8782</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>P2504</t>
+          <t>P2503</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
         <is>
-          <t>R766</t>
+          <t>R711</t>
         </is>
       </c>
       <c r="C163" s="1" t="inlineStr">
         <is>
-          <t>TDX101</t>
+          <t>T386</t>
         </is>
       </c>
       <c r="D163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8032</t>
+          <t>VLINE-8031</t>
         </is>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8152</t>
+          <t>VLINE-8151</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8411</t>
+          <t>VLINE-8410</t>
         </is>
       </c>
       <c r="G163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8717</t>
+          <t>VLINE-8714</t>
         </is>
       </c>
       <c r="H163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8784</t>
+          <t>VLINE-8783</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>P2505</t>
+          <t>P2504</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>R766</t>
         </is>
       </c>
       <c r="C164" s="1" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>TDX101</t>
         </is>
       </c>
       <c r="D164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8036</t>
+          <t>VLINE-8032</t>
         </is>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8153</t>
+          <t>VLINE-8152</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8413</t>
+          <t>VLINE-8411</t>
         </is>
       </c>
       <c r="G164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8720</t>
+          <t>VLINE-8717</t>
         </is>
       </c>
       <c r="H164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8786</t>
+          <t>VLINE-8784</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>P2506</t>
+          <t>P2505</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
         <is>
-          <t>RCTST4</t>
+          <t>RB2353</t>
         </is>
       </c>
       <c r="C165" s="1" t="inlineStr">
         <is>
-          <t>TE2802</t>
+          <t>TE2801</t>
         </is>
       </c>
       <c r="D165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8038</t>
+          <t>VLINE-8036</t>
         </is>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8154</t>
+          <t>VLINE-8153</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8415</t>
+          <t>VLINE-8413</t>
         </is>
       </c>
       <c r="G165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8721</t>
+          <t>VLINE-8720</t>
         </is>
       </c>
       <c r="H165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8787</t>
+          <t>VLINE-8786</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>P2507</t>
+          <t>P2506</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>RCTST4</t>
         </is>
       </c>
       <c r="C166" s="1" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>TE2802</t>
         </is>
       </c>
       <c r="D166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8039</t>
+          <t>VLINE-8038</t>
         </is>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8155</t>
+          <t>VLINE-8154</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8417</t>
+          <t>VLINE-8415</t>
         </is>
       </c>
       <c r="G166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8723</t>
+          <t>VLINE-8721</t>
         </is>
       </c>
       <c r="H166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8788</t>
+          <t>VLINE-8787</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>P2508</t>
+          <t>P2507</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
         <is>
-          <t>RL302</t>
+          <t>RL301</t>
         </is>
       </c>
       <c r="C167" s="1" t="inlineStr">
         <is>
-          <t>TE2804</t>
+          <t>TE2803</t>
         </is>
       </c>
       <c r="D167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8042</t>
+          <t>VLINE-8039</t>
         </is>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8157</t>
+          <t>VLINE-8155</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8418</t>
+          <t>VLINE-8417</t>
         </is>
       </c>
       <c r="G167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8725</t>
+          <t>VLINE-8723</t>
         </is>
       </c>
       <c r="H167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8790</t>
+          <t>VLINE-8788</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>P2509</t>
+          <t>P2508</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
         <is>
-          <t>RL304</t>
+          <t>RL302</t>
         </is>
       </c>
       <c r="C168" s="1" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>TE2804</t>
         </is>
       </c>
       <c r="D168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8049</t>
+          <t>VLINE-8042</t>
         </is>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8158</t>
+          <t>VLINE-8157</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8419</t>
+          <t>VLINE-8418</t>
         </is>
       </c>
       <c r="G168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8726</t>
+          <t>VLINE-8725</t>
         </is>
       </c>
       <c r="H168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8792</t>
+          <t>VLINE-8790</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>P2510</t>
+          <t>P2509</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
         <is>
-          <t>RL305</t>
+          <t>RL304</t>
         </is>
       </c>
       <c r="C169" s="1" t="inlineStr">
         <is>
-          <t>TE2806</t>
+          <t>TE2805</t>
         </is>
       </c>
       <c r="D169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8050</t>
+          <t>VLINE-8049</t>
         </is>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8159</t>
+          <t>VLINE-8158</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8420</t>
+          <t>VLINE-8419</t>
         </is>
       </c>
       <c r="G169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8727</t>
+          <t>VLINE-8726</t>
         </is>
       </c>
       <c r="H169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8793</t>
+          <t>VLINE-8792</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>P2511</t>
+          <t>P2510</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
         <is>
-          <t>RL306</t>
+          <t>RL305</t>
         </is>
       </c>
       <c r="C170" s="1" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>TE2806</t>
         </is>
       </c>
       <c r="D170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8051</t>
+          <t>VLINE-8050</t>
         </is>
       </c>
       <c r="E170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8160</t>
+          <t>VLINE-8159</t>
         </is>
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8421</t>
+          <t>VLINE-8420</t>
         </is>
       </c>
       <c r="G170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8729</t>
+          <t>VLINE-8727</t>
         </is>
       </c>
       <c r="H170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8794</t>
+          <t>VLINE-8793</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8795</t>
+          <t>VLINE-8794</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
         <is>
-          <t>XP2016</t>
+          <t>XP2013</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8796</t>
+          <t>VLINE-8795</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
         <is>
-          <t>XP2017</t>
+          <t>XP2014</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8797</t>
+          <t>VLINE-8796</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>XP2015</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8799</t>
+          <t>VLINE-8797</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
         <is>
-          <t>XR550</t>
+          <t>XP2016</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8800</t>
+          <t>VLINE-8799</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
         <is>
-          <t>XR552</t>
+          <t>XP2017</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8801</t>
+          <t>VLINE-8800</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
         <is>
-          <t>XR559</t>
+          <t>XP2019</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8802</t>
+          <t>VLINE-8801</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
         <is>
-          <t>XRN001</t>
+          <t>XR550</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8803</t>
+          <t>VLINE-8802</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
         <is>
-          <t>XRN004</t>
+          <t>XR552</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8804</t>
+          <t>VLINE-8803</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>XR559</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8805</t>
+          <t>VLINE-8804</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
         <is>
-          <t>XRN006</t>
+          <t>XRN001</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8806</t>
+          <t>VLINE-8805</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
         <is>
-          <t>XRN007</t>
+          <t>XRN004</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8807</t>
+          <t>VLINE-8806</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>XRN005</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8808</t>
+          <t>VLINE-8807</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
         <is>
-          <t>XRN011</t>
+          <t>XRN006</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8809</t>
+          <t>VLINE-8808</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
         <is>
-          <t>XRN014</t>
+          <t>XRN007</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8810</t>
+          <t>VLINE-8809</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>XRN009</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8811</t>
+          <t>VLINE-8810</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>XRN011</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8812</t>
+          <t>VLINE-8811</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
         <is>
-          <t>XRN020</t>
+          <t>XRN014</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8813</t>
+          <t>VLINE-8812</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>XRN017</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8814</t>
+          <t>VLINE-8813</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
         <is>
-          <t>XRN023</t>
+          <t>XRN018</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8816</t>
+          <t>VLINE-8814</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
         <is>
-          <t>XRN025</t>
+          <t>XRN020</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8817</t>
+          <t>VLINE-8815</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
         <is>
-          <t>XRN026</t>
+          <t>XRN021</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8818</t>
+          <t>VLINE-8816</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
         <is>
-          <t>XRN027</t>
+          <t>XRN023</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8819</t>
+          <t>VLINE-8817</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
         <is>
-          <t>XRN029</t>
+          <t>XRN025</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8822</t>
+          <t>VLINE-8818</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
         <is>
-          <t>Y163</t>
+          <t>XRN026</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8860</t>
+          <t>VLINE-8819</t>
+        </is>
+      </c>
+      <c r="B196" s="1" t="inlineStr">
+        <is>
+          <t>XRN027</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8861</t>
+          <t>VLINE-8820</t>
+        </is>
+      </c>
+      <c r="B197" s="1" t="inlineStr">
+        <is>
+          <t>XRN029</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8862</t>
+          <t>VLINE-8822</t>
+        </is>
+      </c>
+      <c r="B198" s="1" t="inlineStr">
+        <is>
+          <t>Y163</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8863</t>
+          <t>VLINE-8860</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8864</t>
+          <t>VLINE-8861</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8865</t>
+          <t>VLINE-8862</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8866</t>
+          <t>VLINE-8863</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8867</t>
+          <t>VLINE-8864</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8868</t>
+          <t>VLINE-8865</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8869</t>
+          <t>VLINE-8866</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8890</t>
+          <t>VLINE-8867</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8891</t>
+          <t>VLINE-8868</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8893</t>
+          <t>VLINE-8869</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8895</t>
+          <t>VLINE-8890</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>WH001</t>
+          <t>VLINE-8891</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>WH003</t>
+          <t>VLINE-8893</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>WL02</t>
+          <t>VLINE-8895</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>X12-X14</t>
+          <t>WH001</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>X31</t>
+          <t>WH003</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>XP2000</t>
+          <t>WL02</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>XP2001</t>
+          <t>X12-X14</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>XP2003</t>
+          <t>X31</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>XP2004</t>
+          <t>XP2000</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>XP2001</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>XP2007</t>
+          <t>XP2003</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>XP2004</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>XP2010</t>
+          <t>XP2005</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>XP2007</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>XP2008</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>XP2010</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>XP2011</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>XP2012</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update trains and loco export 2026-04-06 14:59:26
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -2819,7 +2819,7 @@
       </c>
       <c r="H58" s="1" t="inlineStr">
         <is>
-          <t>N454</t>
+          <t>N453</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2861,7 @@
       </c>
       <c r="H59" s="1" t="inlineStr">
         <is>
-          <t>N457</t>
+          <t>N454</t>
         </is>
       </c>
     </row>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="H60" s="1" t="inlineStr">
         <is>
-          <t>N458</t>
+          <t>N457</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="H61" s="1" t="inlineStr">
         <is>
-          <t>N460</t>
+          <t>N458</t>
         </is>
       </c>
     </row>
@@ -2987,7 +2987,7 @@
       </c>
       <c r="H62" s="1" t="inlineStr">
         <is>
-          <t>N461</t>
+          <t>N460</t>
         </is>
       </c>
     </row>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="H63" s="1" t="inlineStr">
         <is>
-          <t>N465</t>
+          <t>N461</t>
         </is>
       </c>
     </row>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="H64" s="1" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>N465</t>
         </is>
       </c>
     </row>
@@ -3113,7 +3113,7 @@
       </c>
       <c r="H65" s="1" t="inlineStr">
         <is>
-          <t>N467</t>
+          <t>N466</t>
         </is>
       </c>
     </row>
@@ -3155,7 +3155,7 @@
       </c>
       <c r="H66" s="1" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>N467</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
       </c>
       <c r="H67" s="1" t="inlineStr">
         <is>
-          <t>N473</t>
+          <t>N469</t>
         </is>
       </c>
     </row>
@@ -3239,7 +3239,7 @@
       </c>
       <c r="H68" s="1" t="inlineStr">
         <is>
-          <t>NR1</t>
+          <t>N473</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="H69" s="1" t="inlineStr">
         <is>
-          <t>NR2</t>
+          <t>NR1</t>
         </is>
       </c>
     </row>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="H70" s="1" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>NR2</t>
         </is>
       </c>
     </row>
@@ -3365,7 +3365,7 @@
       </c>
       <c r="H71" s="1" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>NR4</t>
         </is>
       </c>
     </row>
@@ -3407,7 +3407,7 @@
       </c>
       <c r="H72" s="1" t="inlineStr">
         <is>
-          <t>NR7</t>
+          <t>NR5</t>
         </is>
       </c>
     </row>
@@ -3444,12 +3444,12 @@
       </c>
       <c r="G73" s="1" t="inlineStr">
         <is>
-          <t>MM-9926M</t>
+          <t>MM-9925M</t>
         </is>
       </c>
       <c r="H73" s="1" t="inlineStr">
         <is>
-          <t>NR8</t>
+          <t>NR7</t>
         </is>
       </c>
     </row>
@@ -3486,12 +3486,12 @@
       </c>
       <c r="G74" s="1" t="inlineStr">
         <is>
-          <t>MM-9928M</t>
+          <t>MM-9926M</t>
         </is>
       </c>
       <c r="H74" s="1" t="inlineStr">
         <is>
-          <t>NR9</t>
+          <t>NR8</t>
         </is>
       </c>
     </row>
@@ -3528,12 +3528,12 @@
       </c>
       <c r="G75" s="1" t="inlineStr">
         <is>
-          <t>MM-9929M</t>
+          <t>MM-9928M</t>
         </is>
       </c>
       <c r="H75" s="1" t="inlineStr">
         <is>
-          <t>NR10</t>
+          <t>NR9</t>
         </is>
       </c>
     </row>
@@ -3570,12 +3570,12 @@
       </c>
       <c r="G76" s="1" t="inlineStr">
         <is>
-          <t>MM-9932M</t>
+          <t>MM-9929M</t>
         </is>
       </c>
       <c r="H76" s="1" t="inlineStr">
         <is>
-          <t>NR12</t>
+          <t>NR10</t>
         </is>
       </c>
     </row>
@@ -3612,12 +3612,12 @@
       </c>
       <c r="G77" s="1" t="inlineStr">
         <is>
-          <t>MM-9933M</t>
+          <t>MM-9932M</t>
         </is>
       </c>
       <c r="H77" s="1" t="inlineStr">
         <is>
-          <t>NR13</t>
+          <t>NR12</t>
         </is>
       </c>
     </row>
@@ -3654,12 +3654,12 @@
       </c>
       <c r="G78" s="1" t="inlineStr">
         <is>
-          <t>MM-9934M</t>
+          <t>MM-9933M</t>
         </is>
       </c>
       <c r="H78" s="1" t="inlineStr">
         <is>
-          <t>NR15</t>
+          <t>NR13</t>
         </is>
       </c>
     </row>
@@ -3696,12 +3696,12 @@
       </c>
       <c r="G79" s="1" t="inlineStr">
         <is>
-          <t>MM-9936M</t>
+          <t>MM-9934M</t>
         </is>
       </c>
       <c r="H79" s="1" t="inlineStr">
         <is>
-          <t>NR16</t>
+          <t>NR15</t>
         </is>
       </c>
     </row>
@@ -3738,12 +3738,12 @@
       </c>
       <c r="G80" s="1" t="inlineStr">
         <is>
-          <t>MM-9938M</t>
+          <t>MM-9936M</t>
         </is>
       </c>
       <c r="H80" s="1" t="inlineStr">
         <is>
-          <t>NR18</t>
+          <t>NR16</t>
         </is>
       </c>
     </row>
@@ -3780,12 +3780,12 @@
       </c>
       <c r="G81" s="1" t="inlineStr">
         <is>
-          <t>MM-9941M</t>
+          <t>MM-9938M</t>
         </is>
       </c>
       <c r="H81" s="1" t="inlineStr">
         <is>
-          <t>NR19</t>
+          <t>NR18</t>
         </is>
       </c>
     </row>
@@ -3822,12 +3822,12 @@
       </c>
       <c r="G82" s="1" t="inlineStr">
         <is>
-          <t>MM-9943M</t>
+          <t>MM-9941M</t>
         </is>
       </c>
       <c r="H82" s="1" t="inlineStr">
         <is>
-          <t>NR20</t>
+          <t>NR19</t>
         </is>
       </c>
     </row>
@@ -3864,12 +3864,12 @@
       </c>
       <c r="G83" s="1" t="inlineStr">
         <is>
-          <t>MM-9945M</t>
+          <t>MM-9943M</t>
         </is>
       </c>
       <c r="H83" s="1" t="inlineStr">
         <is>
-          <t>NR21</t>
+          <t>NR20</t>
         </is>
       </c>
     </row>
@@ -3906,12 +3906,12 @@
       </c>
       <c r="G84" s="1" t="inlineStr">
         <is>
-          <t>MM-9946M</t>
+          <t>MM-9945M</t>
         </is>
       </c>
       <c r="H84" s="1" t="inlineStr">
         <is>
-          <t>NR25</t>
+          <t>NR21</t>
         </is>
       </c>
     </row>
@@ -3948,12 +3948,12 @@
       </c>
       <c r="G85" s="1" t="inlineStr">
         <is>
-          <t>MM-9949M</t>
+          <t>MM-9946M</t>
         </is>
       </c>
       <c r="H85" s="1" t="inlineStr">
         <is>
-          <t>NR27</t>
+          <t>NR25</t>
         </is>
       </c>
     </row>
@@ -3990,12 +3990,12 @@
       </c>
       <c r="G86" s="1" t="inlineStr">
         <is>
-          <t>MM-9950M</t>
+          <t>MM-9949M</t>
         </is>
       </c>
       <c r="H86" s="1" t="inlineStr">
         <is>
-          <t>NR28</t>
+          <t>NR27</t>
         </is>
       </c>
     </row>
@@ -4032,12 +4032,12 @@
       </c>
       <c r="G87" s="1" t="inlineStr">
         <is>
-          <t>MM-9951M</t>
+          <t>MM-9950M</t>
         </is>
       </c>
       <c r="H87" s="1" t="inlineStr">
         <is>
-          <t>NR29</t>
+          <t>NR28</t>
         </is>
       </c>
     </row>
@@ -4074,12 +4074,12 @@
       </c>
       <c r="G88" s="1" t="inlineStr">
         <is>
-          <t>MM-9952M</t>
+          <t>MM-9951M</t>
         </is>
       </c>
       <c r="H88" s="1" t="inlineStr">
         <is>
-          <t>NR30</t>
+          <t>NR29</t>
         </is>
       </c>
     </row>
@@ -4116,12 +4116,12 @@
       </c>
       <c r="G89" s="1" t="inlineStr">
         <is>
-          <t>MM-9953M</t>
+          <t>MM-9952M</t>
         </is>
       </c>
       <c r="H89" s="1" t="inlineStr">
         <is>
-          <t>NR31</t>
+          <t>NR30</t>
         </is>
       </c>
     </row>
@@ -4158,12 +4158,12 @@
       </c>
       <c r="G90" s="1" t="inlineStr">
         <is>
-          <t>MM-9954M</t>
+          <t>MM-9953M</t>
         </is>
       </c>
       <c r="H90" s="1" t="inlineStr">
         <is>
-          <t>NR34</t>
+          <t>NR31</t>
         </is>
       </c>
     </row>
@@ -4200,12 +4200,12 @@
       </c>
       <c r="G91" s="1" t="inlineStr">
         <is>
-          <t>MM-9955M</t>
+          <t>MM-9954M</t>
         </is>
       </c>
       <c r="H91" s="1" t="inlineStr">
         <is>
-          <t>NR36</t>
+          <t>NR34</t>
         </is>
       </c>
     </row>
@@ -4242,12 +4242,12 @@
       </c>
       <c r="G92" s="1" t="inlineStr">
         <is>
-          <t>MM-9957M</t>
+          <t>MM-9955M</t>
         </is>
       </c>
       <c r="H92" s="1" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>NR36</t>
         </is>
       </c>
     </row>
@@ -4284,12 +4284,12 @@
       </c>
       <c r="G93" s="1" t="inlineStr">
         <is>
-          <t>MM-9958M</t>
+          <t>MM-9957M</t>
         </is>
       </c>
       <c r="H93" s="1" t="inlineStr">
         <is>
-          <t>NR38</t>
+          <t>NR37</t>
         </is>
       </c>
     </row>
@@ -4326,12 +4326,12 @@
       </c>
       <c r="G94" s="1" t="inlineStr">
         <is>
-          <t>MM-9959M</t>
+          <t>MM-9958M</t>
         </is>
       </c>
       <c r="H94" s="1" t="inlineStr">
         <is>
-          <t>NR39</t>
+          <t>NR38</t>
         </is>
       </c>
     </row>
@@ -4368,12 +4368,12 @@
       </c>
       <c r="G95" s="1" t="inlineStr">
         <is>
-          <t>MM-9960M</t>
+          <t>MM-9959M</t>
         </is>
       </c>
       <c r="H95" s="1" t="inlineStr">
         <is>
-          <t>NR40</t>
+          <t>NR39</t>
         </is>
       </c>
     </row>
@@ -4410,12 +4410,12 @@
       </c>
       <c r="G96" s="1" t="inlineStr">
         <is>
-          <t>MM-9961M</t>
+          <t>MM-9960M</t>
         </is>
       </c>
       <c r="H96" s="1" t="inlineStr">
         <is>
-          <t>NR43</t>
+          <t>NR40</t>
         </is>
       </c>
     </row>
@@ -4452,12 +4452,12 @@
       </c>
       <c r="G97" s="1" t="inlineStr">
         <is>
-          <t>MM-9962M</t>
+          <t>MM-9961M</t>
         </is>
       </c>
       <c r="H97" s="1" t="inlineStr">
         <is>
-          <t>NR44</t>
+          <t>NR43</t>
         </is>
       </c>
     </row>
@@ -4494,12 +4494,12 @@
       </c>
       <c r="G98" s="1" t="inlineStr">
         <is>
-          <t>MM-9963M</t>
+          <t>MM-9962M</t>
         </is>
       </c>
       <c r="H98" s="1" t="inlineStr">
         <is>
-          <t>NR45</t>
+          <t>NR44</t>
         </is>
       </c>
     </row>
@@ -4536,12 +4536,12 @@
       </c>
       <c r="G99" s="1" t="inlineStr">
         <is>
-          <t>MM-9964M</t>
+          <t>MM-9963M</t>
         </is>
       </c>
       <c r="H99" s="1" t="inlineStr">
         <is>
-          <t>NR46</t>
+          <t>NR45</t>
         </is>
       </c>
     </row>
@@ -4578,12 +4578,12 @@
       </c>
       <c r="G100" s="1" t="inlineStr">
         <is>
-          <t>MM-9965M</t>
+          <t>MM-9964M</t>
         </is>
       </c>
       <c r="H100" s="1" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>NR46</t>
         </is>
       </c>
     </row>
@@ -4620,12 +4620,12 @@
       </c>
       <c r="G101" s="1" t="inlineStr">
         <is>
-          <t>MM-9966M</t>
+          <t>MM-9965M</t>
         </is>
       </c>
       <c r="H101" s="1" t="inlineStr">
         <is>
-          <t>NR48</t>
+          <t>NR47</t>
         </is>
       </c>
     </row>
@@ -4662,12 +4662,12 @@
       </c>
       <c r="G102" s="1" t="inlineStr">
         <is>
-          <t>MM-9967M</t>
+          <t>MM-9966M</t>
         </is>
       </c>
       <c r="H102" s="1" t="inlineStr">
         <is>
-          <t>NR51</t>
+          <t>NR48</t>
         </is>
       </c>
     </row>
@@ -4704,12 +4704,12 @@
       </c>
       <c r="G103" s="1" t="inlineStr">
         <is>
-          <t>MM-9968M</t>
+          <t>MM-9967M</t>
         </is>
       </c>
       <c r="H103" s="1" t="inlineStr">
         <is>
-          <t>NR52</t>
+          <t>NR51</t>
         </is>
       </c>
     </row>
@@ -4746,12 +4746,12 @@
       </c>
       <c r="G104" s="1" t="inlineStr">
         <is>
-          <t>MM-9969M</t>
+          <t>MM-9968M</t>
         </is>
       </c>
       <c r="H104" s="1" t="inlineStr">
         <is>
-          <t>NR53</t>
+          <t>NR52</t>
         </is>
       </c>
     </row>
@@ -4788,12 +4788,12 @@
       </c>
       <c r="G105" s="1" t="inlineStr">
         <is>
-          <t>MM-9970M</t>
+          <t>MM-9969M</t>
         </is>
       </c>
       <c r="H105" s="1" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>NR53</t>
         </is>
       </c>
     </row>
@@ -4830,12 +4830,12 @@
       </c>
       <c r="G106" s="1" t="inlineStr">
         <is>
-          <t>MMY032</t>
+          <t>MM-9970M</t>
         </is>
       </c>
       <c r="H106" s="1" t="inlineStr">
         <is>
-          <t>NR57</t>
+          <t>NR54</t>
         </is>
       </c>
     </row>
@@ -4872,12 +4872,12 @@
       </c>
       <c r="G107" s="1" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MMY032</t>
         </is>
       </c>
       <c r="H107" s="1" t="inlineStr">
         <is>
-          <t>NR58</t>
+          <t>NR57</t>
         </is>
       </c>
     </row>
@@ -4914,12 +4914,12 @@
       </c>
       <c r="G108" s="1" t="inlineStr">
         <is>
-          <t>MRL004</t>
+          <t>MRL001</t>
         </is>
       </c>
       <c r="H108" s="1" t="inlineStr">
         <is>
-          <t>NR59</t>
+          <t>NR58</t>
         </is>
       </c>
     </row>
@@ -4956,12 +4956,12 @@
       </c>
       <c r="G109" s="1" t="inlineStr">
         <is>
-          <t>MRL005</t>
+          <t>MRL004</t>
         </is>
       </c>
       <c r="H109" s="1" t="inlineStr">
         <is>
-          <t>NR61</t>
+          <t>NR59</t>
         </is>
       </c>
     </row>
@@ -4998,12 +4998,12 @@
       </c>
       <c r="G110" s="1" t="inlineStr">
         <is>
-          <t>MRL006</t>
+          <t>MRL005</t>
         </is>
       </c>
       <c r="H110" s="1" t="inlineStr">
         <is>
-          <t>NR62</t>
+          <t>NR61</t>
         </is>
       </c>
     </row>
@@ -5040,12 +5040,12 @@
       </c>
       <c r="G111" s="1" t="inlineStr">
         <is>
-          <t>MTPV2</t>
+          <t>MRL006</t>
         </is>
       </c>
       <c r="H111" s="1" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR62</t>
         </is>
       </c>
     </row>
@@ -5082,12 +5082,12 @@
       </c>
       <c r="G112" s="1" t="inlineStr">
         <is>
-          <t>N452</t>
+          <t>MTPV2</t>
         </is>
       </c>
       <c r="H112" s="1" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR64</t>
         </is>
       </c>
     </row>
@@ -5124,2896 +5124,2911 @@
       </c>
       <c r="G113" s="1" t="inlineStr">
         <is>
-          <t>N453</t>
+          <t>N452</t>
         </is>
       </c>
       <c r="H113" s="1" t="inlineStr">
         <is>
-          <t>NR66</t>
+          <t>NR65</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>NR67</t>
+          <t>NR66</t>
         </is>
       </c>
       <c r="B115" s="1" t="inlineStr">
         <is>
-          <t>P2510</t>
+          <t>P2509</t>
         </is>
       </c>
       <c r="C115" s="1" t="inlineStr">
         <is>
-          <t>RL305</t>
+          <t>RL304</t>
         </is>
       </c>
       <c r="D115" s="1" t="inlineStr">
         <is>
-          <t>TE2806</t>
+          <t>TE2805</t>
         </is>
       </c>
       <c r="E115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8050</t>
+          <t>VLINE-8049</t>
         </is>
       </c>
       <c r="F115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8159</t>
+          <t>VLINE-8158</t>
         </is>
       </c>
       <c r="G115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8420</t>
+          <t>VLINE-8418</t>
         </is>
       </c>
       <c r="H115" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8727</t>
+          <t>VLINE-8725</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR67</t>
         </is>
       </c>
       <c r="B116" s="1" t="inlineStr">
         <is>
-          <t>P2511</t>
+          <t>P2510</t>
         </is>
       </c>
       <c r="C116" s="1" t="inlineStr">
         <is>
-          <t>RL306</t>
+          <t>RL305</t>
         </is>
       </c>
       <c r="D116" s="1" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>TE2806</t>
         </is>
       </c>
       <c r="E116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8051</t>
+          <t>VLINE-8050</t>
         </is>
       </c>
       <c r="F116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8160</t>
+          <t>VLINE-8159</t>
         </is>
       </c>
       <c r="G116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8421</t>
+          <t>VLINE-8419</t>
         </is>
       </c>
       <c r="H116" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8729</t>
+          <t>VLINE-8726</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>NR69</t>
+          <t>NR68</t>
         </is>
       </c>
       <c r="B117" s="1" t="inlineStr">
         <is>
-          <t>P2513</t>
+          <t>P2511</t>
         </is>
       </c>
       <c r="C117" s="1" t="inlineStr">
         <is>
-          <t>RL307</t>
+          <t>RL306</t>
         </is>
       </c>
       <c r="D117" s="1" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>TE2807</t>
         </is>
       </c>
       <c r="E117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8052</t>
+          <t>VLINE-8051</t>
         </is>
       </c>
       <c r="F117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8161</t>
+          <t>VLINE-8160</t>
         </is>
       </c>
       <c r="G117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8422</t>
+          <t>VLINE-8420</t>
         </is>
       </c>
       <c r="H117" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8730</t>
+          <t>VLINE-8727</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>NR71</t>
+          <t>NR69</t>
         </is>
       </c>
       <c r="B118" s="1" t="inlineStr">
         <is>
-          <t>P2514</t>
+          <t>P2513</t>
         </is>
       </c>
       <c r="C118" s="1" t="inlineStr">
         <is>
-          <t>RL309</t>
+          <t>RL307</t>
         </is>
       </c>
       <c r="D118" s="1" t="inlineStr">
         <is>
-          <t>TE2809</t>
+          <t>TE2808</t>
         </is>
       </c>
       <c r="E118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8053</t>
+          <t>VLINE-8052</t>
         </is>
       </c>
       <c r="F118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8162</t>
+          <t>VLINE-8161</t>
         </is>
       </c>
       <c r="G118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8424</t>
+          <t>VLINE-8421</t>
         </is>
       </c>
       <c r="H118" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8731</t>
+          <t>VLINE-8729</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>NR72</t>
+          <t>NR71</t>
         </is>
       </c>
       <c r="B119" s="1" t="inlineStr">
         <is>
-          <t>P2515</t>
+          <t>P2514</t>
         </is>
       </c>
       <c r="C119" s="1" t="inlineStr">
         <is>
-          <t>RL310</t>
+          <t>RL309</t>
         </is>
       </c>
       <c r="D119" s="1" t="inlineStr">
         <is>
-          <t>TE2810</t>
+          <t>TE2809</t>
         </is>
       </c>
       <c r="E119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8055</t>
+          <t>VLINE-8053</t>
         </is>
       </c>
       <c r="F119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8171</t>
+          <t>VLINE-8162</t>
         </is>
       </c>
       <c r="G119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8425</t>
+          <t>VLINE-8422</t>
         </is>
       </c>
       <c r="H119" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8733</t>
+          <t>VLINE-8730</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR72</t>
         </is>
       </c>
       <c r="B120" s="1" t="inlineStr">
         <is>
-          <t>P2516</t>
+          <t>P2515</t>
         </is>
       </c>
       <c r="C120" s="1" t="inlineStr">
         <is>
-          <t>S312</t>
+          <t>RL310</t>
         </is>
       </c>
       <c r="D120" s="1" t="inlineStr">
         <is>
-          <t>TE2812</t>
+          <t>TE2810</t>
         </is>
       </c>
       <c r="E120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8056</t>
+          <t>VLINE-8055</t>
         </is>
       </c>
       <c r="F120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8172</t>
+          <t>VLINE-8165</t>
         </is>
       </c>
       <c r="G120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8426</t>
+          <t>VLINE-8424</t>
         </is>
       </c>
       <c r="H120" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8735</t>
+          <t>VLINE-8731</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t>NR77</t>
+          <t>NR75</t>
         </is>
       </c>
       <c r="B121" s="1" t="inlineStr">
         <is>
-          <t>PB1</t>
+          <t>P2516</t>
         </is>
       </c>
       <c r="C121" s="1" t="inlineStr">
         <is>
-          <t>S317</t>
+          <t>S312</t>
         </is>
       </c>
       <c r="D121" s="1" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>TE2812</t>
         </is>
       </c>
       <c r="E121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8057</t>
+          <t>VLINE-8056</t>
         </is>
       </c>
       <c r="F121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8176</t>
+          <t>VLINE-8171</t>
         </is>
       </c>
       <c r="G121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8427</t>
+          <t>VLINE-8425</t>
         </is>
       </c>
       <c r="H121" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8736</t>
+          <t>VLINE-8733</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR77</t>
         </is>
       </c>
       <c r="B122" s="1" t="inlineStr">
         <is>
-          <t>PB2</t>
+          <t>PB1</t>
         </is>
       </c>
       <c r="C122" s="1" t="inlineStr">
         <is>
-          <t>S3301</t>
+          <t>S317</t>
         </is>
       </c>
       <c r="D122" s="1" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>TE2813</t>
         </is>
       </c>
       <c r="E122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8058</t>
+          <t>VLINE-8057</t>
         </is>
       </c>
       <c r="F122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8179</t>
+          <t>VLINE-8172</t>
         </is>
       </c>
       <c r="G122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8428</t>
+          <t>VLINE-8426</t>
         </is>
       </c>
       <c r="H122" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8737</t>
+          <t>VLINE-8735</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t>NR81</t>
+          <t>NR78</t>
         </is>
       </c>
       <c r="B123" s="1" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>PB2</t>
         </is>
       </c>
       <c r="C123" s="1" t="inlineStr">
         <is>
-          <t>S3302</t>
+          <t>S3301</t>
         </is>
       </c>
       <c r="D123" s="1" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>TE2814</t>
         </is>
       </c>
       <c r="E123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8059</t>
+          <t>VLINE-8058</t>
         </is>
       </c>
       <c r="F123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8180</t>
+          <t>VLINE-8176</t>
         </is>
       </c>
       <c r="G123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8429</t>
+          <t>VLINE-8427</t>
         </is>
       </c>
       <c r="H123" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8739</t>
+          <t>VLINE-8736</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR81</t>
         </is>
       </c>
       <c r="B124" s="1" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>PB4</t>
         </is>
       </c>
       <c r="C124" s="1" t="inlineStr">
         <is>
-          <t>S3304</t>
+          <t>S3302</t>
         </is>
       </c>
       <c r="D124" s="1" t="inlineStr">
         <is>
-          <t>TJ107</t>
+          <t>TJ096</t>
         </is>
       </c>
       <c r="E124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8061</t>
+          <t>VLINE-8059</t>
         </is>
       </c>
       <c r="F124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8181</t>
+          <t>VLINE-8179</t>
         </is>
       </c>
       <c r="G124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8430</t>
+          <t>VLINE-8428</t>
         </is>
       </c>
       <c r="H124" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8740</t>
+          <t>VLINE-8737</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR82</t>
         </is>
       </c>
       <c r="B125" s="1" t="inlineStr">
         <is>
-          <t>PHC002</t>
+          <t>PHC001</t>
         </is>
       </c>
       <c r="C125" s="1" t="inlineStr">
         <is>
-          <t>S3305</t>
+          <t>S3304</t>
         </is>
       </c>
       <c r="D125" s="1" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TJ107</t>
         </is>
       </c>
       <c r="E125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8072</t>
+          <t>VLINE-8061</t>
         </is>
       </c>
       <c r="F125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8182</t>
+          <t>VLINE-8180</t>
         </is>
       </c>
       <c r="G125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8431</t>
+          <t>VLINE-8429</t>
         </is>
       </c>
       <c r="H125" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8741</t>
+          <t>VLINE-8739</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>NR84</t>
+          <t>NR83</t>
         </is>
       </c>
       <c r="B126" s="1" t="inlineStr">
         <is>
-          <t>Q4001</t>
+          <t>PHC002</t>
         </is>
       </c>
       <c r="C126" s="1" t="inlineStr">
         <is>
-          <t>S3306</t>
+          <t>S3305</t>
         </is>
       </c>
       <c r="D126" s="1" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TT03</t>
         </is>
       </c>
       <c r="E126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8074</t>
+          <t>VLINE-8072</t>
         </is>
       </c>
       <c r="F126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8183</t>
+          <t>VLINE-8181</t>
         </is>
       </c>
       <c r="G126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8432</t>
+          <t>VLINE-8430</t>
         </is>
       </c>
       <c r="H126" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8742</t>
+          <t>VLINE-8740</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>NR85</t>
+          <t>NR84</t>
         </is>
       </c>
       <c r="B127" s="1" t="inlineStr">
         <is>
-          <t>Q4003</t>
+          <t>Q4001</t>
         </is>
       </c>
       <c r="C127" s="1" t="inlineStr">
         <is>
-          <t>S3307</t>
+          <t>S3306</t>
         </is>
       </c>
       <c r="D127" s="1" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TT04</t>
         </is>
       </c>
       <c r="E127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8075</t>
+          <t>VLINE-8074</t>
         </is>
       </c>
       <c r="F127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8184</t>
+          <t>VLINE-8182</t>
         </is>
       </c>
       <c r="G127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8433</t>
+          <t>VLINE-8431</t>
         </is>
       </c>
       <c r="H127" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8743</t>
+          <t>VLINE-8741</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>NR86</t>
+          <t>NR85</t>
         </is>
       </c>
       <c r="B128" s="1" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>Q4003</t>
         </is>
       </c>
       <c r="C128" s="1" t="inlineStr">
         <is>
-          <t>S3309</t>
+          <t>S3307</t>
         </is>
       </c>
       <c r="D128" s="1" t="inlineStr">
         <is>
-          <t>TT07</t>
+          <t>TT05</t>
         </is>
       </c>
       <c r="E128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8076</t>
+          <t>VLINE-8075</t>
         </is>
       </c>
       <c r="F128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8185</t>
+          <t>VLINE-8183</t>
         </is>
       </c>
       <c r="G128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8434</t>
+          <t>VLINE-8432</t>
         </is>
       </c>
       <c r="H128" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8744</t>
+          <t>VLINE-8742</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>NR87</t>
+          <t>NR86</t>
         </is>
       </c>
       <c r="B129" s="1" t="inlineStr">
         <is>
-          <t>Q4005</t>
+          <t>Q4004</t>
         </is>
       </c>
       <c r="C129" s="1" t="inlineStr">
         <is>
-          <t>S3310</t>
+          <t>S3309</t>
         </is>
       </c>
       <c r="D129" s="1" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TT07</t>
         </is>
       </c>
       <c r="E129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8077</t>
+          <t>VLINE-8076</t>
         </is>
       </c>
       <c r="F129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8186</t>
+          <t>VLINE-8184</t>
         </is>
       </c>
       <c r="G129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8435</t>
+          <t>VLINE-8433</t>
         </is>
       </c>
       <c r="H129" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8745</t>
+          <t>VLINE-8743</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>NR88</t>
+          <t>NR87</t>
         </is>
       </c>
       <c r="B130" s="1" t="inlineStr">
         <is>
-          <t>Q4006</t>
+          <t>Q4005</t>
         </is>
       </c>
       <c r="C130" s="1" t="inlineStr">
         <is>
-          <t>S7001</t>
+          <t>S3310</t>
         </is>
       </c>
       <c r="D130" s="1" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TT08</t>
         </is>
       </c>
       <c r="E130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8080</t>
+          <t>VLINE-8077</t>
         </is>
       </c>
       <c r="F130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8187</t>
+          <t>VLINE-8185</t>
         </is>
       </c>
       <c r="G130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8438</t>
+          <t>VLINE-8434</t>
         </is>
       </c>
       <c r="H130" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8746</t>
+          <t>VLINE-8744</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>NR89</t>
+          <t>NR88</t>
         </is>
       </c>
       <c r="B131" s="1" t="inlineStr">
         <is>
-          <t>Q4007</t>
+          <t>Q4006</t>
         </is>
       </c>
       <c r="C131" s="1" t="inlineStr">
         <is>
-          <t>S7002</t>
+          <t>S7001</t>
         </is>
       </c>
       <c r="D131" s="1" t="inlineStr">
         <is>
-          <t>TT106</t>
+          <t>TT103</t>
         </is>
       </c>
       <c r="E131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8081</t>
+          <t>VLINE-8080</t>
         </is>
       </c>
       <c r="F131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8188</t>
+          <t>VLINE-8186</t>
         </is>
       </c>
       <c r="G131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8440</t>
+          <t>VLINE-8435</t>
         </is>
       </c>
       <c r="H131" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8747</t>
+          <t>VLINE-8745</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>NR90</t>
+          <t>NR89</t>
         </is>
       </c>
       <c r="B132" s="1" t="inlineStr">
         <is>
-          <t>Q4009</t>
+          <t>Q4007</t>
         </is>
       </c>
       <c r="C132" s="1" t="inlineStr">
         <is>
-          <t>S7003</t>
+          <t>S7002</t>
         </is>
       </c>
       <c r="D132" s="1" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TT106</t>
         </is>
       </c>
       <c r="E132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8084</t>
+          <t>VLINE-8081</t>
         </is>
       </c>
       <c r="F132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8189</t>
+          <t>VLINE-8187</t>
         </is>
       </c>
       <c r="G132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8441</t>
+          <t>VLINE-8438</t>
         </is>
       </c>
       <c r="H132" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8748</t>
+          <t>VLINE-8746</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>NR91</t>
+          <t>NR90</t>
         </is>
       </c>
       <c r="B133" s="1" t="inlineStr">
         <is>
-          <t>Q4011</t>
+          <t>Q4009</t>
         </is>
       </c>
       <c r="C133" s="1" t="inlineStr">
         <is>
-          <t>S7004</t>
+          <t>S7003</t>
         </is>
       </c>
       <c r="D133" s="1" t="inlineStr">
         <is>
-          <t>TT108</t>
+          <t>TT107</t>
         </is>
       </c>
       <c r="E133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8088</t>
+          <t>VLINE-8084</t>
         </is>
       </c>
       <c r="F133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8291</t>
+          <t>VLINE-8188</t>
         </is>
       </c>
       <c r="G133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8442</t>
+          <t>VLINE-8440</t>
         </is>
       </c>
       <c r="H133" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8749</t>
+          <t>VLINE-8747</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>NR92</t>
+          <t>NR91</t>
         </is>
       </c>
       <c r="B134" s="1" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>Q4011</t>
         </is>
       </c>
       <c r="C134" s="1" t="inlineStr">
         <is>
-          <t>S7005</t>
+          <t>S7004</t>
         </is>
       </c>
       <c r="D134" s="1" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TT108</t>
         </is>
       </c>
       <c r="E134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8089</t>
+          <t>VLINE-8088</t>
         </is>
       </c>
       <c r="F134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8293</t>
+          <t>VLINE-8189</t>
         </is>
       </c>
       <c r="G134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8443</t>
+          <t>VLINE-8441</t>
         </is>
       </c>
       <c r="H134" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8750</t>
+          <t>VLINE-8748</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR92</t>
         </is>
       </c>
       <c r="B135" s="1" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>Q4012</t>
         </is>
       </c>
       <c r="C135" s="1" t="inlineStr">
         <is>
-          <t>S7006</t>
+          <t>S7005</t>
         </is>
       </c>
       <c r="D135" s="1" t="inlineStr">
         <is>
-          <t>TT113</t>
+          <t>TT110</t>
         </is>
       </c>
       <c r="E135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8104</t>
+          <t>VLINE-8089</t>
         </is>
       </c>
       <c r="F135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8303</t>
+          <t>VLINE-8291</t>
         </is>
       </c>
       <c r="G135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8444</t>
+          <t>VLINE-8442</t>
         </is>
       </c>
       <c r="H135" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8751</t>
+          <t>VLINE-8749</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR93</t>
         </is>
       </c>
       <c r="B136" s="1" t="inlineStr">
         <is>
-          <t>Q4014</t>
+          <t>Q4013</t>
         </is>
       </c>
       <c r="C136" s="1" t="inlineStr">
         <is>
-          <t>S7007</t>
+          <t>S7006</t>
         </is>
       </c>
       <c r="D136" s="1" t="inlineStr">
         <is>
-          <t>TT114</t>
+          <t>TT113</t>
         </is>
       </c>
       <c r="E136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8107</t>
+          <t>VLINE-8104</t>
         </is>
       </c>
       <c r="F136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8304</t>
+          <t>VLINE-8293</t>
         </is>
       </c>
       <c r="G136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8446</t>
+          <t>VLINE-8443</t>
         </is>
       </c>
       <c r="H136" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8752</t>
+          <t>VLINE-8750</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR94</t>
         </is>
       </c>
       <c r="B137" s="1" t="inlineStr">
         <is>
-          <t>Q4015</t>
+          <t>Q4014</t>
         </is>
       </c>
       <c r="C137" s="1" t="inlineStr">
         <is>
-          <t>S7008</t>
+          <t>S7007</t>
         </is>
       </c>
       <c r="D137" s="1" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT114</t>
         </is>
       </c>
       <c r="E137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8110</t>
+          <t>VLINE-8107</t>
         </is>
       </c>
       <c r="F137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8306</t>
+          <t>VLINE-8303</t>
         </is>
       </c>
       <c r="G137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8447</t>
+          <t>VLINE-8444</t>
         </is>
       </c>
       <c r="H137" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8753</t>
+          <t>VLINE-8751</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>NR96</t>
+          <t>NR95</t>
         </is>
       </c>
       <c r="B138" s="1" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>Q4015</t>
         </is>
       </c>
       <c r="C138" s="1" t="inlineStr">
         <is>
-          <t>S7009</t>
+          <t>S7008</t>
         </is>
       </c>
       <c r="D138" s="1" t="inlineStr">
         <is>
-          <t>TT116</t>
+          <t>TT115</t>
         </is>
       </c>
       <c r="E138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8111</t>
+          <t>VLINE-8110</t>
         </is>
       </c>
       <c r="F138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8311</t>
+          <t>VLINE-8304</t>
         </is>
       </c>
       <c r="G138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8449</t>
+          <t>VLINE-8446</t>
         </is>
       </c>
       <c r="H138" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8754</t>
+          <t>VLINE-8752</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>NR96</t>
         </is>
       </c>
       <c r="B139" s="1" t="inlineStr">
         <is>
-          <t>Q4017</t>
+          <t>Q4016</t>
         </is>
       </c>
       <c r="C139" s="1" t="inlineStr">
         <is>
-          <t>S7012</t>
+          <t>S7009</t>
         </is>
       </c>
       <c r="D139" s="1" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT116</t>
         </is>
       </c>
       <c r="E139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8113</t>
+          <t>VLINE-8111</t>
         </is>
       </c>
       <c r="F139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8313</t>
+          <t>VLINE-8306</t>
         </is>
       </c>
       <c r="G139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8450</t>
+          <t>VLINE-8447</t>
         </is>
       </c>
       <c r="H139" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8755</t>
+          <t>VLINE-8753</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>NR98</t>
+          <t>NR97</t>
         </is>
       </c>
       <c r="B140" s="1" t="inlineStr">
         <is>
-          <t>Q4019</t>
+          <t>Q4017</t>
         </is>
       </c>
       <c r="C140" s="1" t="inlineStr">
         <is>
-          <t>S7013</t>
+          <t>S7012</t>
         </is>
       </c>
       <c r="D140" s="1" t="inlineStr">
         <is>
-          <t>TT122</t>
+          <t>TT117</t>
         </is>
       </c>
       <c r="E140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8114</t>
+          <t>VLINE-8113</t>
         </is>
       </c>
       <c r="F140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8314</t>
+          <t>VLINE-8311</t>
         </is>
       </c>
       <c r="G140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8451</t>
+          <t>VLINE-8449</t>
         </is>
       </c>
       <c r="H140" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8756</t>
+          <t>VLINE-8754</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>NR99</t>
+          <t>NR98</t>
         </is>
       </c>
       <c r="B141" s="1" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>Q4019</t>
         </is>
       </c>
       <c r="C141" s="1" t="inlineStr">
         <is>
-          <t>S7014</t>
+          <t>S7013</t>
         </is>
       </c>
       <c r="D141" s="1" t="inlineStr">
         <is>
-          <t>TT127</t>
+          <t>TT122</t>
         </is>
       </c>
       <c r="E141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8115</t>
+          <t>VLINE-8114</t>
         </is>
       </c>
       <c r="F141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8316</t>
+          <t>VLINE-8313</t>
         </is>
       </c>
       <c r="G141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8452</t>
+          <t>VLINE-8450</t>
         </is>
       </c>
       <c r="H141" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8757</t>
+          <t>VLINE-8755</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>NR101</t>
+          <t>NR99</t>
         </is>
       </c>
       <c r="B142" s="1" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>QBX003</t>
         </is>
       </c>
       <c r="C142" s="1" t="inlineStr">
         <is>
-          <t>S7015</t>
+          <t>S7014</t>
         </is>
       </c>
       <c r="D142" s="1" t="inlineStr">
         <is>
-          <t>TT128</t>
+          <t>TT127</t>
         </is>
       </c>
       <c r="E142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8119</t>
+          <t>VLINE-8115</t>
         </is>
       </c>
       <c r="F142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8318</t>
+          <t>VLINE-8314</t>
         </is>
       </c>
       <c r="G142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8453</t>
+          <t>VLINE-8451</t>
         </is>
       </c>
       <c r="H142" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8758</t>
+          <t>VLINE-8756</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR101</t>
         </is>
       </c>
       <c r="B143" s="1" t="inlineStr">
         <is>
-          <t>QBX005</t>
+          <t>QBX004</t>
         </is>
       </c>
       <c r="C143" s="1" t="inlineStr">
         <is>
-          <t>S7017</t>
+          <t>S7015</t>
         </is>
       </c>
       <c r="D143" s="1" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT128</t>
         </is>
       </c>
       <c r="E143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8120</t>
+          <t>VLINE-8119</t>
         </is>
       </c>
       <c r="F143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8321</t>
+          <t>VLINE-8316</t>
         </is>
       </c>
       <c r="G143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8454</t>
+          <t>VLINE-8452</t>
         </is>
       </c>
       <c r="H143" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8759</t>
+          <t>VLINE-8757</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>NR103</t>
+          <t>NR102</t>
         </is>
       </c>
       <c r="B144" s="1" t="inlineStr">
         <is>
-          <t>QBX006</t>
+          <t>QBX005</t>
         </is>
       </c>
       <c r="C144" s="1" t="inlineStr">
         <is>
-          <t>S7018</t>
+          <t>S7017</t>
         </is>
       </c>
       <c r="D144" s="1" t="inlineStr">
         <is>
-          <t>TT131</t>
+          <t>TT130</t>
         </is>
       </c>
       <c r="E144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8121</t>
+          <t>VLINE-8120</t>
         </is>
       </c>
       <c r="F144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8323</t>
+          <t>VLINE-8318</t>
         </is>
       </c>
       <c r="G144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8455</t>
+          <t>VLINE-8453</t>
         </is>
       </c>
       <c r="H144" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8760</t>
+          <t>VLINE-8758</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>NR105</t>
+          <t>NR103</t>
         </is>
       </c>
       <c r="B145" s="1" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>QBX006</t>
         </is>
       </c>
       <c r="C145" s="1" t="inlineStr">
         <is>
-          <t>S7020</t>
+          <t>S7018</t>
         </is>
       </c>
       <c r="D145" s="1" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT131</t>
         </is>
       </c>
       <c r="E145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8123</t>
+          <t>VLINE-8121</t>
         </is>
       </c>
       <c r="F145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8324</t>
+          <t>VLINE-8321</t>
         </is>
       </c>
       <c r="G145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8456</t>
+          <t>VLINE-8454</t>
         </is>
       </c>
       <c r="H145" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8761</t>
+          <t>VLINE-8759</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>NR106</t>
+          <t>NR105</t>
         </is>
       </c>
       <c r="B146" s="1" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>QE001</t>
         </is>
       </c>
       <c r="C146" s="1" t="inlineStr">
         <is>
-          <t>S7022</t>
+          <t>S7020</t>
         </is>
       </c>
       <c r="D146" s="1" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT202</t>
         </is>
       </c>
       <c r="E146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8124</t>
+          <t>VLINE-8123</t>
         </is>
       </c>
       <c r="F146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8325</t>
+          <t>VLINE-8323</t>
         </is>
       </c>
       <c r="G146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8457</t>
+          <t>VLINE-8455</t>
         </is>
       </c>
       <c r="H146" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8762</t>
+          <t>VLINE-8760</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>NR107</t>
+          <t>NR106</t>
         </is>
       </c>
       <c r="B147" s="1" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>QE002</t>
         </is>
       </c>
       <c r="C147" s="1" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>S7022</t>
         </is>
       </c>
       <c r="D147" s="1" t="inlineStr">
         <is>
-          <t>VL352</t>
+          <t>TT206</t>
         </is>
       </c>
       <c r="E147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8126</t>
+          <t>VLINE-8124</t>
         </is>
       </c>
       <c r="F147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8328</t>
+          <t>VLINE-8324</t>
         </is>
       </c>
       <c r="G147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8460</t>
+          <t>VLINE-8456</t>
         </is>
       </c>
       <c r="H147" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8763</t>
+          <t>VLINE-8761</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>NR108</t>
+          <t>NR107</t>
         </is>
       </c>
       <c r="B148" s="1" t="inlineStr">
         <is>
-          <t>QE004</t>
+          <t>QE003</t>
         </is>
       </c>
       <c r="C148" s="1" t="inlineStr">
         <is>
-          <t>SCT002</t>
+          <t>SCT001</t>
         </is>
       </c>
       <c r="D148" s="1" t="inlineStr">
         <is>
-          <t>VL353</t>
+          <t>VL352</t>
         </is>
       </c>
       <c r="E148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8127</t>
+          <t>VLINE-8126</t>
         </is>
       </c>
       <c r="F148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8329</t>
+          <t>VLINE-8325</t>
         </is>
       </c>
       <c r="G148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8461</t>
+          <t>VLINE-8457</t>
         </is>
       </c>
       <c r="H148" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8764</t>
+          <t>VLINE-8762</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR108</t>
         </is>
       </c>
       <c r="B149" s="1" t="inlineStr">
         <is>
-          <t>QE006</t>
+          <t>QE004</t>
         </is>
       </c>
       <c r="C149" s="1" t="inlineStr">
         <is>
-          <t>SCT006</t>
+          <t>SCT002</t>
         </is>
       </c>
       <c r="D149" s="1" t="inlineStr">
         <is>
-          <t>VL357</t>
+          <t>VL353</t>
         </is>
       </c>
       <c r="E149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8128</t>
+          <t>VLINE-8127</t>
         </is>
       </c>
       <c r="F149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8332</t>
+          <t>VLINE-8328</t>
         </is>
       </c>
       <c r="G149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8464</t>
+          <t>VLINE-8460</t>
         </is>
       </c>
       <c r="H149" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8765</t>
+          <t>VLINE-8763</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>NR110</t>
+          <t>NR109</t>
         </is>
       </c>
       <c r="B150" s="1" t="inlineStr">
         <is>
-          <t>QL001</t>
+          <t>QE006</t>
         </is>
       </c>
       <c r="C150" s="1" t="inlineStr">
         <is>
-          <t>SCT007</t>
+          <t>SCT006</t>
         </is>
       </c>
       <c r="D150" s="1" t="inlineStr">
         <is>
-          <t>VL359</t>
+          <t>VL357</t>
         </is>
       </c>
       <c r="E150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8129</t>
+          <t>VLINE-8128</t>
         </is>
       </c>
       <c r="F150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8336</t>
+          <t>VLINE-8329</t>
         </is>
       </c>
       <c r="G150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8465</t>
+          <t>VLINE-8461</t>
         </is>
       </c>
       <c r="H150" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8766</t>
+          <t>VLINE-8764</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>NR111</t>
+          <t>NR110</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
         <is>
-          <t>QL002</t>
+          <t>QL001</t>
         </is>
       </c>
       <c r="C151" s="1" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>SCT007</t>
         </is>
       </c>
       <c r="D151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8004</t>
+          <t>VL359</t>
         </is>
       </c>
       <c r="E151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8131</t>
+          <t>VLINE-8129</t>
         </is>
       </c>
       <c r="F151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8337</t>
+          <t>VLINE-8332</t>
         </is>
       </c>
       <c r="G151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8468</t>
+          <t>VLINE-8464</t>
         </is>
       </c>
       <c r="H151" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8767</t>
+          <t>VLINE-8765</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR111</t>
         </is>
       </c>
       <c r="B152" s="1" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>QL002</t>
         </is>
       </c>
       <c r="C152" s="1" t="inlineStr">
         <is>
-          <t>SCT011</t>
+          <t>SCT009</t>
         </is>
       </c>
       <c r="D152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8007</t>
+          <t>VLINE-8004</t>
         </is>
       </c>
       <c r="E152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8132</t>
+          <t>VLINE-8131</t>
         </is>
       </c>
       <c r="F152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8338</t>
+          <t>VLINE-8336</t>
         </is>
       </c>
       <c r="G152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8469</t>
+          <t>VLINE-8465</t>
         </is>
       </c>
       <c r="H152" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8768</t>
+          <t>VLINE-8766</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR112</t>
         </is>
       </c>
       <c r="B153" s="1" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>QL004</t>
         </is>
       </c>
       <c r="C153" s="1" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>SCT011</t>
         </is>
       </c>
       <c r="D153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8011</t>
+          <t>VLINE-8007</t>
         </is>
       </c>
       <c r="E153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8133</t>
+          <t>VLINE-8132</t>
         </is>
       </c>
       <c r="F153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8339</t>
+          <t>VLINE-8337</t>
         </is>
       </c>
       <c r="G153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8605</t>
+          <t>VLINE-8468</t>
         </is>
       </c>
       <c r="H153" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8769</t>
+          <t>VLINE-8767</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR113</t>
         </is>
       </c>
       <c r="B154" s="1" t="inlineStr">
         <is>
-          <t>QL008</t>
+          <t>QL007</t>
         </is>
       </c>
       <c r="C154" s="1" t="inlineStr">
         <is>
-          <t>SCT014</t>
+          <t>SCT013</t>
         </is>
       </c>
       <c r="D154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8013</t>
+          <t>VLINE-8011</t>
         </is>
       </c>
       <c r="E154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8134</t>
+          <t>VLINE-8133</t>
         </is>
       </c>
       <c r="F154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8362</t>
+          <t>VLINE-8338</t>
         </is>
       </c>
       <c r="G154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8610</t>
+          <t>VLINE-8469</t>
         </is>
       </c>
       <c r="H154" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8770</t>
+          <t>VLINE-8768</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>NR118</t>
+          <t>NR115</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
         <is>
-          <t>QL010</t>
+          <t>QL008</t>
         </is>
       </c>
       <c r="C155" s="1" t="inlineStr">
         <is>
-          <t>SCT015</t>
+          <t>SCT014</t>
         </is>
       </c>
       <c r="D155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8019</t>
+          <t>VLINE-8013</t>
         </is>
       </c>
       <c r="E155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8136</t>
+          <t>VLINE-8134</t>
         </is>
       </c>
       <c r="F155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8363</t>
+          <t>VLINE-8339</t>
         </is>
       </c>
       <c r="G155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8612</t>
+          <t>VLINE-8605</t>
         </is>
       </c>
       <c r="H155" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8772</t>
+          <t>VLINE-8769</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>NR119</t>
+          <t>NR118</t>
         </is>
       </c>
       <c r="B156" s="1" t="inlineStr">
         <is>
-          <t>QL011</t>
+          <t>QL010</t>
         </is>
       </c>
       <c r="C156" s="1" t="inlineStr">
         <is>
-          <t>SO2</t>
+          <t>SCT015</t>
         </is>
       </c>
       <c r="D156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8020</t>
+          <t>VLINE-8019</t>
         </is>
       </c>
       <c r="E156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8137</t>
+          <t>VLINE-8136</t>
         </is>
       </c>
       <c r="F156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8365</t>
+          <t>VLINE-8362</t>
         </is>
       </c>
       <c r="G156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8615</t>
+          <t>VLINE-8610</t>
         </is>
       </c>
       <c r="H156" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8773</t>
+          <t>VLINE-8770</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>NR120</t>
+          <t>NR119</t>
         </is>
       </c>
       <c r="B157" s="1" t="inlineStr">
         <is>
-          <t>QL012</t>
+          <t>QL011</t>
         </is>
       </c>
       <c r="C157" s="1" t="inlineStr">
         <is>
-          <t>SO3</t>
+          <t>SO2</t>
         </is>
       </c>
       <c r="D157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8023</t>
+          <t>VLINE-8020</t>
         </is>
       </c>
       <c r="E157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8140</t>
+          <t>VLINE-8137</t>
         </is>
       </c>
       <c r="F157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8366</t>
+          <t>VLINE-8363</t>
         </is>
       </c>
       <c r="G157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8617</t>
+          <t>VLINE-8612</t>
         </is>
       </c>
       <c r="H157" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8774</t>
+          <t>VLINE-8772</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>NR121</t>
+          <t>NR120</t>
         </is>
       </c>
       <c r="B158" s="1" t="inlineStr">
         <is>
-          <t>QL014</t>
+          <t>QL012</t>
         </is>
       </c>
       <c r="C158" s="1" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>SO3</t>
         </is>
       </c>
       <c r="D158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8025</t>
+          <t>VLINE-8023</t>
         </is>
       </c>
       <c r="E158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8141</t>
+          <t>VLINE-8140</t>
         </is>
       </c>
       <c r="F158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8368</t>
+          <t>VLINE-8365</t>
         </is>
       </c>
       <c r="G158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8620</t>
+          <t>VLINE-8615</t>
         </is>
       </c>
       <c r="H158" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8776</t>
+          <t>VLINE-8773</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>NR122</t>
+          <t>NR121</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
         <is>
-          <t>QL017</t>
+          <t>QL014</t>
         </is>
       </c>
       <c r="C159" s="1" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>SSR101</t>
         </is>
       </c>
       <c r="D159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8026</t>
+          <t>VLINE-8025</t>
         </is>
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8142</t>
+          <t>VLINE-8141</t>
         </is>
       </c>
       <c r="F159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8369</t>
+          <t>VLINE-8366</t>
         </is>
       </c>
       <c r="G159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8625</t>
+          <t>VLINE-8617</t>
         </is>
       </c>
       <c r="H159" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8778</t>
+          <t>VLINE-8774</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t>P14</t>
+          <t>NR122</t>
         </is>
       </c>
       <c r="B160" s="1" t="inlineStr">
         <is>
-          <t>QL018</t>
+          <t>QL017</t>
         </is>
       </c>
       <c r="C160" s="1" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>SSR102</t>
         </is>
       </c>
       <c r="D160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8027</t>
+          <t>VLINE-8026</t>
         </is>
       </c>
       <c r="E160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8144</t>
+          <t>VLINE-8142</t>
         </is>
       </c>
       <c r="F160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8403</t>
+          <t>VLINE-8368</t>
         </is>
       </c>
       <c r="G160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8630</t>
+          <t>VLINE-8620</t>
         </is>
       </c>
       <c r="H160" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8779</t>
+          <t>VLINE-8776</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>P16</t>
+          <t>P14</t>
         </is>
       </c>
       <c r="B161" s="1" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QL018</t>
         </is>
       </c>
       <c r="C161" s="1" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>SSR103</t>
         </is>
       </c>
       <c r="D161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8028</t>
+          <t>VLINE-8027</t>
         </is>
       </c>
       <c r="E161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8145</t>
+          <t>VLINE-8144</t>
         </is>
       </c>
       <c r="F161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8404</t>
+          <t>VLINE-8369</t>
         </is>
       </c>
       <c r="G161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8671</t>
+          <t>VLINE-8625</t>
         </is>
       </c>
       <c r="H161" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8780</t>
+          <t>VLINE-8778</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>P2501</t>
+          <t>P16</t>
         </is>
       </c>
       <c r="B162" s="1" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QR1744</t>
         </is>
       </c>
       <c r="C162" s="1" t="inlineStr">
         <is>
-          <t>T363</t>
+          <t>SSR104</t>
         </is>
       </c>
       <c r="D162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8029</t>
+          <t>VLINE-8028</t>
         </is>
       </c>
       <c r="E162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8148</t>
+          <t>VLINE-8145</t>
         </is>
       </c>
       <c r="F162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8406</t>
+          <t>VLINE-8403</t>
         </is>
       </c>
       <c r="G162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8706</t>
+          <t>VLINE-8630</t>
         </is>
       </c>
       <c r="H162" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8781</t>
+          <t>VLINE-8779</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>P2502</t>
+          <t>P2501</t>
         </is>
       </c>
       <c r="B163" s="1" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QR1771</t>
         </is>
       </c>
       <c r="C163" s="1" t="inlineStr">
         <is>
-          <t>T381</t>
+          <t>T363</t>
         </is>
       </c>
       <c r="D163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8030</t>
+          <t>VLINE-8029</t>
         </is>
       </c>
       <c r="E163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8150</t>
+          <t>VLINE-8148</t>
         </is>
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8408</t>
+          <t>VLINE-8404</t>
         </is>
       </c>
       <c r="G163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8711</t>
+          <t>VLINE-8671</t>
         </is>
       </c>
       <c r="H163" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8782</t>
+          <t>VLINE-8780</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>P2503</t>
+          <t>P2502</t>
         </is>
       </c>
       <c r="B164" s="1" t="inlineStr">
         <is>
-          <t>R711</t>
+          <t>QR5404</t>
         </is>
       </c>
       <c r="C164" s="1" t="inlineStr">
         <is>
-          <t>T386</t>
+          <t>T381</t>
         </is>
       </c>
       <c r="D164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8031</t>
+          <t>VLINE-8030</t>
         </is>
       </c>
       <c r="E164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8151</t>
+          <t>VLINE-8150</t>
         </is>
       </c>
       <c r="F164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8410</t>
+          <t>VLINE-8406</t>
         </is>
       </c>
       <c r="G164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8714</t>
+          <t>VLINE-8706</t>
         </is>
       </c>
       <c r="H164" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8783</t>
+          <t>VLINE-8781</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>P2504</t>
+          <t>P2503</t>
         </is>
       </c>
       <c r="B165" s="1" t="inlineStr">
         <is>
-          <t>R766</t>
+          <t>R711</t>
         </is>
       </c>
       <c r="C165" s="1" t="inlineStr">
         <is>
-          <t>TDX101</t>
+          <t>T386</t>
         </is>
       </c>
       <c r="D165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8032</t>
+          <t>VLINE-8031</t>
         </is>
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8152</t>
+          <t>VLINE-8151</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8411</t>
+          <t>VLINE-8408</t>
         </is>
       </c>
       <c r="G165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8717</t>
+          <t>VLINE-8711</t>
         </is>
       </c>
       <c r="H165" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8784</t>
+          <t>VLINE-8782</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>P2505</t>
+          <t>P2504</t>
         </is>
       </c>
       <c r="B166" s="1" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>R766</t>
         </is>
       </c>
       <c r="C166" s="1" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>TDX101</t>
         </is>
       </c>
       <c r="D166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8036</t>
+          <t>VLINE-8032</t>
         </is>
       </c>
       <c r="E166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8153</t>
+          <t>VLINE-8152</t>
         </is>
       </c>
       <c r="F166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8413</t>
+          <t>VLINE-8410</t>
         </is>
       </c>
       <c r="G166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8720</t>
+          <t>VLINE-8714</t>
         </is>
       </c>
       <c r="H166" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8786</t>
+          <t>VLINE-8783</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>P2506</t>
+          <t>P2505</t>
         </is>
       </c>
       <c r="B167" s="1" t="inlineStr">
         <is>
-          <t>RCTST4</t>
+          <t>RB2353</t>
         </is>
       </c>
       <c r="C167" s="1" t="inlineStr">
         <is>
-          <t>TE2802</t>
+          <t>TE2801</t>
         </is>
       </c>
       <c r="D167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8038</t>
+          <t>VLINE-8036</t>
         </is>
       </c>
       <c r="E167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8154</t>
+          <t>VLINE-8153</t>
         </is>
       </c>
       <c r="F167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8415</t>
+          <t>VLINE-8411</t>
         </is>
       </c>
       <c r="G167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8721</t>
+          <t>VLINE-8717</t>
         </is>
       </c>
       <c r="H167" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8787</t>
+          <t>VLINE-8784</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>P2507</t>
+          <t>P2506</t>
         </is>
       </c>
       <c r="B168" s="1" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>RCTST4</t>
         </is>
       </c>
       <c r="C168" s="1" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>TE2802</t>
         </is>
       </c>
       <c r="D168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8039</t>
+          <t>VLINE-8038</t>
         </is>
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8155</t>
+          <t>VLINE-8154</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8417</t>
+          <t>VLINE-8413</t>
         </is>
       </c>
       <c r="G168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8723</t>
+          <t>VLINE-8720</t>
         </is>
       </c>
       <c r="H168" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8788</t>
+          <t>VLINE-8786</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>P2508</t>
+          <t>P2507</t>
         </is>
       </c>
       <c r="B169" s="1" t="inlineStr">
         <is>
-          <t>RL302</t>
+          <t>RL301</t>
         </is>
       </c>
       <c r="C169" s="1" t="inlineStr">
         <is>
-          <t>TE2804</t>
+          <t>TE2803</t>
         </is>
       </c>
       <c r="D169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8042</t>
+          <t>VLINE-8039</t>
         </is>
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8157</t>
+          <t>VLINE-8155</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8418</t>
+          <t>VLINE-8415</t>
         </is>
       </c>
       <c r="G169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8725</t>
+          <t>VLINE-8721</t>
         </is>
       </c>
       <c r="H169" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8790</t>
+          <t>VLINE-8787</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>P2509</t>
+          <t>P2508</t>
         </is>
       </c>
       <c r="B170" s="1" t="inlineStr">
         <is>
-          <t>RL304</t>
+          <t>RL302</t>
         </is>
       </c>
       <c r="C170" s="1" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>TE2804</t>
         </is>
       </c>
       <c r="D170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8049</t>
+          <t>VLINE-8042</t>
         </is>
       </c>
       <c r="E170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8158</t>
+          <t>VLINE-8157</t>
         </is>
       </c>
       <c r="F170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8419</t>
+          <t>VLINE-8417</t>
         </is>
       </c>
       <c r="G170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8726</t>
+          <t>VLINE-8723</t>
         </is>
       </c>
       <c r="H170" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8792</t>
+          <t>VLINE-8788</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8793</t>
+          <t>VLINE-8790</t>
         </is>
       </c>
       <c r="B172" s="1" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>XP2008</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8794</t>
+          <t>VLINE-8792</t>
         </is>
       </c>
       <c r="B173" s="1" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>XP2010</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8795</t>
+          <t>VLINE-8793</t>
         </is>
       </c>
       <c r="B174" s="1" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>XP2011</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8796</t>
+          <t>VLINE-8794</t>
         </is>
       </c>
       <c r="B175" s="1" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>XP2012</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8797</t>
+          <t>VLINE-8795</t>
         </is>
       </c>
       <c r="B176" s="1" t="inlineStr">
         <is>
-          <t>XP2016</t>
+          <t>XP2013</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8799</t>
+          <t>VLINE-8796</t>
         </is>
       </c>
       <c r="B177" s="1" t="inlineStr">
         <is>
-          <t>XP2017</t>
+          <t>XP2014</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8800</t>
+          <t>VLINE-8797</t>
         </is>
       </c>
       <c r="B178" s="1" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>XP2015</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8801</t>
+          <t>VLINE-8799</t>
         </is>
       </c>
       <c r="B179" s="1" t="inlineStr">
         <is>
-          <t>XR550</t>
+          <t>XP2016</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8802</t>
+          <t>VLINE-8800</t>
         </is>
       </c>
       <c r="B180" s="1" t="inlineStr">
         <is>
-          <t>XR552</t>
+          <t>XP2017</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8803</t>
+          <t>VLINE-8801</t>
         </is>
       </c>
       <c r="B181" s="1" t="inlineStr">
         <is>
-          <t>XR559</t>
+          <t>XP2019</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8804</t>
+          <t>VLINE-8802</t>
         </is>
       </c>
       <c r="B182" s="1" t="inlineStr">
         <is>
-          <t>XRN001</t>
+          <t>XR550</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8805</t>
+          <t>VLINE-8803</t>
         </is>
       </c>
       <c r="B183" s="1" t="inlineStr">
         <is>
-          <t>XRN004</t>
+          <t>XR552</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8806</t>
+          <t>VLINE-8804</t>
         </is>
       </c>
       <c r="B184" s="1" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>XR559</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8807</t>
+          <t>VLINE-8805</t>
         </is>
       </c>
       <c r="B185" s="1" t="inlineStr">
         <is>
-          <t>XRN006</t>
+          <t>XRN001</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8808</t>
+          <t>VLINE-8806</t>
         </is>
       </c>
       <c r="B186" s="1" t="inlineStr">
         <is>
-          <t>XRN007</t>
+          <t>XRN004</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8809</t>
+          <t>VLINE-8807</t>
         </is>
       </c>
       <c r="B187" s="1" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>XRN005</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8810</t>
+          <t>VLINE-8808</t>
         </is>
       </c>
       <c r="B188" s="1" t="inlineStr">
         <is>
-          <t>XRN011</t>
+          <t>XRN006</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8811</t>
+          <t>VLINE-8809</t>
         </is>
       </c>
       <c r="B189" s="1" t="inlineStr">
         <is>
-          <t>XRN014</t>
+          <t>XRN007</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8812</t>
+          <t>VLINE-8810</t>
         </is>
       </c>
       <c r="B190" s="1" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>XRN009</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8813</t>
+          <t>VLINE-8811</t>
         </is>
       </c>
       <c r="B191" s="1" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>XRN011</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8814</t>
+          <t>VLINE-8812</t>
         </is>
       </c>
       <c r="B192" s="1" t="inlineStr">
         <is>
-          <t>XRN020</t>
+          <t>XRN014</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8815</t>
+          <t>VLINE-8813</t>
         </is>
       </c>
       <c r="B193" s="1" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>XRN017</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8816</t>
+          <t>VLINE-8814</t>
         </is>
       </c>
       <c r="B194" s="1" t="inlineStr">
         <is>
-          <t>XRN023</t>
+          <t>XRN018</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8817</t>
+          <t>VLINE-8815</t>
         </is>
       </c>
       <c r="B195" s="1" t="inlineStr">
         <is>
-          <t>XRN025</t>
+          <t>XRN020</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8818</t>
+          <t>VLINE-8816</t>
         </is>
       </c>
       <c r="B196" s="1" t="inlineStr">
         <is>
-          <t>XRN026</t>
+          <t>XRN021</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8819</t>
+          <t>VLINE-8817</t>
         </is>
       </c>
       <c r="B197" s="1" t="inlineStr">
         <is>
-          <t>XRN027</t>
+          <t>XRN023</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8820</t>
+          <t>VLINE-8818</t>
         </is>
       </c>
       <c r="B198" s="1" t="inlineStr">
         <is>
-          <t>XRN029</t>
+          <t>XRN025</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8822</t>
+          <t>VLINE-8819</t>
         </is>
       </c>
       <c r="B199" s="1" t="inlineStr">
         <is>
-          <t>Y163</t>
+          <t>XRN026</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8860</t>
+          <t>VLINE-8820</t>
+        </is>
+      </c>
+      <c r="B200" s="1" t="inlineStr">
+        <is>
+          <t>XRN027</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8861</t>
+          <t>VLINE-8821</t>
+        </is>
+      </c>
+      <c r="B201" s="1" t="inlineStr">
+        <is>
+          <t>XRN029</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8862</t>
+          <t>VLINE-8822</t>
+        </is>
+      </c>
+      <c r="B202" s="1" t="inlineStr">
+        <is>
+          <t>Y163</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8863</t>
+          <t>VLINE-8860</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8864</t>
+          <t>VLINE-8861</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8865</t>
+          <t>VLINE-8862</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8866</t>
+          <t>VLINE-8863</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8867</t>
+          <t>VLINE-8864</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8868</t>
+          <t>VLINE-8865</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8869</t>
+          <t>VLINE-8866</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8890</t>
+          <t>VLINE-8867</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8891</t>
+          <t>VLINE-8868</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8893</t>
+          <t>VLINE-8869</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>VLINE-8895</t>
+          <t>VLINE-8890</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>WH001</t>
+          <t>VLINE-8891</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>WH003</t>
+          <t>VLINE-8893</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>WL02</t>
+          <t>VLINE-8895</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>X12-X14</t>
+          <t>WH001</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>X31</t>
+          <t>WH003</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>XP2000</t>
+          <t>WL02</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>XP2001</t>
+          <t>X12-X14</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>XP2003</t>
+          <t>X31</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>XP2004</t>
+          <t>XP2000</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>XP2001</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>XP2007</t>
+          <t>XP2003</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>XP2004</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>XP2010</t>
+          <t>XP2005</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>XP2007</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update RailOps database files - 2026-04-29 17:31:31 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A213"/>
+  <dimension ref="A1:A250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -461,1484 +461,1743 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ACB4404</t>
+          <t>ACB4403</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ACD6047</t>
+          <t>ACB4404</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ACD6052</t>
+          <t>ACD6047</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ACD6056</t>
+          <t>ACD6049</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ACD6057</t>
+          <t>ACD6052</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ACD6058</t>
+          <t>ACD6056</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ACD6059</t>
+          <t>ACD6057</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>ACD6065</t>
+          <t>ACD6058</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ACD6066</t>
+          <t>ACD6059</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>ACD6069</t>
+          <t>ACD6065</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ACD6071</t>
+          <t>ACD6066</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>ACD6074</t>
+          <t>ACD6069</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>C502</t>
+          <t>ACD6071</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>C509</t>
+          <t>ACD6074</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>CEY004</t>
+          <t>BL33</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>CEY006</t>
+          <t>C502</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>CEY007</t>
+          <t>C509</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>CF4401</t>
+          <t>CEY004</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>CF4405</t>
+          <t>CEY006</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>CF4410</t>
+          <t>CEY007</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>CF4421</t>
+          <t>CF4401</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>CF4424</t>
+          <t>CF4405</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>CF4425</t>
+          <t>CF4410</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>CF4427</t>
+          <t>CF4421</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>CLP12</t>
+          <t>CF4424</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>CLP13</t>
+          <t>CF4425</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>CSR010</t>
+          <t>CF4427</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>CSR015</t>
+          <t>CF4429</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>CSR019</t>
+          <t>CLP12</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>CSR020</t>
+          <t>CLP13</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>CSR021</t>
+          <t>CSR010</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>EA2503</t>
+          <t>CSR015</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>FIE001</t>
+          <t>CSR019</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>G513</t>
+          <t>CSR020</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>G514</t>
+          <t>CSR021</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>G516</t>
+          <t>CSR023</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>G534</t>
+          <t>DS003</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>GL103</t>
+          <t>EA2503</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>GL105</t>
+          <t>FIE001</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>GL111</t>
+          <t>G513</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>GWA002</t>
+          <t>G514</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>GWA004</t>
+          <t>G516</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>GWA008</t>
+          <t>G533</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>GWA009</t>
+          <t>G534</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>GWB103</t>
+          <t>G536</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>GWU008</t>
+          <t>GL103</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>GWU014</t>
+          <t>GL105</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>HM2701</t>
+          <t>GL111</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>HM2702</t>
+          <t>GWA002</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>LDP002</t>
+          <t>GWA004</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>LDP008</t>
+          <t>GWA008</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>LE2853</t>
+          <t>GWA009</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>M437</t>
+          <t>GWB103</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>M865</t>
+          <t>GWB104</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>MAN004</t>
+          <t>GWU008</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>MAN007</t>
+          <t>GWU014</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>MAN013</t>
+          <t>HM2701</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>MAN015</t>
+          <t>HM2702</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>MAN017</t>
+          <t>HM2705</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>MM76M</t>
+          <t>HM2755</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>MM82M</t>
+          <t>HM2756</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>MM152M</t>
+          <t>LDP002</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>MM158M</t>
+          <t>LDP004</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>MM172M</t>
+          <t>LDP008</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>MM232M</t>
+          <t>LE2853</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>MM260M</t>
+          <t>LZ3114</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>MM280M</t>
+          <t>M437</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>MM502M</t>
+          <t>M865</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>MM522M</t>
+          <t>MAN004</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>MM624M</t>
+          <t>MAN007</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>MM674M</t>
+          <t>MAN013</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>MM718M</t>
+          <t>MAN015</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>MM810M</t>
+          <t>MAN017</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>MM830M</t>
+          <t>MM76M</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>MM834M</t>
+          <t>MM82M</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>MM838M</t>
+          <t>MM152M</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>MM914M</t>
+          <t>MM158M</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>MM928M</t>
+          <t>MM172M</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>MM934M</t>
+          <t>MM232M</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>MM946M</t>
+          <t>MM260M</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>MM962M</t>
+          <t>MM280M</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>MM982M</t>
+          <t>MM502M</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>MM9914M</t>
+          <t>MM522M</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>MM9924M</t>
+          <t>MM624M</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>MM9946M</t>
+          <t>MM674M</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>MM9965M</t>
+          <t>MM718M</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>MM9966M</t>
+          <t>MM810M</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>MM9970M</t>
+          <t>MM830M</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MM834M</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>MM838M</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>MM914M</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>NR6</t>
+          <t>MM928M</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>NR10</t>
+          <t>MM934M</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>NR11</t>
+          <t>MM946M</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>NR13</t>
+          <t>MM962M</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>NR14</t>
+          <t>MM982M</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>NR20</t>
+          <t>MM9914M</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>NR35</t>
+          <t>MM9924M</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>MM9927M</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>NR46</t>
+          <t>MM9946M</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>MM9965M</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>MM9966M</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>MM9970M</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>MRL001</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR4</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR5</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR6</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR10</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>NR11</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR13</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>NR107</t>
+          <t>NR14</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR20</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR35</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR37</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR46</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>NR47</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>PKLA4</t>
+          <t>NR64</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>NR65</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>NR75</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>NR78</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>NR93</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>NR94</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>NR95</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>QL009</t>
+          <t>NR97</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>QL019</t>
+          <t>NR102</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>QR5400</t>
+          <t>NR107</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>NR109</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>RA2303</t>
+          <t>NR112</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>NR113</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>SCT008</t>
+          <t>NR115</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>PKLA4</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>T373</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>TT123</t>
+          <t>QL009</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>TT126</t>
+          <t>QL019</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>TT129</t>
+          <t>QR5400</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>RA2303</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>VL22</t>
+          <t>SCT001</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>VL57</t>
+          <t>SCT008</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>VLINE8058</t>
+          <t>SCT009</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>VLINE8059</t>
+          <t>SSR102</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>VLINE8061</t>
+          <t>SSR103</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>VLINE8161</t>
+          <t>T373</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>VLINE8163</t>
+          <t>TE2803</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>VLINE8164</t>
+          <t>TE2805</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>VLINE8457</t>
+          <t>TJ096</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>VLINE8459</t>
+          <t>TT02</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>VLINE8819</t>
+          <t>TT03</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>XP2001</t>
+          <t>TT08</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>TT103</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>XP2006</t>
+          <t>TT105</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>TT107</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>TT110</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>TT115</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>TT117</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>TT123</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>XRN022</t>
+          <t>TT126</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>XRN028</t>
+          <t>TT129</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>1102</t>
+          <t>TT130</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>1428</t>
+          <t>TT202</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>5011</t>
+          <t>TT206</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>5021</t>
+          <t>VL22</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>5025</t>
+          <t>VL57</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>5030</t>
+          <t>VLINE8058</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>5034</t>
+          <t>VLINE8059</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>5041</t>
+          <t>VLINE8061</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>5042</t>
+          <t>VLINE8161</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>6001</t>
+          <t>VLINE8163</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>6002</t>
+          <t>VLINE8164</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>6008</t>
+          <t>VLINE8457</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>6011</t>
+          <t>VLINE8459</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>6021</t>
+          <t>VLINE8819</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>6025</t>
+          <t>XP2001</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>6027</t>
+          <t>XP2005</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>6028</t>
+          <t>XP2006</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>6029</t>
+          <t>XP2011</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>XRN005</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>8114</t>
+          <t>XRN009</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>8161</t>
+          <t>XRN017</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>8169</t>
+          <t>XRN018</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>8202</t>
+          <t>XRN021</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>8207</t>
+          <t>XRN022</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>8209</t>
+          <t>XRN028</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>8210</t>
+          <t>XRN029</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>8215</t>
+          <t>1102</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>8217</t>
+          <t>1428</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>8223</t>
+          <t>1437</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>8225</t>
+          <t>5009</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>8239</t>
+          <t>5011</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>8240</t>
+          <t>5021</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>9025</t>
+          <t>5025</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>9029</t>
+          <t>5030</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>9203</t>
+          <t>5031</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>9301</t>
+          <t>5032</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>9302</t>
+          <t>5034</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>9305</t>
+          <t>5041</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>9311</t>
+          <t>5042</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>9312</t>
+          <t>6001</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>9313</t>
+          <t>6002</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>9406</t>
+          <t>6003</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>9408</t>
+          <t>6008</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
+          <t>6011</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>6021</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>6025</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>6027</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>6028</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>6029</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>8030</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>8114</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t>8135</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>8161</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>8169</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>8202</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>8206</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>8207</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="inlineStr">
+        <is>
+          <t>8209</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>8210</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>8215</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>8217</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="inlineStr">
+        <is>
+          <t>8223</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>8225</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="inlineStr">
+        <is>
+          <t>8239</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>8240</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="inlineStr">
+        <is>
+          <t>8249</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>9025</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="inlineStr">
+        <is>
+          <t>9029</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>9203</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="inlineStr">
+        <is>
+          <t>9301</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>9302</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="inlineStr">
+        <is>
+          <t>9305</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>9307</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>9311</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>9312</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>9313</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>9406</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>9408</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
           <t>9410</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>44202</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>44204</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update RailOps database files - 2026-04-29 18:02:14 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A250"/>
+  <dimension ref="A1:A268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -461,1743 +461,1869 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ACB4403</t>
+          <t>1102</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ACB4404</t>
+          <t>1428</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ACD6047</t>
+          <t>1435</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ACD6049</t>
+          <t>1437</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ACD6052</t>
+          <t>5009</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ACD6056</t>
+          <t>5011</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ACD6057</t>
+          <t>5021</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>ACD6058</t>
+          <t>5025</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ACD6059</t>
+          <t>5030</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>ACD6065</t>
+          <t>5031</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ACD6066</t>
+          <t>5032</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>ACD6069</t>
+          <t>5034</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>ACD6071</t>
+          <t>5041</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>ACD6074</t>
+          <t>5042</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>BL33</t>
+          <t>6001</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>C502</t>
+          <t>6002</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>C509</t>
+          <t>6003</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>CEY004</t>
+          <t>6008</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>CEY006</t>
+          <t>6011</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>CEY007</t>
+          <t>6021</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>CF4401</t>
+          <t>6025</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>CF4405</t>
+          <t>6027</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>CF4410</t>
+          <t>6028</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>CF4421</t>
+          <t>6029</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>CF4424</t>
+          <t>8030</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>CF4425</t>
+          <t>8114</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>CF4427</t>
+          <t>8135</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>CF4429</t>
+          <t>8161</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>CLP12</t>
+          <t>8169</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>CLP13</t>
+          <t>8202</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>CSR010</t>
+          <t>8203</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>CSR015</t>
+          <t>8206</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>CSR019</t>
+          <t>8207</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>CSR020</t>
+          <t>8209</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>CSR021</t>
+          <t>8210</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>CSR023</t>
+          <t>8215</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>DS003</t>
+          <t>8217</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>EA2503</t>
+          <t>8223</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>FIE001</t>
+          <t>8225</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>G513</t>
+          <t>8239</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>G514</t>
+          <t>8240</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>G516</t>
+          <t>8249</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>G533</t>
+          <t>9025</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>G534</t>
+          <t>9029</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>G536</t>
+          <t>9203</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>GL103</t>
+          <t>9301</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>GL105</t>
+          <t>9302</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>GL111</t>
+          <t>9305</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>GWA002</t>
+          <t>9307</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>GWA004</t>
+          <t>9311</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>GWA008</t>
+          <t>9312</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>GWA009</t>
+          <t>9313</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>GWB103</t>
+          <t>9406</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>GWB104</t>
+          <t>9408</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>GWU008</t>
+          <t>9410</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>GWU014</t>
+          <t>44202</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>HM2701</t>
+          <t>44204</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>HM2702</t>
+          <t>ACB4403</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>HM2705</t>
+          <t>ACB4404</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>HM2755</t>
+          <t>ACD6047</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>HM2756</t>
+          <t>ACD6049</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>LDP002</t>
+          <t>ACD6052</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>LDP004</t>
+          <t>ACD6056</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>LDP008</t>
+          <t>ACD6057</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>LE2853</t>
+          <t>ACD6058</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>LZ3114</t>
+          <t>ACD6059</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>M437</t>
+          <t>ACD6065</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>M865</t>
+          <t>ACD6066</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>MAN004</t>
+          <t>ACD6069</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>MAN007</t>
+          <t>ACD6071</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>MAN013</t>
+          <t>ACD6074</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>MAN015</t>
+          <t>BL26</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>MAN017</t>
+          <t>BL33</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>MM76M</t>
+          <t>C502</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>MM82M</t>
+          <t>C509</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>MM152M</t>
+          <t>CEY004</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>MM158M</t>
+          <t>CEY006</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>MM172M</t>
+          <t>CEY007</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>MM232M</t>
+          <t>CF4401</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>MM260M</t>
+          <t>CF4405</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>MM280M</t>
+          <t>CF4410</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>MM502M</t>
+          <t>CF4421</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>MM522M</t>
+          <t>CF4424</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>MM624M</t>
+          <t>CF4425</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>MM674M</t>
+          <t>CF4427</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>MM718M</t>
+          <t>CF4429</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>MM810M</t>
+          <t>CLP12</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>MM830M</t>
+          <t>CLP13</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>MM834M</t>
+          <t>CSR010</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>MM838M</t>
+          <t>CSR015</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>MM914M</t>
+          <t>CSR019</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>MM928M</t>
+          <t>CSR020</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>MM934M</t>
+          <t>CSR021</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>MM946M</t>
+          <t>CSR023</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>MM962M</t>
+          <t>DS003</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>MM982M</t>
+          <t>EA2503</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>MM9914M</t>
+          <t>FIE001</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>MM9924M</t>
+          <t>G513</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>MM9927M</t>
+          <t>G514</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>MM9946M</t>
+          <t>G516</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>MM9965M</t>
+          <t>G533</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>MM9966M</t>
+          <t>G534</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>MM9970M</t>
+          <t>G536</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>GL103</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>GL105</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>GL111</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>NR6</t>
+          <t>GWA002</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>NR10</t>
+          <t>GWA004</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>NR11</t>
+          <t>GWA008</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>NR13</t>
+          <t>GWA009</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>NR14</t>
+          <t>GWB102</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>NR20</t>
+          <t>GWB103</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>NR35</t>
+          <t>GWB104</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>GWU008</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>NR46</t>
+          <t>GWU013</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>GWU014</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>HM2701</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>HM2702</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>HM2705</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>HM2706</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>HM2753</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>HM2755</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>HM2756</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>LDP002</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>LDP004</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>NR107</t>
+          <t>LDP008</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>LE2851</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>LE2853</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>LZ3114</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>M437</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>M865</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>PKLA4</t>
+          <t>MAN004</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>MAN007</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>MAN013</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>MAN015</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>MAN017</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>MM76M</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>MM82M</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>MM152M</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>MM158M</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>MM172M</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>QL009</t>
+          <t>MM232M</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>QL019</t>
+          <t>MM260M</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>QR5400</t>
+          <t>MM280M</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>MM502M</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>RA2303</t>
+          <t>MM522M</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>MM624M</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>MM674M</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>SCT008</t>
+          <t>MM718M</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>MM768M</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>MM810M</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>MM830M</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>T373</t>
+          <t>MM834M</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>MM838M</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>MM914M</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>MM928M</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>TT02</t>
+          <t>MM934M</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>MM946M</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>MM962M</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>MM972M</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>TT105</t>
+          <t>MM982M</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>MM9914M</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>MM9924M</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>MM9927M</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>MM9936M</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>TT123</t>
+          <t>MM9938M</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>TT126</t>
+          <t>MM9946M</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>TT129</t>
+          <t>MM9961M</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>MM9963M</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>MM9965M</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>MM9966M</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>VL22</t>
+          <t>MM9970M</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>VL57</t>
+          <t>MRL001</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>VLINE8058</t>
+          <t>NR4</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>VLINE8059</t>
+          <t>NR5</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>VLINE8061</t>
+          <t>NR6</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>VLINE8161</t>
+          <t>NR10</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>VLINE8163</t>
+          <t>NR11</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>VLINE8164</t>
+          <t>NR13</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>VLINE8457</t>
+          <t>NR14</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>VLINE8459</t>
+          <t>NR20</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>VLINE8819</t>
+          <t>NR35</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>XP2001</t>
+          <t>NR37</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>NR46</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>XP2006</t>
+          <t>NR47</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>NR64</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>NR65</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>NR75</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>NR78</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>NR93</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>NR94</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>XRN022</t>
+          <t>NR95</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>XRN028</t>
+          <t>NR97</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>XRN029</t>
+          <t>NR102</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>1102</t>
+          <t>NR107</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>1428</t>
+          <t>NR109</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>1437</t>
+          <t>NR112</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>5009</t>
+          <t>NR113</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>5011</t>
+          <t>NR115</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>5021</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>5025</t>
+          <t>PKLA4</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>5030</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>5031</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>5032</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>5034</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>5041</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>5042</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>6001</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>6002</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>6003</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>6008</t>
+          <t>QL009</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>6011</t>
+          <t>QL019</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>6021</t>
+          <t>QR5400</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>6025</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>6027</t>
+          <t>RA2303</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>6028</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>6029</t>
+          <t>SCT001</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>SCT008</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>8114</t>
+          <t>SCT009</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>8135</t>
+          <t>SSR102</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>8161</t>
+          <t>SSR103</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>8169</t>
+          <t>T373</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>8202</t>
+          <t>TE2803</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>8206</t>
+          <t>TE2805</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>8207</t>
+          <t>TE2807</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>8209</t>
+          <t>TE2808</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>8210</t>
+          <t>TE2813</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>8215</t>
+          <t>TJ096</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>8217</t>
+          <t>TT02</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>8223</t>
+          <t>TT03</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>8225</t>
+          <t>TT05</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>8239</t>
+          <t>TT08</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>8240</t>
+          <t>TT103</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>8249</t>
+          <t>TT105</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>9025</t>
+          <t>TT107</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>9029</t>
+          <t>TT110</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>9203</t>
+          <t>TT115</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>9301</t>
+          <t>TT117</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>9302</t>
+          <t>TT123</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>9305</t>
+          <t>TT126</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>9307</t>
+          <t>TT129</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>9311</t>
+          <t>TT130</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>9312</t>
+          <t>TT202</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>9313</t>
+          <t>TT206</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>9406</t>
+          <t>VL22</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>9408</t>
+          <t>VL57</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>9410</t>
+          <t>VLINE8058</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>44202</t>
+          <t>VLINE8059</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>44204</t>
+          <t>VLINE8061</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8161</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8163</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8164</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8457</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8459</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8819</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>XP2001</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>XP2005</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="inlineStr">
+        <is>
+          <t>XP2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>XP2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="inlineStr">
+        <is>
+          <t>XRN005</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>XRN009</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>XRN017</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>XRN018</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="inlineStr">
+        <is>
+          <t>XRN021</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>XRN022</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="inlineStr">
+        <is>
+          <t>XRN028</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="inlineStr">
+        <is>
+          <t>XRN029</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update RailOps database files - 2026-04-29 18:28:20 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A268"/>
+  <dimension ref="A1:A284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -489,1839 +489,1951 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>5009</t>
+          <t>4829</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>5011</t>
+          <t>5009</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>5021</t>
+          <t>5011</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>5025</t>
+          <t>5021</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>5030</t>
+          <t>5025</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>5031</t>
+          <t>5030</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>5032</t>
+          <t>5031</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>5034</t>
+          <t>5032</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>5041</t>
+          <t>5034</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>5042</t>
+          <t>5041</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>6001</t>
+          <t>5042</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>6002</t>
+          <t>6001</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>6003</t>
+          <t>6002</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>6008</t>
+          <t>6003</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>6011</t>
+          <t>6008</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>6021</t>
+          <t>6011</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>6025</t>
+          <t>6021</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>6027</t>
+          <t>6025</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>6028</t>
+          <t>6027</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>6029</t>
+          <t>6028</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>6029</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>8114</t>
+          <t>8030</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>8135</t>
+          <t>8114</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>8161</t>
+          <t>8115</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>8169</t>
+          <t>8135</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>8202</t>
+          <t>8158</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>8203</t>
+          <t>8161</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>8206</t>
+          <t>8169</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>8207</t>
+          <t>8202</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>8209</t>
+          <t>8203</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>8210</t>
+          <t>8206</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>8215</t>
+          <t>8207</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>8217</t>
+          <t>8209</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>8223</t>
+          <t>8210</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>8225</t>
+          <t>8215</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>8239</t>
+          <t>8217</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>8240</t>
+          <t>8223</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>8249</t>
+          <t>8225</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>9025</t>
+          <t>8239</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>9029</t>
+          <t>8240</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>9203</t>
+          <t>8249</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>9301</t>
+          <t>9025</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>9302</t>
+          <t>9029</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>9305</t>
+          <t>9203</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>9307</t>
+          <t>9301</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>9311</t>
+          <t>9302</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>9312</t>
+          <t>9305</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>9313</t>
+          <t>9307</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>9406</t>
+          <t>9311</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>9408</t>
+          <t>9312</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>9410</t>
+          <t>9313</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>44202</t>
+          <t>9406</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>44204</t>
+          <t>9408</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>ACB4403</t>
+          <t>9410</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>ACB4404</t>
+          <t>44202</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>ACD6047</t>
+          <t>44204</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>ACD6049</t>
+          <t>ACB4403</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>ACD6052</t>
+          <t>ACB4404</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>ACD6056</t>
+          <t>ACD6047</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>ACD6057</t>
+          <t>ACD6049</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>ACD6058</t>
+          <t>ACD6052</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>ACD6059</t>
+          <t>ACD6056</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>ACD6065</t>
+          <t>ACD6057</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>ACD6066</t>
+          <t>ACD6058</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>ACD6069</t>
+          <t>ACD6059</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>ACD6071</t>
+          <t>ACD6065</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>ACD6074</t>
+          <t>ACD6066</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>BL26</t>
+          <t>ACD6069</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>BL33</t>
+          <t>ACD6071</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>C502</t>
+          <t>ACD6074</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>C509</t>
+          <t>BL26</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>CEY004</t>
+          <t>BL33</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>CEY006</t>
+          <t>C502</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>CEY007</t>
+          <t>C509</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>CF4401</t>
+          <t>CEY004</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>CF4405</t>
+          <t>CEY006</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>CF4410</t>
+          <t>CEY007</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>CF4421</t>
+          <t>CF4401</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>CF4424</t>
+          <t>CF4405</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>CF4425</t>
+          <t>CF4410</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>CF4427</t>
+          <t>CF4421</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>CF4429</t>
+          <t>CF4424</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>CLP12</t>
+          <t>CF4425</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>CLP13</t>
+          <t>CF4427</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>CSR010</t>
+          <t>CF4429</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>CSR015</t>
+          <t>CLP12</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>CSR019</t>
+          <t>CLP13</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>CSR020</t>
+          <t>CSR010</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>CSR021</t>
+          <t>CSR015</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>CSR023</t>
+          <t>CSR019</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>DS003</t>
+          <t>CSR020</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>EA2503</t>
+          <t>CSR021</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>FIE001</t>
+          <t>CSR023</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>G513</t>
+          <t>DS003</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>G514</t>
+          <t>EA2503</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>G516</t>
+          <t>FIE001</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>G533</t>
+          <t>G513</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>G534</t>
+          <t>G514</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>G536</t>
+          <t>G516</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>GL103</t>
+          <t>G533</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>GL105</t>
+          <t>G534</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>GL111</t>
+          <t>G536</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>GWA002</t>
+          <t>GL103</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>GWA004</t>
+          <t>GL105</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>GWA008</t>
+          <t>GL111</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>GWA009</t>
+          <t>GWA002</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>GWB102</t>
+          <t>GWA004</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>GWB103</t>
+          <t>GWA008</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>GWB104</t>
+          <t>GWA009</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>GWU008</t>
+          <t>GWB102</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>GWU013</t>
+          <t>GWB103</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>GWU014</t>
+          <t>GWB104</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>HM2701</t>
+          <t>GWU008</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>HM2702</t>
+          <t>GWU013</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>HM2705</t>
+          <t>GWU014</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>HM2706</t>
+          <t>HM2701</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>HM2753</t>
+          <t>HM2702</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>HM2755</t>
+          <t>HM2703</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>HM2756</t>
+          <t>HM2705</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>LDP002</t>
+          <t>HM2706</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>LDP004</t>
+          <t>HM2753</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>LDP008</t>
+          <t>HM2755</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>LE2851</t>
+          <t>HM2756</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>LE2853</t>
+          <t>LDP002</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>LZ3114</t>
+          <t>LDP004</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>M437</t>
+          <t>LDP008</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>M865</t>
+          <t>LE2851</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>MAN004</t>
+          <t>LE2853</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>MAN007</t>
+          <t>LE2855</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>MAN013</t>
+          <t>LZ3114</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>MAN015</t>
+          <t>M437</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>MAN017</t>
+          <t>M865</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>MM76M</t>
+          <t>MAN004</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>MM82M</t>
+          <t>MAN007</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>MM152M</t>
+          <t>MAN013</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>MM158M</t>
+          <t>MAN015</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>MM172M</t>
+          <t>MAN017</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>MM232M</t>
+          <t>MM14M</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>MM260M</t>
+          <t>MM76M</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>MM280M</t>
+          <t>MM82M</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>MM502M</t>
+          <t>MM152M</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>MM522M</t>
+          <t>MM158M</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>MM624M</t>
+          <t>MM172M</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>MM674M</t>
+          <t>MM212M</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>MM718M</t>
+          <t>MM232M</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>MM768M</t>
+          <t>MM246M</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>MM810M</t>
+          <t>MM260M</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>MM830M</t>
+          <t>MM280M</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>MM834M</t>
+          <t>MM502M</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>MM838M</t>
+          <t>MM522M</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>MM914M</t>
+          <t>MM624M</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>MM928M</t>
+          <t>MM674M</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>MM934M</t>
+          <t>MM718M</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>MM946M</t>
+          <t>MM768M</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>MM962M</t>
+          <t>MM810M</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>MM972M</t>
+          <t>MM830M</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>MM982M</t>
+          <t>MM834M</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>MM9914M</t>
+          <t>MM838M</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>MM9924M</t>
+          <t>MM864M</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>MM9927M</t>
+          <t>MM880M</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>MM9936M</t>
+          <t>MM914M</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>MM9938M</t>
+          <t>MM928M</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>MM9946M</t>
+          <t>MM934M</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>MM9961M</t>
+          <t>MM946M</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>MM9963M</t>
+          <t>MM962M</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>MM9965M</t>
+          <t>MM972M</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>MM9966M</t>
+          <t>MM982M</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>MM9970M</t>
+          <t>MM9914M</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MM9924M</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>MM9927M</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>MM9931M</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>NR6</t>
+          <t>MM9936M</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>NR10</t>
+          <t>MM9938M</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>NR11</t>
+          <t>MM9946M</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>NR13</t>
+          <t>MM9952M</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>NR14</t>
+          <t>MM9961M</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>NR20</t>
+          <t>MM9963M</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>NR35</t>
+          <t>MM9965M</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>MM9966M</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>NR46</t>
+          <t>MM9970M</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>MRL001</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR4</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR5</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR6</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR10</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR11</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR13</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR14</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>NR20</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR35</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>NR107</t>
+          <t>NR37</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR46</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR47</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR64</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR65</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>NR75</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>PKLA4</t>
+          <t>NR78</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>NR93</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>NR94</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>NR95</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>NR97</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>NR102</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>NR107</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>NR109</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>NR112</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>NR113</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>QL009</t>
+          <t>NR115</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>QL019</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>QR5400</t>
+          <t>PKLA4</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>RA2303</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>SCT008</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>T373</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>QL009</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>QL019</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>QR5400</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>RA2303</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>TT02</t>
+          <t>RL301</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>SCT001</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>SCT008</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>SCT009</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>SSR102</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>TT105</t>
+          <t>SSR103</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>T373</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TE2803</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TE2805</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TE2807</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>TT123</t>
+          <t>TE2808</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>TT126</t>
+          <t>TE2813</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>TT129</t>
+          <t>TJ096</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT02</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT03</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT05</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>VL22</t>
+          <t>TT08</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>VL57</t>
+          <t>TT103</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>VLINE8058</t>
+          <t>TT105</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>VLINE8059</t>
+          <t>TT107</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>VLINE8061</t>
+          <t>TT110</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>VLINE8161</t>
+          <t>TT115</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>VLINE8163</t>
+          <t>TT117</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>VLINE8164</t>
+          <t>TT123</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>VLINE8457</t>
+          <t>TT126</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>VLINE8459</t>
+          <t>TT129</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>VLINE8819</t>
+          <t>TT130</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>XP2001</t>
+          <t>TT202</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>TT206</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>XP2006</t>
+          <t>VL22</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>VL57</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>VLINE8058</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>VLINE8059</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>VLINE8061</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>VLINE8102</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>VLINE8161</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>XRN022</t>
+          <t>VLINE8163</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>XRN028</t>
+          <t>VLINE8164</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8400</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8457</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8459</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8702</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8819</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="2" t="inlineStr">
+        <is>
+          <t>XP2001</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="inlineStr">
+        <is>
+          <t>XP2005</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="inlineStr">
+        <is>
+          <t>XP2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>XP2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="inlineStr">
+        <is>
+          <t>XRN005</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>XRN009</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="2" t="inlineStr">
+        <is>
+          <t>XRN017</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="inlineStr">
+        <is>
+          <t>XRN018</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="2" t="inlineStr">
+        <is>
+          <t>XRN021</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="inlineStr">
+        <is>
+          <t>XRN022</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="2" t="inlineStr">
+        <is>
+          <t>XRN028</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="inlineStr">
         <is>
           <t>XRN029</t>
         </is>

</xml_diff>

<commit_message>
Update RailOps database files - 2026-04-30 00:02:48 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A284"/>
+  <dimension ref="A1:A471"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -496,1944 +496,3253 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>5009</t>
+          <t>4903</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>5011</t>
+          <t>5005</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>5021</t>
+          <t>5009</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>5025</t>
+          <t>5011</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>5030</t>
+          <t>5021</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>5031</t>
+          <t>5025</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>5032</t>
+          <t>5030</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>5034</t>
+          <t>5031</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>5041</t>
+          <t>5032</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>5042</t>
+          <t>5034</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>6001</t>
+          <t>5041</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>6002</t>
+          <t>5042</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>6003</t>
+          <t>6001</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>6008</t>
+          <t>6002</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>6011</t>
+          <t>6003</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>6021</t>
+          <t>6007</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>6025</t>
+          <t>6008</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>6027</t>
+          <t>6011</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>6028</t>
+          <t>6021</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>6029</t>
+          <t>6025</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>6027</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>8114</t>
+          <t>6028</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>8115</t>
+          <t>6029</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>8135</t>
+          <t>8030</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>8158</t>
+          <t>8114</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>8161</t>
+          <t>8115</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>8169</t>
+          <t>8135</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>8202</t>
+          <t>8153</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>8203</t>
+          <t>8158</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>8206</t>
+          <t>8161</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>8207</t>
+          <t>8169</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>8209</t>
+          <t>8172</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>8210</t>
+          <t>8179</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>8215</t>
+          <t>8202</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>8217</t>
+          <t>8203</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>8223</t>
+          <t>8206</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>8225</t>
+          <t>8207</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>8239</t>
+          <t>8209</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>8240</t>
+          <t>8210</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>8249</t>
+          <t>8215</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>9025</t>
+          <t>8217</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>9029</t>
+          <t>8223</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>9203</t>
+          <t>8225</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>9301</t>
+          <t>8226</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>9302</t>
+          <t>8235</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>9305</t>
+          <t>8239</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>9307</t>
+          <t>8240</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>9311</t>
+          <t>8249</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>9312</t>
+          <t>9025</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>9313</t>
+          <t>9029</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>9406</t>
+          <t>9203</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>9408</t>
+          <t>9301</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>9410</t>
+          <t>9302</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>44202</t>
+          <t>9305</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>44204</t>
+          <t>9307</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>ACB4403</t>
+          <t>9311</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>ACB4404</t>
+          <t>9312</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>ACD6047</t>
+          <t>9313</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>ACD6049</t>
+          <t>9406</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>ACD6052</t>
+          <t>9408</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>ACD6056</t>
+          <t>9410</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>ACD6057</t>
+          <t>44202</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>ACD6058</t>
+          <t>44204</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>ACD6059</t>
+          <t>44208</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>ACD6065</t>
+          <t>ACB4403</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>ACD6066</t>
+          <t>ACB4404</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>ACD6069</t>
+          <t>ACD6047</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>ACD6071</t>
+          <t>ACD6049</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>ACD6074</t>
+          <t>ACD6052</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>BL26</t>
+          <t>ACD6056</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>BL33</t>
+          <t>ACD6057</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>C502</t>
+          <t>ACD6058</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>C509</t>
+          <t>ACD6059</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>CEY004</t>
+          <t>ACD6065</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>CEY006</t>
+          <t>ACD6066</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>CEY007</t>
+          <t>ACD6069</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>CF4401</t>
+          <t>ACD6071</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>CF4405</t>
+          <t>ACD6074</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>CF4410</t>
+          <t>BL26</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>CF4421</t>
+          <t>BL31</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>CF4424</t>
+          <t>BL33</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>CF4425</t>
+          <t>C502</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>CF4427</t>
+          <t>C506</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>CF4429</t>
+          <t>C509</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>CLP12</t>
+          <t>CEY004</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>CLP13</t>
+          <t>CEY006</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>CSR010</t>
+          <t>CEY007</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>CSR015</t>
+          <t>CF4401</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>CSR019</t>
+          <t>CF4405</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>CSR020</t>
+          <t>CF4410</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>CSR021</t>
+          <t>CF4412</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>CSR023</t>
+          <t>CF4420</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>DS003</t>
+          <t>CF4421</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>EA2503</t>
+          <t>CF4424</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>FIE001</t>
+          <t>CF4425</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>G513</t>
+          <t>CF4427</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>G514</t>
+          <t>CF4429</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>G516</t>
+          <t>CLP12</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>G533</t>
+          <t>CLP13</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>G534</t>
+          <t>CM3304</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>G536</t>
+          <t>CSR010</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>GL103</t>
+          <t>CSR015</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>GL105</t>
+          <t>CSR017</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>GL111</t>
+          <t>CSR019</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>GWA002</t>
+          <t>CSR020</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>GWA004</t>
+          <t>CSR021</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>GWA008</t>
+          <t>CSR023</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>GWA009</t>
+          <t>DS003</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>GWB102</t>
+          <t>EA2502</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>GWB103</t>
+          <t>EA2503</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>GWB104</t>
+          <t>EA2506</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>GWU008</t>
+          <t>EC2521</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>GWU013</t>
+          <t>EC2525</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>GWU014</t>
+          <t>EC2526</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>HM2701</t>
+          <t>FIE001</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>HM2702</t>
+          <t>FIE003</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>HM2703</t>
+          <t>G513</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>HM2705</t>
+          <t>G514</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>HM2706</t>
+          <t>G516</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>HM2753</t>
+          <t>G533</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>HM2755</t>
+          <t>G534</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>HM2756</t>
+          <t>G536</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>LDP002</t>
+          <t>GL103</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>LDP004</t>
+          <t>GL105</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>LDP008</t>
+          <t>GL108</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>LE2851</t>
+          <t>GL111</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>LE2853</t>
+          <t>GWA002</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>LE2855</t>
+          <t>GWA004</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>LZ3114</t>
+          <t>GWA008</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>M437</t>
+          <t>GWA009</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>M865</t>
+          <t>GWB102</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>MAN004</t>
+          <t>GWB103</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>MAN007</t>
+          <t>GWB104</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>MAN013</t>
+          <t>GWU008</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>MAN015</t>
+          <t>GWU013</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>MAN017</t>
+          <t>GWU014</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>MM14M</t>
+          <t>GWU015</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>MM76M</t>
+          <t>HM2701</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>MM82M</t>
+          <t>HM2702</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>MM152M</t>
+          <t>HM2703</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>MM158M</t>
+          <t>HM2705</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>MM172M</t>
+          <t>HM2706</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>MM212M</t>
+          <t>HM2753</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>MM232M</t>
+          <t>HM2755</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>MM246M</t>
+          <t>HM2756</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>MM260M</t>
+          <t>HM2757</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>MM280M</t>
+          <t>JP9750</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>MM502M</t>
+          <t>LDP002</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>MM522M</t>
+          <t>LDP004</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>MM624M</t>
+          <t>LDP008</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>MM674M</t>
+          <t>LE2851</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>MM718M</t>
+          <t>LE2853</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>MM768M</t>
+          <t>LE2855</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>MM810M</t>
+          <t>LE2858</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>MM830M</t>
+          <t>LE2862</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>MM834M</t>
+          <t>LZ3114</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>MM838M</t>
+          <t>M437</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>MM864M</t>
+          <t>M865</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>MM880M</t>
+          <t>MAN004</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>MM914M</t>
+          <t>MAN005</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>MM928M</t>
+          <t>MAN007</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>MM934M</t>
+          <t>MAN011</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>MM946M</t>
+          <t>MAN013</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>MM962M</t>
+          <t>MAN015</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>MM972M</t>
+          <t>MAN017</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>MM982M</t>
+          <t>MM4M</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>MM9914M</t>
+          <t>MM8M</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>MM9924M</t>
+          <t>MM14M</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>MM9927M</t>
+          <t>MM32M</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>MM9931M</t>
+          <t>MM38M</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>MM9936M</t>
+          <t>MM40M</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>MM9938M</t>
+          <t>MM42M</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>MM9946M</t>
+          <t>MM44M</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>MM9952M</t>
+          <t>MM48M</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>MM9961M</t>
+          <t>MM52M</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>MM9963M</t>
+          <t>MM64M</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>MM9965M</t>
+          <t>MM76M</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>MM9966M</t>
+          <t>MM78M</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>MM9970M</t>
+          <t>MM80M</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MM82M</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>MM84M</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>MM86M</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>NR6</t>
+          <t>MM94M</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>NR10</t>
+          <t>MM96M</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>NR11</t>
+          <t>MM98M</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>NR13</t>
+          <t>MM99M</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>NR14</t>
+          <t>MM122M</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>NR20</t>
+          <t>MM152M</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>NR35</t>
+          <t>MM158M</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>MM172M</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>NR46</t>
+          <t>MM212M</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>MM214M</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>MM216M</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>MM232M</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>MM236M</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>MM240M</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>MM246M</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>MM260M</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>MM264M</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>MM266M</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>MM270M</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>NR107</t>
+          <t>MM280M</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>MM288M</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>MM380M</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>MM456M</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>MM464M</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>MM478M</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>PKLA4</t>
+          <t>MM482M</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>MM502M</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>MM506M</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>MM522M</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>MM542M</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>MM546M</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>MM588M</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>MM592M</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>MM624M</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>MM636M</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>QL009</t>
+          <t>MM638M</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>QL019</t>
+          <t>MM647M</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>QR5400</t>
+          <t>MM656M</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>MM658M</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>RA2303</t>
+          <t>MM660M</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>MM664M</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>MM668M</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>MM673M</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>SCT008</t>
+          <t>MM674M</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>MM676M</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>MM680M</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>MM718M</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>T373</t>
+          <t>MM744M</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>MM752M</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>MM768M</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>MM772M</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>MM774M</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>MM778M</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>MM788M</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>TT02</t>
+          <t>MM798M</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>MM800M</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>MM806M</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>MM808M</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>MM810M</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>TT105</t>
+          <t>MM826M</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>MM830M</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>MM832M</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>MM834M</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>MM838M</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>TT123</t>
+          <t>MM842M</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>TT126</t>
+          <t>MM858M</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>TT129</t>
+          <t>MM860M</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>MM862M</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>MM864M</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>MM872M</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>VL22</t>
+          <t>MM878M</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>VL57</t>
+          <t>MM880M</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>VLINE8058</t>
+          <t>MM886M</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>VLINE8059</t>
+          <t>MM896M</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>VLINE8061</t>
+          <t>MM912M</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>VLINE8102</t>
+          <t>MM914M</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>VLINE8161</t>
+          <t>MM924M</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>VLINE8163</t>
+          <t>MM928M</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>VLINE8164</t>
+          <t>MM934M</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>VLINE8400</t>
+          <t>MM940M</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>VLINE8457</t>
+          <t>MM944M</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>VLINE8459</t>
+          <t>MM946M</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>VLINE8702</t>
+          <t>MM952M</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>VLINE8819</t>
+          <t>MM956M</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>XP2001</t>
+          <t>MM958M</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>MM960M</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>XP2006</t>
+          <t>MM962M</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>MM964M</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>MM968M</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>MM972M</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>MM974M</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>MM976M</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>MM980M</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>XRN022</t>
+          <t>MM982M</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>XRN028</t>
+          <t>MM9901M</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
+        <is>
+          <t>MM9903M</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="2" t="inlineStr">
+        <is>
+          <t>MM9906M</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>MM9908M</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="2" t="inlineStr">
+        <is>
+          <t>MM9910M</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="inlineStr">
+        <is>
+          <t>MM9912M</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="2" t="inlineStr">
+        <is>
+          <t>MM9914M</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="2" t="inlineStr">
+        <is>
+          <t>MM9918M</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="2" t="inlineStr">
+        <is>
+          <t>MM9920M</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="2" t="inlineStr">
+        <is>
+          <t>MM9924M</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="2" t="inlineStr">
+        <is>
+          <t>MM9926M</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="2" t="inlineStr">
+        <is>
+          <t>MM9927M</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="2" t="inlineStr">
+        <is>
+          <t>MM9928M</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="2" t="inlineStr">
+        <is>
+          <t>MM9929M</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="2" t="inlineStr">
+        <is>
+          <t>MM9931M</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="2" t="inlineStr">
+        <is>
+          <t>MM9936M</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="2" t="inlineStr">
+        <is>
+          <t>MM9937M</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="2" t="inlineStr">
+        <is>
+          <t>MM9938M</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="2" t="inlineStr">
+        <is>
+          <t>MM9941M</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="2" t="inlineStr">
+        <is>
+          <t>MM9943M</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="2" t="inlineStr">
+        <is>
+          <t>MM9946M</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="2" t="inlineStr">
+        <is>
+          <t>MM9947M</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="2" t="inlineStr">
+        <is>
+          <t>MM9948M</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="2" t="inlineStr">
+        <is>
+          <t>MM9952M</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="2" t="inlineStr">
+        <is>
+          <t>MM9957M</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="2" t="inlineStr">
+        <is>
+          <t>MM9958M</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="2" t="inlineStr">
+        <is>
+          <t>MM9959M</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="2" t="inlineStr">
+        <is>
+          <t>MM9960M</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="2" t="inlineStr">
+        <is>
+          <t>MM9961M</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="2" t="inlineStr">
+        <is>
+          <t>MM9963M</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="2" t="inlineStr">
+        <is>
+          <t>MM9964M</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="2" t="inlineStr">
+        <is>
+          <t>MM9965M</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="2" t="inlineStr">
+        <is>
+          <t>MM9966M</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="2" t="inlineStr">
+        <is>
+          <t>MM9968M</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="2" t="inlineStr">
+        <is>
+          <t>MM9969M</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="2" t="inlineStr">
+        <is>
+          <t>MM9970M</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="2" t="inlineStr">
+        <is>
+          <t>MRL001</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="2" t="inlineStr">
+        <is>
+          <t>MTPV1</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="2" t="inlineStr">
+        <is>
+          <t>MTPV2</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="2" t="inlineStr">
+        <is>
+          <t>N466</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="2" t="inlineStr">
+        <is>
+          <t>NR4</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="2" t="inlineStr">
+        <is>
+          <t>NR5</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="2" t="inlineStr">
+        <is>
+          <t>NR6</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="2" t="inlineStr">
+        <is>
+          <t>NR10</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="2" t="inlineStr">
+        <is>
+          <t>NR11</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="2" t="inlineStr">
+        <is>
+          <t>NR13</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="2" t="inlineStr">
+        <is>
+          <t>NR14</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="2" t="inlineStr">
+        <is>
+          <t>NR17</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="2" t="inlineStr">
+        <is>
+          <t>NR20</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="2" t="inlineStr">
+        <is>
+          <t>NR35</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="2" t="inlineStr">
+        <is>
+          <t>NR37</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="2" t="inlineStr">
+        <is>
+          <t>NR46</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="2" t="inlineStr">
+        <is>
+          <t>NR47</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="2" t="inlineStr">
+        <is>
+          <t>NR64</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="2" t="inlineStr">
+        <is>
+          <t>NR65</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="2" t="inlineStr">
+        <is>
+          <t>NR75</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="2" t="inlineStr">
+        <is>
+          <t>NR78</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="2" t="inlineStr">
+        <is>
+          <t>NR83</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="2" t="inlineStr">
+        <is>
+          <t>NR93</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="2" t="inlineStr">
+        <is>
+          <t>NR94</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="2" t="inlineStr">
+        <is>
+          <t>NR95</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="2" t="inlineStr">
+        <is>
+          <t>NR97</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="2" t="inlineStr">
+        <is>
+          <t>NR102</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="2" t="inlineStr">
+        <is>
+          <t>NR107</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="2" t="inlineStr">
+        <is>
+          <t>NR109</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="2" t="inlineStr">
+        <is>
+          <t>NR112</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="2" t="inlineStr">
+        <is>
+          <t>NR113</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="2" t="inlineStr">
+        <is>
+          <t>NR115</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="2" t="inlineStr">
+        <is>
+          <t>PHC001</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="2" t="inlineStr">
+        <is>
+          <t>PKLA4</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="2" t="inlineStr">
+        <is>
+          <t>Q4004</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="2" t="inlineStr">
+        <is>
+          <t>Q4012</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="2" t="inlineStr">
+        <is>
+          <t>Q4013</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="2" t="inlineStr">
+        <is>
+          <t>Q4016</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="2" t="inlineStr">
+        <is>
+          <t>QBX003</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="2" t="inlineStr">
+        <is>
+          <t>QBX004</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="2" t="inlineStr">
+        <is>
+          <t>QE001</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="2" t="inlineStr">
+        <is>
+          <t>QE002</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="2" t="inlineStr">
+        <is>
+          <t>QE003</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="2" t="inlineStr">
+        <is>
+          <t>QL004</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="2" t="inlineStr">
+        <is>
+          <t>QL007</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="2" t="inlineStr">
+        <is>
+          <t>QL009</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="2" t="inlineStr">
+        <is>
+          <t>QL019</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="2" t="inlineStr">
+        <is>
+          <t>QR1771</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="2" t="inlineStr">
+        <is>
+          <t>QR5400</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="2" t="inlineStr">
+        <is>
+          <t>QR5404</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="2" t="inlineStr">
+        <is>
+          <t>RA2302</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="2" t="inlineStr">
+        <is>
+          <t>RA2303</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="2" t="inlineStr">
+        <is>
+          <t>RB2353</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="2" t="inlineStr">
+        <is>
+          <t>RL301</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="2" t="inlineStr">
+        <is>
+          <t>RM93</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="2" t="inlineStr">
+        <is>
+          <t>SCT001</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="2" t="inlineStr">
+        <is>
+          <t>SCT008</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="2" t="inlineStr">
+        <is>
+          <t>SCT009</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="2" t="inlineStr">
+        <is>
+          <t>SCT013</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="2" t="inlineStr">
+        <is>
+          <t>SO3</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="2" t="inlineStr">
+        <is>
+          <t>SSR102</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="2" t="inlineStr">
+        <is>
+          <t>SSR103</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="2" t="inlineStr">
+        <is>
+          <t>SSR104</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="2" t="inlineStr">
+        <is>
+          <t>T373</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="2" t="inlineStr">
+        <is>
+          <t>TE2801</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="2" t="inlineStr">
+        <is>
+          <t>TE2803</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="2" t="inlineStr">
+        <is>
+          <t>TE2805</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="2" t="inlineStr">
+        <is>
+          <t>TE2807</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="2" t="inlineStr">
+        <is>
+          <t>TE2808</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="2" t="inlineStr">
+        <is>
+          <t>TE2813</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="2" t="inlineStr">
+        <is>
+          <t>TE2814</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="2" t="inlineStr">
+        <is>
+          <t>TJ096</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="2" t="inlineStr">
+        <is>
+          <t>TT02</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="2" t="inlineStr">
+        <is>
+          <t>TT03</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="2" t="inlineStr">
+        <is>
+          <t>TT05</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="2" t="inlineStr">
+        <is>
+          <t>TT08</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="2" t="inlineStr">
+        <is>
+          <t>TT103</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="2" t="inlineStr">
+        <is>
+          <t>TT105</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="2" t="inlineStr">
+        <is>
+          <t>TT107</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="2" t="inlineStr">
+        <is>
+          <t>TT110</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="2" t="inlineStr">
+        <is>
+          <t>TT115</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="2" t="inlineStr">
+        <is>
+          <t>TT117</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="2" t="inlineStr">
+        <is>
+          <t>TT123</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="2" t="inlineStr">
+        <is>
+          <t>TT126</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="2" t="inlineStr">
+        <is>
+          <t>TT129</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="2" t="inlineStr">
+        <is>
+          <t>TT130</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="2" t="inlineStr">
+        <is>
+          <t>TT202</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="2" t="inlineStr">
+        <is>
+          <t>TT206</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="2" t="inlineStr">
+        <is>
+          <t>VL13</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="2" t="inlineStr">
+        <is>
+          <t>VL22</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="2" t="inlineStr">
+        <is>
+          <t>VL27</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="2" t="inlineStr">
+        <is>
+          <t>VL36</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="2" t="inlineStr">
+        <is>
+          <t>VL38</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="2" t="inlineStr">
+        <is>
+          <t>VL43</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="2" t="inlineStr">
+        <is>
+          <t>VL57</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="2" t="inlineStr">
+        <is>
+          <t>VL67</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="2" t="inlineStr">
+        <is>
+          <t>VL86</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="2" t="inlineStr">
+        <is>
+          <t>VL87</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="2" t="inlineStr">
+        <is>
+          <t>VL88</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="2" t="inlineStr">
+        <is>
+          <t>VL90</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="2" t="inlineStr">
+        <is>
+          <t>VL103</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="2" t="inlineStr">
+        <is>
+          <t>VL107</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="2" t="inlineStr">
+        <is>
+          <t>VL114</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="2" t="inlineStr">
+        <is>
+          <t>VL121</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="2" t="inlineStr">
+        <is>
+          <t>VL122</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="2" t="inlineStr">
+        <is>
+          <t>VL124</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="2" t="inlineStr">
+        <is>
+          <t>VL129</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="2" t="inlineStr">
+        <is>
+          <t>VL139</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8013</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8020</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8058</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8059</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8061</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8102</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8115</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8120</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8161</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8163</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8164</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8172</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8211</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8213</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8226</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8228</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8400</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8405</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8408</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8415</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8457</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8459</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8460</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8702</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8731</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8742</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8744</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8750</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8819</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8863</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="2" t="inlineStr">
+        <is>
+          <t>XP2001</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="2" t="inlineStr">
+        <is>
+          <t>XP2005</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="2" t="inlineStr">
+        <is>
+          <t>XP2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="2" t="inlineStr">
+        <is>
+          <t>XP2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="2" t="inlineStr">
+        <is>
+          <t>XP2013</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="2" t="inlineStr">
+        <is>
+          <t>XRN003</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="2" t="inlineStr">
+        <is>
+          <t>XRN005</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="2" t="inlineStr">
+        <is>
+          <t>XRN009</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="2" t="inlineStr">
+        <is>
+          <t>XRN010</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="2" t="inlineStr">
+        <is>
+          <t>XRN017</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="2" t="inlineStr">
+        <is>
+          <t>XRN018</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="2" t="inlineStr">
+        <is>
+          <t>XRN021</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="2" t="inlineStr">
+        <is>
+          <t>XRN022</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="2" t="inlineStr">
+        <is>
+          <t>XRN028</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="2" t="inlineStr">
         <is>
           <t>XRN029</t>
         </is>

</xml_diff>

<commit_message>
Update RailOps database files - 2026-04-30 00:32:55 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A471"/>
+  <dimension ref="A1:A536"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -489,3260 +489,3715 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>4829</t>
+          <t>4708</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>4903</t>
+          <t>4829</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>5005</t>
+          <t>4903</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>5009</t>
+          <t>5005</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>5011</t>
+          <t>5009</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>5021</t>
+          <t>5011</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>5025</t>
+          <t>5021</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>5030</t>
+          <t>5025</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>5031</t>
+          <t>5030</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>5032</t>
+          <t>5031</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>5034</t>
+          <t>5032</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>5041</t>
+          <t>5034</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>5042</t>
+          <t>5041</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>6001</t>
+          <t>5042</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>6002</t>
+          <t>6001</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>6003</t>
+          <t>6002</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>6007</t>
+          <t>6003</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>6008</t>
+          <t>6007</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>6011</t>
+          <t>6008</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>6021</t>
+          <t>6011</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>6025</t>
+          <t>6021</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>6027</t>
+          <t>6023</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>6028</t>
+          <t>6025</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>6029</t>
+          <t>6027</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>6028</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>8114</t>
+          <t>6029</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>8115</t>
+          <t>8030</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>8135</t>
+          <t>8114</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>8153</t>
+          <t>8115</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>8158</t>
+          <t>8116</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>8161</t>
+          <t>8124</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>8169</t>
+          <t>8135</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>8172</t>
+          <t>8144</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>8179</t>
+          <t>8152</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>8202</t>
+          <t>8153</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>8203</t>
+          <t>8158</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>8206</t>
+          <t>8161</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>8207</t>
+          <t>8163</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>8209</t>
+          <t>8169</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>8210</t>
+          <t>8172</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>8215</t>
+          <t>8178</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>8217</t>
+          <t>8179</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>8223</t>
+          <t>8202</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>8225</t>
+          <t>8203</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>8226</t>
+          <t>8206</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>8235</t>
+          <t>8207</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>8239</t>
+          <t>8209</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>8240</t>
+          <t>8210</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>8249</t>
+          <t>8215</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>9025</t>
+          <t>8217</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>9029</t>
+          <t>8223</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>9203</t>
+          <t>8225</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>9301</t>
+          <t>8226</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>9302</t>
+          <t>8235</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>9305</t>
+          <t>8239</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>9307</t>
+          <t>8240</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>9311</t>
+          <t>8249</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>9312</t>
+          <t>9025</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>9313</t>
+          <t>9029</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>9406</t>
+          <t>9203</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>9408</t>
+          <t>9301</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>9410</t>
+          <t>9302</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>44202</t>
+          <t>9305</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>44204</t>
+          <t>9307</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>44208</t>
+          <t>9311</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>ACB4403</t>
+          <t>9312</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>ACB4404</t>
+          <t>9313</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>ACD6047</t>
+          <t>9406</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>ACD6049</t>
+          <t>9408</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>ACD6052</t>
+          <t>9410</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>ACD6056</t>
+          <t>42103</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>ACD6057</t>
+          <t>44202</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>ACD6058</t>
+          <t>44204</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>ACD6059</t>
+          <t>44208</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>ACD6065</t>
+          <t>ACB4403</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>ACD6066</t>
+          <t>ACB4404</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>ACD6069</t>
+          <t>ACD6047</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>ACD6071</t>
+          <t>ACD6049</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>ACD6074</t>
+          <t>ACD6052</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>BL26</t>
+          <t>ACD6056</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>BL31</t>
+          <t>ACD6057</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>BL33</t>
+          <t>ACD6058</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>C502</t>
+          <t>ACD6059</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>C506</t>
+          <t>ACD6065</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>C509</t>
+          <t>ACD6066</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>CEY004</t>
+          <t>ACD6069</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>CEY006</t>
+          <t>ACD6071</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>CEY007</t>
+          <t>ACD6073</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>CF4401</t>
+          <t>ACD6074</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>CF4405</t>
+          <t>BL26</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>CF4410</t>
+          <t>BL31</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>CF4412</t>
+          <t>BL33</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>CF4420</t>
+          <t>C502</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>CF4421</t>
+          <t>C504</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>CF4424</t>
+          <t>C506</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>CF4425</t>
+          <t>C509</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>CF4427</t>
+          <t>CEY004</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>CF4429</t>
+          <t>CEY006</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>CLP12</t>
+          <t>CEY007</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>CLP13</t>
+          <t>CF4401</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>CM3304</t>
+          <t>CF4405</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>CSR010</t>
+          <t>CF4410</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>CSR015</t>
+          <t>CF4412</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>CSR017</t>
+          <t>CF4420</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>CSR019</t>
+          <t>CF4421</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>CSR020</t>
+          <t>CF4424</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>CSR021</t>
+          <t>CF4425</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>CSR023</t>
+          <t>CF4427</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>DS003</t>
+          <t>CF4429</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>EA2502</t>
+          <t>CLF2</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>EA2503</t>
+          <t>CLP12</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>EA2506</t>
+          <t>CLP13</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>EC2521</t>
+          <t>CM3304</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>EC2525</t>
+          <t>CSR010</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>EC2526</t>
+          <t>CSR015</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>FIE001</t>
+          <t>CSR017</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>FIE003</t>
+          <t>CSR019</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>G513</t>
+          <t>CSR020</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>G514</t>
+          <t>CSR021</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>G516</t>
+          <t>CSR023</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>G533</t>
+          <t>DS003</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>G534</t>
+          <t>EA2502</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>G536</t>
+          <t>EA2503</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>GL103</t>
+          <t>EA2506</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>GL105</t>
+          <t>EC2521</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>GL108</t>
+          <t>EC2525</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>GL111</t>
+          <t>EC2526</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>GWA002</t>
+          <t>FIE001</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>GWA004</t>
+          <t>FIE003</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>GWA008</t>
+          <t>G513</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>GWA009</t>
+          <t>G514</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>GWB102</t>
+          <t>G516</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>GWB103</t>
+          <t>G532</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>GWB104</t>
+          <t>G533</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>GWU008</t>
+          <t>G534</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>GWU013</t>
+          <t>G536</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>GWU014</t>
+          <t>GL103</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>GWU015</t>
+          <t>GL105</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>HM2701</t>
+          <t>GL108</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>HM2702</t>
+          <t>GL111</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>HM2703</t>
+          <t>GWA002</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>HM2705</t>
+          <t>GWA004</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>HM2706</t>
+          <t>GWA008</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>HM2753</t>
+          <t>GWA009</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>HM2755</t>
+          <t>GWB102</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>HM2756</t>
+          <t>GWB103</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>HM2757</t>
+          <t>GWB104</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>JP9750</t>
+          <t>GWU008</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>LDP002</t>
+          <t>GWU013</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>LDP004</t>
+          <t>GWU014</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>LDP008</t>
+          <t>GWU015</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>LE2851</t>
+          <t>HM2701</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>LE2853</t>
+          <t>HM2702</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>LE2855</t>
+          <t>HM2703</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>LE2858</t>
+          <t>HM2705</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>LE2862</t>
+          <t>HM2706</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>LZ3114</t>
+          <t>HM2707</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>M437</t>
+          <t>HM2753</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>M865</t>
+          <t>HM2755</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>MAN004</t>
+          <t>HM2756</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>MAN005</t>
+          <t>HM2757</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>MAN007</t>
+          <t>JP9750</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>MAN011</t>
+          <t>LDP002</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>MAN013</t>
+          <t>LDP004</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>MAN015</t>
+          <t>LDP008</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>MAN017</t>
+          <t>LE2851</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>MM4M</t>
+          <t>LE2853</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>MM8M</t>
+          <t>LE2855</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>MM14M</t>
+          <t>LE2857</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>MM32M</t>
+          <t>LE2858</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>MM38M</t>
+          <t>LE2862</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>MM40M</t>
+          <t>LE2863</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>MM42M</t>
+          <t>LZ3114</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>MM44M</t>
+          <t>M437</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>MM48M</t>
+          <t>M865</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>MM52M</t>
+          <t>MAN004</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>MM64M</t>
+          <t>MAN005</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>MM76M</t>
+          <t>MAN007</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>MM78M</t>
+          <t>MAN011</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>MM80M</t>
+          <t>MAN013</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>MM82M</t>
+          <t>MAN015</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>MM84M</t>
+          <t>MAN017</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>MM86M</t>
+          <t>MM02</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>MM94M</t>
+          <t>MM4M</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>MM96M</t>
+          <t>MM8M</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>MM98M</t>
+          <t>MM14M</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>MM99M</t>
+          <t>MM32M</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>MM122M</t>
+          <t>MM38M</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>MM152M</t>
+          <t>MM40M</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>MM158M</t>
+          <t>MM42M</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>MM172M</t>
+          <t>MM44M</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>MM212M</t>
+          <t>MM48M</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>MM214M</t>
+          <t>MM50M</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>MM216M</t>
+          <t>MM52M</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>MM232M</t>
+          <t>MM64M</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>MM236M</t>
+          <t>MM76M</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>MM240M</t>
+          <t>MM78M</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>MM246M</t>
+          <t>MM80M</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>MM260M</t>
+          <t>MM82M</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>MM264M</t>
+          <t>MM84M</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>MM266M</t>
+          <t>MM86M</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>MM270M</t>
+          <t>MM92M</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>MM280M</t>
+          <t>MM94M</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>MM288M</t>
+          <t>MM96M</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>MM380M</t>
+          <t>MM98M</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>MM456M</t>
+          <t>MM99M</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>MM464M</t>
+          <t>MM122M</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>MM478M</t>
+          <t>MM130M</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>MM482M</t>
+          <t>MM152M</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>MM502M</t>
+          <t>MM158M</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>MM506M</t>
+          <t>MM172M</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>MM522M</t>
+          <t>MM212M</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>MM542M</t>
+          <t>MM214M</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>MM546M</t>
+          <t>MM216M</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>MM588M</t>
+          <t>MM232M</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>MM592M</t>
+          <t>MM236M</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>MM624M</t>
+          <t>MM240M</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>MM636M</t>
+          <t>MM246M</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>MM638M</t>
+          <t>MM260M</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>MM647M</t>
+          <t>MM264M</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>MM656M</t>
+          <t>MM266M</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>MM658M</t>
+          <t>MM268M</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>MM660M</t>
+          <t>MM270M</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>MM664M</t>
+          <t>MM280M</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>MM668M</t>
+          <t>MM288M</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>MM673M</t>
+          <t>MM380M</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>MM674M</t>
+          <t>MM456M</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>MM676M</t>
+          <t>MM464M</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>MM680M</t>
+          <t>MM478M</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>MM718M</t>
+          <t>MM482M</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>MM744M</t>
+          <t>MM486M</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>MM752M</t>
+          <t>MM502M</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>MM768M</t>
+          <t>MM506M</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>MM772M</t>
+          <t>MM514M</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>MM774M</t>
+          <t>MM522M</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>MM778M</t>
+          <t>MM536M</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>MM788M</t>
+          <t>MM542M</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>MM798M</t>
+          <t>MM546M</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>MM800M</t>
+          <t>MM588M</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>MM806M</t>
+          <t>MM592M</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>MM808M</t>
+          <t>MM624M</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>MM810M</t>
+          <t>MM636M</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>MM826M</t>
+          <t>MM638M</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>MM830M</t>
+          <t>MM647M</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>MM832M</t>
+          <t>MM656M</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>MM834M</t>
+          <t>MM658M</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>MM838M</t>
+          <t>MM660M</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>MM842M</t>
+          <t>MM664M</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>MM858M</t>
+          <t>MM668M</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>MM860M</t>
+          <t>MM673M</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>MM862M</t>
+          <t>MM674M</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>MM864M</t>
+          <t>MM676M</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>MM872M</t>
+          <t>MM680M</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>MM878M</t>
+          <t>MM718M</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>MM880M</t>
+          <t>MM742M</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>MM886M</t>
+          <t>MM744M</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>MM896M</t>
+          <t>MM752M</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>MM912M</t>
+          <t>MM768M</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>MM914M</t>
+          <t>MM772M</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>MM924M</t>
+          <t>MM774M</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>MM928M</t>
+          <t>MM778M</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>MM934M</t>
+          <t>MM788M</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>MM940M</t>
+          <t>MM798M</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>MM944M</t>
+          <t>MM800M</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>MM946M</t>
+          <t>MM802M</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>MM952M</t>
+          <t>MM806M</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>MM956M</t>
+          <t>MM808M</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>MM958M</t>
+          <t>MM810M</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>MM960M</t>
+          <t>MM816M</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>MM962M</t>
+          <t>MM826M</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>MM964M</t>
+          <t>MM830M</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>MM968M</t>
+          <t>MM832M</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>MM972M</t>
+          <t>MM834M</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>MM974M</t>
+          <t>MM838M</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>MM976M</t>
+          <t>MM842M</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>MM980M</t>
+          <t>MM858M</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>MM982M</t>
+          <t>MM860M</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>MM9901M</t>
+          <t>MM862M</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>MM9903M</t>
+          <t>MM864M</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>MM9906M</t>
+          <t>MM872M</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>MM9908M</t>
+          <t>MM878M</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>MM9910M</t>
+          <t>MM880M</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>MM9912M</t>
+          <t>MM886M</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>MM9914M</t>
+          <t>MM896M</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>MM9918M</t>
+          <t>MM908M</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>MM9920M</t>
+          <t>MM910M</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>MM9924M</t>
+          <t>MM912M</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>MM9926M</t>
+          <t>MM914M</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>MM9927M</t>
+          <t>MM924M</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>MM9928M</t>
+          <t>MM928M</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>MM9929M</t>
+          <t>MM934M</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>MM9931M</t>
+          <t>MM940M</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>MM9936M</t>
+          <t>MM944M</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>MM9937M</t>
+          <t>MM946M</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>MM9938M</t>
+          <t>MM952M</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>MM9941M</t>
+          <t>MM956M</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>MM9943M</t>
+          <t>MM958M</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>MM9946M</t>
+          <t>MM960M</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>MM9947M</t>
+          <t>MM962M</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>MM9948M</t>
+          <t>MM964M</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>MM9952M</t>
+          <t>MM968M</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>MM9957M</t>
+          <t>MM972M</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>MM9958M</t>
+          <t>MM974M</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>MM9959M</t>
+          <t>MM976M</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>MM9960M</t>
+          <t>MM980M</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>MM9961M</t>
+          <t>MM982M</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>MM9963M</t>
+          <t>MM9901M</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>MM9964M</t>
+          <t>MM9903M</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>MM9965M</t>
+          <t>MM9904M</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>MM9966M</t>
+          <t>MM9906M</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>MM9968M</t>
+          <t>MM9908M</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>MM9969M</t>
+          <t>MM9909M</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>MM9970M</t>
+          <t>MM9910M</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MM9912M</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>MTPV1</t>
+          <t>MM9914M</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>MTPV2</t>
+          <t>MM9916M</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>MM9918M</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>MM9920M</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>MM9924M</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>NR6</t>
+          <t>MM9926M</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>NR10</t>
+          <t>MM9927M</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>NR11</t>
+          <t>MM9928M</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>NR13</t>
+          <t>MM9929M</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>NR14</t>
+          <t>MM9931M</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>NR17</t>
+          <t>MM9936M</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>NR20</t>
+          <t>MM9937M</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>NR35</t>
+          <t>MM9938M</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>MM9941M</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>NR46</t>
+          <t>MM9943M</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>MM9946M</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>MM9947M</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>MM9948M</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>MM9952M</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>MM9954M</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>MM9957M</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>MM9958M</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>MM9959M</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>MM9960M</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>MM9961M</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>MM9963M</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>NR107</t>
+          <t>MM9964M</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>MM9965M</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>MM9966M</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>MM9968M</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>MM9969M</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>MM9970M</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>PKLA4</t>
+          <t>MRL001</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>MTPV1</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>MTPV2</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>N466</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>N469</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>NR4</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>NR5</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>NR6</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>NR10</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>NR11</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>NR13</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>NR14</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>QL009</t>
+          <t>NR17</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>QL019</t>
+          <t>NR20</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>NR35</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>QR5400</t>
+          <t>NR37</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>NR46</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>RA2302</t>
+          <t>NR47</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>RA2303</t>
+          <t>NR54</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>NR56</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>NR64</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t>RM93</t>
+          <t>NR65</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>NR68</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t>SCT008</t>
+          <t>NR75</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>NR78</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>NR83</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>SO3</t>
+          <t>NR93</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>NR94</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>NR95</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>NR97</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>T373</t>
+          <t>NR102</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>NR107</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>NR109</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>NR112</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>NR113</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" s="2" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>NR115</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>PB4</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>PKLA4</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
         <is>
-          <t>TT02</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="2" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" s="2" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
         <is>
-          <t>TT105</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="2" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>QE001</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" s="2" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="2" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>QL004</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" s="2" t="inlineStr">
         <is>
-          <t>TT123</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
         <is>
-          <t>TT126</t>
+          <t>QL009</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" s="2" t="inlineStr">
         <is>
-          <t>TT129</t>
+          <t>QL019</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" s="2" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>QR1744</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>QR1771</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="2" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>QR5400</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
         <is>
-          <t>VL13</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="2" t="inlineStr">
         <is>
-          <t>VL22</t>
+          <t>RA2302</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="2" t="inlineStr">
         <is>
-          <t>VL27</t>
+          <t>RA2303</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" s="2" t="inlineStr">
         <is>
-          <t>VL36</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" s="2" t="inlineStr">
         <is>
-          <t>VL38</t>
+          <t>RL301</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" s="2" t="inlineStr">
         <is>
-          <t>VL43</t>
+          <t>RM93</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" s="2" t="inlineStr">
         <is>
-          <t>VL57</t>
+          <t>SCT001</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" s="2" t="inlineStr">
         <is>
-          <t>VL67</t>
+          <t>SCT008</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" s="2" t="inlineStr">
         <is>
-          <t>VL86</t>
+          <t>SCT009</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" s="2" t="inlineStr">
         <is>
-          <t>VL87</t>
+          <t>SCT013</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" s="2" t="inlineStr">
         <is>
-          <t>VL88</t>
+          <t>SO3</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t>VL90</t>
+          <t>SSR102</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" s="2" t="inlineStr">
         <is>
-          <t>VL103</t>
+          <t>SSR103</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
         <is>
-          <t>VL107</t>
+          <t>SSR104</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" s="2" t="inlineStr">
         <is>
-          <t>VL114</t>
+          <t>T373</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" s="2" t="inlineStr">
         <is>
-          <t>VL121</t>
+          <t>TE2801</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" s="2" t="inlineStr">
         <is>
-          <t>VL122</t>
+          <t>TE2803</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
         <is>
-          <t>VL124</t>
+          <t>TE2805</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="2" t="inlineStr">
         <is>
-          <t>VL129</t>
+          <t>TE2807</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
         <is>
-          <t>VL139</t>
+          <t>TE2808</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
         <is>
-          <t>VLINE8013</t>
+          <t>TE2813</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>VLINE8020</t>
+          <t>TE2814</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" s="2" t="inlineStr">
         <is>
-          <t>VLINE8058</t>
+          <t>TJ096</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
         <is>
-          <t>VLINE8059</t>
+          <t>TT02</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" s="2" t="inlineStr">
         <is>
-          <t>VLINE8061</t>
+          <t>TT03</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
         <is>
-          <t>VLINE8102</t>
+          <t>TT04</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" s="2" t="inlineStr">
         <is>
-          <t>VLINE8115</t>
+          <t>TT05</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t>VLINE8120</t>
+          <t>TT08</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t>VLINE8161</t>
+          <t>TT103</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>VLINE8163</t>
+          <t>TT104</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
         <is>
-          <t>VLINE8164</t>
+          <t>TT105</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
         <is>
-          <t>VLINE8172</t>
+          <t>TT107</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
         <is>
-          <t>VLINE8211</t>
+          <t>TT110</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
         <is>
-          <t>VLINE8213</t>
+          <t>TT115</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
         <is>
-          <t>VLINE8226</t>
+          <t>TT117</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>VLINE8228</t>
+          <t>TT123</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
         <is>
-          <t>VLINE8400</t>
+          <t>TT126</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>VLINE8405</t>
+          <t>TT129</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
         <is>
-          <t>VLINE8408</t>
+          <t>TT130</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>VLINE8415</t>
+          <t>TT202</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
         <is>
-          <t>VLINE8457</t>
+          <t>TT206</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>VLINE8459</t>
+          <t>VL13</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
         <is>
-          <t>VLINE8460</t>
+          <t>VL20</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>VLINE8702</t>
+          <t>VL22</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
         <is>
-          <t>VLINE8731</t>
+          <t>VL27</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>VLINE8742</t>
+          <t>VL36</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="2" t="inlineStr">
         <is>
-          <t>VLINE8744</t>
+          <t>VL38</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
         <is>
-          <t>VLINE8750</t>
+          <t>VL43</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" s="2" t="inlineStr">
         <is>
-          <t>VLINE8819</t>
+          <t>VL49</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
         <is>
-          <t>VLINE8863</t>
+          <t>VL57</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" s="2" t="inlineStr">
         <is>
-          <t>XP2001</t>
+          <t>VL67</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="2" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>VL86</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" s="2" t="inlineStr">
         <is>
-          <t>XP2006</t>
+          <t>VL87</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" s="2" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>VL88</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" s="2" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>VL90</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" s="2" t="inlineStr">
         <is>
-          <t>XRN003</t>
+          <t>VL92</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="2" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>VL100</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="2" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>VL103</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="2" t="inlineStr">
         <is>
-          <t>XRN010</t>
+          <t>VL107</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="2" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>VL114</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="2" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>VL121</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" s="2" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>VL122</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" s="2" t="inlineStr">
         <is>
-          <t>XRN022</t>
+          <t>VL124</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" s="2" t="inlineStr">
         <is>
-          <t>XRN028</t>
+          <t>VL126</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" s="2" t="inlineStr">
+        <is>
+          <t>VL129</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="2" t="inlineStr">
+        <is>
+          <t>VL137</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="2" t="inlineStr">
+        <is>
+          <t>VL139</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="2" t="inlineStr">
+        <is>
+          <t>VL354</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8013</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8020</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8058</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8059</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8061</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8071</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8102</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8111</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8115</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8117</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8120</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8122</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8126</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8161</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8163</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8164</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8172</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8181</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8211</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8213</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8215</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8226</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8228</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8400</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8405</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8408</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8415</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8417</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8418</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8457</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8459</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8460</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8702</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8725</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8727</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8731</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8733</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8735</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8742</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8744</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8746</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8748</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8750</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8819</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8863</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="2" t="inlineStr">
+        <is>
+          <t>XP2001</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" s="2" t="inlineStr">
+        <is>
+          <t>XP2005</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="2" t="inlineStr">
+        <is>
+          <t>XP2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" s="2" t="inlineStr">
+        <is>
+          <t>XP2008</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="2" t="inlineStr">
+        <is>
+          <t>XP2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="2" t="inlineStr">
+        <is>
+          <t>XP2013</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="2" t="inlineStr">
+        <is>
+          <t>XP2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" s="2" t="inlineStr">
+        <is>
+          <t>XRN003</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="2" t="inlineStr">
+        <is>
+          <t>XRN005</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" s="2" t="inlineStr">
+        <is>
+          <t>XRN009</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" s="2" t="inlineStr">
+        <is>
+          <t>XRN010</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" s="2" t="inlineStr">
+        <is>
+          <t>XRN017</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" s="2" t="inlineStr">
+        <is>
+          <t>XRN018</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" s="2" t="inlineStr">
+        <is>
+          <t>XRN021</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" s="2" t="inlineStr">
+        <is>
+          <t>XRN022</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" s="2" t="inlineStr">
+        <is>
+          <t>XRN028</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" s="2" t="inlineStr">
         <is>
           <t>XRN029</t>
         </is>

</xml_diff>

<commit_message>
Update RailOps database files - 2026-04-30 01:03:19 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A536"/>
+  <dimension ref="A1:A574"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -510,3694 +510,3960 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>5005</t>
+          <t>4908</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>5009</t>
+          <t>5005</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>5011</t>
+          <t>5009</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>5021</t>
+          <t>5011</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>5025</t>
+          <t>5021</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>5030</t>
+          <t>5025</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>5031</t>
+          <t>5030</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>5032</t>
+          <t>5031</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>5034</t>
+          <t>5032</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>5041</t>
+          <t>5034</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>5042</t>
+          <t>5041</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>6001</t>
+          <t>5042</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>6002</t>
+          <t>6001</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>6003</t>
+          <t>6002</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>6007</t>
+          <t>6003</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>6008</t>
+          <t>6004</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>6011</t>
+          <t>6007</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>6021</t>
+          <t>6008</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>6023</t>
+          <t>6011</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>6025</t>
+          <t>6021</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>6027</t>
+          <t>6023</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>6028</t>
+          <t>6025</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>6029</t>
+          <t>6027</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>6028</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>8114</t>
+          <t>6029</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>8115</t>
+          <t>8030</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>8116</t>
+          <t>8110</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>8124</t>
+          <t>8114</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>8135</t>
+          <t>8115</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>8144</t>
+          <t>8116</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>8152</t>
+          <t>8124</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>8153</t>
+          <t>8135</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>8158</t>
+          <t>8144</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>8161</t>
+          <t>8152</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>8163</t>
+          <t>8153</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>8169</t>
+          <t>8158</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>8172</t>
+          <t>8161</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>8178</t>
+          <t>8163</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>8179</t>
+          <t>8169</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>8202</t>
+          <t>8172</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>8203</t>
+          <t>8178</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>8206</t>
+          <t>8179</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>8207</t>
+          <t>8202</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>8209</t>
+          <t>8203</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>8210</t>
+          <t>8204</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>8215</t>
+          <t>8206</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>8217</t>
+          <t>8207</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>8223</t>
+          <t>8209</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>8225</t>
+          <t>8210</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>8226</t>
+          <t>8215</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>8235</t>
+          <t>8217</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>8239</t>
+          <t>8222</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>8240</t>
+          <t>8223</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>8249</t>
+          <t>8225</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>9025</t>
+          <t>8226</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>9029</t>
+          <t>8228</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>9203</t>
+          <t>8234</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>9301</t>
+          <t>8235</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>9302</t>
+          <t>8239</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>9305</t>
+          <t>8240</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>9307</t>
+          <t>8249</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>9311</t>
+          <t>9025</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>9312</t>
+          <t>9029</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>9313</t>
+          <t>9203</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>9406</t>
+          <t>9301</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>9408</t>
+          <t>9302</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>9410</t>
+          <t>9305</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>42103</t>
+          <t>9307</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>44202</t>
+          <t>9311</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>44204</t>
+          <t>9312</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>44208</t>
+          <t>9313</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>ACB4403</t>
+          <t>9406</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>ACB4404</t>
+          <t>9408</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>ACD6047</t>
+          <t>9410</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>ACD6049</t>
+          <t>42103</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>ACD6052</t>
+          <t>44202</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>ACD6056</t>
+          <t>44204</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>ACD6057</t>
+          <t>44208</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>ACD6058</t>
+          <t>ACB4403</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>ACD6059</t>
+          <t>ACB4404</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>ACD6065</t>
+          <t>ACD6047</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>ACD6066</t>
+          <t>ACD6049</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>ACD6069</t>
+          <t>ACD6052</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>ACD6071</t>
+          <t>ACD6056</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>ACD6073</t>
+          <t>ACD6057</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>ACD6074</t>
+          <t>ACD6058</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>BL26</t>
+          <t>ACD6059</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>BL31</t>
+          <t>ACD6065</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>BL33</t>
+          <t>ACD6066</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>C502</t>
+          <t>ACD6069</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>C504</t>
+          <t>ACD6071</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>C506</t>
+          <t>ACD6073</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>C509</t>
+          <t>ACD6074</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>CEY004</t>
+          <t>BL26</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>CEY006</t>
+          <t>BL31</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>CEY007</t>
+          <t>BL33</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>CF4401</t>
+          <t>C502</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>CF4405</t>
+          <t>C504</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>CF4410</t>
+          <t>C506</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>CF4412</t>
+          <t>C509</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>CF4420</t>
+          <t>CEY004</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>CF4421</t>
+          <t>CEY006</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>CF4424</t>
+          <t>CEY007</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>CF4425</t>
+          <t>CF4401</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>CF4427</t>
+          <t>CF4405</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>CF4429</t>
+          <t>CF4410</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>CLF2</t>
+          <t>CF4412</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>CLP12</t>
+          <t>CF4420</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>CLP13</t>
+          <t>CF4421</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>CM3304</t>
+          <t>CF4424</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>CSR010</t>
+          <t>CF4425</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>CSR015</t>
+          <t>CF4427</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>CSR017</t>
+          <t>CF4429</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>CSR019</t>
+          <t>CLF2</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>CSR020</t>
+          <t>CLP12</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>CSR021</t>
+          <t>CLP13</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>CSR023</t>
+          <t>CM3304</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>DS003</t>
+          <t>CSR010</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>EA2502</t>
+          <t>CSR015</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>EA2503</t>
+          <t>CSR017</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>EA2506</t>
+          <t>CSR019</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>EC2521</t>
+          <t>CSR020</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>EC2525</t>
+          <t>CSR021</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>EC2526</t>
+          <t>CSR023</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>FIE001</t>
+          <t>DS003</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>FIE003</t>
+          <t>EA2502</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>G513</t>
+          <t>EA2503</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>G514</t>
+          <t>EA2506</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>G516</t>
+          <t>EC2521</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>G532</t>
+          <t>EC2525</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>G533</t>
+          <t>EC2526</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>G534</t>
+          <t>FIE001</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>G536</t>
+          <t>FIE003</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>GL103</t>
+          <t>G513</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>GL105</t>
+          <t>G514</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>GL108</t>
+          <t>G516</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>GL111</t>
+          <t>G532</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>GWA002</t>
+          <t>G533</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>GWA004</t>
+          <t>G534</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>GWA008</t>
+          <t>G536</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>GWA009</t>
+          <t>GL103</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>GWB102</t>
+          <t>GL105</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>GWB103</t>
+          <t>GL108</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>GWB104</t>
+          <t>GL111</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>GWU008</t>
+          <t>GWA002</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>GWU013</t>
+          <t>GWA004</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>GWU014</t>
+          <t>GWA008</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>GWU015</t>
+          <t>GWA009</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>HM2701</t>
+          <t>GWB102</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>HM2702</t>
+          <t>GWB103</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>HM2703</t>
+          <t>GWB104</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>HM2705</t>
+          <t>GWU008</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>HM2706</t>
+          <t>GWU013</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>HM2707</t>
+          <t>GWU014</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>HM2753</t>
+          <t>GWU015</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>HM2755</t>
+          <t>HM2701</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>HM2756</t>
+          <t>HM2702</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>HM2757</t>
+          <t>HM2703</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>JP9750</t>
+          <t>HM2705</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>LDP002</t>
+          <t>HM2706</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>LDP004</t>
+          <t>HM2707</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>LDP008</t>
+          <t>HM2752</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>LE2851</t>
+          <t>HM2753</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>LE2853</t>
+          <t>HM2755</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>LE2855</t>
+          <t>HM2756</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>LE2857</t>
+          <t>HM2757</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>LE2858</t>
+          <t>JP9750</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>LE2862</t>
+          <t>LDP002</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>LE2863</t>
+          <t>LDP004</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>LZ3114</t>
+          <t>LDP008</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>M437</t>
+          <t>LE2851</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>M865</t>
+          <t>LE2853</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>MAN004</t>
+          <t>LE2855</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>MAN005</t>
+          <t>LE2857</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>MAN007</t>
+          <t>LE2858</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>MAN011</t>
+          <t>LE2859</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>MAN013</t>
+          <t>LE2862</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>MAN015</t>
+          <t>LE2863</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>MAN017</t>
+          <t>LZ3114</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>MM02</t>
+          <t>M437</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>MM4M</t>
+          <t>M865</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>MM8M</t>
+          <t>MAN004</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>MM14M</t>
+          <t>MAN005</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>MM32M</t>
+          <t>MAN007</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>MM38M</t>
+          <t>MAN011</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>MM40M</t>
+          <t>MAN013</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>MM42M</t>
+          <t>MAN015</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>MM44M</t>
+          <t>MAN016</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>MM48M</t>
+          <t>MAN017</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>MM50M</t>
+          <t>MM02</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>MM52M</t>
+          <t>MM2M</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>MM64M</t>
+          <t>MM4M</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>MM76M</t>
+          <t>MM8M</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>MM78M</t>
+          <t>MM14M</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>MM80M</t>
+          <t>MM32M</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>MM82M</t>
+          <t>MM38M</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>MM84M</t>
+          <t>MM40M</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>MM86M</t>
+          <t>MM42M</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>MM92M</t>
+          <t>MM44M</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>MM94M</t>
+          <t>MM48M</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>MM96M</t>
+          <t>MM50M</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>MM98M</t>
+          <t>MM52M</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>MM99M</t>
+          <t>MM64M</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>MM122M</t>
+          <t>MM76M</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>MM130M</t>
+          <t>MM78M</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>MM152M</t>
+          <t>MM80M</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>MM158M</t>
+          <t>MM82M</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>MM172M</t>
+          <t>MM84M</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>MM212M</t>
+          <t>MM86M</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>MM214M</t>
+          <t>MM92M</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>MM216M</t>
+          <t>MM94M</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>MM232M</t>
+          <t>MM96M</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>MM236M</t>
+          <t>MM98M</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>MM240M</t>
+          <t>MM99M</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>MM246M</t>
+          <t>MM122M</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>MM260M</t>
+          <t>MM130M</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>MM264M</t>
+          <t>MM152M</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>MM266M</t>
+          <t>MM158M</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>MM268M</t>
+          <t>MM172M</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>MM270M</t>
+          <t>MM178M</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>MM280M</t>
+          <t>MM192M</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>MM288M</t>
+          <t>MM212M</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>MM380M</t>
+          <t>MM214M</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>MM456M</t>
+          <t>MM216M</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>MM464M</t>
+          <t>MM232M</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>MM478M</t>
+          <t>MM236M</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>MM482M</t>
+          <t>MM240M</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>MM486M</t>
+          <t>MM246M</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>MM502M</t>
+          <t>MM260M</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>MM506M</t>
+          <t>MM264M</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>MM514M</t>
+          <t>MM266M</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>MM522M</t>
+          <t>MM268M</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>MM536M</t>
+          <t>MM270M</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>MM542M</t>
+          <t>MM280M</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>MM546M</t>
+          <t>MM288M</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>MM588M</t>
+          <t>MM380M</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>MM592M</t>
+          <t>MM456M</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>MM624M</t>
+          <t>MM464M</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>MM636M</t>
+          <t>MM478M</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>MM638M</t>
+          <t>MM482M</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>MM647M</t>
+          <t>MM486M</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>MM656M</t>
+          <t>MM502M</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>MM658M</t>
+          <t>MM506M</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>MM660M</t>
+          <t>MM514M</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>MM664M</t>
+          <t>MM522M</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>MM668M</t>
+          <t>MM536M</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>MM673M</t>
+          <t>MM542M</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>MM674M</t>
+          <t>MM546M</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>MM676M</t>
+          <t>MM574M</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>MM680M</t>
+          <t>MM588M</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>MM718M</t>
+          <t>MM592M</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>MM742M</t>
+          <t>MM604M</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>MM744M</t>
+          <t>MM624M</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>MM752M</t>
+          <t>MM636M</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>MM768M</t>
+          <t>MM638M</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>MM772M</t>
+          <t>MM647M</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>MM774M</t>
+          <t>MM656M</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>MM778M</t>
+          <t>MM658M</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>MM788M</t>
+          <t>MM660M</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>MM798M</t>
+          <t>MM664M</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>MM800M</t>
+          <t>MM668M</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>MM802M</t>
+          <t>MM673M</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>MM806M</t>
+          <t>MM674M</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>MM808M</t>
+          <t>MM676M</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>MM810M</t>
+          <t>MM680M</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>MM816M</t>
+          <t>MM718M</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>MM826M</t>
+          <t>MM742M</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>MM830M</t>
+          <t>MM744M</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>MM832M</t>
+          <t>MM752M</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>MM834M</t>
+          <t>MM768M</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>MM838M</t>
+          <t>MM772M</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>MM842M</t>
+          <t>MM774M</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>MM858M</t>
+          <t>MM778M</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>MM860M</t>
+          <t>MM788M</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>MM862M</t>
+          <t>MM798M</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>MM864M</t>
+          <t>MM800M</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>MM872M</t>
+          <t>MM802M</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>MM878M</t>
+          <t>MM806M</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>MM880M</t>
+          <t>MM808M</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>MM886M</t>
+          <t>MM810M</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>MM896M</t>
+          <t>MM816M</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>MM908M</t>
+          <t>MM826M</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>MM910M</t>
+          <t>MM830M</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>MM912M</t>
+          <t>MM832M</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>MM914M</t>
+          <t>MM834M</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>MM924M</t>
+          <t>MM838M</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>MM928M</t>
+          <t>MM842M</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>MM934M</t>
+          <t>MM858M</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>MM940M</t>
+          <t>MM860M</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>MM944M</t>
+          <t>MM862M</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>MM946M</t>
+          <t>MM864M</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>MM952M</t>
+          <t>MM866M</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>MM956M</t>
+          <t>MM872M</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>MM958M</t>
+          <t>MM878M</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>MM960M</t>
+          <t>MM880M</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>MM962M</t>
+          <t>MM886M</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>MM964M</t>
+          <t>MM896M</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>MM968M</t>
+          <t>MM908M</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>MM972M</t>
+          <t>MM910M</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>MM974M</t>
+          <t>MM912M</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>MM976M</t>
+          <t>MM914M</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>MM980M</t>
+          <t>MM924M</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>MM982M</t>
+          <t>MM928M</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>MM9901M</t>
+          <t>MM934M</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>MM9903M</t>
+          <t>MM940M</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>MM9904M</t>
+          <t>MM944M</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>MM9906M</t>
+          <t>MM946M</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>MM9908M</t>
+          <t>MM952M</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>MM9909M</t>
+          <t>MM956M</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>MM9910M</t>
+          <t>MM958M</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>MM9912M</t>
+          <t>MM960M</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>MM9914M</t>
+          <t>MM962M</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>MM9916M</t>
+          <t>MM964M</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>MM9918M</t>
+          <t>MM968M</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>MM9920M</t>
+          <t>MM972M</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>MM9924M</t>
+          <t>MM974M</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>MM9926M</t>
+          <t>MM976M</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>MM9927M</t>
+          <t>MM980M</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>MM9928M</t>
+          <t>MM982M</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>MM9929M</t>
+          <t>MM9901M</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>MM9931M</t>
+          <t>MM9903M</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>MM9936M</t>
+          <t>MM9904M</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>MM9937M</t>
+          <t>MM9906M</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>MM9938M</t>
+          <t>MM9908M</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>MM9941M</t>
+          <t>MM9909M</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>MM9943M</t>
+          <t>MM9910M</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>MM9946M</t>
+          <t>MM9912M</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>MM9947M</t>
+          <t>MM9914M</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>MM9948M</t>
+          <t>MM9916M</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>MM9952M</t>
+          <t>MM9918M</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>MM9954M</t>
+          <t>MM9920M</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>MM9957M</t>
+          <t>MM9924M</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>MM9958M</t>
+          <t>MM9926M</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>MM9959M</t>
+          <t>MM9927M</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>MM9960M</t>
+          <t>MM9928M</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>MM9961M</t>
+          <t>MM9929M</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>MM9963M</t>
+          <t>MM9931M</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>MM9964M</t>
+          <t>MM9936M</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>MM9965M</t>
+          <t>MM9937M</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>MM9966M</t>
+          <t>MM9938M</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>MM9968M</t>
+          <t>MM9941M</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>MM9969M</t>
+          <t>MM9943M</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>MM9970M</t>
+          <t>MM9946M</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MM9947M</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>MTPV1</t>
+          <t>MM9948M</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>MTPV2</t>
+          <t>MM9952M</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>MM9953M</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>MM9954M</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>MM9957M</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>MM9958M</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>NR6</t>
+          <t>MM9959M</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>NR10</t>
+          <t>MM9960M</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>NR11</t>
+          <t>MM9961M</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>NR13</t>
+          <t>MM9962M</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>NR14</t>
+          <t>MM9963M</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>NR17</t>
+          <t>MM9964M</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>NR20</t>
+          <t>MM9965M</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>NR35</t>
+          <t>MM9966M</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>MM9968M</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>NR46</t>
+          <t>MM9969M</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>MM9970M</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>MRL001</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>NR56</t>
+          <t>MTPV1</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>MTPV2</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>N460</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>N466</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>N469</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR4</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR5</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR6</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR10</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR11</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>NR13</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR14</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
         <is>
-          <t>NR107</t>
+          <t>NR17</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR20</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR35</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR37</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" s="2" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR46</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>NR47</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>NR54</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>PKLA4</t>
+          <t>NR56</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>NR64</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>NR65</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="2" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>NR68</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>NR75</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" s="2" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>NR78</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>NR82</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="2" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>NR83</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" s="2" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>NR91</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="2" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>NR93</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>NR94</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" s="2" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>NR95</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
         <is>
-          <t>QL009</t>
+          <t>NR97</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" s="2" t="inlineStr">
         <is>
-          <t>QL019</t>
+          <t>NR102</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" s="2" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>NR107</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>NR109</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="2" t="inlineStr">
         <is>
-          <t>QR5400</t>
+          <t>NR112</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>NR113</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="2" t="inlineStr">
         <is>
-          <t>RA2302</t>
+          <t>NR115</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="2" t="inlineStr">
         <is>
-          <t>RA2303</t>
+          <t>PB4</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" s="2" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" s="2" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>PKLA4</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" s="2" t="inlineStr">
         <is>
-          <t>RM93</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" s="2" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" s="2" t="inlineStr">
         <is>
-          <t>SCT008</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" s="2" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" s="2" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" s="2" t="inlineStr">
         <is>
-          <t>SO3</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>QE001</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" s="2" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" s="2" t="inlineStr">
         <is>
-          <t>T373</t>
+          <t>QL004</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" s="2" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" s="2" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>QL009</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>QL016</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="2" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>QL019</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>QR1744</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>QR1771</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>QR5400</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" s="2" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
         <is>
-          <t>TT02</t>
+          <t>RA2302</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" s="2" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>RA2303</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" s="2" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>RL301</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>RM93</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>SCT001</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>TT104</t>
+          <t>SCT008</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
         <is>
-          <t>TT105</t>
+          <t>SCT009</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>SCT013</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>SO3</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>SSR102</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>SSR103</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>TT123</t>
+          <t>SSR104</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
         <is>
-          <t>TT126</t>
+          <t>T373</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>TT129</t>
+          <t>TE2801</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TE2803</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TE2805</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TE2807</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>VL13</t>
+          <t>TE2808</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
         <is>
-          <t>VL20</t>
+          <t>TE2813</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>VL22</t>
+          <t>TE2814</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
         <is>
-          <t>VL27</t>
+          <t>TJ096</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>VL36</t>
+          <t>TT02</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="2" t="inlineStr">
         <is>
-          <t>VL38</t>
+          <t>TT03</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
         <is>
-          <t>VL43</t>
+          <t>TT04</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" s="2" t="inlineStr">
         <is>
-          <t>VL49</t>
+          <t>TT05</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
         <is>
-          <t>VL57</t>
+          <t>TT08</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" s="2" t="inlineStr">
         <is>
-          <t>VL67</t>
+          <t>TT103</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="2" t="inlineStr">
         <is>
-          <t>VL86</t>
+          <t>TT104</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" s="2" t="inlineStr">
         <is>
-          <t>VL87</t>
+          <t>TT105</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" s="2" t="inlineStr">
         <is>
-          <t>VL88</t>
+          <t>TT107</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" s="2" t="inlineStr">
         <is>
-          <t>VL90</t>
+          <t>TT110</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" s="2" t="inlineStr">
         <is>
-          <t>VL92</t>
+          <t>TT115</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="2" t="inlineStr">
         <is>
-          <t>VL100</t>
+          <t>TT117</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="2" t="inlineStr">
         <is>
-          <t>VL103</t>
+          <t>TT123</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="2" t="inlineStr">
         <is>
-          <t>VL107</t>
+          <t>TT126</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="2" t="inlineStr">
         <is>
-          <t>VL114</t>
+          <t>TT129</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="2" t="inlineStr">
         <is>
-          <t>VL121</t>
+          <t>TT130</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" s="2" t="inlineStr">
         <is>
-          <t>VL122</t>
+          <t>TT202</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" s="2" t="inlineStr">
         <is>
-          <t>VL124</t>
+          <t>TT206</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" s="2" t="inlineStr">
         <is>
-          <t>VL126</t>
+          <t>VL13</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" s="2" t="inlineStr">
         <is>
-          <t>VL129</t>
+          <t>VL20</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="A472" s="2" t="inlineStr">
         <is>
-          <t>VL137</t>
+          <t>VL22</t>
         </is>
       </c>
     </row>
     <row r="473">
       <c r="A473" s="2" t="inlineStr">
         <is>
-          <t>VL139</t>
+          <t>VL27</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="A474" s="2" t="inlineStr">
         <is>
-          <t>VL354</t>
+          <t>VL36</t>
         </is>
       </c>
     </row>
     <row r="475">
       <c r="A475" s="2" t="inlineStr">
         <is>
-          <t>VLINE8013</t>
+          <t>VL38</t>
         </is>
       </c>
     </row>
     <row r="476">
       <c r="A476" s="2" t="inlineStr">
         <is>
-          <t>VLINE8020</t>
+          <t>VL43</t>
         </is>
       </c>
     </row>
     <row r="477">
       <c r="A477" s="2" t="inlineStr">
         <is>
-          <t>VLINE8058</t>
+          <t>VL49</t>
         </is>
       </c>
     </row>
     <row r="478">
       <c r="A478" s="2" t="inlineStr">
         <is>
-          <t>VLINE8059</t>
+          <t>VL57</t>
         </is>
       </c>
     </row>
     <row r="479">
       <c r="A479" s="2" t="inlineStr">
         <is>
-          <t>VLINE8061</t>
+          <t>VL62</t>
         </is>
       </c>
     </row>
     <row r="480">
       <c r="A480" s="2" t="inlineStr">
         <is>
-          <t>VLINE8071</t>
+          <t>VL67</t>
         </is>
       </c>
     </row>
     <row r="481">
       <c r="A481" s="2" t="inlineStr">
         <is>
-          <t>VLINE8102</t>
+          <t>VL86</t>
         </is>
       </c>
     </row>
     <row r="482">
       <c r="A482" s="2" t="inlineStr">
         <is>
-          <t>VLINE8111</t>
+          <t>VL87</t>
         </is>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="2" t="inlineStr">
         <is>
-          <t>VLINE8115</t>
+          <t>VL88</t>
         </is>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="2" t="inlineStr">
         <is>
-          <t>VLINE8117</t>
+          <t>VL90</t>
         </is>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="2" t="inlineStr">
         <is>
-          <t>VLINE8120</t>
+          <t>VL92</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="2" t="inlineStr">
         <is>
-          <t>VLINE8122</t>
+          <t>VL100</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="2" t="inlineStr">
         <is>
-          <t>VLINE8126</t>
+          <t>VL101</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" s="2" t="inlineStr">
         <is>
-          <t>VLINE8161</t>
+          <t>VL103</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" s="2" t="inlineStr">
         <is>
-          <t>VLINE8163</t>
+          <t>VL107</t>
         </is>
       </c>
     </row>
     <row r="490">
       <c r="A490" s="2" t="inlineStr">
         <is>
-          <t>VLINE8164</t>
+          <t>VL114</t>
         </is>
       </c>
     </row>
     <row r="491">
       <c r="A491" s="2" t="inlineStr">
         <is>
-          <t>VLINE8172</t>
+          <t>VL115</t>
         </is>
       </c>
     </row>
     <row r="492">
       <c r="A492" s="2" t="inlineStr">
         <is>
-          <t>VLINE8181</t>
+          <t>VL121</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="2" t="inlineStr">
         <is>
-          <t>VLINE8211</t>
+          <t>VL122</t>
         </is>
       </c>
     </row>
     <row r="494">
       <c r="A494" s="2" t="inlineStr">
         <is>
-          <t>VLINE8213</t>
+          <t>VL124</t>
         </is>
       </c>
     </row>
     <row r="495">
       <c r="A495" s="2" t="inlineStr">
         <is>
-          <t>VLINE8215</t>
+          <t>VL125</t>
         </is>
       </c>
     </row>
     <row r="496">
       <c r="A496" s="2" t="inlineStr">
         <is>
-          <t>VLINE8226</t>
+          <t>VL126</t>
         </is>
       </c>
     </row>
     <row r="497">
       <c r="A497" s="2" t="inlineStr">
         <is>
-          <t>VLINE8228</t>
+          <t>VL129</t>
         </is>
       </c>
     </row>
     <row r="498">
       <c r="A498" s="2" t="inlineStr">
         <is>
-          <t>VLINE8400</t>
+          <t>VL134</t>
         </is>
       </c>
     </row>
     <row r="499">
       <c r="A499" s="2" t="inlineStr">
         <is>
-          <t>VLINE8405</t>
+          <t>VL137</t>
         </is>
       </c>
     </row>
     <row r="500">
       <c r="A500" s="2" t="inlineStr">
         <is>
-          <t>VLINE8408</t>
+          <t>VL139</t>
         </is>
       </c>
     </row>
     <row r="501">
       <c r="A501" s="2" t="inlineStr">
         <is>
-          <t>VLINE8415</t>
+          <t>VL354</t>
         </is>
       </c>
     </row>
     <row r="502">
       <c r="A502" s="2" t="inlineStr">
         <is>
-          <t>VLINE8417</t>
+          <t>VLINE8013</t>
         </is>
       </c>
     </row>
     <row r="503">
       <c r="A503" s="2" t="inlineStr">
         <is>
-          <t>VLINE8418</t>
+          <t>VLINE8020</t>
         </is>
       </c>
     </row>
     <row r="504">
       <c r="A504" s="2" t="inlineStr">
         <is>
-          <t>VLINE8457</t>
+          <t>VLINE8058</t>
         </is>
       </c>
     </row>
     <row r="505">
       <c r="A505" s="2" t="inlineStr">
         <is>
-          <t>VLINE8459</t>
+          <t>VLINE8059</t>
         </is>
       </c>
     </row>
     <row r="506">
       <c r="A506" s="2" t="inlineStr">
         <is>
-          <t>VLINE8460</t>
+          <t>VLINE8061</t>
         </is>
       </c>
     </row>
     <row r="507">
       <c r="A507" s="2" t="inlineStr">
         <is>
-          <t>VLINE8702</t>
+          <t>VLINE8071</t>
         </is>
       </c>
     </row>
     <row r="508">
       <c r="A508" s="2" t="inlineStr">
         <is>
-          <t>VLINE8725</t>
+          <t>VLINE8072</t>
         </is>
       </c>
     </row>
     <row r="509">
       <c r="A509" s="2" t="inlineStr">
         <is>
-          <t>VLINE8727</t>
+          <t>VLINE8075</t>
         </is>
       </c>
     </row>
     <row r="510">
       <c r="A510" s="2" t="inlineStr">
         <is>
-          <t>VLINE8731</t>
+          <t>VLINE8102</t>
         </is>
       </c>
     </row>
     <row r="511">
       <c r="A511" s="2" t="inlineStr">
         <is>
-          <t>VLINE8733</t>
+          <t>VLINE8111</t>
         </is>
       </c>
     </row>
     <row r="512">
       <c r="A512" s="2" t="inlineStr">
         <is>
-          <t>VLINE8735</t>
+          <t>VLINE8113</t>
         </is>
       </c>
     </row>
     <row r="513">
       <c r="A513" s="2" t="inlineStr">
         <is>
-          <t>VLINE8742</t>
+          <t>VLINE8115</t>
         </is>
       </c>
     </row>
     <row r="514">
       <c r="A514" s="2" t="inlineStr">
         <is>
-          <t>VLINE8744</t>
+          <t>VLINE8117</t>
         </is>
       </c>
     </row>
     <row r="515">
       <c r="A515" s="2" t="inlineStr">
         <is>
-          <t>VLINE8746</t>
+          <t>VLINE8120</t>
         </is>
       </c>
     </row>
     <row r="516">
       <c r="A516" s="2" t="inlineStr">
         <is>
-          <t>VLINE8748</t>
+          <t>VLINE8122</t>
         </is>
       </c>
     </row>
     <row r="517">
       <c r="A517" s="2" t="inlineStr">
         <is>
-          <t>VLINE8750</t>
+          <t>VLINE8124</t>
         </is>
       </c>
     </row>
     <row r="518">
       <c r="A518" s="2" t="inlineStr">
         <is>
-          <t>VLINE8819</t>
+          <t>VLINE8126</t>
         </is>
       </c>
     </row>
     <row r="519">
       <c r="A519" s="2" t="inlineStr">
         <is>
-          <t>VLINE8863</t>
+          <t>VLINE8161</t>
         </is>
       </c>
     </row>
     <row r="520">
       <c r="A520" s="2" t="inlineStr">
         <is>
-          <t>XP2001</t>
+          <t>VLINE8163</t>
         </is>
       </c>
     </row>
     <row r="521">
       <c r="A521" s="2" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>VLINE8164</t>
         </is>
       </c>
     </row>
     <row r="522">
       <c r="A522" s="2" t="inlineStr">
         <is>
-          <t>XP2006</t>
+          <t>VLINE8172</t>
         </is>
       </c>
     </row>
     <row r="523">
       <c r="A523" s="2" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>VLINE8181</t>
         </is>
       </c>
     </row>
     <row r="524">
       <c r="A524" s="2" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>VLINE8211</t>
         </is>
       </c>
     </row>
     <row r="525">
       <c r="A525" s="2" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>VLINE8213</t>
         </is>
       </c>
     </row>
     <row r="526">
       <c r="A526" s="2" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>VLINE8215</t>
         </is>
       </c>
     </row>
     <row r="527">
       <c r="A527" s="2" t="inlineStr">
         <is>
-          <t>XRN003</t>
+          <t>VLINE8217</t>
         </is>
       </c>
     </row>
     <row r="528">
       <c r="A528" s="2" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>VLINE8226</t>
         </is>
       </c>
     </row>
     <row r="529">
       <c r="A529" s="2" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>VLINE8228</t>
         </is>
       </c>
     </row>
     <row r="530">
       <c r="A530" s="2" t="inlineStr">
         <is>
-          <t>XRN010</t>
+          <t>VLINE8230</t>
         </is>
       </c>
     </row>
     <row r="531">
       <c r="A531" s="2" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>VLINE8400</t>
         </is>
       </c>
     </row>
     <row r="532">
       <c r="A532" s="2" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>VLINE8405</t>
         </is>
       </c>
     </row>
     <row r="533">
       <c r="A533" s="2" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>VLINE8408</t>
         </is>
       </c>
     </row>
     <row r="534">
       <c r="A534" s="2" t="inlineStr">
         <is>
-          <t>XRN022</t>
+          <t>VLINE8415</t>
         </is>
       </c>
     </row>
     <row r="535">
       <c r="A535" s="2" t="inlineStr">
         <is>
-          <t>XRN028</t>
+          <t>VLINE8417</t>
         </is>
       </c>
     </row>
     <row r="536">
       <c r="A536" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8418</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8419</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8420</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8457</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8459</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8460</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8702</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8725</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8727</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8729</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8731</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8733</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8735</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8737</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8742</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8744</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8746</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8748</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8750</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8819</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8863</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" s="2" t="inlineStr">
+        <is>
+          <t>VR77</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="2" t="inlineStr">
+        <is>
+          <t>XP2001</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" s="2" t="inlineStr">
+        <is>
+          <t>XP2005</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" s="2" t="inlineStr">
+        <is>
+          <t>XP2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" s="2" t="inlineStr">
+        <is>
+          <t>XP2008</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" s="2" t="inlineStr">
+        <is>
+          <t>XP2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" s="2" t="inlineStr">
+        <is>
+          <t>XP2013</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" s="2" t="inlineStr">
+        <is>
+          <t>XP2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" s="2" t="inlineStr">
+        <is>
+          <t>XRN003</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" s="2" t="inlineStr">
+        <is>
+          <t>XRN005</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" s="2" t="inlineStr">
+        <is>
+          <t>XRN009</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" s="2" t="inlineStr">
+        <is>
+          <t>XRN010</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" s="2" t="inlineStr">
+        <is>
+          <t>XRN017</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" s="2" t="inlineStr">
+        <is>
+          <t>XRN018</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" s="2" t="inlineStr">
+        <is>
+          <t>XRN021</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" s="2" t="inlineStr">
+        <is>
+          <t>XRN022</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" s="2" t="inlineStr">
+        <is>
+          <t>XRN028</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" s="2" t="inlineStr">
         <is>
           <t>XRN029</t>
         </is>

</xml_diff>

<commit_message>
Update RailOps database files - 2026-04-30 01:31:06 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A574"/>
+  <dimension ref="A1:A609"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -741,3729 +741,3974 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>8152</t>
+          <t>8149</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>8153</t>
+          <t>8152</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>8158</t>
+          <t>8153</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>8161</t>
+          <t>8158</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>8163</t>
+          <t>8161</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>8169</t>
+          <t>8163</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>8172</t>
+          <t>8169</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>8178</t>
+          <t>8172</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>8179</t>
+          <t>8178</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>8202</t>
+          <t>8179</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>8203</t>
+          <t>8202</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>8204</t>
+          <t>8203</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>8206</t>
+          <t>8204</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>8207</t>
+          <t>8206</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>8209</t>
+          <t>8207</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>8210</t>
+          <t>8209</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>8215</t>
+          <t>8210</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>8217</t>
+          <t>8215</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>8222</t>
+          <t>8217</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>8223</t>
+          <t>8222</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>8225</t>
+          <t>8223</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>8226</t>
+          <t>8225</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>8228</t>
+          <t>8226</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>8234</t>
+          <t>8228</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>8235</t>
+          <t>8234</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>8239</t>
+          <t>8235</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>8240</t>
+          <t>8239</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>8249</t>
+          <t>8240</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>9025</t>
+          <t>8249</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>9029</t>
+          <t>9025</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>9203</t>
+          <t>9029</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>9301</t>
+          <t>9203</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>9302</t>
+          <t>9301</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>9305</t>
+          <t>9302</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>9307</t>
+          <t>9305</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>9311</t>
+          <t>9307</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>9312</t>
+          <t>9311</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>9313</t>
+          <t>9312</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>9406</t>
+          <t>9313</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>9408</t>
+          <t>9406</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>9410</t>
+          <t>9408</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>42103</t>
+          <t>9410</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>44202</t>
+          <t>42103</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>44204</t>
+          <t>44202</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>44208</t>
+          <t>44204</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>ACB4403</t>
+          <t>44208</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>ACB4404</t>
+          <t>ACB4403</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>ACD6047</t>
+          <t>ACB4404</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>ACD6049</t>
+          <t>ACD6047</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>ACD6052</t>
+          <t>ACD6049</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>ACD6056</t>
+          <t>ACD6052</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>ACD6057</t>
+          <t>ACD6056</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>ACD6058</t>
+          <t>ACD6057</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>ACD6059</t>
+          <t>ACD6058</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>ACD6065</t>
+          <t>ACD6059</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>ACD6066</t>
+          <t>ACD6065</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>ACD6069</t>
+          <t>ACD6066</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>ACD6071</t>
+          <t>ACD6069</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>ACD6073</t>
+          <t>ACD6071</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>ACD6074</t>
+          <t>ACD6073</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>BL26</t>
+          <t>ACD6074</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>BL31</t>
+          <t>BL26</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>BL33</t>
+          <t>BL31</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>C502</t>
+          <t>BL33</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>C504</t>
+          <t>C502</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>C506</t>
+          <t>C504</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>C509</t>
+          <t>C506</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>CEY004</t>
+          <t>C509</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>CEY006</t>
+          <t>CEY004</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>CEY007</t>
+          <t>CEY006</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>CF4401</t>
+          <t>CEY007</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>CF4405</t>
+          <t>CF4401</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>CF4410</t>
+          <t>CF4405</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>CF4412</t>
+          <t>CF4410</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>CF4420</t>
+          <t>CF4412</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>CF4421</t>
+          <t>CF4420</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>CF4424</t>
+          <t>CF4421</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>CF4425</t>
+          <t>CF4424</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>CF4427</t>
+          <t>CF4425</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>CF4429</t>
+          <t>CF4427</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>CLF2</t>
+          <t>CF4429</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>CLP12</t>
+          <t>CLF2</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>CLP13</t>
+          <t>CLP12</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>CM3304</t>
+          <t>CLP13</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>CSR010</t>
+          <t>CM3304</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>CSR015</t>
+          <t>CSR010</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>CSR017</t>
+          <t>CSR015</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>CSR019</t>
+          <t>CSR017</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>CSR020</t>
+          <t>CSR019</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>CSR021</t>
+          <t>CSR020</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>CSR023</t>
+          <t>CSR021</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>DS003</t>
+          <t>CSR023</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>EA2502</t>
+          <t>DS003</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>EA2503</t>
+          <t>EA2502</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>EA2506</t>
+          <t>EA2503</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>EC2521</t>
+          <t>EA2506</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>EC2525</t>
+          <t>EA2507</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>EC2526</t>
+          <t>EC2521</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>FIE001</t>
+          <t>EC2525</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>FIE003</t>
+          <t>EC2526</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>G513</t>
+          <t>FIE001</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>G514</t>
+          <t>FIE003</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>G516</t>
+          <t>G513</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>G532</t>
+          <t>G514</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>G533</t>
+          <t>G516</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>G534</t>
+          <t>G521</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>G536</t>
+          <t>G532</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>GL103</t>
+          <t>G533</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>GL105</t>
+          <t>G534</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>GL108</t>
+          <t>G536</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>GL111</t>
+          <t>GL103</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>GWA002</t>
+          <t>GL105</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>GWA004</t>
+          <t>GL108</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>GWA008</t>
+          <t>GL111</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>GWA009</t>
+          <t>GM46</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>GWB102</t>
+          <t>GWA002</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>GWB103</t>
+          <t>GWA004</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>GWB104</t>
+          <t>GWA008</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>GWU008</t>
+          <t>GWA009</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>GWU013</t>
+          <t>GWB102</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>GWU014</t>
+          <t>GWB103</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>GWU015</t>
+          <t>GWB104</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>HM2701</t>
+          <t>GWU008</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>HM2702</t>
+          <t>GWU013</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>HM2703</t>
+          <t>GWU014</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>HM2705</t>
+          <t>GWU015</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>HM2706</t>
+          <t>HM2701</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>HM2707</t>
+          <t>HM2702</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>HM2752</t>
+          <t>HM2703</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>HM2753</t>
+          <t>HM2705</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>HM2755</t>
+          <t>HM2706</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>HM2756</t>
+          <t>HM2707</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>HM2757</t>
+          <t>HM2751</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>JP9750</t>
+          <t>HM2752</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>LDP002</t>
+          <t>HM2753</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>LDP004</t>
+          <t>HM2755</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>LDP008</t>
+          <t>HM2756</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>LE2851</t>
+          <t>HM2757</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>LE2853</t>
+          <t>JP9750</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>LE2855</t>
+          <t>LDP002</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>LE2857</t>
+          <t>LDP004</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>LE2858</t>
+          <t>LDP008</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>LE2859</t>
+          <t>LE2851</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>LE2862</t>
+          <t>LE2853</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>LE2863</t>
+          <t>LE2855</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>LZ3114</t>
+          <t>LE2857</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>M437</t>
+          <t>LE2858</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>M865</t>
+          <t>LE2859</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>MAN004</t>
+          <t>LE2862</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>MAN005</t>
+          <t>LE2863</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>MAN007</t>
+          <t>LZ3114</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>MAN011</t>
+          <t>M437</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>MAN013</t>
+          <t>M865</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>MAN015</t>
+          <t>MAN004</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>MAN016</t>
+          <t>MAN005</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>MAN017</t>
+          <t>MAN007</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>MM02</t>
+          <t>MAN011</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>MM2M</t>
+          <t>MAN013</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>MM4M</t>
+          <t>MAN015</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>MM8M</t>
+          <t>MAN016</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>MM14M</t>
+          <t>MAN017</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>MM32M</t>
+          <t>MM02</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>MM38M</t>
+          <t>MM2M</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>MM40M</t>
+          <t>MM4M</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>MM42M</t>
+          <t>MM8M</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>MM44M</t>
+          <t>MM14M</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>MM48M</t>
+          <t>MM32M</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>MM50M</t>
+          <t>MM38M</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>MM52M</t>
+          <t>MM40M</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>MM64M</t>
+          <t>MM42M</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>MM76M</t>
+          <t>MM44M</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>MM78M</t>
+          <t>MM48M</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>MM80M</t>
+          <t>MM50M</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>MM82M</t>
+          <t>MM52M</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>MM84M</t>
+          <t>MM64M</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>MM86M</t>
+          <t>MM76M</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>MM92M</t>
+          <t>MM78M</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>MM94M</t>
+          <t>MM80M</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>MM96M</t>
+          <t>MM82M</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>MM98M</t>
+          <t>MM84M</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>MM99M</t>
+          <t>MM86M</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>MM122M</t>
+          <t>MM92M</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>MM130M</t>
+          <t>MM94M</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>MM152M</t>
+          <t>MM96M</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>MM158M</t>
+          <t>MM98M</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>MM172M</t>
+          <t>MM99M</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>MM178M</t>
+          <t>MM122M</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>MM192M</t>
+          <t>MM130M</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>MM212M</t>
+          <t>MM152M</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>MM214M</t>
+          <t>MM156M</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>MM216M</t>
+          <t>MM158M</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>MM232M</t>
+          <t>MM172M</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>MM236M</t>
+          <t>MM178M</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>MM240M</t>
+          <t>MM192M</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>MM246M</t>
+          <t>MM212M</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>MM260M</t>
+          <t>MM214M</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>MM264M</t>
+          <t>MM216M</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>MM266M</t>
+          <t>MM232M</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>MM268M</t>
+          <t>MM236M</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>MM270M</t>
+          <t>MM240M</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>MM280M</t>
+          <t>MM246M</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>MM288M</t>
+          <t>MM260M</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>MM380M</t>
+          <t>MM264M</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>MM456M</t>
+          <t>MM266M</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>MM464M</t>
+          <t>MM268M</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>MM478M</t>
+          <t>MM270M</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>MM482M</t>
+          <t>MM280M</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>MM486M</t>
+          <t>MM288M</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>MM502M</t>
+          <t>MM380M</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>MM506M</t>
+          <t>MM456M</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>MM514M</t>
+          <t>MM464M</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>MM522M</t>
+          <t>MM478M</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>MM536M</t>
+          <t>MM482M</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>MM542M</t>
+          <t>MM486M</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>MM546M</t>
+          <t>MM502M</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>MM574M</t>
+          <t>MM506M</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>MM588M</t>
+          <t>MM514M</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>MM592M</t>
+          <t>MM522M</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>MM604M</t>
+          <t>MM536M</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>MM624M</t>
+          <t>MM542M</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>MM636M</t>
+          <t>MM544M</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>MM638M</t>
+          <t>MM546M</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>MM647M</t>
+          <t>MM551M</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>MM656M</t>
+          <t>MM574M</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>MM658M</t>
+          <t>MM588M</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>MM660M</t>
+          <t>MM592M</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>MM664M</t>
+          <t>MM604M</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>MM668M</t>
+          <t>MM624M</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>MM673M</t>
+          <t>MM636M</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>MM674M</t>
+          <t>MM638M</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>MM676M</t>
+          <t>MM647M</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>MM680M</t>
+          <t>MM656M</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>MM718M</t>
+          <t>MM658M</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>MM742M</t>
+          <t>MM660M</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>MM744M</t>
+          <t>MM664M</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>MM752M</t>
+          <t>MM668M</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>MM768M</t>
+          <t>MM673M</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>MM772M</t>
+          <t>MM674M</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>MM774M</t>
+          <t>MM676M</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>MM778M</t>
+          <t>MM680M</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>MM788M</t>
+          <t>MM702M</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>MM798M</t>
+          <t>MM718M</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>MM800M</t>
+          <t>MM742M</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>MM802M</t>
+          <t>MM744M</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>MM806M</t>
+          <t>MM752M</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>MM808M</t>
+          <t>MM768M</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>MM810M</t>
+          <t>MM772M</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>MM816M</t>
+          <t>MM774M</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>MM826M</t>
+          <t>MM776M</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>MM830M</t>
+          <t>MM778M</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>MM832M</t>
+          <t>MM788M</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>MM834M</t>
+          <t>MM794M</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>MM838M</t>
+          <t>MM798M</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>MM842M</t>
+          <t>MM800M</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>MM858M</t>
+          <t>MM802M</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>MM860M</t>
+          <t>MM806M</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>MM862M</t>
+          <t>MM808M</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>MM864M</t>
+          <t>MM810M</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>MM866M</t>
+          <t>MM816M</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>MM872M</t>
+          <t>MM826M</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>MM878M</t>
+          <t>MM830M</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>MM880M</t>
+          <t>MM832M</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>MM886M</t>
+          <t>MM834M</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>MM896M</t>
+          <t>MM838M</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>MM908M</t>
+          <t>MM842M</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>MM910M</t>
+          <t>MM858M</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>MM912M</t>
+          <t>MM860M</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>MM914M</t>
+          <t>MM862M</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>MM924M</t>
+          <t>MM864M</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>MM928M</t>
+          <t>MM866M</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>MM934M</t>
+          <t>MM872M</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>MM940M</t>
+          <t>MM878M</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>MM944M</t>
+          <t>MM880M</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>MM946M</t>
+          <t>MM886M</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>MM952M</t>
+          <t>MM896M</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>MM956M</t>
+          <t>MM908M</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>MM958M</t>
+          <t>MM910M</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>MM960M</t>
+          <t>MM912M</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>MM962M</t>
+          <t>MM914M</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>MM964M</t>
+          <t>MM924M</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>MM968M</t>
+          <t>MM928M</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>MM972M</t>
+          <t>MM934M</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>MM974M</t>
+          <t>MM940M</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>MM976M</t>
+          <t>MM944M</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>MM980M</t>
+          <t>MM946M</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>MM982M</t>
+          <t>MM952M</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>MM9901M</t>
+          <t>MM956M</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>MM9903M</t>
+          <t>MM958M</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>MM9904M</t>
+          <t>MM960M</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>MM9906M</t>
+          <t>MM962M</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>MM9908M</t>
+          <t>MM964M</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>MM9909M</t>
+          <t>MM968M</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>MM9910M</t>
+          <t>MM972M</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>MM9912M</t>
+          <t>MM974M</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>MM9914M</t>
+          <t>MM976M</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>MM9916M</t>
+          <t>MM980M</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>MM9918M</t>
+          <t>MM982M</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>MM9920M</t>
+          <t>MM9901M</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>MM9924M</t>
+          <t>MM9903M</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>MM9926M</t>
+          <t>MM9904M</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>MM9927M</t>
+          <t>MM9906M</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>MM9928M</t>
+          <t>MM9908M</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>MM9929M</t>
+          <t>MM9909M</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>MM9931M</t>
+          <t>MM9910M</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>MM9936M</t>
+          <t>MM9912M</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>MM9937M</t>
+          <t>MM9914M</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>MM9938M</t>
+          <t>MM9916M</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>MM9941M</t>
+          <t>MM9918M</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>MM9943M</t>
+          <t>MM9920M</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>MM9946M</t>
+          <t>MM9921M</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>MM9947M</t>
+          <t>MM9924M</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>MM9948M</t>
+          <t>MM9926M</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>MM9952M</t>
+          <t>MM9927M</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>MM9953M</t>
+          <t>MM9928M</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>MM9954M</t>
+          <t>MM9929M</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>MM9957M</t>
+          <t>MM9931M</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>MM9958M</t>
+          <t>MM9936M</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>MM9959M</t>
+          <t>MM9937M</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>MM9960M</t>
+          <t>MM9938M</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>MM9961M</t>
+          <t>MM9941M</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>MM9962M</t>
+          <t>MM9943M</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>MM9963M</t>
+          <t>MM9946M</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>MM9964M</t>
+          <t>MM9947M</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>MM9965M</t>
+          <t>MM9948M</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>MM9966M</t>
+          <t>MM9952M</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>MM9968M</t>
+          <t>MM9953M</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>MM9969M</t>
+          <t>MM9954M</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>MM9970M</t>
+          <t>MM9956M</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MM9957M</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>MTPV1</t>
+          <t>MM9958M</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>MTPV2</t>
+          <t>MM9959M</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t>N460</t>
+          <t>MM9960M</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>MM9961M</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>MM9962M</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>MM9963M</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>MM9964M</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>NR6</t>
+          <t>MM9965M</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>NR10</t>
+          <t>MM9966M</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>NR11</t>
+          <t>MM9968M</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>NR13</t>
+          <t>MM9969M</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>NR14</t>
+          <t>MM9970M</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
         <is>
-          <t>NR17</t>
+          <t>MRL001</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>NR20</t>
+          <t>MTPV1</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
         <is>
-          <t>NR35</t>
+          <t>MTPV2</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>N458</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" s="2" t="inlineStr">
         <is>
-          <t>NR46</t>
+          <t>N460</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>N466</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>N469</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>NR56</t>
+          <t>NR4</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR5</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR6</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="2" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR10</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR11</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" s="2" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR12</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR13</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="2" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR14</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" s="2" t="inlineStr">
         <is>
-          <t>NR91</t>
+          <t>NR17</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="2" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR20</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR35</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" s="2" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR37</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>NR44</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" s="2" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR46</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" s="2" t="inlineStr">
         <is>
-          <t>NR107</t>
+          <t>NR47</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR54</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="2" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR56</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR64</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="2" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR65</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="2" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>NR68</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" s="2" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>NR75</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" s="2" t="inlineStr">
         <is>
-          <t>PKLA4</t>
+          <t>NR76</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" s="2" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>NR78</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" s="2" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>NR82</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" s="2" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>NR83</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" s="2" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>NR88</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" s="2" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>NR91</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" s="2" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>NR93</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>NR94</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" s="2" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>NR95</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>NR97</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" s="2" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>NR102</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" s="2" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>NR107</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" s="2" t="inlineStr">
         <is>
-          <t>QL009</t>
+          <t>NR109</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
         <is>
-          <t>QL016</t>
+          <t>NR112</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="2" t="inlineStr">
         <is>
-          <t>QL019</t>
+          <t>NR113</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>NR115</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>PB4</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>QR5400</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" s="2" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>PKLA4</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
         <is>
-          <t>RA2302</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" s="2" t="inlineStr">
         <is>
-          <t>RA2303</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" s="2" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t>RM93</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>SCT008</t>
+          <t>QE001</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
         <is>
-          <t>SO3</t>
+          <t>QL004</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>QL009</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>QL016</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
         <is>
-          <t>T373</t>
+          <t>QL019</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>QR1744</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>QR1771</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>QR5400</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>RA2302</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>RA2303</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>RL301</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>TT02</t>
+          <t>RM93</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="2" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>SCT001</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>SCT008</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" s="2" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>SCT009</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>SCT013</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" s="2" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>SO3</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="2" t="inlineStr">
         <is>
-          <t>TT104</t>
+          <t>SSR102</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" s="2" t="inlineStr">
         <is>
-          <t>TT105</t>
+          <t>SSR103</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" s="2" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>SSR104</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" s="2" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>T373</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" s="2" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TE2801</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="2" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TE2803</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="2" t="inlineStr">
         <is>
-          <t>TT123</t>
+          <t>TE2805</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="2" t="inlineStr">
         <is>
-          <t>TT126</t>
+          <t>TE2807</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="2" t="inlineStr">
         <is>
-          <t>TT129</t>
+          <t>TE2808</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="2" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TE2813</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" s="2" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TE2814</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" s="2" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TJ096</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" s="2" t="inlineStr">
         <is>
-          <t>VL13</t>
+          <t>TT02</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" s="2" t="inlineStr">
         <is>
-          <t>VL20</t>
+          <t>TT03</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="A472" s="2" t="inlineStr">
         <is>
-          <t>VL22</t>
+          <t>TT04</t>
         </is>
       </c>
     </row>
     <row r="473">
       <c r="A473" s="2" t="inlineStr">
         <is>
-          <t>VL27</t>
+          <t>TT05</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="A474" s="2" t="inlineStr">
         <is>
-          <t>VL36</t>
+          <t>TT08</t>
         </is>
       </c>
     </row>
     <row r="475">
       <c r="A475" s="2" t="inlineStr">
         <is>
-          <t>VL38</t>
+          <t>TT103</t>
         </is>
       </c>
     </row>
     <row r="476">
       <c r="A476" s="2" t="inlineStr">
         <is>
-          <t>VL43</t>
+          <t>TT104</t>
         </is>
       </c>
     </row>
     <row r="477">
       <c r="A477" s="2" t="inlineStr">
         <is>
-          <t>VL49</t>
+          <t>TT105</t>
         </is>
       </c>
     </row>
     <row r="478">
       <c r="A478" s="2" t="inlineStr">
         <is>
-          <t>VL57</t>
+          <t>TT107</t>
         </is>
       </c>
     </row>
     <row r="479">
       <c r="A479" s="2" t="inlineStr">
         <is>
-          <t>VL62</t>
+          <t>TT110</t>
         </is>
       </c>
     </row>
     <row r="480">
       <c r="A480" s="2" t="inlineStr">
         <is>
-          <t>VL67</t>
+          <t>TT115</t>
         </is>
       </c>
     </row>
     <row r="481">
       <c r="A481" s="2" t="inlineStr">
         <is>
-          <t>VL86</t>
+          <t>TT117</t>
         </is>
       </c>
     </row>
     <row r="482">
       <c r="A482" s="2" t="inlineStr">
         <is>
-          <t>VL87</t>
+          <t>TT123</t>
         </is>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="2" t="inlineStr">
         <is>
-          <t>VL88</t>
+          <t>TT126</t>
         </is>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="2" t="inlineStr">
         <is>
-          <t>VL90</t>
+          <t>TT129</t>
         </is>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="2" t="inlineStr">
         <is>
-          <t>VL92</t>
+          <t>TT130</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="2" t="inlineStr">
         <is>
-          <t>VL100</t>
+          <t>TT202</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="2" t="inlineStr">
         <is>
-          <t>VL101</t>
+          <t>TT206</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" s="2" t="inlineStr">
         <is>
-          <t>VL103</t>
+          <t>VL04</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" s="2" t="inlineStr">
         <is>
-          <t>VL107</t>
+          <t>VL11</t>
         </is>
       </c>
     </row>
     <row r="490">
       <c r="A490" s="2" t="inlineStr">
         <is>
-          <t>VL114</t>
+          <t>VL13</t>
         </is>
       </c>
     </row>
     <row r="491">
       <c r="A491" s="2" t="inlineStr">
         <is>
-          <t>VL115</t>
+          <t>VL20</t>
         </is>
       </c>
     </row>
     <row r="492">
       <c r="A492" s="2" t="inlineStr">
         <is>
-          <t>VL121</t>
+          <t>VL22</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="2" t="inlineStr">
         <is>
-          <t>VL122</t>
+          <t>VL27</t>
         </is>
       </c>
     </row>
     <row r="494">
       <c r="A494" s="2" t="inlineStr">
         <is>
-          <t>VL124</t>
+          <t>VL36</t>
         </is>
       </c>
     </row>
     <row r="495">
       <c r="A495" s="2" t="inlineStr">
         <is>
-          <t>VL125</t>
+          <t>VL38</t>
         </is>
       </c>
     </row>
     <row r="496">
       <c r="A496" s="2" t="inlineStr">
         <is>
-          <t>VL126</t>
+          <t>VL43</t>
         </is>
       </c>
     </row>
     <row r="497">
       <c r="A497" s="2" t="inlineStr">
         <is>
-          <t>VL129</t>
+          <t>VL49</t>
         </is>
       </c>
     </row>
     <row r="498">
       <c r="A498" s="2" t="inlineStr">
         <is>
-          <t>VL134</t>
+          <t>VL57</t>
         </is>
       </c>
     </row>
     <row r="499">
       <c r="A499" s="2" t="inlineStr">
         <is>
-          <t>VL137</t>
+          <t>VL62</t>
         </is>
       </c>
     </row>
     <row r="500">
       <c r="A500" s="2" t="inlineStr">
         <is>
-          <t>VL139</t>
+          <t>VL67</t>
         </is>
       </c>
     </row>
     <row r="501">
       <c r="A501" s="2" t="inlineStr">
         <is>
-          <t>VL354</t>
+          <t>VL81</t>
         </is>
       </c>
     </row>
     <row r="502">
       <c r="A502" s="2" t="inlineStr">
         <is>
-          <t>VLINE8013</t>
+          <t>VL86</t>
         </is>
       </c>
     </row>
     <row r="503">
       <c r="A503" s="2" t="inlineStr">
         <is>
-          <t>VLINE8020</t>
+          <t>VL87</t>
         </is>
       </c>
     </row>
     <row r="504">
       <c r="A504" s="2" t="inlineStr">
         <is>
-          <t>VLINE8058</t>
+          <t>VL88</t>
         </is>
       </c>
     </row>
     <row r="505">
       <c r="A505" s="2" t="inlineStr">
         <is>
-          <t>VLINE8059</t>
+          <t>VL90</t>
         </is>
       </c>
     </row>
     <row r="506">
       <c r="A506" s="2" t="inlineStr">
         <is>
-          <t>VLINE8061</t>
+          <t>VL92</t>
         </is>
       </c>
     </row>
     <row r="507">
       <c r="A507" s="2" t="inlineStr">
         <is>
-          <t>VLINE8071</t>
+          <t>VL99</t>
         </is>
       </c>
     </row>
     <row r="508">
       <c r="A508" s="2" t="inlineStr">
         <is>
-          <t>VLINE8072</t>
+          <t>VL100</t>
         </is>
       </c>
     </row>
     <row r="509">
       <c r="A509" s="2" t="inlineStr">
         <is>
-          <t>VLINE8075</t>
+          <t>VL101</t>
         </is>
       </c>
     </row>
     <row r="510">
       <c r="A510" s="2" t="inlineStr">
         <is>
-          <t>VLINE8102</t>
+          <t>VL103</t>
         </is>
       </c>
     </row>
     <row r="511">
       <c r="A511" s="2" t="inlineStr">
         <is>
-          <t>VLINE8111</t>
+          <t>VL107</t>
         </is>
       </c>
     </row>
     <row r="512">
       <c r="A512" s="2" t="inlineStr">
         <is>
-          <t>VLINE8113</t>
+          <t>VL112</t>
         </is>
       </c>
     </row>
     <row r="513">
       <c r="A513" s="2" t="inlineStr">
         <is>
-          <t>VLINE8115</t>
+          <t>VL114</t>
         </is>
       </c>
     </row>
     <row r="514">
       <c r="A514" s="2" t="inlineStr">
         <is>
-          <t>VLINE8117</t>
+          <t>VL115</t>
         </is>
       </c>
     </row>
     <row r="515">
       <c r="A515" s="2" t="inlineStr">
         <is>
-          <t>VLINE8120</t>
+          <t>VL121</t>
         </is>
       </c>
     </row>
     <row r="516">
       <c r="A516" s="2" t="inlineStr">
         <is>
-          <t>VLINE8122</t>
+          <t>VL122</t>
         </is>
       </c>
     </row>
     <row r="517">
       <c r="A517" s="2" t="inlineStr">
         <is>
-          <t>VLINE8124</t>
+          <t>VL124</t>
         </is>
       </c>
     </row>
     <row r="518">
       <c r="A518" s="2" t="inlineStr">
         <is>
-          <t>VLINE8126</t>
+          <t>VL125</t>
         </is>
       </c>
     </row>
     <row r="519">
       <c r="A519" s="2" t="inlineStr">
         <is>
-          <t>VLINE8161</t>
+          <t>VL126</t>
         </is>
       </c>
     </row>
     <row r="520">
       <c r="A520" s="2" t="inlineStr">
         <is>
-          <t>VLINE8163</t>
+          <t>VL129</t>
         </is>
       </c>
     </row>
     <row r="521">
       <c r="A521" s="2" t="inlineStr">
         <is>
-          <t>VLINE8164</t>
+          <t>VL134</t>
         </is>
       </c>
     </row>
     <row r="522">
       <c r="A522" s="2" t="inlineStr">
         <is>
-          <t>VLINE8172</t>
+          <t>VL137</t>
         </is>
       </c>
     </row>
     <row r="523">
       <c r="A523" s="2" t="inlineStr">
         <is>
-          <t>VLINE8181</t>
+          <t>VL139</t>
         </is>
       </c>
     </row>
     <row r="524">
       <c r="A524" s="2" t="inlineStr">
         <is>
-          <t>VLINE8211</t>
+          <t>VL354</t>
         </is>
       </c>
     </row>
     <row r="525">
       <c r="A525" s="2" t="inlineStr">
         <is>
-          <t>VLINE8213</t>
+          <t>VLINE8013</t>
         </is>
       </c>
     </row>
     <row r="526">
       <c r="A526" s="2" t="inlineStr">
         <is>
-          <t>VLINE8215</t>
+          <t>VLINE8020</t>
         </is>
       </c>
     </row>
     <row r="527">
       <c r="A527" s="2" t="inlineStr">
         <is>
-          <t>VLINE8217</t>
+          <t>VLINE8058</t>
         </is>
       </c>
     </row>
     <row r="528">
       <c r="A528" s="2" t="inlineStr">
         <is>
-          <t>VLINE8226</t>
+          <t>VLINE8059</t>
         </is>
       </c>
     </row>
     <row r="529">
       <c r="A529" s="2" t="inlineStr">
         <is>
-          <t>VLINE8228</t>
+          <t>VLINE8061</t>
         </is>
       </c>
     </row>
     <row r="530">
       <c r="A530" s="2" t="inlineStr">
         <is>
-          <t>VLINE8230</t>
+          <t>VLINE8071</t>
         </is>
       </c>
     </row>
     <row r="531">
       <c r="A531" s="2" t="inlineStr">
         <is>
-          <t>VLINE8400</t>
+          <t>VLINE8072</t>
         </is>
       </c>
     </row>
     <row r="532">
       <c r="A532" s="2" t="inlineStr">
         <is>
-          <t>VLINE8405</t>
+          <t>VLINE8075</t>
         </is>
       </c>
     </row>
     <row r="533">
       <c r="A533" s="2" t="inlineStr">
         <is>
-          <t>VLINE8408</t>
+          <t>VLINE8080</t>
         </is>
       </c>
     </row>
     <row r="534">
       <c r="A534" s="2" t="inlineStr">
         <is>
-          <t>VLINE8415</t>
+          <t>VLINE8102</t>
         </is>
       </c>
     </row>
     <row r="535">
       <c r="A535" s="2" t="inlineStr">
         <is>
-          <t>VLINE8417</t>
+          <t>VLINE8111</t>
         </is>
       </c>
     </row>
     <row r="536">
       <c r="A536" s="2" t="inlineStr">
         <is>
-          <t>VLINE8418</t>
+          <t>VLINE8113</t>
         </is>
       </c>
     </row>
     <row r="537">
       <c r="A537" s="2" t="inlineStr">
         <is>
-          <t>VLINE8419</t>
+          <t>VLINE8115</t>
         </is>
       </c>
     </row>
     <row r="538">
       <c r="A538" s="2" t="inlineStr">
         <is>
-          <t>VLINE8420</t>
+          <t>VLINE8117</t>
         </is>
       </c>
     </row>
     <row r="539">
       <c r="A539" s="2" t="inlineStr">
         <is>
-          <t>VLINE8457</t>
+          <t>VLINE8120</t>
         </is>
       </c>
     </row>
     <row r="540">
       <c r="A540" s="2" t="inlineStr">
         <is>
-          <t>VLINE8459</t>
+          <t>VLINE8122</t>
         </is>
       </c>
     </row>
     <row r="541">
       <c r="A541" s="2" t="inlineStr">
         <is>
-          <t>VLINE8460</t>
+          <t>VLINE8124</t>
         </is>
       </c>
     </row>
     <row r="542">
       <c r="A542" s="2" t="inlineStr">
         <is>
-          <t>VLINE8702</t>
+          <t>VLINE8126</t>
         </is>
       </c>
     </row>
     <row r="543">
       <c r="A543" s="2" t="inlineStr">
         <is>
-          <t>VLINE8725</t>
+          <t>VLINE8161</t>
         </is>
       </c>
     </row>
     <row r="544">
       <c r="A544" s="2" t="inlineStr">
         <is>
-          <t>VLINE8727</t>
+          <t>VLINE8163</t>
         </is>
       </c>
     </row>
     <row r="545">
       <c r="A545" s="2" t="inlineStr">
         <is>
-          <t>VLINE8729</t>
+          <t>VLINE8164</t>
         </is>
       </c>
     </row>
     <row r="546">
       <c r="A546" s="2" t="inlineStr">
         <is>
-          <t>VLINE8731</t>
+          <t>VLINE8172</t>
         </is>
       </c>
     </row>
     <row r="547">
       <c r="A547" s="2" t="inlineStr">
         <is>
-          <t>VLINE8733</t>
+          <t>VLINE8181</t>
         </is>
       </c>
     </row>
     <row r="548">
       <c r="A548" s="2" t="inlineStr">
         <is>
-          <t>VLINE8735</t>
+          <t>VLINE8183</t>
         </is>
       </c>
     </row>
     <row r="549">
       <c r="A549" s="2" t="inlineStr">
         <is>
-          <t>VLINE8737</t>
+          <t>VLINE8211</t>
         </is>
       </c>
     </row>
     <row r="550">
       <c r="A550" s="2" t="inlineStr">
         <is>
-          <t>VLINE8742</t>
+          <t>VLINE8213</t>
         </is>
       </c>
     </row>
     <row r="551">
       <c r="A551" s="2" t="inlineStr">
         <is>
-          <t>VLINE8744</t>
+          <t>VLINE8215</t>
         </is>
       </c>
     </row>
     <row r="552">
       <c r="A552" s="2" t="inlineStr">
         <is>
-          <t>VLINE8746</t>
+          <t>VLINE8217</t>
         </is>
       </c>
     </row>
     <row r="553">
       <c r="A553" s="2" t="inlineStr">
         <is>
-          <t>VLINE8748</t>
+          <t>VLINE8219</t>
         </is>
       </c>
     </row>
     <row r="554">
       <c r="A554" s="2" t="inlineStr">
         <is>
-          <t>VLINE8750</t>
+          <t>VLINE8226</t>
         </is>
       </c>
     </row>
     <row r="555">
       <c r="A555" s="2" t="inlineStr">
         <is>
-          <t>VLINE8819</t>
+          <t>VLINE8228</t>
         </is>
       </c>
     </row>
     <row r="556">
       <c r="A556" s="2" t="inlineStr">
         <is>
-          <t>VLINE8863</t>
+          <t>VLINE8230</t>
         </is>
       </c>
     </row>
     <row r="557">
       <c r="A557" s="2" t="inlineStr">
         <is>
-          <t>VR77</t>
+          <t>VLINE8232</t>
         </is>
       </c>
     </row>
     <row r="558">
       <c r="A558" s="2" t="inlineStr">
         <is>
-          <t>XP2001</t>
+          <t>VLINE8400</t>
         </is>
       </c>
     </row>
     <row r="559">
       <c r="A559" s="2" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>VLINE8405</t>
         </is>
       </c>
     </row>
     <row r="560">
       <c r="A560" s="2" t="inlineStr">
         <is>
-          <t>XP2006</t>
+          <t>VLINE8408</t>
         </is>
       </c>
     </row>
     <row r="561">
       <c r="A561" s="2" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>VLINE8413</t>
         </is>
       </c>
     </row>
     <row r="562">
       <c r="A562" s="2" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>VLINE8415</t>
         </is>
       </c>
     </row>
     <row r="563">
       <c r="A563" s="2" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>VLINE8417</t>
         </is>
       </c>
     </row>
     <row r="564">
       <c r="A564" s="2" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>VLINE8418</t>
         </is>
       </c>
     </row>
     <row r="565">
       <c r="A565" s="2" t="inlineStr">
         <is>
-          <t>XRN003</t>
+          <t>VLINE8419</t>
         </is>
       </c>
     </row>
     <row r="566">
       <c r="A566" s="2" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>VLINE8420</t>
         </is>
       </c>
     </row>
     <row r="567">
       <c r="A567" s="2" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>VLINE8421</t>
         </is>
       </c>
     </row>
     <row r="568">
       <c r="A568" s="2" t="inlineStr">
         <is>
-          <t>XRN010</t>
+          <t>VLINE8457</t>
         </is>
       </c>
     </row>
     <row r="569">
       <c r="A569" s="2" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>VLINE8459</t>
         </is>
       </c>
     </row>
     <row r="570">
       <c r="A570" s="2" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>VLINE8460</t>
         </is>
       </c>
     </row>
     <row r="571">
       <c r="A571" s="2" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>VLINE8702</t>
         </is>
       </c>
     </row>
     <row r="572">
       <c r="A572" s="2" t="inlineStr">
         <is>
-          <t>XRN022</t>
+          <t>VLINE8725</t>
         </is>
       </c>
     </row>
     <row r="573">
       <c r="A573" s="2" t="inlineStr">
         <is>
-          <t>XRN028</t>
+          <t>VLINE8727</t>
         </is>
       </c>
     </row>
     <row r="574">
       <c r="A574" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8729</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8731</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8733</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8735</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8737</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8739</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8741</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8742</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8744</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8746</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8748</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8750</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8752</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8754</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8819</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8863</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" s="2" t="inlineStr">
+        <is>
+          <t>VR77</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" s="2" t="inlineStr">
+        <is>
+          <t>XP2001</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" s="2" t="inlineStr">
+        <is>
+          <t>XP2005</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" s="2" t="inlineStr">
+        <is>
+          <t>XP2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" s="2" t="inlineStr">
+        <is>
+          <t>XP2008</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" s="2" t="inlineStr">
+        <is>
+          <t>XP2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" s="2" t="inlineStr">
+        <is>
+          <t>XP2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" s="2" t="inlineStr">
+        <is>
+          <t>XP2013</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" s="2" t="inlineStr">
+        <is>
+          <t>XP2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" s="2" t="inlineStr">
+        <is>
+          <t>XP2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" s="2" t="inlineStr">
+        <is>
+          <t>XRN003</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" s="2" t="inlineStr">
+        <is>
+          <t>XRN005</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" s="2" t="inlineStr">
+        <is>
+          <t>XRN009</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" s="2" t="inlineStr">
+        <is>
+          <t>XRN010</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="2" t="inlineStr">
+        <is>
+          <t>XRN017</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" s="2" t="inlineStr">
+        <is>
+          <t>XRN018</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="2" t="inlineStr">
+        <is>
+          <t>XRN021</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" s="2" t="inlineStr">
+        <is>
+          <t>XRN022</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" s="2" t="inlineStr">
+        <is>
+          <t>XRN028</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" s="2" t="inlineStr">
         <is>
           <t>XRN029</t>
         </is>

</xml_diff>

<commit_message>
Update RailOps database files - 2026-04-30 02:02:42 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A609"/>
+  <dimension ref="A1:A628"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -573,4142 +573,4275 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>5034</t>
+          <t>5033</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>5041</t>
+          <t>5034</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>5042</t>
+          <t>5041</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>6001</t>
+          <t>5042</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>6002</t>
+          <t>6001</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>6003</t>
+          <t>6002</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>6004</t>
+          <t>6003</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>6007</t>
+          <t>6004</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>6008</t>
+          <t>6007</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>6011</t>
+          <t>6008</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>6021</t>
+          <t>6011</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>6023</t>
+          <t>6021</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>6025</t>
+          <t>6023</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>6027</t>
+          <t>6025</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>6028</t>
+          <t>6027</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>6029</t>
+          <t>6028</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>6029</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>8110</t>
+          <t>8030</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>8114</t>
+          <t>8110</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>8115</t>
+          <t>8114</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>8116</t>
+          <t>8115</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>8124</t>
+          <t>8116</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>8135</t>
+          <t>8124</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>8144</t>
+          <t>8135</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>8149</t>
+          <t>8144</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>8152</t>
+          <t>8149</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>8153</t>
+          <t>8151</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>8158</t>
+          <t>8152</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>8161</t>
+          <t>8153</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>8163</t>
+          <t>8158</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>8169</t>
+          <t>8161</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>8172</t>
+          <t>8163</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>8178</t>
+          <t>8169</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>8179</t>
+          <t>8172</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>8202</t>
+          <t>8178</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>8203</t>
+          <t>8179</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>8204</t>
+          <t>8202</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>8206</t>
+          <t>8203</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>8207</t>
+          <t>8204</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>8209</t>
+          <t>8206</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>8210</t>
+          <t>8207</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>8215</t>
+          <t>8209</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>8217</t>
+          <t>8210</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>8222</t>
+          <t>8215</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>8223</t>
+          <t>8217</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>8225</t>
+          <t>8222</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>8226</t>
+          <t>8223</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>8228</t>
+          <t>8225</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>8234</t>
+          <t>8226</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>8235</t>
+          <t>8228</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>8239</t>
+          <t>8234</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>8240</t>
+          <t>8235</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>8249</t>
+          <t>8239</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>9025</t>
+          <t>8240</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>9029</t>
+          <t>8249</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>9203</t>
+          <t>9025</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>9301</t>
+          <t>9029</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>9302</t>
+          <t>9203</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>9305</t>
+          <t>9301</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>9307</t>
+          <t>9302</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>9311</t>
+          <t>9305</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>9312</t>
+          <t>9307</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>9313</t>
+          <t>9311</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>9406</t>
+          <t>9312</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>9408</t>
+          <t>9313</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>9410</t>
+          <t>9406</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>42103</t>
+          <t>9408</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>44202</t>
+          <t>9410</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>44204</t>
+          <t>42103</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>44208</t>
+          <t>44202</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>ACB4403</t>
+          <t>44204</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>ACB4404</t>
+          <t>44208</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>ACD6047</t>
+          <t>ACB4403</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>ACD6049</t>
+          <t>ACB4404</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>ACD6052</t>
+          <t>ACD6046</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>ACD6056</t>
+          <t>ACD6047</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>ACD6057</t>
+          <t>ACD6049</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>ACD6058</t>
+          <t>ACD6052</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>ACD6059</t>
+          <t>ACD6056</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>ACD6065</t>
+          <t>ACD6057</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>ACD6066</t>
+          <t>ACD6058</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>ACD6069</t>
+          <t>ACD6059</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>ACD6071</t>
+          <t>ACD6065</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>ACD6073</t>
+          <t>ACD6066</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>ACD6074</t>
+          <t>ACD6069</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>BL26</t>
+          <t>ACD6071</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>BL31</t>
+          <t>ACD6073</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>BL33</t>
+          <t>ACD6074</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>C502</t>
+          <t>BL26</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>C504</t>
+          <t>BL31</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>C506</t>
+          <t>BL33</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>C509</t>
+          <t>C502</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>CEY004</t>
+          <t>C504</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>CEY006</t>
+          <t>C506</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>CEY007</t>
+          <t>C509</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>CF4401</t>
+          <t>C510</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>CF4405</t>
+          <t>CEY004</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>CF4410</t>
+          <t>CEY006</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>CF4412</t>
+          <t>CEY007</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>CF4420</t>
+          <t>CF4401</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>CF4421</t>
+          <t>CF4405</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>CF4424</t>
+          <t>CF4410</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>CF4425</t>
+          <t>CF4412</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>CF4427</t>
+          <t>CF4420</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>CF4429</t>
+          <t>CF4421</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>CLF2</t>
+          <t>CF4424</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>CLP12</t>
+          <t>CF4425</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>CLP13</t>
+          <t>CF4427</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>CM3304</t>
+          <t>CF4429</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>CSR010</t>
+          <t>CLF2</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>CSR015</t>
+          <t>CLP12</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>CSR017</t>
+          <t>CLP13</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>CSR019</t>
+          <t>CM3304</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>CSR020</t>
+          <t>CSR010</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>CSR021</t>
+          <t>CSR015</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>CSR023</t>
+          <t>CSR017</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>DS003</t>
+          <t>CSR019</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>EA2502</t>
+          <t>CSR020</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>EA2503</t>
+          <t>CSR021</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>EA2506</t>
+          <t>CSR023</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>EA2507</t>
+          <t>DS003</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>EC2521</t>
+          <t>EA2502</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>EC2525</t>
+          <t>EA2503</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>EC2526</t>
+          <t>EA2506</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>FIE001</t>
+          <t>EA2507</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>FIE003</t>
+          <t>EC2521</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>G513</t>
+          <t>EC2525</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>G514</t>
+          <t>EC2526</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>G516</t>
+          <t>FIE001</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>G521</t>
+          <t>FIE003</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>G532</t>
+          <t>G513</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>G533</t>
+          <t>G514</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>G534</t>
+          <t>G516</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>G536</t>
+          <t>G521</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>GL103</t>
+          <t>G532</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>GL105</t>
+          <t>G533</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>GL108</t>
+          <t>G534</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>GL111</t>
+          <t>G536</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>GM46</t>
+          <t>GL103</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>GWA002</t>
+          <t>GL105</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>GWA004</t>
+          <t>GL108</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>GWA008</t>
+          <t>GL111</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>GWA009</t>
+          <t>GM46</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>GWB102</t>
+          <t>GWA002</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>GWB103</t>
+          <t>GWA004</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>GWB104</t>
+          <t>GWA008</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>GWU008</t>
+          <t>GWA009</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>GWU013</t>
+          <t>GWB102</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>GWU014</t>
+          <t>GWB103</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>GWU015</t>
+          <t>GWB104</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>HM2701</t>
+          <t>GWU008</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>HM2702</t>
+          <t>GWU013</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>HM2703</t>
+          <t>GWU014</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>HM2705</t>
+          <t>GWU015</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>HM2706</t>
+          <t>HM2701</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>HM2707</t>
+          <t>HM2702</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>HM2751</t>
+          <t>HM2703</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>HM2752</t>
+          <t>HM2705</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>HM2753</t>
+          <t>HM2706</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>HM2755</t>
+          <t>HM2707</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>HM2756</t>
+          <t>HM2751</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>HM2757</t>
+          <t>HM2752</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>JP9750</t>
+          <t>HM2753</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>LDP002</t>
+          <t>HM2755</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>LDP004</t>
+          <t>HM2756</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>LDP008</t>
+          <t>HM2757</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>LE2851</t>
+          <t>JP9750</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>LE2853</t>
+          <t>LDP002</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>LE2855</t>
+          <t>LDP004</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>LE2857</t>
+          <t>LDP008</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>LE2858</t>
+          <t>LE2851</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>LE2859</t>
+          <t>LE2853</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>LE2862</t>
+          <t>LE2854</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>LE2863</t>
+          <t>LE2855</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>LZ3114</t>
+          <t>LE2857</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>M437</t>
+          <t>LE2858</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>M865</t>
+          <t>LE2859</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>MAN004</t>
+          <t>LE2862</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>MAN005</t>
+          <t>LE2863</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>MAN007</t>
+          <t>LE2864</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>MAN011</t>
+          <t>LZ3114</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>MAN013</t>
+          <t>M437</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>MAN015</t>
+          <t>M865</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>MAN016</t>
+          <t>MAN004</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>MAN017</t>
+          <t>MAN005</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>MM02</t>
+          <t>MAN007</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>MM2M</t>
+          <t>MAN011</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>MM4M</t>
+          <t>MAN013</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>MM8M</t>
+          <t>MAN015</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>MM14M</t>
+          <t>MAN016</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>MM32M</t>
+          <t>MAN017</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>MM38M</t>
+          <t>MM02</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>MM40M</t>
+          <t>MM2M</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>MM42M</t>
+          <t>MM4M</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>MM44M</t>
+          <t>MM8M</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>MM48M</t>
+          <t>MM14M</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>MM50M</t>
+          <t>MM32M</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>MM52M</t>
+          <t>MM38M</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>MM64M</t>
+          <t>MM40M</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>MM76M</t>
+          <t>MM42M</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>MM78M</t>
+          <t>MM44M</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>MM80M</t>
+          <t>MM48M</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>MM82M</t>
+          <t>MM50M</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>MM84M</t>
+          <t>MM52M</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>MM86M</t>
+          <t>MM64M</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>MM92M</t>
+          <t>MM76M</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>MM94M</t>
+          <t>MM78M</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>MM96M</t>
+          <t>MM80M</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>MM98M</t>
+          <t>MM82M</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>MM99M</t>
+          <t>MM84M</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>MM122M</t>
+          <t>MM86M</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>MM130M</t>
+          <t>MM92M</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>MM152M</t>
+          <t>MM94M</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>MM156M</t>
+          <t>MM96M</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>MM158M</t>
+          <t>MM98M</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>MM172M</t>
+          <t>MM99M</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>MM178M</t>
+          <t>MM122M</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>MM192M</t>
+          <t>MM130M</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>MM212M</t>
+          <t>MM152M</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>MM214M</t>
+          <t>MM156M</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>MM216M</t>
+          <t>MM158M</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>MM232M</t>
+          <t>MM172M</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>MM236M</t>
+          <t>MM178M</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>MM240M</t>
+          <t>MM192M</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>MM246M</t>
+          <t>MM212M</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>MM260M</t>
+          <t>MM214M</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>MM264M</t>
+          <t>MM216M</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>MM266M</t>
+          <t>MM232M</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>MM268M</t>
+          <t>MM236M</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>MM270M</t>
+          <t>MM240M</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>MM280M</t>
+          <t>MM246M</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>MM288M</t>
+          <t>MM260M</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>MM380M</t>
+          <t>MM264M</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>MM456M</t>
+          <t>MM266M</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>MM464M</t>
+          <t>MM268M</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>MM478M</t>
+          <t>MM270M</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>MM482M</t>
+          <t>MM280M</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>MM486M</t>
+          <t>MM288M</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>MM502M</t>
+          <t>MM380M</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>MM506M</t>
+          <t>MM456M</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>MM514M</t>
+          <t>MM464M</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>MM522M</t>
+          <t>MM478M</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>MM536M</t>
+          <t>MM482M</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>MM542M</t>
+          <t>MM486M</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>MM544M</t>
+          <t>MM502M</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>MM546M</t>
+          <t>MM506M</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>MM551M</t>
+          <t>MM514M</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>MM574M</t>
+          <t>MM522M</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>MM588M</t>
+          <t>MM536M</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>MM592M</t>
+          <t>MM542M</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>MM604M</t>
+          <t>MM544M</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>MM624M</t>
+          <t>MM546M</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>MM636M</t>
+          <t>MM551M</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>MM638M</t>
+          <t>MM574M</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>MM647M</t>
+          <t>MM588M</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>MM656M</t>
+          <t>MM592M</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>MM658M</t>
+          <t>MM604M</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>MM660M</t>
+          <t>MM624M</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>MM664M</t>
+          <t>MM636M</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>MM668M</t>
+          <t>MM638M</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>MM673M</t>
+          <t>MM647M</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>MM674M</t>
+          <t>MM656M</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>MM676M</t>
+          <t>MM658M</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>MM680M</t>
+          <t>MM660M</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>MM702M</t>
+          <t>MM664M</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>MM718M</t>
+          <t>MM668M</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>MM742M</t>
+          <t>MM673M</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>MM744M</t>
+          <t>MM674M</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>MM752M</t>
+          <t>MM676M</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>MM768M</t>
+          <t>MM680M</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>MM772M</t>
+          <t>MM702M</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>MM774M</t>
+          <t>MM718M</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>MM776M</t>
+          <t>MM742M</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>MM778M</t>
+          <t>MM744M</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>MM788M</t>
+          <t>MM752M</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>MM794M</t>
+          <t>MM768M</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>MM798M</t>
+          <t>MM772M</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>MM800M</t>
+          <t>MM774M</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>MM802M</t>
+          <t>MM776M</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>MM806M</t>
+          <t>MM778M</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>MM808M</t>
+          <t>MM788M</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>MM810M</t>
+          <t>MM794M</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>MM816M</t>
+          <t>MM798M</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>MM826M</t>
+          <t>MM800M</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>MM830M</t>
+          <t>MM802M</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>MM832M</t>
+          <t>MM806M</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>MM834M</t>
+          <t>MM808M</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>MM838M</t>
+          <t>MM810M</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>MM842M</t>
+          <t>MM816M</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>MM858M</t>
+          <t>MM826M</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>MM860M</t>
+          <t>MM830M</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>MM862M</t>
+          <t>MM832M</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>MM864M</t>
+          <t>MM834M</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>MM866M</t>
+          <t>MM838M</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>MM872M</t>
+          <t>MM842M</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>MM878M</t>
+          <t>MM858M</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>MM880M</t>
+          <t>MM860M</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>MM886M</t>
+          <t>MM862M</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>MM896M</t>
+          <t>MM864M</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>MM908M</t>
+          <t>MM866M</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>MM910M</t>
+          <t>MM872M</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>MM912M</t>
+          <t>MM878M</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>MM914M</t>
+          <t>MM880M</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>MM924M</t>
+          <t>MM886M</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>MM928M</t>
+          <t>MM896M</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>MM934M</t>
+          <t>MM908M</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>MM940M</t>
+          <t>MM910M</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>MM944M</t>
+          <t>MM912M</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>MM946M</t>
+          <t>MM914M</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>MM952M</t>
+          <t>MM924M</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>MM956M</t>
+          <t>MM928M</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>MM958M</t>
+          <t>MM934M</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>MM960M</t>
+          <t>MM940M</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>MM962M</t>
+          <t>MM944M</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>MM964M</t>
+          <t>MM946M</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>MM968M</t>
+          <t>MM952M</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>MM972M</t>
+          <t>MM956M</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>MM974M</t>
+          <t>MM958M</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>MM976M</t>
+          <t>MM960M</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>MM980M</t>
+          <t>MM962M</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>MM982M</t>
+          <t>MM964M</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>MM9901M</t>
+          <t>MM968M</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>MM9903M</t>
+          <t>MM972M</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>MM9904M</t>
+          <t>MM974M</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>MM9906M</t>
+          <t>MM976M</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>MM9908M</t>
+          <t>MM980M</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>MM9909M</t>
+          <t>MM982M</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>MM9910M</t>
+          <t>MM9901M</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>MM9912M</t>
+          <t>MM9903M</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>MM9914M</t>
+          <t>MM9904M</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>MM9916M</t>
+          <t>MM9906M</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>MM9918M</t>
+          <t>MM9908M</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>MM9920M</t>
+          <t>MM9909M</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>MM9921M</t>
+          <t>MM9910M</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>MM9924M</t>
+          <t>MM9912M</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>MM9926M</t>
+          <t>MM9914M</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>MM9927M</t>
+          <t>MM9916M</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>MM9928M</t>
+          <t>MM9918M</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>MM9929M</t>
+          <t>MM9920M</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>MM9931M</t>
+          <t>MM9921M</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>MM9936M</t>
+          <t>MM9924M</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>MM9937M</t>
+          <t>MM9926M</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>MM9938M</t>
+          <t>MM9927M</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>MM9941M</t>
+          <t>MM9928M</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>MM9943M</t>
+          <t>MM9929M</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>MM9946M</t>
+          <t>MM9931M</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>MM9947M</t>
+          <t>MM9936M</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>MM9948M</t>
+          <t>MM9937M</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>MM9952M</t>
+          <t>MM9938M</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>MM9953M</t>
+          <t>MM9941M</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>MM9954M</t>
+          <t>MM9943M</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>MM9956M</t>
+          <t>MM9946M</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>MM9957M</t>
+          <t>MM9947M</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>MM9958M</t>
+          <t>MM9948M</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>MM9959M</t>
+          <t>MM9952M</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t>MM9960M</t>
+          <t>MM9953M</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>MM9961M</t>
+          <t>MM9954M</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t>MM9962M</t>
+          <t>MM9956M</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>MM9963M</t>
+          <t>MM9957M</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>MM9964M</t>
+          <t>MM9958M</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>MM9965M</t>
+          <t>MM9959M</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>MM9966M</t>
+          <t>MM9960M</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>MM9968M</t>
+          <t>MM9961M</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>MM9969M</t>
+          <t>MM9962M</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>MM9970M</t>
+          <t>MM9963M</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MM9964M</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>MTPV1</t>
+          <t>MM9965M</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
         <is>
-          <t>MTPV2</t>
+          <t>MM9966M</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
         <is>
-          <t>N458</t>
+          <t>MM9968M</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" s="2" t="inlineStr">
         <is>
-          <t>N460</t>
+          <t>MM9969M</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>MM9970M</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>MRL001</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>MRL002</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>MTPV1</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
         <is>
-          <t>NR6</t>
+          <t>MTPV2</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="2" t="inlineStr">
         <is>
-          <t>NR10</t>
+          <t>N458</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
         <is>
-          <t>NR11</t>
+          <t>N460</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" s="2" t="inlineStr">
         <is>
-          <t>NR12</t>
+          <t>N466</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
         <is>
-          <t>NR13</t>
+          <t>N469</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="2" t="inlineStr">
         <is>
-          <t>NR14</t>
+          <t>NR4</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" s="2" t="inlineStr">
         <is>
-          <t>NR17</t>
+          <t>NR5</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="2" t="inlineStr">
         <is>
-          <t>NR20</t>
+          <t>NR6</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
         <is>
-          <t>NR35</t>
+          <t>NR10</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" s="2" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>NR11</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
         <is>
-          <t>NR44</t>
+          <t>NR12</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" s="2" t="inlineStr">
         <is>
-          <t>NR46</t>
+          <t>NR13</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" s="2" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>NR14</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>NR17</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="2" t="inlineStr">
         <is>
-          <t>NR56</t>
+          <t>NR20</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR35</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="2" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR37</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="2" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR44</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" s="2" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR46</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" s="2" t="inlineStr">
         <is>
-          <t>NR76</t>
+          <t>NR47</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" s="2" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR52</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" s="2" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR54</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" s="2" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR56</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" s="2" t="inlineStr">
         <is>
-          <t>NR88</t>
+          <t>NR64</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" s="2" t="inlineStr">
         <is>
-          <t>NR91</t>
+          <t>NR65</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" s="2" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR68</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR75</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" s="2" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR76</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>NR78</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" s="2" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR82</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" s="2" t="inlineStr">
         <is>
-          <t>NR107</t>
+          <t>NR83</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" s="2" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR88</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR91</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="2" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR93</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR94</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>NR95</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>NR97</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" s="2" t="inlineStr">
         <is>
-          <t>PKLA4</t>
+          <t>NR102</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>NR107</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" s="2" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>NR109</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>NR112</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" s="2" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>NR113</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>NR115</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>PB4</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>PKLA4</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
         <is>
-          <t>QL009</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>QL016</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
         <is>
-          <t>QL019</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QE001</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>QR5400</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QL004</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>RA2302</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
         <is>
-          <t>RA2303</t>
+          <t>QL009</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>QL016</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>QL019</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>RM93</t>
+          <t>QR1744</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="2" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>QR1771</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
         <is>
-          <t>SCT008</t>
+          <t>QR5400</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" s="2" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>RA2302</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" s="2" t="inlineStr">
         <is>
-          <t>SO3</t>
+          <t>RA2303</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="2" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" s="2" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>RL301</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" s="2" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>RM93</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" s="2" t="inlineStr">
         <is>
-          <t>T373</t>
+          <t>SCT001</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" s="2" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>SCT008</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="2" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>SCT009</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="2" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>SCT013</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="2" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>SO3</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="2" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>SSR102</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="2" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>SSR103</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" s="2" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>SSR104</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" s="2" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>T373</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" s="2" t="inlineStr">
         <is>
-          <t>TT02</t>
+          <t>TE2801</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" s="2" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TE2803</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="A472" s="2" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TE2805</t>
         </is>
       </c>
     </row>
     <row r="473">
       <c r="A473" s="2" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TE2807</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="A474" s="2" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TE2808</t>
         </is>
       </c>
     </row>
     <row r="475">
       <c r="A475" s="2" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TE2813</t>
         </is>
       </c>
     </row>
     <row r="476">
       <c r="A476" s="2" t="inlineStr">
         <is>
-          <t>TT104</t>
+          <t>TE2814</t>
         </is>
       </c>
     </row>
     <row r="477">
       <c r="A477" s="2" t="inlineStr">
         <is>
-          <t>TT105</t>
+          <t>TJ096</t>
         </is>
       </c>
     </row>
     <row r="478">
       <c r="A478" s="2" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TT02</t>
         </is>
       </c>
     </row>
     <row r="479">
       <c r="A479" s="2" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TT03</t>
         </is>
       </c>
     </row>
     <row r="480">
       <c r="A480" s="2" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT04</t>
         </is>
       </c>
     </row>
     <row r="481">
       <c r="A481" s="2" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT05</t>
         </is>
       </c>
     </row>
     <row r="482">
       <c r="A482" s="2" t="inlineStr">
         <is>
-          <t>TT123</t>
+          <t>TT08</t>
         </is>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="2" t="inlineStr">
         <is>
-          <t>TT126</t>
+          <t>TT103</t>
         </is>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="2" t="inlineStr">
         <is>
-          <t>TT129</t>
+          <t>TT104</t>
         </is>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="2" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT105</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="2" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT107</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="2" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT110</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" s="2" t="inlineStr">
         <is>
-          <t>VL04</t>
+          <t>TT115</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" s="2" t="inlineStr">
         <is>
-          <t>VL11</t>
+          <t>TT117</t>
         </is>
       </c>
     </row>
     <row r="490">
       <c r="A490" s="2" t="inlineStr">
         <is>
-          <t>VL13</t>
+          <t>TT123</t>
         </is>
       </c>
     </row>
     <row r="491">
       <c r="A491" s="2" t="inlineStr">
         <is>
-          <t>VL20</t>
+          <t>TT126</t>
         </is>
       </c>
     </row>
     <row r="492">
       <c r="A492" s="2" t="inlineStr">
         <is>
-          <t>VL22</t>
+          <t>TT129</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="2" t="inlineStr">
         <is>
-          <t>VL27</t>
+          <t>TT130</t>
         </is>
       </c>
     </row>
     <row r="494">
       <c r="A494" s="2" t="inlineStr">
         <is>
-          <t>VL36</t>
+          <t>TT202</t>
         </is>
       </c>
     </row>
     <row r="495">
       <c r="A495" s="2" t="inlineStr">
         <is>
-          <t>VL38</t>
+          <t>TT206</t>
         </is>
       </c>
     </row>
     <row r="496">
       <c r="A496" s="2" t="inlineStr">
         <is>
-          <t>VL43</t>
+          <t>VL04</t>
         </is>
       </c>
     </row>
     <row r="497">
       <c r="A497" s="2" t="inlineStr">
         <is>
-          <t>VL49</t>
+          <t>VL11</t>
         </is>
       </c>
     </row>
     <row r="498">
       <c r="A498" s="2" t="inlineStr">
         <is>
-          <t>VL57</t>
+          <t>VL13</t>
         </is>
       </c>
     </row>
     <row r="499">
       <c r="A499" s="2" t="inlineStr">
         <is>
-          <t>VL62</t>
+          <t>VL20</t>
         </is>
       </c>
     </row>
     <row r="500">
       <c r="A500" s="2" t="inlineStr">
         <is>
-          <t>VL67</t>
+          <t>VL22</t>
         </is>
       </c>
     </row>
     <row r="501">
       <c r="A501" s="2" t="inlineStr">
         <is>
-          <t>VL81</t>
+          <t>VL27</t>
         </is>
       </c>
     </row>
     <row r="502">
       <c r="A502" s="2" t="inlineStr">
         <is>
-          <t>VL86</t>
+          <t>VL36</t>
         </is>
       </c>
     </row>
     <row r="503">
       <c r="A503" s="2" t="inlineStr">
         <is>
-          <t>VL87</t>
+          <t>VL38</t>
         </is>
       </c>
     </row>
     <row r="504">
       <c r="A504" s="2" t="inlineStr">
         <is>
-          <t>VL88</t>
+          <t>VL43</t>
         </is>
       </c>
     </row>
     <row r="505">
       <c r="A505" s="2" t="inlineStr">
         <is>
-          <t>VL90</t>
+          <t>VL49</t>
         </is>
       </c>
     </row>
     <row r="506">
       <c r="A506" s="2" t="inlineStr">
         <is>
-          <t>VL92</t>
+          <t>VL57</t>
         </is>
       </c>
     </row>
     <row r="507">
       <c r="A507" s="2" t="inlineStr">
         <is>
-          <t>VL99</t>
+          <t>VL62</t>
         </is>
       </c>
     </row>
     <row r="508">
       <c r="A508" s="2" t="inlineStr">
         <is>
-          <t>VL100</t>
+          <t>VL67</t>
         </is>
       </c>
     </row>
     <row r="509">
       <c r="A509" s="2" t="inlineStr">
         <is>
-          <t>VL101</t>
+          <t>VL75</t>
         </is>
       </c>
     </row>
     <row r="510">
       <c r="A510" s="2" t="inlineStr">
         <is>
-          <t>VL103</t>
+          <t>VL81</t>
         </is>
       </c>
     </row>
     <row r="511">
       <c r="A511" s="2" t="inlineStr">
         <is>
-          <t>VL107</t>
+          <t>VL86</t>
         </is>
       </c>
     </row>
     <row r="512">
       <c r="A512" s="2" t="inlineStr">
         <is>
-          <t>VL112</t>
+          <t>VL87</t>
         </is>
       </c>
     </row>
     <row r="513">
       <c r="A513" s="2" t="inlineStr">
         <is>
-          <t>VL114</t>
+          <t>VL88</t>
         </is>
       </c>
     </row>
     <row r="514">
       <c r="A514" s="2" t="inlineStr">
         <is>
-          <t>VL115</t>
+          <t>VL90</t>
         </is>
       </c>
     </row>
     <row r="515">
       <c r="A515" s="2" t="inlineStr">
         <is>
-          <t>VL121</t>
+          <t>VL92</t>
         </is>
       </c>
     </row>
     <row r="516">
       <c r="A516" s="2" t="inlineStr">
         <is>
-          <t>VL122</t>
+          <t>VL99</t>
         </is>
       </c>
     </row>
     <row r="517">
       <c r="A517" s="2" t="inlineStr">
         <is>
-          <t>VL124</t>
+          <t>VL100</t>
         </is>
       </c>
     </row>
     <row r="518">
       <c r="A518" s="2" t="inlineStr">
         <is>
-          <t>VL125</t>
+          <t>VL101</t>
         </is>
       </c>
     </row>
     <row r="519">
       <c r="A519" s="2" t="inlineStr">
         <is>
-          <t>VL126</t>
+          <t>VL103</t>
         </is>
       </c>
     </row>
     <row r="520">
       <c r="A520" s="2" t="inlineStr">
         <is>
-          <t>VL129</t>
+          <t>VL107</t>
         </is>
       </c>
     </row>
     <row r="521">
       <c r="A521" s="2" t="inlineStr">
         <is>
-          <t>VL134</t>
+          <t>VL112</t>
         </is>
       </c>
     </row>
     <row r="522">
       <c r="A522" s="2" t="inlineStr">
         <is>
-          <t>VL137</t>
+          <t>VL114</t>
         </is>
       </c>
     </row>
     <row r="523">
       <c r="A523" s="2" t="inlineStr">
         <is>
-          <t>VL139</t>
+          <t>VL115</t>
         </is>
       </c>
     </row>
     <row r="524">
       <c r="A524" s="2" t="inlineStr">
         <is>
-          <t>VL354</t>
+          <t>VL121</t>
         </is>
       </c>
     </row>
     <row r="525">
       <c r="A525" s="2" t="inlineStr">
         <is>
-          <t>VLINE8013</t>
+          <t>VL122</t>
         </is>
       </c>
     </row>
     <row r="526">
       <c r="A526" s="2" t="inlineStr">
         <is>
-          <t>VLINE8020</t>
+          <t>VL124</t>
         </is>
       </c>
     </row>
     <row r="527">
       <c r="A527" s="2" t="inlineStr">
         <is>
-          <t>VLINE8058</t>
+          <t>VL125</t>
         </is>
       </c>
     </row>
     <row r="528">
       <c r="A528" s="2" t="inlineStr">
         <is>
-          <t>VLINE8059</t>
+          <t>VL126</t>
         </is>
       </c>
     </row>
     <row r="529">
       <c r="A529" s="2" t="inlineStr">
         <is>
-          <t>VLINE8061</t>
+          <t>VL129</t>
         </is>
       </c>
     </row>
     <row r="530">
       <c r="A530" s="2" t="inlineStr">
         <is>
-          <t>VLINE8071</t>
+          <t>VL134</t>
         </is>
       </c>
     </row>
     <row r="531">
       <c r="A531" s="2" t="inlineStr">
         <is>
-          <t>VLINE8072</t>
+          <t>VL137</t>
         </is>
       </c>
     </row>
     <row r="532">
       <c r="A532" s="2" t="inlineStr">
         <is>
-          <t>VLINE8075</t>
+          <t>VL139</t>
         </is>
       </c>
     </row>
     <row r="533">
       <c r="A533" s="2" t="inlineStr">
         <is>
-          <t>VLINE8080</t>
+          <t>VL140</t>
         </is>
       </c>
     </row>
     <row r="534">
       <c r="A534" s="2" t="inlineStr">
         <is>
-          <t>VLINE8102</t>
+          <t>VL354</t>
         </is>
       </c>
     </row>
     <row r="535">
       <c r="A535" s="2" t="inlineStr">
         <is>
-          <t>VLINE8111</t>
+          <t>VLINE8013</t>
         </is>
       </c>
     </row>
     <row r="536">
       <c r="A536" s="2" t="inlineStr">
         <is>
-          <t>VLINE8113</t>
+          <t>VLINE8020</t>
         </is>
       </c>
     </row>
     <row r="537">
       <c r="A537" s="2" t="inlineStr">
         <is>
-          <t>VLINE8115</t>
+          <t>VLINE8021</t>
         </is>
       </c>
     </row>
     <row r="538">
       <c r="A538" s="2" t="inlineStr">
         <is>
-          <t>VLINE8117</t>
+          <t>VLINE8058</t>
         </is>
       </c>
     </row>
     <row r="539">
       <c r="A539" s="2" t="inlineStr">
         <is>
-          <t>VLINE8120</t>
+          <t>VLINE8059</t>
         </is>
       </c>
     </row>
     <row r="540">
       <c r="A540" s="2" t="inlineStr">
         <is>
-          <t>VLINE8122</t>
+          <t>VLINE8061</t>
         </is>
       </c>
     </row>
     <row r="541">
       <c r="A541" s="2" t="inlineStr">
         <is>
-          <t>VLINE8124</t>
+          <t>VLINE8071</t>
         </is>
       </c>
     </row>
     <row r="542">
       <c r="A542" s="2" t="inlineStr">
         <is>
-          <t>VLINE8126</t>
+          <t>VLINE8072</t>
         </is>
       </c>
     </row>
     <row r="543">
       <c r="A543" s="2" t="inlineStr">
         <is>
-          <t>VLINE8161</t>
+          <t>VLINE8075</t>
         </is>
       </c>
     </row>
     <row r="544">
       <c r="A544" s="2" t="inlineStr">
         <is>
-          <t>VLINE8163</t>
+          <t>VLINE8080</t>
         </is>
       </c>
     </row>
     <row r="545">
       <c r="A545" s="2" t="inlineStr">
         <is>
-          <t>VLINE8164</t>
+          <t>VLINE8102</t>
         </is>
       </c>
     </row>
     <row r="546">
       <c r="A546" s="2" t="inlineStr">
         <is>
-          <t>VLINE8172</t>
+          <t>VLINE8111</t>
         </is>
       </c>
     </row>
     <row r="547">
       <c r="A547" s="2" t="inlineStr">
         <is>
-          <t>VLINE8181</t>
+          <t>VLINE8113</t>
         </is>
       </c>
     </row>
     <row r="548">
       <c r="A548" s="2" t="inlineStr">
         <is>
-          <t>VLINE8183</t>
+          <t>VLINE8115</t>
         </is>
       </c>
     </row>
     <row r="549">
       <c r="A549" s="2" t="inlineStr">
         <is>
-          <t>VLINE8211</t>
+          <t>VLINE8117</t>
         </is>
       </c>
     </row>
     <row r="550">
       <c r="A550" s="2" t="inlineStr">
         <is>
-          <t>VLINE8213</t>
+          <t>VLINE8120</t>
         </is>
       </c>
     </row>
     <row r="551">
       <c r="A551" s="2" t="inlineStr">
         <is>
-          <t>VLINE8215</t>
+          <t>VLINE8121</t>
         </is>
       </c>
     </row>
     <row r="552">
       <c r="A552" s="2" t="inlineStr">
         <is>
-          <t>VLINE8217</t>
+          <t>VLINE8122</t>
         </is>
       </c>
     </row>
     <row r="553">
       <c r="A553" s="2" t="inlineStr">
         <is>
-          <t>VLINE8219</t>
+          <t>VLINE8124</t>
         </is>
       </c>
     </row>
     <row r="554">
       <c r="A554" s="2" t="inlineStr">
         <is>
-          <t>VLINE8226</t>
+          <t>VLINE8126</t>
         </is>
       </c>
     </row>
     <row r="555">
       <c r="A555" s="2" t="inlineStr">
         <is>
-          <t>VLINE8228</t>
+          <t>VLINE8161</t>
         </is>
       </c>
     </row>
     <row r="556">
       <c r="A556" s="2" t="inlineStr">
         <is>
-          <t>VLINE8230</t>
+          <t>VLINE8163</t>
         </is>
       </c>
     </row>
     <row r="557">
       <c r="A557" s="2" t="inlineStr">
         <is>
-          <t>VLINE8232</t>
+          <t>VLINE8164</t>
         </is>
       </c>
     </row>
     <row r="558">
       <c r="A558" s="2" t="inlineStr">
         <is>
-          <t>VLINE8400</t>
+          <t>VLINE8172</t>
         </is>
       </c>
     </row>
     <row r="559">
       <c r="A559" s="2" t="inlineStr">
         <is>
-          <t>VLINE8405</t>
+          <t>VLINE8181</t>
         </is>
       </c>
     </row>
     <row r="560">
       <c r="A560" s="2" t="inlineStr">
         <is>
-          <t>VLINE8408</t>
+          <t>VLINE8183</t>
         </is>
       </c>
     </row>
     <row r="561">
       <c r="A561" s="2" t="inlineStr">
         <is>
-          <t>VLINE8413</t>
+          <t>VLINE8211</t>
         </is>
       </c>
     </row>
     <row r="562">
       <c r="A562" s="2" t="inlineStr">
         <is>
-          <t>VLINE8415</t>
+          <t>VLINE8213</t>
         </is>
       </c>
     </row>
     <row r="563">
       <c r="A563" s="2" t="inlineStr">
         <is>
-          <t>VLINE8417</t>
+          <t>VLINE8215</t>
         </is>
       </c>
     </row>
     <row r="564">
       <c r="A564" s="2" t="inlineStr">
         <is>
-          <t>VLINE8418</t>
+          <t>VLINE8217</t>
         </is>
       </c>
     </row>
     <row r="565">
       <c r="A565" s="2" t="inlineStr">
         <is>
-          <t>VLINE8419</t>
+          <t>VLINE8219</t>
         </is>
       </c>
     </row>
     <row r="566">
       <c r="A566" s="2" t="inlineStr">
         <is>
-          <t>VLINE8420</t>
+          <t>VLINE8226</t>
         </is>
       </c>
     </row>
     <row r="567">
       <c r="A567" s="2" t="inlineStr">
         <is>
-          <t>VLINE8421</t>
+          <t>VLINE8228</t>
         </is>
       </c>
     </row>
     <row r="568">
       <c r="A568" s="2" t="inlineStr">
         <is>
-          <t>VLINE8457</t>
+          <t>VLINE8230</t>
         </is>
       </c>
     </row>
     <row r="569">
       <c r="A569" s="2" t="inlineStr">
         <is>
-          <t>VLINE8459</t>
+          <t>VLINE8232</t>
         </is>
       </c>
     </row>
     <row r="570">
       <c r="A570" s="2" t="inlineStr">
         <is>
-          <t>VLINE8460</t>
+          <t>VLINE8234</t>
         </is>
       </c>
     </row>
     <row r="571">
       <c r="A571" s="2" t="inlineStr">
         <is>
-          <t>VLINE8702</t>
+          <t>VLINE8400</t>
         </is>
       </c>
     </row>
     <row r="572">
       <c r="A572" s="2" t="inlineStr">
         <is>
-          <t>VLINE8725</t>
+          <t>VLINE8405</t>
         </is>
       </c>
     </row>
     <row r="573">
       <c r="A573" s="2" t="inlineStr">
         <is>
-          <t>VLINE8727</t>
+          <t>VLINE8408</t>
         </is>
       </c>
     </row>
     <row r="574">
       <c r="A574" s="2" t="inlineStr">
         <is>
-          <t>VLINE8729</t>
+          <t>VLINE8413</t>
         </is>
       </c>
     </row>
     <row r="575">
       <c r="A575" s="2" t="inlineStr">
         <is>
-          <t>VLINE8731</t>
+          <t>VLINE8415</t>
         </is>
       </c>
     </row>
     <row r="576">
       <c r="A576" s="2" t="inlineStr">
         <is>
-          <t>VLINE8733</t>
+          <t>VLINE8417</t>
         </is>
       </c>
     </row>
     <row r="577">
       <c r="A577" s="2" t="inlineStr">
         <is>
-          <t>VLINE8735</t>
+          <t>VLINE8418</t>
         </is>
       </c>
     </row>
     <row r="578">
       <c r="A578" s="2" t="inlineStr">
         <is>
-          <t>VLINE8737</t>
+          <t>VLINE8419</t>
         </is>
       </c>
     </row>
     <row r="579">
       <c r="A579" s="2" t="inlineStr">
         <is>
-          <t>VLINE8739</t>
+          <t>VLINE8420</t>
         </is>
       </c>
     </row>
     <row r="580">
       <c r="A580" s="2" t="inlineStr">
         <is>
-          <t>VLINE8741</t>
+          <t>VLINE8421</t>
         </is>
       </c>
     </row>
     <row r="581">
       <c r="A581" s="2" t="inlineStr">
         <is>
-          <t>VLINE8742</t>
+          <t>VLINE8422</t>
         </is>
       </c>
     </row>
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>VLINE8744</t>
+          <t>VLINE8457</t>
         </is>
       </c>
     </row>
     <row r="583">
       <c r="A583" s="2" t="inlineStr">
         <is>
-          <t>VLINE8746</t>
+          <t>VLINE8459</t>
         </is>
       </c>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>VLINE8748</t>
+          <t>VLINE8460</t>
         </is>
       </c>
     </row>
     <row r="585">
       <c r="A585" s="2" t="inlineStr">
         <is>
-          <t>VLINE8750</t>
+          <t>VLINE8702</t>
         </is>
       </c>
     </row>
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>VLINE8752</t>
+          <t>VLINE8725</t>
         </is>
       </c>
     </row>
     <row r="587">
       <c r="A587" s="2" t="inlineStr">
         <is>
-          <t>VLINE8754</t>
+          <t>VLINE8727</t>
         </is>
       </c>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>VLINE8819</t>
+          <t>VLINE8729</t>
         </is>
       </c>
     </row>
     <row r="589">
       <c r="A589" s="2" t="inlineStr">
         <is>
-          <t>VLINE8863</t>
+          <t>VLINE8731</t>
         </is>
       </c>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>VR77</t>
+          <t>VLINE8733</t>
         </is>
       </c>
     </row>
     <row r="591">
       <c r="A591" s="2" t="inlineStr">
         <is>
-          <t>XP2001</t>
+          <t>VLINE8735</t>
         </is>
       </c>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>VLINE8737</t>
         </is>
       </c>
     </row>
     <row r="593">
       <c r="A593" s="2" t="inlineStr">
         <is>
-          <t>XP2006</t>
+          <t>VLINE8739</t>
         </is>
       </c>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>VLINE8741</t>
         </is>
       </c>
     </row>
     <row r="595">
       <c r="A595" s="2" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>VLINE8742</t>
         </is>
       </c>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>VLINE8743</t>
         </is>
       </c>
     </row>
     <row r="597">
       <c r="A597" s="2" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>VLINE8744</t>
         </is>
       </c>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>VLINE8745</t>
         </is>
       </c>
     </row>
     <row r="599">
       <c r="A599" s="2" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>VLINE8746</t>
         </is>
       </c>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>XRN003</t>
+          <t>VLINE8748</t>
         </is>
       </c>
     </row>
     <row r="601">
       <c r="A601" s="2" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>VLINE8750</t>
         </is>
       </c>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>VLINE8752</t>
         </is>
       </c>
     </row>
     <row r="603">
       <c r="A603" s="2" t="inlineStr">
         <is>
-          <t>XRN010</t>
+          <t>VLINE8754</t>
         </is>
       </c>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>VLINE8756</t>
         </is>
       </c>
     </row>
     <row r="605">
       <c r="A605" s="2" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>VLINE8762</t>
         </is>
       </c>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>VLINE8819</t>
         </is>
       </c>
     </row>
     <row r="607">
       <c r="A607" s="2" t="inlineStr">
         <is>
-          <t>XRN022</t>
+          <t>VLINE8863</t>
         </is>
       </c>
     </row>
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>XRN028</t>
+          <t>VR77</t>
         </is>
       </c>
     </row>
     <row r="609">
       <c r="A609" s="2" t="inlineStr">
+        <is>
+          <t>XP2001</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" s="2" t="inlineStr">
+        <is>
+          <t>XP2005</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" s="2" t="inlineStr">
+        <is>
+          <t>XP2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" s="2" t="inlineStr">
+        <is>
+          <t>XP2008</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" s="2" t="inlineStr">
+        <is>
+          <t>XP2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="2" t="inlineStr">
+        <is>
+          <t>XP2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" s="2" t="inlineStr">
+        <is>
+          <t>XP2013</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" s="2" t="inlineStr">
+        <is>
+          <t>XP2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" s="2" t="inlineStr">
+        <is>
+          <t>XP2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="2" t="inlineStr">
+        <is>
+          <t>XP2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" s="2" t="inlineStr">
+        <is>
+          <t>XRN003</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="2" t="inlineStr">
+        <is>
+          <t>XRN005</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="2" t="inlineStr">
+        <is>
+          <t>XRN009</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="2" t="inlineStr">
+        <is>
+          <t>XRN010</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="2" t="inlineStr">
+        <is>
+          <t>XRN017</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="2" t="inlineStr">
+        <is>
+          <t>XRN018</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="2" t="inlineStr">
+        <is>
+          <t>XRN021</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="2" t="inlineStr">
+        <is>
+          <t>XRN022</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="2" t="inlineStr">
+        <is>
+          <t>XRN028</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="2" t="inlineStr">
         <is>
           <t>XRN029</t>
         </is>

</xml_diff>

<commit_message>
Update RailOps database files - 2026-04-30 02:31:29 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A628"/>
+  <dimension ref="A1:A662"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1056,3792 +1056,4030 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>44202</t>
+          <t>42107</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>44204</t>
+          <t>44202</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>44208</t>
+          <t>44204</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>ACB4403</t>
+          <t>44208</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>ACB4404</t>
+          <t>ACB4403</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>ACD6046</t>
+          <t>ACB4404</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>ACD6047</t>
+          <t>ACD6046</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>ACD6049</t>
+          <t>ACD6047</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>ACD6052</t>
+          <t>ACD6049</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>ACD6056</t>
+          <t>ACD6052</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>ACD6057</t>
+          <t>ACD6056</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>ACD6058</t>
+          <t>ACD6057</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>ACD6059</t>
+          <t>ACD6058</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>ACD6065</t>
+          <t>ACD6059</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>ACD6066</t>
+          <t>ACD6065</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>ACD6069</t>
+          <t>ACD6066</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>ACD6071</t>
+          <t>ACD6069</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>ACD6073</t>
+          <t>ACD6071</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>ACD6074</t>
+          <t>ACD6073</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>BL26</t>
+          <t>ACD6074</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>BL31</t>
+          <t>BL26</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>BL33</t>
+          <t>BL31</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>C502</t>
+          <t>BL33</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>C504</t>
+          <t>C502</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>C506</t>
+          <t>C504</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>C509</t>
+          <t>C506</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>C510</t>
+          <t>C509</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>CEY004</t>
+          <t>C510</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>CEY006</t>
+          <t>CEY004</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>CEY007</t>
+          <t>CEY006</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>CF4401</t>
+          <t>CEY007</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>CF4405</t>
+          <t>CF4401</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>CF4410</t>
+          <t>CF4405</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>CF4412</t>
+          <t>CF4407</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>CF4420</t>
+          <t>CF4410</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>CF4421</t>
+          <t>CF4412</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>CF4424</t>
+          <t>CF4420</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>CF4425</t>
+          <t>CF4421</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>CF4427</t>
+          <t>CF4424</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>CF4429</t>
+          <t>CF4425</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>CLF2</t>
+          <t>CF4427</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>CLP12</t>
+          <t>CF4429</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>CLP13</t>
+          <t>CLF2</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>CM3304</t>
+          <t>CLP12</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>CSR010</t>
+          <t>CLP13</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>CSR015</t>
+          <t>CLP17</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>CSR017</t>
+          <t>CM3304</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>CSR019</t>
+          <t>CM3307</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>CSR020</t>
+          <t>CSR010</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>CSR021</t>
+          <t>CSR015</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>CSR023</t>
+          <t>CSR017</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>DS003</t>
+          <t>CSR019</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>EA2502</t>
+          <t>CSR020</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>EA2503</t>
+          <t>CSR021</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>EA2506</t>
+          <t>CSR023</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>EA2507</t>
+          <t>DS003</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>EC2521</t>
+          <t>EA2502</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>EC2525</t>
+          <t>EA2503</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>EC2526</t>
+          <t>EA2506</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>FIE001</t>
+          <t>EA2507</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>FIE003</t>
+          <t>EC2521</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>G513</t>
+          <t>EC2525</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>G514</t>
+          <t>EC2526</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>G516</t>
+          <t>FIE001</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>G521</t>
+          <t>FIE003</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>G532</t>
+          <t>G513</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>G533</t>
+          <t>G514</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>G534</t>
+          <t>G516</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>G536</t>
+          <t>G521</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>GL103</t>
+          <t>G532</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>GL105</t>
+          <t>G533</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>GL108</t>
+          <t>G534</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>GL111</t>
+          <t>G536</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>GM46</t>
+          <t>GL103</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>GWA002</t>
+          <t>GL105</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>GWA004</t>
+          <t>GL108</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>GWA008</t>
+          <t>GL111</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>GWA009</t>
+          <t>GM46</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>GWB102</t>
+          <t>GWA002</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>GWB103</t>
+          <t>GWA004</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>GWB104</t>
+          <t>GWA008</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>GWU008</t>
+          <t>GWA009</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>GWU013</t>
+          <t>GWB102</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>GWU014</t>
+          <t>GWB103</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>GWU015</t>
+          <t>GWB104</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>HM2701</t>
+          <t>GWU008</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>HM2702</t>
+          <t>GWU013</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>HM2703</t>
+          <t>GWU014</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>HM2705</t>
+          <t>GWU015</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>HM2706</t>
+          <t>HM2701</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>HM2707</t>
+          <t>HM2702</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>HM2751</t>
+          <t>HM2703</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>HM2752</t>
+          <t>HM2705</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>HM2753</t>
+          <t>HM2706</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>HM2755</t>
+          <t>HM2707</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>HM2756</t>
+          <t>HM2751</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>HM2757</t>
+          <t>HM2752</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>JP9750</t>
+          <t>HM2753</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>LDP002</t>
+          <t>HM2755</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>LDP004</t>
+          <t>HM2756</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>LDP008</t>
+          <t>HM2757</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>LE2851</t>
+          <t>JP9750</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>LE2853</t>
+          <t>LDP002</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>LE2854</t>
+          <t>LDP004</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>LE2855</t>
+          <t>LDP008</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>LE2857</t>
+          <t>LE2851</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>LE2858</t>
+          <t>LE2853</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>LE2859</t>
+          <t>LE2854</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>LE2862</t>
+          <t>LE2855</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>LE2863</t>
+          <t>LE2857</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>LE2864</t>
+          <t>LE2858</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>LZ3114</t>
+          <t>LE2859</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>M437</t>
+          <t>LE2862</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>M865</t>
+          <t>LE2863</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>MAN004</t>
+          <t>LE2864</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>MAN005</t>
+          <t>LZ3114</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>MAN007</t>
+          <t>M437</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>MAN011</t>
+          <t>M865</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>MAN013</t>
+          <t>MAN004</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>MAN015</t>
+          <t>MAN005</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>MAN016</t>
+          <t>MAN007</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>MAN017</t>
+          <t>MAN011</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>MM02</t>
+          <t>MAN013</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>MM2M</t>
+          <t>MAN015</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>MM4M</t>
+          <t>MAN016</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>MM8M</t>
+          <t>MAN017</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>MM14M</t>
+          <t>MM02</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>MM32M</t>
+          <t>MM2M</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>MM38M</t>
+          <t>MM4M</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>MM40M</t>
+          <t>MM8M</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>MM42M</t>
+          <t>MM14M</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>MM44M</t>
+          <t>MM32M</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>MM48M</t>
+          <t>MM38M</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>MM50M</t>
+          <t>MM40M</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>MM52M</t>
+          <t>MM42M</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>MM64M</t>
+          <t>MM44M</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>MM76M</t>
+          <t>MM48M</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>MM78M</t>
+          <t>MM50M</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>MM80M</t>
+          <t>MM52M</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>MM82M</t>
+          <t>MM64M</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>MM84M</t>
+          <t>MM76M</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>MM86M</t>
+          <t>MM78M</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>MM92M</t>
+          <t>MM80M</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>MM94M</t>
+          <t>MM82M</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>MM96M</t>
+          <t>MM84M</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>MM98M</t>
+          <t>MM86M</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>MM99M</t>
+          <t>MM92M</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>MM122M</t>
+          <t>MM94M</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>MM130M</t>
+          <t>MM96M</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>MM152M</t>
+          <t>MM98M</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>MM156M</t>
+          <t>MM99M</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>MM158M</t>
+          <t>MM122M</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>MM172M</t>
+          <t>MM130M</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>MM178M</t>
+          <t>MM152M</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>MM192M</t>
+          <t>MM156M</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>MM212M</t>
+          <t>MM158M</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>MM214M</t>
+          <t>MM172M</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>MM216M</t>
+          <t>MM178M</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>MM232M</t>
+          <t>MM192M</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>MM236M</t>
+          <t>MM212M</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>MM240M</t>
+          <t>MM214M</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>MM246M</t>
+          <t>MM216M</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>MM260M</t>
+          <t>MM232M</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>MM264M</t>
+          <t>MM236M</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>MM266M</t>
+          <t>MM240M</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>MM268M</t>
+          <t>MM246M</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>MM270M</t>
+          <t>MM260M</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>MM280M</t>
+          <t>MM264M</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>MM288M</t>
+          <t>MM266M</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>MM380M</t>
+          <t>MM268M</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>MM456M</t>
+          <t>MM270M</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>MM464M</t>
+          <t>MM280M</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>MM478M</t>
+          <t>MM288M</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>MM482M</t>
+          <t>MM380M</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>MM486M</t>
+          <t>MM456M</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>MM502M</t>
+          <t>MM464M</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>MM506M</t>
+          <t>MM478M</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>MM514M</t>
+          <t>MM482M</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>MM522M</t>
+          <t>MM486M</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>MM536M</t>
+          <t>MM502M</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>MM542M</t>
+          <t>MM506M</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>MM544M</t>
+          <t>MM514M</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>MM546M</t>
+          <t>MM522M</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>MM551M</t>
+          <t>MM536M</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>MM574M</t>
+          <t>MM542M</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>MM588M</t>
+          <t>MM544M</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>MM592M</t>
+          <t>MM546M</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>MM604M</t>
+          <t>MM551M</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>MM624M</t>
+          <t>MM574M</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>MM636M</t>
+          <t>MM588M</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>MM638M</t>
+          <t>MM592M</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>MM647M</t>
+          <t>MM604M</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>MM656M</t>
+          <t>MM624M</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>MM658M</t>
+          <t>MM636M</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>MM660M</t>
+          <t>MM638M</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>MM664M</t>
+          <t>MM647M</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>MM668M</t>
+          <t>MM656M</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>MM673M</t>
+          <t>MM658M</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>MM674M</t>
+          <t>MM660M</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>MM676M</t>
+          <t>MM664M</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>MM680M</t>
+          <t>MM668M</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>MM702M</t>
+          <t>MM673M</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>MM718M</t>
+          <t>MM674M</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>MM742M</t>
+          <t>MM676M</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>MM744M</t>
+          <t>MM680M</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>MM752M</t>
+          <t>MM702M</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>MM768M</t>
+          <t>MM718M</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>MM772M</t>
+          <t>MM742M</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>MM774M</t>
+          <t>MM744M</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>MM776M</t>
+          <t>MM752M</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>MM778M</t>
+          <t>MM768M</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>MM788M</t>
+          <t>MM772M</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>MM794M</t>
+          <t>MM774M</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>MM798M</t>
+          <t>MM776M</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>MM800M</t>
+          <t>MM778M</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>MM802M</t>
+          <t>MM788M</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>MM806M</t>
+          <t>MM794M</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>MM808M</t>
+          <t>MM798M</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>MM810M</t>
+          <t>MM800M</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>MM816M</t>
+          <t>MM802M</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>MM826M</t>
+          <t>MM806M</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>MM830M</t>
+          <t>MM808M</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>MM832M</t>
+          <t>MM810M</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>MM834M</t>
+          <t>MM816M</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>MM838M</t>
+          <t>MM826M</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>MM842M</t>
+          <t>MM830M</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>MM858M</t>
+          <t>MM832M</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>MM860M</t>
+          <t>MM834M</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>MM862M</t>
+          <t>MM838M</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>MM864M</t>
+          <t>MM842M</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>MM866M</t>
+          <t>MM858M</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>MM872M</t>
+          <t>MM860M</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>MM878M</t>
+          <t>MM862M</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>MM880M</t>
+          <t>MM864M</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>MM886M</t>
+          <t>MM866M</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>MM896M</t>
+          <t>MM872M</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>MM908M</t>
+          <t>MM878M</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>MM910M</t>
+          <t>MM880M</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>MM912M</t>
+          <t>MM886M</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>MM914M</t>
+          <t>MM896M</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>MM924M</t>
+          <t>MM908M</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>MM928M</t>
+          <t>MM910M</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>MM934M</t>
+          <t>MM912M</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>MM940M</t>
+          <t>MM914M</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>MM944M</t>
+          <t>MM924M</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>MM946M</t>
+          <t>MM928M</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>MM952M</t>
+          <t>MM934M</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>MM956M</t>
+          <t>MM940M</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>MM958M</t>
+          <t>MM944M</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>MM960M</t>
+          <t>MM946M</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>MM962M</t>
+          <t>MM952M</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>MM964M</t>
+          <t>MM956M</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>MM968M</t>
+          <t>MM958M</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>MM972M</t>
+          <t>MM960M</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>MM974M</t>
+          <t>MM962M</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>MM976M</t>
+          <t>MM964M</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>MM980M</t>
+          <t>MM968M</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>MM982M</t>
+          <t>MM972M</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>MM9901M</t>
+          <t>MM974M</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>MM9903M</t>
+          <t>MM976M</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>MM9904M</t>
+          <t>MM980M</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>MM9906M</t>
+          <t>MM982M</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>MM9908M</t>
+          <t>MM9901M</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>MM9909M</t>
+          <t>MM9903M</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>MM9910M</t>
+          <t>MM9904M</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>MM9912M</t>
+          <t>MM9906M</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>MM9914M</t>
+          <t>MM9908M</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>MM9916M</t>
+          <t>MM9909M</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>MM9918M</t>
+          <t>MM9910M</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>MM9920M</t>
+          <t>MM9912M</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>MM9921M</t>
+          <t>MM9914M</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>MM9924M</t>
+          <t>MM9916M</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>MM9926M</t>
+          <t>MM9918M</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>MM9927M</t>
+          <t>MM9920M</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>MM9928M</t>
+          <t>MM9921M</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>MM9929M</t>
+          <t>MM9924M</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>MM9931M</t>
+          <t>MM9926M</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>MM9936M</t>
+          <t>MM9927M</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>MM9937M</t>
+          <t>MM9928M</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>MM9938M</t>
+          <t>MM9929M</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>MM9941M</t>
+          <t>MM9931M</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>MM9943M</t>
+          <t>MM9936M</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>MM9946M</t>
+          <t>MM9937M</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>MM9947M</t>
+          <t>MM9938M</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>MM9948M</t>
+          <t>MM9941M</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>MM9952M</t>
+          <t>MM9943M</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t>MM9953M</t>
+          <t>MM9946M</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>MM9954M</t>
+          <t>MM9947M</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t>MM9956M</t>
+          <t>MM9948M</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>MM9957M</t>
+          <t>MM9952M</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>MM9958M</t>
+          <t>MM9953M</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>MM9959M</t>
+          <t>MM9954M</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>MM9960M</t>
+          <t>MM9956M</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>MM9961M</t>
+          <t>MM9957M</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>MM9962M</t>
+          <t>MM9958M</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>MM9963M</t>
+          <t>MM9959M</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
         <is>
-          <t>MM9964M</t>
+          <t>MM9960M</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>MM9965M</t>
+          <t>MM9961M</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
         <is>
-          <t>MM9966M</t>
+          <t>MM9962M</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
         <is>
-          <t>MM9968M</t>
+          <t>MM9963M</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" s="2" t="inlineStr">
         <is>
-          <t>MM9969M</t>
+          <t>MM9964M</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
         <is>
-          <t>MM9970M</t>
+          <t>MM9965M</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MM9966M</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>MRL002</t>
+          <t>MM9968M</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
         <is>
-          <t>MTPV1</t>
+          <t>MM9969M</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
         <is>
-          <t>MTPV2</t>
+          <t>MM9970M</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="2" t="inlineStr">
         <is>
-          <t>N458</t>
+          <t>MRL001</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
         <is>
-          <t>N460</t>
+          <t>MRL002</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" s="2" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>MTPV1</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>MTPV2</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="2" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>N458</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" s="2" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>N460</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="2" t="inlineStr">
         <is>
-          <t>NR6</t>
+          <t>N466</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
         <is>
-          <t>NR10</t>
+          <t>N469</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" s="2" t="inlineStr">
         <is>
-          <t>NR11</t>
+          <t>NR4</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
         <is>
-          <t>NR12</t>
+          <t>NR5</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" s="2" t="inlineStr">
         <is>
-          <t>NR13</t>
+          <t>NR6</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" s="2" t="inlineStr">
         <is>
-          <t>NR14</t>
+          <t>NR10</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
         <is>
-          <t>NR17</t>
+          <t>NR11</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="2" t="inlineStr">
         <is>
-          <t>NR20</t>
+          <t>NR12</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
         <is>
-          <t>NR35</t>
+          <t>NR13</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="2" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>NR14</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="2" t="inlineStr">
         <is>
-          <t>NR44</t>
+          <t>NR17</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" s="2" t="inlineStr">
         <is>
-          <t>NR46</t>
+          <t>NR20</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" s="2" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>NR35</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" s="2" t="inlineStr">
         <is>
-          <t>NR52</t>
+          <t>NR37</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" s="2" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>NR44</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" s="2" t="inlineStr">
         <is>
-          <t>NR56</t>
+          <t>NR46</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" s="2" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR47</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" s="2" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR52</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" s="2" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR54</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR56</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" s="2" t="inlineStr">
         <is>
-          <t>NR76</t>
+          <t>NR64</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR65</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" s="2" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR68</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" s="2" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR75</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" s="2" t="inlineStr">
         <is>
-          <t>NR88</t>
+          <t>NR76</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
         <is>
-          <t>NR91</t>
+          <t>NR78</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="2" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR82</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR83</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR88</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>NR91</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" s="2" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR93</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
         <is>
-          <t>NR107</t>
+          <t>NR94</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" s="2" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR95</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR97</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" s="2" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR102</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR107</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>NR109</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>NR112</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
         <is>
-          <t>PKLA4</t>
+          <t>NR113</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>NR115</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>PB4</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>PKLA4</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>QE001</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
         <is>
-          <t>QL009</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>QL016</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
         <is>
-          <t>QL019</t>
+          <t>QL004</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="2" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QL009</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
         <is>
-          <t>QR5400</t>
+          <t>QL016</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" s="2" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QL019</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
         <is>
-          <t>RA2302</t>
+          <t>QR1744</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" s="2" t="inlineStr">
         <is>
-          <t>RA2303</t>
+          <t>QR1771</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="2" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>QR5400</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" s="2" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" s="2" t="inlineStr">
         <is>
-          <t>RM93</t>
+          <t>RA2302</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" s="2" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>RA2303</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" s="2" t="inlineStr">
         <is>
-          <t>SCT008</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="2" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>RL301</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="2" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>RM93</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="2" t="inlineStr">
         <is>
-          <t>SO3</t>
+          <t>SCT001</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="2" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>SCT008</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="2" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>SCT009</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" s="2" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>SCT013</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" s="2" t="inlineStr">
         <is>
-          <t>T373</t>
+          <t>SO3</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" s="2" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>SSR101</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" s="2" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>SSR102</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="A472" s="2" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>SSR103</t>
         </is>
       </c>
     </row>
     <row r="473">
       <c r="A473" s="2" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>SSR104</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="A474" s="2" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>T373</t>
         </is>
       </c>
     </row>
     <row r="475">
       <c r="A475" s="2" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>TE2801</t>
         </is>
       </c>
     </row>
     <row r="476">
       <c r="A476" s="2" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>TE2803</t>
         </is>
       </c>
     </row>
     <row r="477">
       <c r="A477" s="2" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>TE2805</t>
         </is>
       </c>
     </row>
     <row r="478">
       <c r="A478" s="2" t="inlineStr">
         <is>
-          <t>TT02</t>
+          <t>TE2807</t>
         </is>
       </c>
     </row>
     <row r="479">
       <c r="A479" s="2" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TE2808</t>
         </is>
       </c>
     </row>
     <row r="480">
       <c r="A480" s="2" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TE2813</t>
         </is>
       </c>
     </row>
     <row r="481">
       <c r="A481" s="2" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TE2814</t>
         </is>
       </c>
     </row>
     <row r="482">
       <c r="A482" s="2" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TJ096</t>
         </is>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="2" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TT02</t>
         </is>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="2" t="inlineStr">
         <is>
-          <t>TT104</t>
+          <t>TT03</t>
         </is>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="2" t="inlineStr">
         <is>
-          <t>TT105</t>
+          <t>TT04</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="2" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TT05</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="2" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TT08</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" s="2" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT103</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" s="2" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT104</t>
         </is>
       </c>
     </row>
     <row r="490">
       <c r="A490" s="2" t="inlineStr">
         <is>
-          <t>TT123</t>
+          <t>TT105</t>
         </is>
       </c>
     </row>
     <row r="491">
       <c r="A491" s="2" t="inlineStr">
         <is>
-          <t>TT126</t>
+          <t>TT107</t>
         </is>
       </c>
     </row>
     <row r="492">
       <c r="A492" s="2" t="inlineStr">
         <is>
-          <t>TT129</t>
+          <t>TT110</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="2" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT115</t>
         </is>
       </c>
     </row>
     <row r="494">
       <c r="A494" s="2" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT117</t>
         </is>
       </c>
     </row>
     <row r="495">
       <c r="A495" s="2" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT123</t>
         </is>
       </c>
     </row>
     <row r="496">
       <c r="A496" s="2" t="inlineStr">
         <is>
-          <t>VL04</t>
+          <t>TT126</t>
         </is>
       </c>
     </row>
     <row r="497">
       <c r="A497" s="2" t="inlineStr">
         <is>
-          <t>VL11</t>
+          <t>TT129</t>
         </is>
       </c>
     </row>
     <row r="498">
       <c r="A498" s="2" t="inlineStr">
         <is>
-          <t>VL13</t>
+          <t>TT130</t>
         </is>
       </c>
     </row>
     <row r="499">
       <c r="A499" s="2" t="inlineStr">
         <is>
-          <t>VL20</t>
+          <t>TT202</t>
         </is>
       </c>
     </row>
     <row r="500">
       <c r="A500" s="2" t="inlineStr">
         <is>
-          <t>VL22</t>
+          <t>TT206</t>
         </is>
       </c>
     </row>
     <row r="501">
       <c r="A501" s="2" t="inlineStr">
         <is>
-          <t>VL27</t>
+          <t>VL01</t>
         </is>
       </c>
     </row>
     <row r="502">
       <c r="A502" s="2" t="inlineStr">
         <is>
-          <t>VL36</t>
+          <t>VL03</t>
         </is>
       </c>
     </row>
     <row r="503">
       <c r="A503" s="2" t="inlineStr">
         <is>
-          <t>VL38</t>
+          <t>VL04</t>
         </is>
       </c>
     </row>
     <row r="504">
       <c r="A504" s="2" t="inlineStr">
         <is>
-          <t>VL43</t>
+          <t>VL11</t>
         </is>
       </c>
     </row>
     <row r="505">
       <c r="A505" s="2" t="inlineStr">
         <is>
-          <t>VL49</t>
+          <t>VL13</t>
         </is>
       </c>
     </row>
     <row r="506">
       <c r="A506" s="2" t="inlineStr">
         <is>
-          <t>VL57</t>
+          <t>VL20</t>
         </is>
       </c>
     </row>
     <row r="507">
       <c r="A507" s="2" t="inlineStr">
         <is>
-          <t>VL62</t>
+          <t>VL22</t>
         </is>
       </c>
     </row>
     <row r="508">
       <c r="A508" s="2" t="inlineStr">
         <is>
-          <t>VL67</t>
+          <t>VL27</t>
         </is>
       </c>
     </row>
     <row r="509">
       <c r="A509" s="2" t="inlineStr">
         <is>
-          <t>VL75</t>
+          <t>VL35</t>
         </is>
       </c>
     </row>
     <row r="510">
       <c r="A510" s="2" t="inlineStr">
         <is>
-          <t>VL81</t>
+          <t>VL36</t>
         </is>
       </c>
     </row>
     <row r="511">
       <c r="A511" s="2" t="inlineStr">
         <is>
-          <t>VL86</t>
+          <t>VL38</t>
         </is>
       </c>
     </row>
     <row r="512">
       <c r="A512" s="2" t="inlineStr">
         <is>
-          <t>VL87</t>
+          <t>VL43</t>
         </is>
       </c>
     </row>
     <row r="513">
       <c r="A513" s="2" t="inlineStr">
         <is>
-          <t>VL88</t>
+          <t>VL47</t>
         </is>
       </c>
     </row>
     <row r="514">
       <c r="A514" s="2" t="inlineStr">
         <is>
-          <t>VL90</t>
+          <t>VL49</t>
         </is>
       </c>
     </row>
     <row r="515">
       <c r="A515" s="2" t="inlineStr">
         <is>
-          <t>VL92</t>
+          <t>VL57</t>
         </is>
       </c>
     </row>
     <row r="516">
       <c r="A516" s="2" t="inlineStr">
         <is>
-          <t>VL99</t>
+          <t>VL62</t>
         </is>
       </c>
     </row>
     <row r="517">
       <c r="A517" s="2" t="inlineStr">
         <is>
-          <t>VL100</t>
+          <t>VL67</t>
         </is>
       </c>
     </row>
     <row r="518">
       <c r="A518" s="2" t="inlineStr">
         <is>
-          <t>VL101</t>
+          <t>VL75</t>
         </is>
       </c>
     </row>
     <row r="519">
       <c r="A519" s="2" t="inlineStr">
         <is>
-          <t>VL103</t>
+          <t>VL81</t>
         </is>
       </c>
     </row>
     <row r="520">
       <c r="A520" s="2" t="inlineStr">
         <is>
-          <t>VL107</t>
+          <t>VL86</t>
         </is>
       </c>
     </row>
     <row r="521">
       <c r="A521" s="2" t="inlineStr">
         <is>
-          <t>VL112</t>
+          <t>VL87</t>
         </is>
       </c>
     </row>
     <row r="522">
       <c r="A522" s="2" t="inlineStr">
         <is>
-          <t>VL114</t>
+          <t>VL88</t>
         </is>
       </c>
     </row>
     <row r="523">
       <c r="A523" s="2" t="inlineStr">
         <is>
-          <t>VL115</t>
+          <t>VL90</t>
         </is>
       </c>
     </row>
     <row r="524">
       <c r="A524" s="2" t="inlineStr">
         <is>
-          <t>VL121</t>
+          <t>VL92</t>
         </is>
       </c>
     </row>
     <row r="525">
       <c r="A525" s="2" t="inlineStr">
         <is>
-          <t>VL122</t>
+          <t>VL99</t>
         </is>
       </c>
     </row>
     <row r="526">
       <c r="A526" s="2" t="inlineStr">
         <is>
-          <t>VL124</t>
+          <t>VL100</t>
         </is>
       </c>
     </row>
     <row r="527">
       <c r="A527" s="2" t="inlineStr">
         <is>
-          <t>VL125</t>
+          <t>VL101</t>
         </is>
       </c>
     </row>
     <row r="528">
       <c r="A528" s="2" t="inlineStr">
         <is>
-          <t>VL126</t>
+          <t>VL103</t>
         </is>
       </c>
     </row>
     <row r="529">
       <c r="A529" s="2" t="inlineStr">
         <is>
-          <t>VL129</t>
+          <t>VL107</t>
         </is>
       </c>
     </row>
     <row r="530">
       <c r="A530" s="2" t="inlineStr">
         <is>
-          <t>VL134</t>
+          <t>VL112</t>
         </is>
       </c>
     </row>
     <row r="531">
       <c r="A531" s="2" t="inlineStr">
         <is>
-          <t>VL137</t>
+          <t>VL114</t>
         </is>
       </c>
     </row>
     <row r="532">
       <c r="A532" s="2" t="inlineStr">
         <is>
-          <t>VL139</t>
+          <t>VL115</t>
         </is>
       </c>
     </row>
     <row r="533">
       <c r="A533" s="2" t="inlineStr">
         <is>
-          <t>VL140</t>
+          <t>VL121</t>
         </is>
       </c>
     </row>
     <row r="534">
       <c r="A534" s="2" t="inlineStr">
         <is>
-          <t>VL354</t>
+          <t>VL122</t>
         </is>
       </c>
     </row>
     <row r="535">
       <c r="A535" s="2" t="inlineStr">
         <is>
-          <t>VLINE8013</t>
+          <t>VL123</t>
         </is>
       </c>
     </row>
     <row r="536">
       <c r="A536" s="2" t="inlineStr">
         <is>
-          <t>VLINE8020</t>
+          <t>VL124</t>
         </is>
       </c>
     </row>
     <row r="537">
       <c r="A537" s="2" t="inlineStr">
         <is>
-          <t>VLINE8021</t>
+          <t>VL125</t>
         </is>
       </c>
     </row>
     <row r="538">
       <c r="A538" s="2" t="inlineStr">
         <is>
-          <t>VLINE8058</t>
+          <t>VL126</t>
         </is>
       </c>
     </row>
     <row r="539">
       <c r="A539" s="2" t="inlineStr">
         <is>
-          <t>VLINE8059</t>
+          <t>VL129</t>
         </is>
       </c>
     </row>
     <row r="540">
       <c r="A540" s="2" t="inlineStr">
         <is>
-          <t>VLINE8061</t>
+          <t>VL132</t>
         </is>
       </c>
     </row>
     <row r="541">
       <c r="A541" s="2" t="inlineStr">
         <is>
-          <t>VLINE8071</t>
+          <t>VL134</t>
         </is>
       </c>
     </row>
     <row r="542">
       <c r="A542" s="2" t="inlineStr">
         <is>
-          <t>VLINE8072</t>
+          <t>VL137</t>
         </is>
       </c>
     </row>
     <row r="543">
       <c r="A543" s="2" t="inlineStr">
         <is>
-          <t>VLINE8075</t>
+          <t>VL139</t>
         </is>
       </c>
     </row>
     <row r="544">
       <c r="A544" s="2" t="inlineStr">
         <is>
-          <t>VLINE8080</t>
+          <t>VL140</t>
         </is>
       </c>
     </row>
     <row r="545">
       <c r="A545" s="2" t="inlineStr">
         <is>
-          <t>VLINE8102</t>
+          <t>VL354</t>
         </is>
       </c>
     </row>
     <row r="546">
       <c r="A546" s="2" t="inlineStr">
         <is>
-          <t>VLINE8111</t>
+          <t>VLINE8013</t>
         </is>
       </c>
     </row>
     <row r="547">
       <c r="A547" s="2" t="inlineStr">
         <is>
-          <t>VLINE8113</t>
+          <t>VLINE8020</t>
         </is>
       </c>
     </row>
     <row r="548">
       <c r="A548" s="2" t="inlineStr">
         <is>
-          <t>VLINE8115</t>
+          <t>VLINE8021</t>
         </is>
       </c>
     </row>
     <row r="549">
       <c r="A549" s="2" t="inlineStr">
         <is>
-          <t>VLINE8117</t>
+          <t>VLINE8028</t>
         </is>
       </c>
     </row>
     <row r="550">
       <c r="A550" s="2" t="inlineStr">
         <is>
-          <t>VLINE8120</t>
+          <t>VLINE8030</t>
         </is>
       </c>
     </row>
     <row r="551">
       <c r="A551" s="2" t="inlineStr">
         <is>
-          <t>VLINE8121</t>
+          <t>VLINE8058</t>
         </is>
       </c>
     </row>
     <row r="552">
       <c r="A552" s="2" t="inlineStr">
         <is>
-          <t>VLINE8122</t>
+          <t>VLINE8059</t>
         </is>
       </c>
     </row>
     <row r="553">
       <c r="A553" s="2" t="inlineStr">
         <is>
-          <t>VLINE8124</t>
+          <t>VLINE8061</t>
         </is>
       </c>
     </row>
     <row r="554">
       <c r="A554" s="2" t="inlineStr">
         <is>
-          <t>VLINE8126</t>
+          <t>VLINE8071</t>
         </is>
       </c>
     </row>
     <row r="555">
       <c r="A555" s="2" t="inlineStr">
         <is>
-          <t>VLINE8161</t>
+          <t>VLINE8072</t>
         </is>
       </c>
     </row>
     <row r="556">
       <c r="A556" s="2" t="inlineStr">
         <is>
-          <t>VLINE8163</t>
+          <t>VLINE8074</t>
         </is>
       </c>
     </row>
     <row r="557">
       <c r="A557" s="2" t="inlineStr">
         <is>
-          <t>VLINE8164</t>
+          <t>VLINE8075</t>
         </is>
       </c>
     </row>
     <row r="558">
       <c r="A558" s="2" t="inlineStr">
         <is>
-          <t>VLINE8172</t>
+          <t>VLINE8080</t>
         </is>
       </c>
     </row>
     <row r="559">
       <c r="A559" s="2" t="inlineStr">
         <is>
-          <t>VLINE8181</t>
+          <t>VLINE8081</t>
         </is>
       </c>
     </row>
     <row r="560">
       <c r="A560" s="2" t="inlineStr">
         <is>
-          <t>VLINE8183</t>
+          <t>VLINE8102</t>
         </is>
       </c>
     </row>
     <row r="561">
       <c r="A561" s="2" t="inlineStr">
         <is>
-          <t>VLINE8211</t>
+          <t>VLINE8111</t>
         </is>
       </c>
     </row>
     <row r="562">
       <c r="A562" s="2" t="inlineStr">
         <is>
-          <t>VLINE8213</t>
+          <t>VLINE8113</t>
         </is>
       </c>
     </row>
     <row r="563">
       <c r="A563" s="2" t="inlineStr">
         <is>
-          <t>VLINE8215</t>
+          <t>VLINE8115</t>
         </is>
       </c>
     </row>
     <row r="564">
       <c r="A564" s="2" t="inlineStr">
         <is>
-          <t>VLINE8217</t>
+          <t>VLINE8117</t>
         </is>
       </c>
     </row>
     <row r="565">
       <c r="A565" s="2" t="inlineStr">
         <is>
-          <t>VLINE8219</t>
+          <t>VLINE8120</t>
         </is>
       </c>
     </row>
     <row r="566">
       <c r="A566" s="2" t="inlineStr">
         <is>
-          <t>VLINE8226</t>
+          <t>VLINE8121</t>
         </is>
       </c>
     </row>
     <row r="567">
       <c r="A567" s="2" t="inlineStr">
         <is>
-          <t>VLINE8228</t>
+          <t>VLINE8122</t>
         </is>
       </c>
     </row>
     <row r="568">
       <c r="A568" s="2" t="inlineStr">
         <is>
-          <t>VLINE8230</t>
+          <t>VLINE8123</t>
         </is>
       </c>
     </row>
     <row r="569">
       <c r="A569" s="2" t="inlineStr">
         <is>
-          <t>VLINE8232</t>
+          <t>VLINE8124</t>
         </is>
       </c>
     </row>
     <row r="570">
       <c r="A570" s="2" t="inlineStr">
         <is>
-          <t>VLINE8234</t>
+          <t>VLINE8126</t>
         </is>
       </c>
     </row>
     <row r="571">
       <c r="A571" s="2" t="inlineStr">
         <is>
-          <t>VLINE8400</t>
+          <t>VLINE8128</t>
         </is>
       </c>
     </row>
     <row r="572">
       <c r="A572" s="2" t="inlineStr">
         <is>
-          <t>VLINE8405</t>
+          <t>VLINE8130</t>
         </is>
       </c>
     </row>
     <row r="573">
       <c r="A573" s="2" t="inlineStr">
         <is>
-          <t>VLINE8408</t>
+          <t>VLINE8161</t>
         </is>
       </c>
     </row>
     <row r="574">
       <c r="A574" s="2" t="inlineStr">
         <is>
-          <t>VLINE8413</t>
+          <t>VLINE8163</t>
         </is>
       </c>
     </row>
     <row r="575">
       <c r="A575" s="2" t="inlineStr">
         <is>
-          <t>VLINE8415</t>
+          <t>VLINE8164</t>
         </is>
       </c>
     </row>
     <row r="576">
       <c r="A576" s="2" t="inlineStr">
         <is>
-          <t>VLINE8417</t>
+          <t>VLINE8172</t>
         </is>
       </c>
     </row>
     <row r="577">
       <c r="A577" s="2" t="inlineStr">
         <is>
-          <t>VLINE8418</t>
+          <t>VLINE8181</t>
         </is>
       </c>
     </row>
     <row r="578">
       <c r="A578" s="2" t="inlineStr">
         <is>
-          <t>VLINE8419</t>
+          <t>VLINE8183</t>
         </is>
       </c>
     </row>
     <row r="579">
       <c r="A579" s="2" t="inlineStr">
         <is>
-          <t>VLINE8420</t>
+          <t>VLINE8184</t>
         </is>
       </c>
     </row>
     <row r="580">
       <c r="A580" s="2" t="inlineStr">
         <is>
-          <t>VLINE8421</t>
+          <t>VLINE8211</t>
         </is>
       </c>
     </row>
     <row r="581">
       <c r="A581" s="2" t="inlineStr">
         <is>
-          <t>VLINE8422</t>
+          <t>VLINE8213</t>
         </is>
       </c>
     </row>
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>VLINE8457</t>
+          <t>VLINE8215</t>
         </is>
       </c>
     </row>
     <row r="583">
       <c r="A583" s="2" t="inlineStr">
         <is>
-          <t>VLINE8459</t>
+          <t>VLINE8217</t>
         </is>
       </c>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>VLINE8460</t>
+          <t>VLINE8219</t>
         </is>
       </c>
     </row>
     <row r="585">
       <c r="A585" s="2" t="inlineStr">
         <is>
-          <t>VLINE8702</t>
+          <t>VLINE8221</t>
         </is>
       </c>
     </row>
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>VLINE8725</t>
+          <t>VLINE8226</t>
         </is>
       </c>
     </row>
     <row r="587">
       <c r="A587" s="2" t="inlineStr">
         <is>
-          <t>VLINE8727</t>
+          <t>VLINE8228</t>
         </is>
       </c>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>VLINE8729</t>
+          <t>VLINE8230</t>
         </is>
       </c>
     </row>
     <row r="589">
       <c r="A589" s="2" t="inlineStr">
         <is>
-          <t>VLINE8731</t>
+          <t>VLINE8232</t>
         </is>
       </c>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>VLINE8733</t>
+          <t>VLINE8234</t>
         </is>
       </c>
     </row>
     <row r="591">
       <c r="A591" s="2" t="inlineStr">
         <is>
-          <t>VLINE8735</t>
+          <t>VLINE8236</t>
         </is>
       </c>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>VLINE8737</t>
+          <t>VLINE8400</t>
         </is>
       </c>
     </row>
     <row r="593">
       <c r="A593" s="2" t="inlineStr">
         <is>
-          <t>VLINE8739</t>
+          <t>VLINE8405</t>
         </is>
       </c>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>VLINE8741</t>
+          <t>VLINE8408</t>
         </is>
       </c>
     </row>
     <row r="595">
       <c r="A595" s="2" t="inlineStr">
         <is>
-          <t>VLINE8742</t>
+          <t>VLINE8413</t>
         </is>
       </c>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>VLINE8743</t>
+          <t>VLINE8415</t>
         </is>
       </c>
     </row>
     <row r="597">
       <c r="A597" s="2" t="inlineStr">
         <is>
-          <t>VLINE8744</t>
+          <t>VLINE8417</t>
         </is>
       </c>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>VLINE8745</t>
+          <t>VLINE8418</t>
         </is>
       </c>
     </row>
     <row r="599">
       <c r="A599" s="2" t="inlineStr">
         <is>
-          <t>VLINE8746</t>
+          <t>VLINE8419</t>
         </is>
       </c>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>VLINE8748</t>
+          <t>VLINE8420</t>
         </is>
       </c>
     </row>
     <row r="601">
       <c r="A601" s="2" t="inlineStr">
         <is>
-          <t>VLINE8750</t>
+          <t>VLINE8421</t>
         </is>
       </c>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>VLINE8752</t>
+          <t>VLINE8422</t>
         </is>
       </c>
     </row>
     <row r="603">
       <c r="A603" s="2" t="inlineStr">
         <is>
-          <t>VLINE8754</t>
+          <t>VLINE8423</t>
         </is>
       </c>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>VLINE8756</t>
+          <t>VLINE8424</t>
         </is>
       </c>
     </row>
     <row r="605">
       <c r="A605" s="2" t="inlineStr">
         <is>
-          <t>VLINE8762</t>
+          <t>VLINE8428</t>
         </is>
       </c>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>VLINE8819</t>
+          <t>VLINE8430</t>
         </is>
       </c>
     </row>
     <row r="607">
       <c r="A607" s="2" t="inlineStr">
         <is>
-          <t>VLINE8863</t>
+          <t>VLINE8457</t>
         </is>
       </c>
     </row>
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>VR77</t>
+          <t>VLINE8459</t>
         </is>
       </c>
     </row>
     <row r="609">
       <c r="A609" s="2" t="inlineStr">
         <is>
-          <t>XP2001</t>
+          <t>VLINE8460</t>
         </is>
       </c>
     </row>
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>VLINE8461</t>
         </is>
       </c>
     </row>
     <row r="611">
       <c r="A611" s="2" t="inlineStr">
         <is>
-          <t>XP2006</t>
+          <t>VLINE8702</t>
         </is>
       </c>
     </row>
     <row r="612">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>VLINE8725</t>
         </is>
       </c>
     </row>
     <row r="613">
       <c r="A613" s="2" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>VLINE8727</t>
         </is>
       </c>
     </row>
     <row r="614">
       <c r="A614" s="2" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>VLINE8729</t>
         </is>
       </c>
     </row>
     <row r="615">
       <c r="A615" s="2" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>VLINE8731</t>
         </is>
       </c>
     </row>
     <row r="616">
       <c r="A616" s="2" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>VLINE8733</t>
         </is>
       </c>
     </row>
     <row r="617">
       <c r="A617" s="2" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>VLINE8735</t>
         </is>
       </c>
     </row>
     <row r="618">
       <c r="A618" s="2" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>VLINE8737</t>
         </is>
       </c>
     </row>
     <row r="619">
       <c r="A619" s="2" t="inlineStr">
         <is>
-          <t>XRN003</t>
+          <t>VLINE8739</t>
         </is>
       </c>
     </row>
     <row r="620">
       <c r="A620" s="2" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>VLINE8741</t>
         </is>
       </c>
     </row>
     <row r="621">
       <c r="A621" s="2" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>VLINE8742</t>
         </is>
       </c>
     </row>
     <row r="622">
       <c r="A622" s="2" t="inlineStr">
         <is>
-          <t>XRN010</t>
+          <t>VLINE8743</t>
         </is>
       </c>
     </row>
     <row r="623">
       <c r="A623" s="2" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>VLINE8744</t>
         </is>
       </c>
     </row>
     <row r="624">
       <c r="A624" s="2" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>VLINE8745</t>
         </is>
       </c>
     </row>
     <row r="625">
       <c r="A625" s="2" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>VLINE8746</t>
         </is>
       </c>
     </row>
     <row r="626">
       <c r="A626" s="2" t="inlineStr">
         <is>
-          <t>XRN022</t>
+          <t>VLINE8747</t>
         </is>
       </c>
     </row>
     <row r="627">
       <c r="A627" s="2" t="inlineStr">
         <is>
-          <t>XRN028</t>
+          <t>VLINE8748</t>
         </is>
       </c>
     </row>
     <row r="628">
       <c r="A628" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8750</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8752</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8754</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8756</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8758</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8760</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8762</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8764</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8819</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8862</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="2" t="inlineStr">
+        <is>
+          <t>VLINE8863</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="2" t="inlineStr">
+        <is>
+          <t>VR77</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="2" t="inlineStr">
+        <is>
+          <t>WOLL408</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="2" t="inlineStr">
+        <is>
+          <t>WOLL430</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="2" t="inlineStr">
+        <is>
+          <t>XP2001</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="2" t="inlineStr">
+        <is>
+          <t>XP2005</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="2" t="inlineStr">
+        <is>
+          <t>XP2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="2" t="inlineStr">
+        <is>
+          <t>XP2008</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="2" t="inlineStr">
+        <is>
+          <t>XP2009</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="2" t="inlineStr">
+        <is>
+          <t>XP2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="2" t="inlineStr">
+        <is>
+          <t>XP2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="2" t="inlineStr">
+        <is>
+          <t>XP2013</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" s="2" t="inlineStr">
+        <is>
+          <t>XP2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" s="2" t="inlineStr">
+        <is>
+          <t>XP2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" s="2" t="inlineStr">
+        <is>
+          <t>XP2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" s="2" t="inlineStr">
+        <is>
+          <t>XRN003</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" s="2" t="inlineStr">
+        <is>
+          <t>XRN005</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="2" t="inlineStr">
+        <is>
+          <t>XRN009</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="2" t="inlineStr">
+        <is>
+          <t>XRN010</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" s="2" t="inlineStr">
+        <is>
+          <t>XRN017</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="2" t="inlineStr">
+        <is>
+          <t>XRN018</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="2" t="inlineStr">
+        <is>
+          <t>XRN021</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" s="2" t="inlineStr">
+        <is>
+          <t>XRN022</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" s="2" t="inlineStr">
+        <is>
+          <t>XRN028</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="2" t="inlineStr">
         <is>
           <t>XRN029</t>
         </is>

</xml_diff>

<commit_message>
Update RailOps database files - 2026-04-30 03:03:31 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A662"/>
+  <dimension ref="A1:A679"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -937,4149 +937,4268 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>8239</t>
+          <t>8238</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>8240</t>
+          <t>8239</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>8249</t>
+          <t>8240</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>9025</t>
+          <t>8249</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>9029</t>
+          <t>9025</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>9203</t>
+          <t>9029</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>9301</t>
+          <t>9203</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>9302</t>
+          <t>9301</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>9305</t>
+          <t>9302</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>9307</t>
+          <t>9305</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>9311</t>
+          <t>9307</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>9312</t>
+          <t>9311</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>9313</t>
+          <t>9312</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>9406</t>
+          <t>9313</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>9408</t>
+          <t>9406</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>9410</t>
+          <t>9408</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>42103</t>
+          <t>9410</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>42107</t>
+          <t>42103</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>44202</t>
+          <t>42107</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>44204</t>
+          <t>44202</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>44208</t>
+          <t>44204</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>ACB4403</t>
+          <t>44208</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>ACB4404</t>
+          <t>ACB4403</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>ACD6046</t>
+          <t>ACB4404</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>ACD6047</t>
+          <t>ACD6046</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>ACD6049</t>
+          <t>ACD6047</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>ACD6052</t>
+          <t>ACD6049</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>ACD6056</t>
+          <t>ACD6052</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>ACD6057</t>
+          <t>ACD6056</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>ACD6058</t>
+          <t>ACD6057</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>ACD6059</t>
+          <t>ACD6058</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>ACD6065</t>
+          <t>ACD6059</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>ACD6066</t>
+          <t>ACD6065</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>ACD6069</t>
+          <t>ACD6066</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>ACD6071</t>
+          <t>ACD6069</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>ACD6073</t>
+          <t>ACD6071</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>ACD6074</t>
+          <t>ACD6073</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>BL26</t>
+          <t>ACD6074</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>BL31</t>
+          <t>BL26</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>BL33</t>
+          <t>BL31</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>C502</t>
+          <t>BL33</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>C504</t>
+          <t>BX056</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>C506</t>
+          <t>C502</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>C509</t>
+          <t>C504</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>C510</t>
+          <t>C506</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>CEY004</t>
+          <t>C509</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>CEY006</t>
+          <t>C510</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>CEY007</t>
+          <t>CEY004</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>CF4401</t>
+          <t>CEY006</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>CF4405</t>
+          <t>CEY007</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>CF4407</t>
+          <t>CF4401</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>CF4410</t>
+          <t>CF4405</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>CF4412</t>
+          <t>CF4407</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>CF4420</t>
+          <t>CF4410</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>CF4421</t>
+          <t>CF4412</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>CF4424</t>
+          <t>CF4420</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>CF4425</t>
+          <t>CF4421</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>CF4427</t>
+          <t>CF4424</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>CF4429</t>
+          <t>CF4425</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>CLF2</t>
+          <t>CF4427</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>CLP12</t>
+          <t>CF4429</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>CLP13</t>
+          <t>CLF2</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>CLP17</t>
+          <t>CLP12</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>CM3304</t>
+          <t>CLP13</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>CM3307</t>
+          <t>CLP17</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>CSR010</t>
+          <t>CM3304</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>CSR015</t>
+          <t>CM3307</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>CSR017</t>
+          <t>CSR010</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>CSR019</t>
+          <t>CSR015</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>CSR020</t>
+          <t>CSR017</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>CSR021</t>
+          <t>CSR019</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>CSR023</t>
+          <t>CSR020</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>DS003</t>
+          <t>CSR021</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>EA2502</t>
+          <t>CSR023</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>EA2503</t>
+          <t>DS003</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>EA2506</t>
+          <t>EA2502</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>EA2507</t>
+          <t>EA2503</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>EC2521</t>
+          <t>EA2506</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>EC2525</t>
+          <t>EA2507</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>EC2526</t>
+          <t>EC2521</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>FIE001</t>
+          <t>EC2525</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>FIE003</t>
+          <t>EC2526</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>G513</t>
+          <t>FIE001</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>G514</t>
+          <t>FIE003</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>G516</t>
+          <t>G513</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>G521</t>
+          <t>G514</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>G532</t>
+          <t>G516</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>G533</t>
+          <t>G521</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>G534</t>
+          <t>G532</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>G536</t>
+          <t>G533</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>GL103</t>
+          <t>G534</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>GL105</t>
+          <t>G536</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>GL108</t>
+          <t>GL103</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>GL111</t>
+          <t>GL105</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>GM46</t>
+          <t>GL108</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>GWA002</t>
+          <t>GL111</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>GWA004</t>
+          <t>GM37</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>GWA008</t>
+          <t>GM46</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>GWA009</t>
+          <t>GWA002</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>GWB102</t>
+          <t>GWA004</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>GWB103</t>
+          <t>GWA008</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>GWB104</t>
+          <t>GWA009</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>GWU008</t>
+          <t>GWB102</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>GWU013</t>
+          <t>GWB103</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>GWU014</t>
+          <t>GWB104</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>GWU015</t>
+          <t>GWU008</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>HM2701</t>
+          <t>GWU012</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>HM2702</t>
+          <t>GWU013</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>HM2703</t>
+          <t>GWU014</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>HM2705</t>
+          <t>GWU015</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>HM2706</t>
+          <t>HM2701</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>HM2707</t>
+          <t>HM2702</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>HM2751</t>
+          <t>HM2703</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>HM2752</t>
+          <t>HM2705</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>HM2753</t>
+          <t>HM2706</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>HM2755</t>
+          <t>HM2707</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>HM2756</t>
+          <t>HM2751</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>HM2757</t>
+          <t>HM2752</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>JP9750</t>
+          <t>HM2753</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>LDP002</t>
+          <t>HM2755</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>LDP004</t>
+          <t>HM2756</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>LDP008</t>
+          <t>HM2757</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>LE2851</t>
+          <t>JP9750</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>LE2853</t>
+          <t>LDP002</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>LE2854</t>
+          <t>LDP004</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>LE2855</t>
+          <t>LDP008</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>LE2857</t>
+          <t>LE2851</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>LE2858</t>
+          <t>LE2853</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>LE2859</t>
+          <t>LE2854</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>LE2862</t>
+          <t>LE2855</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>LE2863</t>
+          <t>LE2857</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>LE2864</t>
+          <t>LE2858</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>LZ3114</t>
+          <t>LE2859</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>M437</t>
+          <t>LE2862</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>M865</t>
+          <t>LE2863</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>MAN004</t>
+          <t>LE2864</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>MAN005</t>
+          <t>LZ3114</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>MAN007</t>
+          <t>M437</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>MAN011</t>
+          <t>M865</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>MAN013</t>
+          <t>MAN004</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>MAN015</t>
+          <t>MAN005</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>MAN016</t>
+          <t>MAN007</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>MAN017</t>
+          <t>MAN011</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>MM02</t>
+          <t>MAN013</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>MM2M</t>
+          <t>MAN015</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>MM4M</t>
+          <t>MAN016</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>MM8M</t>
+          <t>MAN017</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>MM14M</t>
+          <t>MM02</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>MM32M</t>
+          <t>MM2M</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>MM38M</t>
+          <t>MM4M</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>MM40M</t>
+          <t>MM8M</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>MM42M</t>
+          <t>MM14M</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>MM44M</t>
+          <t>MM32M</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>MM48M</t>
+          <t>MM38M</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>MM50M</t>
+          <t>MM40M</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>MM52M</t>
+          <t>MM42M</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>MM64M</t>
+          <t>MM44M</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>MM76M</t>
+          <t>MM48M</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>MM78M</t>
+          <t>MM50M</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>MM80M</t>
+          <t>MM52M</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>MM82M</t>
+          <t>MM64M</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>MM84M</t>
+          <t>MM76M</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>MM86M</t>
+          <t>MM78M</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>MM92M</t>
+          <t>MM80M</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>MM94M</t>
+          <t>MM82M</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>MM96M</t>
+          <t>MM84M</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>MM98M</t>
+          <t>MM86M</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>MM99M</t>
+          <t>MM92M</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>MM122M</t>
+          <t>MM94M</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>MM130M</t>
+          <t>MM96M</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>MM152M</t>
+          <t>MM98M</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>MM156M</t>
+          <t>MM99M</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>MM158M</t>
+          <t>MM122M</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>MM172M</t>
+          <t>MM130M</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>MM178M</t>
+          <t>MM152M</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>MM192M</t>
+          <t>MM156M</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>MM212M</t>
+          <t>MM158M</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>MM214M</t>
+          <t>MM172M</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>MM216M</t>
+          <t>MM178M</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>MM232M</t>
+          <t>MM192M</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>MM236M</t>
+          <t>MM212M</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>MM240M</t>
+          <t>MM214M</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>MM246M</t>
+          <t>MM216M</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>MM260M</t>
+          <t>MM232M</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>MM264M</t>
+          <t>MM236M</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>MM266M</t>
+          <t>MM240M</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>MM268M</t>
+          <t>MM246M</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>MM270M</t>
+          <t>MM260M</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>MM280M</t>
+          <t>MM264M</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>MM288M</t>
+          <t>MM266M</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>MM380M</t>
+          <t>MM268M</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>MM456M</t>
+          <t>MM270M</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>MM464M</t>
+          <t>MM280M</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>MM478M</t>
+          <t>MM288M</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>MM482M</t>
+          <t>MM380M</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>MM486M</t>
+          <t>MM456M</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>MM502M</t>
+          <t>MM464M</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>MM506M</t>
+          <t>MM478M</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>MM514M</t>
+          <t>MM482M</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>MM522M</t>
+          <t>MM486M</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>MM536M</t>
+          <t>MM502M</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>MM542M</t>
+          <t>MM506M</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>MM544M</t>
+          <t>MM514M</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>MM546M</t>
+          <t>MM522M</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>MM551M</t>
+          <t>MM536M</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>MM574M</t>
+          <t>MM542M</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>MM588M</t>
+          <t>MM544M</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>MM592M</t>
+          <t>MM546M</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>MM604M</t>
+          <t>MM551M</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>MM624M</t>
+          <t>MM574M</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>MM636M</t>
+          <t>MM588M</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>MM638M</t>
+          <t>MM592M</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>MM647M</t>
+          <t>MM604M</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>MM656M</t>
+          <t>MM624M</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>MM658M</t>
+          <t>MM636M</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>MM660M</t>
+          <t>MM638M</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>MM664M</t>
+          <t>MM647M</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>MM668M</t>
+          <t>MM656M</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>MM673M</t>
+          <t>MM658M</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>MM674M</t>
+          <t>MM660M</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>MM676M</t>
+          <t>MM664M</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>MM680M</t>
+          <t>MM668M</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>MM702M</t>
+          <t>MM673M</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>MM718M</t>
+          <t>MM674M</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>MM742M</t>
+          <t>MM676M</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>MM744M</t>
+          <t>MM680M</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>MM752M</t>
+          <t>MM702M</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>MM768M</t>
+          <t>MM718M</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>MM772M</t>
+          <t>MM742M</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>MM774M</t>
+          <t>MM744M</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>MM776M</t>
+          <t>MM752M</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>MM778M</t>
+          <t>MM768M</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>MM788M</t>
+          <t>MM772M</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>MM794M</t>
+          <t>MM774M</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>MM798M</t>
+          <t>MM776M</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>MM800M</t>
+          <t>MM778M</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>MM802M</t>
+          <t>MM784M</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>MM806M</t>
+          <t>MM788M</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>MM808M</t>
+          <t>MM794M</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>MM810M</t>
+          <t>MM798M</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>MM816M</t>
+          <t>MM800M</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>MM826M</t>
+          <t>MM802M</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>MM830M</t>
+          <t>MM806M</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>MM832M</t>
+          <t>MM808M</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>MM834M</t>
+          <t>MM810M</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>MM838M</t>
+          <t>MM816M</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>MM842M</t>
+          <t>MM826M</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>MM858M</t>
+          <t>MM830M</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>MM860M</t>
+          <t>MM832M</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>MM862M</t>
+          <t>MM834M</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>MM864M</t>
+          <t>MM838M</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>MM866M</t>
+          <t>MM842M</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>MM872M</t>
+          <t>MM858M</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>MM878M</t>
+          <t>MM860M</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>MM880M</t>
+          <t>MM862M</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>MM886M</t>
+          <t>MM864M</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>MM896M</t>
+          <t>MM866M</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>MM908M</t>
+          <t>MM872M</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>MM910M</t>
+          <t>MM878M</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>MM912M</t>
+          <t>MM880M</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>MM914M</t>
+          <t>MM886M</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>MM924M</t>
+          <t>MM896M</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>MM928M</t>
+          <t>MM908M</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>MM934M</t>
+          <t>MM910M</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>MM940M</t>
+          <t>MM912M</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>MM944M</t>
+          <t>MM914M</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>MM946M</t>
+          <t>MM924M</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>MM952M</t>
+          <t>MM928M</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>MM956M</t>
+          <t>MM934M</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>MM958M</t>
+          <t>MM940M</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>MM960M</t>
+          <t>MM944M</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>MM962M</t>
+          <t>MM946M</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>MM964M</t>
+          <t>MM952M</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>MM968M</t>
+          <t>MM956M</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>MM972M</t>
+          <t>MM958M</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>MM974M</t>
+          <t>MM960M</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>MM976M</t>
+          <t>MM962M</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>MM980M</t>
+          <t>MM964M</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>MM982M</t>
+          <t>MM968M</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>MM9901M</t>
+          <t>MM972M</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>MM9903M</t>
+          <t>MM974M</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>MM9904M</t>
+          <t>MM976M</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>MM9906M</t>
+          <t>MM980M</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>MM9908M</t>
+          <t>MM982M</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>MM9909M</t>
+          <t>MM9901M</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>MM9910M</t>
+          <t>MM9903M</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>MM9912M</t>
+          <t>MM9904M</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>MM9914M</t>
+          <t>MM9906M</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>MM9916M</t>
+          <t>MM9908M</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>MM9918M</t>
+          <t>MM9909M</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>MM9920M</t>
+          <t>MM9910M</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>MM9921M</t>
+          <t>MM9912M</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>MM9924M</t>
+          <t>MM9914M</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>MM9926M</t>
+          <t>MM9916M</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>MM9927M</t>
+          <t>MM9918M</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>MM9928M</t>
+          <t>MM9920M</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>MM9929M</t>
+          <t>MM9921M</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>MM9931M</t>
+          <t>MM9924M</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>MM9936M</t>
+          <t>MM9926M</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>MM9937M</t>
+          <t>MM9927M</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>MM9938M</t>
+          <t>MM9928M</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>MM9941M</t>
+          <t>MM9929M</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>MM9943M</t>
+          <t>MM9931M</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t>MM9946M</t>
+          <t>MM9936M</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>MM9947M</t>
+          <t>MM9937M</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t>MM9948M</t>
+          <t>MM9938M</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>MM9952M</t>
+          <t>MM9941M</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>MM9953M</t>
+          <t>MM9943M</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>MM9954M</t>
+          <t>MM9946M</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>MM9956M</t>
+          <t>MM9947M</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>MM9957M</t>
+          <t>MM9948M</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>MM9958M</t>
+          <t>MM9952M</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>MM9959M</t>
+          <t>MM9953M</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
         <is>
-          <t>MM9960M</t>
+          <t>MM9954M</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>MM9961M</t>
+          <t>MM9956M</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
         <is>
-          <t>MM9962M</t>
+          <t>MM9957M</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
         <is>
-          <t>MM9963M</t>
+          <t>MM9958M</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" s="2" t="inlineStr">
         <is>
-          <t>MM9964M</t>
+          <t>MM9959M</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
         <is>
-          <t>MM9965M</t>
+          <t>MM9960M</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
         <is>
-          <t>MM9966M</t>
+          <t>MM9961M</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>MM9968M</t>
+          <t>MM9962M</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
         <is>
-          <t>MM9969M</t>
+          <t>MM9963M</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
         <is>
-          <t>MM9970M</t>
+          <t>MM9964M</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="2" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MM9965M</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
         <is>
-          <t>MRL002</t>
+          <t>MM9966M</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" s="2" t="inlineStr">
         <is>
-          <t>MTPV1</t>
+          <t>MM9968M</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
         <is>
-          <t>MTPV2</t>
+          <t>MM9969M</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="2" t="inlineStr">
         <is>
-          <t>N458</t>
+          <t>MM9970M</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" s="2" t="inlineStr">
         <is>
-          <t>N460</t>
+          <t>MRL001</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="2" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>MRL002</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>MTPV1</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" s="2" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>MTPV2</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>N453</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" s="2" t="inlineStr">
         <is>
-          <t>NR6</t>
+          <t>N458</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" s="2" t="inlineStr">
         <is>
-          <t>NR10</t>
+          <t>N460</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
         <is>
-          <t>NR11</t>
+          <t>N466</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="2" t="inlineStr">
         <is>
-          <t>NR12</t>
+          <t>N469</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
         <is>
-          <t>NR13</t>
+          <t>NR4</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="2" t="inlineStr">
         <is>
-          <t>NR14</t>
+          <t>NR5</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="2" t="inlineStr">
         <is>
-          <t>NR17</t>
+          <t>NR6</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" s="2" t="inlineStr">
         <is>
-          <t>NR20</t>
+          <t>NR10</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" s="2" t="inlineStr">
         <is>
-          <t>NR35</t>
+          <t>NR11</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" s="2" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>NR12</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" s="2" t="inlineStr">
         <is>
-          <t>NR44</t>
+          <t>NR13</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" s="2" t="inlineStr">
         <is>
-          <t>NR46</t>
+          <t>NR14</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" s="2" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>NR17</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" s="2" t="inlineStr">
         <is>
-          <t>NR52</t>
+          <t>NR20</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" s="2" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>NR31</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t>NR56</t>
+          <t>NR35</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" s="2" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR37</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR44</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" s="2" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR46</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" s="2" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR47</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" s="2" t="inlineStr">
         <is>
-          <t>NR76</t>
+          <t>NR52</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR54</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="2" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR56</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR64</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
         <is>
-          <t>NR88</t>
+          <t>NR65</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>NR91</t>
+          <t>NR68</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" s="2" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR75</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR76</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" s="2" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR78</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>NR82</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" s="2" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR83</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t>NR107</t>
+          <t>NR88</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR91</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR93</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR94</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR95</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>NR97</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>NR102</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
         <is>
-          <t>PKLA4</t>
+          <t>NR107</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>NR109</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>NR112</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>NR113</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>NR115</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>PB4</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>PKLA4</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="2" t="inlineStr">
         <is>
-          <t>QL009</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
         <is>
-          <t>QL016</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" s="2" t="inlineStr">
         <is>
-          <t>QL019</t>
+          <t>QE001</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" s="2" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="2" t="inlineStr">
         <is>
-          <t>QR5400</t>
+          <t>QL004</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" s="2" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" s="2" t="inlineStr">
         <is>
-          <t>RA2302</t>
+          <t>QL009</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" s="2" t="inlineStr">
         <is>
-          <t>RA2303</t>
+          <t>QL016</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" s="2" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>QL019</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="2" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>QR1744</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="2" t="inlineStr">
         <is>
-          <t>RM93</t>
+          <t>QR1771</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="2" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>QR5400</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="2" t="inlineStr">
         <is>
-          <t>SCT008</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="2" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>RA2302</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" s="2" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>RA2303</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" s="2" t="inlineStr">
         <is>
-          <t>SO3</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" s="2" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>RL301</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" s="2" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>RL309</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="A472" s="2" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>RM93</t>
         </is>
       </c>
     </row>
     <row r="473">
       <c r="A473" s="2" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>SCT001</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="A474" s="2" t="inlineStr">
         <is>
-          <t>T373</t>
+          <t>SCT008</t>
         </is>
       </c>
     </row>
     <row r="475">
       <c r="A475" s="2" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>SCT009</t>
         </is>
       </c>
     </row>
     <row r="476">
       <c r="A476" s="2" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>SCT013</t>
         </is>
       </c>
     </row>
     <row r="477">
       <c r="A477" s="2" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>SM636B</t>
         </is>
       </c>
     </row>
     <row r="478">
       <c r="A478" s="2" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>SO3</t>
         </is>
       </c>
     </row>
     <row r="479">
       <c r="A479" s="2" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>SSR101</t>
         </is>
       </c>
     </row>
     <row r="480">
       <c r="A480" s="2" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>SSR102</t>
         </is>
       </c>
     </row>
     <row r="481">
       <c r="A481" s="2" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>SSR103</t>
         </is>
       </c>
     </row>
     <row r="482">
       <c r="A482" s="2" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>SSR104</t>
         </is>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="2" t="inlineStr">
         <is>
-          <t>TT02</t>
+          <t>T373</t>
         </is>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="2" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TE2801</t>
         </is>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="2" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TE2803</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="2" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TE2804</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="2" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TE2805</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" s="2" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TE2807</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" s="2" t="inlineStr">
         <is>
-          <t>TT104</t>
+          <t>TE2808</t>
         </is>
       </c>
     </row>
     <row r="490">
       <c r="A490" s="2" t="inlineStr">
         <is>
-          <t>TT105</t>
+          <t>TE2813</t>
         </is>
       </c>
     </row>
     <row r="491">
       <c r="A491" s="2" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TE2814</t>
         </is>
       </c>
     </row>
     <row r="492">
       <c r="A492" s="2" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TJ096</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="2" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT02</t>
         </is>
       </c>
     </row>
     <row r="494">
       <c r="A494" s="2" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT03</t>
         </is>
       </c>
     </row>
     <row r="495">
       <c r="A495" s="2" t="inlineStr">
         <is>
-          <t>TT123</t>
+          <t>TT04</t>
         </is>
       </c>
     </row>
     <row r="496">
       <c r="A496" s="2" t="inlineStr">
         <is>
-          <t>TT126</t>
+          <t>TT05</t>
         </is>
       </c>
     </row>
     <row r="497">
       <c r="A497" s="2" t="inlineStr">
         <is>
-          <t>TT129</t>
+          <t>TT08</t>
         </is>
       </c>
     </row>
     <row r="498">
       <c r="A498" s="2" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT103</t>
         </is>
       </c>
     </row>
     <row r="499">
       <c r="A499" s="2" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT104</t>
         </is>
       </c>
     </row>
     <row r="500">
       <c r="A500" s="2" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT105</t>
         </is>
       </c>
     </row>
     <row r="501">
       <c r="A501" s="2" t="inlineStr">
         <is>
-          <t>VL01</t>
+          <t>TT107</t>
         </is>
       </c>
     </row>
     <row r="502">
       <c r="A502" s="2" t="inlineStr">
         <is>
-          <t>VL03</t>
+          <t>TT110</t>
         </is>
       </c>
     </row>
     <row r="503">
       <c r="A503" s="2" t="inlineStr">
         <is>
-          <t>VL04</t>
+          <t>TT115</t>
         </is>
       </c>
     </row>
     <row r="504">
       <c r="A504" s="2" t="inlineStr">
         <is>
-          <t>VL11</t>
+          <t>TT117</t>
         </is>
       </c>
     </row>
     <row r="505">
       <c r="A505" s="2" t="inlineStr">
         <is>
-          <t>VL13</t>
+          <t>TT123</t>
         </is>
       </c>
     </row>
     <row r="506">
       <c r="A506" s="2" t="inlineStr">
         <is>
-          <t>VL20</t>
+          <t>TT126</t>
         </is>
       </c>
     </row>
     <row r="507">
       <c r="A507" s="2" t="inlineStr">
         <is>
-          <t>VL22</t>
+          <t>TT129</t>
         </is>
       </c>
     </row>
     <row r="508">
       <c r="A508" s="2" t="inlineStr">
         <is>
-          <t>VL27</t>
+          <t>TT130</t>
         </is>
       </c>
     </row>
     <row r="509">
       <c r="A509" s="2" t="inlineStr">
         <is>
-          <t>VL35</t>
+          <t>TT202</t>
         </is>
       </c>
     </row>
     <row r="510">
       <c r="A510" s="2" t="inlineStr">
         <is>
-          <t>VL36</t>
+          <t>TT206</t>
         </is>
       </c>
     </row>
     <row r="511">
       <c r="A511" s="2" t="inlineStr">
         <is>
-          <t>VL38</t>
+          <t>VL01</t>
         </is>
       </c>
     </row>
     <row r="512">
       <c r="A512" s="2" t="inlineStr">
         <is>
-          <t>VL43</t>
+          <t>VL03</t>
         </is>
       </c>
     </row>
     <row r="513">
       <c r="A513" s="2" t="inlineStr">
         <is>
-          <t>VL47</t>
+          <t>VL04</t>
         </is>
       </c>
     </row>
     <row r="514">
       <c r="A514" s="2" t="inlineStr">
         <is>
-          <t>VL49</t>
+          <t>VL11</t>
         </is>
       </c>
     </row>
     <row r="515">
       <c r="A515" s="2" t="inlineStr">
         <is>
-          <t>VL57</t>
+          <t>VL13</t>
         </is>
       </c>
     </row>
     <row r="516">
       <c r="A516" s="2" t="inlineStr">
         <is>
-          <t>VL62</t>
+          <t>VL20</t>
         </is>
       </c>
     </row>
     <row r="517">
       <c r="A517" s="2" t="inlineStr">
         <is>
-          <t>VL67</t>
+          <t>VL22</t>
         </is>
       </c>
     </row>
     <row r="518">
       <c r="A518" s="2" t="inlineStr">
         <is>
-          <t>VL75</t>
+          <t>VL27</t>
         </is>
       </c>
     </row>
     <row r="519">
       <c r="A519" s="2" t="inlineStr">
         <is>
-          <t>VL81</t>
+          <t>VL30</t>
         </is>
       </c>
     </row>
     <row r="520">
       <c r="A520" s="2" t="inlineStr">
         <is>
-          <t>VL86</t>
+          <t>VL35</t>
         </is>
       </c>
     </row>
     <row r="521">
       <c r="A521" s="2" t="inlineStr">
         <is>
-          <t>VL87</t>
+          <t>VL36</t>
         </is>
       </c>
     </row>
     <row r="522">
       <c r="A522" s="2" t="inlineStr">
         <is>
-          <t>VL88</t>
+          <t>VL38</t>
         </is>
       </c>
     </row>
     <row r="523">
       <c r="A523" s="2" t="inlineStr">
         <is>
-          <t>VL90</t>
+          <t>VL43</t>
         </is>
       </c>
     </row>
     <row r="524">
       <c r="A524" s="2" t="inlineStr">
         <is>
-          <t>VL92</t>
+          <t>VL47</t>
         </is>
       </c>
     </row>
     <row r="525">
       <c r="A525" s="2" t="inlineStr">
         <is>
-          <t>VL99</t>
+          <t>VL49</t>
         </is>
       </c>
     </row>
     <row r="526">
       <c r="A526" s="2" t="inlineStr">
         <is>
-          <t>VL100</t>
+          <t>VL57</t>
         </is>
       </c>
     </row>
     <row r="527">
       <c r="A527" s="2" t="inlineStr">
         <is>
-          <t>VL101</t>
+          <t>VL62</t>
         </is>
       </c>
     </row>
     <row r="528">
       <c r="A528" s="2" t="inlineStr">
         <is>
-          <t>VL103</t>
+          <t>VL67</t>
         </is>
       </c>
     </row>
     <row r="529">
       <c r="A529" s="2" t="inlineStr">
         <is>
-          <t>VL107</t>
+          <t>VL75</t>
         </is>
       </c>
     </row>
     <row r="530">
       <c r="A530" s="2" t="inlineStr">
         <is>
-          <t>VL112</t>
+          <t>VL81</t>
         </is>
       </c>
     </row>
     <row r="531">
       <c r="A531" s="2" t="inlineStr">
         <is>
-          <t>VL114</t>
+          <t>VL86</t>
         </is>
       </c>
     </row>
     <row r="532">
       <c r="A532" s="2" t="inlineStr">
         <is>
-          <t>VL115</t>
+          <t>VL87</t>
         </is>
       </c>
     </row>
     <row r="533">
       <c r="A533" s="2" t="inlineStr">
         <is>
-          <t>VL121</t>
+          <t>VL88</t>
         </is>
       </c>
     </row>
     <row r="534">
       <c r="A534" s="2" t="inlineStr">
         <is>
-          <t>VL122</t>
+          <t>VL90</t>
         </is>
       </c>
     </row>
     <row r="535">
       <c r="A535" s="2" t="inlineStr">
         <is>
-          <t>VL123</t>
+          <t>VL92</t>
         </is>
       </c>
     </row>
     <row r="536">
       <c r="A536" s="2" t="inlineStr">
         <is>
-          <t>VL124</t>
+          <t>VL99</t>
         </is>
       </c>
     </row>
     <row r="537">
       <c r="A537" s="2" t="inlineStr">
         <is>
-          <t>VL125</t>
+          <t>VL100</t>
         </is>
       </c>
     </row>
     <row r="538">
       <c r="A538" s="2" t="inlineStr">
         <is>
-          <t>VL126</t>
+          <t>VL101</t>
         </is>
       </c>
     </row>
     <row r="539">
       <c r="A539" s="2" t="inlineStr">
         <is>
-          <t>VL129</t>
+          <t>VL103</t>
         </is>
       </c>
     </row>
     <row r="540">
       <c r="A540" s="2" t="inlineStr">
         <is>
-          <t>VL132</t>
+          <t>VL107</t>
         </is>
       </c>
     </row>
     <row r="541">
       <c r="A541" s="2" t="inlineStr">
         <is>
-          <t>VL134</t>
+          <t>VL112</t>
         </is>
       </c>
     </row>
     <row r="542">
       <c r="A542" s="2" t="inlineStr">
         <is>
-          <t>VL137</t>
+          <t>VL114</t>
         </is>
       </c>
     </row>
     <row r="543">
       <c r="A543" s="2" t="inlineStr">
         <is>
-          <t>VL139</t>
+          <t>VL115</t>
         </is>
       </c>
     </row>
     <row r="544">
       <c r="A544" s="2" t="inlineStr">
         <is>
-          <t>VL140</t>
+          <t>VL121</t>
         </is>
       </c>
     </row>
     <row r="545">
       <c r="A545" s="2" t="inlineStr">
         <is>
-          <t>VL354</t>
+          <t>VL122</t>
         </is>
       </c>
     </row>
     <row r="546">
       <c r="A546" s="2" t="inlineStr">
         <is>
-          <t>VLINE8013</t>
+          <t>VL123</t>
         </is>
       </c>
     </row>
     <row r="547">
       <c r="A547" s="2" t="inlineStr">
         <is>
-          <t>VLINE8020</t>
+          <t>VL124</t>
         </is>
       </c>
     </row>
     <row r="548">
       <c r="A548" s="2" t="inlineStr">
         <is>
-          <t>VLINE8021</t>
+          <t>VL125</t>
         </is>
       </c>
     </row>
     <row r="549">
       <c r="A549" s="2" t="inlineStr">
         <is>
-          <t>VLINE8028</t>
+          <t>VL126</t>
         </is>
       </c>
     </row>
     <row r="550">
       <c r="A550" s="2" t="inlineStr">
         <is>
-          <t>VLINE8030</t>
+          <t>VL127</t>
         </is>
       </c>
     </row>
     <row r="551">
       <c r="A551" s="2" t="inlineStr">
         <is>
-          <t>VLINE8058</t>
+          <t>VL129</t>
         </is>
       </c>
     </row>
     <row r="552">
       <c r="A552" s="2" t="inlineStr">
         <is>
-          <t>VLINE8059</t>
+          <t>VL132</t>
         </is>
       </c>
     </row>
     <row r="553">
       <c r="A553" s="2" t="inlineStr">
         <is>
-          <t>VLINE8061</t>
+          <t>VL134</t>
         </is>
       </c>
     </row>
     <row r="554">
       <c r="A554" s="2" t="inlineStr">
         <is>
-          <t>VLINE8071</t>
+          <t>VL137</t>
         </is>
       </c>
     </row>
     <row r="555">
       <c r="A555" s="2" t="inlineStr">
         <is>
-          <t>VLINE8072</t>
+          <t>VL139</t>
         </is>
       </c>
     </row>
     <row r="556">
       <c r="A556" s="2" t="inlineStr">
         <is>
-          <t>VLINE8074</t>
+          <t>VL140</t>
         </is>
       </c>
     </row>
     <row r="557">
       <c r="A557" s="2" t="inlineStr">
         <is>
-          <t>VLINE8075</t>
+          <t>VL354</t>
         </is>
       </c>
     </row>
     <row r="558">
       <c r="A558" s="2" t="inlineStr">
         <is>
-          <t>VLINE8080</t>
+          <t>VLINE8013</t>
         </is>
       </c>
     </row>
     <row r="559">
       <c r="A559" s="2" t="inlineStr">
         <is>
-          <t>VLINE8081</t>
+          <t>VLINE8020</t>
         </is>
       </c>
     </row>
     <row r="560">
       <c r="A560" s="2" t="inlineStr">
         <is>
-          <t>VLINE8102</t>
+          <t>VLINE8021</t>
         </is>
       </c>
     </row>
     <row r="561">
       <c r="A561" s="2" t="inlineStr">
         <is>
-          <t>VLINE8111</t>
+          <t>VLINE8023</t>
         </is>
       </c>
     </row>
     <row r="562">
       <c r="A562" s="2" t="inlineStr">
         <is>
-          <t>VLINE8113</t>
+          <t>VLINE8028</t>
         </is>
       </c>
     </row>
     <row r="563">
       <c r="A563" s="2" t="inlineStr">
         <is>
-          <t>VLINE8115</t>
+          <t>VLINE8030</t>
         </is>
       </c>
     </row>
     <row r="564">
       <c r="A564" s="2" t="inlineStr">
         <is>
-          <t>VLINE8117</t>
+          <t>VLINE8058</t>
         </is>
       </c>
     </row>
     <row r="565">
       <c r="A565" s="2" t="inlineStr">
         <is>
-          <t>VLINE8120</t>
+          <t>VLINE8059</t>
         </is>
       </c>
     </row>
     <row r="566">
       <c r="A566" s="2" t="inlineStr">
         <is>
-          <t>VLINE8121</t>
+          <t>VLINE8061</t>
         </is>
       </c>
     </row>
     <row r="567">
       <c r="A567" s="2" t="inlineStr">
         <is>
-          <t>VLINE8122</t>
+          <t>VLINE8071</t>
         </is>
       </c>
     </row>
     <row r="568">
       <c r="A568" s="2" t="inlineStr">
         <is>
-          <t>VLINE8123</t>
+          <t>VLINE8072</t>
         </is>
       </c>
     </row>
     <row r="569">
       <c r="A569" s="2" t="inlineStr">
         <is>
-          <t>VLINE8124</t>
+          <t>VLINE8074</t>
         </is>
       </c>
     </row>
     <row r="570">
       <c r="A570" s="2" t="inlineStr">
         <is>
-          <t>VLINE8126</t>
+          <t>VLINE8075</t>
         </is>
       </c>
     </row>
     <row r="571">
       <c r="A571" s="2" t="inlineStr">
         <is>
-          <t>VLINE8128</t>
+          <t>VLINE8080</t>
         </is>
       </c>
     </row>
     <row r="572">
       <c r="A572" s="2" t="inlineStr">
         <is>
-          <t>VLINE8130</t>
+          <t>VLINE8081</t>
         </is>
       </c>
     </row>
     <row r="573">
       <c r="A573" s="2" t="inlineStr">
         <is>
-          <t>VLINE8161</t>
+          <t>VLINE8102</t>
         </is>
       </c>
     </row>
     <row r="574">
       <c r="A574" s="2" t="inlineStr">
         <is>
-          <t>VLINE8163</t>
+          <t>VLINE8111</t>
         </is>
       </c>
     </row>
     <row r="575">
       <c r="A575" s="2" t="inlineStr">
         <is>
-          <t>VLINE8164</t>
+          <t>VLINE8113</t>
         </is>
       </c>
     </row>
     <row r="576">
       <c r="A576" s="2" t="inlineStr">
         <is>
-          <t>VLINE8172</t>
+          <t>VLINE8115</t>
         </is>
       </c>
     </row>
     <row r="577">
       <c r="A577" s="2" t="inlineStr">
         <is>
-          <t>VLINE8181</t>
+          <t>VLINE8117</t>
         </is>
       </c>
     </row>
     <row r="578">
       <c r="A578" s="2" t="inlineStr">
         <is>
-          <t>VLINE8183</t>
+          <t>VLINE8120</t>
         </is>
       </c>
     </row>
     <row r="579">
       <c r="A579" s="2" t="inlineStr">
         <is>
-          <t>VLINE8184</t>
+          <t>VLINE8121</t>
         </is>
       </c>
     </row>
     <row r="580">
       <c r="A580" s="2" t="inlineStr">
         <is>
-          <t>VLINE8211</t>
+          <t>VLINE8122</t>
         </is>
       </c>
     </row>
     <row r="581">
       <c r="A581" s="2" t="inlineStr">
         <is>
-          <t>VLINE8213</t>
+          <t>VLINE8123</t>
         </is>
       </c>
     </row>
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>VLINE8215</t>
+          <t>VLINE8124</t>
         </is>
       </c>
     </row>
     <row r="583">
       <c r="A583" s="2" t="inlineStr">
         <is>
-          <t>VLINE8217</t>
+          <t>VLINE8126</t>
         </is>
       </c>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>VLINE8219</t>
+          <t>VLINE8128</t>
         </is>
       </c>
     </row>
     <row r="585">
       <c r="A585" s="2" t="inlineStr">
         <is>
-          <t>VLINE8221</t>
+          <t>VLINE8130</t>
         </is>
       </c>
     </row>
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>VLINE8226</t>
+          <t>VLINE8161</t>
         </is>
       </c>
     </row>
     <row r="587">
       <c r="A587" s="2" t="inlineStr">
         <is>
-          <t>VLINE8228</t>
+          <t>VLINE8163</t>
         </is>
       </c>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>VLINE8230</t>
+          <t>VLINE8164</t>
         </is>
       </c>
     </row>
     <row r="589">
       <c r="A589" s="2" t="inlineStr">
         <is>
-          <t>VLINE8232</t>
+          <t>VLINE8172</t>
         </is>
       </c>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>VLINE8234</t>
+          <t>VLINE8181</t>
         </is>
       </c>
     </row>
     <row r="591">
       <c r="A591" s="2" t="inlineStr">
         <is>
-          <t>VLINE8236</t>
+          <t>VLINE8183</t>
         </is>
       </c>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>VLINE8400</t>
+          <t>VLINE8184</t>
         </is>
       </c>
     </row>
     <row r="593">
       <c r="A593" s="2" t="inlineStr">
         <is>
-          <t>VLINE8405</t>
+          <t>VLINE8211</t>
         </is>
       </c>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>VLINE8408</t>
+          <t>VLINE8213</t>
         </is>
       </c>
     </row>
     <row r="595">
       <c r="A595" s="2" t="inlineStr">
         <is>
-          <t>VLINE8413</t>
+          <t>VLINE8215</t>
         </is>
       </c>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>VLINE8415</t>
+          <t>VLINE8217</t>
         </is>
       </c>
     </row>
     <row r="597">
       <c r="A597" s="2" t="inlineStr">
         <is>
-          <t>VLINE8417</t>
+          <t>VLINE8219</t>
         </is>
       </c>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>VLINE8418</t>
+          <t>VLINE8221</t>
         </is>
       </c>
     </row>
     <row r="599">
       <c r="A599" s="2" t="inlineStr">
         <is>
-          <t>VLINE8419</t>
+          <t>VLINE8223</t>
         </is>
       </c>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>VLINE8420</t>
+          <t>VLINE8226</t>
         </is>
       </c>
     </row>
     <row r="601">
       <c r="A601" s="2" t="inlineStr">
         <is>
-          <t>VLINE8421</t>
+          <t>VLINE8228</t>
         </is>
       </c>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>VLINE8422</t>
+          <t>VLINE8230</t>
         </is>
       </c>
     </row>
     <row r="603">
       <c r="A603" s="2" t="inlineStr">
         <is>
-          <t>VLINE8423</t>
+          <t>VLINE8232</t>
         </is>
       </c>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>VLINE8424</t>
+          <t>VLINE8234</t>
         </is>
       </c>
     </row>
     <row r="605">
       <c r="A605" s="2" t="inlineStr">
         <is>
-          <t>VLINE8428</t>
+          <t>VLINE8236</t>
         </is>
       </c>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>VLINE8430</t>
+          <t>VLINE8400</t>
         </is>
       </c>
     </row>
     <row r="607">
       <c r="A607" s="2" t="inlineStr">
         <is>
-          <t>VLINE8457</t>
+          <t>VLINE8405</t>
         </is>
       </c>
     </row>
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>VLINE8459</t>
+          <t>VLINE8408</t>
         </is>
       </c>
     </row>
     <row r="609">
       <c r="A609" s="2" t="inlineStr">
         <is>
-          <t>VLINE8460</t>
+          <t>VLINE8413</t>
         </is>
       </c>
     </row>
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>VLINE8461</t>
+          <t>VLINE8415</t>
         </is>
       </c>
     </row>
     <row r="611">
       <c r="A611" s="2" t="inlineStr">
         <is>
-          <t>VLINE8702</t>
+          <t>VLINE8417</t>
         </is>
       </c>
     </row>
     <row r="612">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>VLINE8725</t>
+          <t>VLINE8418</t>
         </is>
       </c>
     </row>
     <row r="613">
       <c r="A613" s="2" t="inlineStr">
         <is>
-          <t>VLINE8727</t>
+          <t>VLINE8419</t>
         </is>
       </c>
     </row>
     <row r="614">
       <c r="A614" s="2" t="inlineStr">
         <is>
-          <t>VLINE8729</t>
+          <t>VLINE8420</t>
         </is>
       </c>
     </row>
     <row r="615">
       <c r="A615" s="2" t="inlineStr">
         <is>
-          <t>VLINE8731</t>
+          <t>VLINE8421</t>
         </is>
       </c>
     </row>
     <row r="616">
       <c r="A616" s="2" t="inlineStr">
         <is>
-          <t>VLINE8733</t>
+          <t>VLINE8422</t>
         </is>
       </c>
     </row>
     <row r="617">
       <c r="A617" s="2" t="inlineStr">
         <is>
-          <t>VLINE8735</t>
+          <t>VLINE8423</t>
         </is>
       </c>
     </row>
     <row r="618">
       <c r="A618" s="2" t="inlineStr">
         <is>
-          <t>VLINE8737</t>
+          <t>VLINE8424</t>
         </is>
       </c>
     </row>
     <row r="619">
       <c r="A619" s="2" t="inlineStr">
         <is>
-          <t>VLINE8739</t>
+          <t>VLINE8428</t>
         </is>
       </c>
     </row>
     <row r="620">
       <c r="A620" s="2" t="inlineStr">
         <is>
-          <t>VLINE8741</t>
+          <t>VLINE8430</t>
         </is>
       </c>
     </row>
     <row r="621">
       <c r="A621" s="2" t="inlineStr">
         <is>
-          <t>VLINE8742</t>
+          <t>VLINE8457</t>
         </is>
       </c>
     </row>
     <row r="622">
       <c r="A622" s="2" t="inlineStr">
         <is>
-          <t>VLINE8743</t>
+          <t>VLINE8459</t>
         </is>
       </c>
     </row>
     <row r="623">
       <c r="A623" s="2" t="inlineStr">
         <is>
-          <t>VLINE8744</t>
+          <t>VLINE8460</t>
         </is>
       </c>
     </row>
     <row r="624">
       <c r="A624" s="2" t="inlineStr">
         <is>
-          <t>VLINE8745</t>
+          <t>VLINE8461</t>
         </is>
       </c>
     </row>
     <row r="625">
       <c r="A625" s="2" t="inlineStr">
         <is>
-          <t>VLINE8746</t>
+          <t>VLINE8465</t>
         </is>
       </c>
     </row>
     <row r="626">
       <c r="A626" s="2" t="inlineStr">
         <is>
-          <t>VLINE8747</t>
+          <t>VLINE8702</t>
         </is>
       </c>
     </row>
     <row r="627">
       <c r="A627" s="2" t="inlineStr">
         <is>
-          <t>VLINE8748</t>
+          <t>VLINE8725</t>
         </is>
       </c>
     </row>
     <row r="628">
       <c r="A628" s="2" t="inlineStr">
         <is>
-          <t>VLINE8750</t>
+          <t>VLINE8727</t>
         </is>
       </c>
     </row>
     <row r="629">
       <c r="A629" s="2" t="inlineStr">
         <is>
-          <t>VLINE8752</t>
+          <t>VLINE8729</t>
         </is>
       </c>
     </row>
     <row r="630">
       <c r="A630" s="2" t="inlineStr">
         <is>
-          <t>VLINE8754</t>
+          <t>VLINE8731</t>
         </is>
       </c>
     </row>
     <row r="631">
       <c r="A631" s="2" t="inlineStr">
         <is>
-          <t>VLINE8756</t>
+          <t>VLINE8733</t>
         </is>
       </c>
     </row>
     <row r="632">
       <c r="A632" s="2" t="inlineStr">
         <is>
-          <t>VLINE8758</t>
+          <t>VLINE8735</t>
         </is>
       </c>
     </row>
     <row r="633">
       <c r="A633" s="2" t="inlineStr">
         <is>
-          <t>VLINE8760</t>
+          <t>VLINE8737</t>
         </is>
       </c>
     </row>
     <row r="634">
       <c r="A634" s="2" t="inlineStr">
         <is>
-          <t>VLINE8762</t>
+          <t>VLINE8739</t>
         </is>
       </c>
     </row>
     <row r="635">
       <c r="A635" s="2" t="inlineStr">
         <is>
-          <t>VLINE8764</t>
+          <t>VLINE8741</t>
         </is>
       </c>
     </row>
     <row r="636">
       <c r="A636" s="2" t="inlineStr">
         <is>
-          <t>VLINE8819</t>
+          <t>VLINE8742</t>
         </is>
       </c>
     </row>
     <row r="637">
       <c r="A637" s="2" t="inlineStr">
         <is>
-          <t>VLINE8862</t>
+          <t>VLINE8743</t>
         </is>
       </c>
     </row>
     <row r="638">
       <c r="A638" s="2" t="inlineStr">
         <is>
-          <t>VLINE8863</t>
+          <t>VLINE8744</t>
         </is>
       </c>
     </row>
     <row r="639">
       <c r="A639" s="2" t="inlineStr">
         <is>
-          <t>VR77</t>
+          <t>VLINE8745</t>
         </is>
       </c>
     </row>
     <row r="640">
       <c r="A640" s="2" t="inlineStr">
         <is>
-          <t>WOLL408</t>
+          <t>VLINE8746</t>
         </is>
       </c>
     </row>
     <row r="641">
       <c r="A641" s="2" t="inlineStr">
         <is>
-          <t>WOLL430</t>
+          <t>VLINE8747</t>
         </is>
       </c>
     </row>
     <row r="642">
       <c r="A642" s="2" t="inlineStr">
         <is>
-          <t>XP2001</t>
+          <t>VLINE8748</t>
         </is>
       </c>
     </row>
     <row r="643">
       <c r="A643" s="2" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>VLINE8749</t>
         </is>
       </c>
     </row>
     <row r="644">
       <c r="A644" s="2" t="inlineStr">
         <is>
-          <t>XP2006</t>
+          <t>VLINE8750</t>
         </is>
       </c>
     </row>
     <row r="645">
       <c r="A645" s="2" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>VLINE8751</t>
         </is>
       </c>
     </row>
     <row r="646">
       <c r="A646" s="2" t="inlineStr">
         <is>
-          <t>XP2009</t>
+          <t>VLINE8752</t>
         </is>
       </c>
     </row>
     <row r="647">
       <c r="A647" s="2" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>VLINE8754</t>
         </is>
       </c>
     </row>
     <row r="648">
       <c r="A648" s="2" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>VLINE8756</t>
         </is>
       </c>
     </row>
     <row r="649">
       <c r="A649" s="2" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>VLINE8758</t>
         </is>
       </c>
     </row>
     <row r="650">
       <c r="A650" s="2" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>VLINE8760</t>
         </is>
       </c>
     </row>
     <row r="651">
       <c r="A651" s="2" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>VLINE8762</t>
         </is>
       </c>
     </row>
     <row r="652">
       <c r="A652" s="2" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>VLINE8764</t>
         </is>
       </c>
     </row>
     <row r="653">
       <c r="A653" s="2" t="inlineStr">
         <is>
-          <t>XRN003</t>
+          <t>VLINE8819</t>
         </is>
       </c>
     </row>
     <row r="654">
       <c r="A654" s="2" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>VLINE8862</t>
         </is>
       </c>
     </row>
     <row r="655">
       <c r="A655" s="2" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>VLINE8863</t>
         </is>
       </c>
     </row>
     <row r="656">
       <c r="A656" s="2" t="inlineStr">
         <is>
-          <t>XRN010</t>
+          <t>VR77</t>
         </is>
       </c>
     </row>
     <row r="657">
       <c r="A657" s="2" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>WOLL408</t>
         </is>
       </c>
     </row>
     <row r="658">
       <c r="A658" s="2" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>WOLL430</t>
         </is>
       </c>
     </row>
     <row r="659">
       <c r="A659" s="2" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>XP2001</t>
         </is>
       </c>
     </row>
     <row r="660">
       <c r="A660" s="2" t="inlineStr">
         <is>
-          <t>XRN022</t>
+          <t>XP2005</t>
         </is>
       </c>
     </row>
     <row r="661">
       <c r="A661" s="2" t="inlineStr">
         <is>
-          <t>XRN028</t>
+          <t>XP2006</t>
         </is>
       </c>
     </row>
     <row r="662">
       <c r="A662" s="2" t="inlineStr">
+        <is>
+          <t>XP2008</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="2" t="inlineStr">
+        <is>
+          <t>XP2009</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" s="2" t="inlineStr">
+        <is>
+          <t>XP2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="2" t="inlineStr">
+        <is>
+          <t>XP2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" s="2" t="inlineStr">
+        <is>
+          <t>XP2013</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" s="2" t="inlineStr">
+        <is>
+          <t>XP2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" s="2" t="inlineStr">
+        <is>
+          <t>XP2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" s="2" t="inlineStr">
+        <is>
+          <t>XP2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" s="2" t="inlineStr">
+        <is>
+          <t>XRN003</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="2" t="inlineStr">
+        <is>
+          <t>XRN005</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="2" t="inlineStr">
+        <is>
+          <t>XRN009</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" s="2" t="inlineStr">
+        <is>
+          <t>XRN010</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" s="2" t="inlineStr">
+        <is>
+          <t>XRN017</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="2" t="inlineStr">
+        <is>
+          <t>XRN018</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="2" t="inlineStr">
+        <is>
+          <t>XRN021</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" s="2" t="inlineStr">
+        <is>
+          <t>XRN022</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="2" t="inlineStr">
+        <is>
+          <t>XRN028</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="2" t="inlineStr">
         <is>
           <t>XRN029</t>
         </is>

</xml_diff>

<commit_message>
Update RailOps database files - 2026-04-30 03:31:43 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A679"/>
+  <dimension ref="A1:A692"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1476,3729 +1476,3820 @@
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>EA2506</t>
+          <t>EA2505</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>EA2507</t>
+          <t>EA2506</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>EC2521</t>
+          <t>EA2507</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>EC2525</t>
+          <t>EC2521</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>EC2526</t>
+          <t>EC2525</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>FIE001</t>
+          <t>EC2526</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>FIE003</t>
+          <t>FIE001</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>G513</t>
+          <t>FIE003</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>G514</t>
+          <t>G513</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>G516</t>
+          <t>G514</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>G521</t>
+          <t>G516</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>G532</t>
+          <t>G521</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>G533</t>
+          <t>G532</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>G534</t>
+          <t>G533</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>G536</t>
+          <t>G534</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>GL103</t>
+          <t>G536</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>GL105</t>
+          <t>GL103</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>GL108</t>
+          <t>GL105</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>GL111</t>
+          <t>GL108</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>GM37</t>
+          <t>GL111</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>GM46</t>
+          <t>GM37</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>GWA002</t>
+          <t>GM46</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>GWA004</t>
+          <t>GWA002</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>GWA008</t>
+          <t>GWA004</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>GWA009</t>
+          <t>GWA008</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>GWB102</t>
+          <t>GWA009</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>GWB103</t>
+          <t>GWB102</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>GWB104</t>
+          <t>GWB103</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>GWU008</t>
+          <t>GWB104</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>GWU012</t>
+          <t>GWU008</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>GWU013</t>
+          <t>GWU012</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>GWU014</t>
+          <t>GWU013</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>GWU015</t>
+          <t>GWU014</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>HM2701</t>
+          <t>GWU015</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>HM2702</t>
+          <t>HM2701</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>HM2703</t>
+          <t>HM2702</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>HM2705</t>
+          <t>HM2703</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>HM2706</t>
+          <t>HM2705</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>HM2707</t>
+          <t>HM2706</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>HM2751</t>
+          <t>HM2707</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>HM2752</t>
+          <t>HM2751</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>HM2753</t>
+          <t>HM2752</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>HM2755</t>
+          <t>HM2753</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>HM2756</t>
+          <t>HM2755</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>HM2757</t>
+          <t>HM2756</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>JP9750</t>
+          <t>HM2757</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>LDP002</t>
+          <t>JP9750</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>LDP004</t>
+          <t>K183</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>LDP008</t>
+          <t>L277</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>LE2851</t>
+          <t>LDP002</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>LE2853</t>
+          <t>LDP004</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>LE2854</t>
+          <t>LDP008</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>LE2855</t>
+          <t>LE2851</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>LE2857</t>
+          <t>LE2853</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>LE2858</t>
+          <t>LE2854</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>LE2859</t>
+          <t>LE2855</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>LE2862</t>
+          <t>LE2857</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>LE2863</t>
+          <t>LE2858</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>LE2864</t>
+          <t>LE2859</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>LZ3114</t>
+          <t>LE2862</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>M437</t>
+          <t>LE2863</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>M865</t>
+          <t>LE2864</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>MAN004</t>
+          <t>LZ3114</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>MAN005</t>
+          <t>M437</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>MAN007</t>
+          <t>M865</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>MAN011</t>
+          <t>MAN004</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>MAN013</t>
+          <t>MAN005</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>MAN015</t>
+          <t>MAN007</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>MAN016</t>
+          <t>MAN011</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>MAN017</t>
+          <t>MAN013</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>MM02</t>
+          <t>MAN015</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>MM2M</t>
+          <t>MAN016</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>MM4M</t>
+          <t>MAN017</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>MM8M</t>
+          <t>MM02</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>MM14M</t>
+          <t>MM2M</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>MM32M</t>
+          <t>MM4M</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>MM38M</t>
+          <t>MM8M</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>MM40M</t>
+          <t>MM14M</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>MM42M</t>
+          <t>MM32M</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>MM44M</t>
+          <t>MM38M</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>MM48M</t>
+          <t>MM40M</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>MM50M</t>
+          <t>MM42M</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>MM52M</t>
+          <t>MM44M</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>MM64M</t>
+          <t>MM48M</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>MM76M</t>
+          <t>MM50M</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>MM78M</t>
+          <t>MM52M</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>MM80M</t>
+          <t>MM64M</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>MM82M</t>
+          <t>MM76M</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>MM84M</t>
+          <t>MM78M</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>MM86M</t>
+          <t>MM80M</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>MM92M</t>
+          <t>MM82M</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>MM94M</t>
+          <t>MM84M</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>MM96M</t>
+          <t>MM86M</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>MM98M</t>
+          <t>MM92M</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>MM99M</t>
+          <t>MM94M</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>MM122M</t>
+          <t>MM96M</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>MM130M</t>
+          <t>MM98M</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>MM152M</t>
+          <t>MM99M</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>MM156M</t>
+          <t>MM122M</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>MM158M</t>
+          <t>MM130M</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>MM172M</t>
+          <t>MM152M</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>MM178M</t>
+          <t>MM156M</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>MM192M</t>
+          <t>MM158M</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>MM212M</t>
+          <t>MM172M</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>MM214M</t>
+          <t>MM178M</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>MM216M</t>
+          <t>MM192M</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>MM232M</t>
+          <t>MM212M</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>MM236M</t>
+          <t>MM214M</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>MM240M</t>
+          <t>MM216M</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>MM246M</t>
+          <t>MM232M</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>MM260M</t>
+          <t>MM236M</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>MM264M</t>
+          <t>MM240M</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>MM266M</t>
+          <t>MM246M</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>MM268M</t>
+          <t>MM260M</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>MM270M</t>
+          <t>MM264M</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>MM280M</t>
+          <t>MM266M</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>MM288M</t>
+          <t>MM268M</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>MM380M</t>
+          <t>MM270M</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>MM456M</t>
+          <t>MM280M</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>MM464M</t>
+          <t>MM288M</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>MM478M</t>
+          <t>MM380M</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>MM482M</t>
+          <t>MM456M</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>MM486M</t>
+          <t>MM464M</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>MM502M</t>
+          <t>MM478M</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>MM506M</t>
+          <t>MM482M</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>MM514M</t>
+          <t>MM486M</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>MM522M</t>
+          <t>MM502M</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>MM536M</t>
+          <t>MM506M</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>MM542M</t>
+          <t>MM514M</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>MM544M</t>
+          <t>MM522M</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>MM546M</t>
+          <t>MM536M</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>MM551M</t>
+          <t>MM542M</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>MM574M</t>
+          <t>MM544M</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>MM588M</t>
+          <t>MM546M</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>MM592M</t>
+          <t>MM551M</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>MM604M</t>
+          <t>MM574M</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>MM624M</t>
+          <t>MM588M</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>MM636M</t>
+          <t>MM592M</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>MM638M</t>
+          <t>MM604M</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>MM647M</t>
+          <t>MM624M</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>MM656M</t>
+          <t>MM636M</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>MM658M</t>
+          <t>MM638M</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>MM660M</t>
+          <t>MM647M</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>MM664M</t>
+          <t>MM656M</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>MM668M</t>
+          <t>MM658M</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>MM673M</t>
+          <t>MM660M</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>MM674M</t>
+          <t>MM664M</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>MM676M</t>
+          <t>MM668M</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>MM680M</t>
+          <t>MM673M</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>MM702M</t>
+          <t>MM674M</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>MM718M</t>
+          <t>MM676M</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>MM742M</t>
+          <t>MM680M</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>MM744M</t>
+          <t>MM702M</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>MM752M</t>
+          <t>MM718M</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>MM768M</t>
+          <t>MM742M</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>MM772M</t>
+          <t>MM744M</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>MM774M</t>
+          <t>MM752M</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>MM776M</t>
+          <t>MM768M</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>MM778M</t>
+          <t>MM772M</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>MM784M</t>
+          <t>MM774M</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>MM788M</t>
+          <t>MM776M</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>MM794M</t>
+          <t>MM778M</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>MM798M</t>
+          <t>MM784M</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>MM800M</t>
+          <t>MM788M</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>MM802M</t>
+          <t>MM794M</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>MM806M</t>
+          <t>MM798M</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>MM808M</t>
+          <t>MM800M</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>MM810M</t>
+          <t>MM802M</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>MM816M</t>
+          <t>MM806M</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>MM826M</t>
+          <t>MM808M</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>MM830M</t>
+          <t>MM810M</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>MM832M</t>
+          <t>MM816M</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>MM834M</t>
+          <t>MM826M</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>MM838M</t>
+          <t>MM830M</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>MM842M</t>
+          <t>MM832M</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>MM858M</t>
+          <t>MM834M</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>MM860M</t>
+          <t>MM838M</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>MM862M</t>
+          <t>MM842M</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>MM864M</t>
+          <t>MM858M</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>MM866M</t>
+          <t>MM860M</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>MM872M</t>
+          <t>MM862M</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>MM878M</t>
+          <t>MM864M</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>MM880M</t>
+          <t>MM866M</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>MM886M</t>
+          <t>MM872M</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>MM896M</t>
+          <t>MM878M</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>MM908M</t>
+          <t>MM880M</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>MM910M</t>
+          <t>MM886M</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>MM912M</t>
+          <t>MM896M</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>MM914M</t>
+          <t>MM908M</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>MM924M</t>
+          <t>MM910M</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>MM928M</t>
+          <t>MM912M</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>MM934M</t>
+          <t>MM914M</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>MM940M</t>
+          <t>MM924M</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>MM944M</t>
+          <t>MM928M</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>MM946M</t>
+          <t>MM934M</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>MM952M</t>
+          <t>MM940M</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>MM956M</t>
+          <t>MM944M</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>MM958M</t>
+          <t>MM946M</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>MM960M</t>
+          <t>MM952M</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>MM962M</t>
+          <t>MM956M</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>MM964M</t>
+          <t>MM958M</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>MM968M</t>
+          <t>MM960M</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>MM972M</t>
+          <t>MM962M</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>MM974M</t>
+          <t>MM964M</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>MM976M</t>
+          <t>MM968M</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>MM980M</t>
+          <t>MM972M</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>MM982M</t>
+          <t>MM974M</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>MM9901M</t>
+          <t>MM976M</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>MM9903M</t>
+          <t>MM980M</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>MM9904M</t>
+          <t>MM982M</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>MM9906M</t>
+          <t>MM9901M</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>MM9908M</t>
+          <t>MM9903M</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>MM9909M</t>
+          <t>MM9904M</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>MM9910M</t>
+          <t>MM9906M</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>MM9912M</t>
+          <t>MM9908M</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>MM9914M</t>
+          <t>MM9909M</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>MM9916M</t>
+          <t>MM9910M</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>MM9918M</t>
+          <t>MM9912M</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>MM9920M</t>
+          <t>MM9914M</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>MM9921M</t>
+          <t>MM9916M</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>MM9924M</t>
+          <t>MM9918M</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>MM9926M</t>
+          <t>MM9920M</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>MM9927M</t>
+          <t>MM9921M</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>MM9928M</t>
+          <t>MM9924M</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>MM9929M</t>
+          <t>MM9926M</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>MM9931M</t>
+          <t>MM9927M</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t>MM9936M</t>
+          <t>MM9928M</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>MM9937M</t>
+          <t>MM9929M</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t>MM9938M</t>
+          <t>MM9931M</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>MM9941M</t>
+          <t>MM9936M</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>MM9943M</t>
+          <t>MM9937M</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>MM9946M</t>
+          <t>MM9938M</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>MM9947M</t>
+          <t>MM9941M</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>MM9948M</t>
+          <t>MM9943M</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>MM9952M</t>
+          <t>MM9946M</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>MM9953M</t>
+          <t>MM9947M</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
         <is>
-          <t>MM9954M</t>
+          <t>MM9948M</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>MM9956M</t>
+          <t>MM9952M</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
         <is>
-          <t>MM9957M</t>
+          <t>MM9953M</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
         <is>
-          <t>MM9958M</t>
+          <t>MM9954M</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" s="2" t="inlineStr">
         <is>
-          <t>MM9959M</t>
+          <t>MM9956M</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
         <is>
-          <t>MM9960M</t>
+          <t>MM9957M</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
         <is>
-          <t>MM9961M</t>
+          <t>MM9958M</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>MM9962M</t>
+          <t>MM9959M</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
         <is>
-          <t>MM9963M</t>
+          <t>MM9960M</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
         <is>
-          <t>MM9964M</t>
+          <t>MM9961M</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="2" t="inlineStr">
         <is>
-          <t>MM9965M</t>
+          <t>MM9962M</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
         <is>
-          <t>MM9966M</t>
+          <t>MM9963M</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" s="2" t="inlineStr">
         <is>
-          <t>MM9968M</t>
+          <t>MM9964M</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
         <is>
-          <t>MM9969M</t>
+          <t>MM9965M</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="2" t="inlineStr">
         <is>
-          <t>MM9970M</t>
+          <t>MM9966M</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" s="2" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MM9968M</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="2" t="inlineStr">
         <is>
-          <t>MRL002</t>
+          <t>MM9969M</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
         <is>
-          <t>MTPV1</t>
+          <t>MM9970M</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" s="2" t="inlineStr">
         <is>
-          <t>MTPV2</t>
+          <t>MRL001</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
         <is>
-          <t>N453</t>
+          <t>MRL002</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" s="2" t="inlineStr">
         <is>
-          <t>N458</t>
+          <t>MTPV1</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" s="2" t="inlineStr">
         <is>
-          <t>N460</t>
+          <t>MTPV2</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>N453</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="2" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>N458</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>N460</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="2" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>N466</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="2" t="inlineStr">
         <is>
-          <t>NR6</t>
+          <t>N469</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" s="2" t="inlineStr">
         <is>
-          <t>NR10</t>
+          <t>NR4</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" s="2" t="inlineStr">
         <is>
-          <t>NR11</t>
+          <t>NR5</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" s="2" t="inlineStr">
         <is>
-          <t>NR12</t>
+          <t>NR6</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" s="2" t="inlineStr">
         <is>
-          <t>NR13</t>
+          <t>NR10</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" s="2" t="inlineStr">
         <is>
-          <t>NR14</t>
+          <t>NR11</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" s="2" t="inlineStr">
         <is>
-          <t>NR17</t>
+          <t>NR12</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" s="2" t="inlineStr">
         <is>
-          <t>NR20</t>
+          <t>NR13</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" s="2" t="inlineStr">
         <is>
-          <t>NR31</t>
+          <t>NR14</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t>NR35</t>
+          <t>NR17</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" s="2" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>NR20</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
         <is>
-          <t>NR44</t>
+          <t>NR31</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" s="2" t="inlineStr">
         <is>
-          <t>NR46</t>
+          <t>NR35</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" s="2" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>NR37</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" s="2" t="inlineStr">
         <is>
-          <t>NR52</t>
+          <t>NR44</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>NR46</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="2" t="inlineStr">
         <is>
-          <t>NR56</t>
+          <t>NR47</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR52</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR54</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR56</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" s="2" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR60</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
         <is>
-          <t>NR76</t>
+          <t>NR64</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" s="2" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR65</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR68</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" s="2" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR75</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t>NR88</t>
+          <t>NR76</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t>NR91</t>
+          <t>NR78</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR82</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR83</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR88</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>NR91</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR93</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
         <is>
-          <t>NR107</t>
+          <t>NR94</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR95</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR97</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR102</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR106</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>NR107</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>NR109</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>PKLA4</t>
+          <t>NR112</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>NR113</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>NR115</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>PB4</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="2" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>PKLA4</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" s="2" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" s="2" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="2" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" s="2" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" s="2" t="inlineStr">
         <is>
-          <t>QL009</t>
+          <t>QE001</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" s="2" t="inlineStr">
         <is>
-          <t>QL016</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" s="2" t="inlineStr">
         <is>
-          <t>QL019</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="2" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QL004</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="2" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="2" t="inlineStr">
         <is>
-          <t>QR5400</t>
+          <t>QL009</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="2" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QL016</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="2" t="inlineStr">
         <is>
-          <t>RA2302</t>
+          <t>QL019</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" s="2" t="inlineStr">
         <is>
-          <t>RA2303</t>
+          <t>QR1744</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" s="2" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>QR1771</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" s="2" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>QR5400</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" s="2" t="inlineStr">
         <is>
-          <t>RL309</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="A472" s="2" t="inlineStr">
         <is>
-          <t>RM93</t>
+          <t>RA2302</t>
         </is>
       </c>
     </row>
     <row r="473">
       <c r="A473" s="2" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>RA2303</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="A474" s="2" t="inlineStr">
         <is>
-          <t>SCT008</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
     <row r="475">
       <c r="A475" s="2" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>RL301</t>
         </is>
       </c>
     </row>
     <row r="476">
       <c r="A476" s="2" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>RL309</t>
         </is>
       </c>
     </row>
     <row r="477">
       <c r="A477" s="2" t="inlineStr">
         <is>
-          <t>SM636B</t>
+          <t>RM93</t>
         </is>
       </c>
     </row>
     <row r="478">
       <c r="A478" s="2" t="inlineStr">
         <is>
-          <t>SO3</t>
+          <t>SCT001</t>
         </is>
       </c>
     </row>
     <row r="479">
       <c r="A479" s="2" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>SCT008</t>
         </is>
       </c>
     </row>
     <row r="480">
       <c r="A480" s="2" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>SCT009</t>
         </is>
       </c>
     </row>
     <row r="481">
       <c r="A481" s="2" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>SCT013</t>
         </is>
       </c>
     </row>
     <row r="482">
       <c r="A482" s="2" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>SM636B</t>
         </is>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="2" t="inlineStr">
         <is>
-          <t>T373</t>
+          <t>SO3</t>
         </is>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="2" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>SSR101</t>
         </is>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="2" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>SSR102</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="2" t="inlineStr">
         <is>
-          <t>TE2804</t>
+          <t>SSR103</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="2" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>SSR104</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" s="2" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>T373</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" s="2" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>TE2801</t>
         </is>
       </c>
     </row>
     <row r="490">
       <c r="A490" s="2" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>TE2803</t>
         </is>
       </c>
     </row>
     <row r="491">
       <c r="A491" s="2" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>TE2804</t>
         </is>
       </c>
     </row>
     <row r="492">
       <c r="A492" s="2" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>TE2805</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="2" t="inlineStr">
         <is>
-          <t>TT02</t>
+          <t>TE2807</t>
         </is>
       </c>
     </row>
     <row r="494">
       <c r="A494" s="2" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TE2808</t>
         </is>
       </c>
     </row>
     <row r="495">
       <c r="A495" s="2" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TE2813</t>
         </is>
       </c>
     </row>
     <row r="496">
       <c r="A496" s="2" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TE2814</t>
         </is>
       </c>
     </row>
     <row r="497">
       <c r="A497" s="2" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TJ096</t>
         </is>
       </c>
     </row>
     <row r="498">
       <c r="A498" s="2" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TT02</t>
         </is>
       </c>
     </row>
     <row r="499">
       <c r="A499" s="2" t="inlineStr">
         <is>
-          <t>TT104</t>
+          <t>TT03</t>
         </is>
       </c>
     </row>
     <row r="500">
       <c r="A500" s="2" t="inlineStr">
         <is>
-          <t>TT105</t>
+          <t>TT04</t>
         </is>
       </c>
     </row>
     <row r="501">
       <c r="A501" s="2" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TT05</t>
         </is>
       </c>
     </row>
     <row r="502">
       <c r="A502" s="2" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TT08</t>
         </is>
       </c>
     </row>
     <row r="503">
       <c r="A503" s="2" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT103</t>
         </is>
       </c>
     </row>
     <row r="504">
       <c r="A504" s="2" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT104</t>
         </is>
       </c>
     </row>
     <row r="505">
       <c r="A505" s="2" t="inlineStr">
         <is>
-          <t>TT123</t>
+          <t>TT105</t>
         </is>
       </c>
     </row>
     <row r="506">
       <c r="A506" s="2" t="inlineStr">
         <is>
-          <t>TT126</t>
+          <t>TT107</t>
         </is>
       </c>
     </row>
     <row r="507">
       <c r="A507" s="2" t="inlineStr">
         <is>
-          <t>TT129</t>
+          <t>TT110</t>
         </is>
       </c>
     </row>
     <row r="508">
       <c r="A508" s="2" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT115</t>
         </is>
       </c>
     </row>
     <row r="509">
       <c r="A509" s="2" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT117</t>
         </is>
       </c>
     </row>
     <row r="510">
       <c r="A510" s="2" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT123</t>
         </is>
       </c>
     </row>
     <row r="511">
       <c r="A511" s="2" t="inlineStr">
         <is>
-          <t>VL01</t>
+          <t>TT126</t>
         </is>
       </c>
     </row>
     <row r="512">
       <c r="A512" s="2" t="inlineStr">
         <is>
-          <t>VL03</t>
+          <t>TT129</t>
         </is>
       </c>
     </row>
     <row r="513">
       <c r="A513" s="2" t="inlineStr">
         <is>
-          <t>VL04</t>
+          <t>TT130</t>
         </is>
       </c>
     </row>
     <row r="514">
       <c r="A514" s="2" t="inlineStr">
         <is>
-          <t>VL11</t>
+          <t>TT202</t>
         </is>
       </c>
     </row>
     <row r="515">
       <c r="A515" s="2" t="inlineStr">
         <is>
-          <t>VL13</t>
+          <t>TT206</t>
         </is>
       </c>
     </row>
     <row r="516">
       <c r="A516" s="2" t="inlineStr">
         <is>
-          <t>VL20</t>
+          <t>VL01</t>
         </is>
       </c>
     </row>
     <row r="517">
       <c r="A517" s="2" t="inlineStr">
         <is>
-          <t>VL22</t>
+          <t>VL03</t>
         </is>
       </c>
     </row>
     <row r="518">
       <c r="A518" s="2" t="inlineStr">
         <is>
-          <t>VL27</t>
+          <t>VL04</t>
         </is>
       </c>
     </row>
     <row r="519">
       <c r="A519" s="2" t="inlineStr">
         <is>
-          <t>VL30</t>
+          <t>VL11</t>
         </is>
       </c>
     </row>
     <row r="520">
       <c r="A520" s="2" t="inlineStr">
         <is>
-          <t>VL35</t>
+          <t>VL13</t>
         </is>
       </c>
     </row>
     <row r="521">
       <c r="A521" s="2" t="inlineStr">
         <is>
-          <t>VL36</t>
+          <t>VL20</t>
         </is>
       </c>
     </row>
     <row r="522">
       <c r="A522" s="2" t="inlineStr">
         <is>
-          <t>VL38</t>
+          <t>VL22</t>
         </is>
       </c>
     </row>
     <row r="523">
       <c r="A523" s="2" t="inlineStr">
         <is>
-          <t>VL43</t>
+          <t>VL27</t>
         </is>
       </c>
     </row>
     <row r="524">
       <c r="A524" s="2" t="inlineStr">
         <is>
-          <t>VL47</t>
+          <t>VL30</t>
         </is>
       </c>
     </row>
     <row r="525">
       <c r="A525" s="2" t="inlineStr">
         <is>
-          <t>VL49</t>
+          <t>VL35</t>
         </is>
       </c>
     </row>
     <row r="526">
       <c r="A526" s="2" t="inlineStr">
         <is>
-          <t>VL57</t>
+          <t>VL36</t>
         </is>
       </c>
     </row>
     <row r="527">
       <c r="A527" s="2" t="inlineStr">
         <is>
-          <t>VL62</t>
+          <t>VL38</t>
         </is>
       </c>
     </row>
     <row r="528">
       <c r="A528" s="2" t="inlineStr">
         <is>
-          <t>VL67</t>
+          <t>VL43</t>
         </is>
       </c>
     </row>
     <row r="529">
       <c r="A529" s="2" t="inlineStr">
         <is>
-          <t>VL75</t>
+          <t>VL47</t>
         </is>
       </c>
     </row>
     <row r="530">
       <c r="A530" s="2" t="inlineStr">
         <is>
-          <t>VL81</t>
+          <t>VL49</t>
         </is>
       </c>
     </row>
     <row r="531">
       <c r="A531" s="2" t="inlineStr">
         <is>
-          <t>VL86</t>
+          <t>VL57</t>
         </is>
       </c>
     </row>
     <row r="532">
       <c r="A532" s="2" t="inlineStr">
         <is>
-          <t>VL87</t>
+          <t>VL62</t>
         </is>
       </c>
     </row>
     <row r="533">
       <c r="A533" s="2" t="inlineStr">
         <is>
-          <t>VL88</t>
+          <t>VL67</t>
         </is>
       </c>
     </row>
     <row r="534">
       <c r="A534" s="2" t="inlineStr">
         <is>
-          <t>VL90</t>
+          <t>VL68</t>
         </is>
       </c>
     </row>
     <row r="535">
       <c r="A535" s="2" t="inlineStr">
         <is>
-          <t>VL92</t>
+          <t>VL75</t>
         </is>
       </c>
     </row>
     <row r="536">
       <c r="A536" s="2" t="inlineStr">
         <is>
-          <t>VL99</t>
+          <t>VL81</t>
         </is>
       </c>
     </row>
     <row r="537">
       <c r="A537" s="2" t="inlineStr">
         <is>
-          <t>VL100</t>
+          <t>VL86</t>
         </is>
       </c>
     </row>
     <row r="538">
       <c r="A538" s="2" t="inlineStr">
         <is>
-          <t>VL101</t>
+          <t>VL87</t>
         </is>
       </c>
     </row>
     <row r="539">
       <c r="A539" s="2" t="inlineStr">
         <is>
-          <t>VL103</t>
+          <t>VL88</t>
         </is>
       </c>
     </row>
     <row r="540">
       <c r="A540" s="2" t="inlineStr">
         <is>
-          <t>VL107</t>
+          <t>VL90</t>
         </is>
       </c>
     </row>
     <row r="541">
       <c r="A541" s="2" t="inlineStr">
         <is>
-          <t>VL112</t>
+          <t>VL92</t>
         </is>
       </c>
     </row>
     <row r="542">
       <c r="A542" s="2" t="inlineStr">
         <is>
-          <t>VL114</t>
+          <t>VL99</t>
         </is>
       </c>
     </row>
     <row r="543">
       <c r="A543" s="2" t="inlineStr">
         <is>
-          <t>VL115</t>
+          <t>VL100</t>
         </is>
       </c>
     </row>
     <row r="544">
       <c r="A544" s="2" t="inlineStr">
         <is>
-          <t>VL121</t>
+          <t>VL101</t>
         </is>
       </c>
     </row>
     <row r="545">
       <c r="A545" s="2" t="inlineStr">
         <is>
-          <t>VL122</t>
+          <t>VL103</t>
         </is>
       </c>
     </row>
     <row r="546">
       <c r="A546" s="2" t="inlineStr">
         <is>
-          <t>VL123</t>
+          <t>VL107</t>
         </is>
       </c>
     </row>
     <row r="547">
       <c r="A547" s="2" t="inlineStr">
         <is>
-          <t>VL124</t>
+          <t>VL112</t>
         </is>
       </c>
     </row>
     <row r="548">
       <c r="A548" s="2" t="inlineStr">
         <is>
-          <t>VL125</t>
+          <t>VL114</t>
         </is>
       </c>
     </row>
     <row r="549">
       <c r="A549" s="2" t="inlineStr">
         <is>
-          <t>VL126</t>
+          <t>VL115</t>
         </is>
       </c>
     </row>
     <row r="550">
       <c r="A550" s="2" t="inlineStr">
         <is>
-          <t>VL127</t>
+          <t>VL121</t>
         </is>
       </c>
     </row>
     <row r="551">
       <c r="A551" s="2" t="inlineStr">
         <is>
-          <t>VL129</t>
+          <t>VL122</t>
         </is>
       </c>
     </row>
     <row r="552">
       <c r="A552" s="2" t="inlineStr">
         <is>
-          <t>VL132</t>
+          <t>VL123</t>
         </is>
       </c>
     </row>
     <row r="553">
       <c r="A553" s="2" t="inlineStr">
         <is>
-          <t>VL134</t>
+          <t>VL124</t>
         </is>
       </c>
     </row>
     <row r="554">
       <c r="A554" s="2" t="inlineStr">
         <is>
-          <t>VL137</t>
+          <t>VL125</t>
         </is>
       </c>
     </row>
     <row r="555">
       <c r="A555" s="2" t="inlineStr">
         <is>
-          <t>VL139</t>
+          <t>VL126</t>
         </is>
       </c>
     </row>
     <row r="556">
       <c r="A556" s="2" t="inlineStr">
         <is>
-          <t>VL140</t>
+          <t>VL127</t>
         </is>
       </c>
     </row>
     <row r="557">
       <c r="A557" s="2" t="inlineStr">
         <is>
-          <t>VL354</t>
+          <t>VL129</t>
         </is>
       </c>
     </row>
     <row r="558">
       <c r="A558" s="2" t="inlineStr">
         <is>
-          <t>VLINE8013</t>
+          <t>VL132</t>
         </is>
       </c>
     </row>
     <row r="559">
       <c r="A559" s="2" t="inlineStr">
         <is>
-          <t>VLINE8020</t>
+          <t>VL134</t>
         </is>
       </c>
     </row>
     <row r="560">
       <c r="A560" s="2" t="inlineStr">
         <is>
-          <t>VLINE8021</t>
+          <t>VL137</t>
         </is>
       </c>
     </row>
     <row r="561">
       <c r="A561" s="2" t="inlineStr">
         <is>
-          <t>VLINE8023</t>
+          <t>VL139</t>
         </is>
       </c>
     </row>
     <row r="562">
       <c r="A562" s="2" t="inlineStr">
         <is>
-          <t>VLINE8028</t>
+          <t>VL140</t>
         </is>
       </c>
     </row>
     <row r="563">
       <c r="A563" s="2" t="inlineStr">
         <is>
-          <t>VLINE8030</t>
+          <t>VL354</t>
         </is>
       </c>
     </row>
     <row r="564">
       <c r="A564" s="2" t="inlineStr">
         <is>
-          <t>VLINE8058</t>
+          <t>VLINE8013</t>
         </is>
       </c>
     </row>
     <row r="565">
       <c r="A565" s="2" t="inlineStr">
         <is>
-          <t>VLINE8059</t>
+          <t>VLINE8020</t>
         </is>
       </c>
     </row>
     <row r="566">
       <c r="A566" s="2" t="inlineStr">
         <is>
-          <t>VLINE8061</t>
+          <t>VLINE8021</t>
         </is>
       </c>
     </row>
     <row r="567">
       <c r="A567" s="2" t="inlineStr">
         <is>
-          <t>VLINE8071</t>
+          <t>VLINE8023</t>
         </is>
       </c>
     </row>
     <row r="568">
       <c r="A568" s="2" t="inlineStr">
         <is>
-          <t>VLINE8072</t>
+          <t>VLINE8028</t>
         </is>
       </c>
     </row>
     <row r="569">
       <c r="A569" s="2" t="inlineStr">
         <is>
-          <t>VLINE8074</t>
+          <t>VLINE8030</t>
         </is>
       </c>
     </row>
     <row r="570">
       <c r="A570" s="2" t="inlineStr">
         <is>
-          <t>VLINE8075</t>
+          <t>VLINE8058</t>
         </is>
       </c>
     </row>
     <row r="571">
       <c r="A571" s="2" t="inlineStr">
         <is>
-          <t>VLINE8080</t>
+          <t>VLINE8059</t>
         </is>
       </c>
     </row>
     <row r="572">
       <c r="A572" s="2" t="inlineStr">
         <is>
-          <t>VLINE8081</t>
+          <t>VLINE8061</t>
         </is>
       </c>
     </row>
     <row r="573">
       <c r="A573" s="2" t="inlineStr">
         <is>
-          <t>VLINE8102</t>
+          <t>VLINE8071</t>
         </is>
       </c>
     </row>
     <row r="574">
       <c r="A574" s="2" t="inlineStr">
         <is>
-          <t>VLINE8111</t>
+          <t>VLINE8072</t>
         </is>
       </c>
     </row>
     <row r="575">
       <c r="A575" s="2" t="inlineStr">
         <is>
-          <t>VLINE8113</t>
+          <t>VLINE8074</t>
         </is>
       </c>
     </row>
     <row r="576">
       <c r="A576" s="2" t="inlineStr">
         <is>
-          <t>VLINE8115</t>
+          <t>VLINE8075</t>
         </is>
       </c>
     </row>
     <row r="577">
       <c r="A577" s="2" t="inlineStr">
         <is>
-          <t>VLINE8117</t>
+          <t>VLINE8080</t>
         </is>
       </c>
     </row>
     <row r="578">
       <c r="A578" s="2" t="inlineStr">
         <is>
-          <t>VLINE8120</t>
+          <t>VLINE8081</t>
         </is>
       </c>
     </row>
     <row r="579">
       <c r="A579" s="2" t="inlineStr">
         <is>
-          <t>VLINE8121</t>
+          <t>VLINE8102</t>
         </is>
       </c>
     </row>
     <row r="580">
       <c r="A580" s="2" t="inlineStr">
         <is>
-          <t>VLINE8122</t>
+          <t>VLINE8111</t>
         </is>
       </c>
     </row>
     <row r="581">
       <c r="A581" s="2" t="inlineStr">
         <is>
-          <t>VLINE8123</t>
+          <t>VLINE8113</t>
         </is>
       </c>
     </row>
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>VLINE8124</t>
+          <t>VLINE8115</t>
         </is>
       </c>
     </row>
     <row r="583">
       <c r="A583" s="2" t="inlineStr">
         <is>
-          <t>VLINE8126</t>
+          <t>VLINE8117</t>
         </is>
       </c>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>VLINE8128</t>
+          <t>VLINE8120</t>
         </is>
       </c>
     </row>
     <row r="585">
       <c r="A585" s="2" t="inlineStr">
         <is>
-          <t>VLINE8130</t>
+          <t>VLINE8121</t>
         </is>
       </c>
     </row>
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>VLINE8161</t>
+          <t>VLINE8122</t>
         </is>
       </c>
     </row>
     <row r="587">
       <c r="A587" s="2" t="inlineStr">
         <is>
-          <t>VLINE8163</t>
+          <t>VLINE8123</t>
         </is>
       </c>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>VLINE8164</t>
+          <t>VLINE8124</t>
         </is>
       </c>
     </row>
     <row r="589">
       <c r="A589" s="2" t="inlineStr">
         <is>
-          <t>VLINE8172</t>
+          <t>VLINE8125</t>
         </is>
       </c>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>VLINE8181</t>
+          <t>VLINE8126</t>
         </is>
       </c>
     </row>
     <row r="591">
       <c r="A591" s="2" t="inlineStr">
         <is>
-          <t>VLINE8183</t>
+          <t>VLINE8128</t>
         </is>
       </c>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>VLINE8184</t>
+          <t>VLINE8130</t>
         </is>
       </c>
     </row>
     <row r="593">
       <c r="A593" s="2" t="inlineStr">
         <is>
-          <t>VLINE8211</t>
+          <t>VLINE8161</t>
         </is>
       </c>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>VLINE8213</t>
+          <t>VLINE8163</t>
         </is>
       </c>
     </row>
     <row r="595">
       <c r="A595" s="2" t="inlineStr">
         <is>
-          <t>VLINE8215</t>
+          <t>VLINE8164</t>
         </is>
       </c>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>VLINE8217</t>
+          <t>VLINE8172</t>
         </is>
       </c>
     </row>
     <row r="597">
       <c r="A597" s="2" t="inlineStr">
         <is>
-          <t>VLINE8219</t>
+          <t>VLINE8181</t>
         </is>
       </c>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>VLINE8221</t>
+          <t>VLINE8183</t>
         </is>
       </c>
     </row>
     <row r="599">
       <c r="A599" s="2" t="inlineStr">
         <is>
-          <t>VLINE8223</t>
+          <t>VLINE8184</t>
         </is>
       </c>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>VLINE8226</t>
+          <t>VLINE8211</t>
         </is>
       </c>
     </row>
     <row r="601">
       <c r="A601" s="2" t="inlineStr">
         <is>
-          <t>VLINE8228</t>
+          <t>VLINE8213</t>
         </is>
       </c>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>VLINE8230</t>
+          <t>VLINE8215</t>
         </is>
       </c>
     </row>
     <row r="603">
       <c r="A603" s="2" t="inlineStr">
         <is>
-          <t>VLINE8232</t>
+          <t>VLINE8217</t>
         </is>
       </c>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>VLINE8234</t>
+          <t>VLINE8219</t>
         </is>
       </c>
     </row>
     <row r="605">
       <c r="A605" s="2" t="inlineStr">
         <is>
-          <t>VLINE8236</t>
+          <t>VLINE8221</t>
         </is>
       </c>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>VLINE8400</t>
+          <t>VLINE8223</t>
         </is>
       </c>
     </row>
     <row r="607">
       <c r="A607" s="2" t="inlineStr">
         <is>
-          <t>VLINE8405</t>
+          <t>VLINE8225</t>
         </is>
       </c>
     </row>
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>VLINE8408</t>
+          <t>VLINE8226</t>
         </is>
       </c>
     </row>
     <row r="609">
       <c r="A609" s="2" t="inlineStr">
         <is>
-          <t>VLINE8413</t>
+          <t>VLINE8228</t>
         </is>
       </c>
     </row>
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>VLINE8415</t>
+          <t>VLINE8230</t>
         </is>
       </c>
     </row>
     <row r="611">
       <c r="A611" s="2" t="inlineStr">
         <is>
-          <t>VLINE8417</t>
+          <t>VLINE8232</t>
         </is>
       </c>
     </row>
     <row r="612">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>VLINE8418</t>
+          <t>VLINE8234</t>
         </is>
       </c>
     </row>
     <row r="613">
       <c r="A613" s="2" t="inlineStr">
         <is>
-          <t>VLINE8419</t>
+          <t>VLINE8236</t>
         </is>
       </c>
     </row>
     <row r="614">
       <c r="A614" s="2" t="inlineStr">
         <is>
-          <t>VLINE8420</t>
+          <t>VLINE8238</t>
         </is>
       </c>
     </row>
     <row r="615">
       <c r="A615" s="2" t="inlineStr">
         <is>
-          <t>VLINE8421</t>
+          <t>VLINE8400</t>
         </is>
       </c>
     </row>
     <row r="616">
       <c r="A616" s="2" t="inlineStr">
         <is>
-          <t>VLINE8422</t>
+          <t>VLINE8405</t>
         </is>
       </c>
     </row>
     <row r="617">
       <c r="A617" s="2" t="inlineStr">
         <is>
-          <t>VLINE8423</t>
+          <t>VLINE8408</t>
         </is>
       </c>
     </row>
     <row r="618">
       <c r="A618" s="2" t="inlineStr">
         <is>
-          <t>VLINE8424</t>
+          <t>VLINE8413</t>
         </is>
       </c>
     </row>
     <row r="619">
       <c r="A619" s="2" t="inlineStr">
         <is>
-          <t>VLINE8428</t>
+          <t>VLINE8415</t>
         </is>
       </c>
     </row>
     <row r="620">
       <c r="A620" s="2" t="inlineStr">
         <is>
-          <t>VLINE8430</t>
+          <t>VLINE8417</t>
         </is>
       </c>
     </row>
     <row r="621">
       <c r="A621" s="2" t="inlineStr">
         <is>
-          <t>VLINE8457</t>
+          <t>VLINE8418</t>
         </is>
       </c>
     </row>
     <row r="622">
       <c r="A622" s="2" t="inlineStr">
         <is>
-          <t>VLINE8459</t>
+          <t>VLINE8419</t>
         </is>
       </c>
     </row>
     <row r="623">
       <c r="A623" s="2" t="inlineStr">
         <is>
-          <t>VLINE8460</t>
+          <t>VLINE8420</t>
         </is>
       </c>
     </row>
     <row r="624">
       <c r="A624" s="2" t="inlineStr">
         <is>
-          <t>VLINE8461</t>
+          <t>VLINE8421</t>
         </is>
       </c>
     </row>
     <row r="625">
       <c r="A625" s="2" t="inlineStr">
         <is>
-          <t>VLINE8465</t>
+          <t>VLINE8422</t>
         </is>
       </c>
     </row>
     <row r="626">
       <c r="A626" s="2" t="inlineStr">
         <is>
-          <t>VLINE8702</t>
+          <t>VLINE8423</t>
         </is>
       </c>
     </row>
     <row r="627">
       <c r="A627" s="2" t="inlineStr">
         <is>
-          <t>VLINE8725</t>
+          <t>VLINE8424</t>
         </is>
       </c>
     </row>
     <row r="628">
       <c r="A628" s="2" t="inlineStr">
         <is>
-          <t>VLINE8727</t>
+          <t>VLINE8428</t>
         </is>
       </c>
     </row>
     <row r="629">
       <c r="A629" s="2" t="inlineStr">
         <is>
-          <t>VLINE8729</t>
+          <t>VLINE8430</t>
         </is>
       </c>
     </row>
     <row r="630">
       <c r="A630" s="2" t="inlineStr">
         <is>
-          <t>VLINE8731</t>
+          <t>VLINE8457</t>
         </is>
       </c>
     </row>
     <row r="631">
       <c r="A631" s="2" t="inlineStr">
         <is>
-          <t>VLINE8733</t>
+          <t>VLINE8459</t>
         </is>
       </c>
     </row>
     <row r="632">
       <c r="A632" s="2" t="inlineStr">
         <is>
-          <t>VLINE8735</t>
+          <t>VLINE8460</t>
         </is>
       </c>
     </row>
     <row r="633">
       <c r="A633" s="2" t="inlineStr">
         <is>
-          <t>VLINE8737</t>
+          <t>VLINE8461</t>
         </is>
       </c>
     </row>
     <row r="634">
       <c r="A634" s="2" t="inlineStr">
         <is>
-          <t>VLINE8739</t>
+          <t>VLINE8465</t>
         </is>
       </c>
     </row>
     <row r="635">
       <c r="A635" s="2" t="inlineStr">
         <is>
-          <t>VLINE8741</t>
+          <t>VLINE8702</t>
         </is>
       </c>
     </row>
     <row r="636">
       <c r="A636" s="2" t="inlineStr">
         <is>
-          <t>VLINE8742</t>
+          <t>VLINE8725</t>
         </is>
       </c>
     </row>
     <row r="637">
       <c r="A637" s="2" t="inlineStr">
         <is>
-          <t>VLINE8743</t>
+          <t>VLINE8727</t>
         </is>
       </c>
     </row>
     <row r="638">
       <c r="A638" s="2" t="inlineStr">
         <is>
-          <t>VLINE8744</t>
+          <t>VLINE8729</t>
         </is>
       </c>
     </row>
     <row r="639">
       <c r="A639" s="2" t="inlineStr">
         <is>
-          <t>VLINE8745</t>
+          <t>VLINE8731</t>
         </is>
       </c>
     </row>
     <row r="640">
       <c r="A640" s="2" t="inlineStr">
         <is>
-          <t>VLINE8746</t>
+          <t>VLINE8733</t>
         </is>
       </c>
     </row>
     <row r="641">
       <c r="A641" s="2" t="inlineStr">
         <is>
-          <t>VLINE8747</t>
+          <t>VLINE8735</t>
         </is>
       </c>
     </row>
     <row r="642">
       <c r="A642" s="2" t="inlineStr">
         <is>
-          <t>VLINE8748</t>
+          <t>VLINE8737</t>
         </is>
       </c>
     </row>
     <row r="643">
       <c r="A643" s="2" t="inlineStr">
         <is>
-          <t>VLINE8749</t>
+          <t>VLINE8739</t>
         </is>
       </c>
     </row>
     <row r="644">
       <c r="A644" s="2" t="inlineStr">
         <is>
-          <t>VLINE8750</t>
+          <t>VLINE8741</t>
         </is>
       </c>
     </row>
     <row r="645">
       <c r="A645" s="2" t="inlineStr">
         <is>
-          <t>VLINE8751</t>
+          <t>VLINE8742</t>
         </is>
       </c>
     </row>
     <row r="646">
       <c r="A646" s="2" t="inlineStr">
         <is>
-          <t>VLINE8752</t>
+          <t>VLINE8743</t>
         </is>
       </c>
     </row>
     <row r="647">
       <c r="A647" s="2" t="inlineStr">
         <is>
-          <t>VLINE8754</t>
+          <t>VLINE8744</t>
         </is>
       </c>
     </row>
     <row r="648">
       <c r="A648" s="2" t="inlineStr">
         <is>
-          <t>VLINE8756</t>
+          <t>VLINE8745</t>
         </is>
       </c>
     </row>
     <row r="649">
       <c r="A649" s="2" t="inlineStr">
         <is>
-          <t>VLINE8758</t>
+          <t>VLINE8746</t>
         </is>
       </c>
     </row>
     <row r="650">
       <c r="A650" s="2" t="inlineStr">
         <is>
-          <t>VLINE8760</t>
+          <t>VLINE8747</t>
         </is>
       </c>
     </row>
     <row r="651">
       <c r="A651" s="2" t="inlineStr">
         <is>
-          <t>VLINE8762</t>
+          <t>VLINE8748</t>
         </is>
       </c>
     </row>
     <row r="652">
       <c r="A652" s="2" t="inlineStr">
         <is>
-          <t>VLINE8764</t>
+          <t>VLINE8749</t>
         </is>
       </c>
     </row>
     <row r="653">
       <c r="A653" s="2" t="inlineStr">
         <is>
-          <t>VLINE8819</t>
+          <t>VLINE8750</t>
         </is>
       </c>
     </row>
     <row r="654">
       <c r="A654" s="2" t="inlineStr">
         <is>
-          <t>VLINE8862</t>
+          <t>VLINE8751</t>
         </is>
       </c>
     </row>
     <row r="655">
       <c r="A655" s="2" t="inlineStr">
         <is>
-          <t>VLINE8863</t>
+          <t>VLINE8752</t>
         </is>
       </c>
     </row>
     <row r="656">
       <c r="A656" s="2" t="inlineStr">
         <is>
-          <t>VR77</t>
+          <t>VLINE8753</t>
         </is>
       </c>
     </row>
     <row r="657">
       <c r="A657" s="2" t="inlineStr">
         <is>
-          <t>WOLL408</t>
+          <t>VLINE8754</t>
         </is>
       </c>
     </row>
     <row r="658">
       <c r="A658" s="2" t="inlineStr">
         <is>
-          <t>WOLL430</t>
+          <t>VLINE8756</t>
         </is>
       </c>
     </row>
     <row r="659">
       <c r="A659" s="2" t="inlineStr">
         <is>
-          <t>XP2001</t>
+          <t>VLINE8758</t>
         </is>
       </c>
     </row>
     <row r="660">
       <c r="A660" s="2" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>VLINE8760</t>
         </is>
       </c>
     </row>
     <row r="661">
       <c r="A661" s="2" t="inlineStr">
         <is>
-          <t>XP2006</t>
+          <t>VLINE8762</t>
         </is>
       </c>
     </row>
     <row r="662">
       <c r="A662" s="2" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>VLINE8764</t>
         </is>
       </c>
     </row>
     <row r="663">
       <c r="A663" s="2" t="inlineStr">
         <is>
-          <t>XP2009</t>
+          <t>VLINE8766</t>
         </is>
       </c>
     </row>
     <row r="664">
       <c r="A664" s="2" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>VLINE8819</t>
         </is>
       </c>
     </row>
     <row r="665">
       <c r="A665" s="2" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>VLINE8862</t>
         </is>
       </c>
     </row>
     <row r="666">
       <c r="A666" s="2" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>VLINE8863</t>
         </is>
       </c>
     </row>
     <row r="667">
       <c r="A667" s="2" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>VLINE8865</t>
         </is>
       </c>
     </row>
     <row r="668">
       <c r="A668" s="2" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>VR76</t>
         </is>
       </c>
     </row>
     <row r="669">
       <c r="A669" s="2" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>VR77</t>
         </is>
       </c>
     </row>
     <row r="670">
       <c r="A670" s="2" t="inlineStr">
         <is>
-          <t>XRN003</t>
+          <t>WOLL408</t>
         </is>
       </c>
     </row>
     <row r="671">
       <c r="A671" s="2" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>WOLL430</t>
         </is>
       </c>
     </row>
     <row r="672">
       <c r="A672" s="2" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>XP2001</t>
         </is>
       </c>
     </row>
     <row r="673">
       <c r="A673" s="2" t="inlineStr">
         <is>
-          <t>XRN010</t>
+          <t>XP2005</t>
         </is>
       </c>
     </row>
     <row r="674">
       <c r="A674" s="2" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>XP2006</t>
         </is>
       </c>
     </row>
     <row r="675">
       <c r="A675" s="2" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>XP2008</t>
         </is>
       </c>
     </row>
     <row r="676">
       <c r="A676" s="2" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>XP2009</t>
         </is>
       </c>
     </row>
     <row r="677">
       <c r="A677" s="2" t="inlineStr">
         <is>
-          <t>XRN022</t>
+          <t>XP2011</t>
         </is>
       </c>
     </row>
     <row r="678">
       <c r="A678" s="2" t="inlineStr">
         <is>
-          <t>XRN028</t>
+          <t>XP2012</t>
         </is>
       </c>
     </row>
     <row r="679">
       <c r="A679" s="2" t="inlineStr">
+        <is>
+          <t>XP2013</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="2" t="inlineStr">
+        <is>
+          <t>XP2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="2" t="inlineStr">
+        <is>
+          <t>XP2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" s="2" t="inlineStr">
+        <is>
+          <t>XP2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" s="2" t="inlineStr">
+        <is>
+          <t>XRN003</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="2" t="inlineStr">
+        <is>
+          <t>XRN005</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="2" t="inlineStr">
+        <is>
+          <t>XRN009</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" s="2" t="inlineStr">
+        <is>
+          <t>XRN010</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" s="2" t="inlineStr">
+        <is>
+          <t>XRN017</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="2" t="inlineStr">
+        <is>
+          <t>XRN018</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="2" t="inlineStr">
+        <is>
+          <t>XRN021</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="2" t="inlineStr">
+        <is>
+          <t>XRN022</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="2" t="inlineStr">
+        <is>
+          <t>XRN028</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="2" t="inlineStr">
         <is>
           <t>XRN029</t>
         </is>

</xml_diff>

<commit_message>
Update RailOps database files - 2026-04-30 05:02:17 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A729"/>
+  <dimension ref="A1:A751"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2309,3246 +2309,3400 @@
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>MM260M</t>
+          <t>MM256M</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>MM264M</t>
+          <t>MM260M</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>MM266M</t>
+          <t>MM264M</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>MM268M</t>
+          <t>MM266M</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>MM270M</t>
+          <t>MM268M</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>MM280M</t>
+          <t>MM270M</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>MM288M</t>
+          <t>MM280M</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>MM380M</t>
+          <t>MM288M</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>MM456M</t>
+          <t>MM380M</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>MM464M</t>
+          <t>MM418M</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>MM478M</t>
+          <t>MM456M</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>MM482M</t>
+          <t>MM464M</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>MM486M</t>
+          <t>MM478M</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>MM502M</t>
+          <t>MM482M</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>MM506M</t>
+          <t>MM486M</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>MM514M</t>
+          <t>MM502M</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>MM522M</t>
+          <t>MM506M</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>MM536M</t>
+          <t>MM514M</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>MM542M</t>
+          <t>MM522M</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>MM544M</t>
+          <t>MM536M</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>MM546M</t>
+          <t>MM542M</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>MM551M</t>
+          <t>MM544M</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>MM566M</t>
+          <t>MM546M</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>MM574M</t>
+          <t>MM551M</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>MM588M</t>
+          <t>MM566M</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>MM592M</t>
+          <t>MM574M</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>MM604M</t>
+          <t>MM588M</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>MM624M</t>
+          <t>MM592M</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>MM636M</t>
+          <t>MM602M</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>MM638M</t>
+          <t>MM604M</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>MM647M</t>
+          <t>MM624M</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>MM656M</t>
+          <t>MM636M</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>MM658M</t>
+          <t>MM638M</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>MM660M</t>
+          <t>MM647M</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>MM662M</t>
+          <t>MM656M</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>MM664M</t>
+          <t>MM658M</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>MM668M</t>
+          <t>MM660M</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>MM673M</t>
+          <t>MM662M</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>MM674M</t>
+          <t>MM664M</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>MM676M</t>
+          <t>MM668M</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>MM680M</t>
+          <t>MM673M</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>MM702M</t>
+          <t>MM674M</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>MM718M</t>
+          <t>MM676M</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>MM742M</t>
+          <t>MM680M</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>MM744M</t>
+          <t>MM702M</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>MM752M</t>
+          <t>MM708M</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>MM756M</t>
+          <t>MM718M</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>MM768M</t>
+          <t>MM742M</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>MM772M</t>
+          <t>MM744M</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>MM774M</t>
+          <t>MM752M</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>MM776M</t>
+          <t>MM756M</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>MM778M</t>
+          <t>MM768M</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>MM780M</t>
+          <t>MM772M</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>MM784M</t>
+          <t>MM774M</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>MM788M</t>
+          <t>MM776M</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>MM790M</t>
+          <t>MM778M</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>MM794M</t>
+          <t>MM780M</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>MM798M</t>
+          <t>MM784M</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>MM800M</t>
+          <t>MM788M</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>MM802M</t>
+          <t>MM790M</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>MM806M</t>
+          <t>MM794M</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>MM808M</t>
+          <t>MM798M</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>MM810M</t>
+          <t>MM800M</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>MM816M</t>
+          <t>MM802M</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>MM826M</t>
+          <t>MM806M</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>MM830M</t>
+          <t>MM808M</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>MM832M</t>
+          <t>MM810M</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>MM834M</t>
+          <t>MM816M</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>MM838M</t>
+          <t>MM826M</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>MM842M</t>
+          <t>MM830M</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>MM858M</t>
+          <t>MM832M</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>MM860M</t>
+          <t>MM834M</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>MM862M</t>
+          <t>MM836M</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>MM864M</t>
+          <t>MM838M</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>MM866M</t>
+          <t>MM842M</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>MM872M</t>
+          <t>MM858M</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>MM878M</t>
+          <t>MM860M</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>MM880M</t>
+          <t>MM862M</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>MM886M</t>
+          <t>MM864M</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>MM896M</t>
+          <t>MM866M</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>MM908M</t>
+          <t>MM872M</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>MM910M</t>
+          <t>MM878M</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>MM912M</t>
+          <t>MM880M</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>MM914M</t>
+          <t>MM886M</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>MM924M</t>
+          <t>MM896M</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>MM928M</t>
+          <t>MM908M</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>MM934M</t>
+          <t>MM910M</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>MM940M</t>
+          <t>MM912M</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>MM944M</t>
+          <t>MM914M</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>MM946M</t>
+          <t>MM924M</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>MM952M</t>
+          <t>MM928M</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>MM956M</t>
+          <t>MM934M</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>MM958M</t>
+          <t>MM940M</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>MM960M</t>
+          <t>MM944M</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>MM962M</t>
+          <t>MM946M</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>MM964M</t>
+          <t>MM952M</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>MM968M</t>
+          <t>MM956M</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>MM972M</t>
+          <t>MM958M</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>MM974M</t>
+          <t>MM960M</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>MM976M</t>
+          <t>MM962M</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>MM980M</t>
+          <t>MM964M</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>MM982M</t>
+          <t>MM968M</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>MM9901M</t>
+          <t>MM970M</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>MM9903M</t>
+          <t>MM972M</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>MM9904M</t>
+          <t>MM974M</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>MM9906M</t>
+          <t>MM976M</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>MM9908M</t>
+          <t>MM980M</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t>MM9909M</t>
+          <t>MM982M</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>MM9910M</t>
+          <t>MM9901M</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t>MM9912M</t>
+          <t>MM9903M</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>MM9914M</t>
+          <t>MM9904M</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>MM9916M</t>
+          <t>MM9906M</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>MM9918M</t>
+          <t>MM9908M</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>MM9920M</t>
+          <t>MM9909M</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>MM9921M</t>
+          <t>MM9910M</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>MM9924M</t>
+          <t>MM9912M</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>MM9926M</t>
+          <t>MM9914M</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
         <is>
-          <t>MM9927M</t>
+          <t>MM9916M</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>MM9928M</t>
+          <t>MM9918M</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
         <is>
-          <t>MM9929M</t>
+          <t>MM9920M</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
         <is>
-          <t>MM9931M</t>
+          <t>MM9921M</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" s="2" t="inlineStr">
         <is>
-          <t>MM9936M</t>
+          <t>MM9924M</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
         <is>
-          <t>MM9937M</t>
+          <t>MM9926M</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
         <is>
-          <t>MM9938M</t>
+          <t>MM9927M</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>MM9941M</t>
+          <t>MM9928M</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
         <is>
-          <t>MM9943M</t>
+          <t>MM9929M</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
         <is>
-          <t>MM9946M</t>
+          <t>MM9931M</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="2" t="inlineStr">
         <is>
-          <t>MM9947M</t>
+          <t>MM9933M</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
         <is>
-          <t>MM9948M</t>
+          <t>MM9936M</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" s="2" t="inlineStr">
         <is>
-          <t>MM9952M</t>
+          <t>MM9937M</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
         <is>
-          <t>MM9953M</t>
+          <t>MM9938M</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="2" t="inlineStr">
         <is>
-          <t>MM9954M</t>
+          <t>MM9941M</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" s="2" t="inlineStr">
         <is>
-          <t>MM9956M</t>
+          <t>MM9943M</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="2" t="inlineStr">
         <is>
-          <t>MM9957M</t>
+          <t>MM9946M</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
         <is>
-          <t>MM9958M</t>
+          <t>MM9947M</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" s="2" t="inlineStr">
         <is>
-          <t>MM9959M</t>
+          <t>MM9948M</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
         <is>
-          <t>MM9960M</t>
+          <t>MM9952M</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" s="2" t="inlineStr">
         <is>
-          <t>MM9961M</t>
+          <t>MM9953M</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" s="2" t="inlineStr">
         <is>
-          <t>MM9962M</t>
+          <t>MM9954M</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
         <is>
-          <t>MM9963M</t>
+          <t>MM9956M</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="2" t="inlineStr">
         <is>
-          <t>MM9964M</t>
+          <t>MM9957M</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
         <is>
-          <t>MM9965M</t>
+          <t>MM9958M</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="2" t="inlineStr">
         <is>
-          <t>MM9966M</t>
+          <t>MM9959M</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="2" t="inlineStr">
         <is>
-          <t>MM9968M</t>
+          <t>MM9960M</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" s="2" t="inlineStr">
         <is>
-          <t>MM9969M</t>
+          <t>MM9961M</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" s="2" t="inlineStr">
         <is>
-          <t>MM9970M</t>
+          <t>MM9962M</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" s="2" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MM9963M</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" s="2" t="inlineStr">
         <is>
-          <t>MRL002</t>
+          <t>MM9964M</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" s="2" t="inlineStr">
         <is>
-          <t>MTPV1</t>
+          <t>MM9965M</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" s="2" t="inlineStr">
         <is>
-          <t>MTPV2</t>
+          <t>MM9966M</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" s="2" t="inlineStr">
         <is>
-          <t>N453</t>
+          <t>MM9968M</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" s="2" t="inlineStr">
         <is>
-          <t>N458</t>
+          <t>MM9969M</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t>N460</t>
+          <t>MM9970M</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" s="2" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>MRL001</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>MRL002</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" s="2" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>MTPV1</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" s="2" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>MTPV2</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" s="2" t="inlineStr">
         <is>
-          <t>NR6</t>
+          <t>N453</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
         <is>
-          <t>NR10</t>
+          <t>N458</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="2" t="inlineStr">
         <is>
-          <t>NR11</t>
+          <t>N460</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
         <is>
-          <t>NR12</t>
+          <t>N466</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
         <is>
-          <t>NR13</t>
+          <t>N469</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>NR14</t>
+          <t>NR4</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" s="2" t="inlineStr">
         <is>
-          <t>NR17</t>
+          <t>NR5</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
         <is>
-          <t>NR20</t>
+          <t>NR6</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" s="2" t="inlineStr">
         <is>
-          <t>NR31</t>
+          <t>NR10</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
         <is>
-          <t>NR35</t>
+          <t>NR11</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" s="2" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>NR12</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t>NR44</t>
+          <t>NR13</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t>NR46</t>
+          <t>NR14</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>NR17</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
         <is>
-          <t>NR52</t>
+          <t>NR20</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>NR31</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
         <is>
-          <t>NR56</t>
+          <t>NR35</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
         <is>
-          <t>NR60</t>
+          <t>NR37</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR44</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR46</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR47</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR52</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
         <is>
-          <t>NR76</t>
+          <t>NR54</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR56</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR60</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR64</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
         <is>
-          <t>NR88</t>
+          <t>NR65</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>NR91</t>
+          <t>NR68</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR75</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR76</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="2" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR78</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>NR82</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" s="2" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR83</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
         <is>
-          <t>NR106</t>
+          <t>NR88</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" s="2" t="inlineStr">
         <is>
-          <t>NR107</t>
+          <t>NR91</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="2" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR93</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" s="2" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR94</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" s="2" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR95</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" s="2" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR97</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" s="2" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>NR102</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="2" t="inlineStr">
         <is>
-          <t>PB5</t>
+          <t>NR106</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="2" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>NR107</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="2" t="inlineStr">
         <is>
-          <t>PKLA4</t>
+          <t>NR109</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="2" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>NR112</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="2" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>NR113</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" s="2" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>NR115</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" s="2" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>PB4</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" s="2" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>PB5</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" s="2" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="A472" s="2" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>PKLA4</t>
         </is>
       </c>
     </row>
     <row r="473">
       <c r="A473" s="2" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="A474" s="2" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
     <row r="475">
       <c r="A475" s="2" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
     <row r="476">
       <c r="A476" s="2" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
     <row r="477">
       <c r="A477" s="2" t="inlineStr">
         <is>
-          <t>QL009</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
     <row r="478">
       <c r="A478" s="2" t="inlineStr">
         <is>
-          <t>QL016</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
     <row r="479">
       <c r="A479" s="2" t="inlineStr">
         <is>
-          <t>QL019</t>
+          <t>QE001</t>
         </is>
       </c>
     </row>
     <row r="480">
       <c r="A480" s="2" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
     <row r="481">
       <c r="A481" s="2" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
     <row r="482">
       <c r="A482" s="2" t="inlineStr">
         <is>
-          <t>QR5400</t>
+          <t>QL004</t>
         </is>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="2" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="2" t="inlineStr">
         <is>
-          <t>RA2302</t>
+          <t>QL009</t>
         </is>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="2" t="inlineStr">
         <is>
-          <t>RA2303</t>
+          <t>QL016</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="2" t="inlineStr">
         <is>
-          <t>RB2352</t>
+          <t>QL019</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="2" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>QR1744</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" s="2" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>QR1771</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" s="2" t="inlineStr">
         <is>
-          <t>RL309</t>
+          <t>QR5400</t>
         </is>
       </c>
     </row>
     <row r="490">
       <c r="A490" s="2" t="inlineStr">
         <is>
-          <t>RM93</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
     <row r="491">
       <c r="A491" s="2" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>RA2302</t>
         </is>
       </c>
     </row>
     <row r="492">
       <c r="A492" s="2" t="inlineStr">
         <is>
-          <t>SCT008</t>
+          <t>RA2303</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="2" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>RB2352</t>
         </is>
       </c>
     </row>
     <row r="494">
       <c r="A494" s="2" t="inlineStr">
         <is>
-          <t>SCT010</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
     <row r="495">
       <c r="A495" s="2" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>RL301</t>
         </is>
       </c>
     </row>
     <row r="496">
       <c r="A496" s="2" t="inlineStr">
         <is>
-          <t>SM636B</t>
+          <t>RL309</t>
         </is>
       </c>
     </row>
     <row r="497">
       <c r="A497" s="2" t="inlineStr">
         <is>
-          <t>SO3</t>
+          <t>RM93</t>
         </is>
       </c>
     </row>
     <row r="498">
       <c r="A498" s="2" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>SCT001</t>
         </is>
       </c>
     </row>
     <row r="499">
       <c r="A499" s="2" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>SCT008</t>
         </is>
       </c>
     </row>
     <row r="500">
       <c r="A500" s="2" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>SCT009</t>
         </is>
       </c>
     </row>
     <row r="501">
       <c r="A501" s="2" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>SCT010</t>
         </is>
       </c>
     </row>
     <row r="502">
       <c r="A502" s="2" t="inlineStr">
         <is>
-          <t>T373</t>
+          <t>SCT013</t>
         </is>
       </c>
     </row>
     <row r="503">
       <c r="A503" s="2" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>SM636B</t>
         </is>
       </c>
     </row>
     <row r="504">
       <c r="A504" s="2" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>SO3</t>
         </is>
       </c>
     </row>
     <row r="505">
       <c r="A505" s="2" t="inlineStr">
         <is>
-          <t>TE2804</t>
+          <t>SSR101</t>
         </is>
       </c>
     </row>
     <row r="506">
       <c r="A506" s="2" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>SSR102</t>
         </is>
       </c>
     </row>
     <row r="507">
       <c r="A507" s="2" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>SSR103</t>
         </is>
       </c>
     </row>
     <row r="508">
       <c r="A508" s="2" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>SSR104</t>
         </is>
       </c>
     </row>
     <row r="509">
       <c r="A509" s="2" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>T373</t>
         </is>
       </c>
     </row>
     <row r="510">
       <c r="A510" s="2" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>TE2801</t>
         </is>
       </c>
     </row>
     <row r="511">
       <c r="A511" s="2" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>TE2803</t>
         </is>
       </c>
     </row>
     <row r="512">
       <c r="A512" s="2" t="inlineStr">
         <is>
-          <t>TT02</t>
+          <t>TE2804</t>
         </is>
       </c>
     </row>
     <row r="513">
       <c r="A513" s="2" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TE2805</t>
         </is>
       </c>
     </row>
     <row r="514">
       <c r="A514" s="2" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TE2807</t>
         </is>
       </c>
     </row>
     <row r="515">
       <c r="A515" s="2" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TE2808</t>
         </is>
       </c>
     </row>
     <row r="516">
       <c r="A516" s="2" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TE2813</t>
         </is>
       </c>
     </row>
     <row r="517">
       <c r="A517" s="2" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TE2814</t>
         </is>
       </c>
     </row>
     <row r="518">
       <c r="A518" s="2" t="inlineStr">
         <is>
-          <t>TT104</t>
+          <t>TJ096</t>
         </is>
       </c>
     </row>
     <row r="519">
       <c r="A519" s="2" t="inlineStr">
         <is>
-          <t>TT105</t>
+          <t>TT02</t>
         </is>
       </c>
     </row>
     <row r="520">
       <c r="A520" s="2" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TT03</t>
         </is>
       </c>
     </row>
     <row r="521">
       <c r="A521" s="2" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TT04</t>
         </is>
       </c>
     </row>
     <row r="522">
       <c r="A522" s="2" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT05</t>
         </is>
       </c>
     </row>
     <row r="523">
       <c r="A523" s="2" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT08</t>
         </is>
       </c>
     </row>
     <row r="524">
       <c r="A524" s="2" t="inlineStr">
         <is>
-          <t>TT123</t>
+          <t>TT103</t>
         </is>
       </c>
     </row>
     <row r="525">
       <c r="A525" s="2" t="inlineStr">
         <is>
-          <t>TT126</t>
+          <t>TT104</t>
         </is>
       </c>
     </row>
     <row r="526">
       <c r="A526" s="2" t="inlineStr">
         <is>
-          <t>TT129</t>
+          <t>TT105</t>
         </is>
       </c>
     </row>
     <row r="527">
       <c r="A527" s="2" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT107</t>
         </is>
       </c>
     </row>
     <row r="528">
       <c r="A528" s="2" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT110</t>
         </is>
       </c>
     </row>
     <row r="529">
       <c r="A529" s="2" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT115</t>
         </is>
       </c>
     </row>
     <row r="530">
       <c r="A530" s="2" t="inlineStr">
         <is>
-          <t>VL01</t>
+          <t>TT117</t>
         </is>
       </c>
     </row>
     <row r="531">
       <c r="A531" s="2" t="inlineStr">
         <is>
-          <t>VL03</t>
+          <t>TT123</t>
         </is>
       </c>
     </row>
     <row r="532">
       <c r="A532" s="2" t="inlineStr">
         <is>
-          <t>VL04</t>
+          <t>TT126</t>
         </is>
       </c>
     </row>
     <row r="533">
       <c r="A533" s="2" t="inlineStr">
         <is>
-          <t>VL11</t>
+          <t>TT129</t>
         </is>
       </c>
     </row>
     <row r="534">
       <c r="A534" s="2" t="inlineStr">
         <is>
-          <t>VL13</t>
+          <t>TT130</t>
         </is>
       </c>
     </row>
     <row r="535">
       <c r="A535" s="2" t="inlineStr">
         <is>
-          <t>VL20</t>
+          <t>TT202</t>
         </is>
       </c>
     </row>
     <row r="536">
       <c r="A536" s="2" t="inlineStr">
         <is>
-          <t>VL22</t>
+          <t>TT206</t>
         </is>
       </c>
     </row>
     <row r="537">
       <c r="A537" s="2" t="inlineStr">
         <is>
-          <t>VL27</t>
+          <t>VL01</t>
         </is>
       </c>
     </row>
     <row r="538">
       <c r="A538" s="2" t="inlineStr">
         <is>
-          <t>VL30</t>
+          <t>VL03</t>
         </is>
       </c>
     </row>
     <row r="539">
       <c r="A539" s="2" t="inlineStr">
         <is>
-          <t>VL35</t>
+          <t>VL04</t>
         </is>
       </c>
     </row>
     <row r="540">
       <c r="A540" s="2" t="inlineStr">
         <is>
-          <t>VL36</t>
+          <t>VL11</t>
         </is>
       </c>
     </row>
     <row r="541">
       <c r="A541" s="2" t="inlineStr">
         <is>
-          <t>VL38</t>
+          <t>VL13</t>
         </is>
       </c>
     </row>
     <row r="542">
       <c r="A542" s="2" t="inlineStr">
         <is>
-          <t>VL43</t>
+          <t>VL20</t>
         </is>
       </c>
     </row>
     <row r="543">
       <c r="A543" s="2" t="inlineStr">
         <is>
-          <t>VL47</t>
+          <t>VL22</t>
         </is>
       </c>
     </row>
     <row r="544">
       <c r="A544" s="2" t="inlineStr">
         <is>
-          <t>VL49</t>
+          <t>VL27</t>
         </is>
       </c>
     </row>
     <row r="545">
       <c r="A545" s="2" t="inlineStr">
         <is>
-          <t>VL54</t>
+          <t>VL30</t>
         </is>
       </c>
     </row>
     <row r="546">
       <c r="A546" s="2" t="inlineStr">
         <is>
-          <t>VL57</t>
+          <t>VL35</t>
         </is>
       </c>
     </row>
     <row r="547">
       <c r="A547" s="2" t="inlineStr">
         <is>
-          <t>VL62</t>
+          <t>VL36</t>
         </is>
       </c>
     </row>
     <row r="548">
       <c r="A548" s="2" t="inlineStr">
         <is>
-          <t>VL67</t>
+          <t>VL38</t>
         </is>
       </c>
     </row>
     <row r="549">
       <c r="A549" s="2" t="inlineStr">
         <is>
-          <t>VL68</t>
+          <t>VL43</t>
         </is>
       </c>
     </row>
     <row r="550">
       <c r="A550" s="2" t="inlineStr">
         <is>
-          <t>VL75</t>
+          <t>VL47</t>
         </is>
       </c>
     </row>
     <row r="551">
       <c r="A551" s="2" t="inlineStr">
         <is>
-          <t>VL81</t>
+          <t>VL49</t>
         </is>
       </c>
     </row>
     <row r="552">
       <c r="A552" s="2" t="inlineStr">
         <is>
-          <t>VL86</t>
+          <t>VL54</t>
         </is>
       </c>
     </row>
     <row r="553">
       <c r="A553" s="2" t="inlineStr">
         <is>
-          <t>VL87</t>
+          <t>VL57</t>
         </is>
       </c>
     </row>
     <row r="554">
       <c r="A554" s="2" t="inlineStr">
         <is>
-          <t>VL88</t>
+          <t>VL62</t>
         </is>
       </c>
     </row>
     <row r="555">
       <c r="A555" s="2" t="inlineStr">
         <is>
-          <t>VL90</t>
+          <t>VL67</t>
         </is>
       </c>
     </row>
     <row r="556">
       <c r="A556" s="2" t="inlineStr">
         <is>
-          <t>VL92</t>
+          <t>VL68</t>
         </is>
       </c>
     </row>
     <row r="557">
       <c r="A557" s="2" t="inlineStr">
         <is>
-          <t>VL99</t>
+          <t>VL75</t>
         </is>
       </c>
     </row>
     <row r="558">
       <c r="A558" s="2" t="inlineStr">
         <is>
-          <t>VL100</t>
+          <t>VL81</t>
         </is>
       </c>
     </row>
     <row r="559">
       <c r="A559" s="2" t="inlineStr">
         <is>
-          <t>VL101</t>
+          <t>VL86</t>
         </is>
       </c>
     </row>
     <row r="560">
       <c r="A560" s="2" t="inlineStr">
         <is>
-          <t>VL103</t>
+          <t>VL87</t>
         </is>
       </c>
     </row>
     <row r="561">
       <c r="A561" s="2" t="inlineStr">
         <is>
-          <t>VL106</t>
+          <t>VL88</t>
         </is>
       </c>
     </row>
     <row r="562">
       <c r="A562" s="2" t="inlineStr">
         <is>
-          <t>VL107</t>
+          <t>VL90</t>
         </is>
       </c>
     </row>
     <row r="563">
       <c r="A563" s="2" t="inlineStr">
         <is>
-          <t>VL112</t>
+          <t>VL92</t>
         </is>
       </c>
     </row>
     <row r="564">
       <c r="A564" s="2" t="inlineStr">
         <is>
-          <t>VL114</t>
+          <t>VL99</t>
         </is>
       </c>
     </row>
     <row r="565">
       <c r="A565" s="2" t="inlineStr">
         <is>
-          <t>VL115</t>
+          <t>VL100</t>
         </is>
       </c>
     </row>
     <row r="566">
       <c r="A566" s="2" t="inlineStr">
         <is>
-          <t>VL121</t>
+          <t>VL101</t>
         </is>
       </c>
     </row>
     <row r="567">
       <c r="A567" s="2" t="inlineStr">
         <is>
-          <t>VL122</t>
+          <t>VL103</t>
         </is>
       </c>
     </row>
     <row r="568">
       <c r="A568" s="2" t="inlineStr">
         <is>
-          <t>VL123</t>
+          <t>VL106</t>
         </is>
       </c>
     </row>
     <row r="569">
       <c r="A569" s="2" t="inlineStr">
         <is>
-          <t>VL124</t>
+          <t>VL107</t>
         </is>
       </c>
     </row>
     <row r="570">
       <c r="A570" s="2" t="inlineStr">
         <is>
-          <t>VL125</t>
+          <t>VL112</t>
         </is>
       </c>
     </row>
     <row r="571">
       <c r="A571" s="2" t="inlineStr">
         <is>
-          <t>VL126</t>
+          <t>VL114</t>
         </is>
       </c>
     </row>
     <row r="572">
       <c r="A572" s="2" t="inlineStr">
         <is>
-          <t>VL127</t>
+          <t>VL115</t>
         </is>
       </c>
     </row>
     <row r="573">
       <c r="A573" s="2" t="inlineStr">
         <is>
-          <t>VL129</t>
+          <t>VL121</t>
         </is>
       </c>
     </row>
     <row r="574">
       <c r="A574" s="2" t="inlineStr">
         <is>
-          <t>VL132</t>
+          <t>VL122</t>
         </is>
       </c>
     </row>
     <row r="575">
       <c r="A575" s="2" t="inlineStr">
         <is>
-          <t>VL134</t>
+          <t>VL123</t>
         </is>
       </c>
     </row>
     <row r="576">
       <c r="A576" s="2" t="inlineStr">
         <is>
-          <t>VL137</t>
+          <t>VL124</t>
         </is>
       </c>
     </row>
     <row r="577">
       <c r="A577" s="2" t="inlineStr">
         <is>
-          <t>VL139</t>
+          <t>VL125</t>
         </is>
       </c>
     </row>
     <row r="578">
       <c r="A578" s="2" t="inlineStr">
         <is>
-          <t>VL140</t>
+          <t>VL126</t>
         </is>
       </c>
     </row>
     <row r="579">
       <c r="A579" s="2" t="inlineStr">
         <is>
-          <t>VL354</t>
+          <t>VL127</t>
         </is>
       </c>
     </row>
     <row r="580">
       <c r="A580" s="2" t="inlineStr">
         <is>
-          <t>VLINE8013</t>
+          <t>VL129</t>
         </is>
       </c>
     </row>
     <row r="581">
       <c r="A581" s="2" t="inlineStr">
         <is>
-          <t>VLINE8020</t>
+          <t>VL132</t>
         </is>
       </c>
     </row>
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>VLINE8021</t>
+          <t>VL134</t>
         </is>
       </c>
     </row>
     <row r="583">
       <c r="A583" s="2" t="inlineStr">
         <is>
-          <t>VLINE8023</t>
+          <t>VL137</t>
         </is>
       </c>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>VLINE8025</t>
+          <t>VL139</t>
         </is>
       </c>
     </row>
     <row r="585">
       <c r="A585" s="2" t="inlineStr">
         <is>
-          <t>VLINE8028</t>
+          <t>VL140</t>
         </is>
       </c>
     </row>
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>VLINE8030</t>
+          <t>VL354</t>
         </is>
       </c>
     </row>
     <row r="587">
       <c r="A587" s="2" t="inlineStr">
         <is>
-          <t>VLINE8034</t>
+          <t>VLINE8013</t>
         </is>
       </c>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>VLINE8058</t>
+          <t>VLINE8020</t>
         </is>
       </c>
     </row>
     <row r="589">
       <c r="A589" s="2" t="inlineStr">
         <is>
-          <t>VLINE8059</t>
+          <t>VLINE8021</t>
         </is>
       </c>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>VLINE8061</t>
+          <t>VLINE8023</t>
         </is>
       </c>
     </row>
     <row r="591">
       <c r="A591" s="2" t="inlineStr">
         <is>
-          <t>VLINE8071</t>
+          <t>VLINE8025</t>
         </is>
       </c>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>VLINE8072</t>
+          <t>VLINE8028</t>
         </is>
       </c>
     </row>
     <row r="593">
       <c r="A593" s="2" t="inlineStr">
         <is>
-          <t>VLINE8074</t>
+          <t>VLINE8030</t>
         </is>
       </c>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>VLINE8075</t>
+          <t>VLINE8034</t>
         </is>
       </c>
     </row>
     <row r="595">
       <c r="A595" s="2" t="inlineStr">
         <is>
-          <t>VLINE8080</t>
+          <t>VLINE8036</t>
         </is>
       </c>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>VLINE8081</t>
+          <t>VLINE8058</t>
         </is>
       </c>
     </row>
     <row r="597">
       <c r="A597" s="2" t="inlineStr">
         <is>
-          <t>VLINE8102</t>
+          <t>VLINE8059</t>
         </is>
       </c>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>VLINE8111</t>
+          <t>VLINE8061</t>
         </is>
       </c>
     </row>
     <row r="599">
       <c r="A599" s="2" t="inlineStr">
         <is>
-          <t>VLINE8113</t>
+          <t>VLINE8071</t>
         </is>
       </c>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>VLINE8115</t>
+          <t>VLINE8072</t>
         </is>
       </c>
     </row>
     <row r="601">
       <c r="A601" s="2" t="inlineStr">
         <is>
-          <t>VLINE8117</t>
+          <t>VLINE8074</t>
         </is>
       </c>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>VLINE8120</t>
+          <t>VLINE8075</t>
         </is>
       </c>
     </row>
     <row r="603">
       <c r="A603" s="2" t="inlineStr">
         <is>
-          <t>VLINE8121</t>
+          <t>VLINE8077</t>
         </is>
       </c>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>VLINE8122</t>
+          <t>VLINE8080</t>
         </is>
       </c>
     </row>
     <row r="605">
       <c r="A605" s="2" t="inlineStr">
         <is>
-          <t>VLINE8123</t>
+          <t>VLINE8081</t>
         </is>
       </c>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>VLINE8124</t>
+          <t>VLINE8084</t>
         </is>
       </c>
     </row>
     <row r="607">
       <c r="A607" s="2" t="inlineStr">
         <is>
-          <t>VLINE8125</t>
+          <t>VLINE8102</t>
         </is>
       </c>
     </row>
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>VLINE8126</t>
+          <t>VLINE8111</t>
         </is>
       </c>
     </row>
     <row r="609">
       <c r="A609" s="2" t="inlineStr">
         <is>
-          <t>VLINE8127</t>
+          <t>VLINE8113</t>
         </is>
       </c>
     </row>
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>VLINE8128</t>
+          <t>VLINE8115</t>
         </is>
       </c>
     </row>
     <row r="611">
       <c r="A611" s="2" t="inlineStr">
         <is>
-          <t>VLINE8130</t>
+          <t>VLINE8117</t>
         </is>
       </c>
     </row>
     <row r="612">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>VLINE8134</t>
+          <t>VLINE8120</t>
         </is>
       </c>
     </row>
     <row r="613">
       <c r="A613" s="2" t="inlineStr">
         <is>
-          <t>VLINE8136</t>
+          <t>VLINE8121</t>
         </is>
       </c>
     </row>
     <row r="614">
       <c r="A614" s="2" t="inlineStr">
         <is>
-          <t>VLINE8161</t>
+          <t>VLINE8122</t>
         </is>
       </c>
     </row>
     <row r="615">
       <c r="A615" s="2" t="inlineStr">
         <is>
-          <t>VLINE8163</t>
+          <t>VLINE8123</t>
         </is>
       </c>
     </row>
     <row r="616">
       <c r="A616" s="2" t="inlineStr">
         <is>
-          <t>VLINE8164</t>
+          <t>VLINE8124</t>
         </is>
       </c>
     </row>
     <row r="617">
       <c r="A617" s="2" t="inlineStr">
         <is>
-          <t>VLINE8172</t>
+          <t>VLINE8125</t>
         </is>
       </c>
     </row>
     <row r="618">
       <c r="A618" s="2" t="inlineStr">
         <is>
-          <t>VLINE8181</t>
+          <t>VLINE8126</t>
         </is>
       </c>
     </row>
     <row r="619">
       <c r="A619" s="2" t="inlineStr">
         <is>
-          <t>VLINE8183</t>
+          <t>VLINE8127</t>
         </is>
       </c>
     </row>
     <row r="620">
       <c r="A620" s="2" t="inlineStr">
         <is>
-          <t>VLINE8184</t>
+          <t>VLINE8128</t>
         </is>
       </c>
     </row>
     <row r="621">
       <c r="A621" s="2" t="inlineStr">
         <is>
-          <t>VLINE8185</t>
+          <t>VLINE8130</t>
         </is>
       </c>
     </row>
     <row r="622">
       <c r="A622" s="2" t="inlineStr">
         <is>
-          <t>VLINE8211</t>
+          <t>VLINE8134</t>
         </is>
       </c>
     </row>
     <row r="623">
       <c r="A623" s="2" t="inlineStr">
         <is>
-          <t>VLINE8213</t>
+          <t>VLINE8136</t>
         </is>
       </c>
     </row>
     <row r="624">
       <c r="A624" s="2" t="inlineStr">
         <is>
-          <t>VLINE8215</t>
+          <t>VLINE8138</t>
         </is>
       </c>
     </row>
     <row r="625">
       <c r="A625" s="2" t="inlineStr">
         <is>
-          <t>VLINE8217</t>
+          <t>VLINE8161</t>
         </is>
       </c>
     </row>
     <row r="626">
       <c r="A626" s="2" t="inlineStr">
         <is>
-          <t>VLINE8219</t>
+          <t>VLINE8163</t>
         </is>
       </c>
     </row>
     <row r="627">
       <c r="A627" s="2" t="inlineStr">
         <is>
-          <t>VLINE8221</t>
+          <t>VLINE8164</t>
         </is>
       </c>
     </row>
     <row r="628">
       <c r="A628" s="2" t="inlineStr">
         <is>
-          <t>VLINE8223</t>
+          <t>VLINE8172</t>
         </is>
       </c>
     </row>
     <row r="629">
       <c r="A629" s="2" t="inlineStr">
         <is>
-          <t>VLINE8225</t>
+          <t>VLINE8181</t>
         </is>
       </c>
     </row>
     <row r="630">
       <c r="A630" s="2" t="inlineStr">
         <is>
-          <t>VLINE8226</t>
+          <t>VLINE8183</t>
         </is>
       </c>
     </row>
     <row r="631">
       <c r="A631" s="2" t="inlineStr">
         <is>
-          <t>VLINE8227</t>
+          <t>VLINE8184</t>
         </is>
       </c>
     </row>
     <row r="632">
       <c r="A632" s="2" t="inlineStr">
         <is>
-          <t>VLINE8228</t>
+          <t>VLINE8185</t>
         </is>
       </c>
     </row>
     <row r="633">
       <c r="A633" s="2" t="inlineStr">
         <is>
-          <t>VLINE8230</t>
+          <t>VLINE8186</t>
         </is>
       </c>
     </row>
     <row r="634">
       <c r="A634" s="2" t="inlineStr">
         <is>
-          <t>VLINE8232</t>
+          <t>VLINE8211</t>
         </is>
       </c>
     </row>
     <row r="635">
       <c r="A635" s="2" t="inlineStr">
         <is>
-          <t>VLINE8234</t>
+          <t>VLINE8213</t>
         </is>
       </c>
     </row>
     <row r="636">
       <c r="A636" s="2" t="inlineStr">
         <is>
-          <t>VLINE8236</t>
+          <t>VLINE8215</t>
         </is>
       </c>
     </row>
     <row r="637">
       <c r="A637" s="2" t="inlineStr">
         <is>
-          <t>VLINE8238</t>
+          <t>VLINE8217</t>
         </is>
       </c>
     </row>
     <row r="638">
       <c r="A638" s="2" t="inlineStr">
         <is>
-          <t>VLINE8240</t>
+          <t>VLINE8219</t>
         </is>
       </c>
     </row>
     <row r="639">
       <c r="A639" s="2" t="inlineStr">
         <is>
-          <t>VLINE8242</t>
+          <t>VLINE8221</t>
         </is>
       </c>
     </row>
     <row r="640">
       <c r="A640" s="2" t="inlineStr">
         <is>
-          <t>VLINE8400</t>
+          <t>VLINE8223</t>
         </is>
       </c>
     </row>
     <row r="641">
       <c r="A641" s="2" t="inlineStr">
         <is>
-          <t>VLINE8405</t>
+          <t>VLINE8225</t>
         </is>
       </c>
     </row>
     <row r="642">
       <c r="A642" s="2" t="inlineStr">
         <is>
-          <t>VLINE8408</t>
+          <t>VLINE8226</t>
         </is>
       </c>
     </row>
     <row r="643">
       <c r="A643" s="2" t="inlineStr">
         <is>
-          <t>VLINE8413</t>
+          <t>VLINE8227</t>
         </is>
       </c>
     </row>
     <row r="644">
       <c r="A644" s="2" t="inlineStr">
         <is>
-          <t>VLINE8415</t>
+          <t>VLINE8228</t>
         </is>
       </c>
     </row>
     <row r="645">
       <c r="A645" s="2" t="inlineStr">
         <is>
-          <t>VLINE8417</t>
+          <t>VLINE8229</t>
         </is>
       </c>
     </row>
     <row r="646">
       <c r="A646" s="2" t="inlineStr">
         <is>
-          <t>VLINE8418</t>
+          <t>VLINE8230</t>
         </is>
       </c>
     </row>
     <row r="647">
       <c r="A647" s="2" t="inlineStr">
         <is>
-          <t>VLINE8419</t>
+          <t>VLINE8232</t>
         </is>
       </c>
     </row>
     <row r="648">
       <c r="A648" s="2" t="inlineStr">
         <is>
-          <t>VLINE8420</t>
+          <t>VLINE8234</t>
         </is>
       </c>
     </row>
     <row r="649">
       <c r="A649" s="2" t="inlineStr">
         <is>
-          <t>VLINE8421</t>
+          <t>VLINE8236</t>
         </is>
       </c>
     </row>
     <row r="650">
       <c r="A650" s="2" t="inlineStr">
         <is>
-          <t>VLINE8422</t>
+          <t>VLINE8238</t>
         </is>
       </c>
     </row>
     <row r="651">
       <c r="A651" s="2" t="inlineStr">
         <is>
-          <t>VLINE8423</t>
+          <t>VLINE8240</t>
         </is>
       </c>
     </row>
     <row r="652">
       <c r="A652" s="2" t="inlineStr">
         <is>
-          <t>VLINE8424</t>
+          <t>VLINE8242</t>
         </is>
       </c>
     </row>
     <row r="653">
       <c r="A653" s="2" t="inlineStr">
         <is>
-          <t>VLINE8427</t>
+          <t>VLINE8400</t>
         </is>
       </c>
     </row>
     <row r="654">
       <c r="A654" s="2" t="inlineStr">
         <is>
-          <t>VLINE8428</t>
+          <t>VLINE8405</t>
         </is>
       </c>
     </row>
     <row r="655">
       <c r="A655" s="2" t="inlineStr">
         <is>
-          <t>VLINE8429</t>
+          <t>VLINE8408</t>
         </is>
       </c>
     </row>
     <row r="656">
       <c r="A656" s="2" t="inlineStr">
         <is>
-          <t>VLINE8430</t>
+          <t>VLINE8413</t>
         </is>
       </c>
     </row>
     <row r="657">
       <c r="A657" s="2" t="inlineStr">
         <is>
-          <t>VLINE8457</t>
+          <t>VLINE8415</t>
         </is>
       </c>
     </row>
     <row r="658">
       <c r="A658" s="2" t="inlineStr">
         <is>
-          <t>VLINE8459</t>
+          <t>VLINE8417</t>
         </is>
       </c>
     </row>
     <row r="659">
       <c r="A659" s="2" t="inlineStr">
         <is>
-          <t>VLINE8460</t>
+          <t>VLINE8418</t>
         </is>
       </c>
     </row>
     <row r="660">
       <c r="A660" s="2" t="inlineStr">
         <is>
-          <t>VLINE8461</t>
+          <t>VLINE8419</t>
         </is>
       </c>
     </row>
     <row r="661">
       <c r="A661" s="2" t="inlineStr">
         <is>
-          <t>VLINE8464</t>
+          <t>VLINE8420</t>
         </is>
       </c>
     </row>
     <row r="662">
       <c r="A662" s="2" t="inlineStr">
         <is>
-          <t>VLINE8465</t>
+          <t>VLINE8421</t>
         </is>
       </c>
     </row>
     <row r="663">
       <c r="A663" s="2" t="inlineStr">
         <is>
-          <t>VLINE8702</t>
+          <t>VLINE8422</t>
         </is>
       </c>
     </row>
     <row r="664">
       <c r="A664" s="2" t="inlineStr">
         <is>
-          <t>VLINE8725</t>
+          <t>VLINE8423</t>
         </is>
       </c>
     </row>
     <row r="665">
       <c r="A665" s="2" t="inlineStr">
         <is>
-          <t>VLINE8727</t>
+          <t>VLINE8424</t>
         </is>
       </c>
     </row>
     <row r="666">
       <c r="A666" s="2" t="inlineStr">
         <is>
-          <t>VLINE8729</t>
+          <t>VLINE8427</t>
         </is>
       </c>
     </row>
     <row r="667">
       <c r="A667" s="2" t="inlineStr">
         <is>
-          <t>VLINE8731</t>
+          <t>VLINE8428</t>
         </is>
       </c>
     </row>
     <row r="668">
       <c r="A668" s="2" t="inlineStr">
         <is>
-          <t>VLINE8733</t>
+          <t>VLINE8429</t>
         </is>
       </c>
     </row>
     <row r="669">
       <c r="A669" s="2" t="inlineStr">
         <is>
-          <t>VLINE8735</t>
+          <t>VLINE8430</t>
         </is>
       </c>
     </row>
     <row r="670">
       <c r="A670" s="2" t="inlineStr">
         <is>
-          <t>VLINE8737</t>
+          <t>VLINE8431</t>
         </is>
       </c>
     </row>
     <row r="671">
       <c r="A671" s="2" t="inlineStr">
         <is>
-          <t>VLINE8739</t>
+          <t>VLINE8432</t>
         </is>
       </c>
     </row>
     <row r="672">
       <c r="A672" s="2" t="inlineStr">
         <is>
-          <t>VLINE8741</t>
+          <t>VLINE8434</t>
         </is>
       </c>
     </row>
     <row r="673">
       <c r="A673" s="2" t="inlineStr">
         <is>
-          <t>VLINE8742</t>
+          <t>VLINE8438</t>
         </is>
       </c>
     </row>
     <row r="674">
       <c r="A674" s="2" t="inlineStr">
         <is>
-          <t>VLINE8743</t>
+          <t>VLINE8457</t>
         </is>
       </c>
     </row>
     <row r="675">
       <c r="A675" s="2" t="inlineStr">
         <is>
-          <t>VLINE8744</t>
+          <t>VLINE8459</t>
         </is>
       </c>
     </row>
     <row r="676">
       <c r="A676" s="2" t="inlineStr">
         <is>
-          <t>VLINE8745</t>
+          <t>VLINE8460</t>
         </is>
       </c>
     </row>
     <row r="677">
       <c r="A677" s="2" t="inlineStr">
         <is>
-          <t>VLINE8746</t>
+          <t>VLINE8461</t>
         </is>
       </c>
     </row>
     <row r="678">
       <c r="A678" s="2" t="inlineStr">
         <is>
-          <t>VLINE8747</t>
+          <t>VLINE8464</t>
         </is>
       </c>
     </row>
     <row r="679">
       <c r="A679" s="2" t="inlineStr">
         <is>
-          <t>VLINE8748</t>
+          <t>VLINE8465</t>
         </is>
       </c>
     </row>
     <row r="680">
       <c r="A680" s="2" t="inlineStr">
         <is>
-          <t>VLINE8749</t>
+          <t>VLINE8702</t>
         </is>
       </c>
     </row>
     <row r="681">
       <c r="A681" s="2" t="inlineStr">
         <is>
-          <t>VLINE8750</t>
+          <t>VLINE8725</t>
         </is>
       </c>
     </row>
     <row r="682">
       <c r="A682" s="2" t="inlineStr">
         <is>
-          <t>VLINE8751</t>
+          <t>VLINE8727</t>
         </is>
       </c>
     </row>
     <row r="683">
       <c r="A683" s="2" t="inlineStr">
         <is>
-          <t>VLINE8752</t>
+          <t>VLINE8729</t>
         </is>
       </c>
     </row>
     <row r="684">
       <c r="A684" s="2" t="inlineStr">
         <is>
-          <t>VLINE8753</t>
+          <t>VLINE8731</t>
         </is>
       </c>
     </row>
     <row r="685">
       <c r="A685" s="2" t="inlineStr">
         <is>
-          <t>VLINE8754</t>
+          <t>VLINE8733</t>
         </is>
       </c>
     </row>
     <row r="686">
       <c r="A686" s="2" t="inlineStr">
         <is>
-          <t>VLINE8755</t>
+          <t>VLINE8735</t>
         </is>
       </c>
     </row>
     <row r="687">
       <c r="A687" s="2" t="inlineStr">
         <is>
-          <t>VLINE8756</t>
+          <t>VLINE8737</t>
         </is>
       </c>
     </row>
     <row r="688">
       <c r="A688" s="2" t="inlineStr">
         <is>
-          <t>VLINE8757</t>
+          <t>VLINE8739</t>
         </is>
       </c>
     </row>
     <row r="689">
       <c r="A689" s="2" t="inlineStr">
         <is>
-          <t>VLINE8758</t>
+          <t>VLINE8741</t>
         </is>
       </c>
     </row>
     <row r="690">
       <c r="A690" s="2" t="inlineStr">
         <is>
-          <t>VLINE8759</t>
+          <t>VLINE8742</t>
         </is>
       </c>
     </row>
     <row r="691">
       <c r="A691" s="2" t="inlineStr">
         <is>
-          <t>VLINE8760</t>
+          <t>VLINE8743</t>
         </is>
       </c>
     </row>
     <row r="692">
       <c r="A692" s="2" t="inlineStr">
         <is>
-          <t>VLINE8762</t>
+          <t>VLINE8744</t>
         </is>
       </c>
     </row>
     <row r="693">
       <c r="A693" s="2" t="inlineStr">
         <is>
-          <t>VLINE8764</t>
+          <t>VLINE8745</t>
         </is>
       </c>
     </row>
     <row r="694">
       <c r="A694" s="2" t="inlineStr">
         <is>
-          <t>VLINE8766</t>
+          <t>VLINE8746</t>
         </is>
       </c>
     </row>
     <row r="695">
       <c r="A695" s="2" t="inlineStr">
         <is>
-          <t>VLINE8768</t>
+          <t>VLINE8747</t>
         </is>
       </c>
     </row>
     <row r="696">
       <c r="A696" s="2" t="inlineStr">
         <is>
-          <t>VLINE8770</t>
+          <t>VLINE8748</t>
         </is>
       </c>
     </row>
     <row r="697">
       <c r="A697" s="2" t="inlineStr">
         <is>
-          <t>VLINE8772</t>
+          <t>VLINE8749</t>
         </is>
       </c>
     </row>
     <row r="698">
       <c r="A698" s="2" t="inlineStr">
         <is>
-          <t>VLINE8774</t>
+          <t>VLINE8750</t>
         </is>
       </c>
     </row>
     <row r="699">
       <c r="A699" s="2" t="inlineStr">
         <is>
-          <t>VLINE8819</t>
+          <t>VLINE8751</t>
         </is>
       </c>
     </row>
     <row r="700">
       <c r="A700" s="2" t="inlineStr">
         <is>
-          <t>VLINE8862</t>
+          <t>VLINE8752</t>
         </is>
       </c>
     </row>
     <row r="701">
       <c r="A701" s="2" t="inlineStr">
         <is>
-          <t>VLINE8863</t>
+          <t>VLINE8753</t>
         </is>
       </c>
     </row>
     <row r="702">
       <c r="A702" s="2" t="inlineStr">
         <is>
-          <t>VLINE8865</t>
+          <t>VLINE8754</t>
         </is>
       </c>
     </row>
     <row r="703">
       <c r="A703" s="2" t="inlineStr">
         <is>
-          <t>VR76</t>
+          <t>VLINE8755</t>
         </is>
       </c>
     </row>
     <row r="704">
       <c r="A704" s="2" t="inlineStr">
         <is>
-          <t>VR77</t>
+          <t>VLINE8756</t>
         </is>
       </c>
     </row>
     <row r="705">
       <c r="A705" s="2" t="inlineStr">
         <is>
-          <t>WOLL408</t>
+          <t>VLINE8757</t>
         </is>
       </c>
     </row>
     <row r="706">
       <c r="A706" s="2" t="inlineStr">
         <is>
-          <t>WOLL430</t>
+          <t>VLINE8758</t>
         </is>
       </c>
     </row>
     <row r="707">
       <c r="A707" s="2" t="inlineStr">
         <is>
-          <t>XP2001</t>
+          <t>VLINE8759</t>
         </is>
       </c>
     </row>
     <row r="708">
       <c r="A708" s="2" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>VLINE8760</t>
         </is>
       </c>
     </row>
     <row r="709">
       <c r="A709" s="2" t="inlineStr">
         <is>
-          <t>XP2006</t>
+          <t>VLINE8761</t>
         </is>
       </c>
     </row>
     <row r="710">
       <c r="A710" s="2" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>VLINE8762</t>
         </is>
       </c>
     </row>
     <row r="711">
       <c r="A711" s="2" t="inlineStr">
         <is>
-          <t>XP2009</t>
+          <t>VLINE8764</t>
         </is>
       </c>
     </row>
     <row r="712">
       <c r="A712" s="2" t="inlineStr">
         <is>
-          <t>XP2010</t>
+          <t>VLINE8766</t>
         </is>
       </c>
     </row>
     <row r="713">
       <c r="A713" s="2" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>VLINE8768</t>
         </is>
       </c>
     </row>
     <row r="714">
       <c r="A714" s="2" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>VLINE8770</t>
         </is>
       </c>
     </row>
     <row r="715">
       <c r="A715" s="2" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>VLINE8772</t>
         </is>
       </c>
     </row>
     <row r="716">
       <c r="A716" s="2" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>VLINE8774</t>
         </is>
       </c>
     </row>
     <row r="717">
       <c r="A717" s="2" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>VLINE8776</t>
         </is>
       </c>
     </row>
     <row r="718">
       <c r="A718" s="2" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>VLINE8778</t>
         </is>
       </c>
     </row>
     <row r="719">
       <c r="A719" s="2" t="inlineStr">
         <is>
-          <t>XRN003</t>
+          <t>VLINE8780</t>
         </is>
       </c>
     </row>
     <row r="720">
       <c r="A720" s="2" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>VLINE8819</t>
         </is>
       </c>
     </row>
     <row r="721">
       <c r="A721" s="2" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>VLINE8862</t>
         </is>
       </c>
     </row>
     <row r="722">
       <c r="A722" s="2" t="inlineStr">
         <is>
-          <t>XRN010</t>
+          <t>VLINE8863</t>
         </is>
       </c>
     </row>
     <row r="723">
       <c r="A723" s="2" t="inlineStr">
         <is>
-          <t>XRN012</t>
+          <t>VLINE8864</t>
         </is>
       </c>
     </row>
     <row r="724">
       <c r="A724" s="2" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>VLINE8865</t>
         </is>
       </c>
     </row>
     <row r="725">
       <c r="A725" s="2" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>VR76</t>
         </is>
       </c>
     </row>
     <row r="726">
       <c r="A726" s="2" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>VR77</t>
         </is>
       </c>
     </row>
     <row r="727">
       <c r="A727" s="2" t="inlineStr">
         <is>
-          <t>XRN022</t>
+          <t>WOLL408</t>
         </is>
       </c>
     </row>
     <row r="728">
       <c r="A728" s="2" t="inlineStr">
         <is>
-          <t>XRN028</t>
+          <t>WOLL430</t>
         </is>
       </c>
     </row>
     <row r="729">
       <c r="A729" s="2" t="inlineStr">
+        <is>
+          <t>XP2001</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="2" t="inlineStr">
+        <is>
+          <t>XP2005</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="2" t="inlineStr">
+        <is>
+          <t>XP2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" s="2" t="inlineStr">
+        <is>
+          <t>XP2008</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" s="2" t="inlineStr">
+        <is>
+          <t>XP2009</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="2" t="inlineStr">
+        <is>
+          <t>XP2010</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" s="2" t="inlineStr">
+        <is>
+          <t>XP2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="2" t="inlineStr">
+        <is>
+          <t>XP2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="2" t="inlineStr">
+        <is>
+          <t>XP2013</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="2" t="inlineStr">
+        <is>
+          <t>XP2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" s="2" t="inlineStr">
+        <is>
+          <t>XP2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" s="2" t="inlineStr">
+        <is>
+          <t>XP2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="2" t="inlineStr">
+        <is>
+          <t>XRN003</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="2" t="inlineStr">
+        <is>
+          <t>XRN005</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="2" t="inlineStr">
+        <is>
+          <t>XRN009</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" s="2" t="inlineStr">
+        <is>
+          <t>XRN010</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" s="2" t="inlineStr">
+        <is>
+          <t>XRN012</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" s="2" t="inlineStr">
+        <is>
+          <t>XRN017</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" s="2" t="inlineStr">
+        <is>
+          <t>XRN018</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" s="2" t="inlineStr">
+        <is>
+          <t>XRN021</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" s="2" t="inlineStr">
+        <is>
+          <t>XRN022</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="2" t="inlineStr">
+        <is>
+          <t>XRN028</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="2" t="inlineStr">
         <is>
           <t>XRN029</t>
         </is>

</xml_diff>

<commit_message>
Update RailOps database files - 2026-04-30 05:31:53 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A751"/>
+  <dimension ref="A1:A770"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2099,3610 +2099,3743 @@
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>MM48M</t>
+          <t>MM46M</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>MM50M</t>
+          <t>MM48M</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>MM52M</t>
+          <t>MM50M</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>MM64M</t>
+          <t>MM52M</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>MM76M</t>
+          <t>MM54M</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>MM78M</t>
+          <t>MM60M</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>MM80M</t>
+          <t>MM64M</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>MM82M</t>
+          <t>MM76M</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>MM84M</t>
+          <t>MM78M</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>MM86M</t>
+          <t>MM80M</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>MM92M</t>
+          <t>MM82M</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>MM94M</t>
+          <t>MM84M</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>MM96M</t>
+          <t>MM86M</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>MM98M</t>
+          <t>MM92M</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>MM99M</t>
+          <t>MM94M</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>MM122M</t>
+          <t>MM96M</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>MM130M</t>
+          <t>MM98M</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>MM152M</t>
+          <t>MM99M</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>MM156M</t>
+          <t>MM122M</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>MM158M</t>
+          <t>MM130M</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>MM172M</t>
+          <t>MM152M</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>MM178M</t>
+          <t>MM156M</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>MM192M</t>
+          <t>MM158M</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>MM212M</t>
+          <t>MM172M</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>MM214M</t>
+          <t>MM178M</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>MM216M</t>
+          <t>MM192M</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>MM232M</t>
+          <t>MM212M</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>MM236M</t>
+          <t>MM214M</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>MM240M</t>
+          <t>MM216M</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>MM246M</t>
+          <t>MM224M</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>MM256M</t>
+          <t>MM232M</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>MM260M</t>
+          <t>MM236M</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>MM264M</t>
+          <t>MM240M</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>MM266M</t>
+          <t>MM246M</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>MM268M</t>
+          <t>MM256M</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>MM270M</t>
+          <t>MM258M</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>MM280M</t>
+          <t>MM260M</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>MM288M</t>
+          <t>MM264M</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>MM380M</t>
+          <t>MM266M</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>MM418M</t>
+          <t>MM268M</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>MM456M</t>
+          <t>MM270M</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>MM464M</t>
+          <t>MM280M</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>MM478M</t>
+          <t>MM288M</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>MM482M</t>
+          <t>MM380M</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>MM486M</t>
+          <t>MM418M</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>MM502M</t>
+          <t>MM424M</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>MM506M</t>
+          <t>MM456M</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>MM514M</t>
+          <t>MM464M</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>MM522M</t>
+          <t>MM478M</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>MM536M</t>
+          <t>MM482M</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>MM542M</t>
+          <t>MM486M</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>MM544M</t>
+          <t>MM502M</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>MM546M</t>
+          <t>MM506M</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>MM551M</t>
+          <t>MM514M</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>MM566M</t>
+          <t>MM522M</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>MM574M</t>
+          <t>MM536M</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>MM588M</t>
+          <t>MM542M</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>MM592M</t>
+          <t>MM544M</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>MM602M</t>
+          <t>MM546M</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>MM604M</t>
+          <t>MM551M</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>MM624M</t>
+          <t>MM552M</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>MM636M</t>
+          <t>MM566M</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>MM638M</t>
+          <t>MM574M</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>MM647M</t>
+          <t>MM588M</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>MM656M</t>
+          <t>MM592M</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>MM658M</t>
+          <t>MM602M</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>MM660M</t>
+          <t>MM604M</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>MM662M</t>
+          <t>MM620M</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>MM664M</t>
+          <t>MM624M</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>MM668M</t>
+          <t>MM636M</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>MM673M</t>
+          <t>MM638M</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>MM674M</t>
+          <t>MM647M</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>MM676M</t>
+          <t>MM656M</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>MM680M</t>
+          <t>MM658M</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>MM702M</t>
+          <t>MM660M</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>MM708M</t>
+          <t>MM662M</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>MM718M</t>
+          <t>MM664M</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>MM742M</t>
+          <t>MM668M</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>MM744M</t>
+          <t>MM673M</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>MM752M</t>
+          <t>MM674M</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>MM756M</t>
+          <t>MM676M</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>MM768M</t>
+          <t>MM680M</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>MM772M</t>
+          <t>MM702M</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>MM774M</t>
+          <t>MM708M</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>MM776M</t>
+          <t>MM718M</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>MM778M</t>
+          <t>MM742M</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>MM780M</t>
+          <t>MM744M</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>MM784M</t>
+          <t>MM752M</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>MM788M</t>
+          <t>MM756M</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>MM790M</t>
+          <t>MM766M</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>MM794M</t>
+          <t>MM768M</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>MM798M</t>
+          <t>MM772M</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>MM800M</t>
+          <t>MM774M</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>MM802M</t>
+          <t>MM776M</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>MM806M</t>
+          <t>MM778M</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>MM808M</t>
+          <t>MM780M</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>MM810M</t>
+          <t>MM784M</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>MM816M</t>
+          <t>MM788M</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>MM826M</t>
+          <t>MM790M</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>MM830M</t>
+          <t>MM794M</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>MM832M</t>
+          <t>MM798M</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>MM834M</t>
+          <t>MM800M</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>MM836M</t>
+          <t>MM802M</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>MM838M</t>
+          <t>MM806M</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>MM842M</t>
+          <t>MM808M</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>MM858M</t>
+          <t>MM810M</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>MM860M</t>
+          <t>MM816M</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>MM862M</t>
+          <t>MM826M</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>MM864M</t>
+          <t>MM830M</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>MM866M</t>
+          <t>MM832M</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>MM872M</t>
+          <t>MM834M</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>MM878M</t>
+          <t>MM836M</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>MM880M</t>
+          <t>MM838M</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>MM886M</t>
+          <t>MM842M</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>MM896M</t>
+          <t>MM858M</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>MM908M</t>
+          <t>MM860M</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>MM910M</t>
+          <t>MM862M</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>MM912M</t>
+          <t>MM864M</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>MM914M</t>
+          <t>MM866M</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>MM924M</t>
+          <t>MM872M</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>MM928M</t>
+          <t>MM878M</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>MM934M</t>
+          <t>MM880M</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>MM940M</t>
+          <t>MM886M</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>MM944M</t>
+          <t>MM896M</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>MM946M</t>
+          <t>MM908M</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>MM952M</t>
+          <t>MM910M</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>MM956M</t>
+          <t>MM912M</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>MM958M</t>
+          <t>MM914M</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>MM960M</t>
+          <t>MM922M</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>MM962M</t>
+          <t>MM924M</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>MM964M</t>
+          <t>MM928M</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>MM968M</t>
+          <t>MM934M</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>MM970M</t>
+          <t>MM940M</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>MM972M</t>
+          <t>MM944M</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>MM974M</t>
+          <t>MM946M</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>MM976M</t>
+          <t>MM952M</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>MM980M</t>
+          <t>MM956M</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t>MM982M</t>
+          <t>MM958M</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>MM9901M</t>
+          <t>MM960M</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t>MM9903M</t>
+          <t>MM962M</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>MM9904M</t>
+          <t>MM964M</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>MM9906M</t>
+          <t>MM968M</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>MM9908M</t>
+          <t>MM970M</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>MM9909M</t>
+          <t>MM972M</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>MM9910M</t>
+          <t>MM974M</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>MM9912M</t>
+          <t>MM976M</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>MM9914M</t>
+          <t>MM980M</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
         <is>
-          <t>MM9916M</t>
+          <t>MM982M</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>MM9918M</t>
+          <t>MM9901M</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
         <is>
-          <t>MM9920M</t>
+          <t>MM9903M</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
         <is>
-          <t>MM9921M</t>
+          <t>MM9904M</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" s="2" t="inlineStr">
         <is>
-          <t>MM9924M</t>
+          <t>MM9905M</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
         <is>
-          <t>MM9926M</t>
+          <t>MM9906M</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
         <is>
-          <t>MM9927M</t>
+          <t>MM9908M</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>MM9928M</t>
+          <t>MM9909M</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
         <is>
-          <t>MM9929M</t>
+          <t>MM9910M</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
         <is>
-          <t>MM9931M</t>
+          <t>MM9912M</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="2" t="inlineStr">
         <is>
-          <t>MM9933M</t>
+          <t>MM9914M</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
         <is>
-          <t>MM9936M</t>
+          <t>MM9916M</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" s="2" t="inlineStr">
         <is>
-          <t>MM9937M</t>
+          <t>MM9918M</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
         <is>
-          <t>MM9938M</t>
+          <t>MM9920M</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="2" t="inlineStr">
         <is>
-          <t>MM9941M</t>
+          <t>MM9921M</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" s="2" t="inlineStr">
         <is>
-          <t>MM9943M</t>
+          <t>MM9924M</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="2" t="inlineStr">
         <is>
-          <t>MM9946M</t>
+          <t>MM9926M</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
         <is>
-          <t>MM9947M</t>
+          <t>MM9927M</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" s="2" t="inlineStr">
         <is>
-          <t>MM9948M</t>
+          <t>MM9928M</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
         <is>
-          <t>MM9952M</t>
+          <t>MM9929M</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" s="2" t="inlineStr">
         <is>
-          <t>MM9953M</t>
+          <t>MM9931M</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" s="2" t="inlineStr">
         <is>
-          <t>MM9954M</t>
+          <t>MM9933M</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
         <is>
-          <t>MM9956M</t>
+          <t>MM9936M</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="2" t="inlineStr">
         <is>
-          <t>MM9957M</t>
+          <t>MM9937M</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
         <is>
-          <t>MM9958M</t>
+          <t>MM9938M</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="2" t="inlineStr">
         <is>
-          <t>MM9959M</t>
+          <t>MM9941M</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="2" t="inlineStr">
         <is>
-          <t>MM9960M</t>
+          <t>MM9943M</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" s="2" t="inlineStr">
         <is>
-          <t>MM9961M</t>
+          <t>MM9946M</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" s="2" t="inlineStr">
         <is>
-          <t>MM9962M</t>
+          <t>MM9947M</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" s="2" t="inlineStr">
         <is>
-          <t>MM9963M</t>
+          <t>MM9948M</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" s="2" t="inlineStr">
         <is>
-          <t>MM9964M</t>
+          <t>MM9952M</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" s="2" t="inlineStr">
         <is>
-          <t>MM9965M</t>
+          <t>MM9953M</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" s="2" t="inlineStr">
         <is>
-          <t>MM9966M</t>
+          <t>MM9954M</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" s="2" t="inlineStr">
         <is>
-          <t>MM9968M</t>
+          <t>MM9956M</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" s="2" t="inlineStr">
         <is>
-          <t>MM9969M</t>
+          <t>MM9957M</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t>MM9970M</t>
+          <t>MM9958M</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" s="2" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MM9959M</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
         <is>
-          <t>MRL002</t>
+          <t>MM9960M</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" s="2" t="inlineStr">
         <is>
-          <t>MTPV1</t>
+          <t>MM9961M</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" s="2" t="inlineStr">
         <is>
-          <t>MTPV2</t>
+          <t>MM9962M</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" s="2" t="inlineStr">
         <is>
-          <t>N453</t>
+          <t>MM9963M</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
         <is>
-          <t>N458</t>
+          <t>MM9964M</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="2" t="inlineStr">
         <is>
-          <t>N460</t>
+          <t>MM9965M</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>MM9966M</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>MM9968M</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>MM9969M</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" s="2" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>MM9970M</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
         <is>
-          <t>NR6</t>
+          <t>MRL001</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" s="2" t="inlineStr">
         <is>
-          <t>NR10</t>
+          <t>MRL002</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
         <is>
-          <t>NR11</t>
+          <t>MTPV1</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" s="2" t="inlineStr">
         <is>
-          <t>NR12</t>
+          <t>MTPV2</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t>NR13</t>
+          <t>N453</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t>NR14</t>
+          <t>N458</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>NR17</t>
+          <t>N460</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
         <is>
-          <t>NR20</t>
+          <t>N466</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
         <is>
-          <t>NR31</t>
+          <t>N469</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
         <is>
-          <t>NR35</t>
+          <t>NR4</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>NR5</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
         <is>
-          <t>NR44</t>
+          <t>NR6</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>NR46</t>
+          <t>NR10</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>NR11</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>NR52</t>
+          <t>NR12</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>NR13</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>NR56</t>
+          <t>NR14</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
         <is>
-          <t>NR60</t>
+          <t>NR17</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR20</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR31</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR35</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR37</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>NR76</t>
+          <t>NR44</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="2" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR46</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR47</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" s="2" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR52</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
         <is>
-          <t>NR88</t>
+          <t>NR54</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" s="2" t="inlineStr">
         <is>
-          <t>NR91</t>
+          <t>NR56</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="2" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR60</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" s="2" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR64</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" s="2" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR65</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" s="2" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>NR68</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" s="2" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR75</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="2" t="inlineStr">
         <is>
-          <t>NR106</t>
+          <t>NR76</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="2" t="inlineStr">
         <is>
-          <t>NR107</t>
+          <t>NR78</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="2" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR82</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="2" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR83</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="2" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR88</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" s="2" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR91</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" s="2" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>NR93</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" s="2" t="inlineStr">
         <is>
-          <t>PB5</t>
+          <t>NR94</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" s="2" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>NR95</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="A472" s="2" t="inlineStr">
         <is>
-          <t>PKLA4</t>
+          <t>NR97</t>
         </is>
       </c>
     </row>
     <row r="473">
       <c r="A473" s="2" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>NR102</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="A474" s="2" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>NR106</t>
         </is>
       </c>
     </row>
     <row r="475">
       <c r="A475" s="2" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>NR107</t>
         </is>
       </c>
     </row>
     <row r="476">
       <c r="A476" s="2" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>NR109</t>
         </is>
       </c>
     </row>
     <row r="477">
       <c r="A477" s="2" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>NR112</t>
         </is>
       </c>
     </row>
     <row r="478">
       <c r="A478" s="2" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>NR113</t>
         </is>
       </c>
     </row>
     <row r="479">
       <c r="A479" s="2" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>NR115</t>
         </is>
       </c>
     </row>
     <row r="480">
       <c r="A480" s="2" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>PB4</t>
         </is>
       </c>
     </row>
     <row r="481">
       <c r="A481" s="2" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>PB5</t>
         </is>
       </c>
     </row>
     <row r="482">
       <c r="A482" s="2" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="2" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>PKLA4</t>
         </is>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="2" t="inlineStr">
         <is>
-          <t>QL009</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="2" t="inlineStr">
         <is>
-          <t>QL016</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="2" t="inlineStr">
         <is>
-          <t>QL019</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="2" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" s="2" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" s="2" t="inlineStr">
         <is>
-          <t>QR5400</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
     <row r="490">
       <c r="A490" s="2" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QE001</t>
         </is>
       </c>
     </row>
     <row r="491">
       <c r="A491" s="2" t="inlineStr">
         <is>
-          <t>RA2302</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
     <row r="492">
       <c r="A492" s="2" t="inlineStr">
         <is>
-          <t>RA2303</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="2" t="inlineStr">
         <is>
-          <t>RB2352</t>
+          <t>QL004</t>
         </is>
       </c>
     </row>
     <row r="494">
       <c r="A494" s="2" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
     <row r="495">
       <c r="A495" s="2" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>QL009</t>
         </is>
       </c>
     </row>
     <row r="496">
       <c r="A496" s="2" t="inlineStr">
         <is>
-          <t>RL309</t>
+          <t>QL016</t>
         </is>
       </c>
     </row>
     <row r="497">
       <c r="A497" s="2" t="inlineStr">
         <is>
-          <t>RM93</t>
+          <t>QL019</t>
         </is>
       </c>
     </row>
     <row r="498">
       <c r="A498" s="2" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>QR1744</t>
         </is>
       </c>
     </row>
     <row r="499">
       <c r="A499" s="2" t="inlineStr">
         <is>
-          <t>SCT008</t>
+          <t>QR1771</t>
         </is>
       </c>
     </row>
     <row r="500">
       <c r="A500" s="2" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>QR5400</t>
         </is>
       </c>
     </row>
     <row r="501">
       <c r="A501" s="2" t="inlineStr">
         <is>
-          <t>SCT010</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
     <row r="502">
       <c r="A502" s="2" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>RA2302</t>
         </is>
       </c>
     </row>
     <row r="503">
       <c r="A503" s="2" t="inlineStr">
         <is>
-          <t>SM636B</t>
+          <t>RA2303</t>
         </is>
       </c>
     </row>
     <row r="504">
       <c r="A504" s="2" t="inlineStr">
         <is>
-          <t>SO3</t>
+          <t>RB2352</t>
         </is>
       </c>
     </row>
     <row r="505">
       <c r="A505" s="2" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
     <row r="506">
       <c r="A506" s="2" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>RL301</t>
         </is>
       </c>
     </row>
     <row r="507">
       <c r="A507" s="2" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>RL309</t>
         </is>
       </c>
     </row>
     <row r="508">
       <c r="A508" s="2" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>RM93</t>
         </is>
       </c>
     </row>
     <row r="509">
       <c r="A509" s="2" t="inlineStr">
         <is>
-          <t>T373</t>
+          <t>SCT001</t>
         </is>
       </c>
     </row>
     <row r="510">
       <c r="A510" s="2" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>SCT008</t>
         </is>
       </c>
     </row>
     <row r="511">
       <c r="A511" s="2" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>SCT009</t>
         </is>
       </c>
     </row>
     <row r="512">
       <c r="A512" s="2" t="inlineStr">
         <is>
-          <t>TE2804</t>
+          <t>SCT010</t>
         </is>
       </c>
     </row>
     <row r="513">
       <c r="A513" s="2" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>SCT013</t>
         </is>
       </c>
     </row>
     <row r="514">
       <c r="A514" s="2" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>SM636B</t>
         </is>
       </c>
     </row>
     <row r="515">
       <c r="A515" s="2" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>SO3</t>
         </is>
       </c>
     </row>
     <row r="516">
       <c r="A516" s="2" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>SSR101</t>
         </is>
       </c>
     </row>
     <row r="517">
       <c r="A517" s="2" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>SSR102</t>
         </is>
       </c>
     </row>
     <row r="518">
       <c r="A518" s="2" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>SSR103</t>
         </is>
       </c>
     </row>
     <row r="519">
       <c r="A519" s="2" t="inlineStr">
         <is>
-          <t>TT02</t>
+          <t>SSR104</t>
         </is>
       </c>
     </row>
     <row r="520">
       <c r="A520" s="2" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>T373</t>
         </is>
       </c>
     </row>
     <row r="521">
       <c r="A521" s="2" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TE2801</t>
         </is>
       </c>
     </row>
     <row r="522">
       <c r="A522" s="2" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TE2803</t>
         </is>
       </c>
     </row>
     <row r="523">
       <c r="A523" s="2" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TE2804</t>
         </is>
       </c>
     </row>
     <row r="524">
       <c r="A524" s="2" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TE2805</t>
         </is>
       </c>
     </row>
     <row r="525">
       <c r="A525" s="2" t="inlineStr">
         <is>
-          <t>TT104</t>
+          <t>TE2807</t>
         </is>
       </c>
     </row>
     <row r="526">
       <c r="A526" s="2" t="inlineStr">
         <is>
-          <t>TT105</t>
+          <t>TE2808</t>
         </is>
       </c>
     </row>
     <row r="527">
       <c r="A527" s="2" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TE2813</t>
         </is>
       </c>
     </row>
     <row r="528">
       <c r="A528" s="2" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TE2814</t>
         </is>
       </c>
     </row>
     <row r="529">
       <c r="A529" s="2" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TJ096</t>
         </is>
       </c>
     </row>
     <row r="530">
       <c r="A530" s="2" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT02</t>
         </is>
       </c>
     </row>
     <row r="531">
       <c r="A531" s="2" t="inlineStr">
         <is>
-          <t>TT123</t>
+          <t>TT03</t>
         </is>
       </c>
     </row>
     <row r="532">
       <c r="A532" s="2" t="inlineStr">
         <is>
-          <t>TT126</t>
+          <t>TT04</t>
         </is>
       </c>
     </row>
     <row r="533">
       <c r="A533" s="2" t="inlineStr">
         <is>
-          <t>TT129</t>
+          <t>TT05</t>
         </is>
       </c>
     </row>
     <row r="534">
       <c r="A534" s="2" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT08</t>
         </is>
       </c>
     </row>
     <row r="535">
       <c r="A535" s="2" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT103</t>
         </is>
       </c>
     </row>
     <row r="536">
       <c r="A536" s="2" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT104</t>
         </is>
       </c>
     </row>
     <row r="537">
       <c r="A537" s="2" t="inlineStr">
         <is>
-          <t>VL01</t>
+          <t>TT105</t>
         </is>
       </c>
     </row>
     <row r="538">
       <c r="A538" s="2" t="inlineStr">
         <is>
-          <t>VL03</t>
+          <t>TT107</t>
         </is>
       </c>
     </row>
     <row r="539">
       <c r="A539" s="2" t="inlineStr">
         <is>
-          <t>VL04</t>
+          <t>TT110</t>
         </is>
       </c>
     </row>
     <row r="540">
       <c r="A540" s="2" t="inlineStr">
         <is>
-          <t>VL11</t>
+          <t>TT115</t>
         </is>
       </c>
     </row>
     <row r="541">
       <c r="A541" s="2" t="inlineStr">
         <is>
-          <t>VL13</t>
+          <t>TT117</t>
         </is>
       </c>
     </row>
     <row r="542">
       <c r="A542" s="2" t="inlineStr">
         <is>
-          <t>VL20</t>
+          <t>TT123</t>
         </is>
       </c>
     </row>
     <row r="543">
       <c r="A543" s="2" t="inlineStr">
         <is>
-          <t>VL22</t>
+          <t>TT126</t>
         </is>
       </c>
     </row>
     <row r="544">
       <c r="A544" s="2" t="inlineStr">
         <is>
-          <t>VL27</t>
+          <t>TT129</t>
         </is>
       </c>
     </row>
     <row r="545">
       <c r="A545" s="2" t="inlineStr">
         <is>
-          <t>VL30</t>
+          <t>TT130</t>
         </is>
       </c>
     </row>
     <row r="546">
       <c r="A546" s="2" t="inlineStr">
         <is>
-          <t>VL35</t>
+          <t>TT202</t>
         </is>
       </c>
     </row>
     <row r="547">
       <c r="A547" s="2" t="inlineStr">
         <is>
-          <t>VL36</t>
+          <t>TT206</t>
         </is>
       </c>
     </row>
     <row r="548">
       <c r="A548" s="2" t="inlineStr">
         <is>
-          <t>VL38</t>
+          <t>VL01</t>
         </is>
       </c>
     </row>
     <row r="549">
       <c r="A549" s="2" t="inlineStr">
         <is>
-          <t>VL43</t>
+          <t>VL03</t>
         </is>
       </c>
     </row>
     <row r="550">
       <c r="A550" s="2" t="inlineStr">
         <is>
-          <t>VL47</t>
+          <t>VL04</t>
         </is>
       </c>
     </row>
     <row r="551">
       <c r="A551" s="2" t="inlineStr">
         <is>
-          <t>VL49</t>
+          <t>VL11</t>
         </is>
       </c>
     </row>
     <row r="552">
       <c r="A552" s="2" t="inlineStr">
         <is>
-          <t>VL54</t>
+          <t>VL13</t>
         </is>
       </c>
     </row>
     <row r="553">
       <c r="A553" s="2" t="inlineStr">
         <is>
-          <t>VL57</t>
+          <t>VL20</t>
         </is>
       </c>
     </row>
     <row r="554">
       <c r="A554" s="2" t="inlineStr">
         <is>
-          <t>VL62</t>
+          <t>VL22</t>
         </is>
       </c>
     </row>
     <row r="555">
       <c r="A555" s="2" t="inlineStr">
         <is>
-          <t>VL67</t>
+          <t>VL27</t>
         </is>
       </c>
     </row>
     <row r="556">
       <c r="A556" s="2" t="inlineStr">
         <is>
-          <t>VL68</t>
+          <t>VL30</t>
         </is>
       </c>
     </row>
     <row r="557">
       <c r="A557" s="2" t="inlineStr">
         <is>
-          <t>VL75</t>
+          <t>VL35</t>
         </is>
       </c>
     </row>
     <row r="558">
       <c r="A558" s="2" t="inlineStr">
         <is>
-          <t>VL81</t>
+          <t>VL36</t>
         </is>
       </c>
     </row>
     <row r="559">
       <c r="A559" s="2" t="inlineStr">
         <is>
-          <t>VL86</t>
+          <t>VL38</t>
         </is>
       </c>
     </row>
     <row r="560">
       <c r="A560" s="2" t="inlineStr">
         <is>
-          <t>VL87</t>
+          <t>VL43</t>
         </is>
       </c>
     </row>
     <row r="561">
       <c r="A561" s="2" t="inlineStr">
         <is>
-          <t>VL88</t>
+          <t>VL47</t>
         </is>
       </c>
     </row>
     <row r="562">
       <c r="A562" s="2" t="inlineStr">
         <is>
-          <t>VL90</t>
+          <t>VL49</t>
         </is>
       </c>
     </row>
     <row r="563">
       <c r="A563" s="2" t="inlineStr">
         <is>
-          <t>VL92</t>
+          <t>VL54</t>
         </is>
       </c>
     </row>
     <row r="564">
       <c r="A564" s="2" t="inlineStr">
         <is>
-          <t>VL99</t>
+          <t>VL57</t>
         </is>
       </c>
     </row>
     <row r="565">
       <c r="A565" s="2" t="inlineStr">
         <is>
-          <t>VL100</t>
+          <t>VL62</t>
         </is>
       </c>
     </row>
     <row r="566">
       <c r="A566" s="2" t="inlineStr">
         <is>
-          <t>VL101</t>
+          <t>VL67</t>
         </is>
       </c>
     </row>
     <row r="567">
       <c r="A567" s="2" t="inlineStr">
         <is>
-          <t>VL103</t>
+          <t>VL68</t>
         </is>
       </c>
     </row>
     <row r="568">
       <c r="A568" s="2" t="inlineStr">
         <is>
-          <t>VL106</t>
+          <t>VL75</t>
         </is>
       </c>
     </row>
     <row r="569">
       <c r="A569" s="2" t="inlineStr">
         <is>
-          <t>VL107</t>
+          <t>VL81</t>
         </is>
       </c>
     </row>
     <row r="570">
       <c r="A570" s="2" t="inlineStr">
         <is>
-          <t>VL112</t>
+          <t>VL86</t>
         </is>
       </c>
     </row>
     <row r="571">
       <c r="A571" s="2" t="inlineStr">
         <is>
-          <t>VL114</t>
+          <t>VL87</t>
         </is>
       </c>
     </row>
     <row r="572">
       <c r="A572" s="2" t="inlineStr">
         <is>
-          <t>VL115</t>
+          <t>VL88</t>
         </is>
       </c>
     </row>
     <row r="573">
       <c r="A573" s="2" t="inlineStr">
         <is>
-          <t>VL121</t>
+          <t>VL90</t>
         </is>
       </c>
     </row>
     <row r="574">
       <c r="A574" s="2" t="inlineStr">
         <is>
-          <t>VL122</t>
+          <t>VL92</t>
         </is>
       </c>
     </row>
     <row r="575">
       <c r="A575" s="2" t="inlineStr">
         <is>
-          <t>VL123</t>
+          <t>VL99</t>
         </is>
       </c>
     </row>
     <row r="576">
       <c r="A576" s="2" t="inlineStr">
         <is>
-          <t>VL124</t>
+          <t>VL100</t>
         </is>
       </c>
     </row>
     <row r="577">
       <c r="A577" s="2" t="inlineStr">
         <is>
-          <t>VL125</t>
+          <t>VL101</t>
         </is>
       </c>
     </row>
     <row r="578">
       <c r="A578" s="2" t="inlineStr">
         <is>
-          <t>VL126</t>
+          <t>VL103</t>
         </is>
       </c>
     </row>
     <row r="579">
       <c r="A579" s="2" t="inlineStr">
         <is>
-          <t>VL127</t>
+          <t>VL106</t>
         </is>
       </c>
     </row>
     <row r="580">
       <c r="A580" s="2" t="inlineStr">
         <is>
-          <t>VL129</t>
+          <t>VL107</t>
         </is>
       </c>
     </row>
     <row r="581">
       <c r="A581" s="2" t="inlineStr">
         <is>
-          <t>VL132</t>
+          <t>VL112</t>
         </is>
       </c>
     </row>
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>VL134</t>
+          <t>VL114</t>
         </is>
       </c>
     </row>
     <row r="583">
       <c r="A583" s="2" t="inlineStr">
         <is>
-          <t>VL137</t>
+          <t>VL115</t>
         </is>
       </c>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>VL139</t>
+          <t>VL121</t>
         </is>
       </c>
     </row>
     <row r="585">
       <c r="A585" s="2" t="inlineStr">
         <is>
-          <t>VL140</t>
+          <t>VL122</t>
         </is>
       </c>
     </row>
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>VL354</t>
+          <t>VL123</t>
         </is>
       </c>
     </row>
     <row r="587">
       <c r="A587" s="2" t="inlineStr">
         <is>
-          <t>VLINE8013</t>
+          <t>VL124</t>
         </is>
       </c>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>VLINE8020</t>
+          <t>VL125</t>
         </is>
       </c>
     </row>
     <row r="589">
       <c r="A589" s="2" t="inlineStr">
         <is>
-          <t>VLINE8021</t>
+          <t>VL126</t>
         </is>
       </c>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>VLINE8023</t>
+          <t>VL127</t>
         </is>
       </c>
     </row>
     <row r="591">
       <c r="A591" s="2" t="inlineStr">
         <is>
-          <t>VLINE8025</t>
+          <t>VL129</t>
         </is>
       </c>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>VLINE8028</t>
+          <t>VL132</t>
         </is>
       </c>
     </row>
     <row r="593">
       <c r="A593" s="2" t="inlineStr">
         <is>
-          <t>VLINE8030</t>
+          <t>VL134</t>
         </is>
       </c>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>VLINE8034</t>
+          <t>VL137</t>
         </is>
       </c>
     </row>
     <row r="595">
       <c r="A595" s="2" t="inlineStr">
         <is>
-          <t>VLINE8036</t>
+          <t>VL139</t>
         </is>
       </c>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>VLINE8058</t>
+          <t>VL140</t>
         </is>
       </c>
     </row>
     <row r="597">
       <c r="A597" s="2" t="inlineStr">
         <is>
-          <t>VLINE8059</t>
+          <t>VL354</t>
         </is>
       </c>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>VLINE8061</t>
+          <t>VLINE8013</t>
         </is>
       </c>
     </row>
     <row r="599">
       <c r="A599" s="2" t="inlineStr">
         <is>
-          <t>VLINE8071</t>
+          <t>VLINE8020</t>
         </is>
       </c>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>VLINE8072</t>
+          <t>VLINE8021</t>
         </is>
       </c>
     </row>
     <row r="601">
       <c r="A601" s="2" t="inlineStr">
         <is>
-          <t>VLINE8074</t>
+          <t>VLINE8023</t>
         </is>
       </c>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>VLINE8075</t>
+          <t>VLINE8025</t>
         </is>
       </c>
     </row>
     <row r="603">
       <c r="A603" s="2" t="inlineStr">
         <is>
-          <t>VLINE8077</t>
+          <t>VLINE8028</t>
         </is>
       </c>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>VLINE8080</t>
+          <t>VLINE8030</t>
         </is>
       </c>
     </row>
     <row r="605">
       <c r="A605" s="2" t="inlineStr">
         <is>
-          <t>VLINE8081</t>
+          <t>VLINE8034</t>
         </is>
       </c>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>VLINE8084</t>
+          <t>VLINE8036</t>
         </is>
       </c>
     </row>
     <row r="607">
       <c r="A607" s="2" t="inlineStr">
         <is>
-          <t>VLINE8102</t>
+          <t>VLINE8058</t>
         </is>
       </c>
     </row>
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>VLINE8111</t>
+          <t>VLINE8059</t>
         </is>
       </c>
     </row>
     <row r="609">
       <c r="A609" s="2" t="inlineStr">
         <is>
-          <t>VLINE8113</t>
+          <t>VLINE8061</t>
         </is>
       </c>
     </row>
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>VLINE8115</t>
+          <t>VLINE8071</t>
         </is>
       </c>
     </row>
     <row r="611">
       <c r="A611" s="2" t="inlineStr">
         <is>
-          <t>VLINE8117</t>
+          <t>VLINE8072</t>
         </is>
       </c>
     </row>
     <row r="612">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>VLINE8120</t>
+          <t>VLINE8074</t>
         </is>
       </c>
     </row>
     <row r="613">
       <c r="A613" s="2" t="inlineStr">
         <is>
-          <t>VLINE8121</t>
+          <t>VLINE8075</t>
         </is>
       </c>
     </row>
     <row r="614">
       <c r="A614" s="2" t="inlineStr">
         <is>
-          <t>VLINE8122</t>
+          <t>VLINE8076</t>
         </is>
       </c>
     </row>
     <row r="615">
       <c r="A615" s="2" t="inlineStr">
         <is>
-          <t>VLINE8123</t>
+          <t>VLINE8077</t>
         </is>
       </c>
     </row>
     <row r="616">
       <c r="A616" s="2" t="inlineStr">
         <is>
-          <t>VLINE8124</t>
+          <t>VLINE8080</t>
         </is>
       </c>
     </row>
     <row r="617">
       <c r="A617" s="2" t="inlineStr">
         <is>
-          <t>VLINE8125</t>
+          <t>VLINE8081</t>
         </is>
       </c>
     </row>
     <row r="618">
       <c r="A618" s="2" t="inlineStr">
         <is>
-          <t>VLINE8126</t>
+          <t>VLINE8084</t>
         </is>
       </c>
     </row>
     <row r="619">
       <c r="A619" s="2" t="inlineStr">
         <is>
-          <t>VLINE8127</t>
+          <t>VLINE8102</t>
         </is>
       </c>
     </row>
     <row r="620">
       <c r="A620" s="2" t="inlineStr">
         <is>
-          <t>VLINE8128</t>
+          <t>VLINE8111</t>
         </is>
       </c>
     </row>
     <row r="621">
       <c r="A621" s="2" t="inlineStr">
         <is>
-          <t>VLINE8130</t>
+          <t>VLINE8113</t>
         </is>
       </c>
     </row>
     <row r="622">
       <c r="A622" s="2" t="inlineStr">
         <is>
-          <t>VLINE8134</t>
+          <t>VLINE8115</t>
         </is>
       </c>
     </row>
     <row r="623">
       <c r="A623" s="2" t="inlineStr">
         <is>
-          <t>VLINE8136</t>
+          <t>VLINE8117</t>
         </is>
       </c>
     </row>
     <row r="624">
       <c r="A624" s="2" t="inlineStr">
         <is>
-          <t>VLINE8138</t>
+          <t>VLINE8120</t>
         </is>
       </c>
     </row>
     <row r="625">
       <c r="A625" s="2" t="inlineStr">
         <is>
-          <t>VLINE8161</t>
+          <t>VLINE8121</t>
         </is>
       </c>
     </row>
     <row r="626">
       <c r="A626" s="2" t="inlineStr">
         <is>
-          <t>VLINE8163</t>
+          <t>VLINE8122</t>
         </is>
       </c>
     </row>
     <row r="627">
       <c r="A627" s="2" t="inlineStr">
         <is>
-          <t>VLINE8164</t>
+          <t>VLINE8123</t>
         </is>
       </c>
     </row>
     <row r="628">
       <c r="A628" s="2" t="inlineStr">
         <is>
-          <t>VLINE8172</t>
+          <t>VLINE8124</t>
         </is>
       </c>
     </row>
     <row r="629">
       <c r="A629" s="2" t="inlineStr">
         <is>
-          <t>VLINE8181</t>
+          <t>VLINE8125</t>
         </is>
       </c>
     </row>
     <row r="630">
       <c r="A630" s="2" t="inlineStr">
         <is>
-          <t>VLINE8183</t>
+          <t>VLINE8126</t>
         </is>
       </c>
     </row>
     <row r="631">
       <c r="A631" s="2" t="inlineStr">
         <is>
-          <t>VLINE8184</t>
+          <t>VLINE8127</t>
         </is>
       </c>
     </row>
     <row r="632">
       <c r="A632" s="2" t="inlineStr">
         <is>
-          <t>VLINE8185</t>
+          <t>VLINE8128</t>
         </is>
       </c>
     </row>
     <row r="633">
       <c r="A633" s="2" t="inlineStr">
         <is>
-          <t>VLINE8186</t>
+          <t>VLINE8130</t>
         </is>
       </c>
     </row>
     <row r="634">
       <c r="A634" s="2" t="inlineStr">
         <is>
-          <t>VLINE8211</t>
+          <t>VLINE8131</t>
         </is>
       </c>
     </row>
     <row r="635">
       <c r="A635" s="2" t="inlineStr">
         <is>
-          <t>VLINE8213</t>
+          <t>VLINE8134</t>
         </is>
       </c>
     </row>
     <row r="636">
       <c r="A636" s="2" t="inlineStr">
         <is>
-          <t>VLINE8215</t>
+          <t>VLINE8136</t>
         </is>
       </c>
     </row>
     <row r="637">
       <c r="A637" s="2" t="inlineStr">
         <is>
-          <t>VLINE8217</t>
+          <t>VLINE8138</t>
         </is>
       </c>
     </row>
     <row r="638">
       <c r="A638" s="2" t="inlineStr">
         <is>
-          <t>VLINE8219</t>
+          <t>VLINE8161</t>
         </is>
       </c>
     </row>
     <row r="639">
       <c r="A639" s="2" t="inlineStr">
         <is>
-          <t>VLINE8221</t>
+          <t>VLINE8163</t>
         </is>
       </c>
     </row>
     <row r="640">
       <c r="A640" s="2" t="inlineStr">
         <is>
-          <t>VLINE8223</t>
+          <t>VLINE8164</t>
         </is>
       </c>
     </row>
     <row r="641">
       <c r="A641" s="2" t="inlineStr">
         <is>
-          <t>VLINE8225</t>
+          <t>VLINE8172</t>
         </is>
       </c>
     </row>
     <row r="642">
       <c r="A642" s="2" t="inlineStr">
         <is>
-          <t>VLINE8226</t>
+          <t>VLINE8181</t>
         </is>
       </c>
     </row>
     <row r="643">
       <c r="A643" s="2" t="inlineStr">
         <is>
-          <t>VLINE8227</t>
+          <t>VLINE8183</t>
         </is>
       </c>
     </row>
     <row r="644">
       <c r="A644" s="2" t="inlineStr">
         <is>
-          <t>VLINE8228</t>
+          <t>VLINE8184</t>
         </is>
       </c>
     </row>
     <row r="645">
       <c r="A645" s="2" t="inlineStr">
         <is>
-          <t>VLINE8229</t>
+          <t>VLINE8185</t>
         </is>
       </c>
     </row>
     <row r="646">
       <c r="A646" s="2" t="inlineStr">
         <is>
-          <t>VLINE8230</t>
+          <t>VLINE8186</t>
         </is>
       </c>
     </row>
     <row r="647">
       <c r="A647" s="2" t="inlineStr">
         <is>
-          <t>VLINE8232</t>
+          <t>VLINE8211</t>
         </is>
       </c>
     </row>
     <row r="648">
       <c r="A648" s="2" t="inlineStr">
         <is>
-          <t>VLINE8234</t>
+          <t>VLINE8213</t>
         </is>
       </c>
     </row>
     <row r="649">
       <c r="A649" s="2" t="inlineStr">
         <is>
-          <t>VLINE8236</t>
+          <t>VLINE8215</t>
         </is>
       </c>
     </row>
     <row r="650">
       <c r="A650" s="2" t="inlineStr">
         <is>
-          <t>VLINE8238</t>
+          <t>VLINE8217</t>
         </is>
       </c>
     </row>
     <row r="651">
       <c r="A651" s="2" t="inlineStr">
         <is>
-          <t>VLINE8240</t>
+          <t>VLINE8219</t>
         </is>
       </c>
     </row>
     <row r="652">
       <c r="A652" s="2" t="inlineStr">
         <is>
-          <t>VLINE8242</t>
+          <t>VLINE8221</t>
         </is>
       </c>
     </row>
     <row r="653">
       <c r="A653" s="2" t="inlineStr">
         <is>
-          <t>VLINE8400</t>
+          <t>VLINE8223</t>
         </is>
       </c>
     </row>
     <row r="654">
       <c r="A654" s="2" t="inlineStr">
         <is>
-          <t>VLINE8405</t>
+          <t>VLINE8225</t>
         </is>
       </c>
     </row>
     <row r="655">
       <c r="A655" s="2" t="inlineStr">
         <is>
-          <t>VLINE8408</t>
+          <t>VLINE8226</t>
         </is>
       </c>
     </row>
     <row r="656">
       <c r="A656" s="2" t="inlineStr">
         <is>
-          <t>VLINE8413</t>
+          <t>VLINE8227</t>
         </is>
       </c>
     </row>
     <row r="657">
       <c r="A657" s="2" t="inlineStr">
         <is>
-          <t>VLINE8415</t>
+          <t>VLINE8228</t>
         </is>
       </c>
     </row>
     <row r="658">
       <c r="A658" s="2" t="inlineStr">
         <is>
-          <t>VLINE8417</t>
+          <t>VLINE8229</t>
         </is>
       </c>
     </row>
     <row r="659">
       <c r="A659" s="2" t="inlineStr">
         <is>
-          <t>VLINE8418</t>
+          <t>VLINE8230</t>
         </is>
       </c>
     </row>
     <row r="660">
       <c r="A660" s="2" t="inlineStr">
         <is>
-          <t>VLINE8419</t>
+          <t>VLINE8231</t>
         </is>
       </c>
     </row>
     <row r="661">
       <c r="A661" s="2" t="inlineStr">
         <is>
-          <t>VLINE8420</t>
+          <t>VLINE8232</t>
         </is>
       </c>
     </row>
     <row r="662">
       <c r="A662" s="2" t="inlineStr">
         <is>
-          <t>VLINE8421</t>
+          <t>VLINE8234</t>
         </is>
       </c>
     </row>
     <row r="663">
       <c r="A663" s="2" t="inlineStr">
         <is>
-          <t>VLINE8422</t>
+          <t>VLINE8236</t>
         </is>
       </c>
     </row>
     <row r="664">
       <c r="A664" s="2" t="inlineStr">
         <is>
-          <t>VLINE8423</t>
+          <t>VLINE8238</t>
         </is>
       </c>
     </row>
     <row r="665">
       <c r="A665" s="2" t="inlineStr">
         <is>
-          <t>VLINE8424</t>
+          <t>VLINE8240</t>
         </is>
       </c>
     </row>
     <row r="666">
       <c r="A666" s="2" t="inlineStr">
         <is>
-          <t>VLINE8427</t>
+          <t>VLINE8242</t>
         </is>
       </c>
     </row>
     <row r="667">
       <c r="A667" s="2" t="inlineStr">
         <is>
-          <t>VLINE8428</t>
+          <t>VLINE8244</t>
         </is>
       </c>
     </row>
     <row r="668">
       <c r="A668" s="2" t="inlineStr">
         <is>
-          <t>VLINE8429</t>
+          <t>VLINE8400</t>
         </is>
       </c>
     </row>
     <row r="669">
       <c r="A669" s="2" t="inlineStr">
         <is>
-          <t>VLINE8430</t>
+          <t>VLINE8405</t>
         </is>
       </c>
     </row>
     <row r="670">
       <c r="A670" s="2" t="inlineStr">
         <is>
-          <t>VLINE8431</t>
+          <t>VLINE8408</t>
         </is>
       </c>
     </row>
     <row r="671">
       <c r="A671" s="2" t="inlineStr">
         <is>
-          <t>VLINE8432</t>
+          <t>VLINE8413</t>
         </is>
       </c>
     </row>
     <row r="672">
       <c r="A672" s="2" t="inlineStr">
         <is>
-          <t>VLINE8434</t>
+          <t>VLINE8415</t>
         </is>
       </c>
     </row>
     <row r="673">
       <c r="A673" s="2" t="inlineStr">
         <is>
-          <t>VLINE8438</t>
+          <t>VLINE8417</t>
         </is>
       </c>
     </row>
     <row r="674">
       <c r="A674" s="2" t="inlineStr">
         <is>
-          <t>VLINE8457</t>
+          <t>VLINE8418</t>
         </is>
       </c>
     </row>
     <row r="675">
       <c r="A675" s="2" t="inlineStr">
         <is>
-          <t>VLINE8459</t>
+          <t>VLINE8419</t>
         </is>
       </c>
     </row>
     <row r="676">
       <c r="A676" s="2" t="inlineStr">
         <is>
-          <t>VLINE8460</t>
+          <t>VLINE8420</t>
         </is>
       </c>
     </row>
     <row r="677">
       <c r="A677" s="2" t="inlineStr">
         <is>
-          <t>VLINE8461</t>
+          <t>VLINE8421</t>
         </is>
       </c>
     </row>
     <row r="678">
       <c r="A678" s="2" t="inlineStr">
         <is>
-          <t>VLINE8464</t>
+          <t>VLINE8422</t>
         </is>
       </c>
     </row>
     <row r="679">
       <c r="A679" s="2" t="inlineStr">
         <is>
-          <t>VLINE8465</t>
+          <t>VLINE8423</t>
         </is>
       </c>
     </row>
     <row r="680">
       <c r="A680" s="2" t="inlineStr">
         <is>
-          <t>VLINE8702</t>
+          <t>VLINE8424</t>
         </is>
       </c>
     </row>
     <row r="681">
       <c r="A681" s="2" t="inlineStr">
         <is>
-          <t>VLINE8725</t>
+          <t>VLINE8427</t>
         </is>
       </c>
     </row>
     <row r="682">
       <c r="A682" s="2" t="inlineStr">
         <is>
-          <t>VLINE8727</t>
+          <t>VLINE8428</t>
         </is>
       </c>
     </row>
     <row r="683">
       <c r="A683" s="2" t="inlineStr">
         <is>
-          <t>VLINE8729</t>
+          <t>VLINE8429</t>
         </is>
       </c>
     </row>
     <row r="684">
       <c r="A684" s="2" t="inlineStr">
         <is>
-          <t>VLINE8731</t>
+          <t>VLINE8430</t>
         </is>
       </c>
     </row>
     <row r="685">
       <c r="A685" s="2" t="inlineStr">
         <is>
-          <t>VLINE8733</t>
+          <t>VLINE8431</t>
         </is>
       </c>
     </row>
     <row r="686">
       <c r="A686" s="2" t="inlineStr">
         <is>
-          <t>VLINE8735</t>
+          <t>VLINE8432</t>
         </is>
       </c>
     </row>
     <row r="687">
       <c r="A687" s="2" t="inlineStr">
         <is>
-          <t>VLINE8737</t>
+          <t>VLINE8434</t>
         </is>
       </c>
     </row>
     <row r="688">
       <c r="A688" s="2" t="inlineStr">
         <is>
-          <t>VLINE8739</t>
+          <t>VLINE8438</t>
         </is>
       </c>
     </row>
     <row r="689">
       <c r="A689" s="2" t="inlineStr">
         <is>
-          <t>VLINE8741</t>
+          <t>VLINE8457</t>
         </is>
       </c>
     </row>
     <row r="690">
       <c r="A690" s="2" t="inlineStr">
         <is>
-          <t>VLINE8742</t>
+          <t>VLINE8459</t>
         </is>
       </c>
     </row>
     <row r="691">
       <c r="A691" s="2" t="inlineStr">
         <is>
-          <t>VLINE8743</t>
+          <t>VLINE8460</t>
         </is>
       </c>
     </row>
     <row r="692">
       <c r="A692" s="2" t="inlineStr">
         <is>
-          <t>VLINE8744</t>
+          <t>VLINE8461</t>
         </is>
       </c>
     </row>
     <row r="693">
       <c r="A693" s="2" t="inlineStr">
         <is>
-          <t>VLINE8745</t>
+          <t>VLINE8464</t>
         </is>
       </c>
     </row>
     <row r="694">
       <c r="A694" s="2" t="inlineStr">
         <is>
-          <t>VLINE8746</t>
+          <t>VLINE8465</t>
         </is>
       </c>
     </row>
     <row r="695">
       <c r="A695" s="2" t="inlineStr">
         <is>
-          <t>VLINE8747</t>
+          <t>VLINE8702</t>
         </is>
       </c>
     </row>
     <row r="696">
       <c r="A696" s="2" t="inlineStr">
         <is>
-          <t>VLINE8748</t>
+          <t>VLINE8725</t>
         </is>
       </c>
     </row>
     <row r="697">
       <c r="A697" s="2" t="inlineStr">
         <is>
-          <t>VLINE8749</t>
+          <t>VLINE8727</t>
         </is>
       </c>
     </row>
     <row r="698">
       <c r="A698" s="2" t="inlineStr">
         <is>
-          <t>VLINE8750</t>
+          <t>VLINE8729</t>
         </is>
       </c>
     </row>
     <row r="699">
       <c r="A699" s="2" t="inlineStr">
         <is>
-          <t>VLINE8751</t>
+          <t>VLINE8731</t>
         </is>
       </c>
     </row>
     <row r="700">
       <c r="A700" s="2" t="inlineStr">
         <is>
-          <t>VLINE8752</t>
+          <t>VLINE8733</t>
         </is>
       </c>
     </row>
     <row r="701">
       <c r="A701" s="2" t="inlineStr">
         <is>
-          <t>VLINE8753</t>
+          <t>VLINE8735</t>
         </is>
       </c>
     </row>
     <row r="702">
       <c r="A702" s="2" t="inlineStr">
         <is>
-          <t>VLINE8754</t>
+          <t>VLINE8737</t>
         </is>
       </c>
     </row>
     <row r="703">
       <c r="A703" s="2" t="inlineStr">
         <is>
-          <t>VLINE8755</t>
+          <t>VLINE8739</t>
         </is>
       </c>
     </row>
     <row r="704">
       <c r="A704" s="2" t="inlineStr">
         <is>
-          <t>VLINE8756</t>
+          <t>VLINE8741</t>
         </is>
       </c>
     </row>
     <row r="705">
       <c r="A705" s="2" t="inlineStr">
         <is>
-          <t>VLINE8757</t>
+          <t>VLINE8742</t>
         </is>
       </c>
     </row>
     <row r="706">
       <c r="A706" s="2" t="inlineStr">
         <is>
-          <t>VLINE8758</t>
+          <t>VLINE8743</t>
         </is>
       </c>
     </row>
     <row r="707">
       <c r="A707" s="2" t="inlineStr">
         <is>
-          <t>VLINE8759</t>
+          <t>VLINE8744</t>
         </is>
       </c>
     </row>
     <row r="708">
       <c r="A708" s="2" t="inlineStr">
         <is>
-          <t>VLINE8760</t>
+          <t>VLINE8745</t>
         </is>
       </c>
     </row>
     <row r="709">
       <c r="A709" s="2" t="inlineStr">
         <is>
-          <t>VLINE8761</t>
+          <t>VLINE8746</t>
         </is>
       </c>
     </row>
     <row r="710">
       <c r="A710" s="2" t="inlineStr">
         <is>
-          <t>VLINE8762</t>
+          <t>VLINE8747</t>
         </is>
       </c>
     </row>
     <row r="711">
       <c r="A711" s="2" t="inlineStr">
         <is>
-          <t>VLINE8764</t>
+          <t>VLINE8748</t>
         </is>
       </c>
     </row>
     <row r="712">
       <c r="A712" s="2" t="inlineStr">
         <is>
-          <t>VLINE8766</t>
+          <t>VLINE8749</t>
         </is>
       </c>
     </row>
     <row r="713">
       <c r="A713" s="2" t="inlineStr">
         <is>
-          <t>VLINE8768</t>
+          <t>VLINE8750</t>
         </is>
       </c>
     </row>
     <row r="714">
       <c r="A714" s="2" t="inlineStr">
         <is>
-          <t>VLINE8770</t>
+          <t>VLINE8751</t>
         </is>
       </c>
     </row>
     <row r="715">
       <c r="A715" s="2" t="inlineStr">
         <is>
-          <t>VLINE8772</t>
+          <t>VLINE8752</t>
         </is>
       </c>
     </row>
     <row r="716">
       <c r="A716" s="2" t="inlineStr">
         <is>
-          <t>VLINE8774</t>
+          <t>VLINE8753</t>
         </is>
       </c>
     </row>
     <row r="717">
       <c r="A717" s="2" t="inlineStr">
         <is>
-          <t>VLINE8776</t>
+          <t>VLINE8754</t>
         </is>
       </c>
     </row>
     <row r="718">
       <c r="A718" s="2" t="inlineStr">
         <is>
-          <t>VLINE8778</t>
+          <t>VLINE8755</t>
         </is>
       </c>
     </row>
     <row r="719">
       <c r="A719" s="2" t="inlineStr">
         <is>
-          <t>VLINE8780</t>
+          <t>VLINE8756</t>
         </is>
       </c>
     </row>
     <row r="720">
       <c r="A720" s="2" t="inlineStr">
         <is>
-          <t>VLINE8819</t>
+          <t>VLINE8757</t>
         </is>
       </c>
     </row>
     <row r="721">
       <c r="A721" s="2" t="inlineStr">
         <is>
-          <t>VLINE8862</t>
+          <t>VLINE8758</t>
         </is>
       </c>
     </row>
     <row r="722">
       <c r="A722" s="2" t="inlineStr">
         <is>
-          <t>VLINE8863</t>
+          <t>VLINE8759</t>
         </is>
       </c>
     </row>
     <row r="723">
       <c r="A723" s="2" t="inlineStr">
         <is>
-          <t>VLINE8864</t>
+          <t>VLINE8760</t>
         </is>
       </c>
     </row>
     <row r="724">
       <c r="A724" s="2" t="inlineStr">
         <is>
-          <t>VLINE8865</t>
+          <t>VLINE8761</t>
         </is>
       </c>
     </row>
     <row r="725">
       <c r="A725" s="2" t="inlineStr">
         <is>
-          <t>VR76</t>
+          <t>VLINE8762</t>
         </is>
       </c>
     </row>
     <row r="726">
       <c r="A726" s="2" t="inlineStr">
         <is>
-          <t>VR77</t>
+          <t>VLINE8763</t>
         </is>
       </c>
     </row>
     <row r="727">
       <c r="A727" s="2" t="inlineStr">
         <is>
-          <t>WOLL408</t>
+          <t>VLINE8764</t>
         </is>
       </c>
     </row>
     <row r="728">
       <c r="A728" s="2" t="inlineStr">
         <is>
-          <t>WOLL430</t>
+          <t>VLINE8765</t>
         </is>
       </c>
     </row>
     <row r="729">
       <c r="A729" s="2" t="inlineStr">
         <is>
-          <t>XP2001</t>
+          <t>VLINE8766</t>
         </is>
       </c>
     </row>
     <row r="730">
       <c r="A730" s="2" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>VLINE8768</t>
         </is>
       </c>
     </row>
     <row r="731">
       <c r="A731" s="2" t="inlineStr">
         <is>
-          <t>XP2006</t>
+          <t>VLINE8770</t>
         </is>
       </c>
     </row>
     <row r="732">
       <c r="A732" s="2" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>VLINE8772</t>
         </is>
       </c>
     </row>
     <row r="733">
       <c r="A733" s="2" t="inlineStr">
         <is>
-          <t>XP2009</t>
+          <t>VLINE8774</t>
         </is>
       </c>
     </row>
     <row r="734">
       <c r="A734" s="2" t="inlineStr">
         <is>
-          <t>XP2010</t>
+          <t>VLINE8776</t>
         </is>
       </c>
     </row>
     <row r="735">
       <c r="A735" s="2" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>VLINE8778</t>
         </is>
       </c>
     </row>
     <row r="736">
       <c r="A736" s="2" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>VLINE8780</t>
         </is>
       </c>
     </row>
     <row r="737">
       <c r="A737" s="2" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>VLINE8782</t>
         </is>
       </c>
     </row>
     <row r="738">
       <c r="A738" s="2" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>VLINE8819</t>
         </is>
       </c>
     </row>
     <row r="739">
       <c r="A739" s="2" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>VLINE8862</t>
         </is>
       </c>
     </row>
     <row r="740">
       <c r="A740" s="2" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>VLINE8863</t>
         </is>
       </c>
     </row>
     <row r="741">
       <c r="A741" s="2" t="inlineStr">
         <is>
-          <t>XRN003</t>
+          <t>VLINE8864</t>
         </is>
       </c>
     </row>
     <row r="742">
       <c r="A742" s="2" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>VLINE8865</t>
         </is>
       </c>
     </row>
     <row r="743">
       <c r="A743" s="2" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>VR76</t>
         </is>
       </c>
     </row>
     <row r="744">
       <c r="A744" s="2" t="inlineStr">
         <is>
-          <t>XRN010</t>
+          <t>VR77</t>
         </is>
       </c>
     </row>
     <row r="745">
       <c r="A745" s="2" t="inlineStr">
         <is>
-          <t>XRN012</t>
+          <t>WOLL408</t>
         </is>
       </c>
     </row>
     <row r="746">
       <c r="A746" s="2" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>WOLL430</t>
         </is>
       </c>
     </row>
     <row r="747">
       <c r="A747" s="2" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>X21</t>
         </is>
       </c>
     </row>
     <row r="748">
       <c r="A748" s="2" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>XP2001</t>
         </is>
       </c>
     </row>
     <row r="749">
       <c r="A749" s="2" t="inlineStr">
         <is>
-          <t>XRN022</t>
+          <t>XP2005</t>
         </is>
       </c>
     </row>
     <row r="750">
       <c r="A750" s="2" t="inlineStr">
         <is>
-          <t>XRN028</t>
+          <t>XP2006</t>
         </is>
       </c>
     </row>
     <row r="751">
       <c r="A751" s="2" t="inlineStr">
+        <is>
+          <t>XP2008</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="2" t="inlineStr">
+        <is>
+          <t>XP2009</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="2" t="inlineStr">
+        <is>
+          <t>XP2010</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" s="2" t="inlineStr">
+        <is>
+          <t>XP2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" s="2" t="inlineStr">
+        <is>
+          <t>XP2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" s="2" t="inlineStr">
+        <is>
+          <t>XP2013</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="2" t="inlineStr">
+        <is>
+          <t>XP2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="2" t="inlineStr">
+        <is>
+          <t>XP2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" s="2" t="inlineStr">
+        <is>
+          <t>XP2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" s="2" t="inlineStr">
+        <is>
+          <t>XRN003</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="2" t="inlineStr">
+        <is>
+          <t>XRN005</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="2" t="inlineStr">
+        <is>
+          <t>XRN009</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="2" t="inlineStr">
+        <is>
+          <t>XRN010</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" s="2" t="inlineStr">
+        <is>
+          <t>XRN012</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="2" t="inlineStr">
+        <is>
+          <t>XRN017</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="2" t="inlineStr">
+        <is>
+          <t>XRN018</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" s="2" t="inlineStr">
+        <is>
+          <t>XRN021</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="2" t="inlineStr">
+        <is>
+          <t>XRN022</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" s="2" t="inlineStr">
+        <is>
+          <t>XRN028</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="2" t="inlineStr">
         <is>
           <t>XRN029</t>
         </is>

</xml_diff>

<commit_message>
Update RailOps database files - 2026-04-30 06:01:21 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A770"/>
+  <dimension ref="A1:A791"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2141,3701 +2141,3848 @@
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>MM64M</t>
+          <t>MM62M</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>MM76M</t>
+          <t>MM64M</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>MM78M</t>
+          <t>MM76M</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>MM80M</t>
+          <t>MM78M</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>MM82M</t>
+          <t>MM80M</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>MM84M</t>
+          <t>MM82M</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>MM86M</t>
+          <t>MM84M</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>MM92M</t>
+          <t>MM86M</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>MM94M</t>
+          <t>MM92M</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>MM96M</t>
+          <t>MM94M</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>MM98M</t>
+          <t>MM96M</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>MM99M</t>
+          <t>MM98M</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>MM122M</t>
+          <t>MM99M</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>MM130M</t>
+          <t>MM122M</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>MM152M</t>
+          <t>MM130M</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>MM156M</t>
+          <t>MM152M</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>MM158M</t>
+          <t>MM156M</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>MM172M</t>
+          <t>MM158M</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>MM178M</t>
+          <t>MM172M</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>MM192M</t>
+          <t>MM178M</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>MM212M</t>
+          <t>MM192M</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>MM214M</t>
+          <t>MM212M</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>MM216M</t>
+          <t>MM214M</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>MM224M</t>
+          <t>MM216M</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>MM232M</t>
+          <t>MM224M</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>MM236M</t>
+          <t>MM232M</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>MM240M</t>
+          <t>MM236M</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>MM246M</t>
+          <t>MM240M</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>MM256M</t>
+          <t>MM246M</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>MM258M</t>
+          <t>MM256M</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>MM260M</t>
+          <t>MM258M</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>MM264M</t>
+          <t>MM260M</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>MM266M</t>
+          <t>MM264M</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>MM268M</t>
+          <t>MM266M</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>MM270M</t>
+          <t>MM268M</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>MM280M</t>
+          <t>MM270M</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>MM288M</t>
+          <t>MM280M</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>MM380M</t>
+          <t>MM288M</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>MM418M</t>
+          <t>MM380M</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>MM424M</t>
+          <t>MM384M</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>MM456M</t>
+          <t>MM418M</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>MM464M</t>
+          <t>MM424M</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>MM478M</t>
+          <t>MM456M</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>MM482M</t>
+          <t>MM464M</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>MM486M</t>
+          <t>MM478M</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>MM502M</t>
+          <t>MM482M</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>MM506M</t>
+          <t>MM486M</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>MM514M</t>
+          <t>MM502M</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>MM522M</t>
+          <t>MM506M</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>MM536M</t>
+          <t>MM514M</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>MM542M</t>
+          <t>MM522M</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>MM544M</t>
+          <t>MM536M</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>MM546M</t>
+          <t>MM542M</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>MM551M</t>
+          <t>MM544M</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>MM552M</t>
+          <t>MM546M</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>MM566M</t>
+          <t>MM551M</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>MM574M</t>
+          <t>MM552M</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>MM588M</t>
+          <t>MM566M</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>MM592M</t>
+          <t>MM574M</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>MM602M</t>
+          <t>MM588M</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>MM604M</t>
+          <t>MM592M</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>MM620M</t>
+          <t>MM602M</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>MM624M</t>
+          <t>MM604M</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>MM636M</t>
+          <t>MM620M</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>MM638M</t>
+          <t>MM624M</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>MM647M</t>
+          <t>MM636M</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>MM656M</t>
+          <t>MM638M</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>MM658M</t>
+          <t>MM647M</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>MM660M</t>
+          <t>MM656M</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>MM662M</t>
+          <t>MM658M</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>MM664M</t>
+          <t>MM660M</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>MM668M</t>
+          <t>MM662M</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>MM673M</t>
+          <t>MM664M</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>MM674M</t>
+          <t>MM668M</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>MM676M</t>
+          <t>MM673M</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>MM680M</t>
+          <t>MM674M</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>MM702M</t>
+          <t>MM676M</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>MM708M</t>
+          <t>MM680M</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>MM718M</t>
+          <t>MM702M</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>MM742M</t>
+          <t>MM708M</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>MM744M</t>
+          <t>MM718M</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>MM752M</t>
+          <t>MM742M</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>MM756M</t>
+          <t>MM744M</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>MM766M</t>
+          <t>MM752M</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>MM768M</t>
+          <t>MM756M</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>MM772M</t>
+          <t>MM760M</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>MM774M</t>
+          <t>MM766M</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>MM776M</t>
+          <t>MM768M</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>MM778M</t>
+          <t>MM772M</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>MM780M</t>
+          <t>MM774M</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>MM784M</t>
+          <t>MM776M</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>MM788M</t>
+          <t>MM778M</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>MM790M</t>
+          <t>MM780M</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>MM794M</t>
+          <t>MM784M</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>MM798M</t>
+          <t>MM788M</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>MM800M</t>
+          <t>MM790M</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>MM802M</t>
+          <t>MM794M</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>MM806M</t>
+          <t>MM798M</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>MM808M</t>
+          <t>MM800M</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>MM810M</t>
+          <t>MM802M</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>MM816M</t>
+          <t>MM806M</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>MM826M</t>
+          <t>MM808M</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>MM830M</t>
+          <t>MM810M</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>MM832M</t>
+          <t>MM816M</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>MM834M</t>
+          <t>MM820M</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>MM836M</t>
+          <t>MM826M</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>MM838M</t>
+          <t>MM830M</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>MM842M</t>
+          <t>MM832M</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>MM858M</t>
+          <t>MM834M</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>MM860M</t>
+          <t>MM836M</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>MM862M</t>
+          <t>MM838M</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>MM864M</t>
+          <t>MM842M</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>MM866M</t>
+          <t>MM858M</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>MM872M</t>
+          <t>MM860M</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>MM878M</t>
+          <t>MM862M</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>MM880M</t>
+          <t>MM864M</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>MM886M</t>
+          <t>MM866M</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>MM896M</t>
+          <t>MM872M</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>MM908M</t>
+          <t>MM878M</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>MM910M</t>
+          <t>MM880M</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>MM912M</t>
+          <t>MM882M</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>MM914M</t>
+          <t>MM886M</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>MM922M</t>
+          <t>MM896M</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>MM924M</t>
+          <t>MM908M</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>MM928M</t>
+          <t>MM910M</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>MM934M</t>
+          <t>MM912M</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>MM940M</t>
+          <t>MM914M</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>MM944M</t>
+          <t>MM922M</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>MM946M</t>
+          <t>MM924M</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>MM952M</t>
+          <t>MM928M</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>MM956M</t>
+          <t>MM934M</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t>MM958M</t>
+          <t>MM940M</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>MM960M</t>
+          <t>MM944M</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t>MM962M</t>
+          <t>MM946M</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>MM964M</t>
+          <t>MM952M</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>MM968M</t>
+          <t>MM956M</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>MM970M</t>
+          <t>MM958M</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>MM972M</t>
+          <t>MM960M</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>MM974M</t>
+          <t>MM962M</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>MM976M</t>
+          <t>MM964M</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>MM980M</t>
+          <t>MM968M</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
         <is>
-          <t>MM982M</t>
+          <t>MM970M</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>MM9901M</t>
+          <t>MM972M</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
         <is>
-          <t>MM9903M</t>
+          <t>MM974M</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
         <is>
-          <t>MM9904M</t>
+          <t>MM976M</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" s="2" t="inlineStr">
         <is>
-          <t>MM9905M</t>
+          <t>MM980M</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
         <is>
-          <t>MM9906M</t>
+          <t>MM982M</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
         <is>
-          <t>MM9908M</t>
+          <t>MM984M</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>MM9909M</t>
+          <t>MM9901M</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
         <is>
-          <t>MM9910M</t>
+          <t>MM9903M</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
         <is>
-          <t>MM9912M</t>
+          <t>MM9904M</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="2" t="inlineStr">
         <is>
-          <t>MM9914M</t>
+          <t>MM9905M</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
         <is>
-          <t>MM9916M</t>
+          <t>MM9906M</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" s="2" t="inlineStr">
         <is>
-          <t>MM9918M</t>
+          <t>MM9908M</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
         <is>
-          <t>MM9920M</t>
+          <t>MM9909M</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="2" t="inlineStr">
         <is>
-          <t>MM9921M</t>
+          <t>MM9910M</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" s="2" t="inlineStr">
         <is>
-          <t>MM9924M</t>
+          <t>MM9912M</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="2" t="inlineStr">
         <is>
-          <t>MM9926M</t>
+          <t>MM9914M</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
         <is>
-          <t>MM9927M</t>
+          <t>MM9916M</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" s="2" t="inlineStr">
         <is>
-          <t>MM9928M</t>
+          <t>MM9918M</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
         <is>
-          <t>MM9929M</t>
+          <t>MM9919M</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" s="2" t="inlineStr">
         <is>
-          <t>MM9931M</t>
+          <t>MM9920M</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" s="2" t="inlineStr">
         <is>
-          <t>MM9933M</t>
+          <t>MM9921M</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
         <is>
-          <t>MM9936M</t>
+          <t>MM9922M</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="2" t="inlineStr">
         <is>
-          <t>MM9937M</t>
+          <t>MM9924M</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
         <is>
-          <t>MM9938M</t>
+          <t>MM9926M</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="2" t="inlineStr">
         <is>
-          <t>MM9941M</t>
+          <t>MM9927M</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="2" t="inlineStr">
         <is>
-          <t>MM9943M</t>
+          <t>MM9928M</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" s="2" t="inlineStr">
         <is>
-          <t>MM9946M</t>
+          <t>MM9929M</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" s="2" t="inlineStr">
         <is>
-          <t>MM9947M</t>
+          <t>MM9931M</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" s="2" t="inlineStr">
         <is>
-          <t>MM9948M</t>
+          <t>MM9933M</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" s="2" t="inlineStr">
         <is>
-          <t>MM9952M</t>
+          <t>MM9936M</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" s="2" t="inlineStr">
         <is>
-          <t>MM9953M</t>
+          <t>MM9937M</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" s="2" t="inlineStr">
         <is>
-          <t>MM9954M</t>
+          <t>MM9938M</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" s="2" t="inlineStr">
         <is>
-          <t>MM9956M</t>
+          <t>MM9941M</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" s="2" t="inlineStr">
         <is>
-          <t>MM9957M</t>
+          <t>MM9943M</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t>MM9958M</t>
+          <t>MM9946M</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" s="2" t="inlineStr">
         <is>
-          <t>MM9959M</t>
+          <t>MM9947M</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
         <is>
-          <t>MM9960M</t>
+          <t>MM9948M</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" s="2" t="inlineStr">
         <is>
-          <t>MM9961M</t>
+          <t>MM9952M</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" s="2" t="inlineStr">
         <is>
-          <t>MM9962M</t>
+          <t>MM9953M</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" s="2" t="inlineStr">
         <is>
-          <t>MM9963M</t>
+          <t>MM9954M</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
         <is>
-          <t>MM9964M</t>
+          <t>MM9956M</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="2" t="inlineStr">
         <is>
-          <t>MM9965M</t>
+          <t>MM9957M</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
         <is>
-          <t>MM9966M</t>
+          <t>MM9958M</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
         <is>
-          <t>MM9968M</t>
+          <t>MM9959M</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>MM9969M</t>
+          <t>MM9960M</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" s="2" t="inlineStr">
         <is>
-          <t>MM9970M</t>
+          <t>MM9961M</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MM9962M</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" s="2" t="inlineStr">
         <is>
-          <t>MRL002</t>
+          <t>MM9963M</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
         <is>
-          <t>MTPV1</t>
+          <t>MM9964M</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" s="2" t="inlineStr">
         <is>
-          <t>MTPV2</t>
+          <t>MM9965M</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t>N453</t>
+          <t>MM9966M</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t>N458</t>
+          <t>MM9968M</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>N460</t>
+          <t>MM9969M</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>MM9970M</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>MRL001</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>MRL002</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>MTPV1</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
         <is>
-          <t>NR6</t>
+          <t>MTPV2</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>NR10</t>
+          <t>N453</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
         <is>
-          <t>NR11</t>
+          <t>N458</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>NR12</t>
+          <t>N460</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
         <is>
-          <t>NR13</t>
+          <t>N466</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>NR14</t>
+          <t>N469</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
         <is>
-          <t>NR17</t>
+          <t>NR4</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>NR20</t>
+          <t>NR5</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
         <is>
-          <t>NR31</t>
+          <t>NR6</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>NR35</t>
+          <t>NR10</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>NR11</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>NR44</t>
+          <t>NR12</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="2" t="inlineStr">
         <is>
-          <t>NR46</t>
+          <t>NR13</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>NR14</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" s="2" t="inlineStr">
         <is>
-          <t>NR52</t>
+          <t>NR17</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>NR20</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" s="2" t="inlineStr">
         <is>
-          <t>NR56</t>
+          <t>NR31</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="2" t="inlineStr">
         <is>
-          <t>NR60</t>
+          <t>NR35</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" s="2" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR37</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" s="2" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR44</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" s="2" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR46</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" s="2" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR47</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="2" t="inlineStr">
         <is>
-          <t>NR76</t>
+          <t>NR52</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="2" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR54</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="2" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR56</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="2" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR60</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="2" t="inlineStr">
         <is>
-          <t>NR88</t>
+          <t>NR64</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" s="2" t="inlineStr">
         <is>
-          <t>NR91</t>
+          <t>NR65</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" s="2" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR68</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" s="2" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR75</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" s="2" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR76</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="A472" s="2" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>NR78</t>
         </is>
       </c>
     </row>
     <row r="473">
       <c r="A473" s="2" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR82</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="A474" s="2" t="inlineStr">
         <is>
-          <t>NR106</t>
+          <t>NR83</t>
         </is>
       </c>
     </row>
     <row r="475">
       <c r="A475" s="2" t="inlineStr">
         <is>
-          <t>NR107</t>
+          <t>NR88</t>
         </is>
       </c>
     </row>
     <row r="476">
       <c r="A476" s="2" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR91</t>
         </is>
       </c>
     </row>
     <row r="477">
       <c r="A477" s="2" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR93</t>
         </is>
       </c>
     </row>
     <row r="478">
       <c r="A478" s="2" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR94</t>
         </is>
       </c>
     </row>
     <row r="479">
       <c r="A479" s="2" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR95</t>
         </is>
       </c>
     </row>
     <row r="480">
       <c r="A480" s="2" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>NR97</t>
         </is>
       </c>
     </row>
     <row r="481">
       <c r="A481" s="2" t="inlineStr">
         <is>
-          <t>PB5</t>
+          <t>NR102</t>
         </is>
       </c>
     </row>
     <row r="482">
       <c r="A482" s="2" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>NR106</t>
         </is>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="2" t="inlineStr">
         <is>
-          <t>PKLA4</t>
+          <t>NR107</t>
         </is>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="2" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>NR109</t>
         </is>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="2" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>NR112</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="2" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>NR113</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="2" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>NR115</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" s="2" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>PB4</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" s="2" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>PB5</t>
         </is>
       </c>
     </row>
     <row r="490">
       <c r="A490" s="2" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
     <row r="491">
       <c r="A491" s="2" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>PKLA4</t>
         </is>
       </c>
     </row>
     <row r="492">
       <c r="A492" s="2" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="2" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
     <row r="494">
       <c r="A494" s="2" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
     <row r="495">
       <c r="A495" s="2" t="inlineStr">
         <is>
-          <t>QL009</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
     <row r="496">
       <c r="A496" s="2" t="inlineStr">
         <is>
-          <t>QL016</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
     <row r="497">
       <c r="A497" s="2" t="inlineStr">
         <is>
-          <t>QL019</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
     <row r="498">
       <c r="A498" s="2" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>QE001</t>
         </is>
       </c>
     </row>
     <row r="499">
       <c r="A499" s="2" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
     <row r="500">
       <c r="A500" s="2" t="inlineStr">
         <is>
-          <t>QR5400</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
     <row r="501">
       <c r="A501" s="2" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QL004</t>
         </is>
       </c>
     </row>
     <row r="502">
       <c r="A502" s="2" t="inlineStr">
         <is>
-          <t>RA2302</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
     <row r="503">
       <c r="A503" s="2" t="inlineStr">
         <is>
-          <t>RA2303</t>
+          <t>QL009</t>
         </is>
       </c>
     </row>
     <row r="504">
       <c r="A504" s="2" t="inlineStr">
         <is>
-          <t>RB2352</t>
+          <t>QL016</t>
         </is>
       </c>
     </row>
     <row r="505">
       <c r="A505" s="2" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>QL019</t>
         </is>
       </c>
     </row>
     <row r="506">
       <c r="A506" s="2" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>QR1744</t>
         </is>
       </c>
     </row>
     <row r="507">
       <c r="A507" s="2" t="inlineStr">
         <is>
-          <t>RL309</t>
+          <t>QR1771</t>
         </is>
       </c>
     </row>
     <row r="508">
       <c r="A508" s="2" t="inlineStr">
         <is>
-          <t>RM93</t>
+          <t>QR5400</t>
         </is>
       </c>
     </row>
     <row r="509">
       <c r="A509" s="2" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
     <row r="510">
       <c r="A510" s="2" t="inlineStr">
         <is>
-          <t>SCT008</t>
+          <t>RA2302</t>
         </is>
       </c>
     </row>
     <row r="511">
       <c r="A511" s="2" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>RA2303</t>
         </is>
       </c>
     </row>
     <row r="512">
       <c r="A512" s="2" t="inlineStr">
         <is>
-          <t>SCT010</t>
+          <t>RB2352</t>
         </is>
       </c>
     </row>
     <row r="513">
       <c r="A513" s="2" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
     <row r="514">
       <c r="A514" s="2" t="inlineStr">
         <is>
-          <t>SM636B</t>
+          <t>RL301</t>
         </is>
       </c>
     </row>
     <row r="515">
       <c r="A515" s="2" t="inlineStr">
         <is>
-          <t>SO3</t>
+          <t>RL309</t>
         </is>
       </c>
     </row>
     <row r="516">
       <c r="A516" s="2" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>RM93</t>
         </is>
       </c>
     </row>
     <row r="517">
       <c r="A517" s="2" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>SCT001</t>
         </is>
       </c>
     </row>
     <row r="518">
       <c r="A518" s="2" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>SCT008</t>
         </is>
       </c>
     </row>
     <row r="519">
       <c r="A519" s="2" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>SCT009</t>
         </is>
       </c>
     </row>
     <row r="520">
       <c r="A520" s="2" t="inlineStr">
         <is>
-          <t>T373</t>
+          <t>SCT010</t>
         </is>
       </c>
     </row>
     <row r="521">
       <c r="A521" s="2" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>SCT013</t>
         </is>
       </c>
     </row>
     <row r="522">
       <c r="A522" s="2" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>SM636B</t>
         </is>
       </c>
     </row>
     <row r="523">
       <c r="A523" s="2" t="inlineStr">
         <is>
-          <t>TE2804</t>
+          <t>SO3</t>
         </is>
       </c>
     </row>
     <row r="524">
       <c r="A524" s="2" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>SSR101</t>
         </is>
       </c>
     </row>
     <row r="525">
       <c r="A525" s="2" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>SSR102</t>
         </is>
       </c>
     </row>
     <row r="526">
       <c r="A526" s="2" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>SSR103</t>
         </is>
       </c>
     </row>
     <row r="527">
       <c r="A527" s="2" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>SSR104</t>
         </is>
       </c>
     </row>
     <row r="528">
       <c r="A528" s="2" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>T373</t>
         </is>
       </c>
     </row>
     <row r="529">
       <c r="A529" s="2" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>TE2801</t>
         </is>
       </c>
     </row>
     <row r="530">
       <c r="A530" s="2" t="inlineStr">
         <is>
-          <t>TT02</t>
+          <t>TE2803</t>
         </is>
       </c>
     </row>
     <row r="531">
       <c r="A531" s="2" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>TE2804</t>
         </is>
       </c>
     </row>
     <row r="532">
       <c r="A532" s="2" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>TE2805</t>
         </is>
       </c>
     </row>
     <row r="533">
       <c r="A533" s="2" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TE2807</t>
         </is>
       </c>
     </row>
     <row r="534">
       <c r="A534" s="2" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TE2808</t>
         </is>
       </c>
     </row>
     <row r="535">
       <c r="A535" s="2" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TE2813</t>
         </is>
       </c>
     </row>
     <row r="536">
       <c r="A536" s="2" t="inlineStr">
         <is>
-          <t>TT104</t>
+          <t>TE2814</t>
         </is>
       </c>
     </row>
     <row r="537">
       <c r="A537" s="2" t="inlineStr">
         <is>
-          <t>TT105</t>
+          <t>TJ096</t>
         </is>
       </c>
     </row>
     <row r="538">
       <c r="A538" s="2" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TT02</t>
         </is>
       </c>
     </row>
     <row r="539">
       <c r="A539" s="2" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TT03</t>
         </is>
       </c>
     </row>
     <row r="540">
       <c r="A540" s="2" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TT04</t>
         </is>
       </c>
     </row>
     <row r="541">
       <c r="A541" s="2" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TT05</t>
         </is>
       </c>
     </row>
     <row r="542">
       <c r="A542" s="2" t="inlineStr">
         <is>
-          <t>TT123</t>
+          <t>TT08</t>
         </is>
       </c>
     </row>
     <row r="543">
       <c r="A543" s="2" t="inlineStr">
         <is>
-          <t>TT126</t>
+          <t>TT103</t>
         </is>
       </c>
     </row>
     <row r="544">
       <c r="A544" s="2" t="inlineStr">
         <is>
-          <t>TT129</t>
+          <t>TT104</t>
         </is>
       </c>
     </row>
     <row r="545">
       <c r="A545" s="2" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT105</t>
         </is>
       </c>
     </row>
     <row r="546">
       <c r="A546" s="2" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT107</t>
         </is>
       </c>
     </row>
     <row r="547">
       <c r="A547" s="2" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT110</t>
         </is>
       </c>
     </row>
     <row r="548">
       <c r="A548" s="2" t="inlineStr">
         <is>
-          <t>VL01</t>
+          <t>TT115</t>
         </is>
       </c>
     </row>
     <row r="549">
       <c r="A549" s="2" t="inlineStr">
         <is>
-          <t>VL03</t>
+          <t>TT117</t>
         </is>
       </c>
     </row>
     <row r="550">
       <c r="A550" s="2" t="inlineStr">
         <is>
-          <t>VL04</t>
+          <t>TT123</t>
         </is>
       </c>
     </row>
     <row r="551">
       <c r="A551" s="2" t="inlineStr">
         <is>
-          <t>VL11</t>
+          <t>TT126</t>
         </is>
       </c>
     </row>
     <row r="552">
       <c r="A552" s="2" t="inlineStr">
         <is>
-          <t>VL13</t>
+          <t>TT129</t>
         </is>
       </c>
     </row>
     <row r="553">
       <c r="A553" s="2" t="inlineStr">
         <is>
-          <t>VL20</t>
+          <t>TT130</t>
         </is>
       </c>
     </row>
     <row r="554">
       <c r="A554" s="2" t="inlineStr">
         <is>
-          <t>VL22</t>
+          <t>TT202</t>
         </is>
       </c>
     </row>
     <row r="555">
       <c r="A555" s="2" t="inlineStr">
         <is>
-          <t>VL27</t>
+          <t>TT206</t>
         </is>
       </c>
     </row>
     <row r="556">
       <c r="A556" s="2" t="inlineStr">
         <is>
-          <t>VL30</t>
+          <t>VL01</t>
         </is>
       </c>
     </row>
     <row r="557">
       <c r="A557" s="2" t="inlineStr">
         <is>
-          <t>VL35</t>
+          <t>VL03</t>
         </is>
       </c>
     </row>
     <row r="558">
       <c r="A558" s="2" t="inlineStr">
         <is>
-          <t>VL36</t>
+          <t>VL04</t>
         </is>
       </c>
     </row>
     <row r="559">
       <c r="A559" s="2" t="inlineStr">
         <is>
-          <t>VL38</t>
+          <t>VL11</t>
         </is>
       </c>
     </row>
     <row r="560">
       <c r="A560" s="2" t="inlineStr">
         <is>
-          <t>VL43</t>
+          <t>VL13</t>
         </is>
       </c>
     </row>
     <row r="561">
       <c r="A561" s="2" t="inlineStr">
         <is>
-          <t>VL47</t>
+          <t>VL20</t>
         </is>
       </c>
     </row>
     <row r="562">
       <c r="A562" s="2" t="inlineStr">
         <is>
-          <t>VL49</t>
+          <t>VL22</t>
         </is>
       </c>
     </row>
     <row r="563">
       <c r="A563" s="2" t="inlineStr">
         <is>
-          <t>VL54</t>
+          <t>VL27</t>
         </is>
       </c>
     </row>
     <row r="564">
       <c r="A564" s="2" t="inlineStr">
         <is>
-          <t>VL57</t>
+          <t>VL30</t>
         </is>
       </c>
     </row>
     <row r="565">
       <c r="A565" s="2" t="inlineStr">
         <is>
-          <t>VL62</t>
+          <t>VL35</t>
         </is>
       </c>
     </row>
     <row r="566">
       <c r="A566" s="2" t="inlineStr">
         <is>
-          <t>VL67</t>
+          <t>VL36</t>
         </is>
       </c>
     </row>
     <row r="567">
       <c r="A567" s="2" t="inlineStr">
         <is>
-          <t>VL68</t>
+          <t>VL38</t>
         </is>
       </c>
     </row>
     <row r="568">
       <c r="A568" s="2" t="inlineStr">
         <is>
-          <t>VL75</t>
+          <t>VL43</t>
         </is>
       </c>
     </row>
     <row r="569">
       <c r="A569" s="2" t="inlineStr">
         <is>
-          <t>VL81</t>
+          <t>VL47</t>
         </is>
       </c>
     </row>
     <row r="570">
       <c r="A570" s="2" t="inlineStr">
         <is>
-          <t>VL86</t>
+          <t>VL49</t>
         </is>
       </c>
     </row>
     <row r="571">
       <c r="A571" s="2" t="inlineStr">
         <is>
-          <t>VL87</t>
+          <t>VL54</t>
         </is>
       </c>
     </row>
     <row r="572">
       <c r="A572" s="2" t="inlineStr">
         <is>
-          <t>VL88</t>
+          <t>VL57</t>
         </is>
       </c>
     </row>
     <row r="573">
       <c r="A573" s="2" t="inlineStr">
         <is>
-          <t>VL90</t>
+          <t>VL62</t>
         </is>
       </c>
     </row>
     <row r="574">
       <c r="A574" s="2" t="inlineStr">
         <is>
-          <t>VL92</t>
+          <t>VL67</t>
         </is>
       </c>
     </row>
     <row r="575">
       <c r="A575" s="2" t="inlineStr">
         <is>
-          <t>VL99</t>
+          <t>VL68</t>
         </is>
       </c>
     </row>
     <row r="576">
       <c r="A576" s="2" t="inlineStr">
         <is>
-          <t>VL100</t>
+          <t>VL75</t>
         </is>
       </c>
     </row>
     <row r="577">
       <c r="A577" s="2" t="inlineStr">
         <is>
-          <t>VL101</t>
+          <t>VL81</t>
         </is>
       </c>
     </row>
     <row r="578">
       <c r="A578" s="2" t="inlineStr">
         <is>
-          <t>VL103</t>
+          <t>VL86</t>
         </is>
       </c>
     </row>
     <row r="579">
       <c r="A579" s="2" t="inlineStr">
         <is>
-          <t>VL106</t>
+          <t>VL87</t>
         </is>
       </c>
     </row>
     <row r="580">
       <c r="A580" s="2" t="inlineStr">
         <is>
-          <t>VL107</t>
+          <t>VL88</t>
         </is>
       </c>
     </row>
     <row r="581">
       <c r="A581" s="2" t="inlineStr">
         <is>
-          <t>VL112</t>
+          <t>VL90</t>
         </is>
       </c>
     </row>
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>VL114</t>
+          <t>VL92</t>
         </is>
       </c>
     </row>
     <row r="583">
       <c r="A583" s="2" t="inlineStr">
         <is>
-          <t>VL115</t>
+          <t>VL99</t>
         </is>
       </c>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>VL121</t>
+          <t>VL100</t>
         </is>
       </c>
     </row>
     <row r="585">
       <c r="A585" s="2" t="inlineStr">
         <is>
-          <t>VL122</t>
+          <t>VL101</t>
         </is>
       </c>
     </row>
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>VL123</t>
+          <t>VL103</t>
         </is>
       </c>
     </row>
     <row r="587">
       <c r="A587" s="2" t="inlineStr">
         <is>
-          <t>VL124</t>
+          <t>VL106</t>
         </is>
       </c>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>VL125</t>
+          <t>VL107</t>
         </is>
       </c>
     </row>
     <row r="589">
       <c r="A589" s="2" t="inlineStr">
         <is>
-          <t>VL126</t>
+          <t>VL112</t>
         </is>
       </c>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>VL127</t>
+          <t>VL114</t>
         </is>
       </c>
     </row>
     <row r="591">
       <c r="A591" s="2" t="inlineStr">
         <is>
-          <t>VL129</t>
+          <t>VL115</t>
         </is>
       </c>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>VL132</t>
+          <t>VL121</t>
         </is>
       </c>
     </row>
     <row r="593">
       <c r="A593" s="2" t="inlineStr">
         <is>
-          <t>VL134</t>
+          <t>VL122</t>
         </is>
       </c>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>VL137</t>
+          <t>VL123</t>
         </is>
       </c>
     </row>
     <row r="595">
       <c r="A595" s="2" t="inlineStr">
         <is>
-          <t>VL139</t>
+          <t>VL124</t>
         </is>
       </c>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>VL140</t>
+          <t>VL125</t>
         </is>
       </c>
     </row>
     <row r="597">
       <c r="A597" s="2" t="inlineStr">
         <is>
-          <t>VL354</t>
+          <t>VL126</t>
         </is>
       </c>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>VLINE8013</t>
+          <t>VL127</t>
         </is>
       </c>
     </row>
     <row r="599">
       <c r="A599" s="2" t="inlineStr">
         <is>
-          <t>VLINE8020</t>
+          <t>VL129</t>
         </is>
       </c>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>VLINE8021</t>
+          <t>VL132</t>
         </is>
       </c>
     </row>
     <row r="601">
       <c r="A601" s="2" t="inlineStr">
         <is>
-          <t>VLINE8023</t>
+          <t>VL134</t>
         </is>
       </c>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>VLINE8025</t>
+          <t>VL137</t>
         </is>
       </c>
     </row>
     <row r="603">
       <c r="A603" s="2" t="inlineStr">
         <is>
-          <t>VLINE8028</t>
+          <t>VL139</t>
         </is>
       </c>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>VLINE8030</t>
+          <t>VL140</t>
         </is>
       </c>
     </row>
     <row r="605">
       <c r="A605" s="2" t="inlineStr">
         <is>
-          <t>VLINE8034</t>
+          <t>VL354</t>
         </is>
       </c>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>VLINE8036</t>
+          <t>VLINE8013</t>
         </is>
       </c>
     </row>
     <row r="607">
       <c r="A607" s="2" t="inlineStr">
         <is>
-          <t>VLINE8058</t>
+          <t>VLINE8020</t>
         </is>
       </c>
     </row>
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>VLINE8059</t>
+          <t>VLINE8021</t>
         </is>
       </c>
     </row>
     <row r="609">
       <c r="A609" s="2" t="inlineStr">
         <is>
-          <t>VLINE8061</t>
+          <t>VLINE8023</t>
         </is>
       </c>
     </row>
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>VLINE8071</t>
+          <t>VLINE8025</t>
         </is>
       </c>
     </row>
     <row r="611">
       <c r="A611" s="2" t="inlineStr">
         <is>
-          <t>VLINE8072</t>
+          <t>VLINE8028</t>
         </is>
       </c>
     </row>
     <row r="612">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>VLINE8074</t>
+          <t>VLINE8029</t>
         </is>
       </c>
     </row>
     <row r="613">
       <c r="A613" s="2" t="inlineStr">
         <is>
-          <t>VLINE8075</t>
+          <t>VLINE8030</t>
         </is>
       </c>
     </row>
     <row r="614">
       <c r="A614" s="2" t="inlineStr">
         <is>
-          <t>VLINE8076</t>
+          <t>VLINE8034</t>
         </is>
       </c>
     </row>
     <row r="615">
       <c r="A615" s="2" t="inlineStr">
         <is>
-          <t>VLINE8077</t>
+          <t>VLINE8036</t>
         </is>
       </c>
     </row>
     <row r="616">
       <c r="A616" s="2" t="inlineStr">
         <is>
-          <t>VLINE8080</t>
+          <t>VLINE8038</t>
         </is>
       </c>
     </row>
     <row r="617">
       <c r="A617" s="2" t="inlineStr">
         <is>
-          <t>VLINE8081</t>
+          <t>VLINE8058</t>
         </is>
       </c>
     </row>
     <row r="618">
       <c r="A618" s="2" t="inlineStr">
         <is>
-          <t>VLINE8084</t>
+          <t>VLINE8059</t>
         </is>
       </c>
     </row>
     <row r="619">
       <c r="A619" s="2" t="inlineStr">
         <is>
-          <t>VLINE8102</t>
+          <t>VLINE8061</t>
         </is>
       </c>
     </row>
     <row r="620">
       <c r="A620" s="2" t="inlineStr">
         <is>
-          <t>VLINE8111</t>
+          <t>VLINE8071</t>
         </is>
       </c>
     </row>
     <row r="621">
       <c r="A621" s="2" t="inlineStr">
         <is>
-          <t>VLINE8113</t>
+          <t>VLINE8072</t>
         </is>
       </c>
     </row>
     <row r="622">
       <c r="A622" s="2" t="inlineStr">
         <is>
-          <t>VLINE8115</t>
+          <t>VLINE8074</t>
         </is>
       </c>
     </row>
     <row r="623">
       <c r="A623" s="2" t="inlineStr">
         <is>
-          <t>VLINE8117</t>
+          <t>VLINE8075</t>
         </is>
       </c>
     </row>
     <row r="624">
       <c r="A624" s="2" t="inlineStr">
         <is>
-          <t>VLINE8120</t>
+          <t>VLINE8076</t>
         </is>
       </c>
     </row>
     <row r="625">
       <c r="A625" s="2" t="inlineStr">
         <is>
-          <t>VLINE8121</t>
+          <t>VLINE8077</t>
         </is>
       </c>
     </row>
     <row r="626">
       <c r="A626" s="2" t="inlineStr">
         <is>
-          <t>VLINE8122</t>
+          <t>VLINE8080</t>
         </is>
       </c>
     </row>
     <row r="627">
       <c r="A627" s="2" t="inlineStr">
         <is>
-          <t>VLINE8123</t>
+          <t>VLINE8081</t>
         </is>
       </c>
     </row>
     <row r="628">
       <c r="A628" s="2" t="inlineStr">
         <is>
-          <t>VLINE8124</t>
+          <t>VLINE8084</t>
         </is>
       </c>
     </row>
     <row r="629">
       <c r="A629" s="2" t="inlineStr">
         <is>
-          <t>VLINE8125</t>
+          <t>VLINE8102</t>
         </is>
       </c>
     </row>
     <row r="630">
       <c r="A630" s="2" t="inlineStr">
         <is>
-          <t>VLINE8126</t>
+          <t>VLINE8111</t>
         </is>
       </c>
     </row>
     <row r="631">
       <c r="A631" s="2" t="inlineStr">
         <is>
-          <t>VLINE8127</t>
+          <t>VLINE8113</t>
         </is>
       </c>
     </row>
     <row r="632">
       <c r="A632" s="2" t="inlineStr">
         <is>
-          <t>VLINE8128</t>
+          <t>VLINE8115</t>
         </is>
       </c>
     </row>
     <row r="633">
       <c r="A633" s="2" t="inlineStr">
         <is>
-          <t>VLINE8130</t>
+          <t>VLINE8117</t>
         </is>
       </c>
     </row>
     <row r="634">
       <c r="A634" s="2" t="inlineStr">
         <is>
-          <t>VLINE8131</t>
+          <t>VLINE8120</t>
         </is>
       </c>
     </row>
     <row r="635">
       <c r="A635" s="2" t="inlineStr">
         <is>
-          <t>VLINE8134</t>
+          <t>VLINE8121</t>
         </is>
       </c>
     </row>
     <row r="636">
       <c r="A636" s="2" t="inlineStr">
         <is>
-          <t>VLINE8136</t>
+          <t>VLINE8122</t>
         </is>
       </c>
     </row>
     <row r="637">
       <c r="A637" s="2" t="inlineStr">
         <is>
-          <t>VLINE8138</t>
+          <t>VLINE8123</t>
         </is>
       </c>
     </row>
     <row r="638">
       <c r="A638" s="2" t="inlineStr">
         <is>
-          <t>VLINE8161</t>
+          <t>VLINE8124</t>
         </is>
       </c>
     </row>
     <row r="639">
       <c r="A639" s="2" t="inlineStr">
         <is>
-          <t>VLINE8163</t>
+          <t>VLINE8125</t>
         </is>
       </c>
     </row>
     <row r="640">
       <c r="A640" s="2" t="inlineStr">
         <is>
-          <t>VLINE8164</t>
+          <t>VLINE8126</t>
         </is>
       </c>
     </row>
     <row r="641">
       <c r="A641" s="2" t="inlineStr">
         <is>
-          <t>VLINE8172</t>
+          <t>VLINE8127</t>
         </is>
       </c>
     </row>
     <row r="642">
       <c r="A642" s="2" t="inlineStr">
         <is>
-          <t>VLINE8181</t>
+          <t>VLINE8128</t>
         </is>
       </c>
     </row>
     <row r="643">
       <c r="A643" s="2" t="inlineStr">
         <is>
-          <t>VLINE8183</t>
+          <t>VLINE8130</t>
         </is>
       </c>
     </row>
     <row r="644">
       <c r="A644" s="2" t="inlineStr">
         <is>
-          <t>VLINE8184</t>
+          <t>VLINE8131</t>
         </is>
       </c>
     </row>
     <row r="645">
       <c r="A645" s="2" t="inlineStr">
         <is>
-          <t>VLINE8185</t>
+          <t>VLINE8133</t>
         </is>
       </c>
     </row>
     <row r="646">
       <c r="A646" s="2" t="inlineStr">
         <is>
-          <t>VLINE8186</t>
+          <t>VLINE8134</t>
         </is>
       </c>
     </row>
     <row r="647">
       <c r="A647" s="2" t="inlineStr">
         <is>
-          <t>VLINE8211</t>
+          <t>VLINE8136</t>
         </is>
       </c>
     </row>
     <row r="648">
       <c r="A648" s="2" t="inlineStr">
         <is>
-          <t>VLINE8213</t>
+          <t>VLINE8138</t>
         </is>
       </c>
     </row>
     <row r="649">
       <c r="A649" s="2" t="inlineStr">
         <is>
-          <t>VLINE8215</t>
+          <t>VLINE8142</t>
         </is>
       </c>
     </row>
     <row r="650">
       <c r="A650" s="2" t="inlineStr">
         <is>
-          <t>VLINE8217</t>
+          <t>VLINE8161</t>
         </is>
       </c>
     </row>
     <row r="651">
       <c r="A651" s="2" t="inlineStr">
         <is>
-          <t>VLINE8219</t>
+          <t>VLINE8163</t>
         </is>
       </c>
     </row>
     <row r="652">
       <c r="A652" s="2" t="inlineStr">
         <is>
-          <t>VLINE8221</t>
+          <t>VLINE8164</t>
         </is>
       </c>
     </row>
     <row r="653">
       <c r="A653" s="2" t="inlineStr">
         <is>
-          <t>VLINE8223</t>
+          <t>VLINE8172</t>
         </is>
       </c>
     </row>
     <row r="654">
       <c r="A654" s="2" t="inlineStr">
         <is>
-          <t>VLINE8225</t>
+          <t>VLINE8181</t>
         </is>
       </c>
     </row>
     <row r="655">
       <c r="A655" s="2" t="inlineStr">
         <is>
-          <t>VLINE8226</t>
+          <t>VLINE8183</t>
         </is>
       </c>
     </row>
     <row r="656">
       <c r="A656" s="2" t="inlineStr">
         <is>
-          <t>VLINE8227</t>
+          <t>VLINE8184</t>
         </is>
       </c>
     </row>
     <row r="657">
       <c r="A657" s="2" t="inlineStr">
         <is>
-          <t>VLINE8228</t>
+          <t>VLINE8185</t>
         </is>
       </c>
     </row>
     <row r="658">
       <c r="A658" s="2" t="inlineStr">
         <is>
-          <t>VLINE8229</t>
+          <t>VLINE8186</t>
         </is>
       </c>
     </row>
     <row r="659">
       <c r="A659" s="2" t="inlineStr">
         <is>
-          <t>VLINE8230</t>
+          <t>VLINE8211</t>
         </is>
       </c>
     </row>
     <row r="660">
       <c r="A660" s="2" t="inlineStr">
         <is>
-          <t>VLINE8231</t>
+          <t>VLINE8213</t>
         </is>
       </c>
     </row>
     <row r="661">
       <c r="A661" s="2" t="inlineStr">
         <is>
-          <t>VLINE8232</t>
+          <t>VLINE8215</t>
         </is>
       </c>
     </row>
     <row r="662">
       <c r="A662" s="2" t="inlineStr">
         <is>
-          <t>VLINE8234</t>
+          <t>VLINE8217</t>
         </is>
       </c>
     </row>
     <row r="663">
       <c r="A663" s="2" t="inlineStr">
         <is>
-          <t>VLINE8236</t>
+          <t>VLINE8219</t>
         </is>
       </c>
     </row>
     <row r="664">
       <c r="A664" s="2" t="inlineStr">
         <is>
-          <t>VLINE8238</t>
+          <t>VLINE8221</t>
         </is>
       </c>
     </row>
     <row r="665">
       <c r="A665" s="2" t="inlineStr">
         <is>
-          <t>VLINE8240</t>
+          <t>VLINE8223</t>
         </is>
       </c>
     </row>
     <row r="666">
       <c r="A666" s="2" t="inlineStr">
         <is>
-          <t>VLINE8242</t>
+          <t>VLINE8225</t>
         </is>
       </c>
     </row>
     <row r="667">
       <c r="A667" s="2" t="inlineStr">
         <is>
-          <t>VLINE8244</t>
+          <t>VLINE8226</t>
         </is>
       </c>
     </row>
     <row r="668">
       <c r="A668" s="2" t="inlineStr">
         <is>
-          <t>VLINE8400</t>
+          <t>VLINE8227</t>
         </is>
       </c>
     </row>
     <row r="669">
       <c r="A669" s="2" t="inlineStr">
         <is>
-          <t>VLINE8405</t>
+          <t>VLINE8228</t>
         </is>
       </c>
     </row>
     <row r="670">
       <c r="A670" s="2" t="inlineStr">
         <is>
-          <t>VLINE8408</t>
+          <t>VLINE8229</t>
         </is>
       </c>
     </row>
     <row r="671">
       <c r="A671" s="2" t="inlineStr">
         <is>
-          <t>VLINE8413</t>
+          <t>VLINE8230</t>
         </is>
       </c>
     </row>
     <row r="672">
       <c r="A672" s="2" t="inlineStr">
         <is>
-          <t>VLINE8415</t>
+          <t>VLINE8231</t>
         </is>
       </c>
     </row>
     <row r="673">
       <c r="A673" s="2" t="inlineStr">
         <is>
-          <t>VLINE8417</t>
+          <t>VLINE8232</t>
         </is>
       </c>
     </row>
     <row r="674">
       <c r="A674" s="2" t="inlineStr">
         <is>
-          <t>VLINE8418</t>
+          <t>VLINE8233</t>
         </is>
       </c>
     </row>
     <row r="675">
       <c r="A675" s="2" t="inlineStr">
         <is>
-          <t>VLINE8419</t>
+          <t>VLINE8234</t>
         </is>
       </c>
     </row>
     <row r="676">
       <c r="A676" s="2" t="inlineStr">
         <is>
-          <t>VLINE8420</t>
+          <t>VLINE8236</t>
         </is>
       </c>
     </row>
     <row r="677">
       <c r="A677" s="2" t="inlineStr">
         <is>
-          <t>VLINE8421</t>
+          <t>VLINE8238</t>
         </is>
       </c>
     </row>
     <row r="678">
       <c r="A678" s="2" t="inlineStr">
         <is>
-          <t>VLINE8422</t>
+          <t>VLINE8240</t>
         </is>
       </c>
     </row>
     <row r="679">
       <c r="A679" s="2" t="inlineStr">
         <is>
-          <t>VLINE8423</t>
+          <t>VLINE8242</t>
         </is>
       </c>
     </row>
     <row r="680">
       <c r="A680" s="2" t="inlineStr">
         <is>
-          <t>VLINE8424</t>
+          <t>VLINE8244</t>
         </is>
       </c>
     </row>
     <row r="681">
       <c r="A681" s="2" t="inlineStr">
         <is>
-          <t>VLINE8427</t>
+          <t>VLINE8246</t>
         </is>
       </c>
     </row>
     <row r="682">
       <c r="A682" s="2" t="inlineStr">
         <is>
-          <t>VLINE8428</t>
+          <t>VLINE8400</t>
         </is>
       </c>
     </row>
     <row r="683">
       <c r="A683" s="2" t="inlineStr">
         <is>
-          <t>VLINE8429</t>
+          <t>VLINE8405</t>
         </is>
       </c>
     </row>
     <row r="684">
       <c r="A684" s="2" t="inlineStr">
         <is>
-          <t>VLINE8430</t>
+          <t>VLINE8408</t>
         </is>
       </c>
     </row>
     <row r="685">
       <c r="A685" s="2" t="inlineStr">
         <is>
-          <t>VLINE8431</t>
+          <t>VLINE8413</t>
         </is>
       </c>
     </row>
     <row r="686">
       <c r="A686" s="2" t="inlineStr">
         <is>
-          <t>VLINE8432</t>
+          <t>VLINE8415</t>
         </is>
       </c>
     </row>
     <row r="687">
       <c r="A687" s="2" t="inlineStr">
         <is>
-          <t>VLINE8434</t>
+          <t>VLINE8417</t>
         </is>
       </c>
     </row>
     <row r="688">
       <c r="A688" s="2" t="inlineStr">
         <is>
-          <t>VLINE8438</t>
+          <t>VLINE8418</t>
         </is>
       </c>
     </row>
     <row r="689">
       <c r="A689" s="2" t="inlineStr">
         <is>
-          <t>VLINE8457</t>
+          <t>VLINE8419</t>
         </is>
       </c>
     </row>
     <row r="690">
       <c r="A690" s="2" t="inlineStr">
         <is>
-          <t>VLINE8459</t>
+          <t>VLINE8420</t>
         </is>
       </c>
     </row>
     <row r="691">
       <c r="A691" s="2" t="inlineStr">
         <is>
-          <t>VLINE8460</t>
+          <t>VLINE8421</t>
         </is>
       </c>
     </row>
     <row r="692">
       <c r="A692" s="2" t="inlineStr">
         <is>
-          <t>VLINE8461</t>
+          <t>VLINE8422</t>
         </is>
       </c>
     </row>
     <row r="693">
       <c r="A693" s="2" t="inlineStr">
         <is>
-          <t>VLINE8464</t>
+          <t>VLINE8423</t>
         </is>
       </c>
     </row>
     <row r="694">
       <c r="A694" s="2" t="inlineStr">
         <is>
-          <t>VLINE8465</t>
+          <t>VLINE8424</t>
         </is>
       </c>
     </row>
     <row r="695">
       <c r="A695" s="2" t="inlineStr">
         <is>
-          <t>VLINE8702</t>
+          <t>VLINE8427</t>
         </is>
       </c>
     </row>
     <row r="696">
       <c r="A696" s="2" t="inlineStr">
         <is>
-          <t>VLINE8725</t>
+          <t>VLINE8428</t>
         </is>
       </c>
     </row>
     <row r="697">
       <c r="A697" s="2" t="inlineStr">
         <is>
-          <t>VLINE8727</t>
+          <t>VLINE8429</t>
         </is>
       </c>
     </row>
     <row r="698">
       <c r="A698" s="2" t="inlineStr">
         <is>
-          <t>VLINE8729</t>
+          <t>VLINE8430</t>
         </is>
       </c>
     </row>
     <row r="699">
       <c r="A699" s="2" t="inlineStr">
         <is>
-          <t>VLINE8731</t>
+          <t>VLINE8431</t>
         </is>
       </c>
     </row>
     <row r="700">
       <c r="A700" s="2" t="inlineStr">
         <is>
-          <t>VLINE8733</t>
+          <t>VLINE8432</t>
         </is>
       </c>
     </row>
     <row r="701">
       <c r="A701" s="2" t="inlineStr">
         <is>
-          <t>VLINE8735</t>
+          <t>VLINE8433</t>
         </is>
       </c>
     </row>
     <row r="702">
       <c r="A702" s="2" t="inlineStr">
         <is>
-          <t>VLINE8737</t>
+          <t>VLINE8434</t>
         </is>
       </c>
     </row>
     <row r="703">
       <c r="A703" s="2" t="inlineStr">
         <is>
-          <t>VLINE8739</t>
+          <t>VLINE8438</t>
         </is>
       </c>
     </row>
     <row r="704">
       <c r="A704" s="2" t="inlineStr">
         <is>
-          <t>VLINE8741</t>
+          <t>VLINE8440</t>
         </is>
       </c>
     </row>
     <row r="705">
       <c r="A705" s="2" t="inlineStr">
         <is>
-          <t>VLINE8742</t>
+          <t>VLINE8457</t>
         </is>
       </c>
     </row>
     <row r="706">
       <c r="A706" s="2" t="inlineStr">
         <is>
-          <t>VLINE8743</t>
+          <t>VLINE8459</t>
         </is>
       </c>
     </row>
     <row r="707">
       <c r="A707" s="2" t="inlineStr">
         <is>
-          <t>VLINE8744</t>
+          <t>VLINE8460</t>
         </is>
       </c>
     </row>
     <row r="708">
       <c r="A708" s="2" t="inlineStr">
         <is>
-          <t>VLINE8745</t>
+          <t>VLINE8461</t>
         </is>
       </c>
     </row>
     <row r="709">
       <c r="A709" s="2" t="inlineStr">
         <is>
-          <t>VLINE8746</t>
+          <t>VLINE8464</t>
         </is>
       </c>
     </row>
     <row r="710">
       <c r="A710" s="2" t="inlineStr">
         <is>
-          <t>VLINE8747</t>
+          <t>VLINE8465</t>
         </is>
       </c>
     </row>
     <row r="711">
       <c r="A711" s="2" t="inlineStr">
         <is>
-          <t>VLINE8748</t>
+          <t>VLINE8702</t>
         </is>
       </c>
     </row>
     <row r="712">
       <c r="A712" s="2" t="inlineStr">
         <is>
-          <t>VLINE8749</t>
+          <t>VLINE8725</t>
         </is>
       </c>
     </row>
     <row r="713">
       <c r="A713" s="2" t="inlineStr">
         <is>
-          <t>VLINE8750</t>
+          <t>VLINE8727</t>
         </is>
       </c>
     </row>
     <row r="714">
       <c r="A714" s="2" t="inlineStr">
         <is>
-          <t>VLINE8751</t>
+          <t>VLINE8729</t>
         </is>
       </c>
     </row>
     <row r="715">
       <c r="A715" s="2" t="inlineStr">
         <is>
-          <t>VLINE8752</t>
+          <t>VLINE8731</t>
         </is>
       </c>
     </row>
     <row r="716">
       <c r="A716" s="2" t="inlineStr">
         <is>
-          <t>VLINE8753</t>
+          <t>VLINE8733</t>
         </is>
       </c>
     </row>
     <row r="717">
       <c r="A717" s="2" t="inlineStr">
         <is>
-          <t>VLINE8754</t>
+          <t>VLINE8735</t>
         </is>
       </c>
     </row>
     <row r="718">
       <c r="A718" s="2" t="inlineStr">
         <is>
-          <t>VLINE8755</t>
+          <t>VLINE8737</t>
         </is>
       </c>
     </row>
     <row r="719">
       <c r="A719" s="2" t="inlineStr">
         <is>
-          <t>VLINE8756</t>
+          <t>VLINE8739</t>
         </is>
       </c>
     </row>
     <row r="720">
       <c r="A720" s="2" t="inlineStr">
         <is>
-          <t>VLINE8757</t>
+          <t>VLINE8741</t>
         </is>
       </c>
     </row>
     <row r="721">
       <c r="A721" s="2" t="inlineStr">
         <is>
-          <t>VLINE8758</t>
+          <t>VLINE8742</t>
         </is>
       </c>
     </row>
     <row r="722">
       <c r="A722" s="2" t="inlineStr">
         <is>
-          <t>VLINE8759</t>
+          <t>VLINE8743</t>
         </is>
       </c>
     </row>
     <row r="723">
       <c r="A723" s="2" t="inlineStr">
         <is>
-          <t>VLINE8760</t>
+          <t>VLINE8744</t>
         </is>
       </c>
     </row>
     <row r="724">
       <c r="A724" s="2" t="inlineStr">
         <is>
-          <t>VLINE8761</t>
+          <t>VLINE8745</t>
         </is>
       </c>
     </row>
     <row r="725">
       <c r="A725" s="2" t="inlineStr">
         <is>
-          <t>VLINE8762</t>
+          <t>VLINE8746</t>
         </is>
       </c>
     </row>
     <row r="726">
       <c r="A726" s="2" t="inlineStr">
         <is>
-          <t>VLINE8763</t>
+          <t>VLINE8747</t>
         </is>
       </c>
     </row>
     <row r="727">
       <c r="A727" s="2" t="inlineStr">
         <is>
-          <t>VLINE8764</t>
+          <t>VLINE8748</t>
         </is>
       </c>
     </row>
     <row r="728">
       <c r="A728" s="2" t="inlineStr">
         <is>
-          <t>VLINE8765</t>
+          <t>VLINE8749</t>
         </is>
       </c>
     </row>
     <row r="729">
       <c r="A729" s="2" t="inlineStr">
         <is>
-          <t>VLINE8766</t>
+          <t>VLINE8750</t>
         </is>
       </c>
     </row>
     <row r="730">
       <c r="A730" s="2" t="inlineStr">
         <is>
-          <t>VLINE8768</t>
+          <t>VLINE8751</t>
         </is>
       </c>
     </row>
     <row r="731">
       <c r="A731" s="2" t="inlineStr">
         <is>
-          <t>VLINE8770</t>
+          <t>VLINE8752</t>
         </is>
       </c>
     </row>
     <row r="732">
       <c r="A732" s="2" t="inlineStr">
         <is>
-          <t>VLINE8772</t>
+          <t>VLINE8753</t>
         </is>
       </c>
     </row>
     <row r="733">
       <c r="A733" s="2" t="inlineStr">
         <is>
-          <t>VLINE8774</t>
+          <t>VLINE8754</t>
         </is>
       </c>
     </row>
     <row r="734">
       <c r="A734" s="2" t="inlineStr">
         <is>
-          <t>VLINE8776</t>
+          <t>VLINE8755</t>
         </is>
       </c>
     </row>
     <row r="735">
       <c r="A735" s="2" t="inlineStr">
         <is>
-          <t>VLINE8778</t>
+          <t>VLINE8756</t>
         </is>
       </c>
     </row>
     <row r="736">
       <c r="A736" s="2" t="inlineStr">
         <is>
-          <t>VLINE8780</t>
+          <t>VLINE8757</t>
         </is>
       </c>
     </row>
     <row r="737">
       <c r="A737" s="2" t="inlineStr">
         <is>
-          <t>VLINE8782</t>
+          <t>VLINE8758</t>
         </is>
       </c>
     </row>
     <row r="738">
       <c r="A738" s="2" t="inlineStr">
         <is>
-          <t>VLINE8819</t>
+          <t>VLINE8759</t>
         </is>
       </c>
     </row>
     <row r="739">
       <c r="A739" s="2" t="inlineStr">
         <is>
-          <t>VLINE8862</t>
+          <t>VLINE8760</t>
         </is>
       </c>
     </row>
     <row r="740">
       <c r="A740" s="2" t="inlineStr">
         <is>
-          <t>VLINE8863</t>
+          <t>VLINE8761</t>
         </is>
       </c>
     </row>
     <row r="741">
       <c r="A741" s="2" t="inlineStr">
         <is>
-          <t>VLINE8864</t>
+          <t>VLINE8762</t>
         </is>
       </c>
     </row>
     <row r="742">
       <c r="A742" s="2" t="inlineStr">
         <is>
-          <t>VLINE8865</t>
+          <t>VLINE8763</t>
         </is>
       </c>
     </row>
     <row r="743">
       <c r="A743" s="2" t="inlineStr">
         <is>
-          <t>VR76</t>
+          <t>VLINE8764</t>
         </is>
       </c>
     </row>
     <row r="744">
       <c r="A744" s="2" t="inlineStr">
         <is>
-          <t>VR77</t>
+          <t>VLINE8765</t>
         </is>
       </c>
     </row>
     <row r="745">
       <c r="A745" s="2" t="inlineStr">
         <is>
-          <t>WOLL408</t>
+          <t>VLINE8766</t>
         </is>
       </c>
     </row>
     <row r="746">
       <c r="A746" s="2" t="inlineStr">
         <is>
-          <t>WOLL430</t>
+          <t>VLINE8767</t>
         </is>
       </c>
     </row>
     <row r="747">
       <c r="A747" s="2" t="inlineStr">
         <is>
-          <t>X21</t>
+          <t>VLINE8768</t>
         </is>
       </c>
     </row>
     <row r="748">
       <c r="A748" s="2" t="inlineStr">
         <is>
-          <t>XP2001</t>
+          <t>VLINE8770</t>
         </is>
       </c>
     </row>
     <row r="749">
       <c r="A749" s="2" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>VLINE8772</t>
         </is>
       </c>
     </row>
     <row r="750">
       <c r="A750" s="2" t="inlineStr">
         <is>
-          <t>XP2006</t>
+          <t>VLINE8774</t>
         </is>
       </c>
     </row>
     <row r="751">
       <c r="A751" s="2" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>VLINE8776</t>
         </is>
       </c>
     </row>
     <row r="752">
       <c r="A752" s="2" t="inlineStr">
         <is>
-          <t>XP2009</t>
+          <t>VLINE8778</t>
         </is>
       </c>
     </row>
     <row r="753">
       <c r="A753" s="2" t="inlineStr">
         <is>
-          <t>XP2010</t>
+          <t>VLINE8780</t>
         </is>
       </c>
     </row>
     <row r="754">
       <c r="A754" s="2" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>VLINE8782</t>
         </is>
       </c>
     </row>
     <row r="755">
       <c r="A755" s="2" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>VLINE8784</t>
         </is>
       </c>
     </row>
     <row r="756">
       <c r="A756" s="2" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>VLINE8786</t>
         </is>
       </c>
     </row>
     <row r="757">
       <c r="A757" s="2" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>VLINE8819</t>
         </is>
       </c>
     </row>
     <row r="758">
       <c r="A758" s="2" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>VLINE8862</t>
         </is>
       </c>
     </row>
     <row r="759">
       <c r="A759" s="2" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>VLINE8863</t>
         </is>
       </c>
     </row>
     <row r="760">
       <c r="A760" s="2" t="inlineStr">
         <is>
-          <t>XRN003</t>
+          <t>VLINE8864</t>
         </is>
       </c>
     </row>
     <row r="761">
       <c r="A761" s="2" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>VLINE8865</t>
         </is>
       </c>
     </row>
     <row r="762">
       <c r="A762" s="2" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>VLINE8933</t>
         </is>
       </c>
     </row>
     <row r="763">
       <c r="A763" s="2" t="inlineStr">
         <is>
-          <t>XRN010</t>
+          <t>VLINE8935</t>
         </is>
       </c>
     </row>
     <row r="764">
       <c r="A764" s="2" t="inlineStr">
         <is>
-          <t>XRN012</t>
+          <t>VR76</t>
         </is>
       </c>
     </row>
     <row r="765">
       <c r="A765" s="2" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>VR77</t>
         </is>
       </c>
     </row>
     <row r="766">
       <c r="A766" s="2" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>WOLL408</t>
         </is>
       </c>
     </row>
     <row r="767">
       <c r="A767" s="2" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>WOLL430</t>
         </is>
       </c>
     </row>
     <row r="768">
       <c r="A768" s="2" t="inlineStr">
         <is>
-          <t>XRN022</t>
+          <t>X21</t>
         </is>
       </c>
     </row>
     <row r="769">
       <c r="A769" s="2" t="inlineStr">
         <is>
-          <t>XRN028</t>
+          <t>XP2001</t>
         </is>
       </c>
     </row>
     <row r="770">
       <c r="A770" s="2" t="inlineStr">
+        <is>
+          <t>XP2005</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" s="2" t="inlineStr">
+        <is>
+          <t>XP2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" s="2" t="inlineStr">
+        <is>
+          <t>XP2008</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" s="2" t="inlineStr">
+        <is>
+          <t>XP2009</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" s="2" t="inlineStr">
+        <is>
+          <t>XP2010</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" s="2" t="inlineStr">
+        <is>
+          <t>XP2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="2" t="inlineStr">
+        <is>
+          <t>XP2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" s="2" t="inlineStr">
+        <is>
+          <t>XP2013</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="2" t="inlineStr">
+        <is>
+          <t>XP2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="2" t="inlineStr">
+        <is>
+          <t>XP2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="2" t="inlineStr">
+        <is>
+          <t>XP2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="2" t="inlineStr">
+        <is>
+          <t>XRN003</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="2" t="inlineStr">
+        <is>
+          <t>XRN005</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="2" t="inlineStr">
+        <is>
+          <t>XRN009</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="2" t="inlineStr">
+        <is>
+          <t>XRN010</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="2" t="inlineStr">
+        <is>
+          <t>XRN012</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" s="2" t="inlineStr">
+        <is>
+          <t>XRN017</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="2" t="inlineStr">
+        <is>
+          <t>XRN018</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" s="2" t="inlineStr">
+        <is>
+          <t>XRN021</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="2" t="inlineStr">
+        <is>
+          <t>XRN022</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" s="2" t="inlineStr">
+        <is>
+          <t>XRN028</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="2" t="inlineStr">
         <is>
           <t>XRN029</t>
         </is>

</xml_diff>

<commit_message>
Update RailOps database files - 2026-04-30 06:33:59 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A791"/>
+  <dimension ref="A1:A814"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2197,3792 +2197,3953 @@
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>MM92M</t>
+          <t>MM88M</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>MM94M</t>
+          <t>MM92M</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>MM96M</t>
+          <t>MM94M</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>MM98M</t>
+          <t>MM96M</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>MM99M</t>
+          <t>MM98M</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>MM122M</t>
+          <t>MM99M</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>MM130M</t>
+          <t>MM122M</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>MM152M</t>
+          <t>MM130M</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>MM156M</t>
+          <t>MM152M</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>MM158M</t>
+          <t>MM156M</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>MM172M</t>
+          <t>MM158M</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>MM178M</t>
+          <t>MM162M</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>MM192M</t>
+          <t>MM172M</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>MM212M</t>
+          <t>MM178M</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>MM214M</t>
+          <t>MM192M</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>MM216M</t>
+          <t>MM212M</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>MM224M</t>
+          <t>MM214M</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>MM232M</t>
+          <t>MM216M</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>MM236M</t>
+          <t>MM224M</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>MM240M</t>
+          <t>MM232M</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>MM246M</t>
+          <t>MM236M</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>MM256M</t>
+          <t>MM240M</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>MM258M</t>
+          <t>MM242M</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>MM260M</t>
+          <t>MM246M</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>MM264M</t>
+          <t>MM256M</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>MM266M</t>
+          <t>MM258M</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>MM268M</t>
+          <t>MM260M</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>MM270M</t>
+          <t>MM264M</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>MM280M</t>
+          <t>MM266M</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>MM288M</t>
+          <t>MM268M</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>MM380M</t>
+          <t>MM270M</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>MM384M</t>
+          <t>MM280M</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>MM418M</t>
+          <t>MM288M</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>MM424M</t>
+          <t>MM380M</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>MM456M</t>
+          <t>MM384M</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>MM464M</t>
+          <t>MM418M</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>MM478M</t>
+          <t>MM424M</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>MM482M</t>
+          <t>MM456M</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>MM486M</t>
+          <t>MM464M</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>MM502M</t>
+          <t>MM478M</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>MM506M</t>
+          <t>MM482M</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>MM514M</t>
+          <t>MM486M</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>MM522M</t>
+          <t>MM502M</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>MM536M</t>
+          <t>MM506M</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>MM542M</t>
+          <t>MM514M</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>MM544M</t>
+          <t>MM522M</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>MM546M</t>
+          <t>MM536M</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>MM551M</t>
+          <t>MM542M</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>MM552M</t>
+          <t>MM544M</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>MM566M</t>
+          <t>MM546M</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>MM574M</t>
+          <t>MM551M</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>MM588M</t>
+          <t>MM552M</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>MM592M</t>
+          <t>MM566M</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>MM602M</t>
+          <t>MM574M</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>MM604M</t>
+          <t>MM588M</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>MM620M</t>
+          <t>MM592M</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>MM624M</t>
+          <t>MM602M</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>MM636M</t>
+          <t>MM604M</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>MM638M</t>
+          <t>MM608M</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>MM647M</t>
+          <t>MM620M</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>MM656M</t>
+          <t>MM624M</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>MM658M</t>
+          <t>MM636M</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>MM660M</t>
+          <t>MM638M</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>MM662M</t>
+          <t>MM647M</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>MM664M</t>
+          <t>MM656M</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>MM668M</t>
+          <t>MM658M</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>MM673M</t>
+          <t>MM660M</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>MM674M</t>
+          <t>MM661M</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>MM676M</t>
+          <t>MM662M</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>MM680M</t>
+          <t>MM664M</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>MM702M</t>
+          <t>MM668M</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>MM708M</t>
+          <t>MM673M</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>MM718M</t>
+          <t>MM674M</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>MM742M</t>
+          <t>MM676M</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>MM744M</t>
+          <t>MM678M</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>MM752M</t>
+          <t>MM680M</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>MM756M</t>
+          <t>MM702M</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>MM760M</t>
+          <t>MM708M</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>MM766M</t>
+          <t>MM718M</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>MM768M</t>
+          <t>MM742M</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>MM772M</t>
+          <t>MM744M</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>MM774M</t>
+          <t>MM752M</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>MM776M</t>
+          <t>MM756M</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>MM778M</t>
+          <t>MM760M</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>MM780M</t>
+          <t>MM766M</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>MM784M</t>
+          <t>MM768M</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>MM788M</t>
+          <t>MM772M</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>MM790M</t>
+          <t>MM774M</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>MM794M</t>
+          <t>MM776M</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>MM798M</t>
+          <t>MM778M</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>MM800M</t>
+          <t>MM780M</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>MM802M</t>
+          <t>MM784M</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>MM806M</t>
+          <t>MM788M</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>MM808M</t>
+          <t>MM790M</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>MM810M</t>
+          <t>MM794M</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>MM816M</t>
+          <t>MM798M</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>MM820M</t>
+          <t>MM800M</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>MM826M</t>
+          <t>MM802M</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>MM830M</t>
+          <t>MM806M</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>MM832M</t>
+          <t>MM808M</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>MM834M</t>
+          <t>MM810M</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>MM836M</t>
+          <t>MM816M</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>MM838M</t>
+          <t>MM820M</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>MM842M</t>
+          <t>MM826M</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>MM858M</t>
+          <t>MM830M</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>MM860M</t>
+          <t>MM832M</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>MM862M</t>
+          <t>MM834M</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>MM864M</t>
+          <t>MM836M</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>MM866M</t>
+          <t>MM838M</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>MM872M</t>
+          <t>MM840M</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>MM878M</t>
+          <t>MM842M</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>MM880M</t>
+          <t>MM844M</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>MM882M</t>
+          <t>MM858M</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>MM886M</t>
+          <t>MM860M</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>MM896M</t>
+          <t>MM862M</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>MM908M</t>
+          <t>MM864M</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>MM910M</t>
+          <t>MM866M</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>MM912M</t>
+          <t>MM872M</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>MM914M</t>
+          <t>MM878M</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>MM922M</t>
+          <t>MM880M</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>MM924M</t>
+          <t>MM882M</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>MM928M</t>
+          <t>MM886M</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>MM934M</t>
+          <t>MM896M</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t>MM940M</t>
+          <t>MM908M</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>MM944M</t>
+          <t>MM910M</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t>MM946M</t>
+          <t>MM912M</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>MM952M</t>
+          <t>MM914M</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>MM956M</t>
+          <t>MM918M</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>MM958M</t>
+          <t>MM922M</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>MM960M</t>
+          <t>MM924M</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>MM962M</t>
+          <t>MM928M</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>MM964M</t>
+          <t>MM934M</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>MM968M</t>
+          <t>MM940M</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
         <is>
-          <t>MM970M</t>
+          <t>MM944M</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>MM972M</t>
+          <t>MM946M</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
         <is>
-          <t>MM974M</t>
+          <t>MM950M</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
         <is>
-          <t>MM976M</t>
+          <t>MM952M</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" s="2" t="inlineStr">
         <is>
-          <t>MM980M</t>
+          <t>MM956M</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
         <is>
-          <t>MM982M</t>
+          <t>MM958M</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
         <is>
-          <t>MM984M</t>
+          <t>MM960M</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>MM9901M</t>
+          <t>MM962M</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
         <is>
-          <t>MM9903M</t>
+          <t>MM964M</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
         <is>
-          <t>MM9904M</t>
+          <t>MM968M</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="2" t="inlineStr">
         <is>
-          <t>MM9905M</t>
+          <t>MM970M</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
         <is>
-          <t>MM9906M</t>
+          <t>MM972M</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" s="2" t="inlineStr">
         <is>
-          <t>MM9908M</t>
+          <t>MM974M</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
         <is>
-          <t>MM9909M</t>
+          <t>MM976M</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="2" t="inlineStr">
         <is>
-          <t>MM9910M</t>
+          <t>MM980M</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" s="2" t="inlineStr">
         <is>
-          <t>MM9912M</t>
+          <t>MM982M</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="2" t="inlineStr">
         <is>
-          <t>MM9914M</t>
+          <t>MM984M</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
         <is>
-          <t>MM9916M</t>
+          <t>MM9901M</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" s="2" t="inlineStr">
         <is>
-          <t>MM9918M</t>
+          <t>MM9903M</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
         <is>
-          <t>MM9919M</t>
+          <t>MM9904M</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" s="2" t="inlineStr">
         <is>
-          <t>MM9920M</t>
+          <t>MM9905M</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" s="2" t="inlineStr">
         <is>
-          <t>MM9921M</t>
+          <t>MM9906M</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
         <is>
-          <t>MM9922M</t>
+          <t>MM9907M</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="2" t="inlineStr">
         <is>
-          <t>MM9924M</t>
+          <t>MM9908M</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
         <is>
-          <t>MM9926M</t>
+          <t>MM9909M</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="2" t="inlineStr">
         <is>
-          <t>MM9927M</t>
+          <t>MM9910M</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="2" t="inlineStr">
         <is>
-          <t>MM9928M</t>
+          <t>MM9912M</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" s="2" t="inlineStr">
         <is>
-          <t>MM9929M</t>
+          <t>MM9914M</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" s="2" t="inlineStr">
         <is>
-          <t>MM9931M</t>
+          <t>MM9916M</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" s="2" t="inlineStr">
         <is>
-          <t>MM9933M</t>
+          <t>MM9918M</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" s="2" t="inlineStr">
         <is>
-          <t>MM9936M</t>
+          <t>MM9919M</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" s="2" t="inlineStr">
         <is>
-          <t>MM9937M</t>
+          <t>MM9920M</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" s="2" t="inlineStr">
         <is>
-          <t>MM9938M</t>
+          <t>MM9921M</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" s="2" t="inlineStr">
         <is>
-          <t>MM9941M</t>
+          <t>MM9922M</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" s="2" t="inlineStr">
         <is>
-          <t>MM9943M</t>
+          <t>MM9924M</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t>MM9946M</t>
+          <t>MM9926M</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" s="2" t="inlineStr">
         <is>
-          <t>MM9947M</t>
+          <t>MM9927M</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
         <is>
-          <t>MM9948M</t>
+          <t>MM9928M</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" s="2" t="inlineStr">
         <is>
-          <t>MM9952M</t>
+          <t>MM9929M</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" s="2" t="inlineStr">
         <is>
-          <t>MM9953M</t>
+          <t>MM9930M</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" s="2" t="inlineStr">
         <is>
-          <t>MM9954M</t>
+          <t>MM9931M</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
         <is>
-          <t>MM9956M</t>
+          <t>MM9933M</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="2" t="inlineStr">
         <is>
-          <t>MM9957M</t>
+          <t>MM9936M</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
         <is>
-          <t>MM9958M</t>
+          <t>MM9937M</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
         <is>
-          <t>MM9959M</t>
+          <t>MM9938M</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>MM9960M</t>
+          <t>MM9941M</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" s="2" t="inlineStr">
         <is>
-          <t>MM9961M</t>
+          <t>MM9943M</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
         <is>
-          <t>MM9962M</t>
+          <t>MM9946M</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" s="2" t="inlineStr">
         <is>
-          <t>MM9963M</t>
+          <t>MM9947M</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
         <is>
-          <t>MM9964M</t>
+          <t>MM9948M</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" s="2" t="inlineStr">
         <is>
-          <t>MM9965M</t>
+          <t>MM9952M</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t>MM9966M</t>
+          <t>MM9953M</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t>MM9968M</t>
+          <t>MM9954M</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>MM9969M</t>
+          <t>MM9956M</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
         <is>
-          <t>MM9970M</t>
+          <t>MM9957M</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MM9958M</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
         <is>
-          <t>MRL002</t>
+          <t>MM9959M</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
         <is>
-          <t>MTPV1</t>
+          <t>MM9960M</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
         <is>
-          <t>MTPV2</t>
+          <t>MM9961M</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>N453</t>
+          <t>MM9962M</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
         <is>
-          <t>N458</t>
+          <t>MM9963M</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>N460</t>
+          <t>MM9964M</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>MM9965M</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>MM9966M</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>MM9968M</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>MM9969M</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
         <is>
-          <t>NR6</t>
+          <t>MM9970M</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>NR10</t>
+          <t>MRL001</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
         <is>
-          <t>NR11</t>
+          <t>MRL002</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>NR12</t>
+          <t>MTPV1</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="2" t="inlineStr">
         <is>
-          <t>NR13</t>
+          <t>MTPV2</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
         <is>
-          <t>NR14</t>
+          <t>N453</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" s="2" t="inlineStr">
         <is>
-          <t>NR17</t>
+          <t>N458</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
         <is>
-          <t>NR20</t>
+          <t>N460</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" s="2" t="inlineStr">
         <is>
-          <t>NR31</t>
+          <t>N466</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="2" t="inlineStr">
         <is>
-          <t>NR35</t>
+          <t>N469</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" s="2" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>NR4</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" s="2" t="inlineStr">
         <is>
-          <t>NR44</t>
+          <t>NR5</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" s="2" t="inlineStr">
         <is>
-          <t>NR46</t>
+          <t>NR6</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" s="2" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>NR10</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="2" t="inlineStr">
         <is>
-          <t>NR52</t>
+          <t>NR11</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="2" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>NR12</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="2" t="inlineStr">
         <is>
-          <t>NR56</t>
+          <t>NR13</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="2" t="inlineStr">
         <is>
-          <t>NR60</t>
+          <t>NR14</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="2" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR17</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" s="2" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR20</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" s="2" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR31</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" s="2" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR35</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" s="2" t="inlineStr">
         <is>
-          <t>NR76</t>
+          <t>NR37</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="A472" s="2" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR44</t>
         </is>
       </c>
     </row>
     <row r="473">
       <c r="A473" s="2" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR46</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="A474" s="2" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR47</t>
         </is>
       </c>
     </row>
     <row r="475">
       <c r="A475" s="2" t="inlineStr">
         <is>
-          <t>NR88</t>
+          <t>NR52</t>
         </is>
       </c>
     </row>
     <row r="476">
       <c r="A476" s="2" t="inlineStr">
         <is>
-          <t>NR91</t>
+          <t>NR54</t>
         </is>
       </c>
     </row>
     <row r="477">
       <c r="A477" s="2" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR56</t>
         </is>
       </c>
     </row>
     <row r="478">
       <c r="A478" s="2" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR60</t>
         </is>
       </c>
     </row>
     <row r="479">
       <c r="A479" s="2" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR64</t>
         </is>
       </c>
     </row>
     <row r="480">
       <c r="A480" s="2" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>NR65</t>
         </is>
       </c>
     </row>
     <row r="481">
       <c r="A481" s="2" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR68</t>
         </is>
       </c>
     </row>
     <row r="482">
       <c r="A482" s="2" t="inlineStr">
         <is>
-          <t>NR106</t>
+          <t>NR75</t>
         </is>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="2" t="inlineStr">
         <is>
-          <t>NR107</t>
+          <t>NR76</t>
         </is>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="2" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR78</t>
         </is>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="2" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR82</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="2" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR83</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="2" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR88</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" s="2" t="inlineStr">
         <is>
-          <t>PB4</t>
+          <t>NR91</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" s="2" t="inlineStr">
         <is>
-          <t>PB5</t>
+          <t>NR93</t>
         </is>
       </c>
     </row>
     <row r="490">
       <c r="A490" s="2" t="inlineStr">
         <is>
-          <t>PHC001</t>
+          <t>NR94</t>
         </is>
       </c>
     </row>
     <row r="491">
       <c r="A491" s="2" t="inlineStr">
         <is>
-          <t>PKLA4</t>
+          <t>NR95</t>
         </is>
       </c>
     </row>
     <row r="492">
       <c r="A492" s="2" t="inlineStr">
         <is>
-          <t>Q4004</t>
+          <t>NR97</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="2" t="inlineStr">
         <is>
-          <t>Q4012</t>
+          <t>NR102</t>
         </is>
       </c>
     </row>
     <row r="494">
       <c r="A494" s="2" t="inlineStr">
         <is>
-          <t>Q4013</t>
+          <t>NR106</t>
         </is>
       </c>
     </row>
     <row r="495">
       <c r="A495" s="2" t="inlineStr">
         <is>
-          <t>Q4016</t>
+          <t>NR107</t>
         </is>
       </c>
     </row>
     <row r="496">
       <c r="A496" s="2" t="inlineStr">
         <is>
-          <t>QBX003</t>
+          <t>NR109</t>
         </is>
       </c>
     </row>
     <row r="497">
       <c r="A497" s="2" t="inlineStr">
         <is>
-          <t>QBX004</t>
+          <t>NR112</t>
         </is>
       </c>
     </row>
     <row r="498">
       <c r="A498" s="2" t="inlineStr">
         <is>
-          <t>QE001</t>
+          <t>NR113</t>
         </is>
       </c>
     </row>
     <row r="499">
       <c r="A499" s="2" t="inlineStr">
         <is>
-          <t>QE002</t>
+          <t>NR115</t>
         </is>
       </c>
     </row>
     <row r="500">
       <c r="A500" s="2" t="inlineStr">
         <is>
-          <t>QE003</t>
+          <t>PB4</t>
         </is>
       </c>
     </row>
     <row r="501">
       <c r="A501" s="2" t="inlineStr">
         <is>
-          <t>QL004</t>
+          <t>PB5</t>
         </is>
       </c>
     </row>
     <row r="502">
       <c r="A502" s="2" t="inlineStr">
         <is>
-          <t>QL007</t>
+          <t>PHC001</t>
         </is>
       </c>
     </row>
     <row r="503">
       <c r="A503" s="2" t="inlineStr">
         <is>
-          <t>QL009</t>
+          <t>PKLA4</t>
         </is>
       </c>
     </row>
     <row r="504">
       <c r="A504" s="2" t="inlineStr">
         <is>
-          <t>QL016</t>
+          <t>Q4004</t>
         </is>
       </c>
     </row>
     <row r="505">
       <c r="A505" s="2" t="inlineStr">
         <is>
-          <t>QL019</t>
+          <t>Q4012</t>
         </is>
       </c>
     </row>
     <row r="506">
       <c r="A506" s="2" t="inlineStr">
         <is>
-          <t>QR1744</t>
+          <t>Q4013</t>
         </is>
       </c>
     </row>
     <row r="507">
       <c r="A507" s="2" t="inlineStr">
         <is>
-          <t>QR1771</t>
+          <t>Q4016</t>
         </is>
       </c>
     </row>
     <row r="508">
       <c r="A508" s="2" t="inlineStr">
         <is>
-          <t>QR5400</t>
+          <t>QBX003</t>
         </is>
       </c>
     </row>
     <row r="509">
       <c r="A509" s="2" t="inlineStr">
         <is>
-          <t>QR5404</t>
+          <t>QBX004</t>
         </is>
       </c>
     </row>
     <row r="510">
       <c r="A510" s="2" t="inlineStr">
         <is>
-          <t>RA2302</t>
+          <t>QE001</t>
         </is>
       </c>
     </row>
     <row r="511">
       <c r="A511" s="2" t="inlineStr">
         <is>
-          <t>RA2303</t>
+          <t>QE002</t>
         </is>
       </c>
     </row>
     <row r="512">
       <c r="A512" s="2" t="inlineStr">
         <is>
-          <t>RB2352</t>
+          <t>QE003</t>
         </is>
       </c>
     </row>
     <row r="513">
       <c r="A513" s="2" t="inlineStr">
         <is>
-          <t>RB2353</t>
+          <t>QL004</t>
         </is>
       </c>
     </row>
     <row r="514">
       <c r="A514" s="2" t="inlineStr">
         <is>
-          <t>RL301</t>
+          <t>QL007</t>
         </is>
       </c>
     </row>
     <row r="515">
       <c r="A515" s="2" t="inlineStr">
         <is>
-          <t>RL309</t>
+          <t>QL009</t>
         </is>
       </c>
     </row>
     <row r="516">
       <c r="A516" s="2" t="inlineStr">
         <is>
-          <t>RM93</t>
+          <t>QL016</t>
         </is>
       </c>
     </row>
     <row r="517">
       <c r="A517" s="2" t="inlineStr">
         <is>
-          <t>SCT001</t>
+          <t>QL019</t>
         </is>
       </c>
     </row>
     <row r="518">
       <c r="A518" s="2" t="inlineStr">
         <is>
-          <t>SCT008</t>
+          <t>QR1744</t>
         </is>
       </c>
     </row>
     <row r="519">
       <c r="A519" s="2" t="inlineStr">
         <is>
-          <t>SCT009</t>
+          <t>QR1771</t>
         </is>
       </c>
     </row>
     <row r="520">
       <c r="A520" s="2" t="inlineStr">
         <is>
-          <t>SCT010</t>
+          <t>QR5400</t>
         </is>
       </c>
     </row>
     <row r="521">
       <c r="A521" s="2" t="inlineStr">
         <is>
-          <t>SCT013</t>
+          <t>QR5404</t>
         </is>
       </c>
     </row>
     <row r="522">
       <c r="A522" s="2" t="inlineStr">
         <is>
-          <t>SM636B</t>
+          <t>RA2302</t>
         </is>
       </c>
     </row>
     <row r="523">
       <c r="A523" s="2" t="inlineStr">
         <is>
-          <t>SO3</t>
+          <t>RA2303</t>
         </is>
       </c>
     </row>
     <row r="524">
       <c r="A524" s="2" t="inlineStr">
         <is>
-          <t>SSR101</t>
+          <t>RB2352</t>
         </is>
       </c>
     </row>
     <row r="525">
       <c r="A525" s="2" t="inlineStr">
         <is>
-          <t>SSR102</t>
+          <t>RB2353</t>
         </is>
       </c>
     </row>
     <row r="526">
       <c r="A526" s="2" t="inlineStr">
         <is>
-          <t>SSR103</t>
+          <t>RL301</t>
         </is>
       </c>
     </row>
     <row r="527">
       <c r="A527" s="2" t="inlineStr">
         <is>
-          <t>SSR104</t>
+          <t>RL309</t>
         </is>
       </c>
     </row>
     <row r="528">
       <c r="A528" s="2" t="inlineStr">
         <is>
-          <t>T373</t>
+          <t>RM93</t>
         </is>
       </c>
     </row>
     <row r="529">
       <c r="A529" s="2" t="inlineStr">
         <is>
-          <t>TE2801</t>
+          <t>SCT001</t>
         </is>
       </c>
     </row>
     <row r="530">
       <c r="A530" s="2" t="inlineStr">
         <is>
-          <t>TE2803</t>
+          <t>SCT008</t>
         </is>
       </c>
     </row>
     <row r="531">
       <c r="A531" s="2" t="inlineStr">
         <is>
-          <t>TE2804</t>
+          <t>SCT009</t>
         </is>
       </c>
     </row>
     <row r="532">
       <c r="A532" s="2" t="inlineStr">
         <is>
-          <t>TE2805</t>
+          <t>SCT010</t>
         </is>
       </c>
     </row>
     <row r="533">
       <c r="A533" s="2" t="inlineStr">
         <is>
-          <t>TE2807</t>
+          <t>SCT013</t>
         </is>
       </c>
     </row>
     <row r="534">
       <c r="A534" s="2" t="inlineStr">
         <is>
-          <t>TE2808</t>
+          <t>SM636B</t>
         </is>
       </c>
     </row>
     <row r="535">
       <c r="A535" s="2" t="inlineStr">
         <is>
-          <t>TE2813</t>
+          <t>SO3</t>
         </is>
       </c>
     </row>
     <row r="536">
       <c r="A536" s="2" t="inlineStr">
         <is>
-          <t>TE2814</t>
+          <t>SSR101</t>
         </is>
       </c>
     </row>
     <row r="537">
       <c r="A537" s="2" t="inlineStr">
         <is>
-          <t>TJ096</t>
+          <t>SSR102</t>
         </is>
       </c>
     </row>
     <row r="538">
       <c r="A538" s="2" t="inlineStr">
         <is>
-          <t>TT02</t>
+          <t>SSR103</t>
         </is>
       </c>
     </row>
     <row r="539">
       <c r="A539" s="2" t="inlineStr">
         <is>
-          <t>TT03</t>
+          <t>SSR104</t>
         </is>
       </c>
     </row>
     <row r="540">
       <c r="A540" s="2" t="inlineStr">
         <is>
-          <t>TT04</t>
+          <t>T373</t>
         </is>
       </c>
     </row>
     <row r="541">
       <c r="A541" s="2" t="inlineStr">
         <is>
-          <t>TT05</t>
+          <t>TE2801</t>
         </is>
       </c>
     </row>
     <row r="542">
       <c r="A542" s="2" t="inlineStr">
         <is>
-          <t>TT08</t>
+          <t>TE2803</t>
         </is>
       </c>
     </row>
     <row r="543">
       <c r="A543" s="2" t="inlineStr">
         <is>
-          <t>TT103</t>
+          <t>TE2804</t>
         </is>
       </c>
     </row>
     <row r="544">
       <c r="A544" s="2" t="inlineStr">
         <is>
-          <t>TT104</t>
+          <t>TE2805</t>
         </is>
       </c>
     </row>
     <row r="545">
       <c r="A545" s="2" t="inlineStr">
         <is>
-          <t>TT105</t>
+          <t>TE2807</t>
         </is>
       </c>
     </row>
     <row r="546">
       <c r="A546" s="2" t="inlineStr">
         <is>
-          <t>TT107</t>
+          <t>TE2808</t>
         </is>
       </c>
     </row>
     <row r="547">
       <c r="A547" s="2" t="inlineStr">
         <is>
-          <t>TT110</t>
+          <t>TE2813</t>
         </is>
       </c>
     </row>
     <row r="548">
       <c r="A548" s="2" t="inlineStr">
         <is>
-          <t>TT115</t>
+          <t>TE2814</t>
         </is>
       </c>
     </row>
     <row r="549">
       <c r="A549" s="2" t="inlineStr">
         <is>
-          <t>TT117</t>
+          <t>TJ096</t>
         </is>
       </c>
     </row>
     <row r="550">
       <c r="A550" s="2" t="inlineStr">
         <is>
-          <t>TT123</t>
+          <t>TT02</t>
         </is>
       </c>
     </row>
     <row r="551">
       <c r="A551" s="2" t="inlineStr">
         <is>
-          <t>TT126</t>
+          <t>TT03</t>
         </is>
       </c>
     </row>
     <row r="552">
       <c r="A552" s="2" t="inlineStr">
         <is>
-          <t>TT129</t>
+          <t>TT04</t>
         </is>
       </c>
     </row>
     <row r="553">
       <c r="A553" s="2" t="inlineStr">
         <is>
-          <t>TT130</t>
+          <t>TT05</t>
         </is>
       </c>
     </row>
     <row r="554">
       <c r="A554" s="2" t="inlineStr">
         <is>
-          <t>TT202</t>
+          <t>TT08</t>
         </is>
       </c>
     </row>
     <row r="555">
       <c r="A555" s="2" t="inlineStr">
         <is>
-          <t>TT206</t>
+          <t>TT103</t>
         </is>
       </c>
     </row>
     <row r="556">
       <c r="A556" s="2" t="inlineStr">
         <is>
-          <t>VL01</t>
+          <t>TT104</t>
         </is>
       </c>
     </row>
     <row r="557">
       <c r="A557" s="2" t="inlineStr">
         <is>
-          <t>VL03</t>
+          <t>TT105</t>
         </is>
       </c>
     </row>
     <row r="558">
       <c r="A558" s="2" t="inlineStr">
         <is>
-          <t>VL04</t>
+          <t>TT107</t>
         </is>
       </c>
     </row>
     <row r="559">
       <c r="A559" s="2" t="inlineStr">
         <is>
-          <t>VL11</t>
+          <t>TT110</t>
         </is>
       </c>
     </row>
     <row r="560">
       <c r="A560" s="2" t="inlineStr">
         <is>
-          <t>VL13</t>
+          <t>TT115</t>
         </is>
       </c>
     </row>
     <row r="561">
       <c r="A561" s="2" t="inlineStr">
         <is>
-          <t>VL20</t>
+          <t>TT117</t>
         </is>
       </c>
     </row>
     <row r="562">
       <c r="A562" s="2" t="inlineStr">
         <is>
-          <t>VL22</t>
+          <t>TT123</t>
         </is>
       </c>
     </row>
     <row r="563">
       <c r="A563" s="2" t="inlineStr">
         <is>
-          <t>VL27</t>
+          <t>TT126</t>
         </is>
       </c>
     </row>
     <row r="564">
       <c r="A564" s="2" t="inlineStr">
         <is>
-          <t>VL30</t>
+          <t>TT129</t>
         </is>
       </c>
     </row>
     <row r="565">
       <c r="A565" s="2" t="inlineStr">
         <is>
-          <t>VL35</t>
+          <t>TT130</t>
         </is>
       </c>
     </row>
     <row r="566">
       <c r="A566" s="2" t="inlineStr">
         <is>
-          <t>VL36</t>
+          <t>TT202</t>
         </is>
       </c>
     </row>
     <row r="567">
       <c r="A567" s="2" t="inlineStr">
         <is>
-          <t>VL38</t>
+          <t>TT206</t>
         </is>
       </c>
     </row>
     <row r="568">
       <c r="A568" s="2" t="inlineStr">
         <is>
-          <t>VL43</t>
+          <t>VL01</t>
         </is>
       </c>
     </row>
     <row r="569">
       <c r="A569" s="2" t="inlineStr">
         <is>
-          <t>VL47</t>
+          <t>VL03</t>
         </is>
       </c>
     </row>
     <row r="570">
       <c r="A570" s="2" t="inlineStr">
         <is>
-          <t>VL49</t>
+          <t>VL04</t>
         </is>
       </c>
     </row>
     <row r="571">
       <c r="A571" s="2" t="inlineStr">
         <is>
-          <t>VL54</t>
+          <t>VL11</t>
         </is>
       </c>
     </row>
     <row r="572">
       <c r="A572" s="2" t="inlineStr">
         <is>
-          <t>VL57</t>
+          <t>VL13</t>
         </is>
       </c>
     </row>
     <row r="573">
       <c r="A573" s="2" t="inlineStr">
         <is>
-          <t>VL62</t>
+          <t>VL20</t>
         </is>
       </c>
     </row>
     <row r="574">
       <c r="A574" s="2" t="inlineStr">
         <is>
-          <t>VL67</t>
+          <t>VL22</t>
         </is>
       </c>
     </row>
     <row r="575">
       <c r="A575" s="2" t="inlineStr">
         <is>
-          <t>VL68</t>
+          <t>VL27</t>
         </is>
       </c>
     </row>
     <row r="576">
       <c r="A576" s="2" t="inlineStr">
         <is>
-          <t>VL75</t>
+          <t>VL30</t>
         </is>
       </c>
     </row>
     <row r="577">
       <c r="A577" s="2" t="inlineStr">
         <is>
-          <t>VL81</t>
+          <t>VL35</t>
         </is>
       </c>
     </row>
     <row r="578">
       <c r="A578" s="2" t="inlineStr">
         <is>
-          <t>VL86</t>
+          <t>VL36</t>
         </is>
       </c>
     </row>
     <row r="579">
       <c r="A579" s="2" t="inlineStr">
         <is>
-          <t>VL87</t>
+          <t>VL38</t>
         </is>
       </c>
     </row>
     <row r="580">
       <c r="A580" s="2" t="inlineStr">
         <is>
-          <t>VL88</t>
+          <t>VL43</t>
         </is>
       </c>
     </row>
     <row r="581">
       <c r="A581" s="2" t="inlineStr">
         <is>
-          <t>VL90</t>
+          <t>VL47</t>
         </is>
       </c>
     </row>
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>VL92</t>
+          <t>VL49</t>
         </is>
       </c>
     </row>
     <row r="583">
       <c r="A583" s="2" t="inlineStr">
         <is>
-          <t>VL99</t>
+          <t>VL54</t>
         </is>
       </c>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>VL100</t>
+          <t>VL57</t>
         </is>
       </c>
     </row>
     <row r="585">
       <c r="A585" s="2" t="inlineStr">
         <is>
-          <t>VL101</t>
+          <t>VL62</t>
         </is>
       </c>
     </row>
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>VL103</t>
+          <t>VL67</t>
         </is>
       </c>
     </row>
     <row r="587">
       <c r="A587" s="2" t="inlineStr">
         <is>
-          <t>VL106</t>
+          <t>VL68</t>
         </is>
       </c>
     </row>
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>VL107</t>
+          <t>VL75</t>
         </is>
       </c>
     </row>
     <row r="589">
       <c r="A589" s="2" t="inlineStr">
         <is>
-          <t>VL112</t>
+          <t>VL81</t>
         </is>
       </c>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>VL114</t>
+          <t>VL86</t>
         </is>
       </c>
     </row>
     <row r="591">
       <c r="A591" s="2" t="inlineStr">
         <is>
-          <t>VL115</t>
+          <t>VL87</t>
         </is>
       </c>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>VL121</t>
+          <t>VL88</t>
         </is>
       </c>
     </row>
     <row r="593">
       <c r="A593" s="2" t="inlineStr">
         <is>
-          <t>VL122</t>
+          <t>VL90</t>
         </is>
       </c>
     </row>
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>VL123</t>
+          <t>VL92</t>
         </is>
       </c>
     </row>
     <row r="595">
       <c r="A595" s="2" t="inlineStr">
         <is>
-          <t>VL124</t>
+          <t>VL99</t>
         </is>
       </c>
     </row>
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>VL125</t>
+          <t>VL100</t>
         </is>
       </c>
     </row>
     <row r="597">
       <c r="A597" s="2" t="inlineStr">
         <is>
-          <t>VL126</t>
+          <t>VL101</t>
         </is>
       </c>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>VL127</t>
+          <t>VL103</t>
         </is>
       </c>
     </row>
     <row r="599">
       <c r="A599" s="2" t="inlineStr">
         <is>
-          <t>VL129</t>
+          <t>VL106</t>
         </is>
       </c>
     </row>
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>VL132</t>
+          <t>VL107</t>
         </is>
       </c>
     </row>
     <row r="601">
       <c r="A601" s="2" t="inlineStr">
         <is>
-          <t>VL134</t>
+          <t>VL112</t>
         </is>
       </c>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>VL137</t>
+          <t>VL114</t>
         </is>
       </c>
     </row>
     <row r="603">
       <c r="A603" s="2" t="inlineStr">
         <is>
-          <t>VL139</t>
+          <t>VL115</t>
         </is>
       </c>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>VL140</t>
+          <t>VL121</t>
         </is>
       </c>
     </row>
     <row r="605">
       <c r="A605" s="2" t="inlineStr">
         <is>
-          <t>VL354</t>
+          <t>VL122</t>
         </is>
       </c>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>VLINE8013</t>
+          <t>VL123</t>
         </is>
       </c>
     </row>
     <row r="607">
       <c r="A607" s="2" t="inlineStr">
         <is>
-          <t>VLINE8020</t>
+          <t>VL124</t>
         </is>
       </c>
     </row>
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>VLINE8021</t>
+          <t>VL125</t>
         </is>
       </c>
     </row>
     <row r="609">
       <c r="A609" s="2" t="inlineStr">
         <is>
-          <t>VLINE8023</t>
+          <t>VL126</t>
         </is>
       </c>
     </row>
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>VLINE8025</t>
+          <t>VL127</t>
         </is>
       </c>
     </row>
     <row r="611">
       <c r="A611" s="2" t="inlineStr">
         <is>
-          <t>VLINE8028</t>
+          <t>VL129</t>
         </is>
       </c>
     </row>
     <row r="612">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>VLINE8029</t>
+          <t>VL132</t>
         </is>
       </c>
     </row>
     <row r="613">
       <c r="A613" s="2" t="inlineStr">
         <is>
-          <t>VLINE8030</t>
+          <t>VL134</t>
         </is>
       </c>
     </row>
     <row r="614">
       <c r="A614" s="2" t="inlineStr">
         <is>
-          <t>VLINE8034</t>
+          <t>VL137</t>
         </is>
       </c>
     </row>
     <row r="615">
       <c r="A615" s="2" t="inlineStr">
         <is>
-          <t>VLINE8036</t>
+          <t>VL139</t>
         </is>
       </c>
     </row>
     <row r="616">
       <c r="A616" s="2" t="inlineStr">
         <is>
-          <t>VLINE8038</t>
+          <t>VL140</t>
         </is>
       </c>
     </row>
     <row r="617">
       <c r="A617" s="2" t="inlineStr">
         <is>
-          <t>VLINE8058</t>
+          <t>VL354</t>
         </is>
       </c>
     </row>
     <row r="618">
       <c r="A618" s="2" t="inlineStr">
         <is>
-          <t>VLINE8059</t>
+          <t>VLINE8013</t>
         </is>
       </c>
     </row>
     <row r="619">
       <c r="A619" s="2" t="inlineStr">
         <is>
-          <t>VLINE8061</t>
+          <t>VLINE8020</t>
         </is>
       </c>
     </row>
     <row r="620">
       <c r="A620" s="2" t="inlineStr">
         <is>
-          <t>VLINE8071</t>
+          <t>VLINE8021</t>
         </is>
       </c>
     </row>
     <row r="621">
       <c r="A621" s="2" t="inlineStr">
         <is>
-          <t>VLINE8072</t>
+          <t>VLINE8023</t>
         </is>
       </c>
     </row>
     <row r="622">
       <c r="A622" s="2" t="inlineStr">
         <is>
-          <t>VLINE8074</t>
+          <t>VLINE8025</t>
         </is>
       </c>
     </row>
     <row r="623">
       <c r="A623" s="2" t="inlineStr">
         <is>
-          <t>VLINE8075</t>
+          <t>VLINE8028</t>
         </is>
       </c>
     </row>
     <row r="624">
       <c r="A624" s="2" t="inlineStr">
         <is>
-          <t>VLINE8076</t>
+          <t>VLINE8029</t>
         </is>
       </c>
     </row>
     <row r="625">
       <c r="A625" s="2" t="inlineStr">
         <is>
-          <t>VLINE8077</t>
+          <t>VLINE8030</t>
         </is>
       </c>
     </row>
     <row r="626">
       <c r="A626" s="2" t="inlineStr">
         <is>
-          <t>VLINE8080</t>
+          <t>VLINE8031</t>
         </is>
       </c>
     </row>
     <row r="627">
       <c r="A627" s="2" t="inlineStr">
         <is>
-          <t>VLINE8081</t>
+          <t>VLINE8034</t>
         </is>
       </c>
     </row>
     <row r="628">
       <c r="A628" s="2" t="inlineStr">
         <is>
-          <t>VLINE8084</t>
+          <t>VLINE8036</t>
         </is>
       </c>
     </row>
     <row r="629">
       <c r="A629" s="2" t="inlineStr">
         <is>
-          <t>VLINE8102</t>
+          <t>VLINE8038</t>
         </is>
       </c>
     </row>
     <row r="630">
       <c r="A630" s="2" t="inlineStr">
         <is>
-          <t>VLINE8111</t>
+          <t>VLINE8058</t>
         </is>
       </c>
     </row>
     <row r="631">
       <c r="A631" s="2" t="inlineStr">
         <is>
-          <t>VLINE8113</t>
+          <t>VLINE8059</t>
         </is>
       </c>
     </row>
     <row r="632">
       <c r="A632" s="2" t="inlineStr">
         <is>
-          <t>VLINE8115</t>
+          <t>VLINE8061</t>
         </is>
       </c>
     </row>
     <row r="633">
       <c r="A633" s="2" t="inlineStr">
         <is>
-          <t>VLINE8117</t>
+          <t>VLINE8071</t>
         </is>
       </c>
     </row>
     <row r="634">
       <c r="A634" s="2" t="inlineStr">
         <is>
-          <t>VLINE8120</t>
+          <t>VLINE8072</t>
         </is>
       </c>
     </row>
     <row r="635">
       <c r="A635" s="2" t="inlineStr">
         <is>
-          <t>VLINE8121</t>
+          <t>VLINE8074</t>
         </is>
       </c>
     </row>
     <row r="636">
       <c r="A636" s="2" t="inlineStr">
         <is>
-          <t>VLINE8122</t>
+          <t>VLINE8075</t>
         </is>
       </c>
     </row>
     <row r="637">
       <c r="A637" s="2" t="inlineStr">
         <is>
-          <t>VLINE8123</t>
+          <t>VLINE8076</t>
         </is>
       </c>
     </row>
     <row r="638">
       <c r="A638" s="2" t="inlineStr">
         <is>
-          <t>VLINE8124</t>
+          <t>VLINE8077</t>
         </is>
       </c>
     </row>
     <row r="639">
       <c r="A639" s="2" t="inlineStr">
         <is>
-          <t>VLINE8125</t>
+          <t>VLINE8080</t>
         </is>
       </c>
     </row>
     <row r="640">
       <c r="A640" s="2" t="inlineStr">
         <is>
-          <t>VLINE8126</t>
+          <t>VLINE8081</t>
         </is>
       </c>
     </row>
     <row r="641">
       <c r="A641" s="2" t="inlineStr">
         <is>
-          <t>VLINE8127</t>
+          <t>VLINE8084</t>
         </is>
       </c>
     </row>
     <row r="642">
       <c r="A642" s="2" t="inlineStr">
         <is>
-          <t>VLINE8128</t>
+          <t>VLINE8102</t>
         </is>
       </c>
     </row>
     <row r="643">
       <c r="A643" s="2" t="inlineStr">
         <is>
-          <t>VLINE8130</t>
+          <t>VLINE8111</t>
         </is>
       </c>
     </row>
     <row r="644">
       <c r="A644" s="2" t="inlineStr">
         <is>
-          <t>VLINE8131</t>
+          <t>VLINE8113</t>
         </is>
       </c>
     </row>
     <row r="645">
       <c r="A645" s="2" t="inlineStr">
         <is>
-          <t>VLINE8133</t>
+          <t>VLINE8115</t>
         </is>
       </c>
     </row>
     <row r="646">
       <c r="A646" s="2" t="inlineStr">
         <is>
-          <t>VLINE8134</t>
+          <t>VLINE8117</t>
         </is>
       </c>
     </row>
     <row r="647">
       <c r="A647" s="2" t="inlineStr">
         <is>
-          <t>VLINE8136</t>
+          <t>VLINE8120</t>
         </is>
       </c>
     </row>
     <row r="648">
       <c r="A648" s="2" t="inlineStr">
         <is>
-          <t>VLINE8138</t>
+          <t>VLINE8121</t>
         </is>
       </c>
     </row>
     <row r="649">
       <c r="A649" s="2" t="inlineStr">
         <is>
-          <t>VLINE8142</t>
+          <t>VLINE8122</t>
         </is>
       </c>
     </row>
     <row r="650">
       <c r="A650" s="2" t="inlineStr">
         <is>
-          <t>VLINE8161</t>
+          <t>VLINE8123</t>
         </is>
       </c>
     </row>
     <row r="651">
       <c r="A651" s="2" t="inlineStr">
         <is>
-          <t>VLINE8163</t>
+          <t>VLINE8124</t>
         </is>
       </c>
     </row>
     <row r="652">
       <c r="A652" s="2" t="inlineStr">
         <is>
-          <t>VLINE8164</t>
+          <t>VLINE8125</t>
         </is>
       </c>
     </row>
     <row r="653">
       <c r="A653" s="2" t="inlineStr">
         <is>
-          <t>VLINE8172</t>
+          <t>VLINE8126</t>
         </is>
       </c>
     </row>
     <row r="654">
       <c r="A654" s="2" t="inlineStr">
         <is>
-          <t>VLINE8181</t>
+          <t>VLINE8127</t>
         </is>
       </c>
     </row>
     <row r="655">
       <c r="A655" s="2" t="inlineStr">
         <is>
-          <t>VLINE8183</t>
+          <t>VLINE8128</t>
         </is>
       </c>
     </row>
     <row r="656">
       <c r="A656" s="2" t="inlineStr">
         <is>
-          <t>VLINE8184</t>
+          <t>VLINE8130</t>
         </is>
       </c>
     </row>
     <row r="657">
       <c r="A657" s="2" t="inlineStr">
         <is>
-          <t>VLINE8185</t>
+          <t>VLINE8131</t>
         </is>
       </c>
     </row>
     <row r="658">
       <c r="A658" s="2" t="inlineStr">
         <is>
-          <t>VLINE8186</t>
+          <t>VLINE8133</t>
         </is>
       </c>
     </row>
     <row r="659">
       <c r="A659" s="2" t="inlineStr">
         <is>
-          <t>VLINE8211</t>
+          <t>VLINE8134</t>
         </is>
       </c>
     </row>
     <row r="660">
       <c r="A660" s="2" t="inlineStr">
         <is>
-          <t>VLINE8213</t>
+          <t>VLINE8135</t>
         </is>
       </c>
     </row>
     <row r="661">
       <c r="A661" s="2" t="inlineStr">
         <is>
-          <t>VLINE8215</t>
+          <t>VLINE8136</t>
         </is>
       </c>
     </row>
     <row r="662">
       <c r="A662" s="2" t="inlineStr">
         <is>
-          <t>VLINE8217</t>
+          <t>VLINE8138</t>
         </is>
       </c>
     </row>
     <row r="663">
       <c r="A663" s="2" t="inlineStr">
         <is>
-          <t>VLINE8219</t>
+          <t>VLINE8142</t>
         </is>
       </c>
     </row>
     <row r="664">
       <c r="A664" s="2" t="inlineStr">
         <is>
-          <t>VLINE8221</t>
+          <t>VLINE8161</t>
         </is>
       </c>
     </row>
     <row r="665">
       <c r="A665" s="2" t="inlineStr">
         <is>
-          <t>VLINE8223</t>
+          <t>VLINE8163</t>
         </is>
       </c>
     </row>
     <row r="666">
       <c r="A666" s="2" t="inlineStr">
         <is>
-          <t>VLINE8225</t>
+          <t>VLINE8164</t>
         </is>
       </c>
     </row>
     <row r="667">
       <c r="A667" s="2" t="inlineStr">
         <is>
-          <t>VLINE8226</t>
+          <t>VLINE8172</t>
         </is>
       </c>
     </row>
     <row r="668">
       <c r="A668" s="2" t="inlineStr">
         <is>
-          <t>VLINE8227</t>
+          <t>VLINE8181</t>
         </is>
       </c>
     </row>
     <row r="669">
       <c r="A669" s="2" t="inlineStr">
         <is>
-          <t>VLINE8228</t>
+          <t>VLINE8183</t>
         </is>
       </c>
     </row>
     <row r="670">
       <c r="A670" s="2" t="inlineStr">
         <is>
-          <t>VLINE8229</t>
+          <t>VLINE8184</t>
         </is>
       </c>
     </row>
     <row r="671">
       <c r="A671" s="2" t="inlineStr">
         <is>
-          <t>VLINE8230</t>
+          <t>VLINE8185</t>
         </is>
       </c>
     </row>
     <row r="672">
       <c r="A672" s="2" t="inlineStr">
         <is>
-          <t>VLINE8231</t>
+          <t>VLINE8186</t>
         </is>
       </c>
     </row>
     <row r="673">
       <c r="A673" s="2" t="inlineStr">
         <is>
-          <t>VLINE8232</t>
+          <t>VLINE8211</t>
         </is>
       </c>
     </row>
     <row r="674">
       <c r="A674" s="2" t="inlineStr">
         <is>
-          <t>VLINE8233</t>
+          <t>VLINE8213</t>
         </is>
       </c>
     </row>
     <row r="675">
       <c r="A675" s="2" t="inlineStr">
         <is>
-          <t>VLINE8234</t>
+          <t>VLINE8215</t>
         </is>
       </c>
     </row>
     <row r="676">
       <c r="A676" s="2" t="inlineStr">
         <is>
-          <t>VLINE8236</t>
+          <t>VLINE8217</t>
         </is>
       </c>
     </row>
     <row r="677">
       <c r="A677" s="2" t="inlineStr">
         <is>
-          <t>VLINE8238</t>
+          <t>VLINE8219</t>
         </is>
       </c>
     </row>
     <row r="678">
       <c r="A678" s="2" t="inlineStr">
         <is>
-          <t>VLINE8240</t>
+          <t>VLINE8221</t>
         </is>
       </c>
     </row>
     <row r="679">
       <c r="A679" s="2" t="inlineStr">
         <is>
-          <t>VLINE8242</t>
+          <t>VLINE8223</t>
         </is>
       </c>
     </row>
     <row r="680">
       <c r="A680" s="2" t="inlineStr">
         <is>
-          <t>VLINE8244</t>
+          <t>VLINE8225</t>
         </is>
       </c>
     </row>
     <row r="681">
       <c r="A681" s="2" t="inlineStr">
         <is>
-          <t>VLINE8246</t>
+          <t>VLINE8226</t>
         </is>
       </c>
     </row>
     <row r="682">
       <c r="A682" s="2" t="inlineStr">
         <is>
-          <t>VLINE8400</t>
+          <t>VLINE8227</t>
         </is>
       </c>
     </row>
     <row r="683">
       <c r="A683" s="2" t="inlineStr">
         <is>
-          <t>VLINE8405</t>
+          <t>VLINE8228</t>
         </is>
       </c>
     </row>
     <row r="684">
       <c r="A684" s="2" t="inlineStr">
         <is>
-          <t>VLINE8408</t>
+          <t>VLINE8229</t>
         </is>
       </c>
     </row>
     <row r="685">
       <c r="A685" s="2" t="inlineStr">
         <is>
-          <t>VLINE8413</t>
+          <t>VLINE8230</t>
         </is>
       </c>
     </row>
     <row r="686">
       <c r="A686" s="2" t="inlineStr">
         <is>
-          <t>VLINE8415</t>
+          <t>VLINE8231</t>
         </is>
       </c>
     </row>
     <row r="687">
       <c r="A687" s="2" t="inlineStr">
         <is>
-          <t>VLINE8417</t>
+          <t>VLINE8232</t>
         </is>
       </c>
     </row>
     <row r="688">
       <c r="A688" s="2" t="inlineStr">
         <is>
-          <t>VLINE8418</t>
+          <t>VLINE8233</t>
         </is>
       </c>
     </row>
     <row r="689">
       <c r="A689" s="2" t="inlineStr">
         <is>
-          <t>VLINE8419</t>
+          <t>VLINE8234</t>
         </is>
       </c>
     </row>
     <row r="690">
       <c r="A690" s="2" t="inlineStr">
         <is>
-          <t>VLINE8420</t>
+          <t>VLINE8235</t>
         </is>
       </c>
     </row>
     <row r="691">
       <c r="A691" s="2" t="inlineStr">
         <is>
-          <t>VLINE8421</t>
+          <t>VLINE8236</t>
         </is>
       </c>
     </row>
     <row r="692">
       <c r="A692" s="2" t="inlineStr">
         <is>
-          <t>VLINE8422</t>
+          <t>VLINE8238</t>
         </is>
       </c>
     </row>
     <row r="693">
       <c r="A693" s="2" t="inlineStr">
         <is>
-          <t>VLINE8423</t>
+          <t>VLINE8240</t>
         </is>
       </c>
     </row>
     <row r="694">
       <c r="A694" s="2" t="inlineStr">
         <is>
-          <t>VLINE8424</t>
+          <t>VLINE8242</t>
         </is>
       </c>
     </row>
     <row r="695">
       <c r="A695" s="2" t="inlineStr">
         <is>
-          <t>VLINE8427</t>
+          <t>VLINE8244</t>
         </is>
       </c>
     </row>
     <row r="696">
       <c r="A696" s="2" t="inlineStr">
         <is>
-          <t>VLINE8428</t>
+          <t>VLINE8246</t>
         </is>
       </c>
     </row>
     <row r="697">
       <c r="A697" s="2" t="inlineStr">
         <is>
-          <t>VLINE8429</t>
+          <t>VLINE8248</t>
         </is>
       </c>
     </row>
     <row r="698">
       <c r="A698" s="2" t="inlineStr">
         <is>
-          <t>VLINE8430</t>
+          <t>VLINE8400</t>
         </is>
       </c>
     </row>
     <row r="699">
       <c r="A699" s="2" t="inlineStr">
         <is>
-          <t>VLINE8431</t>
+          <t>VLINE8405</t>
         </is>
       </c>
     </row>
     <row r="700">
       <c r="A700" s="2" t="inlineStr">
         <is>
-          <t>VLINE8432</t>
+          <t>VLINE8408</t>
         </is>
       </c>
     </row>
     <row r="701">
       <c r="A701" s="2" t="inlineStr">
         <is>
-          <t>VLINE8433</t>
+          <t>VLINE8413</t>
         </is>
       </c>
     </row>
     <row r="702">
       <c r="A702" s="2" t="inlineStr">
         <is>
-          <t>VLINE8434</t>
+          <t>VLINE8415</t>
         </is>
       </c>
     </row>
     <row r="703">
       <c r="A703" s="2" t="inlineStr">
         <is>
-          <t>VLINE8438</t>
+          <t>VLINE8417</t>
         </is>
       </c>
     </row>
     <row r="704">
       <c r="A704" s="2" t="inlineStr">
         <is>
-          <t>VLINE8440</t>
+          <t>VLINE8418</t>
         </is>
       </c>
     </row>
     <row r="705">
       <c r="A705" s="2" t="inlineStr">
         <is>
-          <t>VLINE8457</t>
+          <t>VLINE8419</t>
         </is>
       </c>
     </row>
     <row r="706">
       <c r="A706" s="2" t="inlineStr">
         <is>
-          <t>VLINE8459</t>
+          <t>VLINE8420</t>
         </is>
       </c>
     </row>
     <row r="707">
       <c r="A707" s="2" t="inlineStr">
         <is>
-          <t>VLINE8460</t>
+          <t>VLINE8421</t>
         </is>
       </c>
     </row>
     <row r="708">
       <c r="A708" s="2" t="inlineStr">
         <is>
-          <t>VLINE8461</t>
+          <t>VLINE8422</t>
         </is>
       </c>
     </row>
     <row r="709">
       <c r="A709" s="2" t="inlineStr">
         <is>
-          <t>VLINE8464</t>
+          <t>VLINE8423</t>
         </is>
       </c>
     </row>
     <row r="710">
       <c r="A710" s="2" t="inlineStr">
         <is>
-          <t>VLINE8465</t>
+          <t>VLINE8424</t>
         </is>
       </c>
     </row>
     <row r="711">
       <c r="A711" s="2" t="inlineStr">
         <is>
-          <t>VLINE8702</t>
+          <t>VLINE8427</t>
         </is>
       </c>
     </row>
     <row r="712">
       <c r="A712" s="2" t="inlineStr">
         <is>
-          <t>VLINE8725</t>
+          <t>VLINE8428</t>
         </is>
       </c>
     </row>
     <row r="713">
       <c r="A713" s="2" t="inlineStr">
         <is>
-          <t>VLINE8727</t>
+          <t>VLINE8429</t>
         </is>
       </c>
     </row>
     <row r="714">
       <c r="A714" s="2" t="inlineStr">
         <is>
-          <t>VLINE8729</t>
+          <t>VLINE8430</t>
         </is>
       </c>
     </row>
     <row r="715">
       <c r="A715" s="2" t="inlineStr">
         <is>
-          <t>VLINE8731</t>
+          <t>VLINE8431</t>
         </is>
       </c>
     </row>
     <row r="716">
       <c r="A716" s="2" t="inlineStr">
         <is>
-          <t>VLINE8733</t>
+          <t>VLINE8432</t>
         </is>
       </c>
     </row>
     <row r="717">
       <c r="A717" s="2" t="inlineStr">
         <is>
-          <t>VLINE8735</t>
+          <t>VLINE8433</t>
         </is>
       </c>
     </row>
     <row r="718">
       <c r="A718" s="2" t="inlineStr">
         <is>
-          <t>VLINE8737</t>
+          <t>VLINE8434</t>
         </is>
       </c>
     </row>
     <row r="719">
       <c r="A719" s="2" t="inlineStr">
         <is>
-          <t>VLINE8739</t>
+          <t>VLINE8435</t>
         </is>
       </c>
     </row>
     <row r="720">
       <c r="A720" s="2" t="inlineStr">
         <is>
-          <t>VLINE8741</t>
+          <t>VLINE8438</t>
         </is>
       </c>
     </row>
     <row r="721">
       <c r="A721" s="2" t="inlineStr">
         <is>
-          <t>VLINE8742</t>
+          <t>VLINE8440</t>
         </is>
       </c>
     </row>
     <row r="722">
       <c r="A722" s="2" t="inlineStr">
         <is>
-          <t>VLINE8743</t>
+          <t>VLINE8442</t>
         </is>
       </c>
     </row>
     <row r="723">
       <c r="A723" s="2" t="inlineStr">
         <is>
-          <t>VLINE8744</t>
+          <t>VLINE8457</t>
         </is>
       </c>
     </row>
     <row r="724">
       <c r="A724" s="2" t="inlineStr">
         <is>
-          <t>VLINE8745</t>
+          <t>VLINE8459</t>
         </is>
       </c>
     </row>
     <row r="725">
       <c r="A725" s="2" t="inlineStr">
         <is>
-          <t>VLINE8746</t>
+          <t>VLINE8460</t>
         </is>
       </c>
     </row>
     <row r="726">
       <c r="A726" s="2" t="inlineStr">
         <is>
-          <t>VLINE8747</t>
+          <t>VLINE8461</t>
         </is>
       </c>
     </row>
     <row r="727">
       <c r="A727" s="2" t="inlineStr">
         <is>
-          <t>VLINE8748</t>
+          <t>VLINE8464</t>
         </is>
       </c>
     </row>
     <row r="728">
       <c r="A728" s="2" t="inlineStr">
         <is>
-          <t>VLINE8749</t>
+          <t>VLINE8465</t>
         </is>
       </c>
     </row>
     <row r="729">
       <c r="A729" s="2" t="inlineStr">
         <is>
-          <t>VLINE8750</t>
+          <t>VLINE8702</t>
         </is>
       </c>
     </row>
     <row r="730">
       <c r="A730" s="2" t="inlineStr">
         <is>
-          <t>VLINE8751</t>
+          <t>VLINE8725</t>
         </is>
       </c>
     </row>
     <row r="731">
       <c r="A731" s="2" t="inlineStr">
         <is>
-          <t>VLINE8752</t>
+          <t>VLINE8727</t>
         </is>
       </c>
     </row>
     <row r="732">
       <c r="A732" s="2" t="inlineStr">
         <is>
-          <t>VLINE8753</t>
+          <t>VLINE8729</t>
         </is>
       </c>
     </row>
     <row r="733">
       <c r="A733" s="2" t="inlineStr">
         <is>
-          <t>VLINE8754</t>
+          <t>VLINE8731</t>
         </is>
       </c>
     </row>
     <row r="734">
       <c r="A734" s="2" t="inlineStr">
         <is>
-          <t>VLINE8755</t>
+          <t>VLINE8733</t>
         </is>
       </c>
     </row>
     <row r="735">
       <c r="A735" s="2" t="inlineStr">
         <is>
-          <t>VLINE8756</t>
+          <t>VLINE8735</t>
         </is>
       </c>
     </row>
     <row r="736">
       <c r="A736" s="2" t="inlineStr">
         <is>
-          <t>VLINE8757</t>
+          <t>VLINE8737</t>
         </is>
       </c>
     </row>
     <row r="737">
       <c r="A737" s="2" t="inlineStr">
         <is>
-          <t>VLINE8758</t>
+          <t>VLINE8739</t>
         </is>
       </c>
     </row>
     <row r="738">
       <c r="A738" s="2" t="inlineStr">
         <is>
-          <t>VLINE8759</t>
+          <t>VLINE8741</t>
         </is>
       </c>
     </row>
     <row r="739">
       <c r="A739" s="2" t="inlineStr">
         <is>
-          <t>VLINE8760</t>
+          <t>VLINE8742</t>
         </is>
       </c>
     </row>
     <row r="740">
       <c r="A740" s="2" t="inlineStr">
         <is>
-          <t>VLINE8761</t>
+          <t>VLINE8743</t>
         </is>
       </c>
     </row>
     <row r="741">
       <c r="A741" s="2" t="inlineStr">
         <is>
-          <t>VLINE8762</t>
+          <t>VLINE8744</t>
         </is>
       </c>
     </row>
     <row r="742">
       <c r="A742" s="2" t="inlineStr">
         <is>
-          <t>VLINE8763</t>
+          <t>VLINE8745</t>
         </is>
       </c>
     </row>
     <row r="743">
       <c r="A743" s="2" t="inlineStr">
         <is>
-          <t>VLINE8764</t>
+          <t>VLINE8746</t>
         </is>
       </c>
     </row>
     <row r="744">
       <c r="A744" s="2" t="inlineStr">
         <is>
-          <t>VLINE8765</t>
+          <t>VLINE8747</t>
         </is>
       </c>
     </row>
     <row r="745">
       <c r="A745" s="2" t="inlineStr">
         <is>
-          <t>VLINE8766</t>
+          <t>VLINE8748</t>
         </is>
       </c>
     </row>
     <row r="746">
       <c r="A746" s="2" t="inlineStr">
         <is>
-          <t>VLINE8767</t>
+          <t>VLINE8749</t>
         </is>
       </c>
     </row>
     <row r="747">
       <c r="A747" s="2" t="inlineStr">
         <is>
-          <t>VLINE8768</t>
+          <t>VLINE8750</t>
         </is>
       </c>
     </row>
     <row r="748">
       <c r="A748" s="2" t="inlineStr">
         <is>
-          <t>VLINE8770</t>
+          <t>VLINE8751</t>
         </is>
       </c>
     </row>
     <row r="749">
       <c r="A749" s="2" t="inlineStr">
         <is>
-          <t>VLINE8772</t>
+          <t>VLINE8752</t>
         </is>
       </c>
     </row>
     <row r="750">
       <c r="A750" s="2" t="inlineStr">
         <is>
-          <t>VLINE8774</t>
+          <t>VLINE8753</t>
         </is>
       </c>
     </row>
     <row r="751">
       <c r="A751" s="2" t="inlineStr">
         <is>
-          <t>VLINE8776</t>
+          <t>VLINE8754</t>
         </is>
       </c>
     </row>
     <row r="752">
       <c r="A752" s="2" t="inlineStr">
         <is>
-          <t>VLINE8778</t>
+          <t>VLINE8755</t>
         </is>
       </c>
     </row>
     <row r="753">
       <c r="A753" s="2" t="inlineStr">
         <is>
-          <t>VLINE8780</t>
+          <t>VLINE8756</t>
         </is>
       </c>
     </row>
     <row r="754">
       <c r="A754" s="2" t="inlineStr">
         <is>
-          <t>VLINE8782</t>
+          <t>VLINE8757</t>
         </is>
       </c>
     </row>
     <row r="755">
       <c r="A755" s="2" t="inlineStr">
         <is>
-          <t>VLINE8784</t>
+          <t>VLINE8758</t>
         </is>
       </c>
     </row>
     <row r="756">
       <c r="A756" s="2" t="inlineStr">
         <is>
-          <t>VLINE8786</t>
+          <t>VLINE8759</t>
         </is>
       </c>
     </row>
     <row r="757">
       <c r="A757" s="2" t="inlineStr">
         <is>
-          <t>VLINE8819</t>
+          <t>VLINE8760</t>
         </is>
       </c>
     </row>
     <row r="758">
       <c r="A758" s="2" t="inlineStr">
         <is>
-          <t>VLINE8862</t>
+          <t>VLINE8761</t>
         </is>
       </c>
     </row>
     <row r="759">
       <c r="A759" s="2" t="inlineStr">
         <is>
-          <t>VLINE8863</t>
+          <t>VLINE8762</t>
         </is>
       </c>
     </row>
     <row r="760">
       <c r="A760" s="2" t="inlineStr">
         <is>
-          <t>VLINE8864</t>
+          <t>VLINE8763</t>
         </is>
       </c>
     </row>
     <row r="761">
       <c r="A761" s="2" t="inlineStr">
         <is>
-          <t>VLINE8865</t>
+          <t>VLINE8764</t>
         </is>
       </c>
     </row>
     <row r="762">
       <c r="A762" s="2" t="inlineStr">
         <is>
-          <t>VLINE8933</t>
+          <t>VLINE8765</t>
         </is>
       </c>
     </row>
     <row r="763">
       <c r="A763" s="2" t="inlineStr">
         <is>
-          <t>VLINE8935</t>
+          <t>VLINE8766</t>
         </is>
       </c>
     </row>
     <row r="764">
       <c r="A764" s="2" t="inlineStr">
         <is>
-          <t>VR76</t>
+          <t>VLINE8767</t>
         </is>
       </c>
     </row>
     <row r="765">
       <c r="A765" s="2" t="inlineStr">
         <is>
-          <t>VR77</t>
+          <t>VLINE8768</t>
         </is>
       </c>
     </row>
     <row r="766">
       <c r="A766" s="2" t="inlineStr">
         <is>
-          <t>WOLL408</t>
+          <t>VLINE8770</t>
         </is>
       </c>
     </row>
     <row r="767">
       <c r="A767" s="2" t="inlineStr">
         <is>
-          <t>WOLL430</t>
+          <t>VLINE8771</t>
         </is>
       </c>
     </row>
     <row r="768">
       <c r="A768" s="2" t="inlineStr">
         <is>
-          <t>X21</t>
+          <t>VLINE8772</t>
         </is>
       </c>
     </row>
     <row r="769">
       <c r="A769" s="2" t="inlineStr">
         <is>
-          <t>XP2001</t>
+          <t>VLINE8773</t>
         </is>
       </c>
     </row>
     <row r="770">
       <c r="A770" s="2" t="inlineStr">
         <is>
-          <t>XP2005</t>
+          <t>VLINE8774</t>
         </is>
       </c>
     </row>
     <row r="771">
       <c r="A771" s="2" t="inlineStr">
         <is>
-          <t>XP2006</t>
+          <t>VLINE8775</t>
         </is>
       </c>
     </row>
     <row r="772">
       <c r="A772" s="2" t="inlineStr">
         <is>
-          <t>XP2008</t>
+          <t>VLINE8776</t>
         </is>
       </c>
     </row>
     <row r="773">
       <c r="A773" s="2" t="inlineStr">
         <is>
-          <t>XP2009</t>
+          <t>VLINE8778</t>
         </is>
       </c>
     </row>
     <row r="774">
       <c r="A774" s="2" t="inlineStr">
         <is>
-          <t>XP2010</t>
+          <t>VLINE8780</t>
         </is>
       </c>
     </row>
     <row r="775">
       <c r="A775" s="2" t="inlineStr">
         <is>
-          <t>XP2011</t>
+          <t>VLINE8782</t>
         </is>
       </c>
     </row>
     <row r="776">
       <c r="A776" s="2" t="inlineStr">
         <is>
-          <t>XP2012</t>
+          <t>VLINE8784</t>
         </is>
       </c>
     </row>
     <row r="777">
       <c r="A777" s="2" t="inlineStr">
         <is>
-          <t>XP2013</t>
+          <t>VLINE8786</t>
         </is>
       </c>
     </row>
     <row r="778">
       <c r="A778" s="2" t="inlineStr">
         <is>
-          <t>XP2014</t>
+          <t>VLINE8788</t>
         </is>
       </c>
     </row>
     <row r="779">
       <c r="A779" s="2" t="inlineStr">
         <is>
-          <t>XP2015</t>
+          <t>VLINE8819</t>
         </is>
       </c>
     </row>
     <row r="780">
       <c r="A780" s="2" t="inlineStr">
         <is>
-          <t>XP2019</t>
+          <t>VLINE8862</t>
         </is>
       </c>
     </row>
     <row r="781">
       <c r="A781" s="2" t="inlineStr">
         <is>
-          <t>XRN003</t>
+          <t>VLINE8863</t>
         </is>
       </c>
     </row>
     <row r="782">
       <c r="A782" s="2" t="inlineStr">
         <is>
-          <t>XRN005</t>
+          <t>VLINE8864</t>
         </is>
       </c>
     </row>
     <row r="783">
       <c r="A783" s="2" t="inlineStr">
         <is>
-          <t>XRN009</t>
+          <t>VLINE8865</t>
         </is>
       </c>
     </row>
     <row r="784">
       <c r="A784" s="2" t="inlineStr">
         <is>
-          <t>XRN010</t>
+          <t>VLINE8933</t>
         </is>
       </c>
     </row>
     <row r="785">
       <c r="A785" s="2" t="inlineStr">
         <is>
-          <t>XRN012</t>
+          <t>VLINE8935</t>
         </is>
       </c>
     </row>
     <row r="786">
       <c r="A786" s="2" t="inlineStr">
         <is>
-          <t>XRN017</t>
+          <t>VLINE8937</t>
         </is>
       </c>
     </row>
     <row r="787">
       <c r="A787" s="2" t="inlineStr">
         <is>
-          <t>XRN018</t>
+          <t>VR76</t>
         </is>
       </c>
     </row>
     <row r="788">
       <c r="A788" s="2" t="inlineStr">
         <is>
-          <t>XRN021</t>
+          <t>VR77</t>
         </is>
       </c>
     </row>
     <row r="789">
       <c r="A789" s="2" t="inlineStr">
         <is>
-          <t>XRN022</t>
+          <t>WOLL408</t>
         </is>
       </c>
     </row>
     <row r="790">
       <c r="A790" s="2" t="inlineStr">
         <is>
-          <t>XRN028</t>
+          <t>WOLL430</t>
         </is>
       </c>
     </row>
     <row r="791">
       <c r="A791" s="2" t="inlineStr">
+        <is>
+          <t>X21</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" s="2" t="inlineStr">
+        <is>
+          <t>XP2001</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" s="2" t="inlineStr">
+        <is>
+          <t>XP2005</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" s="2" t="inlineStr">
+        <is>
+          <t>XP2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="2" t="inlineStr">
+        <is>
+          <t>XP2008</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="2" t="inlineStr">
+        <is>
+          <t>XP2009</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="2" t="inlineStr">
+        <is>
+          <t>XP2010</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="2" t="inlineStr">
+        <is>
+          <t>XP2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" s="2" t="inlineStr">
+        <is>
+          <t>XP2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" s="2" t="inlineStr">
+        <is>
+          <t>XP2013</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" s="2" t="inlineStr">
+        <is>
+          <t>XP2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" s="2" t="inlineStr">
+        <is>
+          <t>XP2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" s="2" t="inlineStr">
+        <is>
+          <t>XP2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="2" t="inlineStr">
+        <is>
+          <t>XRN003</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="2" t="inlineStr">
+        <is>
+          <t>XRN005</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="2" t="inlineStr">
+        <is>
+          <t>XRN009</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="2" t="inlineStr">
+        <is>
+          <t>XRN010</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="2" t="inlineStr">
+        <is>
+          <t>XRN012</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="2" t="inlineStr">
+        <is>
+          <t>XRN017</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="2" t="inlineStr">
+        <is>
+          <t>XRN018</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="2" t="inlineStr">
+        <is>
+          <t>XRN021</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="2" t="inlineStr">
+        <is>
+          <t>XRN022</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="2" t="inlineStr">
+        <is>
+          <t>XRN028</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" s="2" t="inlineStr">
         <is>
           <t>XRN029</t>
         </is>

</xml_diff>

<commit_message>
Update RailOps database files - 2026-04-30 07:02:47 UTC
</commit_message>
<xml_diff>
--- a/static/downloads/loco_numbers_only.xlsx
+++ b/static/downloads/loco_numbers_only.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A814"/>
+  <dimension ref="A1:A838"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2295,3855 +2295,4023 @@
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>MM192M</t>
+          <t>MM180M</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>MM212M</t>
+          <t>MM192M</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>MM214M</t>
+          <t>MM208M</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>MM216M</t>
+          <t>MM212M</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>MM224M</t>
+          <t>MM214M</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>MM232M</t>
+          <t>MM216M</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>MM236M</t>
+          <t>MM224M</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>MM240M</t>
+          <t>MM232M</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>MM242M</t>
+          <t>MM236M</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>MM246M</t>
+          <t>MM240M</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>MM256M</t>
+          <t>MM242M</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>MM258M</t>
+          <t>MM246M</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>MM260M</t>
+          <t>MM248M</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>MM264M</t>
+          <t>MM256M</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>MM266M</t>
+          <t>MM258M</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>MM268M</t>
+          <t>MM260M</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>MM270M</t>
+          <t>MM264M</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>MM280M</t>
+          <t>MM266M</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>MM288M</t>
+          <t>MM268M</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>MM380M</t>
+          <t>MM270M</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>MM384M</t>
+          <t>MM280M</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>MM418M</t>
+          <t>MM288M</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>MM424M</t>
+          <t>MM349M</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>MM456M</t>
+          <t>MM380M</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>MM464M</t>
+          <t>MM384M</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>MM478M</t>
+          <t>MM387M</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>MM482M</t>
+          <t>MM418M</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>MM486M</t>
+          <t>MM424M</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>MM502M</t>
+          <t>MM456M</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>MM506M</t>
+          <t>MM464M</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>MM514M</t>
+          <t>MM472M</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>MM522M</t>
+          <t>MM478M</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>MM536M</t>
+          <t>MM482M</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>MM542M</t>
+          <t>MM486M</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>MM544M</t>
+          <t>MM502M</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>MM546M</t>
+          <t>MM506M</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>MM551M</t>
+          <t>MM514M</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>MM552M</t>
+          <t>MM522M</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>MM566M</t>
+          <t>MM536M</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>MM574M</t>
+          <t>MM542M</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>MM588M</t>
+          <t>MM544M</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>MM592M</t>
+          <t>MM546M</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>MM602M</t>
+          <t>MM551M</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>MM604M</t>
+          <t>MM552M</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>MM608M</t>
+          <t>MM564M</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>MM620M</t>
+          <t>MM566M</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>MM624M</t>
+          <t>MM574M</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>MM636M</t>
+          <t>MM588M</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>MM638M</t>
+          <t>MM592M</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>MM647M</t>
+          <t>MM602M</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>MM656M</t>
+          <t>MM604M</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>MM658M</t>
+          <t>MM608M</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>MM660M</t>
+          <t>MM620M</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>MM661M</t>
+          <t>MM624M</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>MM662M</t>
+          <t>MM636M</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>MM664M</t>
+          <t>MM638M</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>MM668M</t>
+          <t>MM647M</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>MM673M</t>
+          <t>MM656M</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>MM674M</t>
+          <t>MM658M</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>MM676M</t>
+          <t>MM660M</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>MM678M</t>
+          <t>MM661M</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>MM680M</t>
+          <t>MM662M</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>MM702M</t>
+          <t>MM664M</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>MM708M</t>
+          <t>MM668M</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>MM718M</t>
+          <t>MM673M</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>MM742M</t>
+          <t>MM674M</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>MM744M</t>
+          <t>MM676M</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>MM752M</t>
+          <t>MM678M</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>MM756M</t>
+          <t>MM680M</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>MM760M</t>
+          <t>MM702M</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>MM766M</t>
+          <t>MM708M</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>MM768M</t>
+          <t>MM718M</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>MM772M</t>
+          <t>MM742M</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>MM774M</t>
+          <t>MM744M</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>MM776M</t>
+          <t>MM752M</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>MM778M</t>
+          <t>MM756M</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>MM780M</t>
+          <t>MM760M</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>MM784M</t>
+          <t>MM766M</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>MM788M</t>
+          <t>MM768M</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>MM790M</t>
+          <t>MM772M</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>MM794M</t>
+          <t>MM774M</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>MM798M</t>
+          <t>MM776M</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>MM800M</t>
+          <t>MM778M</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>MM802M</t>
+          <t>MM780M</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>MM806M</t>
+          <t>MM784M</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>MM808M</t>
+          <t>MM788M</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>MM810M</t>
+          <t>MM790M</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>MM816M</t>
+          <t>MM794M</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>MM820M</t>
+          <t>MM798M</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>MM826M</t>
+          <t>MM800M</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>MM830M</t>
+          <t>MM802M</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>MM832M</t>
+          <t>MM806M</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>MM834M</t>
+          <t>MM808M</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>MM836M</t>
+          <t>MM810M</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>MM838M</t>
+          <t>MM816M</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>MM840M</t>
+          <t>MM820M</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>MM842M</t>
+          <t>MM826M</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>MM844M</t>
+          <t>MM830M</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>MM858M</t>
+          <t>MM832M</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>MM860M</t>
+          <t>MM834M</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>MM862M</t>
+          <t>MM836M</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>MM864M</t>
+          <t>MM838M</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>MM866M</t>
+          <t>MM840M</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>MM872M</t>
+          <t>MM842M</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>MM878M</t>
+          <t>MM844M</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>MM880M</t>
+          <t>MM858M</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>MM882M</t>
+          <t>MM860M</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>MM886M</t>
+          <t>MM862M</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>MM896M</t>
+          <t>MM864M</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t>MM908M</t>
+          <t>MM866M</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>MM910M</t>
+          <t>MM872M</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t>MM912M</t>
+          <t>MM878M</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>MM914M</t>
+          <t>MM880M</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>MM918M</t>
+          <t>MM882M</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>MM922M</t>
+          <t>MM886M</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>MM924M</t>
+          <t>MM896M</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>MM928M</t>
+          <t>MM908M</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>MM934M</t>
+          <t>MM910M</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>MM940M</t>
+          <t>MM912M</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
         <is>
-          <t>MM944M</t>
+          <t>MM914M</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
         <is>
-          <t>MM946M</t>
+          <t>MM918M</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
         <is>
-          <t>MM950M</t>
+          <t>MM922M</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
         <is>
-          <t>MM952M</t>
+          <t>MM924M</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" s="2" t="inlineStr">
         <is>
-          <t>MM956M</t>
+          <t>MM926M</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
         <is>
-          <t>MM958M</t>
+          <t>MM928M</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
         <is>
-          <t>MM960M</t>
+          <t>MM934M</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>MM962M</t>
+          <t>MM940M</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
         <is>
-          <t>MM964M</t>
+          <t>MM944M</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
         <is>
-          <t>MM968M</t>
+          <t>MM946M</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="2" t="inlineStr">
         <is>
-          <t>MM970M</t>
+          <t>MM950M</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
         <is>
-          <t>MM972M</t>
+          <t>MM952M</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" s="2" t="inlineStr">
         <is>
-          <t>MM974M</t>
+          <t>MM956M</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
         <is>
-          <t>MM976M</t>
+          <t>MM958M</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="2" t="inlineStr">
         <is>
-          <t>MM980M</t>
+          <t>MM960M</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" s="2" t="inlineStr">
         <is>
-          <t>MM982M</t>
+          <t>MM962M</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="2" t="inlineStr">
         <is>
-          <t>MM984M</t>
+          <t>MM964M</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
         <is>
-          <t>MM9901M</t>
+          <t>MM968M</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" s="2" t="inlineStr">
         <is>
-          <t>MM9903M</t>
+          <t>MM970M</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
         <is>
-          <t>MM9904M</t>
+          <t>MM972M</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" s="2" t="inlineStr">
         <is>
-          <t>MM9905M</t>
+          <t>MM974M</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" s="2" t="inlineStr">
         <is>
-          <t>MM9906M</t>
+          <t>MM976M</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
         <is>
-          <t>MM9907M</t>
+          <t>MM980M</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="2" t="inlineStr">
         <is>
-          <t>MM9908M</t>
+          <t>MM982M</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
         <is>
-          <t>MM9909M</t>
+          <t>MM984M</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="2" t="inlineStr">
         <is>
-          <t>MM9910M</t>
+          <t>MM9901M</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="2" t="inlineStr">
         <is>
-          <t>MM9912M</t>
+          <t>MM9903M</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" s="2" t="inlineStr">
         <is>
-          <t>MM9914M</t>
+          <t>MM9904M</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" s="2" t="inlineStr">
         <is>
-          <t>MM9916M</t>
+          <t>MM9905M</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" s="2" t="inlineStr">
         <is>
-          <t>MM9918M</t>
+          <t>MM9906M</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" s="2" t="inlineStr">
         <is>
-          <t>MM9919M</t>
+          <t>MM9907M</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" s="2" t="inlineStr">
         <is>
-          <t>MM9920M</t>
+          <t>MM9908M</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" s="2" t="inlineStr">
         <is>
-          <t>MM9921M</t>
+          <t>MM9909M</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" s="2" t="inlineStr">
         <is>
-          <t>MM9922M</t>
+          <t>MM9910M</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" s="2" t="inlineStr">
         <is>
-          <t>MM9924M</t>
+          <t>MM9912M</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t>MM9926M</t>
+          <t>MM9914M</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" s="2" t="inlineStr">
         <is>
-          <t>MM9927M</t>
+          <t>MM9916M</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
         <is>
-          <t>MM9928M</t>
+          <t>MM9918M</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" s="2" t="inlineStr">
         <is>
-          <t>MM9929M</t>
+          <t>MM9919M</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" s="2" t="inlineStr">
         <is>
-          <t>MM9930M</t>
+          <t>MM9920M</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" s="2" t="inlineStr">
         <is>
-          <t>MM9931M</t>
+          <t>MM9921M</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
         <is>
-          <t>MM9933M</t>
+          <t>MM9922M</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="2" t="inlineStr">
         <is>
-          <t>MM9936M</t>
+          <t>MM9924M</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
         <is>
-          <t>MM9937M</t>
+          <t>MM9925M</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
         <is>
-          <t>MM9938M</t>
+          <t>MM9926M</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>MM9941M</t>
+          <t>MM9927M</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" s="2" t="inlineStr">
         <is>
-          <t>MM9943M</t>
+          <t>MM9928M</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
         <is>
-          <t>MM9946M</t>
+          <t>MM9929M</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" s="2" t="inlineStr">
         <is>
-          <t>MM9947M</t>
+          <t>MM9930M</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
         <is>
-          <t>MM9948M</t>
+          <t>MM9931M</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" s="2" t="inlineStr">
         <is>
-          <t>MM9952M</t>
+          <t>MM9933M</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t>MM9953M</t>
+          <t>MM9934M</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t>MM9954M</t>
+          <t>MM9936M</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>MM9956M</t>
+          <t>MM9937M</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
         <is>
-          <t>MM9957M</t>
+          <t>MM9938M</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
         <is>
-          <t>MM9958M</t>
+          <t>MM9941M</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
         <is>
-          <t>MM9959M</t>
+          <t>MM9943M</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
         <is>
-          <t>MM9960M</t>
+          <t>MM9946M</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
         <is>
-          <t>MM9961M</t>
+          <t>MM9947M</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>MM9962M</t>
+          <t>MM9948M</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
         <is>
-          <t>MM9963M</t>
+          <t>MM9950M</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>MM9964M</t>
+          <t>MM9952M</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
         <is>
-          <t>MM9965M</t>
+          <t>MM9953M</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>MM9966M</t>
+          <t>MM9954M</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
         <is>
-          <t>MM9968M</t>
+          <t>MM9956M</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>MM9969M</t>
+          <t>MM9957M</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
         <is>
-          <t>MM9970M</t>
+          <t>MM9958M</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>MRL001</t>
+          <t>MM9959M</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
         <is>
-          <t>MRL002</t>
+          <t>MM9960M</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>MTPV1</t>
+          <t>MM9961M</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="2" t="inlineStr">
         <is>
-          <t>MTPV2</t>
+          <t>MM9962M</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
         <is>
-          <t>N453</t>
+          <t>MM9963M</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" s="2" t="inlineStr">
         <is>
-          <t>N458</t>
+          <t>MM9964M</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
         <is>
-          <t>N460</t>
+          <t>MM9965M</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" s="2" t="inlineStr">
         <is>
-          <t>N466</t>
+          <t>MM9966M</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="2" t="inlineStr">
         <is>
-          <t>N469</t>
+          <t>MM9968M</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" s="2" t="inlineStr">
         <is>
-          <t>NR4</t>
+          <t>MM9969M</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" s="2" t="inlineStr">
         <is>
-          <t>NR5</t>
+          <t>MM9970M</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" s="2" t="inlineStr">
         <is>
-          <t>NR6</t>
+          <t>MRL001</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" s="2" t="inlineStr">
         <is>
-          <t>NR10</t>
+          <t>MRL002</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="2" t="inlineStr">
         <is>
-          <t>NR11</t>
+          <t>MTPV1</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="2" t="inlineStr">
         <is>
-          <t>NR12</t>
+          <t>MTPV2</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="2" t="inlineStr">
         <is>
-          <t>NR13</t>
+          <t>N453</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="2" t="inlineStr">
         <is>
-          <t>NR14</t>
+          <t>N458</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="2" t="inlineStr">
         <is>
-          <t>NR17</t>
+          <t>N460</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" s="2" t="inlineStr">
         <is>
-          <t>NR20</t>
+          <t>N466</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" s="2" t="inlineStr">
         <is>
-          <t>NR31</t>
+          <t>N469</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" s="2" t="inlineStr">
         <is>
-          <t>NR35</t>
+          <t>NR4</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" s="2" t="inlineStr">
         <is>
-          <t>NR37</t>
+          <t>NR5</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="A472" s="2" t="inlineStr">
         <is>
-          <t>NR44</t>
+          <t>NR6</t>
         </is>
       </c>
     </row>
     <row r="473">
       <c r="A473" s="2" t="inlineStr">
         <is>
-          <t>NR46</t>
+          <t>NR10</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="A474" s="2" t="inlineStr">
         <is>
-          <t>NR47</t>
+          <t>NR11</t>
         </is>
       </c>
     </row>
     <row r="475">
       <c r="A475" s="2" t="inlineStr">
         <is>
-          <t>NR52</t>
+          <t>NR12</t>
         </is>
       </c>
     </row>
     <row r="476">
       <c r="A476" s="2" t="inlineStr">
         <is>
-          <t>NR54</t>
+          <t>NR13</t>
         </is>
       </c>
     </row>
     <row r="477">
       <c r="A477" s="2" t="inlineStr">
         <is>
-          <t>NR56</t>
+          <t>NR14</t>
         </is>
       </c>
     </row>
     <row r="478">
       <c r="A478" s="2" t="inlineStr">
         <is>
-          <t>NR60</t>
+          <t>NR17</t>
         </is>
       </c>
     </row>
     <row r="479">
       <c r="A479" s="2" t="inlineStr">
         <is>
-          <t>NR64</t>
+          <t>NR20</t>
         </is>
       </c>
     </row>
     <row r="480">
       <c r="A480" s="2" t="inlineStr">
         <is>
-          <t>NR65</t>
+          <t>NR31</t>
         </is>
       </c>
     </row>
     <row r="481">
       <c r="A481" s="2" t="inlineStr">
         <is>
-          <t>NR68</t>
+          <t>NR35</t>
         </is>
       </c>
     </row>
     <row r="482">
       <c r="A482" s="2" t="inlineStr">
         <is>
-          <t>NR75</t>
+          <t>NR37</t>
         </is>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="2" t="inlineStr">
         <is>
-          <t>NR76</t>
+          <t>NR44</t>
         </is>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="2" t="inlineStr">
         <is>
-          <t>NR78</t>
+          <t>NR46</t>
         </is>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="2" t="inlineStr">
         <is>
-          <t>NR82</t>
+          <t>NR47</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="2" t="inlineStr">
         <is>
-          <t>NR83</t>
+          <t>NR52</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="2" t="inlineStr">
         <is>
-          <t>NR88</t>
+          <t>NR54</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" s="2" t="inlineStr">
         <is>
-          <t>NR91</t>
+          <t>NR56</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" s="2" t="inlineStr">
         <is>
-          <t>NR93</t>
+          <t>NR60</t>
         </is>
       </c>
     </row>
     <row r="490">
       <c r="A490" s="2" t="inlineStr">
         <is>
-          <t>NR94</t>
+          <t>NR64</t>
         </is>
       </c>
     </row>
     <row r="491">
       <c r="A491" s="2" t="inlineStr">
         <is>
-          <t>NR95</t>
+          <t>NR65</t>
         </is>
       </c>
     </row>
     <row r="492">
       <c r="A492" s="2" t="inlineStr">
         <is>
-          <t>NR97</t>
+          <t>NR68</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="2" t="inlineStr">
         <is>
-          <t>NR102</t>
+          <t>NR75</t>
         </is>
       </c>
     </row>
     <row r="494">
       <c r="A494" s="2" t="inlineStr">
         <is>
-          <t>NR106</t>
+          <t>NR76</t>
         </is>
       </c>
     </row>
     <row r="495">
       <c r="A495" s="2" t="inlineStr">
         <is>
-          <t>NR107</t>
+          <t>NR78</t>
         </is>
       </c>
     </row>
     <row r="496">
       <c r="A496" s="2" t="inlineStr">
         <is>
-          <t>NR109</t>
+          <t>NR82</t>
         </is>
       </c>
     </row>
     <row r="497">
       <c r="A497" s="2" t="inlineStr">
         <is>
-          <t>NR112</t>
+          <t>NR83</t>
         </is>
       </c>
     </row>
     <row r="498">
       <c r="A498" s="2" t="inlineStr">
         <is>
-          <t>NR113</t>
+          <t>NR88</t>
         </is>
       </c>
     </row>
     <row r="499">
       <c r="A499" s="2" t="inlineStr">
         <is>
-          <t>NR115</t>
+          <t>NR91</t>
         </